<commit_message>
Expand item brainstorming with field gear resources and hybrid fauna
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,11 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R83fb3b97ed824eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R91a466bd7b1d490e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R21edbf3232504ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R43da7ce8a76841ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R6645d5f18f0c469c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="Rc9dd72c09de341c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R08d3808e22594dfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R5fb7f71d37554fed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Ra7bf41a8f1e64e12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R31bd2a341b8f47b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R02b1924a016d46c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rf405ec8950354877"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -50,7 +52,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -77,6 +79,21 @@
         <x:fgColor rgb="FFFFF5D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF423B35"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -90,7 +107,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -170,15 +187,37 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="1">
+  <x:dxfs count="2">
     <x:dxf>
       <x:font>
         <x:color rgb="FF8A5B22"/>
       </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF87521B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF0D9"/>
+        </x:patternFill>
+      </x:fill>
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
@@ -202,7 +241,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -282,10 +321,43 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ResourcechainsTable" displayName="ResourcechainsTable" ref="A5:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Input concept ID"/>
+    <x:tableColumn id="2" name="Output concept ID"/>
+    <x:tableColumn id="3" name="Processing concept"/>
+    <x:tableColumn id="4" name="Potential use"/>
+    <x:tableColumn id="5" name="Work location"/>
+    <x:tableColumn id="6" name="Open constraint"/>
+    <x:tableColumn id="7" name="Status"/>
+    <x:tableColumn id="8" name="Basis"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="CreatureconceptsTable" displayName="CreatureconceptsTable" ref="A5:I10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="Concept ID"/>
+    <x:tableColumn id="2" name="Working description"/>
+    <x:tableColumn id="3" name="Hybrid anatomy"/>
+    <x:tableColumn id="4" name="Ecological role"/>
+    <x:tableColumn id="5" name="Expedition decision"/>
+    <x:tableColumn id="6" name="Resource concept IDs"/>
+    <x:tableColumn id="7" name="Collection alternative"/>
+    <x:tableColumn id="8" name="Open design issue"/>
+    <x:tableColumn id="9" name="Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -565,7 +637,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>Filter by category or scope. Blank stats are undecided. Trial values are shown where overrides exist.</x:v>
+        <x:v>Existing items plus user direction and new proposals. Filter Implementation scope before comparing stats.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -1687,9 +1759,1676 @@
         <x:v>Assets/_Project/Settings/Items/CampLoopIronstone/2-MineralSand.asset; Docs/Evidence/Gameplay/CampIronstone20261014/README.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="66" customHeight="1">
+      <x:c r="A24" s="9" t="str">
+        <x:v>proposal.gear.magnets</x:v>
+      </x:c>
+      <x:c r="B24" s="9" t="str">
+        <x:v>Field magnets</x:v>
+      </x:c>
+      <x:c r="C24" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D24" s="9" t="str">
+        <x:v>Magnetic recovery</x:v>
+      </x:c>
+      <x:c r="E24" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F24" s="9" t="str">
+        <x:v>Carry magnets for field work. Proposed uses: recover ferrous fragments and hold small workpieces.</x:v>
+      </x:c>
+      <x:c r="G24" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H24" s="9" t="str">
+        <x:v>Booter intended; storage TBD</x:v>
+      </x:c>
+      <x:c r="I24" s="13"/>
+      <x:c r="J24" s="15"/>
+      <x:c r="K24" s="9" t="str">
+        <x:v>Booter-carried equipment requested by author</x:v>
+      </x:c>
+      <x:c r="L24" s="9" t="str">
+        <x:v>Links to magnetite/iron and salvage chains</x:v>
+      </x:c>
+      <x:c r="M24" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N24" s="9" t="str">
+        <x:v>Magnet use, strength and mounting are proposals; not all materials are magnetic.</x:v>
+      </x:c>
+      <x:c r="O24" s="22"/>
+      <x:c r="P24" s="22"/>
+      <x:c r="Q24" s="22"/>
+      <x:c r="R24" s="22"/>
+      <x:c r="S24" s="22"/>
+      <x:c r="T24" s="9" t="str">
+        <x:v>Permanent versus powered; handling controls; carry location</x:v>
+      </x:c>
+      <x:c r="U24" s="23"/>
+      <x:c r="V24" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="66" customHeight="1">
+      <x:c r="A25" s="9" t="str">
+        <x:v>proposal.gear.grounding_kit</x:v>
+      </x:c>
+      <x:c r="B25" s="9" t="str">
+        <x:v>Static grounding kit</x:v>
+      </x:c>
+      <x:c r="C25" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D25" s="9" t="str">
+        <x:v>Charge management</x:v>
+      </x:c>
+      <x:c r="E25" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F25" s="9" t="str">
+        <x:v>Ground Booter against atmospheric static. Proposed kit: body contact, controlled discharge lead and ground contact.</x:v>
+      </x:c>
+      <x:c r="G25" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H25" s="9" t="str">
+        <x:v>Booter intended; storage TBD</x:v>
+      </x:c>
+      <x:c r="I25" s="13"/>
+      <x:c r="J25" s="15"/>
+      <x:c r="K25" s="9" t="str">
+        <x:v>Booter-carried equipment requested by author</x:v>
+      </x:c>
+      <x:c r="L25" s="9" t="str">
+        <x:v>Potential conductive braid, graphite and insulating ceramic components</x:v>
+      </x:c>
+      <x:c r="M25" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N25" s="9" t="str">
+        <x:v>Fictional game mechanic to design; contact quality matters; no immunity to lightning assumed.</x:v>
+      </x:c>
+      <x:c r="O25" s="22"/>
+      <x:c r="P25" s="22"/>
+      <x:c r="Q25" s="22"/>
+      <x:c r="R25" s="22"/>
+      <x:c r="S25" s="22"/>
+      <x:c r="T25" s="9" t="str">
+        <x:v>Ground-contact suitability; deployment; feedback; relation to storms; carry location</x:v>
+      </x:c>
+      <x:c r="U25" s="23"/>
+      <x:c r="V25" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="66" customHeight="1">
+      <x:c r="A26" s="9" t="str">
+        <x:v>proposal.natural.magnetite</x:v>
+      </x:c>
+      <x:c r="B26" s="9" t="str">
+        <x:v>Magnetite-rich stone</x:v>
+      </x:c>
+      <x:c r="C26" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D26" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E26" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F26" s="9" t="str">
+        <x:v>Iron feed and magnetic tool research</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H26" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I26" s="13"/>
+      <x:c r="J26" s="15"/>
+      <x:c r="K26" s="9" t="str">
+        <x:v>Magnetic mineral seams and dense dark nodules</x:v>
+      </x:c>
+      <x:c r="L26" s="9" t="str">
+        <x:v>Dry crush and magnetic separation</x:v>
+      </x:c>
+      <x:c r="M26" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N26" s="9" t="str">
+        <x:v>New deposit and processing design; no free natural liquid water.</x:v>
+      </x:c>
+      <x:c r="O26" s="22"/>
+      <x:c r="P26" s="22"/>
+      <x:c r="Q26" s="22"/>
+      <x:c r="R26" s="22"/>
+      <x:c r="S26" s="22"/>
+      <x:c r="T26" s="9" t="str">
+        <x:v>Distribution, collection tool, processing constraints and balance</x:v>
+      </x:c>
+      <x:c r="U26" s="23"/>
+      <x:c r="V26" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="66" customHeight="1">
+      <x:c r="A27" s="9" t="str">
+        <x:v>proposal.natural.silica</x:v>
+      </x:c>
+      <x:c r="B27" s="9" t="str">
+        <x:v>Silica-rich grit</x:v>
+      </x:c>
+      <x:c r="C27" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D27" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E27" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F27" s="9" t="str">
+        <x:v>Sharpening, finishing and repair</x:v>
+      </x:c>
+      <x:c r="G27" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H27" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I27" s="13"/>
+      <x:c r="J27" s="15"/>
+      <x:c r="K27" s="9" t="str">
+        <x:v>Dry canyon scree and exposed mineral beds</x:v>
+      </x:c>
+      <x:c r="L27" s="9" t="str">
+        <x:v>Grade into abrasive; high-heat glass route left open</x:v>
+      </x:c>
+      <x:c r="M27" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N27" s="9" t="str">
+        <x:v>New deposit and processing design; no free natural liquid water.</x:v>
+      </x:c>
+      <x:c r="O27" s="22"/>
+      <x:c r="P27" s="22"/>
+      <x:c r="Q27" s="22"/>
+      <x:c r="R27" s="22"/>
+      <x:c r="S27" s="22"/>
+      <x:c r="T27" s="9" t="str">
+        <x:v>Distribution, collection tool, processing constraints and balance</x:v>
+      </x:c>
+      <x:c r="U27" s="23"/>
+      <x:c r="V27" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="66" customHeight="1">
+      <x:c r="A28" s="9" t="str">
+        <x:v>proposal.natural.alumina</x:v>
+      </x:c>
+      <x:c r="B28" s="9" t="str">
+        <x:v>Alumina-rich rock</x:v>
+      </x:c>
+      <x:c r="C28" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D28" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E28" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F28" s="9" t="str">
+        <x:v>Hard ceramic and electrical separation parts</x:v>
+      </x:c>
+      <x:c r="G28" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H28" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I28" s="13"/>
+      <x:c r="J28" s="15"/>
+      <x:c r="K28" s="9" t="str">
+        <x:v>Authored mineral outcrops</x:v>
+      </x:c>
+      <x:c r="L28" s="9" t="str">
+        <x:v>Crush, grade and fire with suitable binder</x:v>
+      </x:c>
+      <x:c r="M28" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N28" s="9" t="str">
+        <x:v>New deposit and processing design; no free natural liquid water.</x:v>
+      </x:c>
+      <x:c r="O28" s="22"/>
+      <x:c r="P28" s="22"/>
+      <x:c r="Q28" s="22"/>
+      <x:c r="R28" s="22"/>
+      <x:c r="S28" s="22"/>
+      <x:c r="T28" s="9" t="str">
+        <x:v>Distribution, collection tool, processing constraints and balance</x:v>
+      </x:c>
+      <x:c r="U28" s="23"/>
+      <x:c r="V28" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="66" customHeight="1">
+      <x:c r="A29" s="9" t="str">
+        <x:v>proposal.natural.claystone</x:v>
+      </x:c>
+      <x:c r="B29" s="9" t="str">
+        <x:v>Claystone</x:v>
+      </x:c>
+      <x:c r="C29" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D29" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E29" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F29" s="9" t="str">
+        <x:v>Ceramic bodies and refractory parts</x:v>
+      </x:c>
+      <x:c r="G29" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H29" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I29" s="13"/>
+      <x:c r="J29" s="15"/>
+      <x:c r="K29" s="9" t="str">
+        <x:v>Ancient dry sediment beds</x:v>
+      </x:c>
+      <x:c r="L29" s="9" t="str">
+        <x:v>Dry mill for ceramic feed; binder method unresolved</x:v>
+      </x:c>
+      <x:c r="M29" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N29" s="9" t="str">
+        <x:v>New deposit and processing design; no free natural liquid water.</x:v>
+      </x:c>
+      <x:c r="O29" s="22"/>
+      <x:c r="P29" s="22"/>
+      <x:c r="Q29" s="22"/>
+      <x:c r="R29" s="22"/>
+      <x:c r="S29" s="22"/>
+      <x:c r="T29" s="9" t="str">
+        <x:v>Distribution, collection tool, processing constraints and balance</x:v>
+      </x:c>
+      <x:c r="U29" s="23"/>
+      <x:c r="V29" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="66" customHeight="1">
+      <x:c r="A30" s="9" t="str">
+        <x:v>proposal.natural.carbonate</x:v>
+      </x:c>
+      <x:c r="B30" s="9" t="str">
+        <x:v>Carbonate stone</x:v>
+      </x:c>
+      <x:c r="C30" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D30" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E30" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F30" s="9" t="str">
+        <x:v>Mineral binder and construction research</x:v>
+      </x:c>
+      <x:c r="G30" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H30" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I30" s="13"/>
+      <x:c r="J30" s="15"/>
+      <x:c r="K30" s="9" t="str">
+        <x:v>Ancient exposed deposits</x:v>
+      </x:c>
+      <x:c r="L30" s="9" t="str">
+        <x:v>Heat to lime; use dry aggregate formulation</x:v>
+      </x:c>
+      <x:c r="M30" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N30" s="9" t="str">
+        <x:v>New deposit and processing design; no free natural liquid water.</x:v>
+      </x:c>
+      <x:c r="O30" s="22"/>
+      <x:c r="P30" s="22"/>
+      <x:c r="Q30" s="22"/>
+      <x:c r="R30" s="22"/>
+      <x:c r="S30" s="22"/>
+      <x:c r="T30" s="9" t="str">
+        <x:v>Distribution, collection tool, processing constraints and balance</x:v>
+      </x:c>
+      <x:c r="U30" s="23"/>
+      <x:c r="V30" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="66" customHeight="1">
+      <x:c r="A31" s="9" t="str">
+        <x:v>proposal.natural.salts</x:v>
+      </x:c>
+      <x:c r="B31" s="9" t="str">
+        <x:v>Dry mineral salts</x:v>
+      </x:c>
+      <x:c r="C31" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D31" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E31" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F31" s="9" t="str">
+        <x:v>Algae culture mineral inputs, subject to biology design</x:v>
+      </x:c>
+      <x:c r="G31" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H31" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I31" s="13"/>
+      <x:c r="J31" s="15"/>
+      <x:c r="K31" s="9" t="str">
+        <x:v>Ancient evaporite seams; no current water required</x:v>
+      </x:c>
+      <x:c r="L31" s="9" t="str">
+        <x:v>Sort and grade dry crystals</x:v>
+      </x:c>
+      <x:c r="M31" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N31" s="9" t="str">
+        <x:v>New deposit and processing design; no free natural liquid water.</x:v>
+      </x:c>
+      <x:c r="O31" s="22"/>
+      <x:c r="P31" s="22"/>
+      <x:c r="Q31" s="22"/>
+      <x:c r="R31" s="22"/>
+      <x:c r="S31" s="22"/>
+      <x:c r="T31" s="9" t="str">
+        <x:v>Distribution, collection tool, processing constraints and balance</x:v>
+      </x:c>
+      <x:c r="U31" s="23"/>
+      <x:c r="V31" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="66" customHeight="1">
+      <x:c r="A32" s="9" t="str">
+        <x:v>proposal.natural.graphite</x:v>
+      </x:c>
+      <x:c r="B32" s="9" t="str">
+        <x:v>Graphite-bearing stone</x:v>
+      </x:c>
+      <x:c r="C32" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D32" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E32" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F32" s="9" t="str">
+        <x:v>Dry lubrication and conductive composites</x:v>
+      </x:c>
+      <x:c r="G32" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H32" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I32" s="13"/>
+      <x:c r="J32" s="15"/>
+      <x:c r="K32" s="9" t="str">
+        <x:v>Sparse mineral seams</x:v>
+      </x:c>
+      <x:c r="L32" s="9" t="str">
+        <x:v>Separate and grade carbon flakes</x:v>
+      </x:c>
+      <x:c r="M32" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N32" s="9" t="str">
+        <x:v>New deposit and processing design; no free natural liquid water.</x:v>
+      </x:c>
+      <x:c r="O32" s="22"/>
+      <x:c r="P32" s="22"/>
+      <x:c r="Q32" s="22"/>
+      <x:c r="R32" s="22"/>
+      <x:c r="S32" s="22"/>
+      <x:c r="T32" s="9" t="str">
+        <x:v>Distribution, collection tool, processing constraints and balance</x:v>
+      </x:c>
+      <x:c r="U32" s="23"/>
+      <x:c r="V32" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="66" customHeight="1">
+      <x:c r="A33" s="9" t="str">
+        <x:v>proposal.natural.mica</x:v>
+      </x:c>
+      <x:c r="B33" s="9" t="str">
+        <x:v>Mica sheets</x:v>
+      </x:c>
+      <x:c r="C33" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D33" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E33" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F33" s="9" t="str">
+        <x:v>Insulating separators and heat shields</x:v>
+      </x:c>
+      <x:c r="G33" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H33" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I33" s="13"/>
+      <x:c r="J33" s="15"/>
+      <x:c r="K33" s="9" t="str">
+        <x:v>Layered mineral outcrops</x:v>
+      </x:c>
+      <x:c r="L33" s="9" t="str">
+        <x:v>Split and trim plates</x:v>
+      </x:c>
+      <x:c r="M33" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N33" s="9" t="str">
+        <x:v>New deposit and processing design; no free natural liquid water.</x:v>
+      </x:c>
+      <x:c r="O33" s="22"/>
+      <x:c r="P33" s="22"/>
+      <x:c r="Q33" s="22"/>
+      <x:c r="R33" s="22"/>
+      <x:c r="S33" s="22"/>
+      <x:c r="T33" s="9" t="str">
+        <x:v>Distribution, collection tool, processing constraints and balance</x:v>
+      </x:c>
+      <x:c r="U33" s="23"/>
+      <x:c r="V33" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="66" customHeight="1">
+      <x:c r="A34" s="9" t="str">
+        <x:v>proposal.natural.iron_feed</x:v>
+      </x:c>
+      <x:c r="B34" s="9" t="str">
+        <x:v>Iron-rich mineral feed</x:v>
+      </x:c>
+      <x:c r="C34" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D34" s="9" t="str">
+        <x:v>Processed mineral</x:v>
+      </x:c>
+      <x:c r="E34" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F34" s="9" t="str">
+        <x:v>Intermediate feed for an eventual furnace</x:v>
+      </x:c>
+      <x:c r="G34" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H34" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I34" s="13"/>
+      <x:c r="J34" s="15"/>
+      <x:c r="K34" s="9" t="str">
+        <x:v>Process magnetite</x:v>
+      </x:c>
+      <x:c r="L34" s="9" t="str">
+        <x:v>Dry crush and magnetic separation</x:v>
+      </x:c>
+      <x:c r="M34" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N34" s="9" t="str">
+        <x:v>Distinct proposal from existing Iron-rich Concentrate; decide whether to merge them.</x:v>
+      </x:c>
+      <x:c r="O34" s="22"/>
+      <x:c r="P34" s="22"/>
+      <x:c r="Q34" s="22"/>
+      <x:c r="R34" s="22"/>
+      <x:c r="S34" s="22"/>
+      <x:c r="T34" s="9" t="str">
+        <x:v>Choose production chain and possible reuse of existing item definitions</x:v>
+      </x:c>
+      <x:c r="U34" s="23"/>
+      <x:c r="V34" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="66" customHeight="1">
+      <x:c r="A35" s="9" t="str">
+        <x:v>proposal.natural.iron_stock</x:v>
+      </x:c>
+      <x:c r="B35" s="9" t="str">
+        <x:v>Worked iron stock</x:v>
+      </x:c>
+      <x:c r="C35" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D35" s="9" t="str">
+        <x:v>Processed mineral</x:v>
+      </x:c>
+      <x:c r="E35" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F35" s="9" t="str">
+        <x:v>Repair stock, fasteners and structural tool parts</x:v>
+      </x:c>
+      <x:c r="G35" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H35" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I35" s="13"/>
+      <x:c r="J35" s="15"/>
+      <x:c r="K35" s="9" t="str">
+        <x:v>Process iron_feed</x:v>
+      </x:c>
+      <x:c r="L35" s="9" t="str">
+        <x:v>Smelt, forge and finish at a stationary facility</x:v>
+      </x:c>
+      <x:c r="M35" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N35" s="9" t="str">
+        <x:v>Fuel, furnace, alloy and process choices unresolved; no Legger crafting platform.</x:v>
+      </x:c>
+      <x:c r="O35" s="22"/>
+      <x:c r="P35" s="22"/>
+      <x:c r="Q35" s="22"/>
+      <x:c r="R35" s="22"/>
+      <x:c r="S35" s="22"/>
+      <x:c r="T35" s="9" t="str">
+        <x:v>Choose production chain and possible reuse of existing item definitions</x:v>
+      </x:c>
+      <x:c r="U35" s="23"/>
+      <x:c r="V35" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="66" customHeight="1">
+      <x:c r="A36" s="9" t="str">
+        <x:v>proposal.natural.abrasive</x:v>
+      </x:c>
+      <x:c r="B36" s="9" t="str">
+        <x:v>Graded abrasive grit</x:v>
+      </x:c>
+      <x:c r="C36" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D36" s="9" t="str">
+        <x:v>Processed mineral</x:v>
+      </x:c>
+      <x:c r="E36" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F36" s="9" t="str">
+        <x:v>Tool sharpening and surface preparation</x:v>
+      </x:c>
+      <x:c r="G36" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H36" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I36" s="13"/>
+      <x:c r="J36" s="15"/>
+      <x:c r="K36" s="9" t="str">
+        <x:v>Process silica</x:v>
+      </x:c>
+      <x:c r="L36" s="9" t="str">
+        <x:v>Dry sieve and grade</x:v>
+      </x:c>
+      <x:c r="M36" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N36" s="9" t="str">
+        <x:v>Could reuse existing Mineral Sand instead; resolve before implementation.</x:v>
+      </x:c>
+      <x:c r="O36" s="22"/>
+      <x:c r="P36" s="22"/>
+      <x:c r="Q36" s="22"/>
+      <x:c r="R36" s="22"/>
+      <x:c r="S36" s="22"/>
+      <x:c r="T36" s="9" t="str">
+        <x:v>Choose production chain and possible reuse of existing item definitions</x:v>
+      </x:c>
+      <x:c r="U36" s="23"/>
+      <x:c r="V36" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="66" customHeight="1">
+      <x:c r="A37" s="9" t="str">
+        <x:v>proposal.natural.ceramic</x:v>
+      </x:c>
+      <x:c r="B37" s="9" t="str">
+        <x:v>Insulating ceramic blanks</x:v>
+      </x:c>
+      <x:c r="C37" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D37" s="9" t="str">
+        <x:v>Processed mineral</x:v>
+      </x:c>
+      <x:c r="E37" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F37" s="9" t="str">
+        <x:v>Grounding-kit spacers and heat-resistant fixtures</x:v>
+      </x:c>
+      <x:c r="G37" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H37" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I37" s="13"/>
+      <x:c r="J37" s="15"/>
+      <x:c r="K37" s="9" t="str">
+        <x:v>Process alumina</x:v>
+      </x:c>
+      <x:c r="L37" s="9" t="str">
+        <x:v>Dry feed preparation, forming and firing</x:v>
+      </x:c>
+      <x:c r="M37" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N37" s="9" t="str">
+        <x:v>Claystone may be a co-input; forming binder/energy not settled.</x:v>
+      </x:c>
+      <x:c r="O37" s="22"/>
+      <x:c r="P37" s="22"/>
+      <x:c r="Q37" s="22"/>
+      <x:c r="R37" s="22"/>
+      <x:c r="S37" s="22"/>
+      <x:c r="T37" s="9" t="str">
+        <x:v>Choose production chain and possible reuse of existing item definitions</x:v>
+      </x:c>
+      <x:c r="U37" s="23"/>
+      <x:c r="V37" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="66" customHeight="1">
+      <x:c r="A38" s="9" t="str">
+        <x:v>proposal.natural.lime</x:v>
+      </x:c>
+      <x:c r="B38" s="9" t="str">
+        <x:v>Calcined mineral binder</x:v>
+      </x:c>
+      <x:c r="C38" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D38" s="9" t="str">
+        <x:v>Processed mineral</x:v>
+      </x:c>
+      <x:c r="E38" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F38" s="9" t="str">
+        <x:v>Dry composite repair and construction</x:v>
+      </x:c>
+      <x:c r="G38" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H38" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I38" s="13"/>
+      <x:c r="J38" s="15"/>
+      <x:c r="K38" s="9" t="str">
+        <x:v>Process carbonate</x:v>
+      </x:c>
+      <x:c r="L38" s="9" t="str">
+        <x:v>Heat mineral feed; retain dry product</x:v>
+      </x:c>
+      <x:c r="M38" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N38" s="9" t="str">
+        <x:v>No conventional water-based cement recipe assumed.</x:v>
+      </x:c>
+      <x:c r="O38" s="22"/>
+      <x:c r="P38" s="22"/>
+      <x:c r="Q38" s="22"/>
+      <x:c r="R38" s="22"/>
+      <x:c r="S38" s="22"/>
+      <x:c r="T38" s="9" t="str">
+        <x:v>Choose production chain and possible reuse of existing item definitions</x:v>
+      </x:c>
+      <x:c r="U38" s="23"/>
+      <x:c r="V38" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="66" customHeight="1">
+      <x:c r="A39" s="9" t="str">
+        <x:v>proposal.natural.carbon</x:v>
+      </x:c>
+      <x:c r="B39" s="9" t="str">
+        <x:v>Graded graphite flakes</x:v>
+      </x:c>
+      <x:c r="C39" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D39" s="9" t="str">
+        <x:v>Processed mineral</x:v>
+      </x:c>
+      <x:c r="E39" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F39" s="9" t="str">
+        <x:v>Dry lubricant; conductive composite ingredient</x:v>
+      </x:c>
+      <x:c r="G39" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H39" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I39" s="13"/>
+      <x:c r="J39" s="15"/>
+      <x:c r="K39" s="9" t="str">
+        <x:v>Process graphite</x:v>
+      </x:c>
+      <x:c r="L39" s="9" t="str">
+        <x:v>Crush and dry grade</x:v>
+      </x:c>
+      <x:c r="M39" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N39" s="9" t="str">
+        <x:v>Not a power source; graphite behavior and recipe details remain provisional.</x:v>
+      </x:c>
+      <x:c r="O39" s="22"/>
+      <x:c r="P39" s="22"/>
+      <x:c r="Q39" s="22"/>
+      <x:c r="R39" s="22"/>
+      <x:c r="S39" s="22"/>
+      <x:c r="T39" s="9" t="str">
+        <x:v>Choose production chain and possible reuse of existing item definitions</x:v>
+      </x:c>
+      <x:c r="U39" s="23"/>
+      <x:c r="V39" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="66" customHeight="1">
+      <x:c r="A40" s="9" t="str">
+        <x:v>proposal.bio.shell</x:v>
+      </x:c>
+      <x:c r="B40" s="9" t="str">
+        <x:v>Shed shell plates</x:v>
+      </x:c>
+      <x:c r="C40" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D40" s="9" t="str">
+        <x:v>Molted exoskeleton</x:v>
+      </x:c>
+      <x:c r="E40" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F40" s="9" t="str">
+        <x:v>Layered armor, shields and tool guards</x:v>
+      </x:c>
+      <x:c r="G40" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H40" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I40" s="13"/>
+      <x:c r="J40" s="15"/>
+      <x:c r="K40" s="9" t="str">
+        <x:v>Molts and carcasses of plate-backed fauna</x:v>
+      </x:c>
+      <x:c r="L40" s="9" t="str">
+        <x:v>See Resource chains</x:v>
+      </x:c>
+      <x:c r="M40" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N40" s="9" t="str">
+        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+      </x:c>
+      <x:c r="O40" s="22"/>
+      <x:c r="P40" s="22"/>
+      <x:c r="Q40" s="22"/>
+      <x:c r="R40" s="22"/>
+      <x:c r="S40" s="22"/>
+      <x:c r="T40" s="9" t="str">
+        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+      </x:c>
+      <x:c r="U40" s="23"/>
+      <x:c r="V40" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="66" customHeight="1">
+      <x:c r="A41" s="9" t="str">
+        <x:v>proposal.bio.tendon</x:v>
+      </x:c>
+      <x:c r="B41" s="9" t="str">
+        <x:v>Dried tendon bundles</x:v>
+      </x:c>
+      <x:c r="C41" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D41" s="9" t="str">
+        <x:v>Connective tissue</x:v>
+      </x:c>
+      <x:c r="E41" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F41" s="9" t="str">
+        <x:v>Cordage and flexible bindings</x:v>
+      </x:c>
+      <x:c r="G41" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H41" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I41" s="13"/>
+      <x:c r="J41" s="15"/>
+      <x:c r="K41" s="9" t="str">
+        <x:v>Carcass joints and limb anchors</x:v>
+      </x:c>
+      <x:c r="L41" s="9" t="str">
+        <x:v>See Resource chains</x:v>
+      </x:c>
+      <x:c r="M41" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N41" s="9" t="str">
+        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+      </x:c>
+      <x:c r="O41" s="22"/>
+      <x:c r="P41" s="22"/>
+      <x:c r="Q41" s="22"/>
+      <x:c r="R41" s="22"/>
+      <x:c r="S41" s="22"/>
+      <x:c r="T41" s="9" t="str">
+        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+      </x:c>
+      <x:c r="U41" s="23"/>
+      <x:c r="V41" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="66" customHeight="1">
+      <x:c r="A42" s="9" t="str">
+        <x:v>proposal.bio.bristles</x:v>
+      </x:c>
+      <x:c r="B42" s="9" t="str">
+        <x:v>Coarse sensory bristles</x:v>
+      </x:c>
+      <x:c r="C42" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D42" s="9" t="str">
+        <x:v>Dry fibers</x:v>
+      </x:c>
+      <x:c r="E42" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F42" s="9" t="str">
+        <x:v>Dust seals, brushes and filter research</x:v>
+      </x:c>
+      <x:c r="G42" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H42" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I42" s="13"/>
+      <x:c r="J42" s="15"/>
+      <x:c r="K42" s="9" t="str">
+        <x:v>Shed bristles and carcass brushes</x:v>
+      </x:c>
+      <x:c r="L42" s="9" t="str">
+        <x:v>See Resource chains</x:v>
+      </x:c>
+      <x:c r="M42" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N42" s="9" t="str">
+        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+      </x:c>
+      <x:c r="O42" s="22"/>
+      <x:c r="P42" s="22"/>
+      <x:c r="Q42" s="22"/>
+      <x:c r="R42" s="22"/>
+      <x:c r="S42" s="22"/>
+      <x:c r="T42" s="9" t="str">
+        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+      </x:c>
+      <x:c r="U42" s="23"/>
+      <x:c r="V42" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="66" customHeight="1">
+      <x:c r="A43" s="9" t="str">
+        <x:v>proposal.bio.underfur</x:v>
+      </x:c>
+      <x:c r="B43" s="9" t="str">
+        <x:v>Shed underfur</x:v>
+      </x:c>
+      <x:c r="C43" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D43" s="9" t="str">
+        <x:v>Dry fibers</x:v>
+      </x:c>
+      <x:c r="E43" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F43" s="9" t="str">
+        <x:v>Clothing liners and dust buffers</x:v>
+      </x:c>
+      <x:c r="G43" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H43" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I43" s="13"/>
+      <x:c r="J43" s="15"/>
+      <x:c r="K43" s="9" t="str">
+        <x:v>Abandoned resting hollows and natural shedding</x:v>
+      </x:c>
+      <x:c r="L43" s="9" t="str">
+        <x:v>See Resource chains</x:v>
+      </x:c>
+      <x:c r="M43" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N43" s="9" t="str">
+        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+      </x:c>
+      <x:c r="O43" s="22"/>
+      <x:c r="P43" s="22"/>
+      <x:c r="Q43" s="22"/>
+      <x:c r="R43" s="22"/>
+      <x:c r="S43" s="22"/>
+      <x:c r="T43" s="9" t="str">
+        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+      </x:c>
+      <x:c r="U43" s="23"/>
+      <x:c r="V43" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="66" customHeight="1">
+      <x:c r="A44" s="9" t="str">
+        <x:v>proposal.bio.jaw</x:v>
+      </x:c>
+      <x:c r="B44" s="9" t="str">
+        <x:v>Dense jaw plates</x:v>
+      </x:c>
+      <x:c r="C44" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D44" s="9" t="str">
+        <x:v>Hard tissue</x:v>
+      </x:c>
+      <x:c r="E44" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F44" s="9" t="str">
+        <x:v>Tool edges and wear inserts</x:v>
+      </x:c>
+      <x:c r="G44" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H44" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I44" s="13"/>
+      <x:c r="J44" s="15"/>
+      <x:c r="K44" s="9" t="str">
+        <x:v>Carcass chewing and digging mouthparts</x:v>
+      </x:c>
+      <x:c r="L44" s="9" t="str">
+        <x:v>See Resource chains</x:v>
+      </x:c>
+      <x:c r="M44" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N44" s="9" t="str">
+        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+      </x:c>
+      <x:c r="O44" s="22"/>
+      <x:c r="P44" s="22"/>
+      <x:c r="Q44" s="22"/>
+      <x:c r="R44" s="22"/>
+      <x:c r="S44" s="22"/>
+      <x:c r="T44" s="9" t="str">
+        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+      </x:c>
+      <x:c r="U44" s="23"/>
+      <x:c r="V44" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="66" customHeight="1">
+      <x:c r="A45" s="9" t="str">
+        <x:v>proposal.bio.membrane</x:v>
+      </x:c>
+      <x:c r="B45" s="9" t="str">
+        <x:v>Dried joint membrane</x:v>
+      </x:c>
+      <x:c r="C45" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D45" s="9" t="str">
+        <x:v>Flexible tissue</x:v>
+      </x:c>
+      <x:c r="E45" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F45" s="9" t="str">
+        <x:v>Flexible seals and patch material</x:v>
+      </x:c>
+      <x:c r="G45" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H45" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I45" s="13"/>
+      <x:c r="J45" s="15"/>
+      <x:c r="K45" s="9" t="str">
+        <x:v>Carcass limb joints and body folds</x:v>
+      </x:c>
+      <x:c r="L45" s="9" t="str">
+        <x:v>See Resource chains</x:v>
+      </x:c>
+      <x:c r="M45" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N45" s="9" t="str">
+        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+      </x:c>
+      <x:c r="O45" s="22"/>
+      <x:c r="P45" s="22"/>
+      <x:c r="Q45" s="22"/>
+      <x:c r="R45" s="22"/>
+      <x:c r="S45" s="22"/>
+      <x:c r="T45" s="9" t="str">
+        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+      </x:c>
+      <x:c r="U45" s="23"/>
+      <x:c r="V45" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="66" customHeight="1">
+      <x:c r="A46" s="9" t="str">
+        <x:v>proposal.bio.fat</x:v>
+      </x:c>
+      <x:c r="B46" s="9" t="str">
+        <x:v>Fresh fat-bearing tissue</x:v>
+      </x:c>
+      <x:c r="C46" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D46" s="9" t="str">
+        <x:v>Perishable tissue</x:v>
+      </x:c>
+      <x:c r="E46" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F46" s="9" t="str">
+        <x:v>Dry solid lubricant and binder research</x:v>
+      </x:c>
+      <x:c r="G46" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H46" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I46" s="13"/>
+      <x:c r="J46" s="15"/>
+      <x:c r="K46" s="9" t="str">
+        <x:v>Recent carcass; preservation rules required</x:v>
+      </x:c>
+      <x:c r="L46" s="9" t="str">
+        <x:v>See Resource chains</x:v>
+      </x:c>
+      <x:c r="M46" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N46" s="9" t="str">
+        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+      </x:c>
+      <x:c r="O46" s="22"/>
+      <x:c r="P46" s="22"/>
+      <x:c r="Q46" s="22"/>
+      <x:c r="R46" s="22"/>
+      <x:c r="S46" s="22"/>
+      <x:c r="T46" s="9" t="str">
+        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+      </x:c>
+      <x:c r="U46" s="23"/>
+      <x:c r="V46" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="66" customHeight="1">
+      <x:c r="A47" s="9" t="str">
+        <x:v>proposal.bio.organ</x:v>
+      </x:c>
+      <x:c r="B47" s="9" t="str">
+        <x:v>Charge-organ tissue</x:v>
+      </x:c>
+      <x:c r="C47" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D47" s="9" t="str">
+        <x:v>Specialized tissue</x:v>
+      </x:c>
+      <x:c r="E47" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F47" s="9" t="str">
+        <x:v>Dry electrode scaffold research, not bottled electricity</x:v>
+      </x:c>
+      <x:c r="G47" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H47" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I47" s="13"/>
+      <x:c r="J47" s="15"/>
+      <x:c r="K47" s="9" t="str">
+        <x:v>Rare storm-adapted fauna; anatomy provisional</x:v>
+      </x:c>
+      <x:c r="L47" s="9" t="str">
+        <x:v>See Resource chains</x:v>
+      </x:c>
+      <x:c r="M47" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N47" s="9" t="str">
+        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+      </x:c>
+      <x:c r="O47" s="22"/>
+      <x:c r="P47" s="22"/>
+      <x:c r="Q47" s="22"/>
+      <x:c r="R47" s="22"/>
+      <x:c r="S47" s="22"/>
+      <x:c r="T47" s="9" t="str">
+        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+      </x:c>
+      <x:c r="U47" s="23"/>
+      <x:c r="V47" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="66" customHeight="1">
+      <x:c r="A48" s="9" t="str">
+        <x:v>proposal.bio.laminate</x:v>
+      </x:c>
+      <x:c r="B48" s="9" t="str">
+        <x:v>Shell laminate</x:v>
+      </x:c>
+      <x:c r="C48" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D48" s="9" t="str">
+        <x:v>Processed biological</x:v>
+      </x:c>
+      <x:c r="E48" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F48" s="9" t="str">
+        <x:v>Light armor panels and impact guards</x:v>
+      </x:c>
+      <x:c r="G48" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H48" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I48" s="13"/>
+      <x:c r="J48" s="15"/>
+      <x:c r="K48" s="9" t="str">
+        <x:v>Process shell</x:v>
+      </x:c>
+      <x:c r="L48" s="9" t="str">
+        <x:v>Trim, layer and bind dry plates</x:v>
+      </x:c>
+      <x:c r="M48" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N48" s="9" t="str">
+        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+      </x:c>
+      <x:c r="O48" s="22"/>
+      <x:c r="P48" s="22"/>
+      <x:c r="Q48" s="22"/>
+      <x:c r="R48" s="22"/>
+      <x:c r="S48" s="22"/>
+      <x:c r="T48" s="9" t="str">
+        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+      </x:c>
+      <x:c r="U48" s="23"/>
+      <x:c r="V48" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="66" customHeight="1">
+      <x:c r="A49" s="9" t="str">
+        <x:v>proposal.bio.cord</x:v>
+      </x:c>
+      <x:c r="B49" s="9" t="str">
+        <x:v>Tendon cord</x:v>
+      </x:c>
+      <x:c r="C49" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D49" s="9" t="str">
+        <x:v>Processed biological</x:v>
+      </x:c>
+      <x:c r="E49" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F49" s="9" t="str">
+        <x:v>Tool lashings and field repairs</x:v>
+      </x:c>
+      <x:c r="G49" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H49" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I49" s="13"/>
+      <x:c r="J49" s="15"/>
+      <x:c r="K49" s="9" t="str">
+        <x:v>Process tendon</x:v>
+      </x:c>
+      <x:c r="L49" s="9" t="str">
+        <x:v>Dry, split, twist and bind</x:v>
+      </x:c>
+      <x:c r="M49" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N49" s="9" t="str">
+        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+      </x:c>
+      <x:c r="O49" s="22"/>
+      <x:c r="P49" s="22"/>
+      <x:c r="Q49" s="22"/>
+      <x:c r="R49" s="22"/>
+      <x:c r="S49" s="22"/>
+      <x:c r="T49" s="9" t="str">
+        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+      </x:c>
+      <x:c r="U49" s="23"/>
+      <x:c r="V49" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="66" customHeight="1">
+      <x:c r="A50" s="9" t="str">
+        <x:v>proposal.bio.brush</x:v>
+      </x:c>
+      <x:c r="B50" s="9" t="str">
+        <x:v>Bristle brush strips</x:v>
+      </x:c>
+      <x:c r="C50" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D50" s="9" t="str">
+        <x:v>Processed biological</x:v>
+      </x:c>
+      <x:c r="E50" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F50" s="9" t="str">
+        <x:v>Dust exclusion at joints and equipment closures</x:v>
+      </x:c>
+      <x:c r="G50" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H50" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I50" s="13"/>
+      <x:c r="J50" s="15"/>
+      <x:c r="K50" s="9" t="str">
+        <x:v>Process bristles</x:v>
+      </x:c>
+      <x:c r="L50" s="9" t="str">
+        <x:v>Sort fibers and bind into a backing</x:v>
+      </x:c>
+      <x:c r="M50" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N50" s="9" t="str">
+        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+      </x:c>
+      <x:c r="O50" s="22"/>
+      <x:c r="P50" s="22"/>
+      <x:c r="Q50" s="22"/>
+      <x:c r="R50" s="22"/>
+      <x:c r="S50" s="22"/>
+      <x:c r="T50" s="9" t="str">
+        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+      </x:c>
+      <x:c r="U50" s="23"/>
+      <x:c r="V50" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="66" customHeight="1">
+      <x:c r="A51" s="9" t="str">
+        <x:v>proposal.bio.liner</x:v>
+      </x:c>
+      <x:c r="B51" s="9" t="str">
+        <x:v>Felted underfur liner</x:v>
+      </x:c>
+      <x:c r="C51" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D51" s="9" t="str">
+        <x:v>Processed biological</x:v>
+      </x:c>
+      <x:c r="E51" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F51" s="9" t="str">
+        <x:v>Replaceable jacket/cloak liners</x:v>
+      </x:c>
+      <x:c r="G51" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H51" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I51" s="13"/>
+      <x:c r="J51" s="15"/>
+      <x:c r="K51" s="9" t="str">
+        <x:v>Process underfur</x:v>
+      </x:c>
+      <x:c r="L51" s="9" t="str">
+        <x:v>Dry clean, card and compress</x:v>
+      </x:c>
+      <x:c r="M51" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N51" s="9" t="str">
+        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+      </x:c>
+      <x:c r="O51" s="22"/>
+      <x:c r="P51" s="22"/>
+      <x:c r="Q51" s="22"/>
+      <x:c r="R51" s="22"/>
+      <x:c r="S51" s="22"/>
+      <x:c r="T51" s="9" t="str">
+        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+      </x:c>
+      <x:c r="U51" s="23"/>
+      <x:c r="V51" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="66" customHeight="1">
+      <x:c r="A52" s="9" t="str">
+        <x:v>proposal.bio.insert</x:v>
+      </x:c>
+      <x:c r="B52" s="9" t="str">
+        <x:v>Jaw cutting insert</x:v>
+      </x:c>
+      <x:c r="C52" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D52" s="9" t="str">
+        <x:v>Processed biological</x:v>
+      </x:c>
+      <x:c r="E52" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F52" s="9" t="str">
+        <x:v>Replaceable excavation-tool wear part</x:v>
+      </x:c>
+      <x:c r="G52" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H52" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I52" s="13"/>
+      <x:c r="J52" s="15"/>
+      <x:c r="K52" s="9" t="str">
+        <x:v>Process jaw</x:v>
+      </x:c>
+      <x:c r="L52" s="9" t="str">
+        <x:v>Cut and grind dense tissue</x:v>
+      </x:c>
+      <x:c r="M52" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N52" s="9" t="str">
+        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+      </x:c>
+      <x:c r="O52" s="22"/>
+      <x:c r="P52" s="22"/>
+      <x:c r="Q52" s="22"/>
+      <x:c r="R52" s="22"/>
+      <x:c r="S52" s="22"/>
+      <x:c r="T52" s="9" t="str">
+        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+      </x:c>
+      <x:c r="U52" s="23"/>
+      <x:c r="V52" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="66" customHeight="1">
+      <x:c r="A53" s="9" t="str">
+        <x:v>proposal.bio.seal</x:v>
+      </x:c>
+      <x:c r="B53" s="9" t="str">
+        <x:v>Membrane seal patches</x:v>
+      </x:c>
+      <x:c r="C53" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D53" s="9" t="str">
+        <x:v>Processed biological</x:v>
+      </x:c>
+      <x:c r="E53" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F53" s="9" t="str">
+        <x:v>Flexible equipment repairs</x:v>
+      </x:c>
+      <x:c r="G53" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H53" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I53" s="13"/>
+      <x:c r="J53" s="15"/>
+      <x:c r="K53" s="9" t="str">
+        <x:v>Process membrane</x:v>
+      </x:c>
+      <x:c r="L53" s="9" t="str">
+        <x:v>Dry preserve, cut and laminate</x:v>
+      </x:c>
+      <x:c r="M53" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N53" s="9" t="str">
+        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+      </x:c>
+      <x:c r="O53" s="22"/>
+      <x:c r="P53" s="22"/>
+      <x:c r="Q53" s="22"/>
+      <x:c r="R53" s="22"/>
+      <x:c r="S53" s="22"/>
+      <x:c r="T53" s="9" t="str">
+        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+      </x:c>
+      <x:c r="U53" s="23"/>
+      <x:c r="V53" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="66" customHeight="1">
+      <x:c r="A54" s="9" t="str">
+        <x:v>proposal.bio.wax</x:v>
+      </x:c>
+      <x:c r="B54" s="9" t="str">
+        <x:v>Solid biological wax</x:v>
+      </x:c>
+      <x:c r="C54" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D54" s="9" t="str">
+        <x:v>Processed biological</x:v>
+      </x:c>
+      <x:c r="E54" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F54" s="9" t="str">
+        <x:v>Sealing compounds and dry lubricant research</x:v>
+      </x:c>
+      <x:c r="G54" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H54" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I54" s="13"/>
+      <x:c r="J54" s="15"/>
+      <x:c r="K54" s="9" t="str">
+        <x:v>Process fat</x:v>
+      </x:c>
+      <x:c r="L54" s="9" t="str">
+        <x:v>Process tissue into a retained solid; no free-liquid commodity</x:v>
+      </x:c>
+      <x:c r="M54" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N54" s="9" t="str">
+        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+      </x:c>
+      <x:c r="O54" s="22"/>
+      <x:c r="P54" s="22"/>
+      <x:c r="Q54" s="22"/>
+      <x:c r="R54" s="22"/>
+      <x:c r="S54" s="22"/>
+      <x:c r="T54" s="9" t="str">
+        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+      </x:c>
+      <x:c r="U54" s="23"/>
+      <x:c r="V54" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="66" customHeight="1">
+      <x:c r="A55" s="9" t="str">
+        <x:v>proposal.bio.electrode</x:v>
+      </x:c>
+      <x:c r="B55" s="9" t="str">
+        <x:v>Dry organ electrode scaffold</x:v>
+      </x:c>
+      <x:c r="C55" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D55" s="9" t="str">
+        <x:v>Processed biological</x:v>
+      </x:c>
+      <x:c r="E55" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F55" s="9" t="str">
+        <x:v>Possible charged-battery component research</x:v>
+      </x:c>
+      <x:c r="G55" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H55" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I55" s="13"/>
+      <x:c r="J55" s="15"/>
+      <x:c r="K55" s="9" t="str">
+        <x:v>Process organ</x:v>
+      </x:c>
+      <x:c r="L55" s="9" t="str">
+        <x:v>Dry preserve and stabilize structure</x:v>
+      </x:c>
+      <x:c r="M55" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N55" s="9" t="str">
+        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+      </x:c>
+      <x:c r="O55" s="22"/>
+      <x:c r="P55" s="22"/>
+      <x:c r="Q55" s="22"/>
+      <x:c r="R55" s="22"/>
+      <x:c r="S55" s="22"/>
+      <x:c r="T55" s="9" t="str">
+        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+      </x:c>
+      <x:c r="U55" s="23"/>
+      <x:c r="V55" s="9" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E24:E55">
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="proposal"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C6:C23">
@@ -1698,7 +3437,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0db29f1724574820"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ad7a8aaab04472b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2606,7 +4345,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref4aec266be14a9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d923ef0b70741cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2972,7 +4711,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5116ad69fe2340a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d45700b8fd42c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3033,13 +4772,13 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>Six fitted gear types</x:v>
+        <x:v>Six existing fitted types plus two user-directed carried gear concepts</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>Weapons/armor variants require later design</x:v>
+        <x:v>Magnets/grounding kit have no assigned equipment slot</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
@@ -3054,7 +4793,7 @@
         <x:v>Pop-up camp and two battery states</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>Other food, medicine and ammunition not defined</x:v>
+        <x:v>Additional supplies await later design</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
@@ -3063,13 +4802,13 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>6</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Ore, airborne dust and four processed minerals</x:v>
+        <x:v>Existing mineral resources plus proposed natural and biological inputs</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Scrap, iron and biological resources occur as broad canon concepts</x:v>
+        <x:v>Proposals have no authored deposits, yields or runtime definitions</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -3078,13 +4817,13 @@
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A9)</x:f>
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
-        <x:v>Three trial salvage parts</x:v>
+        <x:v>Three trial salvage parts plus proposed biological products</x:v>
       </x:c>
       <x:c r="D9" s="4" t="str">
-        <x:v>Additional components and recipes await brainstorming</x:v>
+        <x:v>Recipes and properties remain proposals</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -3174,7 +4913,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re41eec55410a45a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R801906c34cb54139"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3237,7 +4976,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>One row per existing stable item ID. 18 items from 20 serialized definitions.</x:v>
+        <x:v>50 design entries: 18 existing item IDs plus 2 user-directed gear concepts and 30 new resource/material proposals.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -3301,7 +5040,7 @@
         <x:v>Algae</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str">
-        <x:v>Algae is living reserve state, not a loose-stack item. Eat, Drink and Treat do not restore sleep/Reserve.</x:v>
+        <x:v>Algae remains the survival backbone. Fauna products do not establish alternate food/hydration or free-liquid supplies.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="38" customHeight="1">
@@ -3376,10 +5115,799 @@
         <x:v>Active Assets/_Project and local game design/canon reviewed. Frozen engine/Unreal/historical Unity catalogs are excluded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="52" customHeight="1">
+      <x:c r="A26" s="3" t="str">
+        <x:v>Design scope</x:v>
+      </x:c>
+      <x:c r="B26" s="3" t="str">
+        <x:v>User direction is limited to carried magnets, grounding equipment and the insectoid/crustacean/mammal hybrid fauna direction. Specific forms, species and materials are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="52" customHeight="1">
+      <x:c r="A27" s="3" t="str">
+        <x:v>Proposal IDs</x:v>
+      </x:c>
+      <x:c r="B27" s="3" t="str">
+        <x:v>proposal.* keys exist only in this workbook. They are not Unity IDs and do not reserve new equipment slots.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="52" customHeight="1">
+      <x:c r="A28" s="3" t="str">
+        <x:v>Resource chains</x:v>
+      </x:c>
+      <x:c r="B28" s="3" t="str">
+        <x:v>Qualitative relationships only: no quantities, chemistry recipes or balance values are approved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="52" customHeight="1">
+      <x:c r="A29" s="3" t="str">
+        <x:v>Fauna ecology</x:v>
+      </x:c>
+      <x:c r="B29" s="3" t="str">
+        <x:v>No plant food chain assumed. Metabolism, primary energy and reproduction need a later ecology decision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="52" customHeight="1">
+      <x:c r="A30" s="3" t="str">
+        <x:v>Electrical design</x:v>
+      </x:c>
+      <x:c r="B30" s="3" t="str">
+        <x:v>Static discharge and electrical-storm danger need distinct game rules. Proposed gear does not imply real lightning protection.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9afc9614d67c43dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fe53715704a4c8a"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="38" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="70" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="65" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Proposed resource processing chains</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="1"/>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="35" customHeight="1">
+      <x:c r="A5" s="25" t="str">
+        <x:v>Input concept ID</x:v>
+      </x:c>
+      <x:c r="B5" s="25" t="str">
+        <x:v>Output concept ID</x:v>
+      </x:c>
+      <x:c r="C5" s="25" t="str">
+        <x:v>Processing concept</x:v>
+      </x:c>
+      <x:c r="D5" s="25" t="str">
+        <x:v>Potential use</x:v>
+      </x:c>
+      <x:c r="E5" s="25" t="str">
+        <x:v>Work location</x:v>
+      </x:c>
+      <x:c r="F5" s="25" t="str">
+        <x:v>Open constraint</x:v>
+      </x:c>
+      <x:c r="G5" s="25" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="H5" s="25" t="str">
+        <x:v>Basis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="85" customHeight="1">
+      <x:c r="A6" s="4" t="str">
+        <x:v>proposal.natural.magnetite</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>proposal.natural.iron_feed</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>Dry crush and magnetic separation</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>Intermediate feed for an eventual furnace</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>Stationary camp/settlement processing proposed</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>Distinct proposal from existing Iron-rich Concentrate; decide whether to merge them.</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="85" customHeight="1">
+      <x:c r="A7" s="4" t="str">
+        <x:v>proposal.natural.iron_feed</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>proposal.natural.iron_stock</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>Smelt, forge and finish at a stationary facility</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>Repair stock, fasteners and structural tool parts</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>Stationary camp/settlement processing proposed</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>Fuel, furnace, alloy and process choices unresolved; no Legger crafting platform.</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="85" customHeight="1">
+      <x:c r="A8" s="4" t="str">
+        <x:v>proposal.natural.silica</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>proposal.natural.abrasive</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>Dry sieve and grade</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>Tool sharpening and surface preparation</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>Stationary camp/settlement processing proposed</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>Could reuse existing Mineral Sand instead; resolve before implementation.</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="85" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>proposal.natural.alumina</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>proposal.natural.ceramic</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>Dry feed preparation, forming and firing</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Grounding-kit spacers and heat-resistant fixtures</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Stationary camp/settlement processing proposed</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>Claystone may be a co-input; forming binder/energy not settled.</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="85" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>proposal.natural.carbonate</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>proposal.natural.lime</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>Heat mineral feed; retain dry product</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Dry composite repair and construction</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>Stationary camp/settlement processing proposed</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>No conventional water-based cement recipe assumed.</x:v>
+      </x:c>
+      <x:c r="G10" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="85" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>proposal.natural.graphite</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>proposal.natural.carbon</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>Crush and dry grade</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>Dry lubricant; conductive composite ingredient</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>Stationary camp/settlement processing proposed</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>Not a power source; graphite behavior and recipe details remain provisional.</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="85" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>proposal.bio.shell</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>proposal.bio.laminate</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>Trim, layer and bind dry plates</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>Light armor panels and impact guards</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>Stationary preservation/workbench proposed</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="85" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>proposal.bio.tendon</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>proposal.bio.cord</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>Dry, split, twist and bind</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Tool lashings and field repairs</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>Stationary preservation/workbench proposed</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="85" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>proposal.bio.bristles</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>proposal.bio.brush</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>Sort fibers and bind into a backing</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>Dust exclusion at joints and equipment closures</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>Stationary preservation/workbench proposed</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="85" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>proposal.bio.underfur</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>proposal.bio.liner</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>Dry clean, card and compress</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Replaceable jacket/cloak liners</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>Stationary preservation/workbench proposed</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="85" customHeight="1">
+      <x:c r="A16" s="4" t="str">
+        <x:v>proposal.bio.jaw</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>proposal.bio.insert</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>Cut and grind dense tissue</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Replaceable excavation-tool wear part</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>Stationary preservation/workbench proposed</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+      </x:c>
+      <x:c r="G16" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="85" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>proposal.bio.membrane</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>proposal.bio.seal</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>Dry preserve, cut and laminate</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Flexible equipment repairs</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Stationary preservation/workbench proposed</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="85" customHeight="1">
+      <x:c r="A18" s="4" t="str">
+        <x:v>proposal.bio.fat</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>proposal.bio.wax</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>Process tissue into a retained solid; no free-liquid commodity</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>Sealing compounds and dry lubricant research</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>Stationary preservation/workbench proposed</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="85" customHeight="1">
+      <x:c r="A19" s="4" t="str">
+        <x:v>proposal.bio.organ</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>proposal.bio.electrode</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>Dry preserve and stabilize structure</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Possible charged-battery component research</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>Stationary preservation/workbench proposed</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="str">
+        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+      </x:c>
+      <x:c r="G19" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H19" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="85" customHeight="1">
+      <x:c r="A20" s="4" t="str">
+        <x:v>proposal.natural.mica</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>proposal.gear.grounding_kit</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>Trim insulating separator</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>Separates selected contact surfaces; not the discharge path</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>Field fitting proposed</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="str">
+        <x:v>Kit also needs an authored conductive path and game-valid ground contact</x:v>
+      </x:c>
+      <x:c r="G20" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H20" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="85" customHeight="1">
+      <x:c r="A21" s="4" t="str">
+        <x:v>proposal.natural.carbon</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>proposal.gear.grounding_kit</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>Potential conductive composite ingredient</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>Charge-control kit component research</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>Workbench proposed</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="str">
+        <x:v>Does not establish a complete working kit or physical safety claim</x:v>
+      </x:c>
+      <x:c r="G21" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H21" s="4" t="str">
+        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd506d206b9564fad"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="62" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="70" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="62" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="72" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Megafauna concepts and material sources</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+      <x:c r="I2" s="1"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="1"/>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+      <x:c r="I3" s="1"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="35" customHeight="1">
+      <x:c r="A5" s="25" t="str">
+        <x:v>Concept ID</x:v>
+      </x:c>
+      <x:c r="B5" s="25" t="str">
+        <x:v>Working description</x:v>
+      </x:c>
+      <x:c r="C5" s="25" t="str">
+        <x:v>Hybrid anatomy</x:v>
+      </x:c>
+      <x:c r="D5" s="25" t="str">
+        <x:v>Ecological role</x:v>
+      </x:c>
+      <x:c r="E5" s="25" t="str">
+        <x:v>Expedition decision</x:v>
+      </x:c>
+      <x:c r="F5" s="25" t="str">
+        <x:v>Resource concept IDs</x:v>
+      </x:c>
+      <x:c r="G5" s="25" t="str">
+        <x:v>Collection alternative</x:v>
+      </x:c>
+      <x:c r="H5" s="25" t="str">
+        <x:v>Open design issue</x:v>
+      </x:c>
+      <x:c r="I5" s="25" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="85" customHeight="1">
+      <x:c r="A6" s="4" t="str">
+        <x:v>fauna.plate_grazer</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>Plate-backed grazer</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>Broad low body; overlapping crustacean plates, six load-bearing legs, furred joint recesses</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>Slow herd browser of proposed dry microbial/mineral crusts</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>Quiet feedstock supply via abandoned molts; hunt only when worthwhile</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>proposal.bio.shell; proposal.bio.underfur; proposal.bio.tendon</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="str">
+        <x:v>Molts and bedding can supply modest materials without a kill</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="str">
+        <x:v>Primary productivity and crust biology unresolved; no plant grazing</x:v>
+      </x:c>
+      <x:c r="I6" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="85" customHeight="1">
+      <x:c r="A7" s="4" t="str">
+        <x:v>fauna.burrower</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>Canyon burrower</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>Wedge-shaped armored head, mole-like digging posture, shovel forelimbs, mandibular cutters</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>Excavates old scree fans; diet and nutrient sources unresolved</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>Excavation competes with access to mineral seams</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>proposal.bio.jaw; proposal.bio.bristles; proposal.bio.membrane</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="str">
+        <x:v>Old bristle-lined burrows provide low-yield scavenging opportunities</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="str">
+        <x:v>Burrows and collapse rules must respect fixed terrain; no terrain system authorized</x:v>
+      </x:c>
+      <x:c r="I7" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="85" customHeight="1">
+      <x:c r="A8" s="4" t="str">
+        <x:v>fauna.storm_migrant</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>Storm-following giant</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>Tall segmented body, shell ridges, furred underside, many broad feet</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>Fictional charge-sensitive migration near storms; diet unresolved</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>Storm timing creates a dangerous optional expedition target</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>proposal.bio.organ; proposal.bio.shell; proposal.bio.tendon</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="str">
+        <x:v>Abandoned molts available after migrations; rare tissue requires a carcass</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="str">
+        <x:v>Charge sensing/storage biology and electrical behavior are speculative</x:v>
+      </x:c>
+      <x:c r="I8" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="85" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>fauna.carrion_crusher</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>Carrion crusher</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>Heavy crab-like claws, mandibular mouth, muscular mammal-like trunk and gait</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Scavenges large carcasses; competes with Booter for remains</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Carcass harvesting attracts competition and encourages selective removal</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>proposal.bio.jaw; proposal.bio.shell; proposal.bio.fat</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="str">
+        <x:v>Track feeding sites for discarded dry fragments</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>Population depends on a viable food web; no established species or combat kit</x:v>
+      </x:c>
+      <x:c r="I9" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="85" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>fauna.shelf_climber</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>Shelf-climbing browser</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>Compact furred torso, hooked insectoid feet, flexible shell bands and springing limbs</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Uses narrow canyon ledges; diet unresolved</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>Source of flexible materials where bulk hauling is awkward</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>proposal.bio.membrane; proposal.bio.underfur; proposal.bio.tendon</x:v>
+      </x:c>
+      <x:c r="G10" s="4" t="str">
+        <x:v>Shed fur and abandoned rests provide a low-impact collection option</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="str">
+        <x:v>Movement, size, ecology and hunt behavior need design</x:v>
+      </x:c>
+      <x:c r="I10" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04deea109feb4ad6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expand mineral item register with Death Valley references
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="Rc9dd72c09de341c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R08d3808e22594dfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R5fb7f71d37554fed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Ra7bf41a8f1e64e12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R31bd2a341b8f47b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R02b1924a016d46c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rf405ec8950354877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R6bb67b5580a44387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rd9f55d6f849c4eac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rf058577461184423"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R068b950b0e1a4c5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rfdbb605f1e5f4943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R2de8e5c966974c95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rcca507fbe8ed42ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52,7 +52,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -94,6 +94,16 @@
         <x:fgColor rgb="FF423B35"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -107,7 +117,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -199,15 +209,31 @@
     <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="3">
     <x:dxf>
       <x:font>
         <x:color rgb="FF8A5B22"/>
       </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF87521B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF0D9"/>
+        </x:patternFill>
+      </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
@@ -241,7 +267,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V74" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -321,7 +347,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -331,7 +357,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ResourcechainsTable" displayName="ResourcechainsTable" ref="A5:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ResourcechainsTable" displayName="ResourcechainsTable" ref="A5:H27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Input concept ID"/>
     <x:tableColumn id="2" name="Output concept ID"/>
@@ -1640,7 +1666,7 @@
       <x:c r="R21" s="17"/>
       <x:c r="S21" s="17"/>
       <x:c r="T21" s="4" t="str">
-        <x:v>Production economy and final balance</x:v>
+        <x:v>Author wording: unprocessed iron-rich stones. Existing Ironstone Ore is the generic candidate; decide whether hematite/magnetite deserve separate resources.</x:v>
       </x:c>
       <x:c r="U21" s="11"/>
       <x:c r="V21" s="4" t="str">
@@ -3423,12 +3449,1003 @@
         <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
       </x:c>
     </x:row>
+    <x:row r="56" ht="75" customHeight="1">
+      <x:c r="A56" s="9" t="str">
+        <x:v>proposal.natural.charcoal</x:v>
+      </x:c>
+      <x:c r="B56" s="9" t="str">
+        <x:v>Charcoal</x:v>
+      </x:c>
+      <x:c r="C56" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D56" s="9" t="str">
+        <x:v>Processed fuel</x:v>
+      </x:c>
+      <x:c r="E56" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F56" s="9" t="str">
+        <x:v>Solid carbon fuel and possible metallurgical feedstock</x:v>
+      </x:c>
+      <x:c r="G56" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H56" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I56" s="13"/>
+      <x:c r="J56" s="15"/>
+      <x:c r="K56" s="9" t="str">
+        <x:v>Carbonize biological feedstock or recover old fuel; source undecided</x:v>
+      </x:c>
+      <x:c r="L56" s="9" t="str">
+        <x:v>Fuel and reduction research</x:v>
+      </x:c>
+      <x:c r="M56" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N56" s="9" t="str">
+        <x:v>Requested item; not a naturally mined metal. No wood/forest source introduced.</x:v>
+      </x:c>
+      <x:c r="O56" s="26"/>
+      <x:c r="P56" s="26"/>
+      <x:c r="Q56" s="26"/>
+      <x:c r="R56" s="26"/>
+      <x:c r="S56" s="26"/>
+      <x:c r="T56" s="9" t="str">
+        <x:v>Biological feedstock, scarcity and survival-versus-fuel tradeoff</x:v>
+      </x:c>
+      <x:c r="U56" s="27"/>
+      <x:c r="V56" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/historyculture/charcoalkilns.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="75" customHeight="1">
+      <x:c r="A57" s="9" t="str">
+        <x:v>proposal.natural.copper_stone</x:v>
+      </x:c>
+      <x:c r="B57" s="9" t="str">
+        <x:v>Unprocessed copper-rich stone</x:v>
+      </x:c>
+      <x:c r="C57" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D57" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E57" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F57" s="9" t="str">
+        <x:v>Bulk copper-bearing rock before sorting</x:v>
+      </x:c>
+      <x:c r="G57" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H57" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I57" s="13"/>
+      <x:c r="J57" s="15"/>
+      <x:c r="K57" s="9" t="str">
+        <x:v>Authored copper-bearing outcrop proposal</x:v>
+      </x:c>
+      <x:c r="L57" s="9" t="str">
+        <x:v>Sort into richer copper ore</x:v>
+      </x:c>
+      <x:c r="M57" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N57" s="9" t="str">
+        <x:v>Requested copper-rich feed represented separately from sorted ore provisionally.</x:v>
+      </x:c>
+      <x:c r="O57" s="26"/>
+      <x:c r="P57" s="26"/>
+      <x:c r="Q57" s="26"/>
+      <x:c r="R57" s="26"/>
+      <x:c r="S57" s="26"/>
+      <x:c r="T57" s="9" t="str">
+        <x:v>Merge with copper ore if the extra stage adds no useful choice</x:v>
+      </x:c>
+      <x:c r="U57" s="27"/>
+      <x:c r="V57" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="75" customHeight="1">
+      <x:c r="A58" s="9" t="str">
+        <x:v>proposal.natural.copper_ore</x:v>
+      </x:c>
+      <x:c r="B58" s="9" t="str">
+        <x:v>Copper ore</x:v>
+      </x:c>
+      <x:c r="C58" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D58" s="9" t="str">
+        <x:v>Sorted ore</x:v>
+      </x:c>
+      <x:c r="E58" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F58" s="9" t="str">
+        <x:v>Copper-bearing mineral feed for refining</x:v>
+      </x:c>
+      <x:c r="G58" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H58" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I58" s="13"/>
+      <x:c r="J58" s="15"/>
+      <x:c r="K58" s="9" t="str">
+        <x:v>Sort copper-rich stone; exact mineral species open</x:v>
+      </x:c>
+      <x:c r="L58" s="9" t="str">
+        <x:v>Refine into unworked copper</x:v>
+      </x:c>
+      <x:c r="M58" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N58" s="9" t="str">
+        <x:v>Ore is still mineral-bearing material, not metallic copper.</x:v>
+      </x:c>
+      <x:c r="O58" s="26"/>
+      <x:c r="P58" s="26"/>
+      <x:c r="Q58" s="26"/>
+      <x:c r="R58" s="26"/>
+      <x:c r="S58" s="26"/>
+      <x:c r="T58" s="9" t="str">
+        <x:v>Ore species, grade, impurities and refining method</x:v>
+      </x:c>
+      <x:c r="U58" s="27"/>
+      <x:c r="V58" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="75" customHeight="1">
+      <x:c r="A59" s="9" t="str">
+        <x:v>proposal.natural.raw_copper</x:v>
+      </x:c>
+      <x:c r="B59" s="9" t="str">
+        <x:v>Raw copper lump</x:v>
+      </x:c>
+      <x:c r="C59" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D59" s="9" t="str">
+        <x:v>Unworked metal</x:v>
+      </x:c>
+      <x:c r="E59" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F59" s="9" t="str">
+        <x:v>Unworked copper metal for conductors and small fittings</x:v>
+      </x:c>
+      <x:c r="G59" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H59" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I59" s="13"/>
+      <x:c r="J59" s="15"/>
+      <x:c r="K59" s="9" t="str">
+        <x:v>Refine ore or recover unworked metal from salvage</x:v>
+      </x:c>
+      <x:c r="L59" s="9" t="str">
+        <x:v>Potential wire, contacts and grounding-kit parts</x:v>
+      </x:c>
+      <x:c r="M59" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N59" s="9" t="str">
+        <x:v>Raw means unworked metal here; native copper occurrence is not established by the cited regional mining list.</x:v>
+      </x:c>
+      <x:c r="O59" s="26"/>
+      <x:c r="P59" s="26"/>
+      <x:c r="Q59" s="26"/>
+      <x:c r="R59" s="26"/>
+      <x:c r="S59" s="26"/>
+      <x:c r="T59" s="9" t="str">
+        <x:v>Decide whether native copper is also available; define manufacturing steps</x:v>
+      </x:c>
+      <x:c r="U59" s="27"/>
+      <x:c r="V59" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="75" customHeight="1">
+      <x:c r="A60" s="9" t="str">
+        <x:v>proposal.natural.tungsten_ore</x:v>
+      </x:c>
+      <x:c r="B60" s="9" t="str">
+        <x:v>Tungsten-bearing ore</x:v>
+      </x:c>
+      <x:c r="C60" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D60" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E60" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F60" s="9" t="str">
+        <x:v>Dense mineral feed for advanced wear-resistant material research</x:v>
+      </x:c>
+      <x:c r="G60" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H60" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I60" s="13"/>
+      <x:c r="J60" s="15"/>
+      <x:c r="K60" s="9" t="str">
+        <x:v>Authored mineral vein proposal</x:v>
+      </x:c>
+      <x:c r="L60" s="9" t="str">
+        <x:v>Advanced tool/alloy ingredient research</x:v>
+      </x:c>
+      <x:c r="M60" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N60" s="9" t="str">
+        <x:v>Tungsten ore is separate from copper ore; mineral choice unapproved. Scheelite/wolframite are general reference candidates.</x:v>
+      </x:c>
+      <x:c r="O60" s="26"/>
+      <x:c r="P60" s="26"/>
+      <x:c r="Q60" s="26"/>
+      <x:c r="R60" s="26"/>
+      <x:c r="S60" s="26"/>
+      <x:c r="T60" s="9" t="str">
+        <x:v>Deposit mineral, processing tier and worthwhile uses</x:v>
+      </x:c>
+      <x:c r="U60" s="27"/>
+      <x:c r="V60" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm; https://www.usgs.gov/data/tungsten-deposits-united-states</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="75" customHeight="1">
+      <x:c r="A61" s="9" t="str">
+        <x:v>proposal.natural.magnesium_rock</x:v>
+      </x:c>
+      <x:c r="B61" s="9" t="str">
+        <x:v>Magnesium-bearing rock</x:v>
+      </x:c>
+      <x:c r="C61" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D61" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E61" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F61" s="9" t="str">
+        <x:v>Mineral feed containing magnesium compounds</x:v>
+      </x:c>
+      <x:c r="G61" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H61" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I61" s="13"/>
+      <x:c r="J61" s="15"/>
+      <x:c r="K61" s="9" t="str">
+        <x:v>Magnesium-bearing mineral/salt deposit proposal</x:v>
+      </x:c>
+      <x:c r="L61" s="9" t="str">
+        <x:v>Refining research; possible refractory route</x:v>
+      </x:c>
+      <x:c r="M61" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N61" s="9" t="str">
+        <x:v>Death Valley Mg-bearing evaporites are documented; they do not establish loose native magnesium metal.</x:v>
+      </x:c>
+      <x:c r="O61" s="26"/>
+      <x:c r="P61" s="26"/>
+      <x:c r="Q61" s="26"/>
+      <x:c r="R61" s="26"/>
+      <x:c r="S61" s="26"/>
+      <x:c r="T61" s="9" t="str">
+        <x:v>Choose mineral, dry-world adaptation and refining route</x:v>
+      </x:c>
+      <x:c r="U61" s="27"/>
+      <x:c r="V61" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://pubs.usgs.gov/publication/70018701</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="75" customHeight="1">
+      <x:c r="A62" s="9" t="str">
+        <x:v>proposal.natural.raw_magnesium</x:v>
+      </x:c>
+      <x:c r="B62" s="9" t="str">
+        <x:v>Raw magnesium metal</x:v>
+      </x:c>
+      <x:c r="C62" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D62" s="9" t="str">
+        <x:v>Unworked metal</x:v>
+      </x:c>
+      <x:c r="E62" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F62" s="9" t="str">
+        <x:v>Unworked manufactured magnesium metal</x:v>
+      </x:c>
+      <x:c r="G62" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H62" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I62" s="13"/>
+      <x:c r="J62" s="15"/>
+      <x:c r="K62" s="9" t="str">
+        <x:v>Specialist refining or industrial salvage proposal</x:v>
+      </x:c>
+      <x:c r="L62" s="9" t="str">
+        <x:v>Lightweight alloy research</x:v>
+      </x:c>
+      <x:c r="M62" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N62" s="9" t="str">
+        <x:v>Not presented as a common native metal picked up from the ground.</x:v>
+      </x:c>
+      <x:c r="O62" s="26"/>
+      <x:c r="P62" s="26"/>
+      <x:c r="Q62" s="26"/>
+      <x:c r="R62" s="26"/>
+      <x:c r="S62" s="26"/>
+      <x:c r="T62" s="9" t="str">
+        <x:v>Processing burden, alloy uses and whether a separate item is useful</x:v>
+      </x:c>
+      <x:c r="U62" s="27"/>
+      <x:c r="V62" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://pubs.usgs.gov/publication/70018701</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="75" customHeight="1">
+      <x:c r="A63" s="9" t="str">
+        <x:v>proposal.natural.hematite</x:v>
+      </x:c>
+      <x:c r="B63" s="9" t="str">
+        <x:v>Raw hematite</x:v>
+      </x:c>
+      <x:c r="C63" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D63" s="9" t="str">
+        <x:v>Iron oxide mineral</x:v>
+      </x:c>
+      <x:c r="E63" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F63" s="9" t="str">
+        <x:v>Specific iron-rich mineral feed distinct from generic field stone</x:v>
+      </x:c>
+      <x:c r="G63" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H63" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I63" s="13"/>
+      <x:c r="J63" s="15"/>
+      <x:c r="K63" s="9" t="str">
+        <x:v>User-requested outcrop candidate</x:v>
+      </x:c>
+      <x:c r="L63" s="9" t="str">
+        <x:v>Possible iron-feed input</x:v>
+      </x:c>
+      <x:c r="M63" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N63" s="9" t="str">
+        <x:v>Requested game candidate; specific Death Valley occurrence not verified in this research pass.</x:v>
+      </x:c>
+      <x:c r="O63" s="26"/>
+      <x:c r="P63" s="26"/>
+      <x:c r="Q63" s="26"/>
+      <x:c r="R63" s="26"/>
+      <x:c r="S63" s="26"/>
+      <x:c r="T63" s="9" t="str">
+        <x:v>Overlap with Ironstone Ore and magnetite; retain only useful distinctions</x:v>
+      </x:c>
+      <x:c r="U63" s="27"/>
+      <x:c r="V63" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: User direction, October 14, 2026; specific local geology unverified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="75" customHeight="1">
+      <x:c r="A64" s="9" t="str">
+        <x:v>proposal.natural.sulfur</x:v>
+      </x:c>
+      <x:c r="B64" s="9" t="str">
+        <x:v>Raw sulfur</x:v>
+      </x:c>
+      <x:c r="C64" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D64" s="9" t="str">
+        <x:v>Native nonmetal</x:v>
+      </x:c>
+      <x:c r="E64" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F64" s="9" t="str">
+        <x:v>Nonmetallic mineral feed for specialist crafting research</x:v>
+      </x:c>
+      <x:c r="G64" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H64" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I64" s="13"/>
+      <x:c r="J64" s="15"/>
+      <x:c r="K64" s="9" t="str">
+        <x:v>Authored sulfur deposit proposal</x:v>
+      </x:c>
+      <x:c r="L64" s="9" t="str">
+        <x:v>Industrial reagent research; recipes open</x:v>
+      </x:c>
+      <x:c r="M64" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N64" s="9" t="str">
+        <x:v>Regional sulfur mining documented; no chemical or explosive recipe approved.</x:v>
+      </x:c>
+      <x:c r="O64" s="26"/>
+      <x:c r="P64" s="26"/>
+      <x:c r="Q64" s="26"/>
+      <x:c r="R64" s="26"/>
+      <x:c r="S64" s="26"/>
+      <x:c r="T64" s="9" t="str">
+        <x:v>Uses, gathering presentation and storage requirements</x:v>
+      </x:c>
+      <x:c r="U64" s="27"/>
+      <x:c r="V64" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="75" customHeight="1">
+      <x:c r="A65" s="9" t="str">
+        <x:v>proposal.natural.borate</x:v>
+      </x:c>
+      <x:c r="B65" s="9" t="str">
+        <x:v>Raw borate minerals</x:v>
+      </x:c>
+      <x:c r="C65" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D65" s="9" t="str">
+        <x:v>Evaporite mineral</x:v>
+      </x:c>
+      <x:c r="E65" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F65" s="9" t="str">
+        <x:v>Borate-rich feed for proposed glass/ceramic processing</x:v>
+      </x:c>
+      <x:c r="G65" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H65" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I65" s="13"/>
+      <x:c r="J65" s="15"/>
+      <x:c r="K65" s="9" t="str">
+        <x:v>Ancient dry mineral deposits</x:v>
+      </x:c>
+      <x:c r="L65" s="9" t="str">
+        <x:v>Flux and glass/ceramic research</x:v>
+      </x:c>
+      <x:c r="M65" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N65" s="9" t="str">
+        <x:v>Borate minerals are not elemental boron. No current water cycle is required for ancient deposits.</x:v>
+      </x:c>
+      <x:c r="O65" s="26"/>
+      <x:c r="P65" s="26"/>
+      <x:c r="Q65" s="26"/>
+      <x:c r="R65" s="26"/>
+      <x:c r="S65" s="26"/>
+      <x:c r="T65" s="9" t="str">
+        <x:v>Select borax/colemanite/ulexite versus one simplified item</x:v>
+      </x:c>
+      <x:c r="U65" s="27"/>
+      <x:c r="V65" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="75" customHeight="1">
+      <x:c r="A66" s="9" t="str">
+        <x:v>proposal.natural.gypsum</x:v>
+      </x:c>
+      <x:c r="B66" s="9" t="str">
+        <x:v>Raw gypsum</x:v>
+      </x:c>
+      <x:c r="C66" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D66" s="9" t="str">
+        <x:v>Sulfate mineral</x:v>
+      </x:c>
+      <x:c r="E66" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F66" s="9" t="str">
+        <x:v>Soft mineral feed for molds and mineral products</x:v>
+      </x:c>
+      <x:c r="G66" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H66" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I66" s="13"/>
+      <x:c r="J66" s="15"/>
+      <x:c r="K66" s="9" t="str">
+        <x:v>Ancient evaporite beds</x:v>
+      </x:c>
+      <x:c r="L66" s="9" t="str">
+        <x:v>Mold/binder research</x:v>
+      </x:c>
+      <x:c r="M66" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N66" s="9" t="str">
+        <x:v>Water bound in a mineral is not a free-liquid supply; no hydration mechanic proposed.</x:v>
+      </x:c>
+      <x:c r="O66" s="26"/>
+      <x:c r="P66" s="26"/>
+      <x:c r="Q66" s="26"/>
+      <x:c r="R66" s="26"/>
+      <x:c r="S66" s="26"/>
+      <x:c r="T66" s="9" t="str">
+        <x:v>Dry-world processing and overlap with existing binders</x:v>
+      </x:c>
+      <x:c r="U66" s="27"/>
+      <x:c r="V66" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://pubs.usgs.gov/publication/70018701</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="75" customHeight="1">
+      <x:c r="A67" s="9" t="str">
+        <x:v>proposal.natural.talc</x:v>
+      </x:c>
+      <x:c r="B67" s="9" t="str">
+        <x:v>Raw talc</x:v>
+      </x:c>
+      <x:c r="C67" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D67" s="9" t="str">
+        <x:v>Industrial mineral</x:v>
+      </x:c>
+      <x:c r="E67" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F67" s="9" t="str">
+        <x:v>Soft mineral feed for proposed dry powders and ceramics</x:v>
+      </x:c>
+      <x:c r="G67" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H67" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I67" s="13"/>
+      <x:c r="J67" s="15"/>
+      <x:c r="K67" s="9" t="str">
+        <x:v>Authored mineral seam proposal</x:v>
+      </x:c>
+      <x:c r="L67" s="9" t="str">
+        <x:v>Dry lubricant/filler research</x:v>
+      </x:c>
+      <x:c r="M67" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N67" s="9" t="str">
+        <x:v>Regional talc mining is reference evidence, not an implemented deposit.</x:v>
+      </x:c>
+      <x:c r="O67" s="26"/>
+      <x:c r="P67" s="26"/>
+      <x:c r="Q67" s="26"/>
+      <x:c r="R67" s="26"/>
+      <x:c r="S67" s="26"/>
+      <x:c r="T67" s="9" t="str">
+        <x:v>Useful difference from graphite and existing dust materials</x:v>
+      </x:c>
+      <x:c r="U67" s="27"/>
+      <x:c r="V67" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="75" customHeight="1">
+      <x:c r="A68" s="9" t="str">
+        <x:v>proposal.natural.manganese_ore</x:v>
+      </x:c>
+      <x:c r="B68" s="9" t="str">
+        <x:v>Manganese-bearing ore</x:v>
+      </x:c>
+      <x:c r="C68" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D68" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E68" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F68" s="9" t="str">
+        <x:v>Mineral feed for alloy and pigment research</x:v>
+      </x:c>
+      <x:c r="G68" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H68" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I68" s="13"/>
+      <x:c r="J68" s="15"/>
+      <x:c r="K68" s="9" t="str">
+        <x:v>Authored mineral deposit proposal</x:v>
+      </x:c>
+      <x:c r="L68" s="9" t="str">
+        <x:v>Advanced metallurgy research</x:v>
+      </x:c>
+      <x:c r="M68" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N68" s="9" t="str">
+        <x:v>Regional commodity listed by NPS; exact ore mineral remains unselected.</x:v>
+      </x:c>
+      <x:c r="O68" s="26"/>
+      <x:c r="P68" s="26"/>
+      <x:c r="Q68" s="26"/>
+      <x:c r="R68" s="26"/>
+      <x:c r="S68" s="26"/>
+      <x:c r="T68" s="9" t="str">
+        <x:v>Mineral species, steelmaking role and processing tier</x:v>
+      </x:c>
+      <x:c r="U68" s="27"/>
+      <x:c r="V68" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://home.nps.gov/deva/faqs.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="75" customHeight="1">
+      <x:c r="A69" s="9" t="str">
+        <x:v>proposal.natural.lead_ore</x:v>
+      </x:c>
+      <x:c r="B69" s="9" t="str">
+        <x:v>Lead-bearing ore</x:v>
+      </x:c>
+      <x:c r="C69" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D69" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E69" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F69" s="9" t="str">
+        <x:v>Heavy mineral feed for specialized industrial material</x:v>
+      </x:c>
+      <x:c r="G69" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H69" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I69" s="13"/>
+      <x:c r="J69" s="15"/>
+      <x:c r="K69" s="9" t="str">
+        <x:v>Authored mineral deposit proposal</x:v>
+      </x:c>
+      <x:c r="L69" s="9" t="str">
+        <x:v>Specialist refining and dense-component research</x:v>
+      </x:c>
+      <x:c r="M69" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N69" s="9" t="str">
+        <x:v>Regional lead mining documented; item does not establish easy field refining.</x:v>
+      </x:c>
+      <x:c r="O69" s="26"/>
+      <x:c r="P69" s="26"/>
+      <x:c r="Q69" s="26"/>
+      <x:c r="R69" s="26"/>
+      <x:c r="S69" s="26"/>
+      <x:c r="T69" s="9" t="str">
+        <x:v>Whether its mass and uses create a worthwhile haul</x:v>
+      </x:c>
+      <x:c r="U69" s="27"/>
+      <x:c r="V69" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="75" customHeight="1">
+      <x:c r="A70" s="9" t="str">
+        <x:v>proposal.natural.zinc_ore</x:v>
+      </x:c>
+      <x:c r="B70" s="9" t="str">
+        <x:v>Zinc-bearing ore</x:v>
+      </x:c>
+      <x:c r="C70" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D70" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E70" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F70" s="9" t="str">
+        <x:v>Mineral feed for alloy and protective-coating research</x:v>
+      </x:c>
+      <x:c r="G70" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H70" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I70" s="13"/>
+      <x:c r="J70" s="15"/>
+      <x:c r="K70" s="9" t="str">
+        <x:v>Authored mineral deposit proposal</x:v>
+      </x:c>
+      <x:c r="L70" s="9" t="str">
+        <x:v>Brass/coating research with copper</x:v>
+      </x:c>
+      <x:c r="M70" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N70" s="9" t="str">
+        <x:v>Regional zinc commodity documented; no alloy recipe approved.</x:v>
+      </x:c>
+      <x:c r="O70" s="26"/>
+      <x:c r="P70" s="26"/>
+      <x:c r="Q70" s="26"/>
+      <x:c r="R70" s="26"/>
+      <x:c r="S70" s="26"/>
+      <x:c r="T70" s="9" t="str">
+        <x:v>Mineral, processing and final equipment uses</x:v>
+      </x:c>
+      <x:c r="U70" s="27"/>
+      <x:c r="V70" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="75" customHeight="1">
+      <x:c r="A71" s="9" t="str">
+        <x:v>proposal.natural.silver_ore</x:v>
+      </x:c>
+      <x:c r="B71" s="9" t="str">
+        <x:v>Silver-bearing ore</x:v>
+      </x:c>
+      <x:c r="C71" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D71" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E71" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F71" s="9" t="str">
+        <x:v>Mineral feed for trade and specialist contact research</x:v>
+      </x:c>
+      <x:c r="G71" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H71" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I71" s="13"/>
+      <x:c r="J71" s="15"/>
+      <x:c r="K71" s="9" t="str">
+        <x:v>Authored high-grade seam proposal</x:v>
+      </x:c>
+      <x:c r="L71" s="9" t="str">
+        <x:v>Refining and trade research</x:v>
+      </x:c>
+      <x:c r="M71" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N71" s="9" t="str">
+        <x:v>Regional silver mining documented; value is undecided.</x:v>
+      </x:c>
+      <x:c r="O71" s="26"/>
+      <x:c r="P71" s="26"/>
+      <x:c r="Q71" s="26"/>
+      <x:c r="R71" s="26"/>
+      <x:c r="S71" s="26"/>
+      <x:c r="T71" s="9" t="str">
+        <x:v>Use beyond trade and relation to copper conductors</x:v>
+      </x:c>
+      <x:c r="U71" s="27"/>
+      <x:c r="V71" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="75" customHeight="1">
+      <x:c r="A72" s="9" t="str">
+        <x:v>proposal.natural.gold_rock</x:v>
+      </x:c>
+      <x:c r="B72" s="9" t="str">
+        <x:v>Gold-bearing rock</x:v>
+      </x:c>
+      <x:c r="C72" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D72" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E72" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F72" s="9" t="str">
+        <x:v>Scarce mineral feed for trade and specialist components</x:v>
+      </x:c>
+      <x:c r="G72" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H72" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I72" s="13"/>
+      <x:c r="J72" s="15"/>
+      <x:c r="K72" s="9" t="str">
+        <x:v>Authored mineral deposit proposal</x:v>
+      </x:c>
+      <x:c r="L72" s="9" t="str">
+        <x:v>Separation/refining and trade research</x:v>
+      </x:c>
+      <x:c r="M72" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N72" s="9" t="str">
+        <x:v>Regional gold mining documented; no currency or rarity value set.</x:v>
+      </x:c>
+      <x:c r="O72" s="26"/>
+      <x:c r="P72" s="26"/>
+      <x:c r="Q72" s="26"/>
+      <x:c r="R72" s="26"/>
+      <x:c r="S72" s="26"/>
+      <x:c r="T72" s="9" t="str">
+        <x:v>Whether gold has a meaningful survival-economy role</x:v>
+      </x:c>
+      <x:c r="U72" s="27"/>
+      <x:c r="V72" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="75" customHeight="1">
+      <x:c r="A73" s="9" t="str">
+        <x:v>proposal.natural.fluorite</x:v>
+      </x:c>
+      <x:c r="B73" s="9" t="str">
+        <x:v>Raw fluorite</x:v>
+      </x:c>
+      <x:c r="C73" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D73" s="9" t="str">
+        <x:v>Industrial mineral</x:v>
+      </x:c>
+      <x:c r="E73" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F73" s="9" t="str">
+        <x:v>Mineral feed for specialist ceramic/metallurgical research</x:v>
+      </x:c>
+      <x:c r="G73" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H73" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I73" s="13"/>
+      <x:c r="J73" s="15"/>
+      <x:c r="K73" s="9" t="str">
+        <x:v>Authored mineral deposit proposal</x:v>
+      </x:c>
+      <x:c r="L73" s="9" t="str">
+        <x:v>Flux/optical-material research</x:v>
+      </x:c>
+      <x:c r="M73" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N73" s="9" t="str">
+        <x:v>NPS lists fluorspar; proposed manufacturing uses need their own design.</x:v>
+      </x:c>
+      <x:c r="O73" s="26"/>
+      <x:c r="P73" s="26"/>
+      <x:c r="Q73" s="26"/>
+      <x:c r="R73" s="26"/>
+      <x:c r="S73" s="26"/>
+      <x:c r="T73" s="9" t="str">
+        <x:v>Distinct use, processing and game naming</x:v>
+      </x:c>
+      <x:c r="U73" s="27"/>
+      <x:c r="V73" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://home.nps.gov/deva/faqs.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="75" customHeight="1">
+      <x:c r="A74" s="9" t="str">
+        <x:v>proposal.natural.antimony_ore</x:v>
+      </x:c>
+      <x:c r="B74" s="9" t="str">
+        <x:v>Antimony-bearing ore</x:v>
+      </x:c>
+      <x:c r="C74" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D74" s="9" t="str">
+        <x:v>Raw mineral</x:v>
+      </x:c>
+      <x:c r="E74" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F74" s="9" t="str">
+        <x:v>Mineral feed for specialist alloy research</x:v>
+      </x:c>
+      <x:c r="G74" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H74" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I74" s="13"/>
+      <x:c r="J74" s="15"/>
+      <x:c r="K74" s="9" t="str">
+        <x:v>Authored mineral deposit proposal</x:v>
+      </x:c>
+      <x:c r="L74" s="9" t="str">
+        <x:v>Advanced alloy research</x:v>
+      </x:c>
+      <x:c r="M74" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N74" s="9" t="str">
+        <x:v>Regional antimony commodity documented; no final ore species or recipe selected.</x:v>
+      </x:c>
+      <x:c r="O74" s="26"/>
+      <x:c r="P74" s="26"/>
+      <x:c r="Q74" s="26"/>
+      <x:c r="R74" s="26"/>
+      <x:c r="S74" s="26"/>
+      <x:c r="T74" s="9" t="str">
+        <x:v>Keep only if advanced crafting needs this separate material</x:v>
+      </x:c>
+      <x:c r="U74" s="27"/>
+      <x:c r="V74" s="9" t="str">
+        <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="E24:E55">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="proposal"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E56:E74">
+    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="proposal"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C6:C23">
@@ -3437,7 +4454,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ad7a8aaab04472b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R117d4bb2fbc84a92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4345,7 +5362,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d923ef0b70741cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4ba61aaeecf4417"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4711,7 +5728,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d45700b8fd42c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2088468a270246d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4802,13 +5819,13 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>28</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Existing mineral resources plus proposed natural and biological inputs</x:v>
+        <x:v>Existing resources plus natural minerals, unworked metals, charcoal and biological proposals</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Proposals have no authored deposits, yields or runtime definitions</x:v>
+        <x:v>Regional evidence supports candidate selection; availability and processing stay open</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -4913,7 +5930,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R801906c34cb54139"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1c2f2589b54738"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4976,7 +5993,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>50 design entries: 18 existing item IDs plus 2 user-directed gear concepts and 30 new resource/material proposals.</x:v>
+        <x:v>69 design entries: 18 existing item IDs, 11 user-directed concepts, and 40 proposed resources/materials. Implementation remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -5120,7 +6137,7 @@
         <x:v>Design scope</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
-        <x:v>User direction is limited to carried magnets, grounding equipment and the insectoid/crustacean/mammal hybrid fauna direction. Specific forms, species and materials are proposals.</x:v>
+        <x:v>User direction includes carried magnets/grounding gear, hybrid fauna, and requested charcoal, copper, tungsten, magnesium, hematite and sulfur materials. Specific species, geology and processing remain proposals.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="52" customHeight="1">
@@ -5155,10 +6172,50 @@
         <x:v>Static discharge and electrical-storm danger need distinct game rules. Proposed gear does not imply real lightning protection.</x:v>
       </x:c>
     </x:row>
+    <x:row r="31" ht="58" customHeight="1">
+      <x:c r="A31" s="4" t="str">
+        <x:v>Mineral naming</x:v>
+      </x:c>
+      <x:c r="B31" s="4" t="str">
+        <x:v>Copper-rich stone, sorted copper ore and unworked copper are provisional stages. Copper and tungsten were interpreted as separate requested resources.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="58" customHeight="1">
+      <x:c r="A32" s="4" t="str">
+        <x:v>Raw magnesium</x:v>
+      </x:c>
+      <x:c r="B32" s="4" t="str">
+        <x:v>Magnesium-bearing rock is separate from unworked manufactured magnesium metal; native metal deposits are not assumed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="58" customHeight="1">
+      <x:c r="A33" s="4" t="str">
+        <x:v>Charcoal source</x:v>
+      </x:c>
+      <x:c r="B33" s="4" t="str">
+        <x:v>Charcoal is a processed carbon material. Biological offcuts or recovered fuel are options; no wood or living plants added to the world.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="58" customHeight="1">
+      <x:c r="A34" s="4" t="str">
+        <x:v>Regional evidence</x:v>
+      </x:c>
+      <x:c r="B34" s="4" t="str">
+        <x:v>NPS/USGS URLs support reference geology/history only. Game deposits, locations, yields and uses remain unimplemented; hematite locality was not verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="58" customHeight="1">
+      <x:c r="A35" s="4" t="str">
+        <x:v>Generic iron alias</x:v>
+      </x:c>
+      <x:c r="B35" s="4" t="str">
+        <x:v>Unprocessed iron-rich stones maps to the existing Ironstone Ore candidate. Specific hematite/magnetite distinctions remain open rather than creating another duplicate generic item.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fe53715704a4c8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a253a4df8d14f7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5661,10 +6718,166 @@
         <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="85" customHeight="1">
+      <x:c r="A22" s="4" t="str">
+        <x:v>proposal.natural.copper_stone</x:v>
+      </x:c>
+      <x:c r="B22" s="4" t="str">
+        <x:v>proposal.natural.copper_ore</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="str">
+        <x:v>Dry sort / concentrate; method to design</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>Higher-grade copper feed</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="str">
+        <x:v>Stationary processing proposed</x:v>
+      </x:c>
+      <x:c r="F22" s="4" t="str">
+        <x:v>Optional extra stage; merge these entries if sorting is busywork</x:v>
+      </x:c>
+      <x:c r="G22" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H22" s="4" t="str">
+        <x:v>https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="85" customHeight="1">
+      <x:c r="A23" s="4" t="str">
+        <x:v>proposal.natural.copper_ore</x:v>
+      </x:c>
+      <x:c r="B23" s="4" t="str">
+        <x:v>proposal.natural.raw_copper</x:v>
+      </x:c>
+      <x:c r="C23" s="4" t="str">
+        <x:v>Refine; process and energy unresolved</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="str">
+        <x:v>Unworked copper for manufacturing</x:v>
+      </x:c>
+      <x:c r="E23" s="4" t="str">
+        <x:v>Stationary specialist facility proposed</x:v>
+      </x:c>
+      <x:c r="F23" s="4" t="str">
+        <x:v>No direct conversion rate or field-smelting recipe approved</x:v>
+      </x:c>
+      <x:c r="G23" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H23" s="4" t="str">
+        <x:v>https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="85" customHeight="1">
+      <x:c r="A24" s="4" t="str">
+        <x:v>proposal.natural.magnesium_rock</x:v>
+      </x:c>
+      <x:c r="B24" s="4" t="str">
+        <x:v>proposal.natural.raw_magnesium</x:v>
+      </x:c>
+      <x:c r="C24" s="4" t="str">
+        <x:v>Specialist extraction; method unresolved</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:v>Unworked metal for alloy research</x:v>
+      </x:c>
+      <x:c r="E24" s="4" t="str">
+        <x:v>Settlement-scale facility or salvage proposed</x:v>
+      </x:c>
+      <x:c r="F24" s="4" t="str">
+        <x:v>Mineral occurrence does not establish native magnesium metal</x:v>
+      </x:c>
+      <x:c r="G24" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H24" s="4" t="str">
+        <x:v>https://pubs.usgs.gov/publication/70018701</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="85" customHeight="1">
+      <x:c r="A25" s="4" t="str">
+        <x:v>proposal.natural.hematite</x:v>
+      </x:c>
+      <x:c r="B25" s="4" t="str">
+        <x:v>proposal.natural.iron_feed</x:v>
+      </x:c>
+      <x:c r="C25" s="4" t="str">
+        <x:v>Sort and prepare iron-bearing feed</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>Common iron-refining intermediate candidate</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="str">
+        <x:v>Stationary processing proposed</x:v>
+      </x:c>
+      <x:c r="F25" s="4" t="str">
+        <x:v>Hematite game entry user-requested; local occurrence not verified here</x:v>
+      </x:c>
+      <x:c r="G25" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H25" s="4" t="str">
+        <x:v>User direction, October 14, 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="85" customHeight="1">
+      <x:c r="A26" s="4" t="str">
+        <x:v>proposal.bio.tendon</x:v>
+      </x:c>
+      <x:c r="B26" s="4" t="str">
+        <x:v>proposal.natural.charcoal</x:v>
+      </x:c>
+      <x:c r="C26" s="4" t="str">
+        <x:v>Possible carbonization of dried biological offcuts</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:v>Fuel from non-wood biological material</x:v>
+      </x:c>
+      <x:c r="E26" s="4" t="str">
+        <x:v>Stationary retort proposed</x:v>
+      </x:c>
+      <x:c r="F26" s="4" t="str">
+        <x:v>Illustrative pathway only; consumes valuable biomass; source/yield and ecology unapproved</x:v>
+      </x:c>
+      <x:c r="G26" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H26" s="4" t="str">
+        <x:v>https://www.nps.gov/deva/learn/historyculture/charcoalkilns.htm; game feedstock is a new proposal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="85" customHeight="1">
+      <x:c r="A27" s="4" t="str">
+        <x:v>proposal.natural.raw_copper</x:v>
+      </x:c>
+      <x:c r="B27" s="4" t="str">
+        <x:v>proposal.gear.grounding_kit</x:v>
+      </x:c>
+      <x:c r="C27" s="4" t="str">
+        <x:v>Manufacture conductive parts; kit design unresolved</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="str">
+        <x:v>Charge-management gear</x:v>
+      </x:c>
+      <x:c r="E27" s="4" t="str">
+        <x:v>Workbench proposed</x:v>
+      </x:c>
+      <x:c r="F27" s="4" t="str">
+        <x:v>Material link only; not a complete electrical design</x:v>
+      </x:c>
+      <x:c r="G27" s="4" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="H27" s="4" t="str">
+        <x:v>User direction; proposed crafting relationship</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd506d206b9564fad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc28d6f4ba88f4222"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5907,7 +7120,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04deea109feb4ad6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R211a51648a82418b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record husk fiber paper and no-cloth material rules
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R6bb67b5580a44387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rd9f55d6f849c4eac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rf058577461184423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R068b950b0e1a4c5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rfdbb605f1e5f4943"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R2de8e5c966974c95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rcca507fbe8ed42ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R7c7839909cc94067"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R75ab1c9bb144465f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R4a034556bca247d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R3570054a1ff645e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R3e127f52146b4c44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R5b65cf6fa26e419d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R070361ad3a944f6f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52,7 +52,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -104,6 +104,16 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -117,7 +127,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,6 +225,12 @@
     <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -240,7 +256,7 @@
         <x:color rgb="FF87521B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D9"/>
         </x:patternFill>
       </x:fill>
@@ -267,7 +283,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V74" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -347,7 +363,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -357,7 +373,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ResourcechainsTable" displayName="ResourcechainsTable" ref="A5:H27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ResourcechainsTable" displayName="ResourcechainsTable" ref="A5:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Input concept ID"/>
     <x:tableColumn id="2" name="Output concept ID"/>
@@ -1050,7 +1066,7 @@
       <x:c r="R10" s="17"/>
       <x:c r="S10" s="17"/>
       <x:c r="T10" s="9" t="str">
-        <x:v>Protection and material progression</x:v>
+        <x:v>Protection and material progression; material composition unresolved under no-cloth rule</x:v>
       </x:c>
       <x:c r="U10" s="11"/>
       <x:c r="V10" s="9" t="str">
@@ -1274,7 +1290,7 @@
       <x:c r="R14" s="17"/>
       <x:c r="S14" s="17"/>
       <x:c r="T14" s="9" t="str">
-        <x:v>Protection, exposure rules and progression</x:v>
+        <x:v>Protection, exposure rules and progression; material composition unresolved under no-cloth rule</x:v>
       </x:c>
       <x:c r="U14" s="11"/>
       <x:c r="V14" s="9" t="str">
@@ -2622,7 +2638,7 @@
         <x:v>proposal.bio.shell</x:v>
       </x:c>
       <x:c r="B40" s="9" t="str">
-        <x:v>Shed shell plates</x:v>
+        <x:v>Shell husks / shed plates</x:v>
       </x:c>
       <x:c r="C40" s="9" t="str">
         <x:v>Resources</x:v>
@@ -2634,7 +2650,7 @@
         <x:v>New proposal</x:v>
       </x:c>
       <x:c r="F40" s="9" t="str">
-        <x:v>Layered armor, shields and tool guards</x:v>
+        <x:v>Source of abundant scraped chitin and icore fibers; possible structural plate uses.</x:v>
       </x:c>
       <x:c r="G40" s="9" t="str">
         <x:v>None</x:v>
@@ -2645,16 +2661,16 @@
       <x:c r="I40" s="13"/>
       <x:c r="J40" s="15"/>
       <x:c r="K40" s="9" t="str">
-        <x:v>Molts and carcasses of plate-backed fauna</x:v>
+        <x:v>Discarded shell husks; creature-specific collection remains proposed</x:v>
       </x:c>
       <x:c r="L40" s="9" t="str">
-        <x:v>See Resource chains</x:v>
+        <x:v>Scrape fibers for paper and difficult pressed textile processing</x:v>
       </x:c>
       <x:c r="M40" s="9" t="str">
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N40" s="9" t="str">
-        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+        <x:v>Raw fiber abundance does not imply easy finished textile production; no cloth.</x:v>
       </x:c>
       <x:c r="O40" s="22"/>
       <x:c r="P40" s="22"/>
@@ -2662,11 +2678,11 @@
       <x:c r="R40" s="22"/>
       <x:c r="S40" s="22"/>
       <x:c r="T40" s="9" t="str">
-        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+        <x:v>Species-specific shell properties and structural uses remain proposals</x:v>
       </x:c>
       <x:c r="U40" s="23"/>
       <x:c r="V40" s="9" t="str">
-        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="66" customHeight="1">
@@ -2790,7 +2806,7 @@
         <x:v>New proposal</x:v>
       </x:c>
       <x:c r="F43" s="9" t="str">
-        <x:v>Clothing liners and dust buffers</x:v>
+        <x:v>Raw fur for extremely low-yield material processing.</x:v>
       </x:c>
       <x:c r="G43" s="9" t="str">
         <x:v>None</x:v>
@@ -2804,13 +2820,13 @@
         <x:v>Abandoned resting hollows and natural shedding</x:v>
       </x:c>
       <x:c r="L43" s="9" t="str">
-        <x:v>See Resource chains</x:v>
+        <x:v>Extremely low usable yield for textile/material processing</x:v>
       </x:c>
       <x:c r="M43" s="9" t="str">
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N43" s="9" t="str">
-        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+        <x:v>No cloth. Raw collection amount does not establish processed yield.</x:v>
       </x:c>
       <x:c r="O43" s="22"/>
       <x:c r="P43" s="22"/>
@@ -2818,11 +2834,11 @@
       <x:c r="R43" s="22"/>
       <x:c r="S43" s="22"/>
       <x:c r="T43" s="9" t="str">
-        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+        <x:v>Specific fur types and outputs remain proposals; no numeric yield</x:v>
       </x:c>
       <x:c r="U43" s="23"/>
       <x:c r="V43" s="9" t="str">
-        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="66" customHeight="1">
@@ -2914,7 +2930,7 @@
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N45" s="9" t="str">
-        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+        <x:v>Flexible tissue proposal; does not establish cloth. Processing and preservation remain open.</x:v>
       </x:c>
       <x:c r="O45" s="22"/>
       <x:c r="P45" s="22"/>
@@ -3194,7 +3210,7 @@
         <x:v>proposal.bio.liner</x:v>
       </x:c>
       <x:c r="B51" s="9" t="str">
-        <x:v>Felted underfur liner</x:v>
+        <x:v>Pressed fur-fiber material</x:v>
       </x:c>
       <x:c r="C51" s="9" t="str">
         <x:v>Crafting components</x:v>
@@ -3206,7 +3222,7 @@
         <x:v>New proposal</x:v>
       </x:c>
       <x:c r="F51" s="9" t="str">
-        <x:v>Replaceable jacket/cloak liners</x:v>
+        <x:v>Candidate scarce pressed material; former liner proposal requires reassessment.</x:v>
       </x:c>
       <x:c r="G51" s="9" t="str">
         <x:v>None</x:v>
@@ -3220,13 +3236,13 @@
         <x:v>Process underfur</x:v>
       </x:c>
       <x:c r="L51" s="9" t="str">
-        <x:v>Dry clean, card and compress</x:v>
+        <x:v>Very low-yield fur processing; pressing/finish details unapproved</x:v>
       </x:c>
       <x:c r="M51" s="9" t="str">
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N51" s="9" t="str">
-        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+        <x:v>Extremely low usable yield. No cloth or routine clothing-liner supply implied.</x:v>
       </x:c>
       <x:c r="O51" s="22"/>
       <x:c r="P51" s="22"/>
@@ -3234,11 +3250,11 @@
       <x:c r="R51" s="22"/>
       <x:c r="S51" s="22"/>
       <x:c r="T51" s="9" t="str">
-        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+        <x:v>Product form and garment use remain proposals; old felted-liner assumption superseded</x:v>
       </x:c>
       <x:c r="U51" s="23"/>
       <x:c r="V51" s="9" t="str">
-        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="66" customHeight="1">
@@ -4435,6 +4451,318 @@
       <x:c r="U74" s="27"/>
       <x:c r="V74" s="9" t="str">
         <x:v>User brainstorming, October 14, 2026; game uses proposed. Reference: https://www.nps.gov/deva/learn/nature/mining-in-death-valley.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="75" customHeight="1">
+      <x:c r="A75" s="9" t="str">
+        <x:v>proposal.bio.chitin_fibers</x:v>
+      </x:c>
+      <x:c r="B75" s="9" t="str">
+        <x:v>Scraped chitin fibers</x:v>
+      </x:c>
+      <x:c r="C75" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D75" s="9" t="str">
+        <x:v>Raw husk fiber</x:v>
+      </x:c>
+      <x:c r="E75" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F75" s="9" t="str">
+        <x:v>Abundant husk fiber feed for paper and difficult pressed textiles.</x:v>
+      </x:c>
+      <x:c r="G75" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H75" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I75" s="13"/>
+      <x:c r="J75" s="15"/>
+      <x:c r="K75" s="9" t="str">
+        <x:v>Scrape shell husks</x:v>
+      </x:c>
+      <x:c r="L75" s="9" t="str">
+        <x:v>Main paper feedstock; textile conversion very difficult</x:v>
+      </x:c>
+      <x:c r="M75" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N75" s="9" t="str">
+        <x:v>Abundance applies to raw fibers; no numeric output yield approved.</x:v>
+      </x:c>
+      <x:c r="O75" s="28"/>
+      <x:c r="P75" s="28"/>
+      <x:c r="Q75" s="28"/>
+      <x:c r="R75" s="28"/>
+      <x:c r="S75" s="28"/>
+      <x:c r="T75" s="9" t="str">
+        <x:v>Distinction from icore and exact processing</x:v>
+      </x:c>
+      <x:c r="U75" s="29"/>
+      <x:c r="V75" s="9" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="75" customHeight="1">
+      <x:c r="A76" s="9" t="str">
+        <x:v>proposal.bio.icore_fibers</x:v>
+      </x:c>
+      <x:c r="B76" s="9" t="str">
+        <x:v>Scraped icore fibers</x:v>
+      </x:c>
+      <x:c r="C76" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D76" s="9" t="str">
+        <x:v>Raw husk fiber</x:v>
+      </x:c>
+      <x:c r="E76" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F76" s="9" t="str">
+        <x:v>Abundant fibers scraped from shell husks.</x:v>
+      </x:c>
+      <x:c r="G76" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H76" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I76" s="13"/>
+      <x:c r="J76" s="15"/>
+      <x:c r="K76" s="9" t="str">
+        <x:v>Scrape shell husks</x:v>
+      </x:c>
+      <x:c r="L76" s="9" t="str">
+        <x:v>Paper feedstock and difficult pressed-textile material</x:v>
+      </x:c>
+      <x:c r="M76" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N76" s="9" t="str">
+        <x:v>Author spelling retained; no composition, fluid identity or special property invented.</x:v>
+      </x:c>
+      <x:c r="O76" s="28"/>
+      <x:c r="P76" s="28"/>
+      <x:c r="Q76" s="28"/>
+      <x:c r="R76" s="28"/>
+      <x:c r="S76" s="28"/>
+      <x:c r="T76" s="9" t="str">
+        <x:v>Define icore and whether paper uses one or both fiber types</x:v>
+      </x:c>
+      <x:c r="U76" s="29"/>
+      <x:c r="V76" s="9" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="75" customHeight="1">
+      <x:c r="A77" s="9" t="str">
+        <x:v>proposal.bio.husk_paper</x:v>
+      </x:c>
+      <x:c r="B77" s="9" t="str">
+        <x:v>Husk-fiber paper</x:v>
+      </x:c>
+      <x:c r="C77" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D77" s="9" t="str">
+        <x:v>Paper</x:v>
+      </x:c>
+      <x:c r="E77" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F77" s="9" t="str">
+        <x:v>The main paper material comes from scraped shell-husk fibers.</x:v>
+      </x:c>
+      <x:c r="G77" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H77" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I77" s="13"/>
+      <x:c r="J77" s="15"/>
+      <x:c r="K77" s="9" t="str">
+        <x:v>Process scraped husk fibers</x:v>
+      </x:c>
+      <x:c r="L77" s="9" t="str">
+        <x:v>Paper sheets; end uses remain open</x:v>
+      </x:c>
+      <x:c r="M77" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N77" s="9" t="str">
+        <x:v>Main source established; paper recipe, difficulty and yield not yet specified.</x:v>
+      </x:c>
+      <x:c r="O77" s="28"/>
+      <x:c r="P77" s="28"/>
+      <x:c r="Q77" s="28"/>
+      <x:c r="R77" s="28"/>
+      <x:c r="S77" s="28"/>
+      <x:c r="T77" s="9" t="str">
+        <x:v>Sheet sizes, paper properties and production method</x:v>
+      </x:c>
+      <x:c r="U77" s="29"/>
+      <x:c r="V77" s="9" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="75" customHeight="1">
+      <x:c r="A78" s="9" t="str">
+        <x:v>proposal.bio.pressed_husk</x:v>
+      </x:c>
+      <x:c r="B78" s="9" t="str">
+        <x:v>Pressed husk-fiber textile material</x:v>
+      </x:c>
+      <x:c r="C78" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D78" s="9" t="str">
+        <x:v>Pressed textile material</x:v>
+      </x:c>
+      <x:c r="E78" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F78" s="9" t="str">
+        <x:v>Difficult processed/pressed husk-fiber material.</x:v>
+      </x:c>
+      <x:c r="G78" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H78" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I78" s="13"/>
+      <x:c r="J78" s="15"/>
+      <x:c r="K78" s="9" t="str">
+        <x:v>Very difficult processing and pressing of husk fibers</x:v>
+      </x:c>
+      <x:c r="L78" s="9" t="str">
+        <x:v>Textile-material use under the no-cloth rule</x:v>
+      </x:c>
+      <x:c r="M78" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N78" s="9" t="str">
+        <x:v>No cloth of any kind; exact product form, flexibility and uses are unapproved.</x:v>
+      </x:c>
+      <x:c r="O78" s="28"/>
+      <x:c r="P78" s="28"/>
+      <x:c r="Q78" s="28"/>
+      <x:c r="R78" s="28"/>
+      <x:c r="S78" s="28"/>
+      <x:c r="T78" s="9" t="str">
+        <x:v>Binder, equipment, work and finished properties</x:v>
+      </x:c>
+      <x:c r="U78" s="29"/>
+      <x:c r="V78" s="9" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="75" customHeight="1">
+      <x:c r="A79" s="9" t="str">
+        <x:v>proposal.bio.hide</x:v>
+      </x:c>
+      <x:c r="B79" s="9" t="str">
+        <x:v>Raw hide</x:v>
+      </x:c>
+      <x:c r="C79" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D79" s="9" t="str">
+        <x:v>Animal hide</x:v>
+      </x:c>
+      <x:c r="E79" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F79" s="9" t="str">
+        <x:v>Hide feedstock for extremely low-yield material processing.</x:v>
+      </x:c>
+      <x:c r="G79" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H79" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I79" s="13"/>
+      <x:c r="J79" s="15"/>
+      <x:c r="K79" s="9" t="str">
+        <x:v>Creature hide collection; species and method unapproved</x:v>
+      </x:c>
+      <x:c r="L79" s="9" t="str">
+        <x:v>Textile and other material processing with extremely low yield</x:v>
+      </x:c>
+      <x:c r="M79" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N79" s="9" t="str">
+        <x:v>Low yield concerns conversion into usable material; does not define carcass yield.</x:v>
+      </x:c>
+      <x:c r="O79" s="28"/>
+      <x:c r="P79" s="28"/>
+      <x:c r="Q79" s="28"/>
+      <x:c r="R79" s="28"/>
+      <x:c r="S79" s="28"/>
+      <x:c r="T79" s="9" t="str">
+        <x:v>Species, preservation and workable output forms</x:v>
+      </x:c>
+      <x:c r="U79" s="29"/>
+      <x:c r="V79" s="9" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="75" customHeight="1">
+      <x:c r="A80" s="9" t="str">
+        <x:v>proposal.bio.hide_material</x:v>
+      </x:c>
+      <x:c r="B80" s="9" t="str">
+        <x:v>Processed hide material</x:v>
+      </x:c>
+      <x:c r="C80" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D80" s="9" t="str">
+        <x:v>Processed biological</x:v>
+      </x:c>
+      <x:c r="E80" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F80" s="9" t="str">
+        <x:v>Scarce usable material obtained from hide processing.</x:v>
+      </x:c>
+      <x:c r="G80" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H80" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I80" s="13"/>
+      <x:c r="J80" s="15"/>
+      <x:c r="K80" s="9" t="str">
+        <x:v>Process raw hide</x:v>
+      </x:c>
+      <x:c r="L80" s="9" t="str">
+        <x:v>Candidate material for later product design</x:v>
+      </x:c>
+      <x:c r="M80" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N80" s="9" t="str">
+        <x:v>Extremely low usable yield. No cloth; output form and properties remain proposals.</x:v>
+      </x:c>
+      <x:c r="O80" s="28"/>
+      <x:c r="P80" s="28"/>
+      <x:c r="Q80" s="28"/>
+      <x:c r="R80" s="28"/>
+      <x:c r="S80" s="28"/>
+      <x:c r="T80" s="9" t="str">
+        <x:v>Processing method, intended products and balance</x:v>
+      </x:c>
+      <x:c r="U80" s="29"/>
+      <x:c r="V80" s="9" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4454,7 +4782,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R117d4bb2fbc84a92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff7cfb275b04c7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5362,7 +5690,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4ba61aaeecf4417"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a67be037dd844cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5728,7 +6056,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2088468a270246d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb68dcc88279498b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5819,7 +6147,7 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Existing resources plus natural minerals, unworked metals, charcoal and biological proposals</x:v>
@@ -5834,13 +6162,13 @@
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A9)</x:f>
-        <x:v>11</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
-        <x:v>Three trial salvage parts plus proposed biological products</x:v>
+        <x:v>Existing salvage and proposed materials, including husk-fiber paper and difficult pressed textiles</x:v>
       </x:c>
       <x:c r="D9" s="4" t="str">
-        <x:v>Recipes and properties remain proposals</x:v>
+        <x:v>No cloth. Hide/fur conversion yields extremely little usable material.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -5930,7 +6258,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1c2f2589b54738"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32b5acf433784cfd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5993,7 +6321,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>69 design entries: 18 existing item IDs, 11 user-directed concepts, and 40 proposed resources/materials. Implementation remains unchanged.</x:v>
+        <x:v>75 design entries: 18 existing item IDs and 57 design concepts. Six husk/paper/hide entries record the author's material direction; no runtime items added.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -6212,10 +6540,50 @@
         <x:v>Unprocessed iron-rich stones maps to the existing Ironstone Ore candidate. Specific hematite/magnetite distinctions remain open rather than creating another duplicate generic item.</x:v>
       </x:c>
     </x:row>
+    <x:row r="36" ht="60" customHeight="1">
+      <x:c r="A36" s="4" t="str">
+        <x:v>No cloth</x:v>
+      </x:c>
+      <x:c r="B36" s="4" t="str">
+        <x:v>No cloth of any kind. Pressed textile/material processing does not establish cloth items or an easy fabric economy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="60" customHeight="1">
+      <x:c r="A37" s="4" t="str">
+        <x:v>Husk fibers and paper</x:v>
+      </x:c>
+      <x:c r="B37" s="4" t="str">
+        <x:v>Shell husks supply abundant chitin/icore fibers. Scraped husk fibers supply the main paper. Textile processing/pressing is very difficult.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="60" customHeight="1">
+      <x:c r="A38" s="4" t="str">
+        <x:v>Hide and fur yield</x:v>
+      </x:c>
+      <x:c r="B38" s="4" t="str">
+        <x:v>Extremely low usable yield from hide/fur processing. No numeric ratio, easy liner production or finished garment recipe approved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="60" customHeight="1">
+      <x:c r="A39" s="4" t="str">
+        <x:v>Icore</x:v>
+      </x:c>
+      <x:c r="B39" s="4" t="str">
+        <x:v>Author spelling preserved exactly. Composition and differences from chitin remain undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="60" customHeight="1">
+      <x:c r="A40" s="4" t="str">
+        <x:v>Prior garment proposals</x:v>
+      </x:c>
+      <x:c r="B40" s="4" t="str">
+        <x:v>The previous felted underfur liner is now a candidate pressed fur material requiring reassessment. Cloak/shade prototype appearance does not establish cloth composition.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a253a4df8d14f7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3102a32fce194374"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6544,22 +6912,22 @@
         <x:v>proposal.bio.liner</x:v>
       </x:c>
       <x:c r="C15" s="4" t="str">
-        <x:v>Dry clean, card and compress</x:v>
+        <x:v>Process fur into a candidate pressed material</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:v>Replaceable jacket/cloak liners</x:v>
+        <x:v>Scarce usable material; garment application undecided</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
-        <x:v>Stationary preservation/workbench proposed</x:v>
+        <x:v>Specialist stationary processing proposed</x:v>
       </x:c>
       <x:c r="F15" s="4" t="str">
-        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+        <x:v>Extremely low usable yield; no cloth; previous routine liner/felting assumption superseded</x:v>
       </x:c>
       <x:c r="G15" s="4" t="str">
-        <x:v>New proposal</x:v>
+        <x:v>User constraint; product form proposed</x:v>
       </x:c>
       <x:c r="H15" s="4" t="str">
-        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="85" customHeight="1">
@@ -6874,10 +7242,192 @@
         <x:v>User direction; proposed crafting relationship</x:v>
       </x:c>
     </x:row>
+    <x:row r="28" ht="90" customHeight="1">
+      <x:c r="A28" s="4" t="str">
+        <x:v>proposal.bio.shell</x:v>
+      </x:c>
+      <x:c r="B28" s="4" t="str">
+        <x:v>proposal.bio.chitin_fibers</x:v>
+      </x:c>
+      <x:c r="C28" s="4" t="str">
+        <x:v>Scrape fibers from shell husks</x:v>
+      </x:c>
+      <x:c r="D28" s="4" t="str">
+        <x:v>Abundant raw chitin fiber feed</x:v>
+      </x:c>
+      <x:c r="E28" s="4" t="str">
+        <x:v>Work location not yet defined</x:v>
+      </x:c>
+      <x:c r="F28" s="4" t="str">
+        <x:v>Scraping rate, tools and actual collectible yield unapproved</x:v>
+      </x:c>
+      <x:c r="G28" s="4" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="H28" s="4" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="90" customHeight="1">
+      <x:c r="A29" s="4" t="str">
+        <x:v>proposal.bio.shell</x:v>
+      </x:c>
+      <x:c r="B29" s="4" t="str">
+        <x:v>proposal.bio.icore_fibers</x:v>
+      </x:c>
+      <x:c r="C29" s="4" t="str">
+        <x:v>Scrape fibers from shell husks</x:v>
+      </x:c>
+      <x:c r="D29" s="4" t="str">
+        <x:v>Abundant raw icore fiber feed</x:v>
+      </x:c>
+      <x:c r="E29" s="4" t="str">
+        <x:v>Work location not yet defined</x:v>
+      </x:c>
+      <x:c r="F29" s="4" t="str">
+        <x:v>Icore composition undefined; no invented special properties</x:v>
+      </x:c>
+      <x:c r="G29" s="4" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="H29" s="4" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="90" customHeight="1">
+      <x:c r="A30" s="4" t="str">
+        <x:v>proposal.bio.chitin_fibers</x:v>
+      </x:c>
+      <x:c r="B30" s="4" t="str">
+        <x:v>proposal.bio.husk_paper</x:v>
+      </x:c>
+      <x:c r="C30" s="4" t="str">
+        <x:v>Process scraped husk fibers into paper</x:v>
+      </x:c>
+      <x:c r="D30" s="4" t="str">
+        <x:v>Main paper material</x:v>
+      </x:c>
+      <x:c r="E30" s="4" t="str">
+        <x:v>Paper-processing station not yet defined</x:v>
+      </x:c>
+      <x:c r="F30" s="4" t="str">
+        <x:v>No numeric yield, paper recipe or processing difficulty approved</x:v>
+      </x:c>
+      <x:c r="G30" s="4" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="H30" s="4" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="90" customHeight="1">
+      <x:c r="A31" s="4" t="str">
+        <x:v>proposal.bio.icore_fibers</x:v>
+      </x:c>
+      <x:c r="B31" s="4" t="str">
+        <x:v>proposal.bio.husk_paper</x:v>
+      </x:c>
+      <x:c r="C31" s="4" t="str">
+        <x:v>Use scraped husk fibers for paper</x:v>
+      </x:c>
+      <x:c r="D31" s="4" t="str">
+        <x:v>Main paper material</x:v>
+      </x:c>
+      <x:c r="E31" s="4" t="str">
+        <x:v>Paper-processing station not yet defined</x:v>
+      </x:c>
+      <x:c r="F31" s="4" t="str">
+        <x:v>Two fiber inputs shown as alternatives/options; mixing requirement not settled</x:v>
+      </x:c>
+      <x:c r="G31" s="4" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="H31" s="4" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="90" customHeight="1">
+      <x:c r="A32" s="4" t="str">
+        <x:v>proposal.bio.chitin_fibers</x:v>
+      </x:c>
+      <x:c r="B32" s="4" t="str">
+        <x:v>proposal.bio.pressed_husk</x:v>
+      </x:c>
+      <x:c r="C32" s="4" t="str">
+        <x:v>Difficult processing and pressing</x:v>
+      </x:c>
+      <x:c r="D32" s="4" t="str">
+        <x:v>Pressed textile material</x:v>
+      </x:c>
+      <x:c r="E32" s="4" t="str">
+        <x:v>Specialist processing proposed</x:v>
+      </x:c>
+      <x:c r="F32" s="4" t="str">
+        <x:v>Very difficult; no cloth; exact recipe and product properties unresolved</x:v>
+      </x:c>
+      <x:c r="G32" s="4" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="H32" s="4" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="90" customHeight="1">
+      <x:c r="A33" s="4" t="str">
+        <x:v>proposal.bio.icore_fibers</x:v>
+      </x:c>
+      <x:c r="B33" s="4" t="str">
+        <x:v>proposal.bio.pressed_husk</x:v>
+      </x:c>
+      <x:c r="C33" s="4" t="str">
+        <x:v>Difficult processing and pressing</x:v>
+      </x:c>
+      <x:c r="D33" s="4" t="str">
+        <x:v>Pressed textile material</x:v>
+      </x:c>
+      <x:c r="E33" s="4" t="str">
+        <x:v>Specialist processing proposed</x:v>
+      </x:c>
+      <x:c r="F33" s="4" t="str">
+        <x:v>Fiber combination unresolved; this is not a two-input recipe specification</x:v>
+      </x:c>
+      <x:c r="G33" s="4" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="H33" s="4" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="90" customHeight="1">
+      <x:c r="A34" s="4" t="str">
+        <x:v>proposal.bio.hide</x:v>
+      </x:c>
+      <x:c r="B34" s="4" t="str">
+        <x:v>proposal.bio.hide_material</x:v>
+      </x:c>
+      <x:c r="C34" s="4" t="str">
+        <x:v>Process hide into usable material</x:v>
+      </x:c>
+      <x:c r="D34" s="4" t="str">
+        <x:v>Scarce material output</x:v>
+      </x:c>
+      <x:c r="E34" s="4" t="str">
+        <x:v>Specialist processing proposed</x:v>
+      </x:c>
+      <x:c r="F34" s="4" t="str">
+        <x:v>Extremely low yield; no cloth; no numeric ratio specified</x:v>
+      </x:c>
+      <x:c r="G34" s="4" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="H34" s="4" t="str">
+        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc28d6f4ba88f4222"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refceae31ddf34b4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6989,13 +7539,13 @@
         <x:v>Quiet feedstock supply via abandoned molts; hunt only when worthwhile</x:v>
       </x:c>
       <x:c r="F6" s="4" t="str">
-        <x:v>proposal.bio.shell; proposal.bio.underfur; proposal.bio.tendon</x:v>
+        <x:v>proposal.bio.shell; proposal.bio.underfur; proposal.bio.tendon; proposal.bio.chitin_fibers; proposal.bio.icore_fibers</x:v>
       </x:c>
       <x:c r="G6" s="4" t="str">
         <x:v>Molts and bedding can supply modest materials without a kill</x:v>
       </x:c>
       <x:c r="H6" s="4" t="str">
-        <x:v>Primary productivity and crust biology unresolved; no plant grazing</x:v>
+        <x:v>Primary productivity and crust biology unresolved; no plant grazing; fiber supply follows husk rule, but species-specific yields remain unapproved; fur conversion has extremely low usable yield; no cloth</x:v>
       </x:c>
       <x:c r="I6" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -7047,13 +7597,13 @@
         <x:v>Storm timing creates a dangerous optional expedition target</x:v>
       </x:c>
       <x:c r="F8" s="4" t="str">
-        <x:v>proposal.bio.organ; proposal.bio.shell; proposal.bio.tendon</x:v>
+        <x:v>proposal.bio.organ; proposal.bio.shell; proposal.bio.tendon; proposal.bio.chitin_fibers; proposal.bio.icore_fibers</x:v>
       </x:c>
       <x:c r="G8" s="4" t="str">
         <x:v>Abandoned molts available after migrations; rare tissue requires a carcass</x:v>
       </x:c>
       <x:c r="H8" s="4" t="str">
-        <x:v>Charge sensing/storage biology and electrical behavior are speculative</x:v>
+        <x:v>Charge sensing/storage biology and electrical behavior are speculative; fiber supply follows husk rule, but species-specific yields remain unapproved</x:v>
       </x:c>
       <x:c r="I8" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -7076,13 +7626,13 @@
         <x:v>Carcass harvesting attracts competition and encourages selective removal</x:v>
       </x:c>
       <x:c r="F9" s="4" t="str">
-        <x:v>proposal.bio.jaw; proposal.bio.shell; proposal.bio.fat</x:v>
+        <x:v>proposal.bio.jaw; proposal.bio.shell; proposal.bio.fat; proposal.bio.chitin_fibers; proposal.bio.icore_fibers</x:v>
       </x:c>
       <x:c r="G9" s="4" t="str">
         <x:v>Track feeding sites for discarded dry fragments</x:v>
       </x:c>
       <x:c r="H9" s="4" t="str">
-        <x:v>Population depends on a viable food web; no established species or combat kit</x:v>
+        <x:v>Population depends on a viable food web; no established species or combat kit; fiber supply follows husk rule, but species-specific yields remain unapproved</x:v>
       </x:c>
       <x:c r="I9" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -7111,7 +7661,7 @@
         <x:v>Shed fur and abandoned rests provide a low-impact collection option</x:v>
       </x:c>
       <x:c r="H10" s="4" t="str">
-        <x:v>Movement, size, ecology and hunt behavior need design</x:v>
+        <x:v>Movement, size, ecology and hunt behavior need design; fur conversion has extremely low usable yield; no cloth</x:v>
       </x:c>
       <x:c r="I10" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -7120,7 +7670,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R211a51648a82418b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcaca3ea7c1554ba7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record Burden Beasts anatomy boundary and faunal material rules
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R7c7839909cc94067"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R75ab1c9bb144465f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R4a034556bca247d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R3570054a1ff645e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R3e127f52146b4c44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R5b65cf6fa26e419d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R070361ad3a944f6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R2bb57a32ecd4436c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R5bae113c85de4a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R7e8a203c11cb4c93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R9966bb4b89454b87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R16cb4c6545b64079"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R51c38aade7bf49dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R98dc64d063be4a21"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52,7 +52,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -114,6 +114,16 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -127,7 +137,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -231,6 +241,12 @@
     <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -283,7 +299,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -363,7 +379,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -2722,7 +2738,7 @@
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N41" s="9" t="str">
-        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+        <x:v>No yield numbers. Internal chemistry is mostly toxic to humans; faunal chemicals/liquids can be materials. Anatomy and containment remain unresolved.</x:v>
       </x:c>
       <x:c r="O41" s="22"/>
       <x:c r="P41" s="22"/>
@@ -2774,7 +2790,7 @@
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N42" s="9" t="str">
-        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+        <x:v>No yield numbers. Internal chemistry is mostly toxic to humans; faunal chemicals/liquids can be materials. Anatomy and containment remain unresolved.</x:v>
       </x:c>
       <x:c r="O42" s="22"/>
       <x:c r="P42" s="22"/>
@@ -2878,7 +2894,7 @@
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N44" s="9" t="str">
-        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+        <x:v>No yield numbers. Internal chemistry is mostly toxic to humans; faunal chemicals/liquids can be materials. Anatomy and containment remain unresolved.</x:v>
       </x:c>
       <x:c r="O44" s="22"/>
       <x:c r="P44" s="22"/>
@@ -2950,7 +2966,7 @@
         <x:v>proposal.bio.fat</x:v>
       </x:c>
       <x:c r="B46" s="9" t="str">
-        <x:v>Fresh fat-bearing tissue</x:v>
+        <x:v>Unverified fat-like tissue concept</x:v>
       </x:c>
       <x:c r="C46" s="9" t="str">
         <x:v>Resources</x:v>
@@ -2959,10 +2975,10 @@
         <x:v>Perishable tissue</x:v>
       </x:c>
       <x:c r="E46" s="9" t="str">
-        <x:v>New proposal</x:v>
+        <x:v>Needs lore anatomy review</x:v>
       </x:c>
       <x:c r="F46" s="9" t="str">
-        <x:v>Dry solid lubricant and binder research</x:v>
+        <x:v>Earlier conventional-fat assumption withheld pending Burden Beasts anatomy review.</x:v>
       </x:c>
       <x:c r="G46" s="9" t="str">
         <x:v>None</x:v>
@@ -2973,16 +2989,16 @@
       <x:c r="I46" s="13"/>
       <x:c r="J46" s="15"/>
       <x:c r="K46" s="9" t="str">
-        <x:v>Recent carcass; preservation rules required</x:v>
+        <x:v>No validated species or anatomy source</x:v>
       </x:c>
       <x:c r="L46" s="9" t="str">
-        <x:v>See Resource chains</x:v>
+        <x:v>Prior wax/lubricant route is a conditional proposal only</x:v>
       </x:c>
       <x:c r="M46" s="9" t="str">
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N46" s="9" t="str">
-        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+        <x:v>Most fauna lacks traditional flesh; conventional mammalian fat cannot be assumed. Not an established food.</x:v>
       </x:c>
       <x:c r="O46" s="22"/>
       <x:c r="P46" s="22"/>
@@ -2990,11 +3006,11 @@
       <x:c r="R46" s="22"/>
       <x:c r="S46" s="22"/>
       <x:c r="T46" s="9" t="str">
-        <x:v>Ecology, tissue preservation, safe fiction, processing and final naming</x:v>
+        <x:v>Review actual Burden Beasts anatomy before assigning tissue properties</x:v>
       </x:c>
       <x:c r="U46" s="23"/>
       <x:c r="V46" s="9" t="str">
-        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="66" customHeight="1">
@@ -3034,7 +3050,7 @@
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N47" s="9" t="str">
-        <x:v>No yield numbers; fluids outside living organisms remain a canon question. Molt collection where feasible.</x:v>
+        <x:v>No yield numbers. Internal chemistry is mostly toxic to humans; faunal chemicals/liquids can be materials. Anatomy and containment remain unresolved.</x:v>
       </x:c>
       <x:c r="O47" s="22"/>
       <x:c r="P47" s="22"/>
@@ -3375,10 +3391,10 @@
         <x:v>Processed biological</x:v>
       </x:c>
       <x:c r="E54" s="9" t="str">
-        <x:v>New proposal</x:v>
+        <x:v>Needs lore anatomy review</x:v>
       </x:c>
       <x:c r="F54" s="9" t="str">
-        <x:v>Sealing compounds and dry lubricant research</x:v>
+        <x:v>Conditional solid biological product; the earlier fat precursor is unverified.</x:v>
       </x:c>
       <x:c r="G54" s="9" t="str">
         <x:v>None</x:v>
@@ -3389,16 +3405,16 @@
       <x:c r="I54" s="13"/>
       <x:c r="J54" s="15"/>
       <x:c r="K54" s="9" t="str">
-        <x:v>Process fat</x:v>
+        <x:v>Precursor and conversion await anatomy review</x:v>
       </x:c>
       <x:c r="L54" s="9" t="str">
-        <x:v>Process tissue into a retained solid; no free-liquid commodity</x:v>
+        <x:v>Potential sealing/lubricant use remains a proposal</x:v>
       </x:c>
       <x:c r="M54" s="9" t="str">
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N54" s="9" t="str">
-        <x:v>Speculative material capability; no effects or real processing instructions established.</x:v>
+        <x:v>No approved fat source, chemical identity or conversion. Not an established material property.</x:v>
       </x:c>
       <x:c r="O54" s="22"/>
       <x:c r="P54" s="22"/>
@@ -3406,11 +3422,11 @@
       <x:c r="R54" s="22"/>
       <x:c r="S54" s="22"/>
       <x:c r="T54" s="9" t="str">
-        <x:v>Material properties, additives, station, balance and world-rule compatibility</x:v>
+        <x:v>Review precursor and chemistry against Burden Beasts anatomy</x:v>
       </x:c>
       <x:c r="U54" s="23"/>
       <x:c r="V54" s="9" t="str">
-        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="66" customHeight="1">
@@ -4763,6 +4779,162 @@
       <x:c r="U80" s="29"/>
       <x:c r="V80" s="9" t="str">
         <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="80" customHeight="1">
+      <x:c r="A81" s="9" t="str">
+        <x:v>proposal.bio.edible_fraction</x:v>
+      </x:c>
+      <x:c r="B81" s="9" t="str">
+        <x:v>Edible fauna fraction (species TBD)</x:v>
+      </x:c>
+      <x:c r="C81" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D81" s="9" t="str">
+        <x:v>Food candidate</x:v>
+      </x:c>
+      <x:c r="E81" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F81" s="9" t="str">
+        <x:v>Some fauna can be eaten, but provides poor nutrition.</x:v>
+      </x:c>
+      <x:c r="G81" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H81" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I81" s="13"/>
+      <x:c r="J81" s="15"/>
+      <x:c r="K81" s="9" t="str">
+        <x:v>Only explicitly edible species/parts; preparation undefined</x:v>
+      </x:c>
+      <x:c r="L81" s="9" t="str">
+        <x:v>Potential supplementary food; does not replace algae</x:v>
+      </x:c>
+      <x:c r="M81" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N81" s="9" t="str">
+        <x:v>Most fauna lacks traditional flesh; no meat model, calorie values or safe preparation assigned.</x:v>
+      </x:c>
+      <x:c r="O81" s="30"/>
+      <x:c r="P81" s="30"/>
+      <x:c r="Q81" s="30"/>
+      <x:c r="R81" s="30"/>
+      <x:c r="S81" s="30"/>
+      <x:c r="T81" s="9" t="str">
+        <x:v>Identify species/parts from Burden Beasts anatomy; carrier/use rules not implemented</x:v>
+      </x:c>
+      <x:c r="U81" s="31"/>
+      <x:c r="V81" s="9" t="str">
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="80" customHeight="1">
+      <x:c r="A82" s="9" t="str">
+        <x:v>proposal.bio.chemical_material</x:v>
+      </x:c>
+      <x:c r="B82" s="9" t="str">
+        <x:v>Faunal chemical material (unspecified)</x:v>
+      </x:c>
+      <x:c r="C82" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D82" s="9" t="str">
+        <x:v>Chemical material</x:v>
+      </x:c>
+      <x:c r="E82" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F82" s="9" t="str">
+        <x:v>Internal faunal chemicals can be used as materials despite toxicity to humans.</x:v>
+      </x:c>
+      <x:c r="G82" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H82" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I82" s="13"/>
+      <x:c r="J82" s="15"/>
+      <x:c r="K82" s="9" t="str">
+        <x:v>Species-specific extraction remains undefined</x:v>
+      </x:c>
+      <x:c r="L82" s="9" t="str">
+        <x:v>Material processing uses to be established</x:v>
+      </x:c>
+      <x:c r="M82" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N82" s="9" t="str">
+        <x:v>Most internal chemistry is toxic. No named reagent, solvent, fuel or recipe established.</x:v>
+      </x:c>
+      <x:c r="O82" s="30"/>
+      <x:c r="P82" s="30"/>
+      <x:c r="Q82" s="30"/>
+      <x:c r="R82" s="30"/>
+      <x:c r="S82" s="30"/>
+      <x:c r="T82" s="9" t="str">
+        <x:v>Chemical identities, useful properties, extraction and containment</x:v>
+      </x:c>
+      <x:c r="U82" s="31"/>
+      <x:c r="V82" s="9" t="str">
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="80" customHeight="1">
+      <x:c r="A83" s="9" t="str">
+        <x:v>proposal.bio.liquid_material</x:v>
+      </x:c>
+      <x:c r="B83" s="9" t="str">
+        <x:v>Faunal liquid material (unspecified)</x:v>
+      </x:c>
+      <x:c r="C83" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D83" s="9" t="str">
+        <x:v>Biological liquid material</x:v>
+      </x:c>
+      <x:c r="E83" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F83" s="9" t="str">
+        <x:v>Biological liquids may be extracted for use as materials.</x:v>
+      </x:c>
+      <x:c r="G83" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H83" s="9" t="str">
+        <x:v>Legger / local storage proposed</x:v>
+      </x:c>
+      <x:c r="I83" s="13"/>
+      <x:c r="J83" s="15"/>
+      <x:c r="K83" s="9" t="str">
+        <x:v>Faunal interiors; species-specific extraction undefined</x:v>
+      </x:c>
+      <x:c r="L83" s="9" t="str">
+        <x:v>Material use; not presumed drinkable</x:v>
+      </x:c>
+      <x:c r="M83" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N83" s="9" t="str">
+        <x:v>No natural free water or edible-liquid assumption. Storage, stability and specific uses unresolved.</x:v>
+      </x:c>
+      <x:c r="O83" s="30"/>
+      <x:c r="P83" s="30"/>
+      <x:c r="Q83" s="30"/>
+      <x:c r="R83" s="30"/>
+      <x:c r="S83" s="30"/>
+      <x:c r="T83" s="9" t="str">
+        <x:v>Liquid identities, containers, extraction conditions and processing</x:v>
+      </x:c>
+      <x:c r="U83" s="31"/>
+      <x:c r="V83" s="9" t="str">
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4782,7 +4954,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff7cfb275b04c7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6244e3b33add40f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5690,7 +5862,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a67be037dd844cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a0e06fe4ed24cbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6056,7 +6228,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb68dcc88279498b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94af4ea1b9664462"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6147,13 +6319,13 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>50</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Existing resources plus natural minerals, unworked metals, charcoal and biological proposals</x:v>
+        <x:v>Existing resources plus proposed minerals, biological materials and unspecified fauna chemistry</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Regional evidence supports candidate selection; availability and processing stay open</x:v>
+        <x:v>Some fauna edible but poorly nutritious; most internal chemistry toxic; species/uses unresolved</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -6258,7 +6430,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32b5acf433784cfd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b37eb7933644f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6321,7 +6493,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>75 design entries: 18 existing item IDs and 57 design concepts. Six husk/paper/hide entries record the author's material direction; no runtime items added.</x:v>
+        <x:v>78 design entries: 18 existing item IDs and 60 design concepts. Generic fauna chemistry/food placeholders are not named species, chemicals or implemented items.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -6385,7 +6557,7 @@
         <x:v>Algae</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str">
-        <x:v>Algae remains the survival backbone. Fauna products do not establish alternate food/hydration or free-liquid supplies.</x:v>
+        <x:v>Algae remains the survival backbone. Some fauna is edible but poorly nutritious; this does not make other fauna/parts edible or establish an alternate hydration supply.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="38" customHeight="1">
@@ -6580,10 +6752,50 @@
         <x:v>The previous felted underfur liner is now a candidate pressed fur material requiring reassessment. Cloak/shade prototype appearance does not establish cloth composition.</x:v>
       </x:c>
     </x:row>
+    <x:row r="41" ht="60" customHeight="1">
+      <x:c r="A41" s="4" t="str">
+        <x:v>Fauna edibility</x:v>
+      </x:c>
+      <x:c r="B41" s="4" t="str">
+        <x:v>Some fauna can be eaten but is not nutritious. No universal meat resource, edible species list or preparation method is established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="60" customHeight="1">
+      <x:c r="A42" s="4" t="str">
+        <x:v>Fauna anatomy</x:v>
+      </x:c>
+      <x:c r="B42" s="4" t="str">
+        <x:v>Most fauna lacks flesh in the traditional sense. Earlier mammalian fat/muscle assumptions await source review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="60" customHeight="1">
+      <x:c r="A43" s="4" t="str">
+        <x:v>Chemical materials</x:v>
+      </x:c>
+      <x:c r="B43" s="4" t="str">
+        <x:v>Most internal fauna chemistry is toxic to humans; chemicals and liquids can nevertheless be material resources. Specific properties and processing remain undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="60" customHeight="1">
+      <x:c r="A44" s="4" t="str">
+        <x:v>Liquid rule clarification</x:v>
+      </x:c>
+      <x:c r="B44" s="4" t="str">
+        <x:v>Extracted faunal liquids can be materials. This supersedes earlier blanket doubts about out-of-body liquids while preserving no natural free water.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="60" customHeight="1">
+      <x:c r="A45" s="4" t="str">
+        <x:v>Burden Beasts reference</x:v>
+      </x:c>
+      <x:c r="B45" s="4" t="str">
+        <x:v>The author corrected the anatomy reference to Burden Beasts. Separate lore repo remains unavailable; no source-specific anatomy is claimed.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3102a32fce194374"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R459e4aaab7454ce9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6843,7 +7055,7 @@
         <x:v>Stationary preservation/workbench proposed</x:v>
       </x:c>
       <x:c r="F12" s="4" t="str">
-        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+        <x:v>This dry-product route has no approved yield/recipe. Faunal liquids are separately valid material candidates.</x:v>
       </x:c>
       <x:c r="G12" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -6869,7 +7081,7 @@
         <x:v>Stationary preservation/workbench proposed</x:v>
       </x:c>
       <x:c r="F13" s="4" t="str">
-        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+        <x:v>This dry-product route has no approved yield/recipe. Faunal liquids are separately valid material candidates.</x:v>
       </x:c>
       <x:c r="G13" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -6895,7 +7107,7 @@
         <x:v>Stationary preservation/workbench proposed</x:v>
       </x:c>
       <x:c r="F14" s="4" t="str">
-        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+        <x:v>This dry-product route has no approved yield/recipe. Faunal liquids are separately valid material candidates.</x:v>
       </x:c>
       <x:c r="G14" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -6947,7 +7159,7 @@
         <x:v>Stationary preservation/workbench proposed</x:v>
       </x:c>
       <x:c r="F16" s="4" t="str">
-        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+        <x:v>This dry-product route has no approved yield/recipe. Faunal liquids are separately valid material candidates.</x:v>
       </x:c>
       <x:c r="G16" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -6973,7 +7185,7 @@
         <x:v>Stationary preservation/workbench proposed</x:v>
       </x:c>
       <x:c r="F17" s="4" t="str">
-        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+        <x:v>This dry-product route has no approved yield/recipe. Faunal liquids are separately valid material candidates.</x:v>
       </x:c>
       <x:c r="G17" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -6990,22 +7202,22 @@
         <x:v>proposal.bio.wax</x:v>
       </x:c>
       <x:c r="C18" s="4" t="str">
-        <x:v>Process tissue into a retained solid; no free-liquid commodity</x:v>
+        <x:v>Unverified conversion; await actual anatomy</x:v>
       </x:c>
       <x:c r="D18" s="4" t="str">
-        <x:v>Sealing compounds and dry lubricant research</x:v>
+        <x:v>Conditional solid product only</x:v>
       </x:c>
       <x:c r="E18" s="4" t="str">
-        <x:v>Stationary preservation/workbench proposed</x:v>
+        <x:v>Processing undefined</x:v>
       </x:c>
       <x:c r="F18" s="4" t="str">
-        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+        <x:v>Conventional fat precursor not established; Burden Beasts source must be reviewed</x:v>
       </x:c>
       <x:c r="G18" s="4" t="str">
-        <x:v>New proposal</x:v>
+        <x:v>Needs lore anatomy review</x:v>
       </x:c>
       <x:c r="H18" s="4" t="str">
-        <x:v>User design direction, October 14, 2026; local brainstorming. New proposal unless explicitly marked User direction.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="85" customHeight="1">
@@ -7025,7 +7237,7 @@
         <x:v>Stationary preservation/workbench proposed</x:v>
       </x:c>
       <x:c r="F19" s="4" t="str">
-        <x:v>No liquid commodity, numeric yield or finished recipe approved</x:v>
+        <x:v>This dry-product route has no approved yield/recipe. Faunal liquids are separately valid material candidates.</x:v>
       </x:c>
       <x:c r="G19" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -7427,7 +7639,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refceae31ddf34b4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7280da0587084ad1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7522,7 +7734,7 @@
         <x:v>Status</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="85" customHeight="1">
+    <x:row r="6" ht="115" customHeight="1">
       <x:c r="A6" s="4" t="str">
         <x:v>fauna.plate_grazer</x:v>
       </x:c>
@@ -7545,13 +7757,13 @@
         <x:v>Molts and bedding can supply modest materials without a kill</x:v>
       </x:c>
       <x:c r="H6" s="4" t="str">
-        <x:v>Primary productivity and crust biology unresolved; no plant grazing; fiber supply follows husk rule, but species-specific yields remain unapproved; fur conversion has extremely low usable yield; no cloth</x:v>
+        <x:v>Primary productivity and crust biology unresolved; no plant grazing; fiber supply follows husk rule, but species-specific yields remain unapproved; fur conversion has extremely low usable yield; no cloth; Burden Beasts anatomy unreviewed; no species-specific edibility or chemistry assigned</x:v>
       </x:c>
       <x:c r="I6" s="4" t="str">
         <x:v>New proposal</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="85" customHeight="1">
+    <x:row r="7" ht="115" customHeight="1">
       <x:c r="A7" s="4" t="str">
         <x:v>fauna.burrower</x:v>
       </x:c>
@@ -7574,13 +7786,13 @@
         <x:v>Old bristle-lined burrows provide low-yield scavenging opportunities</x:v>
       </x:c>
       <x:c r="H7" s="4" t="str">
-        <x:v>Burrows and collapse rules must respect fixed terrain; no terrain system authorized</x:v>
+        <x:v>Burrows and collapse rules must respect fixed terrain; no terrain system authorized; Burden Beasts anatomy unreviewed; no species-specific edibility or chemistry assigned</x:v>
       </x:c>
       <x:c r="I7" s="4" t="str">
         <x:v>New proposal</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="85" customHeight="1">
+    <x:row r="8" ht="115" customHeight="1">
       <x:c r="A8" s="4" t="str">
         <x:v>fauna.storm_migrant</x:v>
       </x:c>
@@ -7603,13 +7815,13 @@
         <x:v>Abandoned molts available after migrations; rare tissue requires a carcass</x:v>
       </x:c>
       <x:c r="H8" s="4" t="str">
-        <x:v>Charge sensing/storage biology and electrical behavior are speculative; fiber supply follows husk rule, but species-specific yields remain unapproved</x:v>
+        <x:v>Charge sensing/storage biology and electrical behavior are speculative; fiber supply follows husk rule, but species-specific yields remain unapproved; Burden Beasts anatomy unreviewed; no species-specific edibility or chemistry assigned</x:v>
       </x:c>
       <x:c r="I8" s="4" t="str">
         <x:v>New proposal</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="85" customHeight="1">
+    <x:row r="9" ht="115" customHeight="1">
       <x:c r="A9" s="4" t="str">
         <x:v>fauna.carrion_crusher</x:v>
       </x:c>
@@ -7617,7 +7829,7 @@
         <x:v>Carrion crusher</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
-        <x:v>Heavy crab-like claws, mandibular mouth, muscular mammal-like trunk and gait</x:v>
+        <x:v>Heavy crab-like claws, mandibular mouth and a bulky trunk; internal structure unverified</x:v>
       </x:c>
       <x:c r="D9" s="4" t="str">
         <x:v>Scavenges large carcasses; competes with Booter for remains</x:v>
@@ -7626,19 +7838,19 @@
         <x:v>Carcass harvesting attracts competition and encourages selective removal</x:v>
       </x:c>
       <x:c r="F9" s="4" t="str">
-        <x:v>proposal.bio.jaw; proposal.bio.shell; proposal.bio.fat; proposal.bio.chitin_fibers; proposal.bio.icore_fibers</x:v>
+        <x:v>proposal.bio.jaw; proposal.bio.shell; proposal.bio.chitin_fibers; proposal.bio.icore_fibers</x:v>
       </x:c>
       <x:c r="G9" s="4" t="str">
         <x:v>Track feeding sites for discarded dry fragments</x:v>
       </x:c>
       <x:c r="H9" s="4" t="str">
-        <x:v>Population depends on a viable food web; no established species or combat kit; fiber supply follows husk rule, but species-specific yields remain unapproved</x:v>
+        <x:v>Population depends on a viable food web; no established species or combat kit; fiber supply follows husk rule, but species-specific yields remain unapproved; Burden Beasts anatomy unreviewed; no species-specific edibility or chemistry assigned</x:v>
       </x:c>
       <x:c r="I9" s="4" t="str">
         <x:v>New proposal</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="85" customHeight="1">
+    <x:row r="10" ht="115" customHeight="1">
       <x:c r="A10" s="4" t="str">
         <x:v>fauna.shelf_climber</x:v>
       </x:c>
@@ -7661,7 +7873,7 @@
         <x:v>Shed fur and abandoned rests provide a low-impact collection option</x:v>
       </x:c>
       <x:c r="H10" s="4" t="str">
-        <x:v>Movement, size, ecology and hunt behavior need design; fur conversion has extremely low usable yield; no cloth</x:v>
+        <x:v>Movement, size, ecology and hunt behavior need design; fur conversion has extremely low usable yield; no cloth; Burden Beasts anatomy unreviewed; no species-specific edibility or chemistry assigned</x:v>
       </x:c>
       <x:c r="I10" s="4" t="str">
         <x:v>New proposal</x:v>
@@ -7670,7 +7882,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcaca3ea7c1554ba7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2c000a50716448b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Restore read-only Arc-Dust lore reference access
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R2bb57a32ecd4436c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R5bae113c85de4a14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R7e8a203c11cb4c93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R9966bb4b89454b87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R16cb4c6545b64079"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R51c38aade7bf49dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R98dc64d063be4a21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R049a2a85dc9e4356"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R687cbf64f39649d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Ra46c5b88d68d4738"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R77d24152b0c34689"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rb1f6936ab9bd4adc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R91ac93323c4b4328"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rba837219a57d4d55"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -379,7 +379,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -804,7 +804,7 @@
       <x:c r="T5" s="8" t="str">
         <x:v>Open design decisions</x:v>
       </x:c>
-      <x:c r="U5" s="10" t="str"/>
+      <x:c r="U5" s="10"/>
       <x:c r="V5" s="12" t="str">
         <x:v>Sources</x:v>
       </x:c>
@@ -3010,7 +3010,7 @@
       </x:c>
       <x:c r="U46" s="23"/>
       <x:c r="V46" s="9" t="str">
-        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Related source anatomy proposals now accessible at f6f98515; this item awaits reconciliation; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="66" customHeight="1">
@@ -3426,7 +3426,7 @@
       </x:c>
       <x:c r="U54" s="23"/>
       <x:c r="V54" s="9" t="str">
-        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Related source anatomy proposals now accessible at f6f98515; this item awaits reconciliation; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="66" customHeight="1">
@@ -4830,7 +4830,7 @@
       </x:c>
       <x:c r="U81" s="31"/>
       <x:c r="V81" s="9" t="str">
-        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Related source anatomy proposals now accessible at f6f98515; this item awaits reconciliation; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="80" customHeight="1">
@@ -4882,7 +4882,7 @@
       </x:c>
       <x:c r="U82" s="31"/>
       <x:c r="V82" s="9" t="str">
-        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Related source anatomy proposals now accessible at f6f98515; this item awaits reconciliation; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="80" customHeight="1">
@@ -4934,7 +4934,7 @@
       </x:c>
       <x:c r="U83" s="31"/>
       <x:c r="V83" s="9" t="str">
-        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Related source anatomy proposals now accessible at f6f98515; this item awaits reconciliation; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4954,7 +4954,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6244e3b33add40f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raee8f2a624b741db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5862,7 +5862,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a0e06fe4ed24cbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c3c910994ce471b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6228,7 +6228,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94af4ea1b9664462"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a17e9ab66f4ff0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6430,7 +6430,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b37eb7933644f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0f0d4a67f5e4a0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6621,7 +6621,7 @@
         <x:v>External lore</x:v>
       </x:c>
       <x:c r="B24" s="9" t="str">
-        <x:v>The separate Arc &amp; Dust source repository is unavailable on this machine; no external roster is claimed.</x:v>
+        <x:v>Read-only source access restored October 14: github.com/sleepyseamonster/Arc-Dust, master at f6f98515. No external item roster imported.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
@@ -6789,13 +6789,29 @@
         <x:v>Burden Beasts reference</x:v>
       </x:c>
       <x:c r="B45" s="4" t="str">
-        <x:v>The author corrected the anatomy reference to Burden Beasts. Separate lore repo remains unavailable; no source-specific anatomy is claimed.</x:v>
+        <x:v>The author corrected the anatomy reference to Burden Beasts. Authenticated source Git access restored October 14 at f6f98515. Related fauna records are proposals; exact Burden Beasts owning record not identified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="65" customHeight="1">
+      <x:c r="A46" s="4" t="str">
+        <x:v>Source reconnection</x:v>
+      </x:c>
+      <x:c r="B46" s="4" t="str">
+        <x:v>Read-only Git access verified to sleepyseamonster/Arc-Dust, master at f6f98515c005dc3c73cccd9cbc031691745740c6. No source content was edited.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="65" customHeight="1">
+      <x:c r="A47" s="4" t="str">
+        <x:v>Source reconciliation</x:v>
+      </x:c>
+      <x:c r="B47" s="4" t="str">
+        <x:v>Native biology, domestic burden beetle and chitin/Phagia material records are proposals. Their woven textile assumptions conflict with newer game no-cloth direction. No source species or recipes adopted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R459e4aaab7454ce9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d1990e4a9cd41ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7217,7 +7233,7 @@
         <x:v>Needs lore anatomy review</x:v>
       </x:c>
       <x:c r="H18" s="4" t="str">
-        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Burden Beasts anatomy source unavailable; identities and processing remain undefined.</x:v>
+        <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Related source anatomy proposals now accessible at f6f98515; this item awaits reconciliation; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="85" customHeight="1">
@@ -7639,7 +7655,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7280da0587084ad1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5eedab1f81d447e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7882,7 +7898,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2c000a50716448b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd36be8b266d046e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Brainstorm faunal chemicals toxins and material applications
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R049a2a85dc9e4356"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R687cbf64f39649d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Ra46c5b88d68d4738"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R77d24152b0c34689"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rb1f6936ab9bd4adc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R91ac93323c4b4328"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rba837219a57d4d55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R5173927b2edb4801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Radc4e641995c4637"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R0fbdf3504da74c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R96ab48cee52848b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Re3bf5b8362b14df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rf7d84e54c2294f04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R50822fd1223d4609"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Rca82e73cd2f24217"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52,7 +53,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -124,6 +125,21 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF423B35"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -137,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -247,15 +263,37 @@
     <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="4">
     <x:dxf>
       <x:font>
         <x:color rgb="FF8A5B22"/>
       </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF87521B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF0D9"/>
+        </x:patternFill>
+      </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
@@ -299,7 +337,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V95" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -379,7 +417,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -416,6 +454,22 @@
     <x:tableColumn id="7" name="Collection alternative"/>
     <x:tableColumn id="8" name="Open design issue"/>
     <x:tableColumn id="9" name="Status"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ChemicalConceptsTable" displayName="ChemicalConceptsTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Concept ID"/>
+    <x:tableColumn id="2" name="Working label"/>
+    <x:tableColumn id="3" name="Biological source / role"/>
+    <x:tableColumn id="4" name="Human hazard"/>
+    <x:tableColumn id="5" name="Potential material use"/>
+    <x:tableColumn id="6" name="Design constraint"/>
+    <x:tableColumn id="7" name="Source relationship"/>
+    <x:tableColumn id="8" name="Reference"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -4937,6 +4991,630 @@
         <x:v>Docs/WORLD_BASIS.md#faunal-biology-and-material-use; direct author direction October 14, 2026. Related source anatomy proposals now accessible at f6f98515; this item awaits reconciliation; identities and processing remain undefined.</x:v>
       </x:c>
     </x:row>
+    <x:row r="84" ht="80" customHeight="1">
+      <x:c r="A84" s="9" t="str">
+        <x:v>proposal.chemical.digestive_etchant</x:v>
+      </x:c>
+      <x:c r="B84" s="9" t="str">
+        <x:v>Digestive etchant</x:v>
+      </x:c>
+      <x:c r="C84" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D84" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E84" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F84" s="9" t="str">
+        <x:v>Mineral separation and metal surface preparation</x:v>
+      </x:c>
+      <x:c r="G84" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H84" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I84" s="13"/>
+      <x:c r="J84" s="15"/>
+      <x:c r="K84" s="9" t="str">
+        <x:v>Contained digestive liquor in geological feeders; exposes useful mineral compounds</x:v>
+      </x:c>
+      <x:c r="L84" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M84" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N84" s="9" t="str">
+        <x:v>Corrosive tissue injury; inedible; Could damage containers and useful shell; reusable containment and selectivity need design</x:v>
+      </x:c>
+      <x:c r="O84" s="32"/>
+      <x:c r="P84" s="32"/>
+      <x:c r="Q84" s="32"/>
+      <x:c r="R84" s="32"/>
+      <x:c r="S84" s="32"/>
+      <x:c r="T84" s="9" t="str">
+        <x:v>Source draft describes digestive acids/catalysts; this harvestable agent and uses are new proposals</x:v>
+      </x:c>
+      <x:c r="U84" s="33"/>
+      <x:c r="V84" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="80" customHeight="1">
+      <x:c r="A85" s="9" t="str">
+        <x:v>proposal.chemical.husk_enzyme</x:v>
+      </x:c>
+      <x:c r="B85" s="9" t="str">
+        <x:v>Husk-separation enzyme</x:v>
+      </x:c>
+      <x:c r="C85" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D85" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E85" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F85" s="9" t="str">
+        <x:v>Help release chitin/icore fibers for paper and difficult pressed materials</x:v>
+      </x:c>
+      <x:c r="G85" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H85" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I85" s="13"/>
+      <x:c r="J85" s="15"/>
+      <x:c r="K85" s="9" t="str">
+        <x:v>Proposed catalytic fraction associated with shell renewal or digestion</x:v>
+      </x:c>
+      <x:c r="L85" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M85" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N85" s="9" t="str">
+        <x:v>Biologically active irritant; effects species-dependent; Slow specialist processing still required; must not turn abundant husks into easy cloth</x:v>
+      </x:c>
+      <x:c r="O85" s="32"/>
+      <x:c r="P85" s="32"/>
+      <x:c r="Q85" s="32"/>
+      <x:c r="R85" s="32"/>
+      <x:c r="S85" s="32"/>
+      <x:c r="T85" s="9" t="str">
+        <x:v>Source draft includes industrial enzymes, but fauna origin and this fiber application are new proposals</x:v>
+      </x:c>
+      <x:c r="U85" s="33"/>
+      <x:c r="V85" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="80" customHeight="1">
+      <x:c r="A86" s="9" t="str">
+        <x:v>proposal.chemical.shell_binder</x:v>
+      </x:c>
+      <x:c r="B86" s="9" t="str">
+        <x:v>Shell-binding secretion</x:v>
+      </x:c>
+      <x:c r="C86" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D86" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E86" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F86" s="9" t="str">
+        <x:v>Bind mineral aggregate, shell laminates and pressed fiber materials</x:v>
+      </x:c>
+      <x:c r="G86" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H86" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I86" s="13"/>
+      <x:c r="J86" s="15"/>
+      <x:c r="K86" s="9" t="str">
+        <x:v>Proposed armor-building secretion that binds deposited minerals</x:v>
+      </x:c>
+      <x:c r="L86" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M86" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N86" s="9" t="str">
+        <x:v>Adheres to exposed surfaces; contaminated residue may be toxic; Durable bonding is a proposal; curing conditions and unwanted adhesion remain unresolved</x:v>
+      </x:c>
+      <x:c r="O86" s="32"/>
+      <x:c r="P86" s="32"/>
+      <x:c r="Q86" s="32"/>
+      <x:c r="R86" s="32"/>
+      <x:c r="S86" s="32"/>
+      <x:c r="T86" s="9" t="str">
+        <x:v>Armor-building organs and chitin-derived binders are source-draft seeds; secretion/product is new</x:v>
+      </x:c>
+      <x:c r="U86" s="33"/>
+      <x:c r="V86" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="80" customHeight="1">
+      <x:c r="A87" s="9" t="str">
+        <x:v>proposal.chemical.clotting_compound</x:v>
+      </x:c>
+      <x:c r="B87" s="9" t="str">
+        <x:v>Mineral clotting compound</x:v>
+      </x:c>
+      <x:c r="C87" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D87" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E87" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F87" s="9" t="str">
+        <x:v>Quick hard-setting equipment patches and temporary container seals</x:v>
+      </x:c>
+      <x:c r="G87" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H87" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I87" s="13"/>
+      <x:c r="J87" s="15"/>
+      <x:c r="K87" s="9" t="str">
+        <x:v>Ichor wound response; suspended minerals harden into a protective clot</x:v>
+      </x:c>
+      <x:c r="L87" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M87" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N87" s="9" t="str">
+        <x:v>Not human-compatible medicine; contact/ingestion toxicity unresolved; Brittleness and shelf stability can distinguish it from a permanent binder</x:v>
+      </x:c>
+      <x:c r="O87" s="32"/>
+      <x:c r="P87" s="32"/>
+      <x:c r="Q87" s="32"/>
+      <x:c r="R87" s="32"/>
+      <x:c r="S87" s="32"/>
+      <x:c r="T87" s="9" t="str">
+        <x:v>Source draft describes mineral-hardened clots; repair-material use is new</x:v>
+      </x:c>
+      <x:c r="U87" s="33"/>
+      <x:c r="V87" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="80" customHeight="1">
+      <x:c r="A88" s="9" t="str">
+        <x:v>proposal.chemical.mineral_ichor</x:v>
+      </x:c>
+      <x:c r="B88" s="9" t="str">
+        <x:v>Mineral-rich ichor</x:v>
+      </x:c>
+      <x:c r="C88" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D88" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E88" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F88" s="9" t="str">
+        <x:v>Potential feed for pigments, recovered mineral fractions and binder research</x:v>
+      </x:c>
+      <x:c r="G88" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H88" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I88" s="13"/>
+      <x:c r="J88" s="15"/>
+      <x:c r="K88" s="9" t="str">
+        <x:v>Circulatory fluid carrying minerals, energy compounds and metabolic wastes</x:v>
+      </x:c>
+      <x:c r="L88" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M88" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N88" s="9" t="str">
+        <x:v>Species-dependent toxicity and mineral contamination; not drinkable by default; Mixed contents vary by diet; do not assume a universal reagent or battery electrolyte</x:v>
+      </x:c>
+      <x:c r="O88" s="32"/>
+      <x:c r="P88" s="32"/>
+      <x:c r="Q88" s="32"/>
+      <x:c r="R88" s="32"/>
+      <x:c r="S88" s="32"/>
+      <x:c r="T88" s="9" t="str">
+        <x:v>Ichor contents are source-draft biology; separated material uses are new proposals</x:v>
+      </x:c>
+      <x:c r="U88" s="33"/>
+      <x:c r="V88" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="80" customHeight="1">
+      <x:c r="A89" s="9" t="str">
+        <x:v>proposal.chemical.joint_lubricant</x:v>
+      </x:c>
+      <x:c r="B89" s="9" t="str">
+        <x:v>Joint-lubricating secretion</x:v>
+      </x:c>
+      <x:c r="C89" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D89" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E89" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F89" s="9" t="str">
+        <x:v>Dust-resistant equipment lubrication and flexible-seal conditioning</x:v>
+      </x:c>
+      <x:c r="G89" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H89" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I89" s="13"/>
+      <x:c r="J89" s="15"/>
+      <x:c r="K89" s="9" t="str">
+        <x:v>Proposed secretion that protects sliding plate/joint surfaces</x:v>
+      </x:c>
+      <x:c r="L89" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M89" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N89" s="9" t="str">
+        <x:v>Toxic if ingested; skin compatibility unapproved; Dust capture versus useful lubrication needs design; does not restore conventional fat anatomy</x:v>
+      </x:c>
+      <x:c r="O89" s="32"/>
+      <x:c r="P89" s="32"/>
+      <x:c r="Q89" s="32"/>
+      <x:c r="R89" s="32"/>
+      <x:c r="S89" s="32"/>
+      <x:c r="T89" s="9" t="str">
+        <x:v>New proposed secretion; source processing draft discusses biological oils without validating this anatomy</x:v>
+      </x:c>
+      <x:c r="U89" s="33"/>
+      <x:c r="V89" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="80" customHeight="1">
+      <x:c r="A90" s="9" t="str">
+        <x:v>proposal.chemical.insulating_secretion</x:v>
+      </x:c>
+      <x:c r="B90" s="9" t="str">
+        <x:v>Insulating secretion</x:v>
+      </x:c>
+      <x:c r="C90" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D90" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E90" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F90" s="9" t="str">
+        <x:v>Candidate electrical separators and equipment coating</x:v>
+      </x:c>
+      <x:c r="G90" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H90" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I90" s="13"/>
+      <x:c r="J90" s="15"/>
+      <x:c r="K90" s="9" t="str">
+        <x:v>Proposed barrier layer that helps fauna manage electrical exposure</x:v>
+      </x:c>
+      <x:c r="L90" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M90" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N90" s="9" t="str">
+        <x:v>Irritating/toxic residue; no human-contact assumption; Electrical behavior and wear are unproven; never blanket lightning immunity</x:v>
+      </x:c>
+      <x:c r="O90" s="32"/>
+      <x:c r="P90" s="32"/>
+      <x:c r="Q90" s="32"/>
+      <x:c r="R90" s="32"/>
+      <x:c r="S90" s="32"/>
+      <x:c r="T90" s="9" t="str">
+        <x:v>Source draft includes insulation/charge shedding; this material capability is a new proposal</x:v>
+      </x:c>
+      <x:c r="U90" s="33"/>
+      <x:c r="V90" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="80" customHeight="1">
+      <x:c r="A91" s="9" t="str">
+        <x:v>proposal.chemical.conductive_gel</x:v>
+      </x:c>
+      <x:c r="B91" s="9" t="str">
+        <x:v>Charge-conducting gel</x:v>
+      </x:c>
+      <x:c r="C91" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D91" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E91" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F91" s="9" t="str">
+        <x:v>Candidate contained equipment contacts and sensing components</x:v>
+      </x:c>
+      <x:c r="G91" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H91" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I91" s="13"/>
+      <x:c r="J91" s="15"/>
+      <x:c r="K91" s="9" t="str">
+        <x:v>Proposed contained medium supporting electroactive tissue</x:v>
+      </x:c>
+      <x:c r="L91" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M91" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N91" s="9" t="str">
+        <x:v>Contact could create an unwanted charge path; chemically toxic; Can worsen charge exposure; no direct body application or power generation assumed</x:v>
+      </x:c>
+      <x:c r="O91" s="32"/>
+      <x:c r="P91" s="32"/>
+      <x:c r="Q91" s="32"/>
+      <x:c r="R91" s="32"/>
+      <x:c r="S91" s="32"/>
+      <x:c r="T91" s="9" t="str">
+        <x:v>Source draft has electroactive fibers and conductive tissue; gel and applications are new proposals</x:v>
+      </x:c>
+      <x:c r="U91" s="33"/>
+      <x:c r="V91" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="80" customHeight="1">
+      <x:c r="A92" s="9" t="str">
+        <x:v>proposal.chemical.molt_release</x:v>
+      </x:c>
+      <x:c r="B92" s="9" t="str">
+        <x:v>Molt-release compound</x:v>
+      </x:c>
+      <x:c r="C92" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D92" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E92" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F92" s="9" t="str">
+        <x:v>Controlled plate-layer release and husk surface preparation</x:v>
+      </x:c>
+      <x:c r="G92" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H92" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I92" s="13"/>
+      <x:c r="J92" s="15"/>
+      <x:c r="K92" s="9" t="str">
+        <x:v>Proposed agent that separates old outer husk layers during renewal</x:v>
+      </x:c>
+      <x:c r="L92" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M92" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N92" s="9" t="str">
+        <x:v>Tissue/surface damage on contact; species-dependent; May spoil recovered fibers or structural plate; usefulness must differ from enzyme fraction</x:v>
+      </x:c>
+      <x:c r="O92" s="32"/>
+      <x:c r="P92" s="32"/>
+      <x:c r="Q92" s="32"/>
+      <x:c r="R92" s="32"/>
+      <x:c r="S92" s="32"/>
+      <x:c r="T92" s="9" t="str">
+        <x:v>New biological/material proposal; no specific molt chemistry established</x:v>
+      </x:c>
+      <x:c r="U92" s="33"/>
+      <x:c r="V92" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="80" customHeight="1">
+      <x:c r="A93" s="9" t="str">
+        <x:v>proposal.chemical.defensive_irritant</x:v>
+      </x:c>
+      <x:c r="B93" s="9" t="str">
+        <x:v>Defensive irritant secretion</x:v>
+      </x:c>
+      <x:c r="C93" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D93" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E93" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F93" s="9" t="str">
+        <x:v>Candidate exclusion coatings around equipment or stored materials</x:v>
+      </x:c>
+      <x:c r="G93" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H93" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I93" s="13"/>
+      <x:c r="J93" s="15"/>
+      <x:c r="K93" s="9" t="str">
+        <x:v>Proposed deterrent gland output in defensive species</x:v>
+      </x:c>
+      <x:c r="L93" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M93" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N93" s="9" t="str">
+        <x:v>Painful surface irritation and temporary sensory disruption; Repellent target response is unproven; deliberate containment only, no ambient liquid pools</x:v>
+      </x:c>
+      <x:c r="O93" s="32"/>
+      <x:c r="P93" s="32"/>
+      <x:c r="Q93" s="32"/>
+      <x:c r="R93" s="32"/>
+      <x:c r="S93" s="32"/>
+      <x:c r="T93" s="9" t="str">
+        <x:v>New toxin and application proposal; not assigned to any existing species</x:v>
+      </x:c>
+      <x:c r="U93" s="33"/>
+      <x:c r="V93" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="80" customHeight="1">
+      <x:c r="A94" s="9" t="str">
+        <x:v>proposal.chemical.disabling_venom</x:v>
+      </x:c>
+      <x:c r="B94" s="9" t="str">
+        <x:v>Disabling venom fraction</x:v>
+      </x:c>
+      <x:c r="C94" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D94" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E94" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F94" s="9" t="str">
+        <x:v>Candidate specialist trade/sample material for later design</x:v>
+      </x:c>
+      <x:c r="G94" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H94" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I94" s="13"/>
+      <x:c r="J94" s="15"/>
+      <x:c r="K94" s="9" t="str">
+        <x:v>Proposed specialized predator secretion for subduing native prey</x:v>
+      </x:c>
+      <x:c r="L94" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M94" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N94" s="9" t="str">
+        <x:v>Neurological disruption; human severity undefined; No human/animal potency equivalence, cure, delivery method or combat system established</x:v>
+      </x:c>
+      <x:c r="O94" s="32"/>
+      <x:c r="P94" s="32"/>
+      <x:c r="Q94" s="32"/>
+      <x:c r="R94" s="32"/>
+      <x:c r="S94" s="32"/>
+      <x:c r="T94" s="9" t="str">
+        <x:v>New proposal; source predation does not establish a specific venom</x:v>
+      </x:c>
+      <x:c r="U94" s="33"/>
+      <x:c r="V94" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="80" customHeight="1">
+      <x:c r="A95" s="9" t="str">
+        <x:v>proposal.chemical.scent_marker</x:v>
+      </x:c>
+      <x:c r="B95" s="9" t="str">
+        <x:v>Chemical scent marker</x:v>
+      </x:c>
+      <x:c r="C95" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D95" s="9" t="str">
+        <x:v>Faunal chemical concept</x:v>
+      </x:c>
+      <x:c r="E95" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F95" s="9" t="str">
+        <x:v>Possible lure, trail concealment or animal-avoidance research</x:v>
+      </x:c>
+      <x:c r="G95" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H95" s="9" t="str">
+        <x:v>Contained Legger/local storage proposed</x:v>
+      </x:c>
+      <x:c r="I95" s="13"/>
+      <x:c r="J95" s="15"/>
+      <x:c r="K95" s="9" t="str">
+        <x:v>Proposed territorial or social signal secretion</x:v>
+      </x:c>
+      <x:c r="L95" s="9" t="str">
+        <x:v>Qualitative material concept; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M95" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N95" s="9" t="str">
+        <x:v>Irritant or toxic to humans despite its signaling role; Species-specific response; a signal may attract unwanted animals rather than repel them</x:v>
+      </x:c>
+      <x:c r="O95" s="32"/>
+      <x:c r="P95" s="32"/>
+      <x:c r="Q95" s="32"/>
+      <x:c r="R95" s="32"/>
+      <x:c r="S95" s="32"/>
+      <x:c r="T95" s="9" t="str">
+        <x:v>New proposal; no accepted behavioral response or universal bait chemistry</x:v>
+      </x:c>
+      <x:c r="U95" s="33"/>
+      <x:c r="V95" s="9" t="str">
+        <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
@@ -4947,6 +5625,9 @@
   <x:conditionalFormatting sqref="E56:E74">
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="proposal"/>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E84:E95">
+    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="proposal"/>
+  </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C6:C23">
       <x:formula1>"Equipment,Field supplies,Resources,Crafting components,Weapons,Ammunition,Quest items,Trade goods"</x:formula1>
@@ -4954,7 +5635,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raee8f2a624b741db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d0940bd6efa40df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5862,7 +6543,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c3c910994ce471b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb0ca6f067fa48d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6228,7 +6909,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a17e9ab66f4ff0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5adb5314a14c4b0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6319,13 +7000,13 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>53</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Existing resources plus proposed minerals, biological materials and unspecified fauna chemistry</x:v>
+        <x:v>Minerals, biological resources, generic chemistry placeholders and twelve new chemical concepts</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Some fauna edible but poorly nutritious; most internal chemistry toxic; species/uses unresolved</x:v>
+        <x:v>Some concepts may merge: etchant/enzyme/molt agent, or binder/clot compound. No new canon.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -6430,7 +7111,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0f0d4a67f5e4a0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree1e5780f5884b8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6493,7 +7174,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>78 design entries: 18 existing item IDs and 60 design concepts. Generic fauna chemistry/food placeholders are not named species, chemicals or implemented items.</x:v>
+        <x:v>90 design entries: 18 existing item IDs and 72 design concepts. Twelve named chemical concepts are new brainstorming proposals; three earlier generic fauna food/chemistry placeholders remain grouping candidates.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -6808,10 +7489,50 @@
         <x:v>Native biology, domestic burden beetle and chitin/Phagia material records are proposals. Their woven textile assumptions conflict with newer game no-cloth direction. No source species or recipes adopted.</x:v>
       </x:c>
     </x:row>
+    <x:row r="48" ht="65" customHeight="1">
+      <x:c r="A48" s="4" t="str">
+        <x:v>Chemical concepts</x:v>
+      </x:c>
+      <x:c r="B48" s="4" t="str">
+        <x:v>Twelve descriptive working labels explore biology, human hazard and possible material use. No new species, chemical identities, numerical effects or recipes are accepted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="65" customHeight="1">
+      <x:c r="A49" s="4" t="str">
+        <x:v>Draft versus invention</x:v>
+      </x:c>
+      <x:c r="B49" s="4" t="str">
+        <x:v>Reference column identifies source-draft biology and processing seeds. The Source relationship column states which abilities or uses were invented for this brainstorm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="65" customHeight="1">
+      <x:c r="A50" s="4" t="str">
+        <x:v>Useful does not mean edible</x:v>
+      </x:c>
+      <x:c r="B50" s="4" t="str">
+        <x:v>Toxicity, nutrition and industrial usefulness remain separate. No candidate replaces algae or becomes a drink/medicine by default.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="65" customHeight="1">
+      <x:c r="A51" s="4" t="str">
+        <x:v>Scarce workshop skill</x:v>
+      </x:c>
+      <x:c r="B51" s="4" t="str">
+        <x:v>Husk-fiber processing remains very difficult and hide/fur output extremely low. Enzyme/binder concepts do not create cloth or bypass processing costs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="65" customHeight="1">
+      <x:c r="A52" s="4" t="str">
+        <x:v>Contained chemicals</x:v>
+      </x:c>
+      <x:c r="B52" s="4" t="str">
+        <x:v>Liquid candidates require deliberate containment. Native liquid landscapes, real synthesis procedures and harvesting/weapon delivery rules are not introduced.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d1990e4a9cd41ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16ab484d720e473f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7655,7 +8376,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5eedab1f81d447e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58961db48a024f27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7898,7 +8619,411 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd36be8b266d046e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39fba1ca96dd4540"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="55" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="72" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="110" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Faunal chemicals and toxins</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="1" t="str">
+        <x:v>New game proposals. Descriptive labels; no accepted chemical identities, species assignments, recipes or numeric effects.</x:v>
+      </x:c>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="35" customHeight="1">
+      <x:c r="A5" s="35" t="str">
+        <x:v>Concept ID</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="str">
+        <x:v>Working label</x:v>
+      </x:c>
+      <x:c r="C5" s="35" t="str">
+        <x:v>Biological source / role</x:v>
+      </x:c>
+      <x:c r="D5" s="35" t="str">
+        <x:v>Human hazard</x:v>
+      </x:c>
+      <x:c r="E5" s="35" t="str">
+        <x:v>Potential material use</x:v>
+      </x:c>
+      <x:c r="F5" s="35" t="str">
+        <x:v>Design constraint</x:v>
+      </x:c>
+      <x:c r="G5" s="35" t="str">
+        <x:v>Source relationship</x:v>
+      </x:c>
+      <x:c r="H5" s="35" t="str">
+        <x:v>Reference</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="75" customHeight="1">
+      <x:c r="A6" s="4" t="str">
+        <x:v>proposal.chemical.digestive_etchant</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>Digestive etchant</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>Contained digestive liquor in geological feeders; exposes useful mineral compounds</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>Corrosive tissue injury; inedible</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>Mineral separation and metal surface preparation</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>Could damage containers and useful shell; reusable containment and selectivity need design</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="str">
+        <x:v>Source draft describes digestive acids/catalysts; this harvestable agent and uses are new proposals</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="75" customHeight="1">
+      <x:c r="A7" s="4" t="str">
+        <x:v>proposal.chemical.husk_enzyme</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>Husk-separation enzyme</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>Proposed catalytic fraction associated with shell renewal or digestion</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>Biologically active irritant; effects species-dependent</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>Help release chitin/icore fibers for paper and difficult pressed materials</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>Slow specialist processing still required; must not turn abundant husks into easy cloth</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="str">
+        <x:v>Source draft includes industrial enzymes, but fauna origin and this fiber application are new proposals</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="75" customHeight="1">
+      <x:c r="A8" s="4" t="str">
+        <x:v>proposal.chemical.shell_binder</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>Shell-binding secretion</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>Proposed armor-building secretion that binds deposited minerals</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>Adheres to exposed surfaces; contaminated residue may be toxic</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>Bind mineral aggregate, shell laminates and pressed fiber materials</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>Durable bonding is a proposal; curing conditions and unwanted adhesion remain unresolved</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="str">
+        <x:v>Armor-building organs and chitin-derived binders are source-draft seeds; secretion/product is new</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="75" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>proposal.chemical.clotting_compound</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>Mineral clotting compound</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>Ichor wound response; suspended minerals harden into a protective clot</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Not human-compatible medicine; contact/ingestion toxicity unresolved</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Quick hard-setting equipment patches and temporary container seals</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>Brittleness and shelf stability can distinguish it from a permanent binder</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="str">
+        <x:v>Source draft describes mineral-hardened clots; repair-material use is new</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="75" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>proposal.chemical.mineral_ichor</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>Mineral-rich ichor</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>Circulatory fluid carrying minerals, energy compounds and metabolic wastes</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Species-dependent toxicity and mineral contamination; not drinkable by default</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>Potential feed for pigments, recovered mineral fractions and binder research</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>Mixed contents vary by diet; do not assume a universal reagent or battery electrolyte</x:v>
+      </x:c>
+      <x:c r="G10" s="4" t="str">
+        <x:v>Ichor contents are source-draft biology; separated material uses are new proposals</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="75" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>proposal.chemical.joint_lubricant</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>Joint-lubricating secretion</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>Proposed secretion that protects sliding plate/joint surfaces</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>Toxic if ingested; skin compatibility unapproved</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>Dust-resistant equipment lubrication and flexible-seal conditioning</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>Dust capture versus useful lubrication needs design; does not restore conventional fat anatomy</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str">
+        <x:v>New proposed secretion; source processing draft discusses biological oils without validating this anatomy</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="75" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>proposal.chemical.insulating_secretion</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>Insulating secretion</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>Proposed barrier layer that helps fauna manage electrical exposure</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>Irritating/toxic residue; no human-contact assumption</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>Candidate electrical separators and equipment coating</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>Electrical behavior and wear are unproven; never blanket lightning immunity</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="str">
+        <x:v>Source draft includes insulation/charge shedding; this material capability is a new proposal</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="75" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>proposal.chemical.conductive_gel</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>Charge-conducting gel</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>Proposed contained medium supporting electroactive tissue</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Contact could create an unwanted charge path; chemically toxic</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>Candidate contained equipment contacts and sensing components</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>Can worsen charge exposure; no direct body application or power generation assumed</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>Source draft has electroactive fibers and conductive tissue; gel and applications are new proposals</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="75" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>proposal.chemical.molt_release</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>Molt-release compound</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>Proposed agent that separates old outer husk layers during renewal</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>Tissue/surface damage on contact; species-dependent</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>Controlled plate-layer release and husk surface preparation</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>May spoil recovered fibers or structural plate; usefulness must differ from enzyme fraction</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="str">
+        <x:v>New biological/material proposal; no specific molt chemistry established</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="75" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>proposal.chemical.defensive_irritant</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>Defensive irritant secretion</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>Proposed deterrent gland output in defensive species</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Painful surface irritation and temporary sensory disruption</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>Candidate exclusion coatings around equipment or stored materials</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>Repellent target response is unproven; deliberate containment only, no ambient liquid pools</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>New toxin and application proposal; not assigned to any existing species</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="75" customHeight="1">
+      <x:c r="A16" s="4" t="str">
+        <x:v>proposal.chemical.disabling_venom</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>Disabling venom fraction</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>Proposed specialized predator secretion for subduing native prey</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Neurological disruption; human severity undefined</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>Candidate specialist trade/sample material for later design</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>No human/animal potency equivalence, cure, delivery method or combat system established</x:v>
+      </x:c>
+      <x:c r="G16" s="4" t="str">
+        <x:v>New proposal; source predation does not establish a specific venom</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="75" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>proposal.chemical.scent_marker</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>Chemical scent marker</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>Proposed territorial or social signal secretion</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Irritant or toxic to humans despite its signaling role</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Possible lure, trail concealment or animal-avoidance research</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>Species-specific response; a signal may attract unwanted animals rather than repel them</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>New proposal; no accepted behavioral response or universal bait chemistry</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9990cc1ee1b5413d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Brainstorm liquid containers cargo cases and transfer glassware
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R5173927b2edb4801"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Radc4e641995c4637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R0fbdf3504da74c0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R96ab48cee52848b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Re3bf5b8362b14df7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rf7d84e54c2294f04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R50822fd1223d4609"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Rca82e73cd2f24217"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R25769ec2bf91410b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rf57a656733944a7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rbabdf7f2634e421a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R3e477107a9c242cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R4d9b2650177a496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R0e69858b132a4bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Ra5040fb927254a93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R5a1123767d044a6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Ra41986f3017e4d0c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -53,7 +54,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -140,6 +141,21 @@
         <x:fgColor rgb="FF423B35"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF423B35"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -153,7 +169,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="42">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -275,6 +291,24 @@
     <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -337,7 +371,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V95" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V111" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -405,7 +439,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -417,7 +451,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -470,6 +504,25 @@
     <x:tableColumn id="6" name="Design constraint"/>
     <x:tableColumn id="7" name="Source relationship"/>
     <x:tableColumn id="8" name="Reference"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ContainerConceptsTable" displayName="ContainerConceptsTable" ref="A5:K21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Concept ID"/>
+    <x:tableColumn id="2" name="Working label"/>
+    <x:tableColumn id="3" name="Form"/>
+    <x:tableColumn id="4" name="Proposed materials"/>
+    <x:tableColumn id="5" name="Purpose"/>
+    <x:tableColumn id="6" name="Qualitative size"/>
+    <x:tableColumn id="7" name="Closure concept"/>
+    <x:tableColumn id="8" name="Contents / contact"/>
+    <x:tableColumn id="9" name="Design constraint"/>
+    <x:tableColumn id="10" name="Source relationship"/>
+    <x:tableColumn id="11" name="References"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -5615,6 +5668,838 @@
         <x:v>New game brainstorm, October 14, 2026; source records are proposals. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/native-fauna-biology.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="96" ht="100" customHeight="1">
+      <x:c r="A96" s="9" t="str">
+        <x:v>proposal.container.sample_vial</x:v>
+      </x:c>
+      <x:c r="B96" s="9" t="str">
+        <x:v>Clear sample vial</x:v>
+      </x:c>
+      <x:c r="C96" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D96" s="9" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="E96" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F96" s="9" t="str">
+        <x:v>Inspect a small ichor or chemical sample without opening it</x:v>
+      </x:c>
+      <x:c r="G96" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H96" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I96" s="13"/>
+      <x:c r="J96" s="15"/>
+      <x:c r="K96" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L96" s="9" t="str">
+        <x:v>Materials: Scarce clear glass</x:v>
+      </x:c>
+      <x:c r="M96" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N96" s="9" t="str">
+        <x:v>Clear glass cost; liquid compatibility and fill limit unapproved</x:v>
+      </x:c>
+      <x:c r="O96" s="36"/>
+      <x:c r="P96" s="36"/>
+      <x:c r="Q96" s="36"/>
+      <x:c r="R96" s="36"/>
+      <x:c r="S96" s="36"/>
+      <x:c r="T96" s="9" t="str">
+        <x:v>Qualitative size: Small sample. Closure: Matched stopper with retained cover proposed. Contents: Species-tagged ichor; compatible chemical samples</x:v>
+      </x:c>
+      <x:c r="U96" s="37"/>
+      <x:c r="V96" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. Glass draft supports costly transparent material; this vessel is a new proposal. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="100" customHeight="1">
+      <x:c r="A97" s="9" t="str">
+        <x:v>proposal.container.reagent_bottle</x:v>
+      </x:c>
+      <x:c r="B97" s="9" t="str">
+        <x:v>Opaque reagent bottle</x:v>
+      </x:c>
+      <x:c r="C97" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D97" s="9" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="E97" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F97" s="9" t="str">
+        <x:v>Everyday transport of one known material</x:v>
+      </x:c>
+      <x:c r="G97" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H97" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I97" s="13"/>
+      <x:c r="J97" s="15"/>
+      <x:c r="K97" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L97" s="9" t="str">
+        <x:v>Materials: Opaque mineral glass; shell/metal cap</x:v>
+      </x:c>
+      <x:c r="M97" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N97" s="9" t="str">
+        <x:v>Cannot inspect contents through the wall; external identity label matters</x:v>
+      </x:c>
+      <x:c r="O97" s="36"/>
+      <x:c r="P97" s="36"/>
+      <x:c r="Q97" s="36"/>
+      <x:c r="R97" s="36"/>
+      <x:c r="S97" s="36"/>
+      <x:c r="T97" s="9" t="str">
+        <x:v>Qualitative size: Hand-sized. Closure: Compression cap and compatible seat proposed. Contents: One identified ichor or reagent batch</x:v>
+      </x:c>
+      <x:c r="U97" s="37"/>
+      <x:c r="V97" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. Standard opaque glass vessels have a source-draft basis; exact item new. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="100" customHeight="1">
+      <x:c r="A98" s="9" t="str">
+        <x:v>proposal.container.wide_jar</x:v>
+      </x:c>
+      <x:c r="B98" s="9" t="str">
+        <x:v>Wide-mouth sample jar</x:v>
+      </x:c>
+      <x:c r="C98" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D98" s="9" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="E98" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F98" s="9" t="str">
+        <x:v>Carry thick gels, clot samples and mineral-rich slurry</x:v>
+      </x:c>
+      <x:c r="G98" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H98" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I98" s="13"/>
+      <x:c r="J98" s="15"/>
+      <x:c r="K98" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L98" s="9" t="str">
+        <x:v>Materials: Glass body; rigid broad lid</x:v>
+      </x:c>
+      <x:c r="M98" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N98" s="9" t="str">
+        <x:v>Wide opening aids access but makes transfers less controlled; no scoop rules set</x:v>
+      </x:c>
+      <x:c r="O98" s="36"/>
+      <x:c r="P98" s="36"/>
+      <x:c r="Q98" s="36"/>
+      <x:c r="R98" s="36"/>
+      <x:c r="S98" s="36"/>
+      <x:c r="T98" s="9" t="str">
+        <x:v>Qualitative size: Small to medium. Closure: Broad fitted lid with compatible sealing seat. Contents: Viscous material or solid/liquid sample</x:v>
+      </x:c>
+      <x:c r="U98" s="37"/>
+      <x:c r="V98" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. Glass vessel basis; wide-mouth item and uses proposed. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="100" customHeight="1">
+      <x:c r="A99" s="9" t="str">
+        <x:v>proposal.container.ampoule</x:v>
+      </x:c>
+      <x:c r="B99" s="9" t="str">
+        <x:v>Sealed sample ampoule</x:v>
+      </x:c>
+      <x:c r="C99" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D99" s="9" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="E99" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F99" s="9" t="str">
+        <x:v>Preserve an isolated small specimen for later analysis or trade</x:v>
+      </x:c>
+      <x:c r="G99" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H99" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I99" s="13"/>
+      <x:c r="J99" s="15"/>
+      <x:c r="K99" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L99" s="9" t="str">
+        <x:v>Materials: Sealed clear glass</x:v>
+      </x:c>
+      <x:c r="M99" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N99" s="9" t="str">
+        <x:v>Opening and reuse undecided; no mandatory single-use depletion rule approved</x:v>
+      </x:c>
+      <x:c r="O99" s="36"/>
+      <x:c r="P99" s="36"/>
+      <x:c r="Q99" s="36"/>
+      <x:c r="R99" s="36"/>
+      <x:c r="S99" s="36"/>
+      <x:c r="T99" s="9" t="str">
+        <x:v>Qualitative size: Very small. Closure: Factory/workshop sealed. Contents: One specimen; chemistry compatibility unresolved</x:v>
+      </x:c>
+      <x:c r="U99" s="37"/>
+      <x:c r="V99" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New sealed-glass form inspired by source glasswork. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="100" customHeight="1">
+      <x:c r="A100" s="9" t="str">
+        <x:v>proposal.container.marked_flask</x:v>
+      </x:c>
+      <x:c r="B100" s="9" t="str">
+        <x:v>Marked glass flask</x:v>
+      </x:c>
+      <x:c r="C100" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D100" s="9" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="E100" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F100" s="9" t="str">
+        <x:v>Read fill and compare a specimen before transfer</x:v>
+      </x:c>
+      <x:c r="G100" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H100" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I100" s="13"/>
+      <x:c r="J100" s="15"/>
+      <x:c r="K100" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L100" s="9" t="str">
+        <x:v>Materials: Clear glass with etched marks</x:v>
+      </x:c>
+      <x:c r="M100" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N100" s="9" t="str">
+        <x:v>Marks do not establish numeric volume, chemistry analysis or automatic quality grading</x:v>
+      </x:c>
+      <x:c r="O100" s="36"/>
+      <x:c r="P100" s="36"/>
+      <x:c r="Q100" s="36"/>
+      <x:c r="R100" s="36"/>
+      <x:c r="S100" s="36"/>
+      <x:c r="T100" s="9" t="str">
+        <x:v>Qualitative size: Small sample / workshop. Closure: Matched stopper proposed. Contents: Compatible samples and liquids</x:v>
+      </x:c>
+      <x:c r="U100" s="37"/>
+      <x:c r="V100" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New measuring/inspection use; no authored volume system. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="100" customHeight="1">
+      <x:c r="A101" s="9" t="str">
+        <x:v>proposal.container.shell_cage</x:v>
+      </x:c>
+      <x:c r="B101" s="9" t="str">
+        <x:v>Shell-caged glass flask</x:v>
+      </x:c>
+      <x:c r="C101" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D101" s="9" t="str">
+        <x:v>Protected vessel assembly</x:v>
+      </x:c>
+      <x:c r="E101" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F101" s="9" t="str">
+        <x:v>Protect a carried specimen while keeping a viewing opening</x:v>
+      </x:c>
+      <x:c r="G101" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H101" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I101" s="13"/>
+      <x:c r="J101" s="15"/>
+      <x:c r="K101" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L101" s="9" t="str">
+        <x:v>Materials: Glass inner vessel; slotted shell outer cage</x:v>
+      </x:c>
+      <x:c r="M101" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N101" s="9" t="str">
+        <x:v>One assembled container, not two copies of storage; protection behavior undecided</x:v>
+      </x:c>
+      <x:c r="O101" s="36"/>
+      <x:c r="P101" s="36"/>
+      <x:c r="Q101" s="36"/>
+      <x:c r="R101" s="36"/>
+      <x:c r="S101" s="36"/>
+      <x:c r="T101" s="9" t="str">
+        <x:v>Qualitative size: Medium. Closure: Retained cap and inspectable seat proposed. Contents: One compatible liquid payload</x:v>
+      </x:c>
+      <x:c r="U101" s="37"/>
+      <x:c r="V101" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. Chitin plate/curved vessel and glass drafts inspire assembly; item new. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="100" customHeight="1">
+      <x:c r="A102" s="9" t="str">
+        <x:v>proposal.container.lined_canister</x:v>
+      </x:c>
+      <x:c r="B102" s="9" t="str">
+        <x:v>Glass-lined haul canister</x:v>
+      </x:c>
+      <x:c r="C102" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D102" s="9" t="str">
+        <x:v>Protected vessel assembly</x:v>
+      </x:c>
+      <x:c r="E102" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F102" s="9" t="str">
+        <x:v>Transport larger quantities to a processing workshop</x:v>
+      </x:c>
+      <x:c r="G102" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H102" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I102" s="13"/>
+      <x:c r="J102" s="15"/>
+      <x:c r="K102" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L102" s="9" t="str">
+        <x:v>Materials: Metal/shell outer body; replaceable glass liner</x:v>
+      </x:c>
+      <x:c r="M102" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N102" s="9" t="str">
+        <x:v>Liner, seal and contents must all be compatible; filled payload belongs in resource cargo</x:v>
+      </x:c>
+      <x:c r="O102" s="36"/>
+      <x:c r="P102" s="36"/>
+      <x:c r="Q102" s="36"/>
+      <x:c r="R102" s="36"/>
+      <x:c r="S102" s="36"/>
+      <x:c r="T102" s="9" t="str">
+        <x:v>Qualitative size: Medium haul. Closure: Compression lid with replaceable compatible seat. Contents: One identified raw ichor or chemical batch</x:v>
+      </x:c>
+      <x:c r="U102" s="37"/>
+      <x:c r="V102" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. Glass draft includes internal canister linings; haul role and item new. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="100" customHeight="1">
+      <x:c r="A103" s="9" t="str">
+        <x:v>proposal.container.ceramic_jar</x:v>
+      </x:c>
+      <x:c r="B103" s="9" t="str">
+        <x:v>Glazed ceramic reagent jar</x:v>
+      </x:c>
+      <x:c r="C103" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D103" s="9" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="E103" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F103" s="9" t="str">
+        <x:v>Alternative storage for selected processing compounds</x:v>
+      </x:c>
+      <x:c r="G103" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H103" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I103" s="13"/>
+      <x:c r="J103" s="15"/>
+      <x:c r="K103" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L103" s="9" t="str">
+        <x:v>Materials: Fired ceramic; proposed glaze; rigid lid</x:v>
+      </x:c>
+      <x:c r="M103" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N103" s="9" t="str">
+        <x:v>Opaque; heavier/bulkier tradeoff proposed; glaze is not universally chemical-resistant</x:v>
+      </x:c>
+      <x:c r="O103" s="36"/>
+      <x:c r="P103" s="36"/>
+      <x:c r="Q103" s="36"/>
+      <x:c r="R103" s="36"/>
+      <x:c r="S103" s="36"/>
+      <x:c r="T103" s="9" t="str">
+        <x:v>Qualitative size: Medium. Closure: Fitted rigid lid and compatible seal. Contents: Only compounds qualified for that jar</x:v>
+      </x:c>
+      <x:c r="U103" s="37"/>
+      <x:c r="V103" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New ceramic vessel proposal; not a validated recipe/material capability. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="100" customHeight="1">
+      <x:c r="A104" s="9" t="str">
+        <x:v>proposal.container.bulk_ichor</x:v>
+      </x:c>
+      <x:c r="B104" s="9" t="str">
+        <x:v>Bulk ichor vessel</x:v>
+      </x:c>
+      <x:c r="C104" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D104" s="9" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="E104" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F104" s="9" t="str">
+        <x:v>Make a large harvest an expedition haul decision</x:v>
+      </x:c>
+      <x:c r="G104" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H104" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I104" s="13"/>
+      <x:c r="J104" s="15"/>
+      <x:c r="K104" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L104" s="9" t="str">
+        <x:v>Materials: Reinforced outer body; qualified inner lining TBD</x:v>
+      </x:c>
+      <x:c r="M104" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N104" s="9" t="str">
+        <x:v>Finite Legger cargo and contents mass; no backpack resource exception or free capacity</x:v>
+      </x:c>
+      <x:c r="O104" s="36"/>
+      <x:c r="P104" s="36"/>
+      <x:c r="Q104" s="36"/>
+      <x:c r="R104" s="36"/>
+      <x:c r="S104" s="36"/>
+      <x:c r="T104" s="9" t="str">
+        <x:v>Qualitative size: Bulk cargo. Closure: Service lid and separate transfer fitting proposed. Contents: One species/batch of gathered ichor</x:v>
+      </x:c>
+      <x:c r="U104" s="37"/>
+      <x:c r="V104" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New bulk vessel proposal; no liter capacity, hose or extraction mechanic approved. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="100" customHeight="1">
+      <x:c r="A105" s="9" t="str">
+        <x:v>proposal.container.vial_case</x:v>
+      </x:c>
+      <x:c r="B105" s="9" t="str">
+        <x:v>Divided vial case</x:v>
+      </x:c>
+      <x:c r="C105" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D105" s="9" t="str">
+        <x:v>Protective carrier</x:v>
+      </x:c>
+      <x:c r="E105" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F105" s="9" t="str">
+        <x:v>Keep separately sealed specimens organized and supported</x:v>
+      </x:c>
+      <x:c r="G105" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H105" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I105" s="13"/>
+      <x:c r="J105" s="15"/>
+      <x:c r="K105" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L105" s="9" t="str">
+        <x:v>Materials: Shell/metal case; shaped mineral seats</x:v>
+      </x:c>
+      <x:c r="M105" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N105" s="9" t="str">
+        <x:v>Does not create extra inventory capacity; inserts use no assumed wood, cork or cloth</x:v>
+      </x:c>
+      <x:c r="O105" s="36"/>
+      <x:c r="P105" s="36"/>
+      <x:c r="Q105" s="36"/>
+      <x:c r="R105" s="36"/>
+      <x:c r="S105" s="36"/>
+      <x:c r="T105" s="9" t="str">
+        <x:v>Qualitative size: Several small vessels. Closure: Rigid latched case; each vial has its own seal. Contents: Sealed vials only; no direct liquid payload</x:v>
+      </x:c>
+      <x:c r="U105" s="37"/>
+      <x:c r="V105" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New case proposal; materials chosen under current no-cloth game rule. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="100" customHeight="1">
+      <x:c r="A106" s="9" t="str">
+        <x:v>proposal.container.sealed_box</x:v>
+      </x:c>
+      <x:c r="B106" s="9" t="str">
+        <x:v>Sealed cargo box</x:v>
+      </x:c>
+      <x:c r="C106" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D106" s="9" t="str">
+        <x:v>Protective carrier</x:v>
+      </x:c>
+      <x:c r="E106" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F106" s="9" t="str">
+        <x:v>Carry containers and dry sample packets together</x:v>
+      </x:c>
+      <x:c r="G106" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H106" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I106" s="13"/>
+      <x:c r="J106" s="15"/>
+      <x:c r="K106" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L106" s="9" t="str">
+        <x:v>Materials: Shell panels or metal; rigid dividers</x:v>
+      </x:c>
+      <x:c r="M106" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N106" s="9" t="str">
+        <x:v>Outer dust seal is not liquid or vapor certification; all nested contents still count</x:v>
+      </x:c>
+      <x:c r="O106" s="36"/>
+      <x:c r="P106" s="36"/>
+      <x:c r="Q106" s="36"/>
+      <x:c r="R106" s="36"/>
+      <x:c r="S106" s="36"/>
+      <x:c r="T106" s="9" t="str">
+        <x:v>Qualitative size: Cargo package. Closure: Latched lid with dust-excluding seat proposed. Contents: Separately sealed contents</x:v>
+      </x:c>
+      <x:c r="U106" s="37"/>
+      <x:c r="V106" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New protective box proposal; not automatic liquid containment. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="100" customHeight="1">
+      <x:c r="A107" s="9" t="str">
+        <x:v>proposal.container.field_chest</x:v>
+      </x:c>
+      <x:c r="B107" s="9" t="str">
+        <x:v>Locking field chest</x:v>
+      </x:c>
+      <x:c r="C107" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D107" s="9" t="str">
+        <x:v>Storage object candidate</x:v>
+      </x:c>
+      <x:c r="E107" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F107" s="9" t="str">
+        <x:v>Secure expedition samples at a physical camp/worksite</x:v>
+      </x:c>
+      <x:c r="G107" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H107" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I107" s="13"/>
+      <x:c r="J107" s="15"/>
+      <x:c r="K107" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L107" s="9" t="str">
+        <x:v>Materials: Metal/shell chest; rigid compartment tray</x:v>
+      </x:c>
+      <x:c r="M107" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N107" s="9" t="str">
+        <x:v>Physical local owner; no global stockpile. Portable versus fixed identity undecided</x:v>
+      </x:c>
+      <x:c r="O107" s="36"/>
+      <x:c r="P107" s="36"/>
+      <x:c r="Q107" s="36"/>
+      <x:c r="R107" s="36"/>
+      <x:c r="S107" s="36"/>
+      <x:c r="T107" s="9" t="str">
+        <x:v>Qualitative size: Local storage. Closure: Mechanical lock and rigid lid proposed. Contents: Sealed vessels and dry material</x:v>
+      </x:c>
+      <x:c r="U107" s="37"/>
+      <x:c r="V107" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New storage-object candidate; not another implemented camp chest. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="100" customHeight="1">
+      <x:c r="A108" s="9" t="str">
+        <x:v>proposal.container.funnel</x:v>
+      </x:c>
+      <x:c r="B108" s="9" t="str">
+        <x:v>Glass transfer funnel</x:v>
+      </x:c>
+      <x:c r="C108" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D108" s="9" t="str">
+        <x:v>Transfer glassware</x:v>
+      </x:c>
+      <x:c r="E108" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F108" s="9" t="str">
+        <x:v>Assist transfers into a compatible narrow-neck vessel</x:v>
+      </x:c>
+      <x:c r="G108" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H108" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I108" s="13"/>
+      <x:c r="J108" s="15"/>
+      <x:c r="K108" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L108" s="9" t="str">
+        <x:v>Materials: Glass bowl and stem</x:v>
+      </x:c>
+      <x:c r="M108" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N108" s="9" t="str">
+        <x:v>Residue/cross-contamination and workshop reconditioning unresolved; no ambient fluid pooling</x:v>
+      </x:c>
+      <x:c r="O108" s="36"/>
+      <x:c r="P108" s="36"/>
+      <x:c r="Q108" s="36"/>
+      <x:c r="R108" s="36"/>
+      <x:c r="S108" s="36"/>
+      <x:c r="T108" s="9" t="str">
+        <x:v>Qualitative size: Tool-sized. Closure: No closure; never a storage vessel. Contents: Temporary transfer contact only</x:v>
+      </x:c>
+      <x:c r="U108" s="37"/>
+      <x:c r="V108" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New glassworking tool proposal. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="100" customHeight="1">
+      <x:c r="A109" s="9" t="str">
+        <x:v>proposal.container.draw_tube</x:v>
+      </x:c>
+      <x:c r="B109" s="9" t="str">
+        <x:v>Glass draw tube</x:v>
+      </x:c>
+      <x:c r="C109" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D109" s="9" t="str">
+        <x:v>Transfer glassware</x:v>
+      </x:c>
+      <x:c r="E109" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F109" s="9" t="str">
+        <x:v>Move a small sample through an inspectable transfer path</x:v>
+      </x:c>
+      <x:c r="G109" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H109" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I109" s="13"/>
+      <x:c r="J109" s="15"/>
+      <x:c r="K109" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L109" s="9" t="str">
+        <x:v>Materials: Glass tube; proposed mechanical fitting</x:v>
+      </x:c>
+      <x:c r="M109" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N109" s="9" t="str">
+        <x:v>No mouth operation or real extraction procedure; gameplay tool and fittings unapproved</x:v>
+      </x:c>
+      <x:c r="O109" s="36"/>
+      <x:c r="P109" s="36"/>
+      <x:c r="Q109" s="36"/>
+      <x:c r="R109" s="36"/>
+      <x:c r="S109" s="36"/>
+      <x:c r="T109" s="9" t="str">
+        <x:v>Qualitative size: Tool-sized. Closure: Closed mechanical interface to design. Contents: Compatible small specimen transfer</x:v>
+      </x:c>
+      <x:c r="U109" s="37"/>
+      <x:c r="V109" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New mechanical sample-transfer tool proposal. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="100" customHeight="1">
+      <x:c r="A110" s="9" t="str">
+        <x:v>proposal.container.glass_stopper</x:v>
+      </x:c>
+      <x:c r="B110" s="9" t="str">
+        <x:v>Matched glass stopper</x:v>
+      </x:c>
+      <x:c r="C110" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D110" s="9" t="str">
+        <x:v>Closure component</x:v>
+      </x:c>
+      <x:c r="E110" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F110" s="9" t="str">
+        <x:v>Close its matching vessel without cork or cloth</x:v>
+      </x:c>
+      <x:c r="G110" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H110" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I110" s="13"/>
+      <x:c r="J110" s="15"/>
+      <x:c r="K110" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L110" s="9" t="str">
+        <x:v>Materials: Ground glass seat; retaining clip optional</x:v>
+      </x:c>
+      <x:c r="M110" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N110" s="9" t="str">
+        <x:v>Fit and material compatibility matter; no universal stopper or separate durability chore assumed</x:v>
+      </x:c>
+      <x:c r="O110" s="36"/>
+      <x:c r="P110" s="36"/>
+      <x:c r="Q110" s="36"/>
+      <x:c r="R110" s="36"/>
+      <x:c r="S110" s="36"/>
+      <x:c r="T110" s="9" t="str">
+        <x:v>Qualitative size: Part-sized. Closure: Matched seat. Contents: Vessel closure, not an independent payload</x:v>
+      </x:c>
+      <x:c r="U110" s="37"/>
+      <x:c r="V110" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New glass closure component proposal. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="100" customHeight="1">
+      <x:c r="A111" s="9" t="str">
+        <x:v>proposal.container.seal_collar</x:v>
+      </x:c>
+      <x:c r="B111" s="9" t="str">
+        <x:v>Compression seal collar</x:v>
+      </x:c>
+      <x:c r="C111" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D111" s="9" t="str">
+        <x:v>Closure component</x:v>
+      </x:c>
+      <x:c r="E111" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F111" s="9" t="str">
+        <x:v>Retain and compress a vessel lid/seat</x:v>
+      </x:c>
+      <x:c r="G111" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H111" s="9" t="str">
+        <x:v>Filled raw-resource vessel: Legger/local owner; other carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I111" s="13"/>
+      <x:c r="J111" s="15"/>
+      <x:c r="K111" s="9" t="str">
+        <x:v>Glassworker/fabricator or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L111" s="9" t="str">
+        <x:v>Materials: Metal/shell collar; compatible mineral/biological seal insert TBD</x:v>
+      </x:c>
+      <x:c r="M111" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N111" s="9" t="str">
+        <x:v>Biological membrane is not automatically compatible; no fat/oil/gasket recipe accepted</x:v>
+      </x:c>
+      <x:c r="O111" s="36"/>
+      <x:c r="P111" s="36"/>
+      <x:c r="Q111" s="36"/>
+      <x:c r="R111" s="36"/>
+      <x:c r="S111" s="36"/>
+      <x:c r="T111" s="9" t="str">
+        <x:v>Qualitative size: Part-sized. Closure: Mechanical collar. Contents: Vessel closure, not a liquid container</x:v>
+      </x:c>
+      <x:c r="U111" s="37"/>
+      <x:c r="V111" s="9" t="str">
+        <x:v>New game proposal, October 14, 2026. New closure assembly proposal; exact seal material unresolved. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
@@ -5628,14 +6513,17 @@
   <x:conditionalFormatting sqref="E84:E95">
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="proposal"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C6:C23">
       <x:formula1>"Equipment,Field supplies,Resources,Crafting components,Weapons,Ammunition,Quest items,Trade goods"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C96:C111">
+      <x:formula1>"Equipment,Field supplies,Resources,Crafting components,Containers,Weapons,Ammunition,Quest items,Trade goods"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d0940bd6efa40df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re583605c66c2436d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6543,7 +7431,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb0ca6f067fa48d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raefaf1fd551940f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6909,7 +7797,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5adb5314a14c4b0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b4e89d903b24d5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7108,10 +7996,25 @@
         <x:v>Currency, prices, quest-item roster and rarity remain open</x:v>
       </x:c>
     </x:row>
+    <x:row r="16" ht="70" customHeight="1">
+      <x:c r="A16" s="41" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="B16" s="41" t="n">
+        <x:f>COUNTIF(Items!$C$6:$C$1005,A16)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C16" s="41" t="str">
+        <x:v>Primary vessels, protective carriers, transfer glassware and closures</x:v>
+      </x:c>
+      <x:c r="D16" s="41" t="str">
+        <x:v>16 proposals; form distinguishes actual vessels from boxes, tools and the possible fixed chest</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree1e5780f5884b8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd822c5ee14654ae6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7174,7 +8077,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>90 design entries: 18 existing item IDs and 72 design concepts. Twelve named chemical concepts are new brainstorming proposals; three earlier generic fauna food/chemistry placeholders remain grouping candidates.</x:v>
+        <x:v>106 design entries: 18 existing item IDs and 88 design concepts. Sixteen container-family proposals include vessels, protective cases, transfer tools, closures and one possible local chest.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -7529,10 +8432,66 @@
         <x:v>Liquid candidates require deliberate containment. Native liquid landscapes, real synthesis procedures and harvesting/weapon delivery rules are not introduced.</x:v>
       </x:c>
     </x:row>
+    <x:row r="53" ht="70" customHeight="1">
+      <x:c r="A53" s="4" t="str">
+        <x:v>Container ownership</x:v>
+      </x:c>
+      <x:c r="B53" s="4" t="str">
+        <x:v>Proposed filled vessel = one container instance with one contained payload. Transfer preserves vessel identity, content identity/quantity and ownership; no duplicate empty/full item stacks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="70" customHeight="1">
+      <x:c r="A54" s="4" t="str">
+        <x:v>Cargo and packaging</x:v>
+      </x:c>
+      <x:c r="B54" s="4" t="str">
+        <x:v>Gathered ichor and raw chemicals remain Legger/local resources. Boxes, cases and nested vessels grant no extra inventory capacity. All material and contents mass must be counted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="70" customHeight="1">
+      <x:c r="A55" s="4" t="str">
+        <x:v>Capacity and compatibility</x:v>
+      </x:c>
+      <x:c r="B55" s="4" t="str">
+        <x:v>Sizes are qualitative. Capacity, seal, liner and material compatibility are undecided per vessel/content pair. Glass is not assumed universally acid-proof or electrically insulating.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="70" customHeight="1">
+      <x:c r="A56" s="4" t="str">
+        <x:v>No cloth packing</x:v>
+      </x:c>
+      <x:c r="B56" s="4" t="str">
+        <x:v>No cork, wood crates or cloth padding assumed. Proposed outer protection uses shell cages, metal partitions and shaped mineral supports.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="70" customHeight="1">
+      <x:c r="A57" s="4" t="str">
+        <x:v>Workshop and reuse</x:v>
+      </x:c>
+      <x:c r="B57" s="4" t="str">
+        <x:v>Glassworks is a stationary craft/trade source proposal, not an inventory item or Legger platform. Returning empty vessels and workshop reconditioning could form a useful loop; methods/costs remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="70" customHeight="1">
+      <x:c r="A58" s="4" t="str">
+        <x:v>Container costs</x:v>
+      </x:c>
+      <x:c r="B58" s="4" t="str">
+        <x:v>No random breakage, leakage penalties, item durability chores or mandatory nested packing are introduced. Protective forms describe design options, not implemented mechanics.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="70" customHeight="1">
+      <x:c r="A59" s="4" t="str">
+        <x:v>World and save boundary</x:v>
+      </x:c>
+      <x:c r="B59" s="4" t="str">
+        <x:v>Documentation only. No terrain, spawn, streaming or persistence changes. Future container ownership needs stable instances and versioned payloads; prototype canister code does not implement these new vessels.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16ab484d720e473f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59b8b0026a6f4cea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8376,7 +9335,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58961db48a024f27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R110e7303c1ab44db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8619,7 +9578,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39fba1ca96dd4540"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe6abf7039ed46df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9023,7 +9982,683 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9990cc1ee1b5413d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c8b07c6161544bb"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="50" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="55" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="50" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="50" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="70" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="78" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="110" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+      <x:c r="K1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Liquid vessels, protective carriers and glasswork</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+      <x:c r="I2" s="1"/>
+      <x:c r="J2" s="1"/>
+      <x:c r="K2" s="1"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="1" t="str">
+        <x:v>All new proposals. Sizes are qualitative; filled resource vessels use finite Legger/local storage.</x:v>
+      </x:c>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+      <x:c r="I3" s="1"/>
+      <x:c r="J3" s="1"/>
+      <x:c r="K3" s="1"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+      <x:c r="J4" s="1"/>
+      <x:c r="K4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="35" customHeight="1">
+      <x:c r="A5" s="40" t="str">
+        <x:v>Concept ID</x:v>
+      </x:c>
+      <x:c r="B5" s="40" t="str">
+        <x:v>Working label</x:v>
+      </x:c>
+      <x:c r="C5" s="40" t="str">
+        <x:v>Form</x:v>
+      </x:c>
+      <x:c r="D5" s="40" t="str">
+        <x:v>Proposed materials</x:v>
+      </x:c>
+      <x:c r="E5" s="40" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="F5" s="40" t="str">
+        <x:v>Qualitative size</x:v>
+      </x:c>
+      <x:c r="G5" s="40" t="str">
+        <x:v>Closure concept</x:v>
+      </x:c>
+      <x:c r="H5" s="40" t="str">
+        <x:v>Contents / contact</x:v>
+      </x:c>
+      <x:c r="I5" s="40" t="str">
+        <x:v>Design constraint</x:v>
+      </x:c>
+      <x:c r="J5" s="40" t="str">
+        <x:v>Source relationship</x:v>
+      </x:c>
+      <x:c r="K5" s="40" t="str">
+        <x:v>References</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="90" customHeight="1">
+      <x:c r="A6" s="4" t="str">
+        <x:v>proposal.container.sample_vial</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>Clear sample vial</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>Scarce clear glass</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>Inspect a small ichor or chemical sample without opening it</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>Small sample</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="str">
+        <x:v>Matched stopper with retained cover proposed</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="str">
+        <x:v>Species-tagged ichor; compatible chemical samples</x:v>
+      </x:c>
+      <x:c r="I6" s="4" t="str">
+        <x:v>Clear glass cost; liquid compatibility and fill limit unapproved</x:v>
+      </x:c>
+      <x:c r="J6" s="4" t="str">
+        <x:v>Glass draft supports costly transparent material; this vessel is a new proposal</x:v>
+      </x:c>
+      <x:c r="K6" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="90" customHeight="1">
+      <x:c r="A7" s="4" t="str">
+        <x:v>proposal.container.reagent_bottle</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>Opaque reagent bottle</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>Opaque mineral glass; shell/metal cap</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>Everyday transport of one known material</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>Hand-sized</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="str">
+        <x:v>Compression cap and compatible seat proposed</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="str">
+        <x:v>One identified ichor or reagent batch</x:v>
+      </x:c>
+      <x:c r="I7" s="4" t="str">
+        <x:v>Cannot inspect contents through the wall; external identity label matters</x:v>
+      </x:c>
+      <x:c r="J7" s="4" t="str">
+        <x:v>Standard opaque glass vessels have a source-draft basis; exact item new</x:v>
+      </x:c>
+      <x:c r="K7" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="90" customHeight="1">
+      <x:c r="A8" s="4" t="str">
+        <x:v>proposal.container.wide_jar</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>Wide-mouth sample jar</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>Glass body; rigid broad lid</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>Carry thick gels, clot samples and mineral-rich slurry</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>Small to medium</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="str">
+        <x:v>Broad fitted lid with compatible sealing seat</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="str">
+        <x:v>Viscous material or solid/liquid sample</x:v>
+      </x:c>
+      <x:c r="I8" s="4" t="str">
+        <x:v>Wide opening aids access but makes transfers less controlled; no scoop rules set</x:v>
+      </x:c>
+      <x:c r="J8" s="4" t="str">
+        <x:v>Glass vessel basis; wide-mouth item and uses proposed</x:v>
+      </x:c>
+      <x:c r="K8" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="90" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>proposal.container.ampoule</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>Sealed sample ampoule</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Sealed clear glass</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Preserve an isolated small specimen for later analysis or trade</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>Very small</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="str">
+        <x:v>Factory/workshop sealed</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>One specimen; chemistry compatibility unresolved</x:v>
+      </x:c>
+      <x:c r="I9" s="4" t="str">
+        <x:v>Opening and reuse undecided; no mandatory single-use depletion rule approved</x:v>
+      </x:c>
+      <x:c r="J9" s="4" t="str">
+        <x:v>New sealed-glass form inspired by source glasswork</x:v>
+      </x:c>
+      <x:c r="K9" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="90" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>proposal.container.marked_flask</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>Marked glass flask</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Clear glass with etched marks</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>Read fill and compare a specimen before transfer</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>Small sample / workshop</x:v>
+      </x:c>
+      <x:c r="G10" s="4" t="str">
+        <x:v>Matched stopper proposed</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="str">
+        <x:v>Compatible samples and liquids</x:v>
+      </x:c>
+      <x:c r="I10" s="4" t="str">
+        <x:v>Marks do not establish numeric volume, chemistry analysis or automatic quality grading</x:v>
+      </x:c>
+      <x:c r="J10" s="4" t="str">
+        <x:v>New measuring/inspection use; no authored volume system</x:v>
+      </x:c>
+      <x:c r="K10" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="90" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>proposal.container.shell_cage</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>Shell-caged glass flask</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>Protected vessel assembly</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>Glass inner vessel; slotted shell outer cage</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>Protect a carried specimen while keeping a viewing opening</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str">
+        <x:v>Retained cap and inspectable seat proposed</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="str">
+        <x:v>One compatible liquid payload</x:v>
+      </x:c>
+      <x:c r="I11" s="4" t="str">
+        <x:v>One assembled container, not two copies of storage; protection behavior undecided</x:v>
+      </x:c>
+      <x:c r="J11" s="4" t="str">
+        <x:v>Chitin plate/curved vessel and glass drafts inspire assembly; item new</x:v>
+      </x:c>
+      <x:c r="K11" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="90" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>proposal.container.lined_canister</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>Glass-lined haul canister</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>Protected vessel assembly</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>Metal/shell outer body; replaceable glass liner</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>Transport larger quantities to a processing workshop</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>Medium haul</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="str">
+        <x:v>Compression lid with replaceable compatible seat</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str">
+        <x:v>One identified raw ichor or chemical batch</x:v>
+      </x:c>
+      <x:c r="I12" s="4" t="str">
+        <x:v>Liner, seal and contents must all be compatible; filled payload belongs in resource cargo</x:v>
+      </x:c>
+      <x:c r="J12" s="4" t="str">
+        <x:v>Glass draft includes internal canister linings; haul role and item new</x:v>
+      </x:c>
+      <x:c r="K12" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="90" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>proposal.container.ceramic_jar</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>Glazed ceramic reagent jar</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Fired ceramic; proposed glaze; rigid lid</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>Alternative storage for selected processing compounds</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>Fitted rigid lid and compatible seal</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str">
+        <x:v>Only compounds qualified for that jar</x:v>
+      </x:c>
+      <x:c r="I13" s="4" t="str">
+        <x:v>Opaque; heavier/bulkier tradeoff proposed; glaze is not universally chemical-resistant</x:v>
+      </x:c>
+      <x:c r="J13" s="4" t="str">
+        <x:v>New ceramic vessel proposal; not a validated recipe/material capability</x:v>
+      </x:c>
+      <x:c r="K13" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="90" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>proposal.container.bulk_ichor</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>Bulk ichor vessel</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>Primary vessel</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>Reinforced outer body; qualified inner lining TBD</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>Make a large harvest an expedition haul decision</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>Bulk cargo</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="str">
+        <x:v>Service lid and separate transfer fitting proposed</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str">
+        <x:v>One species/batch of gathered ichor</x:v>
+      </x:c>
+      <x:c r="I14" s="4" t="str">
+        <x:v>Finite Legger cargo and contents mass; no backpack resource exception or free capacity</x:v>
+      </x:c>
+      <x:c r="J14" s="4" t="str">
+        <x:v>New bulk vessel proposal; no liter capacity, hose or extraction mechanic approved</x:v>
+      </x:c>
+      <x:c r="K14" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="90" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>proposal.container.vial_case</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>Divided vial case</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>Protective carrier</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Shell/metal case; shaped mineral seats</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>Keep separately sealed specimens organized and supported</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>Several small vessels</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>Rigid latched case; each vial has its own seal</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str">
+        <x:v>Sealed vials only; no direct liquid payload</x:v>
+      </x:c>
+      <x:c r="I15" s="4" t="str">
+        <x:v>Does not create extra inventory capacity; inserts use no assumed wood, cork or cloth</x:v>
+      </x:c>
+      <x:c r="J15" s="4" t="str">
+        <x:v>New case proposal; materials chosen under current no-cloth game rule</x:v>
+      </x:c>
+      <x:c r="K15" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="90" customHeight="1">
+      <x:c r="A16" s="4" t="str">
+        <x:v>proposal.container.sealed_box</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>Sealed cargo box</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>Protective carrier</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Shell panels or metal; rigid dividers</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>Carry containers and dry sample packets together</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>Cargo package</x:v>
+      </x:c>
+      <x:c r="G16" s="4" t="str">
+        <x:v>Latched lid with dust-excluding seat proposed</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="str">
+        <x:v>Separately sealed contents</x:v>
+      </x:c>
+      <x:c r="I16" s="4" t="str">
+        <x:v>Outer dust seal is not liquid or vapor certification; all nested contents still count</x:v>
+      </x:c>
+      <x:c r="J16" s="4" t="str">
+        <x:v>New protective box proposal; not automatic liquid containment</x:v>
+      </x:c>
+      <x:c r="K16" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="90" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>proposal.container.field_chest</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>Locking field chest</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>Storage object candidate</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Metal/shell chest; rigid compartment tray</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Secure expedition samples at a physical camp/worksite</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>Local storage</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>Mechanical lock and rigid lid proposed</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>Sealed vessels and dry material</x:v>
+      </x:c>
+      <x:c r="I17" s="4" t="str">
+        <x:v>Physical local owner; no global stockpile. Portable versus fixed identity undecided</x:v>
+      </x:c>
+      <x:c r="J17" s="4" t="str">
+        <x:v>New storage-object candidate; not another implemented camp chest</x:v>
+      </x:c>
+      <x:c r="K17" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="90" customHeight="1">
+      <x:c r="A18" s="4" t="str">
+        <x:v>proposal.container.funnel</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>Glass transfer funnel</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>Transfer glassware</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>Glass bowl and stem</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>Assist transfers into a compatible narrow-neck vessel</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>Tool-sized</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="str">
+        <x:v>No closure; never a storage vessel</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="str">
+        <x:v>Temporary transfer contact only</x:v>
+      </x:c>
+      <x:c r="I18" s="4" t="str">
+        <x:v>Residue/cross-contamination and workshop reconditioning unresolved; no ambient fluid pooling</x:v>
+      </x:c>
+      <x:c r="J18" s="4" t="str">
+        <x:v>New glassworking tool proposal</x:v>
+      </x:c>
+      <x:c r="K18" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="90" customHeight="1">
+      <x:c r="A19" s="4" t="str">
+        <x:v>proposal.container.draw_tube</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>Glass draw tube</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>Transfer glassware</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Glass tube; proposed mechanical fitting</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>Move a small sample through an inspectable transfer path</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="str">
+        <x:v>Tool-sized</x:v>
+      </x:c>
+      <x:c r="G19" s="4" t="str">
+        <x:v>Closed mechanical interface to design</x:v>
+      </x:c>
+      <x:c r="H19" s="4" t="str">
+        <x:v>Compatible small specimen transfer</x:v>
+      </x:c>
+      <x:c r="I19" s="4" t="str">
+        <x:v>No mouth operation or real extraction procedure; gameplay tool and fittings unapproved</x:v>
+      </x:c>
+      <x:c r="J19" s="4" t="str">
+        <x:v>New mechanical sample-transfer tool proposal</x:v>
+      </x:c>
+      <x:c r="K19" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="90" customHeight="1">
+      <x:c r="A20" s="4" t="str">
+        <x:v>proposal.container.glass_stopper</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>Matched glass stopper</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>Closure component</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>Ground glass seat; retaining clip optional</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>Close its matching vessel without cork or cloth</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="str">
+        <x:v>Part-sized</x:v>
+      </x:c>
+      <x:c r="G20" s="4" t="str">
+        <x:v>Matched seat</x:v>
+      </x:c>
+      <x:c r="H20" s="4" t="str">
+        <x:v>Vessel closure, not an independent payload</x:v>
+      </x:c>
+      <x:c r="I20" s="4" t="str">
+        <x:v>Fit and material compatibility matter; no universal stopper or separate durability chore assumed</x:v>
+      </x:c>
+      <x:c r="J20" s="4" t="str">
+        <x:v>New glass closure component proposal</x:v>
+      </x:c>
+      <x:c r="K20" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="90" customHeight="1">
+      <x:c r="A21" s="4" t="str">
+        <x:v>proposal.container.seal_collar</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>Compression seal collar</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>Closure component</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>Metal/shell collar; compatible mineral/biological seal insert TBD</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>Retain and compress a vessel lid/seat</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="str">
+        <x:v>Part-sized</x:v>
+      </x:c>
+      <x:c r="G21" s="4" t="str">
+        <x:v>Mechanical collar</x:v>
+      </x:c>
+      <x:c r="H21" s="4" t="str">
+        <x:v>Vessel closure, not a liquid container</x:v>
+      </x:c>
+      <x:c r="I21" s="4" t="str">
+        <x:v>Biological membrane is not automatically compatible; no fat/oil/gasket recipe accepted</x:v>
+      </x:c>
+      <x:c r="J21" s="4" t="str">
+        <x:v>New closure assembly proposal; exact seal material unresolved</x:v>
+      </x:c>
+      <x:c r="K21" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6c1c1572fe647d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add armor shield and backpack equipment families
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R25769ec2bf91410b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rf57a656733944a7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rbabdf7f2634e421a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R3e477107a9c242cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R4d9b2650177a496e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R0e69858b132a4bc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Ra5040fb927254a93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R5a1123767d044a6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Ra41986f3017e4d0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R1f2b35aedcb245e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R5a9b37e260e34280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R21d70c0fc2cb4e12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R4b374c134cc34113"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Re6f6da5ef06d4369"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R4f78fa28ca35478e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rec93710b9ddf47b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Rc8ed5f54af564e49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R2b46736a5d134709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R959242ebd96041f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -54,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -156,6 +157,21 @@
         <x:fgColor rgb="FF423B35"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF423B35"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -169,7 +185,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="42">
+  <x:cellXfs count="46">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -309,6 +325,18 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -371,7 +399,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V111" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V121" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -395,6 +423,24 @@
     <x:tableColumn id="20" name="Open design decisions"/>
     <x:tableColumn id="21" name="Column21"/>
     <x:tableColumn id="22" name="Sources"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="EquipmentConceptsTable" displayName="EquipmentConceptsTable" ref="A5:J15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="Concept ID"/>
+    <x:tableColumn id="2" name="Item family"/>
+    <x:tableColumn id="3" name="Region / form"/>
+    <x:tableColumn id="4" name="Crude concept"/>
+    <x:tableColumn id="5" name="Serviceable concept"/>
+    <x:tableColumn id="6" name="Elaborate concept"/>
+    <x:tableColumn id="7" name="Material candidates"/>
+    <x:tableColumn id="8" name="Design purpose"/>
+    <x:tableColumn id="9" name="Open compatibility / ownership"/>
+    <x:tableColumn id="10" name="Status / basis"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -451,7 +497,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -6500,6 +6546,526 @@
         <x:v>New game proposal, October 14, 2026. New closure assembly proposal; exact seal material unresolved. Source records are proposals: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md; https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="112" ht="105" customHeight="1">
+      <x:c r="A112" s="9" t="str">
+        <x:v>proposal.gear.mail_shirt</x:v>
+      </x:c>
+      <x:c r="B112" s="9" t="str">
+        <x:v>Chainmail shirt</x:v>
+      </x:c>
+      <x:c r="C112" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D112" s="9" t="str">
+        <x:v>Torso layer</x:v>
+      </x:c>
+      <x:c r="E112" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F112" s="9" t="str">
+        <x:v>Flexible linked protection candidate</x:v>
+      </x:c>
+      <x:c r="G112" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H112" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I112" s="13"/>
+      <x:c r="J112" s="15"/>
+      <x:c r="K112" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L112" s="9" t="str">
+        <x:v>Proposed materials: Metal rings; attachment/underlayer material undecided</x:v>
+      </x:c>
+      <x:c r="M112" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N112" s="9" t="str">
+        <x:v>Layering, weight, noise and underlayer requirements need design; no cloth assumed</x:v>
+      </x:c>
+      <x:c r="O112" s="42"/>
+      <x:c r="P112" s="42"/>
+      <x:c r="Q112" s="42"/>
+      <x:c r="R112" s="42"/>
+      <x:c r="S112" s="42"/>
+      <x:c r="T112" s="9" t="str">
+        <x:v>Crude: Patched ring sections with conspicuous repairs. Serviceable: Consistent linked rings and repairable closures. Elaborate: Closely fitted ringwork, shaped sleeves and deliberate detailing</x:v>
+      </x:c>
+      <x:c r="U112" s="43"/>
+      <x:c r="V112" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="105" customHeight="1">
+      <x:c r="A113" s="9" t="str">
+        <x:v>proposal.gear.metal_armor_set</x:v>
+      </x:c>
+      <x:c r="B113" s="9" t="str">
+        <x:v>Assembled metal armor</x:v>
+      </x:c>
+      <x:c r="C113" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D113" s="9" t="str">
+        <x:v>Whole-body assembly candidate</x:v>
+      </x:c>
+      <x:c r="E113" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F113" s="9" t="str">
+        <x:v>A coordinated armor family from crude to elaborate</x:v>
+      </x:c>
+      <x:c r="G113" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H113" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I113" s="13"/>
+      <x:c r="J113" s="15"/>
+      <x:c r="K113" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L113" s="9" t="str">
+        <x:v>Proposed materials: Metal plates; hinges/rivets; backing and connectors undecided</x:v>
+      </x:c>
+      <x:c r="M113" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N113" s="9" t="str">
+        <x:v>Set versus independently owned pieces unresolved; do not count the same plates as both set and components</x:v>
+      </x:c>
+      <x:c r="O113" s="42"/>
+      <x:c r="P113" s="42"/>
+      <x:c r="Q113" s="42"/>
+      <x:c r="R113" s="42"/>
+      <x:c r="S113" s="42"/>
+      <x:c r="T113" s="9" t="str">
+        <x:v>Crude: Mixed scavenged plates on a simple carrier. Serviceable: Coordinated torso and limb pieces. Elaborate: Fitted articulated ensemble with matched joints</x:v>
+      </x:c>
+      <x:c r="U113" s="43"/>
+      <x:c r="V113" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="105" customHeight="1">
+      <x:c r="A114" s="9" t="str">
+        <x:v>proposal.gear.chest_armor</x:v>
+      </x:c>
+      <x:c r="B114" s="9" t="str">
+        <x:v>Chest armor</x:v>
+      </x:c>
+      <x:c r="C114" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D114" s="9" t="str">
+        <x:v>Torso plate</x:v>
+      </x:c>
+      <x:c r="E114" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F114" s="9" t="str">
+        <x:v>Torso protection candidate</x:v>
+      </x:c>
+      <x:c r="G114" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H114" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I114" s="13"/>
+      <x:c r="J114" s="15"/>
+      <x:c r="K114" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L114" s="9" t="str">
+        <x:v>Proposed materials: Worked metal; optional shell/mineral-backed design</x:v>
+      </x:c>
+      <x:c r="M114" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N114" s="9" t="str">
+        <x:v>Relationship to chainmail, jacket, cloak and canisters unresolved; no automatic Jacket-slot compatibility</x:v>
+      </x:c>
+      <x:c r="O114" s="42"/>
+      <x:c r="P114" s="42"/>
+      <x:c r="Q114" s="42"/>
+      <x:c r="R114" s="42"/>
+      <x:c r="S114" s="42"/>
+      <x:c r="T114" s="9" t="str">
+        <x:v>Crude: Single repaired plate and simple retaining hardware. Serviceable: Shaped front/back panels with accessible closures. Elaborate: Fitted articulated chest assembly with replaceable panels</x:v>
+      </x:c>
+      <x:c r="U114" s="43"/>
+      <x:c r="V114" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="105" customHeight="1">
+      <x:c r="A115" s="9" t="str">
+        <x:v>proposal.gear.helmet</x:v>
+      </x:c>
+      <x:c r="B115" s="9" t="str">
+        <x:v>Helmet</x:v>
+      </x:c>
+      <x:c r="C115" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D115" s="9" t="str">
+        <x:v>Head</x:v>
+      </x:c>
+      <x:c r="E115" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F115" s="9" t="str">
+        <x:v>Head protection with readable sight/hearing tradeoffs</x:v>
+      </x:c>
+      <x:c r="G115" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H115" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I115" s="13"/>
+      <x:c r="J115" s="15"/>
+      <x:c r="K115" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L115" s="9" t="str">
+        <x:v>Proposed materials: Metal; optional shell panels; liner material undecided</x:v>
+      </x:c>
+      <x:c r="M115" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N115" s="9" t="str">
+        <x:v>Visibility, hearing, breathing and worn canister interaction need design; no sealed respiratory protection implied</x:v>
+      </x:c>
+      <x:c r="O115" s="42"/>
+      <x:c r="P115" s="42"/>
+      <x:c r="Q115" s="42"/>
+      <x:c r="R115" s="42"/>
+      <x:c r="S115" s="42"/>
+      <x:c r="T115" s="9" t="str">
+        <x:v>Crude: Simple open bowl or salvaged cap. Serviceable: Fitted shell with cheek/neck coverage options. Elaborate: Articulated protective helmet with carefully framed sightlines</x:v>
+      </x:c>
+      <x:c r="U115" s="43"/>
+      <x:c r="V115" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="105" customHeight="1">
+      <x:c r="A116" s="9" t="str">
+        <x:v>proposal.gear.leg_armor</x:v>
+      </x:c>
+      <x:c r="B116" s="9" t="str">
+        <x:v>Leg armor</x:v>
+      </x:c>
+      <x:c r="C116" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D116" s="9" t="str">
+        <x:v>Lower limbs</x:v>
+      </x:c>
+      <x:c r="E116" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F116" s="9" t="str">
+        <x:v>Lower-limb protection candidate</x:v>
+      </x:c>
+      <x:c r="G116" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H116" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I116" s="13"/>
+      <x:c r="J116" s="15"/>
+      <x:c r="K116" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L116" s="9" t="str">
+        <x:v>Proposed materials: Metal plate segments; mechanical/flexible joints TBD</x:v>
+      </x:c>
+      <x:c r="M116" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N116" s="9" t="str">
+        <x:v>Crouch, climb, gait and boots must remain compatible; no movement penalties fixed</x:v>
+      </x:c>
+      <x:c r="O116" s="42"/>
+      <x:c r="P116" s="42"/>
+      <x:c r="Q116" s="42"/>
+      <x:c r="R116" s="42"/>
+      <x:c r="S116" s="42"/>
+      <x:c r="T116" s="9" t="str">
+        <x:v>Crude: Separate shin plates and exposed joints. Serviceable: Matched shin/knee protection. Elaborate: Articulated thigh/knee/shin assembly</x:v>
+      </x:c>
+      <x:c r="U116" s="43"/>
+      <x:c r="V116" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="105" customHeight="1">
+      <x:c r="A117" s="9" t="str">
+        <x:v>proposal.gear.boots</x:v>
+      </x:c>
+      <x:c r="B117" s="9" t="str">
+        <x:v>Boots</x:v>
+      </x:c>
+      <x:c r="C117" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D117" s="9" t="str">
+        <x:v>Feet</x:v>
+      </x:c>
+      <x:c r="E117" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F117" s="9" t="str">
+        <x:v>Footwear for traversal and exposure</x:v>
+      </x:c>
+      <x:c r="G117" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H117" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I117" s="13"/>
+      <x:c r="J117" s="15"/>
+      <x:c r="K117" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L117" s="9" t="str">
+        <x:v>Proposed materials: Metal/shell structure; sole and flexible insert materials TBD</x:v>
+      </x:c>
+      <x:c r="M117" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N117" s="9" t="str">
+        <x:v>Grip, sound, grounding and insulation are separate proposals; no leather, rubber or cloth assumed</x:v>
+      </x:c>
+      <x:c r="O117" s="42"/>
+      <x:c r="P117" s="42"/>
+      <x:c r="Q117" s="42"/>
+      <x:c r="R117" s="42"/>
+      <x:c r="S117" s="42"/>
+      <x:c r="T117" s="9" t="str">
+        <x:v>Crude: Rigid foot shell with basic closure and replaceable sole pieces. Serviceable: Fitted boot with articulated ankle and serviceable tread. Elaborate: Carefully fitted armored boot with replaceable contact surfaces</x:v>
+      </x:c>
+      <x:c r="U117" s="43"/>
+      <x:c r="V117" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="105" customHeight="1">
+      <x:c r="A118" s="9" t="str">
+        <x:v>proposal.gear.gloves</x:v>
+      </x:c>
+      <x:c r="B118" s="9" t="str">
+        <x:v>Gloves</x:v>
+      </x:c>
+      <x:c r="C118" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D118" s="9" t="str">
+        <x:v>Hands</x:v>
+      </x:c>
+      <x:c r="E118" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F118" s="9" t="str">
+        <x:v>Hand protection while handling tools and gear</x:v>
+      </x:c>
+      <x:c r="G118" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H118" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I118" s="13"/>
+      <x:c r="J118" s="15"/>
+      <x:c r="K118" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L118" s="9" t="str">
+        <x:v>Proposed materials: Metal/shell guards; flexible insert material TBD</x:v>
+      </x:c>
+      <x:c r="M118" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N118" s="9" t="str">
+        <x:v>Dexterity, grip and chemical/electrical compatibility need design; no universal protective effect</x:v>
+      </x:c>
+      <x:c r="O118" s="42"/>
+      <x:c r="P118" s="42"/>
+      <x:c r="Q118" s="42"/>
+      <x:c r="R118" s="42"/>
+      <x:c r="S118" s="42"/>
+      <x:c r="T118" s="9" t="str">
+        <x:v>Crude: Palm/knuckle guards on a sparse carrier. Serviceable: Fitted hand protection with usable finger movement. Elaborate: Articulated plated glove with replaceable fingertips</x:v>
+      </x:c>
+      <x:c r="U118" s="43"/>
+      <x:c r="V118" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="105" customHeight="1">
+      <x:c r="A119" s="9" t="str">
+        <x:v>proposal.gear.backpack</x:v>
+      </x:c>
+      <x:c r="B119" s="9" t="str">
+        <x:v>Backpack</x:v>
+      </x:c>
+      <x:c r="C119" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D119" s="9" t="str">
+        <x:v>Back-mounted carrier</x:v>
+      </x:c>
+      <x:c r="E119" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F119" s="9" t="str">
+        <x:v>Booter-carried supplies/tool carrier candidate</x:v>
+      </x:c>
+      <x:c r="G119" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H119" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I119" s="13"/>
+      <x:c r="J119" s="15"/>
+      <x:c r="K119" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L119" s="9" t="str">
+        <x:v>Proposed materials: Shell panels, metal frame, hinges; harness material unresolved</x:v>
+      </x:c>
+      <x:c r="M119" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N119" s="9" t="str">
+        <x:v>No raw-resource carrying exception. Capacity, equipment spares, cloak clearance and mounts remain open</x:v>
+      </x:c>
+      <x:c r="O119" s="42"/>
+      <x:c r="P119" s="42"/>
+      <x:c r="Q119" s="42"/>
+      <x:c r="R119" s="42"/>
+      <x:c r="S119" s="42"/>
+      <x:c r="T119" s="9" t="str">
+        <x:v>Crude: Rigid back basket or simple carrying frame. Serviceable: Compartmented shell/metal case on a fitted frame. Elaborate: Tailored frame with modular tool mounts and access panels</x:v>
+      </x:c>
+      <x:c r="U119" s="43"/>
+      <x:c r="V119" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="105" customHeight="1">
+      <x:c r="A120" s="9" t="str">
+        <x:v>proposal.gear.special_plates</x:v>
+      </x:c>
+      <x:c r="B120" s="9" t="str">
+        <x:v>Specialized armor plates</x:v>
+      </x:c>
+      <x:c r="C120" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D120" s="9" t="str">
+        <x:v>Modular protection</x:v>
+      </x:c>
+      <x:c r="E120" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F120" s="9" t="str">
+        <x:v>Purpose-specific protection modules</x:v>
+      </x:c>
+      <x:c r="G120" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H120" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I120" s="13"/>
+      <x:c r="J120" s="15"/>
+      <x:c r="K120" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L120" s="9" t="str">
+        <x:v>Proposed materials: Metal, shell and optional mineral/ceramic layers; recipes TBD</x:v>
+      </x:c>
+      <x:c r="M120" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N120" s="9" t="str">
+        <x:v>Candidate functions: impact distribution, abrasion protection, joint coverage and electrical separation; all effects unapproved</x:v>
+      </x:c>
+      <x:c r="O120" s="42"/>
+      <x:c r="P120" s="42"/>
+      <x:c r="Q120" s="42"/>
+      <x:c r="R120" s="42"/>
+      <x:c r="S120" s="42"/>
+      <x:c r="T120" s="9" t="str">
+        <x:v>Crude: Replaceable abrasion plate or bolted reinforcement. Serviceable: Purpose-shaped joint cover or impact-spreading module. Elaborate: Integrated interchangeable plate system for specific tasks</x:v>
+      </x:c>
+      <x:c r="U120" s="43"/>
+      <x:c r="V120" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="105" customHeight="1">
+      <x:c r="A121" s="9" t="str">
+        <x:v>proposal.gear.shield</x:v>
+      </x:c>
+      <x:c r="B121" s="9" t="str">
+        <x:v>Shield</x:v>
+      </x:c>
+      <x:c r="C121" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D121" s="9" t="str">
+        <x:v>Held / mounted defensive gear</x:v>
+      </x:c>
+      <x:c r="E121" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F121" s="9" t="str">
+        <x:v>Directional protection candidate</x:v>
+      </x:c>
+      <x:c r="G121" s="9" t="str">
+        <x:v>Unassigned; loadout extension TBD</x:v>
+      </x:c>
+      <x:c r="H121" s="9" t="str">
+        <x:v>Booter-worn/held concept; permitted spares in Legger cargo TBD</x:v>
+      </x:c>
+      <x:c r="I121" s="13"/>
+      <x:c r="J121" s="15"/>
+      <x:c r="K121" s="9" t="str">
+        <x:v>Fabrication, trade or salvage candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L121" s="9" t="str">
+        <x:v>Proposed materials: Metal and/or shell panels; grip and rim materials TBD</x:v>
+      </x:c>
+      <x:c r="M121" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N121" s="9" t="str">
+        <x:v>Hand ownership, tool use, carrying posture and Legger cargo storage need design; no blocking mechanics implemented</x:v>
+      </x:c>
+      <x:c r="O121" s="42"/>
+      <x:c r="P121" s="42"/>
+      <x:c r="Q121" s="42"/>
+      <x:c r="R121" s="42"/>
+      <x:c r="S121" s="42"/>
+      <x:c r="T121" s="9" t="str">
+        <x:v>Crude: Cut salvaged plate with a rigid grip. Serviceable: Shaped shield with reinforced edge and repairable face. Elaborate: Fitted layered shield with deliberate sightline and handling geometry</x:v>
+      </x:c>
+      <x:c r="U121" s="43"/>
+      <x:c r="V121" s="9" t="str">
+        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
@@ -6523,7 +7089,435 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re583605c66c2436d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde26094e25214b78"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="62" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="52" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="78" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="110" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Armor, shields and backpacks</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+      <x:c r="I2" s="1"/>
+      <x:c r="J2" s="1"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="1" t="str">
+        <x:v>Requested families. Construction bands are proposals; slots, layering, capacity and effects remain undecided.</x:v>
+      </x:c>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+      <x:c r="I3" s="1"/>
+      <x:c r="J3" s="1"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+      <x:c r="J4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="45" t="str">
+        <x:v>Concept ID</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>Item family</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>Region / form</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>Crude concept</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>Serviceable concept</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str">
+        <x:v>Elaborate concept</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="str">
+        <x:v>Material candidates</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
+        <x:v>Design purpose</x:v>
+      </x:c>
+      <x:c r="I5" s="45" t="str">
+        <x:v>Open compatibility / ownership</x:v>
+      </x:c>
+      <x:c r="J5" s="45" t="str">
+        <x:v>Status / basis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="100" customHeight="1">
+      <x:c r="A6" s="4" t="str">
+        <x:v>proposal.gear.mail_shirt</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>Chainmail shirt</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>Torso layer</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>Patched ring sections with conspicuous repairs</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>Consistent linked rings and repairable closures</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>Closely fitted ringwork, shaped sleeves and deliberate detailing</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="str">
+        <x:v>Metal rings; attachment/underlayer material undecided</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="str">
+        <x:v>Flexible linked protection candidate</x:v>
+      </x:c>
+      <x:c r="I6" s="4" t="str">
+        <x:v>Layering, weight, noise and underlayer requirements need design; no cloth assumed</x:v>
+      </x:c>
+      <x:c r="J6" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="100" customHeight="1">
+      <x:c r="A7" s="4" t="str">
+        <x:v>proposal.gear.metal_armor_set</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>Assembled metal armor</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>Whole-body assembly candidate</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>Mixed scavenged plates on a simple carrier</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>Coordinated torso and limb pieces</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>Fitted articulated ensemble with matched joints</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="str">
+        <x:v>Metal plates; hinges/rivets; backing and connectors undecided</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="str">
+        <x:v>A coordinated armor family from crude to elaborate</x:v>
+      </x:c>
+      <x:c r="I7" s="4" t="str">
+        <x:v>Set versus independently owned pieces unresolved; do not count the same plates as both set and components</x:v>
+      </x:c>
+      <x:c r="J7" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="100" customHeight="1">
+      <x:c r="A8" s="4" t="str">
+        <x:v>proposal.gear.chest_armor</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>Chest armor</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>Torso plate</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>Single repaired plate and simple retaining hardware</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>Shaped front/back panels with accessible closures</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>Fitted articulated chest assembly with replaceable panels</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="str">
+        <x:v>Worked metal; optional shell/mineral-backed design</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="str">
+        <x:v>Torso protection candidate</x:v>
+      </x:c>
+      <x:c r="I8" s="4" t="str">
+        <x:v>Relationship to chainmail, jacket, cloak and canisters unresolved; no automatic Jacket-slot compatibility</x:v>
+      </x:c>
+      <x:c r="J8" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="100" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>proposal.gear.helmet</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>Helmet</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>Head</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Simple open bowl or salvaged cap</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Fitted shell with cheek/neck coverage options</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>Articulated protective helmet with carefully framed sightlines</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="str">
+        <x:v>Metal; optional shell panels; liner material undecided</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>Head protection with readable sight/hearing tradeoffs</x:v>
+      </x:c>
+      <x:c r="I9" s="4" t="str">
+        <x:v>Visibility, hearing, breathing and worn canister interaction need design; no sealed respiratory protection implied</x:v>
+      </x:c>
+      <x:c r="J9" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="100" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>proposal.gear.leg_armor</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>Leg armor</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>Lower limbs</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Separate shin plates and exposed joints</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>Matched shin/knee protection</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>Articulated thigh/knee/shin assembly</x:v>
+      </x:c>
+      <x:c r="G10" s="4" t="str">
+        <x:v>Metal plate segments; mechanical/flexible joints TBD</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="str">
+        <x:v>Lower-limb protection candidate</x:v>
+      </x:c>
+      <x:c r="I10" s="4" t="str">
+        <x:v>Crouch, climb, gait and boots must remain compatible; no movement penalties fixed</x:v>
+      </x:c>
+      <x:c r="J10" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="100" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>proposal.gear.boots</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>Boots</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>Feet</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>Rigid foot shell with basic closure and replaceable sole pieces</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>Fitted boot with articulated ankle and serviceable tread</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>Carefully fitted armored boot with replaceable contact surfaces</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str">
+        <x:v>Metal/shell structure; sole and flexible insert materials TBD</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="str">
+        <x:v>Footwear for traversal and exposure</x:v>
+      </x:c>
+      <x:c r="I11" s="4" t="str">
+        <x:v>Grip, sound, grounding and insulation are separate proposals; no leather, rubber or cloth assumed</x:v>
+      </x:c>
+      <x:c r="J11" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="100" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>proposal.gear.gloves</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>Gloves</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>Hands</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>Palm/knuckle guards on a sparse carrier</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>Fitted hand protection with usable finger movement</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>Articulated plated glove with replaceable fingertips</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="str">
+        <x:v>Metal/shell guards; flexible insert material TBD</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str">
+        <x:v>Hand protection while handling tools and gear</x:v>
+      </x:c>
+      <x:c r="I12" s="4" t="str">
+        <x:v>Dexterity, grip and chemical/electrical compatibility need design; no universal protective effect</x:v>
+      </x:c>
+      <x:c r="J12" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="100" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>proposal.gear.backpack</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>Backpack</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>Back-mounted carrier</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Rigid back basket or simple carrying frame</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>Compartmented shell/metal case on a fitted frame</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>Tailored frame with modular tool mounts and access panels</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>Shell panels, metal frame, hinges; harness material unresolved</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str">
+        <x:v>Booter-carried supplies/tool carrier candidate</x:v>
+      </x:c>
+      <x:c r="I13" s="4" t="str">
+        <x:v>No raw-resource carrying exception. Capacity, equipment spares, cloak clearance and mounts remain open</x:v>
+      </x:c>
+      <x:c r="J13" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="100" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>proposal.gear.special_plates</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>Specialized armor plates</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>Modular protection</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>Replaceable abrasion plate or bolted reinforcement</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>Purpose-shaped joint cover or impact-spreading module</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>Integrated interchangeable plate system for specific tasks</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="str">
+        <x:v>Metal, shell and optional mineral/ceramic layers; recipes TBD</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str">
+        <x:v>Purpose-specific protection modules</x:v>
+      </x:c>
+      <x:c r="I14" s="4" t="str">
+        <x:v>Candidate functions: impact distribution, abrasion protection, joint coverage and electrical separation; all effects unapproved</x:v>
+      </x:c>
+      <x:c r="J14" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="100" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>proposal.gear.shield</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>Shield</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>Held / mounted defensive gear</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Cut salvaged plate with a rigid grip</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>Shaped shield with reinforced edge and repairable face</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>Fitted layered shield with deliberate sightline and handling geometry</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>Metal and/or shell panels; grip and rim materials TBD</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str">
+        <x:v>Directional protection candidate</x:v>
+      </x:c>
+      <x:c r="I15" s="4" t="str">
+        <x:v>Hand ownership, tool use, carrying posture and Legger cargo storage need design; no blocking mechanics implemented</x:v>
+      </x:c>
+      <x:c r="J15" s="4" t="str">
+        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ee3e0707886437c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7431,7 +8425,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raefaf1fd551940f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7a77a73ec46428a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7797,7 +8791,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b4e89d903b24d5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f2a583e521d467a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7858,13 +8852,13 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>8</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>Six existing fitted types plus two user-directed carried gear concepts</x:v>
+        <x:v>Six existing fitted types, two carried-gear concepts and ten requested armor/carrier families</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>Magnets/grounding kit have no assigned equipment slot</x:v>
+        <x:v>New head/limb/hand/back/shield regions are design concepts; no runtime slots added</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
@@ -8014,7 +9008,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd822c5ee14654ae6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cfb700068134287"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8077,7 +9071,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>106 design entries: 18 existing item IDs and 88 design concepts. Sixteen container-family proposals include vessels, protective cases, transfer tools, closures and one possible local chest.</x:v>
+        <x:v>116 design entries: 18 existing item IDs and 98 design concepts. Armor/carrier families include ten author-requested concepts with proposed construction variants, not additional implemented slots.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -8488,10 +9482,66 @@
         <x:v>Documentation only. No terrain, spawn, streaming or persistence changes. Future container ownership needs stable instances and versioned payloads; prototype canister code does not implement these new vessels.</x:v>
       </x:c>
     </x:row>
+    <x:row r="60" ht="70" customHeight="1">
+      <x:c r="A60" s="4" t="str">
+        <x:v>Armor families</x:v>
+      </x:c>
+      <x:c r="B60" s="4" t="str">
+        <x:v>User direction: chainmail shirts, crude-to-elaborate metal armor, chest armor, helmets, leg armor, boots, gloves, backpacks, specialized plates and shields.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="70" customHeight="1">
+      <x:c r="A61" s="4" t="str">
+        <x:v>Construction variants</x:v>
+      </x:c>
+      <x:c r="B61" s="4" t="str">
+        <x:v>Crude, serviceable and elaborate are descriptive design bands, not rarity or numerical power tiers. Fit, articulation, replaceability and craft detail can differ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="70" customHeight="1">
+      <x:c r="A62" s="4" t="str">
+        <x:v>Loadout extension</x:v>
+      </x:c>
+      <x:c r="B62" s="4" t="str">
+        <x:v>The six current trial slots remain dust/algae canister, grapple, digging tool, cloak and jacket. New worn regions, layering and held-shield ownership need their own approved implementation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="70" customHeight="1">
+      <x:c r="A63" s="4" t="str">
+        <x:v>Armor materials</x:v>
+      </x:c>
+      <x:c r="B63" s="4" t="str">
+        <x:v>No cloth, cork, plant fiber, common leather or rubber assumed. Scarce hide/fur and difficult pressed husk materials remain possible only under established processing constraints.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="70" customHeight="1">
+      <x:c r="A64" s="4" t="str">
+        <x:v>Backpack policy</x:v>
+      </x:c>
+      <x:c r="B64" s="4" t="str">
+        <x:v>A backpack concept does not permit Booter to carry raw resources. Supply capacity, spare equipment, harness, cloak/canister clearance and ground-kit placement remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="70" customHeight="1">
+      <x:c r="A65" s="4" t="str">
+        <x:v>Assembly ownership</x:v>
+      </x:c>
+      <x:c r="B65" s="4" t="str">
+        <x:v>The assembled armor entry is a grouping candidate until set-versus-piece ownership is designed. Do not duplicate plates between a set, a module and separately equipped pieces.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="70" customHeight="1">
+      <x:c r="A66" s="4" t="str">
+        <x:v>Armor effects</x:v>
+      </x:c>
+      <x:c r="B66" s="4" t="str">
+        <x:v>Damage mitigation, mass, durability, movement, electrical behavior, chemical protection and trade values are undecided. Visual metal or elaborate craft alone grants no implemented effect.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59b8b0026a6f4cea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57871cf38cb44f63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9335,7 +10385,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R110e7303c1ab44db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dffaada6c814d30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9578,7 +10628,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe6abf7039ed46df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c0b8072d8ac4f8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9982,7 +11032,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c8b07c6161544bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra518e2a73ce840f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10658,7 +11708,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6c1c1572fe647d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70767ffb50754c8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reserve specialized weapon categories and add caltrops candidate
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R1f2b35aedcb245e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R5a9b37e260e34280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R21d70c0fc2cb4e12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R4b374c134cc34113"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Re6f6da5ef06d4369"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R4f78fa28ca35478e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rec93710b9ddf47b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Rc8ed5f54af564e49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R2b46736a5d134709"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R959242ebd96041f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R4c3a01216e0d4b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rd92b9eca6a7b42dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rf3932ceff7d04ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R734a22109d2344b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R3253f7f72f6a44fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R04d02d969abf4bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rc297cf83ca464585"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R1852260165f64fa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R1f2089a67bef40f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="Rc4d24c51b2e3481c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -399,7 +399,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V121" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V122" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -485,7 +485,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -497,7 +497,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -7066,6 +7066,58 @@
         <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
       </x:c>
     </x:row>
+    <x:row r="122" ht="85" customHeight="1">
+      <x:c r="A122" s="9" t="str">
+        <x:v>proposal.weapon.caltrops</x:v>
+      </x:c>
+      <x:c r="B122" s="9" t="str">
+        <x:v>Caltrops</x:v>
+      </x:c>
+      <x:c r="C122" s="9" t="str">
+        <x:v>Weapons</x:v>
+      </x:c>
+      <x:c r="D122" s="9" t="str">
+        <x:v>Trip-ups</x:v>
+      </x:c>
+      <x:c r="E122" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F122" s="9" t="str">
+        <x:v>First named candidate for specialized, purpose-specific weapon brainstorming.</x:v>
+      </x:c>
+      <x:c r="G122" s="9" t="str">
+        <x:v>Unassigned; future design</x:v>
+      </x:c>
+      <x:c r="H122" s="9" t="str">
+        <x:v>Carrier and quantity policy TBD</x:v>
+      </x:c>
+      <x:c r="I122" s="13"/>
+      <x:c r="J122" s="15"/>
+      <x:c r="K122" s="9" t="str">
+        <x:v>Acquisition and manufacture deferred</x:v>
+      </x:c>
+      <x:c r="L122" s="9" t="str">
+        <x:v>No recipe authored</x:v>
+      </x:c>
+      <x:c r="M122" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N122" s="9" t="str">
+        <x:v>Weapon mechanics, damage, targets and deployment are deferred.</x:v>
+      </x:c>
+      <x:c r="O122" s="17"/>
+      <x:c r="P122" s="17"/>
+      <x:c r="Q122" s="17"/>
+      <x:c r="R122" s="17"/>
+      <x:c r="S122" s="17"/>
+      <x:c r="T122" s="9" t="str">
+        <x:v>Future weapon lanes: offensive weapons, defensive weapons, traps and trip-ups. No additional weapon roster proposed.</x:v>
+      </x:c>
+      <x:c r="U122" s="11"/>
+      <x:c r="V122" s="9" t="str">
+        <x:v>Direct author direction, October 14, 2026. Detailed brainstorming explicitly deferred.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
@@ -7089,7 +7141,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde26094e25214b78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24918f7c2f694dec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7517,7 +7569,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ee3e0707886437c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e36ef076f6842d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8425,7 +8477,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7a77a73ec46428a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R056d8b9d619444fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8791,7 +8843,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f2a583e521d467a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3d84b0ca4e849a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8939,13 +8991,13 @@
         <x:v>Weapons and ammunition</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
-        <x:v>No current item definitions</x:v>
+        <x:v>1 named candidate; design deferred</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>World basis permits crafted weapons</x:v>
+        <x:v>Caltrops; four future specialized-purpose weapon lanes</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>No named weapon or ammunition roster established</x:v>
+        <x:v>Offensive weapons, defensive weapons, traps and trip-ups. No ammunition roster defined.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
@@ -9005,10 +9057,70 @@
         <x:v>16 proposals; form distinguishes actual vessels from boxes, tools and the possible fixed chest</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="60" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>Offensive weapons</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="n">
+        <x:f>COUNTIFS(Items!$C$6:$C$1005,"Weapons",Items!$D$6:$D$1005,A17)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>Reserved category; no named item added</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Specialized purpose and detailed brainstorming deferred</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="60" customHeight="1">
+      <x:c r="A18" s="4" t="str">
+        <x:v>Defensive weapons</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="n">
+        <x:f>COUNTIFS(Items!$C$6:$C$1005,"Weapons",Items!$D$6:$D$1005,A18)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>Reserved category; existing shield concept remains in Equipment</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>No duplicate shield item or new defensive weapon added</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="60" customHeight="1">
+      <x:c r="A19" s="4" t="str">
+        <x:v>Traps</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="n">
+        <x:f>COUNTIFS(Items!$C$6:$C$1005,"Weapons",Items!$D$6:$D$1005,A19)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>Reserved category; no named trap added</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Targets, trigger, recovery and mechanics deferred</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="60" customHeight="1">
+      <x:c r="A20" s="4" t="str">
+        <x:v>Trip-ups</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="n">
+        <x:f>COUNTIFS(Items!$C$6:$C$1005,"Weapons",Items!$D$6:$D$1005,A20)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>Caltrops is the first named candidate</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>No damage, recipe, deployment or target compatibility established</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cfb700068134287"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a435a6716294e65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9071,7 +9183,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>116 design entries: 18 existing item IDs and 98 design concepts. Armor/carrier families include ten author-requested concepts with proposed construction variants, not additional implemented slots.</x:v>
+        <x:v>117 design entries: 18 existing item IDs and 99 design concepts. Caltrops is the only newly named weapon candidate; four purpose-specific weapon lanes are reserved for later brainstorming.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -9538,10 +9650,26 @@
         <x:v>Damage mitigation, mass, durability, movement, electrical behavior, chemical protection and trade values are undecided. Visual metal or elaborate craft alone grants no implemented effect.</x:v>
       </x:c>
     </x:row>
+    <x:row r="67" ht="70" customHeight="1">
+      <x:c r="A67" s="4" t="str">
+        <x:v>Specialized weapon direction</x:v>
+      </x:c>
+      <x:c r="B67" s="4" t="str">
+        <x:v>Reserve offensive weapons, defensive weapons, traps and trip-ups. Caltrops is the first named candidate. Detailed weapon brainstorming is deferred at the author's request.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="70" customHeight="1">
+      <x:c r="A68" s="4" t="str">
+        <x:v>Weapon taxonomy</x:v>
+      </x:c>
+      <x:c r="B68" s="4" t="str">
+        <x:v>Weapon lanes describe intended purpose, not new equipment slots or combat systems. Caltrops is provisionally under Trip-ups; future overlap with traps can be settled later. Existing shield equipment is not duplicated.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57871cf38cb44f63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18d20a55ff0c40a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10385,7 +10513,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dffaada6c814d30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d73ac67262b4559"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10628,7 +10756,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c0b8072d8ac4f8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racf8195972664521"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11032,7 +11160,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra518e2a73ce840f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R642415c6cf244235"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11708,7 +11836,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70767ffb50754c8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc494984be7b4bf3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record extremely rare ancient composite material families
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R4c3a01216e0d4b7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rd92b9eca6a7b42dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rf3932ceff7d04ac7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R734a22109d2344b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R3253f7f72f6a44fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R04d02d969abf4bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rc297cf83ca464585"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R1852260165f64fa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R1f2089a67bef40f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="Rc4d24c51b2e3481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R5df129a4f1784199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R184bdf7fa2b84318"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R59a042f8347d423d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rf8e63faaf64b4883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Redeb9f94543a4e79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rf301270fa9e44c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R106101ca65714a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Rac76479a47484e81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R1209ebdf07594962"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R4841434c94be4da5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="24">
+  <x:fills count="25">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -172,6 +172,11 @@
         <x:fgColor rgb="FF423B35"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3E9D2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -185,7 +190,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="46">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -337,6 +342,9 @@
     <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -399,7 +407,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V122" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V125" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -485,7 +493,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -497,7 +505,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B71" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -7118,6 +7126,168 @@
         <x:v>Direct author direction, October 14, 2026. Detailed brainstorming explicitly deferred.</x:v>
       </x:c>
     </x:row>
+    <x:row r="123" ht="80" customHeight="1">
+      <x:c r="A123" s="9" t="str">
+        <x:v>proposal.ancient.carbon_composite</x:v>
+      </x:c>
+      <x:c r="B123" s="9" t="str">
+        <x:v>Ancient carbon composite</x:v>
+      </x:c>
+      <x:c r="C123" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D123" s="9" t="str">
+        <x:v>Ancient manufactured material</x:v>
+      </x:c>
+      <x:c r="E123" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F123" s="9" t="str">
+        <x:v>Ancient material comparable to carbon-fiber composites.</x:v>
+      </x:c>
+      <x:c r="G123" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H123" s="9" t="str">
+        <x:v>Recovered material: Legger / physical local storage</x:v>
+      </x:c>
+      <x:c r="I123" s="13"/>
+      <x:c r="J123" s="15"/>
+      <x:c r="K123" s="9" t="str">
+        <x:v>Ancient-tech recovery source; specific sites and forms undecided</x:v>
+      </x:c>
+      <x:c r="L123" s="9" t="str">
+        <x:v>Recovery/reuse only as a design candidate; no manufacturing recipe established</x:v>
+      </x:c>
+      <x:c r="M123" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N123" s="9" t="str">
+        <x:v>Recovery form, composition and usable properties need design. No carbon-fabric or cloth item assumed.</x:v>
+      </x:c>
+      <x:c r="O123" s="46" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P123" s="17"/>
+      <x:c r="Q123" s="17"/>
+      <x:c r="R123" s="17"/>
+      <x:c r="S123" s="17"/>
+      <x:c r="T123" s="9" t="str">
+        <x:v>Extremely rare by author direction. Fragment versus intact component, testing, trade and fabrication possibilities remain open.</x:v>
+      </x:c>
+      <x:c r="U123" s="11"/>
+      <x:c r="V123" s="9" t="str">
+        <x:v>Direct author direction October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Related source is a proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/ancient-synthetics.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="80" customHeight="1">
+      <x:c r="A124" s="9" t="str">
+        <x:v>proposal.ancient.nanocarbon</x:v>
+      </x:c>
+      <x:c r="B124" s="9" t="str">
+        <x:v>Ancient nanocarbon material</x:v>
+      </x:c>
+      <x:c r="C124" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D124" s="9" t="str">
+        <x:v>Ancient manufactured material</x:v>
+      </x:c>
+      <x:c r="E124" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F124" s="9" t="str">
+        <x:v>Ancient material comparable to advanced nanocarbon substances.</x:v>
+      </x:c>
+      <x:c r="G124" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H124" s="9" t="str">
+        <x:v>Recovered material: Legger / physical local storage</x:v>
+      </x:c>
+      <x:c r="I124" s="13"/>
+      <x:c r="J124" s="15"/>
+      <x:c r="K124" s="9" t="str">
+        <x:v>Ancient-tech recovery source; specific sites and forms undecided</x:v>
+      </x:c>
+      <x:c r="L124" s="9" t="str">
+        <x:v>Recovery/reuse only as a design candidate; no manufacturing recipe established</x:v>
+      </x:c>
+      <x:c r="M124" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N124" s="9" t="str">
+        <x:v>No self-repair, active nanomachines or extraordinary conductivity inferred from its name.</x:v>
+      </x:c>
+      <x:c r="O124" s="46" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P124" s="17"/>
+      <x:c r="Q124" s="17"/>
+      <x:c r="R124" s="17"/>
+      <x:c r="S124" s="17"/>
+      <x:c r="T124" s="9" t="str">
+        <x:v>Extremely rare by author direction. Fragment versus intact component, testing, trade and fabrication possibilities remain open.</x:v>
+      </x:c>
+      <x:c r="U124" s="11"/>
+      <x:c r="V124" s="9" t="str">
+        <x:v>Direct author direction October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Related source is a proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/ancient-synthetics.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="80" customHeight="1">
+      <x:c r="A125" s="9" t="str">
+        <x:v>proposal.ancient.plasteel</x:v>
+      </x:c>
+      <x:c r="B125" s="9" t="str">
+        <x:v>Ancient plasteel material</x:v>
+      </x:c>
+      <x:c r="C125" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D125" s="9" t="str">
+        <x:v>Ancient manufactured material</x:v>
+      </x:c>
+      <x:c r="E125" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F125" s="9" t="str">
+        <x:v>Ancient manufactured material comparable to plasteel.</x:v>
+      </x:c>
+      <x:c r="G125" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H125" s="9" t="str">
+        <x:v>Recovered material: Legger / physical local storage</x:v>
+      </x:c>
+      <x:c r="I125" s="13"/>
+      <x:c r="J125" s="15"/>
+      <x:c r="K125" s="9" t="str">
+        <x:v>Ancient-tech recovery source; specific sites and forms undecided</x:v>
+      </x:c>
+      <x:c r="L125" s="9" t="str">
+        <x:v>Recovery/reuse only as a design candidate; no manufacturing recipe established</x:v>
+      </x:c>
+      <x:c r="M125" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N125" s="9" t="str">
+        <x:v>Exact formulation and properties undefined; not an ordinary iron/steel ore or alloy recipe.</x:v>
+      </x:c>
+      <x:c r="O125" s="46" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P125" s="17"/>
+      <x:c r="Q125" s="17"/>
+      <x:c r="R125" s="17"/>
+      <x:c r="S125" s="17"/>
+      <x:c r="T125" s="9" t="str">
+        <x:v>Extremely rare by author direction. Fragment versus intact component, testing, trade and fabrication possibilities remain open.</x:v>
+      </x:c>
+      <x:c r="U125" s="11"/>
+      <x:c r="V125" s="9" t="str">
+        <x:v>Direct author direction October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Related source is a proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/ancient-synthetics.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
@@ -7141,7 +7311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24918f7c2f694dec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fc0bba4e5614b41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7569,7 +7739,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e36ef076f6842d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf70e3d50fe1436b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8477,7 +8647,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R056d8b9d619444fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4e16f651e884fe4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8843,7 +9013,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3d84b0ca4e849a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc34dad537d784974"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8934,7 +9104,7 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>65</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Minerals, biological resources, generic chemistry placeholders and twelve new chemical concepts</x:v>
@@ -9117,10 +9287,25 @@
         <x:v>No damage, recipe, deployment or target compatibility established</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="65" customHeight="1">
+      <x:c r="A21" s="4" t="str">
+        <x:v>Ancient technology materials</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="n">
+        <x:f>COUNTIFS(Items!$C$6:$C$1005,"Resources",Items!$D$6:$D$1005,"Ancient manufactured material")</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>Carbon composites, nanocarbon materials, plasteels and related futuristic substances</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>Extremely rare; source of material does not establish repeatable manufacture</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a435a6716294e65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90eb613276f44335"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9183,7 +9368,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>117 design entries: 18 existing item IDs and 99 design concepts. Caltrops is the only newly named weapon candidate; four purpose-specific weapon lanes are reserved for later brainstorming.</x:v>
+        <x:v>120 design entries: 18 existing item IDs and 102 design concepts. Ancient carbon composite, nanocarbon and plasteel are extremely rare author-directed material families; exact properties remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -9666,10 +9851,34 @@
         <x:v>Weapon lanes describe intended purpose, not new equipment slots or combat systems. Caltrops is provisionally under Trip-ups; future overlap with traps can be settled later. Existing shield equipment is not duplicated.</x:v>
       </x:c>
     </x:row>
+    <x:row r="69" ht="65" customHeight="1">
+      <x:c r="A69" s="4" t="str">
+        <x:v>Ancient materials</x:v>
+      </x:c>
+      <x:c r="B69" s="4" t="str">
+        <x:v>Extremely rare manufactured materials analogous to carbon-fiber composites, nanocarbons, plasteels and similar futuristic substances. Three named family entries; other futuristic types remain undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="65" customHeight="1">
+      <x:c r="A70" s="4" t="str">
+        <x:v>Scarcity and manufacture</x:v>
+      </x:c>
+      <x:c r="B70" s="4" t="str">
+        <x:v>Rarity is explicit author direction. No drop rate, quantity, price or ordinary production recipe is assigned. Recovery does not grant manufacturing capability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="65" customHeight="1">
+      <x:c r="A71" s="4" t="str">
+        <x:v>Material distinctions</x:v>
+      </x:c>
+      <x:c r="B71" s="4" t="str">
+        <x:v>Ordinary graphite/charcoal does not become ancient nanocarbon through an assumed recipe. Plasteel is not an ordinary raw metal. Advanced fibers do not establish a cloth exception.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18d20a55ff0c40a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde24c96d6817409b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10513,7 +10722,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d73ac67262b4559"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc383db3f209247ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10756,7 +10965,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racf8195972664521"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d25c20ec50747b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11160,7 +11369,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R642415c6cf244235"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra86fa6994ffc4799"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11836,7 +12045,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc494984be7b4bf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe0dc6235f334f38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record rare fashion clothing and valuable crafting input economy
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R5df129a4f1784199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R184bdf7fa2b84318"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R59a042f8347d423d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rf8e63faaf64b4883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Redeb9f94543a4e79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rf301270fa9e44c82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R106101ca65714a50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Rac76479a47484e81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R1209ebdf07594962"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R4841434c94be4da5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R1070c4c2006347a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R1d47a14dec464e0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R3813aefb25374697"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rffeed6dadb2440e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R83d420ae1c534eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Re14d55c450e142e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R7e45d91ea4854d5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R20f316522ad94f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R56aa3d68dbaf419b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R76a813cfe5ca433d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="25">
+  <x:fills count="26">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -177,6 +177,11 @@
         <x:fgColor rgb="FFF3E9D2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3E9D2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -190,7 +195,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -345,6 +350,9 @@
     <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -407,7 +415,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V125" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -437,7 +445,7 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="EquipmentConceptsTable" displayName="EquipmentConceptsTable" ref="A5:J15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="EquipmentConceptsTable" displayName="EquipmentConceptsTable" ref="A5:J21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Concept ID"/>
     <x:tableColumn id="2" name="Item family"/>
@@ -493,7 +501,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -505,7 +513,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B71" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -3011,7 +3019,7 @@
       <x:c r="R43" s="22"/>
       <x:c r="S43" s="22"/>
       <x:c r="T43" s="9" t="str">
-        <x:v>Specific fur types and outputs remain proposals; no numeric yield</x:v>
+        <x:v>Specific fur types and outputs remain proposals; no numeric yield; fashion-crafting input: high sale-value intent; large material/time demand; exact prices and quantities TBD</x:v>
       </x:c>
       <x:c r="U43" s="23"/>
       <x:c r="V43" s="9" t="str">
@@ -3427,7 +3435,7 @@
       <x:c r="R51" s="22"/>
       <x:c r="S51" s="22"/>
       <x:c r="T51" s="9" t="str">
-        <x:v>Product form and garment use remain proposals; old felted-liner assumption superseded</x:v>
+        <x:v>Product form and garment use remain proposals; old felted-liner assumption superseded; fashion-crafting input: high sale-value intent; large material/time demand; exact prices and quantities TBD</x:v>
       </x:c>
       <x:c r="U51" s="23"/>
       <x:c r="V51" s="9" t="str">
@@ -4675,7 +4683,7 @@
       <x:c r="R75" s="28"/>
       <x:c r="S75" s="28"/>
       <x:c r="T75" s="9" t="str">
-        <x:v>Distinction from icore and exact processing</x:v>
+        <x:v>Distinction from icore and exact processing; fashion-crafting input: high sale-value intent; large material/time demand; exact prices and quantities TBD</x:v>
       </x:c>
       <x:c r="U75" s="29"/>
       <x:c r="V75" s="9" t="str">
@@ -4727,7 +4735,7 @@
       <x:c r="R76" s="28"/>
       <x:c r="S76" s="28"/>
       <x:c r="T76" s="9" t="str">
-        <x:v>Define icore and whether paper uses one or both fiber types</x:v>
+        <x:v>Define icore and whether paper uses one or both fiber types; fashion-crafting input: high sale-value intent; large material/time demand; exact prices and quantities TBD</x:v>
       </x:c>
       <x:c r="U76" s="29"/>
       <x:c r="V76" s="9" t="str">
@@ -4831,7 +4839,7 @@
       <x:c r="R78" s="28"/>
       <x:c r="S78" s="28"/>
       <x:c r="T78" s="9" t="str">
-        <x:v>Binder, equipment, work and finished properties</x:v>
+        <x:v>Binder, equipment, work and finished properties; fashion-crafting input: high sale-value intent; large material/time demand; exact prices and quantities TBD</x:v>
       </x:c>
       <x:c r="U78" s="29"/>
       <x:c r="V78" s="9" t="str">
@@ -4883,7 +4891,7 @@
       <x:c r="R79" s="28"/>
       <x:c r="S79" s="28"/>
       <x:c r="T79" s="9" t="str">
-        <x:v>Species, preservation and workable output forms</x:v>
+        <x:v>Species, preservation and workable output forms; fashion-crafting input: high sale-value intent; large material/time demand; exact prices and quantities TBD</x:v>
       </x:c>
       <x:c r="U79" s="29"/>
       <x:c r="V79" s="9" t="str">
@@ -4935,7 +4943,7 @@
       <x:c r="R80" s="28"/>
       <x:c r="S80" s="28"/>
       <x:c r="T80" s="9" t="str">
-        <x:v>Processing method, intended products and balance</x:v>
+        <x:v>Processing method, intended products and balance; fashion-crafting input: high sale-value intent; large material/time demand; exact prices and quantities TBD</x:v>
       </x:c>
       <x:c r="U80" s="29"/>
       <x:c r="V80" s="9" t="str">
@@ -7286,6 +7294,330 @@
       <x:c r="U125" s="11"/>
       <x:c r="V125" s="9" t="str">
         <x:v>Direct author direction October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Related source is a proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/ancient-synthetics.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="90" customHeight="1">
+      <x:c r="A126" s="9" t="str">
+        <x:v>proposal.fashion.special_spectacles</x:v>
+      </x:c>
+      <x:c r="B126" s="9" t="str">
+        <x:v>Specialized spectacles</x:v>
+      </x:c>
+      <x:c r="C126" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D126" s="9" t="str">
+        <x:v>Specialist eyewear</x:v>
+      </x:c>
+      <x:c r="E126" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F126" s="9" t="str">
+        <x:v>Rare specialized eyewear; precise purpose and optical effect to define.</x:v>
+      </x:c>
+      <x:c r="G126" s="9" t="str">
+        <x:v>Unassigned; fit/layering TBD</x:v>
+      </x:c>
+      <x:c r="H126" s="9" t="str">
+        <x:v>Booter-worn concept; spare/transfer policy TBD</x:v>
+      </x:c>
+      <x:c r="I126" s="13"/>
+      <x:c r="J126" s="15"/>
+      <x:c r="K126" s="9" t="str">
+        <x:v>Specialist crafting/trade candidate; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L126" s="9" t="str">
+        <x:v>Material family: Lens and frame materials/requirements TBD</x:v>
+      </x:c>
+      <x:c r="M126" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N126" s="9" t="str">
+        <x:v>Specific purpose, lens manufacture, face fit and equipment compatibility remain open</x:v>
+      </x:c>
+      <x:c r="O126" s="47" t="str">
+        <x:v>Rare</x:v>
+      </x:c>
+      <x:c r="P126" s="17"/>
+      <x:c r="Q126" s="17"/>
+      <x:c r="R126" s="17"/>
+      <x:c r="S126" s="17"/>
+      <x:c r="T126" s="9" t="str">
+        <x:v>Rare by author direction; fashion versions very rare and expensive. Crafting inputs intended high-value trade goods; no numeric price/time/yield assigned.</x:v>
+      </x:c>
+      <x:c r="U126" s="11"/>
+      <x:c r="V126" s="9" t="str">
+        <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="90" customHeight="1">
+      <x:c r="A127" s="9" t="str">
+        <x:v>proposal.fashion.eyeglasses</x:v>
+      </x:c>
+      <x:c r="B127" s="9" t="str">
+        <x:v>Eyeglasses</x:v>
+      </x:c>
+      <x:c r="C127" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D127" s="9" t="str">
+        <x:v>Eyewear</x:v>
+      </x:c>
+      <x:c r="E127" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F127" s="9" t="str">
+        <x:v>Rare eyeglasses; lens function, frame and fitting need design.</x:v>
+      </x:c>
+      <x:c r="G127" s="9" t="str">
+        <x:v>Unassigned; fit/layering TBD</x:v>
+      </x:c>
+      <x:c r="H127" s="9" t="str">
+        <x:v>Booter-worn concept; spare/transfer policy TBD</x:v>
+      </x:c>
+      <x:c r="I127" s="13"/>
+      <x:c r="J127" s="15"/>
+      <x:c r="K127" s="9" t="str">
+        <x:v>Specialist crafting/trade candidate; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L127" s="9" t="str">
+        <x:v>Material family: Lens and frame materials/requirements TBD</x:v>
+      </x:c>
+      <x:c r="M127" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N127" s="9" t="str">
+        <x:v>Distinction from specialized spectacles and actual vision effects remain open</x:v>
+      </x:c>
+      <x:c r="O127" s="47" t="str">
+        <x:v>Rare</x:v>
+      </x:c>
+      <x:c r="P127" s="17"/>
+      <x:c r="Q127" s="17"/>
+      <x:c r="R127" s="17"/>
+      <x:c r="S127" s="17"/>
+      <x:c r="T127" s="9" t="str">
+        <x:v>Rare by author direction; fashion versions very rare and expensive. Crafting inputs intended high-value trade goods; no numeric price/time/yield assigned.</x:v>
+      </x:c>
+      <x:c r="U127" s="11"/>
+      <x:c r="V127" s="9" t="str">
+        <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="90" customHeight="1">
+      <x:c r="A128" s="9" t="str">
+        <x:v>proposal.fashion.hat</x:v>
+      </x:c>
+      <x:c r="B128" s="9" t="str">
+        <x:v>Hat</x:v>
+      </x:c>
+      <x:c r="C128" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D128" s="9" t="str">
+        <x:v>Headwear</x:v>
+      </x:c>
+      <x:c r="E128" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F128" s="9" t="str">
+        <x:v>Rare headwear; fashion variants belong to the very rare expensive fashion economy.</x:v>
+      </x:c>
+      <x:c r="G128" s="9" t="str">
+        <x:v>Unassigned; fit/layering TBD</x:v>
+      </x:c>
+      <x:c r="H128" s="9" t="str">
+        <x:v>Booter-worn concept; spare/transfer policy TBD</x:v>
+      </x:c>
+      <x:c r="I128" s="13"/>
+      <x:c r="J128" s="15"/>
+      <x:c r="K128" s="9" t="str">
+        <x:v>Specialist crafting/trade candidate; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L128" s="9" t="str">
+        <x:v>Material family: Husk-fiber/fur/hide options proposed; exact construction TBD</x:v>
+      </x:c>
+      <x:c r="M128" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N128" s="9" t="str">
+        <x:v>Hat versus helmet, cloak clearance, shade and decorative function unresolved</x:v>
+      </x:c>
+      <x:c r="O128" s="47" t="str">
+        <x:v>Rare</x:v>
+      </x:c>
+      <x:c r="P128" s="17"/>
+      <x:c r="Q128" s="17"/>
+      <x:c r="R128" s="17"/>
+      <x:c r="S128" s="17"/>
+      <x:c r="T128" s="9" t="str">
+        <x:v>Rare by author direction; fashion versions very rare and expensive. Crafting inputs intended high-value trade goods; no numeric price/time/yield assigned.</x:v>
+      </x:c>
+      <x:c r="U128" s="11"/>
+      <x:c r="V128" s="9" t="str">
+        <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="90" customHeight="1">
+      <x:c r="A129" s="9" t="str">
+        <x:v>proposal.fashion.husk_garment</x:v>
+      </x:c>
+      <x:c r="B129" s="9" t="str">
+        <x:v>Husk-fiber clothing</x:v>
+      </x:c>
+      <x:c r="C129" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D129" s="9" t="str">
+        <x:v>Fashion garment</x:v>
+      </x:c>
+      <x:c r="E129" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F129" s="9" t="str">
+        <x:v>Expensive clothing made from processed husk fibers.</x:v>
+      </x:c>
+      <x:c r="G129" s="9" t="str">
+        <x:v>Unassigned; fit/layering TBD</x:v>
+      </x:c>
+      <x:c r="H129" s="9" t="str">
+        <x:v>Booter-worn concept; spare/transfer policy TBD</x:v>
+      </x:c>
+      <x:c r="I129" s="13"/>
+      <x:c r="J129" s="15"/>
+      <x:c r="K129" s="9" t="str">
+        <x:v>Specialist crafting/trade candidate; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L129" s="9" t="str">
+        <x:v>Material family: Husk-fiber material; no cloth</x:v>
+      </x:c>
+      <x:c r="M129" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N129" s="9" t="str">
+        <x:v>Very large material demand and processing/craft time; garment form and construction open</x:v>
+      </x:c>
+      <x:c r="O129" s="47" t="str">
+        <x:v>Very rare</x:v>
+      </x:c>
+      <x:c r="P129" s="17"/>
+      <x:c r="Q129" s="17"/>
+      <x:c r="R129" s="17"/>
+      <x:c r="S129" s="17"/>
+      <x:c r="T129" s="9" t="str">
+        <x:v>Rare by author direction; fashion versions very rare and expensive. Crafting inputs intended high-value trade goods; no numeric price/time/yield assigned.</x:v>
+      </x:c>
+      <x:c r="U129" s="11"/>
+      <x:c r="V129" s="9" t="str">
+        <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="90" customHeight="1">
+      <x:c r="A130" s="9" t="str">
+        <x:v>proposal.fashion.fur_garment</x:v>
+      </x:c>
+      <x:c r="B130" s="9" t="str">
+        <x:v>Fur clothing</x:v>
+      </x:c>
+      <x:c r="C130" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D130" s="9" t="str">
+        <x:v>Fashion garment</x:v>
+      </x:c>
+      <x:c r="E130" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F130" s="9" t="str">
+        <x:v>Expensive clothing made using processed animal fur.</x:v>
+      </x:c>
+      <x:c r="G130" s="9" t="str">
+        <x:v>Unassigned; fit/layering TBD</x:v>
+      </x:c>
+      <x:c r="H130" s="9" t="str">
+        <x:v>Booter-worn concept; spare/transfer policy TBD</x:v>
+      </x:c>
+      <x:c r="I130" s="13"/>
+      <x:c r="J130" s="15"/>
+      <x:c r="K130" s="9" t="str">
+        <x:v>Specialist crafting/trade candidate; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L130" s="9" t="str">
+        <x:v>Material family: Animal fur; supporting material TBD; no cloth</x:v>
+      </x:c>
+      <x:c r="M130" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N130" s="9" t="str">
+        <x:v>Extremely low usable processing yield; very large material/time demand; no cheap/common liner chain</x:v>
+      </x:c>
+      <x:c r="O130" s="47" t="str">
+        <x:v>Very rare</x:v>
+      </x:c>
+      <x:c r="P130" s="17"/>
+      <x:c r="Q130" s="17"/>
+      <x:c r="R130" s="17"/>
+      <x:c r="S130" s="17"/>
+      <x:c r="T130" s="9" t="str">
+        <x:v>Rare by author direction; fashion versions very rare and expensive. Crafting inputs intended high-value trade goods; no numeric price/time/yield assigned.</x:v>
+      </x:c>
+      <x:c r="U130" s="11"/>
+      <x:c r="V130" s="9" t="str">
+        <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="90" customHeight="1">
+      <x:c r="A131" s="9" t="str">
+        <x:v>proposal.fashion.hide_garment</x:v>
+      </x:c>
+      <x:c r="B131" s="9" t="str">
+        <x:v>Hide clothing</x:v>
+      </x:c>
+      <x:c r="C131" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D131" s="9" t="str">
+        <x:v>Fashion garment</x:v>
+      </x:c>
+      <x:c r="E131" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F131" s="9" t="str">
+        <x:v>Expensive clothing made using processed hides.</x:v>
+      </x:c>
+      <x:c r="G131" s="9" t="str">
+        <x:v>Unassigned; fit/layering TBD</x:v>
+      </x:c>
+      <x:c r="H131" s="9" t="str">
+        <x:v>Booter-worn concept; spare/transfer policy TBD</x:v>
+      </x:c>
+      <x:c r="I131" s="13"/>
+      <x:c r="J131" s="15"/>
+      <x:c r="K131" s="9" t="str">
+        <x:v>Specialist crafting/trade candidate; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L131" s="9" t="str">
+        <x:v>Material family: Processed hide; supporting material TBD; no cloth</x:v>
+      </x:c>
+      <x:c r="M131" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N131" s="9" t="str">
+        <x:v>Extremely low usable processing yield; very large material/time demand; no common leather supply assumed</x:v>
+      </x:c>
+      <x:c r="O131" s="47" t="str">
+        <x:v>Very rare</x:v>
+      </x:c>
+      <x:c r="P131" s="17"/>
+      <x:c r="Q131" s="17"/>
+      <x:c r="R131" s="17"/>
+      <x:c r="S131" s="17"/>
+      <x:c r="T131" s="9" t="str">
+        <x:v>Rare by author direction; fashion versions very rare and expensive. Crafting inputs intended high-value trade goods; no numeric price/time/yield assigned.</x:v>
+      </x:c>
+      <x:c r="U131" s="11"/>
+      <x:c r="V131" s="9" t="str">
+        <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7311,7 +7643,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fc0bba4e5614b41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4f8a4b7cde94fa8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7736,10 +8068,202 @@
         <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
       </x:c>
     </x:row>
+    <x:row r="16" ht="100" customHeight="1">
+      <x:c r="A16" s="4" t="str">
+        <x:v>proposal.fashion.special_spectacles</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>Specialized spectacles</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>Specialist eyewear</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Simple form remains rare; construction TBD</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>Workmanship and fit TBD</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>Fine finish and specialist details TBD</x:v>
+      </x:c>
+      <x:c r="G16" s="4" t="str">
+        <x:v>Lens and frame materials/requirements TBD</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="str">
+        <x:v>Rare specialized eyewear; precise purpose and optical effect to define.</x:v>
+      </x:c>
+      <x:c r="I16" s="4" t="str">
+        <x:v>Specific purpose, lens manufacture, face fit and equipment compatibility remain open</x:v>
+      </x:c>
+      <x:c r="J16" s="4" t="str">
+        <x:v>Family/rarity requested by author. Specific forms, mechanics and craft bands remain proposals. Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="100" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>proposal.fashion.eyeglasses</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>Eyeglasses</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>Eyewear</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Simple form remains rare; construction TBD</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Workmanship and fit TBD</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>Fine finish and specialist details TBD</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>Lens and frame materials/requirements TBD</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>Rare eyeglasses; lens function, frame and fitting need design.</x:v>
+      </x:c>
+      <x:c r="I17" s="4" t="str">
+        <x:v>Distinction from specialized spectacles and actual vision effects remain open</x:v>
+      </x:c>
+      <x:c r="J17" s="4" t="str">
+        <x:v>Family/rarity requested by author. Specific forms, mechanics and craft bands remain proposals. Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="100" customHeight="1">
+      <x:c r="A18" s="4" t="str">
+        <x:v>proposal.fashion.hat</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>Hat</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>Headwear</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>Simple form remains rare; construction TBD</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>Workmanship and fit TBD</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>Fine finish and specialist details TBD</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="str">
+        <x:v>Husk-fiber/fur/hide options proposed; exact construction TBD</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="str">
+        <x:v>Rare headwear; fashion variants belong to the very rare expensive fashion economy.</x:v>
+      </x:c>
+      <x:c r="I18" s="4" t="str">
+        <x:v>Hat versus helmet, cloak clearance, shade and decorative function unresolved</x:v>
+      </x:c>
+      <x:c r="J18" s="4" t="str">
+        <x:v>Family/rarity requested by author. Specific forms, mechanics and craft bands remain proposals. Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="100" customHeight="1">
+      <x:c r="A19" s="4" t="str">
+        <x:v>proposal.fashion.husk_garment</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>Husk-fiber clothing</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>Fashion garment</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Simple form remains rare; construction TBD</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>Workmanship and fit TBD</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="str">
+        <x:v>Fine finish and specialist details TBD</x:v>
+      </x:c>
+      <x:c r="G19" s="4" t="str">
+        <x:v>Husk-fiber material; no cloth</x:v>
+      </x:c>
+      <x:c r="H19" s="4" t="str">
+        <x:v>Expensive clothing made from processed husk fibers.</x:v>
+      </x:c>
+      <x:c r="I19" s="4" t="str">
+        <x:v>Very large material demand and processing/craft time; garment form and construction open</x:v>
+      </x:c>
+      <x:c r="J19" s="4" t="str">
+        <x:v>Family/rarity requested by author. Specific forms, mechanics and craft bands remain proposals. Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="100" customHeight="1">
+      <x:c r="A20" s="4" t="str">
+        <x:v>proposal.fashion.fur_garment</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>Fur clothing</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>Fashion garment</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>Simple form remains rare; construction TBD</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>Workmanship and fit TBD</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="str">
+        <x:v>Fine finish and specialist details TBD</x:v>
+      </x:c>
+      <x:c r="G20" s="4" t="str">
+        <x:v>Animal fur; supporting material TBD; no cloth</x:v>
+      </x:c>
+      <x:c r="H20" s="4" t="str">
+        <x:v>Expensive clothing made using processed animal fur.</x:v>
+      </x:c>
+      <x:c r="I20" s="4" t="str">
+        <x:v>Extremely low usable processing yield; very large material/time demand; no cheap/common liner chain</x:v>
+      </x:c>
+      <x:c r="J20" s="4" t="str">
+        <x:v>Family/rarity requested by author. Specific forms, mechanics and craft bands remain proposals. Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="100" customHeight="1">
+      <x:c r="A21" s="4" t="str">
+        <x:v>proposal.fashion.hide_garment</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>Hide clothing</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>Fashion garment</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>Simple form remains rare; construction TBD</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>Workmanship and fit TBD</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="str">
+        <x:v>Fine finish and specialist details TBD</x:v>
+      </x:c>
+      <x:c r="G21" s="4" t="str">
+        <x:v>Processed hide; supporting material TBD; no cloth</x:v>
+      </x:c>
+      <x:c r="H21" s="4" t="str">
+        <x:v>Expensive clothing made using processed hides.</x:v>
+      </x:c>
+      <x:c r="I21" s="4" t="str">
+        <x:v>Extremely low usable processing yield; very large material/time demand; no common leather supply assumed</x:v>
+      </x:c>
+      <x:c r="J21" s="4" t="str">
+        <x:v>Family/rarity requested by author. Specific forms, mechanics and craft bands remain proposals. Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf70e3d50fe1436b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R927a53fda2424c38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8647,7 +9171,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4e16f651e884fe4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R705c559bf9304274"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9013,7 +9537,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc34dad537d784974"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc837b4bf71e54180"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9074,13 +9598,13 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>18</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>Six existing fitted types, two carried-gear concepts and ten requested armor/carrier families</x:v>
+        <x:v>Existing gear plus armor, carriers, rare eyewear/headwear and very rare fashion families</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>New head/limb/hand/back/shield regions are design concepts; no runtime slots added</x:v>
+        <x:v>New equipment concepts have no implemented slots, effects or layering rules</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
@@ -9302,10 +9826,25 @@
         <x:v>Extremely rare; source of material does not establish repeatable manufacture</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="75" customHeight="1">
+      <x:c r="A22" s="4" t="str">
+        <x:v>Fashion, hats and eyewear</x:v>
+      </x:c>
+      <x:c r="B22" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Specialist eyewear")+COUNTIF(Items!$D$6:$D$1005,"Eyewear")+COUNTIF(Items!$D$6:$D$1005,"Headwear")+COUNTIF(Items!$D$6:$D$1005,"Fashion garment")</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="str">
+        <x:v>Six families: specialized spectacles, eyeglasses, hats, husk-fiber clothing, fur clothing and hide clothing</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>Rare eyewear/hats; very rare expensive fashion. High-value crafting inputs support resource gathering.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90eb613276f44335"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e12393954bf41d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9368,7 +9907,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>120 design entries: 18 existing item IDs and 102 design concepts. Ancient carbon composite, nanocarbon and plasteel are extremely rare author-directed material families; exact properties remain open.</x:v>
+        <x:v>126 design entries: 18 existing item IDs and 108 design concepts. Six rare eyewear/headwear/fashion families added; prices, quantities, crafting times and effects remain undecided.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -9875,10 +10414,58 @@
         <x:v>Ordinary graphite/charcoal does not become ancient nanocarbon through an assumed recipe. Plasteel is not an ordinary raw metal. Advanced fibers do not establish a cloth exception.</x:v>
       </x:c>
     </x:row>
+    <x:row r="72" ht="70" customHeight="1">
+      <x:c r="A72" s="4" t="str">
+        <x:v>Clothing without cloth</x:v>
+      </x:c>
+      <x:c r="B72" s="4" t="str">
+        <x:v>Clothing can be made from husk fibers, animal fur, hides and related processed materials. No-cloth does not mean no clothing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="70" customHeight="1">
+      <x:c r="A73" s="4" t="str">
+        <x:v>Fashion scarcity</x:v>
+      </x:c>
+      <x:c r="B73" s="4" t="str">
+        <x:v>Fashion items are very rare and expensive because production consumes very large quantities of material and very large amounts of time; hide/fur conversion remains extremely low yield.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="70" customHeight="1">
+      <x:c r="A74" s="4" t="str">
+        <x:v>Eyewear and hats</x:v>
+      </x:c>
+      <x:c r="B74" s="4" t="str">
+        <x:v>Specialized spectacles, eyeglasses and hats are rare. Exact optical purposes, lens/frame materials, forms, fit and effects remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="70" customHeight="1">
+      <x:c r="A75" s="4" t="str">
+        <x:v>Fashion input economy</x:v>
+      </x:c>
+      <x:c r="B75" s="4" t="str">
+        <x:v>All inputs used in this expensive fashion economy have high sale-value intent. Seven directly relevant fiber/fur/hide material entries carry that note; membership for other inputs awaits recipes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="70" customHeight="1">
+      <x:c r="A76" s="4" t="str">
+        <x:v>Abundance and value</x:v>
+      </x:c>
+      <x:c r="B76" s="4" t="str">
+        <x:v>Abundant raw husk fiber is compatible with costly fashion production: total input demand, processing loss and skilled labor are separate design factors. Numerical ratios/prices remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="70" customHeight="1">
+      <x:c r="A77" s="4" t="str">
+        <x:v>Utility versus fashion</x:v>
+      </x:c>
+      <x:c r="B77" s="4" t="str">
+        <x:v>Existing starter cloak/jacket, functional armor and containers are not automatically reclassified as luxury fashion. Fashion variants can be defined later.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde24c96d6817409b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e03c748b38b4210"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10722,7 +11309,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc383db3f209247ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5055aeacad044ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10965,7 +11552,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d25c20ec50747b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09c18e8f8142470b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11369,7 +11956,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra86fa6994ffc4799"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6bef2bf20fc40d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12045,7 +12632,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe0dc6235f334f38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cdb2404330e4700"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Brainstorm gemstone families for the material and fashion economy
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R1070c4c2006347a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R1d47a14dec464e0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R3813aefb25374697"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rffeed6dadb2440e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R83d420ae1c534eb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Re14d55c450e142e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R7e45d91ea4854d5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R20f316522ad94f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R56aa3d68dbaf419b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R76a813cfe5ca433d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R2e8e6c09447247a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R68ff341f1ad94bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rd902a5a883944aa7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R2de8b1f2040a47df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R46a728ed62b84b40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rcf18e5b9df2e4b76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R621d8227fdf448ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R70a5b44b03eb458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R1836028243e64df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R52fefabe34314898"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="26">
+  <x:fills count="28">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -182,6 +182,16 @@
         <x:fgColor rgb="FFF3E9D2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -195,7 +205,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -353,6 +363,12 @@
     <x:xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -415,7 +431,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V139" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -501,7 +517,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -513,7 +529,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -7620,6 +7636,422 @@
         <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
       </x:c>
     </x:row>
+    <x:row r="132" ht="90" customHeight="1">
+      <x:c r="A132" s="9" t="str">
+        <x:v>proposal.gem.clear_quartz</x:v>
+      </x:c>
+      <x:c r="B132" s="9" t="str">
+        <x:v>Clear quartz</x:v>
+      </x:c>
+      <x:c r="C132" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D132" s="9" t="str">
+        <x:v>Gemstone concept</x:v>
+      </x:c>
+      <x:c r="E132" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F132" s="9" t="str">
+        <x:v>Proposed appearance: Colorless / clear crystal. Potential use: Small ornaments, polished inserts and premium clear stonework</x:v>
+      </x:c>
+      <x:c r="G132" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H132" s="9" t="str">
+        <x:v>Gathered raw gemstone: Legger / local storage</x:v>
+      </x:c>
+      <x:c r="I132" s="13"/>
+      <x:c r="J132" s="15"/>
+      <x:c r="K132" s="9" t="str">
+        <x:v>Authored ancient mineral-bearing strata candidate; no deposit placement approved</x:v>
+      </x:c>
+      <x:c r="L132" s="9" t="str">
+        <x:v>Sorting, cutting, polishing and setting are future craft concepts</x:v>
+      </x:c>
+      <x:c r="M132" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N132" s="9" t="str">
+        <x:v>Keep distinct from loose silica grit and manufactured glass; optical function is not assumed.</x:v>
+      </x:c>
+      <x:c r="O132" s="48"/>
+      <x:c r="P132" s="48"/>
+      <x:c r="Q132" s="48"/>
+      <x:c r="R132" s="48"/>
+      <x:c r="S132" s="48"/>
+      <x:c r="T132" s="9" t="str">
+        <x:v>Gemstones exist by author direction. This mineral choice, palette, grade, cut and use are proposals. Fashion-suitable inputs intended valuable; no universal rarity or numeric price assigned.</x:v>
+      </x:c>
+      <x:c r="U132" s="49"/>
+      <x:c r="V132" s="9" t="str">
+        <x:v>Author direction October 14, 2026 establishes gemstones generally. Proposed real-mineral inspiration: https://www.gia.edu/gem-encyclopedia; no claim of Death Valley occurrence or game canon for this species.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="90" customHeight="1">
+      <x:c r="A133" s="9" t="str">
+        <x:v>proposal.gem.smoky_quartz</x:v>
+      </x:c>
+      <x:c r="B133" s="9" t="str">
+        <x:v>Smoky quartz</x:v>
+      </x:c>
+      <x:c r="C133" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D133" s="9" t="str">
+        <x:v>Gemstone concept</x:v>
+      </x:c>
+      <x:c r="E133" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F133" s="9" t="str">
+        <x:v>Proposed appearance: Smoke-brown through near-black palette. Potential use: Dark ornaments, clasps and contrasting inlays</x:v>
+      </x:c>
+      <x:c r="G133" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H133" s="9" t="str">
+        <x:v>Gathered raw gemstone: Legger / local storage</x:v>
+      </x:c>
+      <x:c r="I133" s="13"/>
+      <x:c r="J133" s="15"/>
+      <x:c r="K133" s="9" t="str">
+        <x:v>Authored ancient mineral-bearing strata candidate; no deposit placement approved</x:v>
+      </x:c>
+      <x:c r="L133" s="9" t="str">
+        <x:v>Sorting, cutting, polishing and setting are future craft concepts</x:v>
+      </x:c>
+      <x:c r="M133" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N133" s="9" t="str">
+        <x:v>Color/clarity grades and cutting uses are proposals; no storm or charge effect inferred.</x:v>
+      </x:c>
+      <x:c r="O133" s="48"/>
+      <x:c r="P133" s="48"/>
+      <x:c r="Q133" s="48"/>
+      <x:c r="R133" s="48"/>
+      <x:c r="S133" s="48"/>
+      <x:c r="T133" s="9" t="str">
+        <x:v>Gemstones exist by author direction. This mineral choice, palette, grade, cut and use are proposals. Fashion-suitable inputs intended valuable; no universal rarity or numeric price assigned.</x:v>
+      </x:c>
+      <x:c r="U133" s="49"/>
+      <x:c r="V133" s="9" t="str">
+        <x:v>Author direction October 14, 2026 establishes gemstones generally. Proposed real-mineral inspiration: https://www.gia.edu/gem-encyclopedia; no claim of Death Valley occurrence or game canon for this species.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="90" customHeight="1">
+      <x:c r="A134" s="9" t="str">
+        <x:v>proposal.gem.garnet</x:v>
+      </x:c>
+      <x:c r="B134" s="9" t="str">
+        <x:v>Garnet</x:v>
+      </x:c>
+      <x:c r="C134" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D134" s="9" t="str">
+        <x:v>Gemstone concept</x:v>
+      </x:c>
+      <x:c r="E134" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F134" s="9" t="str">
+        <x:v>Proposed appearance: Deep red / rust / orange palette. Potential use: Fashion settings, clasps and detailed inlay</x:v>
+      </x:c>
+      <x:c r="G134" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H134" s="9" t="str">
+        <x:v>Gathered raw gemstone: Legger / local storage</x:v>
+      </x:c>
+      <x:c r="I134" s="13"/>
+      <x:c r="J134" s="15"/>
+      <x:c r="K134" s="9" t="str">
+        <x:v>Authored ancient mineral-bearing strata candidate; no deposit placement approved</x:v>
+      </x:c>
+      <x:c r="L134" s="9" t="str">
+        <x:v>Sorting, cutting, polishing and setting are future craft concepts</x:v>
+      </x:c>
+      <x:c r="M134" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N134" s="9" t="str">
+        <x:v>Garnet is a mineral group; exact species and regional source undecided.</x:v>
+      </x:c>
+      <x:c r="O134" s="48"/>
+      <x:c r="P134" s="48"/>
+      <x:c r="Q134" s="48"/>
+      <x:c r="R134" s="48"/>
+      <x:c r="S134" s="48"/>
+      <x:c r="T134" s="9" t="str">
+        <x:v>Gemstones exist by author direction. This mineral choice, palette, grade, cut and use are proposals. Fashion-suitable inputs intended valuable; no universal rarity or numeric price assigned.</x:v>
+      </x:c>
+      <x:c r="U134" s="49"/>
+      <x:c r="V134" s="9" t="str">
+        <x:v>Author direction October 14, 2026 establishes gemstones generally. Proposed real-mineral inspiration: https://www.gia.edu/gem-encyclopedia; no claim of Death Valley occurrence or game canon for this species.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="90" customHeight="1">
+      <x:c r="A135" s="9" t="str">
+        <x:v>proposal.gem.spinel</x:v>
+      </x:c>
+      <x:c r="B135" s="9" t="str">
+        <x:v>Spinel</x:v>
+      </x:c>
+      <x:c r="C135" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D135" s="9" t="str">
+        <x:v>Gemstone concept</x:v>
+      </x:c>
+      <x:c r="E135" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F135" s="9" t="str">
+        <x:v>Proposed appearance: Black, with other colors left open. Potential use: High-contrast accents and polished dark settings</x:v>
+      </x:c>
+      <x:c r="G135" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H135" s="9" t="str">
+        <x:v>Gathered raw gemstone: Legger / local storage</x:v>
+      </x:c>
+      <x:c r="I135" s="13"/>
+      <x:c r="J135" s="15"/>
+      <x:c r="K135" s="9" t="str">
+        <x:v>Authored ancient mineral-bearing strata candidate; no deposit placement approved</x:v>
+      </x:c>
+      <x:c r="L135" s="9" t="str">
+        <x:v>Sorting, cutting, polishing and setting are future craft concepts</x:v>
+      </x:c>
+      <x:c r="M135" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N135" s="9" t="str">
+        <x:v>Proposed black spinel direction; other colors need not become separate item IDs.</x:v>
+      </x:c>
+      <x:c r="O135" s="48"/>
+      <x:c r="P135" s="48"/>
+      <x:c r="Q135" s="48"/>
+      <x:c r="R135" s="48"/>
+      <x:c r="S135" s="48"/>
+      <x:c r="T135" s="9" t="str">
+        <x:v>Gemstones exist by author direction. This mineral choice, palette, grade, cut and use are proposals. Fashion-suitable inputs intended valuable; no universal rarity or numeric price assigned.</x:v>
+      </x:c>
+      <x:c r="U135" s="49"/>
+      <x:c r="V135" s="9" t="str">
+        <x:v>Author direction October 14, 2026 establishes gemstones generally. Proposed real-mineral inspiration: https://my.gia.edu/gems-gemology/winter-2022-colored-stones-unearthed; no claim of Death Valley occurrence or game canon for this species.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="90" customHeight="1">
+      <x:c r="A136" s="9" t="str">
+        <x:v>proposal.gem.peridot</x:v>
+      </x:c>
+      <x:c r="B136" s="9" t="str">
+        <x:v>Peridot</x:v>
+      </x:c>
+      <x:c r="C136" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D136" s="9" t="str">
+        <x:v>Gemstone concept</x:v>
+      </x:c>
+      <x:c r="E136" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F136" s="9" t="str">
+        <x:v>Proposed appearance: Yellow-green / olive palette. Potential use: Distinctive green accents against iron-colored materials</x:v>
+      </x:c>
+      <x:c r="G136" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H136" s="9" t="str">
+        <x:v>Gathered raw gemstone: Legger / local storage</x:v>
+      </x:c>
+      <x:c r="I136" s="13"/>
+      <x:c r="J136" s="15"/>
+      <x:c r="K136" s="9" t="str">
+        <x:v>Authored ancient mineral-bearing strata candidate; no deposit placement approved</x:v>
+      </x:c>
+      <x:c r="L136" s="9" t="str">
+        <x:v>Sorting, cutting, polishing and setting are future craft concepts</x:v>
+      </x:c>
+      <x:c r="M136" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N136" s="9" t="str">
+        <x:v>Proposed geological gem candidate; not plant material or a source of greenery.</x:v>
+      </x:c>
+      <x:c r="O136" s="48"/>
+      <x:c r="P136" s="48"/>
+      <x:c r="Q136" s="48"/>
+      <x:c r="R136" s="48"/>
+      <x:c r="S136" s="48"/>
+      <x:c r="T136" s="9" t="str">
+        <x:v>Gemstones exist by author direction. This mineral choice, palette, grade, cut and use are proposals. Fashion-suitable inputs intended valuable; no universal rarity or numeric price assigned.</x:v>
+      </x:c>
+      <x:c r="U136" s="49"/>
+      <x:c r="V136" s="9" t="str">
+        <x:v>Author direction October 14, 2026 establishes gemstones generally. Proposed real-mineral inspiration: https://my.gia.edu/gems-gemology/winter-2022-colored-stones-unearthed; no claim of Death Valley occurrence or game canon for this species.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="90" customHeight="1">
+      <x:c r="A137" s="9" t="str">
+        <x:v>proposal.gem.corundum</x:v>
+      </x:c>
+      <x:c r="B137" s="9" t="str">
+        <x:v>Ruby / sapphire corundum</x:v>
+      </x:c>
+      <x:c r="C137" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D137" s="9" t="str">
+        <x:v>Gemstone concept</x:v>
+      </x:c>
+      <x:c r="E137" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F137" s="9" t="str">
+        <x:v>Proposed appearance: Red ruby and blue or other sapphire palette. Potential use: Fine settings and high-craft decorative work</x:v>
+      </x:c>
+      <x:c r="G137" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H137" s="9" t="str">
+        <x:v>Gathered raw gemstone: Legger / local storage</x:v>
+      </x:c>
+      <x:c r="I137" s="13"/>
+      <x:c r="J137" s="15"/>
+      <x:c r="K137" s="9" t="str">
+        <x:v>Authored ancient mineral-bearing strata candidate; no deposit placement approved</x:v>
+      </x:c>
+      <x:c r="L137" s="9" t="str">
+        <x:v>Sorting, cutting, polishing and setting are future craft concepts</x:v>
+      </x:c>
+      <x:c r="M137" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N137" s="9" t="str">
+        <x:v>One family for now; ruby/sapphire variants can split if useful. No armor or tool effect assigned.</x:v>
+      </x:c>
+      <x:c r="O137" s="48"/>
+      <x:c r="P137" s="48"/>
+      <x:c r="Q137" s="48"/>
+      <x:c r="R137" s="48"/>
+      <x:c r="S137" s="48"/>
+      <x:c r="T137" s="9" t="str">
+        <x:v>Gemstones exist by author direction. This mineral choice, palette, grade, cut and use are proposals. Fashion-suitable inputs intended valuable; no universal rarity or numeric price assigned.</x:v>
+      </x:c>
+      <x:c r="U137" s="49"/>
+      <x:c r="V137" s="9" t="str">
+        <x:v>Author direction October 14, 2026 establishes gemstones generally. Proposed real-mineral inspiration: https://my.gia.edu/gems-gemology/winter-2022-colored-stones-unearthed; no claim of Death Valley occurrence or game canon for this species.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="90" customHeight="1">
+      <x:c r="A138" s="9" t="str">
+        <x:v>proposal.gem.tourmaline</x:v>
+      </x:c>
+      <x:c r="B138" s="9" t="str">
+        <x:v>Tourmaline</x:v>
+      </x:c>
+      <x:c r="C138" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D138" s="9" t="str">
+        <x:v>Gemstone concept</x:v>
+      </x:c>
+      <x:c r="E138" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F138" s="9" t="str">
+        <x:v>Proposed appearance: Dark green / multicolor palette to select. Potential use: Regional ornament styles and distinctive settings</x:v>
+      </x:c>
+      <x:c r="G138" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H138" s="9" t="str">
+        <x:v>Gathered raw gemstone: Legger / local storage</x:v>
+      </x:c>
+      <x:c r="I138" s="13"/>
+      <x:c r="J138" s="15"/>
+      <x:c r="K138" s="9" t="str">
+        <x:v>Authored ancient mineral-bearing strata candidate; no deposit placement approved</x:v>
+      </x:c>
+      <x:c r="L138" s="9" t="str">
+        <x:v>Sorting, cutting, polishing and setting are future craft concepts</x:v>
+      </x:c>
+      <x:c r="M138" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N138" s="9" t="str">
+        <x:v>Exact variety and useful color range undecided; no magnetic or electrical powers inferred.</x:v>
+      </x:c>
+      <x:c r="O138" s="48"/>
+      <x:c r="P138" s="48"/>
+      <x:c r="Q138" s="48"/>
+      <x:c r="R138" s="48"/>
+      <x:c r="S138" s="48"/>
+      <x:c r="T138" s="9" t="str">
+        <x:v>Gemstones exist by author direction. This mineral choice, palette, grade, cut and use are proposals. Fashion-suitable inputs intended valuable; no universal rarity or numeric price assigned.</x:v>
+      </x:c>
+      <x:c r="U138" s="49"/>
+      <x:c r="V138" s="9" t="str">
+        <x:v>Author direction October 14, 2026 establishes gemstones generally. Proposed real-mineral inspiration: https://www.gia.edu/gem-encyclopedia; no claim of Death Valley occurrence or game canon for this species.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="90" customHeight="1">
+      <x:c r="A139" s="9" t="str">
+        <x:v>proposal.gem.zircon</x:v>
+      </x:c>
+      <x:c r="B139" s="9" t="str">
+        <x:v>Zircon</x:v>
+      </x:c>
+      <x:c r="C139" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D139" s="9" t="str">
+        <x:v>Gemstone concept</x:v>
+      </x:c>
+      <x:c r="E139" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F139" s="9" t="str">
+        <x:v>Proposed appearance: Honey-brown / warm clear palette. Potential use: Small brilliant accents and fine polished settings</x:v>
+      </x:c>
+      <x:c r="G139" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H139" s="9" t="str">
+        <x:v>Gathered raw gemstone: Legger / local storage</x:v>
+      </x:c>
+      <x:c r="I139" s="13"/>
+      <x:c r="J139" s="15"/>
+      <x:c r="K139" s="9" t="str">
+        <x:v>Authored ancient mineral-bearing strata candidate; no deposit placement approved</x:v>
+      </x:c>
+      <x:c r="L139" s="9" t="str">
+        <x:v>Sorting, cutting, polishing and setting are future craft concepts</x:v>
+      </x:c>
+      <x:c r="M139" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N139" s="9" t="str">
+        <x:v>A natural mineral candidate, distinct from cubic zirconia; no ancient-tech identity assumed.</x:v>
+      </x:c>
+      <x:c r="O139" s="48"/>
+      <x:c r="P139" s="48"/>
+      <x:c r="Q139" s="48"/>
+      <x:c r="R139" s="48"/>
+      <x:c r="S139" s="48"/>
+      <x:c r="T139" s="9" t="str">
+        <x:v>Gemstones exist by author direction. This mineral choice, palette, grade, cut and use are proposals. Fashion-suitable inputs intended valuable; no universal rarity or numeric price assigned.</x:v>
+      </x:c>
+      <x:c r="U139" s="49"/>
+      <x:c r="V139" s="9" t="str">
+        <x:v>Author direction October 14, 2026 establishes gemstones generally. Proposed real-mineral inspiration: https://www.gia.edu/zircon-description; no claim of Death Valley occurrence or game canon for this species.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
@@ -7643,7 +8075,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4f8a4b7cde94fa8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f7e8c92677840e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8263,7 +8695,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R927a53fda2424c38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R526e96dad0de49c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9171,7 +9603,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R705c559bf9304274"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40f9c6334c634fab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9537,7 +9969,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc837b4bf71e54180"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40e8f609c0b1450c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9628,7 +10060,7 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>68</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Minerals, biological resources, generic chemistry placeholders and twelve new chemical concepts</x:v>
@@ -9841,10 +10273,25 @@
         <x:v>Rare eyewear/hats; very rare expensive fashion. High-value crafting inputs support resource gathering.</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="75" customHeight="1">
+      <x:c r="A23" s="4" t="str">
+        <x:v>Gemstones</x:v>
+      </x:c>
+      <x:c r="B23" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Gemstone concept")</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C23" s="4" t="str">
+        <x:v>Eight proposed mineral families: clear/smoky quartz, garnet, spinel, peridot, corundum, tourmaline and zircon</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="str">
+        <x:v>Existence accepted; species, deposits, grades, cutting, rarity and uses remain proposed.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e12393954bf41d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03744211789c450e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9907,7 +10354,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>126 design entries: 18 existing item IDs and 108 design concepts. Six rare eyewear/headwear/fashion families added; prices, quantities, crafting times and effects remain undecided.</x:v>
+        <x:v>134 design entries: 18 existing item IDs and 116 design concepts. Eight gemstone families are brainstorming candidates; only gemstone existence is established by this direction.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -10462,10 +10909,50 @@
         <x:v>Existing starter cloak/jacket, functional armor and containers are not automatically reclassified as luxury fashion. Fashion variants can be defined later.</x:v>
       </x:c>
     </x:row>
+    <x:row r="78" ht="70" customHeight="1">
+      <x:c r="A78" s="4" t="str">
+        <x:v>Gemstone authority</x:v>
+      </x:c>
+      <x:c r="B78" s="4" t="str">
+        <x:v>Gemstones exist. Specific real-mineral candidates, palettes and uses are new game proposals, not accepted lore species or verified Death Valley deposits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="70" customHeight="1">
+      <x:c r="A79" s="4" t="str">
+        <x:v>Gem quality and work</x:v>
+      </x:c>
+      <x:c r="B79" s="4" t="str">
+        <x:v>Proposed value factors: size, clarity, color, inclusions, cutting/polishing skill and setting work. Raw mineral abundance and a fine specimen's value need not be identical.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="70" customHeight="1">
+      <x:c r="A80" s="4" t="str">
+        <x:v>Rough and finished state</x:v>
+      </x:c>
+      <x:c r="B80" s="4" t="str">
+        <x:v>Rough, cut and set forms need a later ownership/craft design. Current entries are families, not duplicate rewards for each processing stage; no gem-cutting recipe or yield implemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="70" customHeight="1">
+      <x:c r="A81" s="4" t="str">
+        <x:v>Fashion use</x:v>
+      </x:c>
+      <x:c r="B81" s="4" t="str">
+        <x:v>Ornaments, clasps and inlays are potential uses. Fashion-qualified inputs follow the high-value economy direction, while exact stone grades, prices and demand remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="70" customHeight="1">
+      <x:c r="A82" s="4" t="str">
+        <x:v>Ancient deposits</x:v>
+      </x:c>
+      <x:c r="B82" s="4" t="str">
+        <x:v>Game deposits could be exposed ancient mineral-bearing strata. These concepts add no present-day water cycle, plant gem source, terrain generation or special elemental powers.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e03c748b38b4210"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304b902371224a1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11309,7 +11796,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5055aeacad044ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f3c66835ce94565"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11552,7 +12039,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09c18e8f8142470b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cebd52385c84789"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11956,7 +12443,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6bef2bf20fc40d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R061ce0042b42449e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12632,7 +13119,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cdb2404330e4700"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fd53b0ee1664203"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify everyday wraps and metal wear versus elaborate fashion
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R2e8e6c09447247a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R68ff341f1ad94bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rd902a5a883944aa7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R2de8b1f2040a47df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R46a728ed62b84b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rcf18e5b9df2e4b76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R621d8227fdf448ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R70a5b44b03eb458a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R1836028243e64df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R52fefabe34314898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R7d8c70ce9d124981"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rf01557ecfe454c92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R48d4ccdb42b845b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rc6c9d63612734444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R282df88cc1b2428f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R838ab625eee54ebe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R7f9ada08577d4c49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R411f56eeacc84545"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R47b9cf5d70404141"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R319b00919f9547ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -431,7 +431,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V139" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V140" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -461,7 +461,7 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="EquipmentConceptsTable" displayName="EquipmentConceptsTable" ref="A5:J21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="EquipmentConceptsTable" displayName="EquipmentConceptsTable" ref="A5:J22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Concept ID"/>
     <x:tableColumn id="2" name="Item family"/>
@@ -517,7 +517,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -529,7 +529,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B85" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -6595,7 +6595,7 @@
         <x:v>User direction; not implemented</x:v>
       </x:c>
       <x:c r="F112" s="9" t="str">
-        <x:v>Flexible linked protection candidate</x:v>
+        <x:v>Everyday metal chainmail clothing; fitted/protective effects remain undecided.</x:v>
       </x:c>
       <x:c r="G112" s="9" t="str">
         <x:v>Unassigned; loadout extension TBD</x:v>
@@ -6623,11 +6623,11 @@
       <x:c r="R112" s="42"/>
       <x:c r="S112" s="42"/>
       <x:c r="T112" s="9" t="str">
-        <x:v>Crude: Patched ring sections with conspicuous repairs. Serviceable: Consistent linked rings and repairable closures. Elaborate: Closely fitted ringwork, shaped sleeves and deliberate detailing</x:v>
+        <x:v>Ordinary simple chainmail belongs to regular clothing. Elaborate variants can be fashion; detailed construction, mass and effects remain open.</x:v>
       </x:c>
       <x:c r="U112" s="43"/>
       <x:c r="V112" s="9" t="str">
-        <x:v>Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="105" customHeight="1">
@@ -7479,7 +7479,7 @@
         <x:v>proposal.fashion.husk_garment</x:v>
       </x:c>
       <x:c r="B129" s="9" t="str">
-        <x:v>Husk-fiber clothing</x:v>
+        <x:v>Elaborate husk-fiber wear</x:v>
       </x:c>
       <x:c r="C129" s="9" t="str">
         <x:v>Equipment</x:v>
@@ -7491,7 +7491,7 @@
         <x:v>User direction; not implemented</x:v>
       </x:c>
       <x:c r="F129" s="9" t="str">
-        <x:v>Expensive clothing made from processed husk fibers.</x:v>
+        <x:v>Very rare expensive fashion clothing using husk fibers.</x:v>
       </x:c>
       <x:c r="G129" s="9" t="str">
         <x:v>Unassigned; fit/layering TBD</x:v>
@@ -7511,7 +7511,7 @@
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N129" s="9" t="str">
-        <x:v>Very large material demand and processing/craft time; garment form and construction open</x:v>
+        <x:v>Luxury workmanship and large material/time demand; does not classify all everyday clothing as rare. Hide/fur processing still has extremely low yield.</x:v>
       </x:c>
       <x:c r="O129" s="47" t="str">
         <x:v>Very rare</x:v>
@@ -7521,11 +7521,11 @@
       <x:c r="R129" s="17"/>
       <x:c r="S129" s="17"/>
       <x:c r="T129" s="9" t="str">
-        <x:v>Rare by author direction; fashion versions very rare and expensive. Crafting inputs intended high-value trade goods; no numeric price/time/yield assigned.</x:v>
+        <x:v>Elaborate fashion variant. Ordinary simple wraps and metal-based wear with minimal fur are a separate everyday baseline.</x:v>
       </x:c>
       <x:c r="U129" s="11"/>
       <x:c r="V129" s="9" t="str">
-        <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="90" customHeight="1">
@@ -7533,7 +7533,7 @@
         <x:v>proposal.fashion.fur_garment</x:v>
       </x:c>
       <x:c r="B130" s="9" t="str">
-        <x:v>Fur clothing</x:v>
+        <x:v>Elaborate fur wear</x:v>
       </x:c>
       <x:c r="C130" s="9" t="str">
         <x:v>Equipment</x:v>
@@ -7545,7 +7545,7 @@
         <x:v>User direction; not implemented</x:v>
       </x:c>
       <x:c r="F130" s="9" t="str">
-        <x:v>Expensive clothing made using processed animal fur.</x:v>
+        <x:v>Very rare expensive fashion clothing using animal fur.</x:v>
       </x:c>
       <x:c r="G130" s="9" t="str">
         <x:v>Unassigned; fit/layering TBD</x:v>
@@ -7565,7 +7565,7 @@
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N130" s="9" t="str">
-        <x:v>Extremely low usable processing yield; very large material/time demand; no cheap/common liner chain</x:v>
+        <x:v>Luxury workmanship and large material/time demand; does not classify all everyday clothing as rare. Hide/fur processing still has extremely low yield.</x:v>
       </x:c>
       <x:c r="O130" s="47" t="str">
         <x:v>Very rare</x:v>
@@ -7575,11 +7575,11 @@
       <x:c r="R130" s="17"/>
       <x:c r="S130" s="17"/>
       <x:c r="T130" s="9" t="str">
-        <x:v>Rare by author direction; fashion versions very rare and expensive. Crafting inputs intended high-value trade goods; no numeric price/time/yield assigned.</x:v>
+        <x:v>Elaborate fashion variant. Ordinary simple wraps and metal-based wear with minimal fur are a separate everyday baseline.</x:v>
       </x:c>
       <x:c r="U130" s="11"/>
       <x:c r="V130" s="9" t="str">
-        <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="90" customHeight="1">
@@ -7587,7 +7587,7 @@
         <x:v>proposal.fashion.hide_garment</x:v>
       </x:c>
       <x:c r="B131" s="9" t="str">
-        <x:v>Hide clothing</x:v>
+        <x:v>Elaborate hide wear</x:v>
       </x:c>
       <x:c r="C131" s="9" t="str">
         <x:v>Equipment</x:v>
@@ -7599,7 +7599,7 @@
         <x:v>User direction; not implemented</x:v>
       </x:c>
       <x:c r="F131" s="9" t="str">
-        <x:v>Expensive clothing made using processed hides.</x:v>
+        <x:v>Very rare expensive fashion clothing using processed hides.</x:v>
       </x:c>
       <x:c r="G131" s="9" t="str">
         <x:v>Unassigned; fit/layering TBD</x:v>
@@ -7619,7 +7619,7 @@
         <x:v>Not implemented</x:v>
       </x:c>
       <x:c r="N131" s="9" t="str">
-        <x:v>Extremely low usable processing yield; very large material/time demand; no common leather supply assumed</x:v>
+        <x:v>Luxury workmanship and large material/time demand; does not classify all everyday clothing as rare. Hide/fur processing still has extremely low yield.</x:v>
       </x:c>
       <x:c r="O131" s="47" t="str">
         <x:v>Very rare</x:v>
@@ -7629,11 +7629,11 @@
       <x:c r="R131" s="17"/>
       <x:c r="S131" s="17"/>
       <x:c r="T131" s="9" t="str">
-        <x:v>Rare by author direction; fashion versions very rare and expensive. Crafting inputs intended high-value trade goods; no numeric price/time/yield assigned.</x:v>
+        <x:v>Elaborate fashion variant. Ordinary simple wraps and metal-based wear with minimal fur are a separate everyday baseline.</x:v>
       </x:c>
       <x:c r="U131" s="11"/>
       <x:c r="V131" s="9" t="str">
-        <x:v>Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="90" customHeight="1">
@@ -8050,6 +8050,58 @@
       <x:c r="U139" s="49"/>
       <x:c r="V139" s="9" t="str">
         <x:v>Author direction October 14, 2026 establishes gemstones generally. Proposed real-mineral inspiration: https://www.gia.edu/zircon-description; no claim of Death Valley occurrence or game canon for this species.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="90" customHeight="1">
+      <x:c r="A140" s="9" t="str">
+        <x:v>proposal.gear.simple_wraps</x:v>
+      </x:c>
+      <x:c r="B140" s="9" t="str">
+        <x:v>Simple everyday wraps</x:v>
+      </x:c>
+      <x:c r="C140" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D140" s="9" t="str">
+        <x:v>Everyday clothing</x:v>
+      </x:c>
+      <x:c r="E140" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F140" s="9" t="str">
+        <x:v>Regular simple wrap-style clothing under the no-cloth material rule.</x:v>
+      </x:c>
+      <x:c r="G140" s="9" t="str">
+        <x:v>Unassigned; layering/fastening TBD</x:v>
+      </x:c>
+      <x:c r="H140" s="9" t="str">
+        <x:v>Booter-worn concept; supply/spare policy TBD</x:v>
+      </x:c>
+      <x:c r="I140" s="13"/>
+      <x:c r="J140" s="15"/>
+      <x:c r="K140" s="9" t="str">
+        <x:v>Ordinary fabrication/trade candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L140" s="9" t="str">
+        <x:v>Construction and material combination TBD; minimal fur with metal-based fastenings/pieces possible</x:v>
+      </x:c>
+      <x:c r="M140" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N140" s="9" t="str">
+        <x:v>No cloth. Wrap material, attachment and coverage remain open; minimal fur is not an abundant processed-fur supply.</x:v>
+      </x:c>
+      <x:c r="O140" s="17"/>
+      <x:c r="P140" s="17"/>
+      <x:c r="Q140" s="17"/>
+      <x:c r="R140" s="17"/>
+      <x:c r="S140" s="17"/>
+      <x:c r="T140" s="9" t="str">
+        <x:v>Everyday baseline by author direction. No fixed rarity, price, garment pattern or material ratio assigned.</x:v>
+      </x:c>
+      <x:c r="U140" s="11"/>
+      <x:c r="V140" s="9" t="str">
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8075,7 +8127,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f7e8c92677840e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7406d226711453b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8203,13 +8255,13 @@
         <x:v>Metal rings; attachment/underlayer material undecided</x:v>
       </x:c>
       <x:c r="H6" s="4" t="str">
-        <x:v>Flexible linked protection candidate</x:v>
+        <x:v>Everyday metal clothing; protective mechanics TBD</x:v>
       </x:c>
       <x:c r="I6" s="4" t="str">
         <x:v>Layering, weight, noise and underlayer requirements need design; no cloth assumed</x:v>
       </x:c>
       <x:c r="J6" s="4" t="str">
-        <x:v>Family requested by author; construction/material details proposed. Author item-family direction, October 14, 2026. Crude/serviceable/elaborate constructions, materials and effects are new proposals. Docs/WORLD_BASIS.md#material-culture; current runtime slot contract: Assets/_Project/Scripts/Runtime/TopDown3D/Inventory/TopDown3DLoadoutLayout.cs</x:v>
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="100" customHeight="1">
@@ -8601,13 +8653,13 @@
         <x:v>proposal.fashion.husk_garment</x:v>
       </x:c>
       <x:c r="B19" s="4" t="str">
-        <x:v>Husk-fiber clothing</x:v>
+        <x:v>Elaborate husk-fiber wear</x:v>
       </x:c>
       <x:c r="C19" s="4" t="str">
         <x:v>Fashion garment</x:v>
       </x:c>
       <x:c r="D19" s="4" t="str">
-        <x:v>Simple form remains rare; construction TBD</x:v>
+        <x:v>Simpler finish within the rare fashion family</x:v>
       </x:c>
       <x:c r="E19" s="4" t="str">
         <x:v>Workmanship and fit TBD</x:v>
@@ -8619,13 +8671,13 @@
         <x:v>Husk-fiber material; no cloth</x:v>
       </x:c>
       <x:c r="H19" s="4" t="str">
-        <x:v>Expensive clothing made from processed husk fibers.</x:v>
+        <x:v>Very rare elaborate fashion; everyday simple wraps/metal wear separate</x:v>
       </x:c>
       <x:c r="I19" s="4" t="str">
-        <x:v>Very large material demand and processing/craft time; garment form and construction open</x:v>
+        <x:v>Large material/time demand; no universal scarcity for ordinary wear</x:v>
       </x:c>
       <x:c r="J19" s="4" t="str">
-        <x:v>Family/rarity requested by author. Specific forms, mechanics and craft bands remain proposals. Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="100" customHeight="1">
@@ -8633,13 +8685,13 @@
         <x:v>proposal.fashion.fur_garment</x:v>
       </x:c>
       <x:c r="B20" s="4" t="str">
-        <x:v>Fur clothing</x:v>
+        <x:v>Elaborate fur wear</x:v>
       </x:c>
       <x:c r="C20" s="4" t="str">
         <x:v>Fashion garment</x:v>
       </x:c>
       <x:c r="D20" s="4" t="str">
-        <x:v>Simple form remains rare; construction TBD</x:v>
+        <x:v>Simpler finish within the rare fashion family</x:v>
       </x:c>
       <x:c r="E20" s="4" t="str">
         <x:v>Workmanship and fit TBD</x:v>
@@ -8651,13 +8703,13 @@
         <x:v>Animal fur; supporting material TBD; no cloth</x:v>
       </x:c>
       <x:c r="H20" s="4" t="str">
-        <x:v>Expensive clothing made using processed animal fur.</x:v>
+        <x:v>Very rare elaborate fashion; everyday simple wraps/metal wear separate</x:v>
       </x:c>
       <x:c r="I20" s="4" t="str">
-        <x:v>Extremely low usable processing yield; very large material/time demand; no cheap/common liner chain</x:v>
+        <x:v>Large material/time demand; no universal scarcity for ordinary wear</x:v>
       </x:c>
       <x:c r="J20" s="4" t="str">
-        <x:v>Family/rarity requested by author. Specific forms, mechanics and craft bands remain proposals. Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="100" customHeight="1">
@@ -8665,13 +8717,13 @@
         <x:v>proposal.fashion.hide_garment</x:v>
       </x:c>
       <x:c r="B21" s="4" t="str">
-        <x:v>Hide clothing</x:v>
+        <x:v>Elaborate hide wear</x:v>
       </x:c>
       <x:c r="C21" s="4" t="str">
         <x:v>Fashion garment</x:v>
       </x:c>
       <x:c r="D21" s="4" t="str">
-        <x:v>Simple form remains rare; construction TBD</x:v>
+        <x:v>Simpler finish within the rare fashion family</x:v>
       </x:c>
       <x:c r="E21" s="4" t="str">
         <x:v>Workmanship and fit TBD</x:v>
@@ -8683,19 +8735,51 @@
         <x:v>Processed hide; supporting material TBD; no cloth</x:v>
       </x:c>
       <x:c r="H21" s="4" t="str">
-        <x:v>Expensive clothing made using processed hides.</x:v>
+        <x:v>Very rare elaborate fashion; everyday simple wraps/metal wear separate</x:v>
       </x:c>
       <x:c r="I21" s="4" t="str">
-        <x:v>Extremely low usable processing yield; very large material/time demand; no common leather supply assumed</x:v>
+        <x:v>Large material/time demand; no universal scarcity for ordinary wear</x:v>
       </x:c>
       <x:c r="J21" s="4" t="str">
-        <x:v>Family/rarity requested by author. Specific forms, mechanics and craft bands remain proposals. Direct author direction, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Clothing exists without cloth; fashion is very rare/expensive and qualifying crafting inputs have high sale-value intent.</x:v>
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="100" customHeight="1">
+      <x:c r="A22" s="4" t="str">
+        <x:v>proposal.gear.simple_wraps</x:v>
+      </x:c>
+      <x:c r="B22" s="4" t="str">
+        <x:v>Simple everyday wraps</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="str">
+        <x:v>Everyday clothing</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>Simple wrap; pattern TBD</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="str">
+        <x:v>Fastening and fit TBD</x:v>
+      </x:c>
+      <x:c r="F22" s="4" t="str">
+        <x:v>Elaborate fashion variant would be separate</x:v>
+      </x:c>
+      <x:c r="G22" s="4" t="str">
+        <x:v>No cloth; exact wrap construction and minimal-fur/metal combination TBD</x:v>
+      </x:c>
+      <x:c r="H22" s="4" t="str">
+        <x:v>Everyday clothing baseline</x:v>
+      </x:c>
+      <x:c r="I22" s="4" t="str">
+        <x:v>Coverage, layering and attachment remain open</x:v>
+      </x:c>
+      <x:c r="J22" s="4" t="str">
+        <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R526e96dad0de49c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36a2655abdf04317"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9603,7 +9687,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40f9c6334c634fab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53746a952862460e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9969,7 +10053,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40e8f609c0b1450c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R568e319411824edf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10030,7 +10114,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>Existing gear plus armor, carriers, rare eyewear/headwear and very rare fashion families</x:v>
@@ -10267,10 +10351,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C22" s="4" t="str">
-        <x:v>Six families: specialized spectacles, eyeglasses, hats, husk-fiber clothing, fur clothing and hide clothing</x:v>
+        <x:v>Six rare eyewear/headwear and elaborate fashion families</x:v>
       </x:c>
       <x:c r="D22" s="4" t="str">
-        <x:v>Rare eyewear/hats; very rare expensive fashion. High-value crafting inputs support resource gathering.</x:v>
+        <x:v>Elaborate fashion is very rare/expensive; everyday simple wraps and chainmail are a separate baseline.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="75" customHeight="1">
@@ -10288,10 +10372,25 @@
         <x:v>Existence accepted; species, deposits, grades, cutting, rarity and uses remain proposed.</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="75" customHeight="1">
+      <x:c r="A24" s="4" t="str">
+        <x:v>Everyday clothing</x:v>
+      </x:c>
+      <x:c r="B24" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Everyday clothing")+COUNTIF(Items!$A$6:$A$1005,"proposal.gear.mail_shirt")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C24" s="4" t="str">
+        <x:v>Simple wraps, metal chainmail and practical metal-based wear with minimal fur</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:v>Chainmail already has an item-family entry; no duplicate mail item or cloth input added.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03744211789c450e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb98a99993c514421"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10354,7 +10453,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>134 design entries: 18 existing item IDs and 116 design concepts. Eight gemstone families are brainstorming candidates; only gemstone existence is established by this direction.</x:v>
+        <x:v>135 design entries: 18 existing item IDs and 117 design concepts. Simple wraps are the new everyday-wear entry; existing chainmail is reused. Three fashion-garment entries explicitly describe elaborate wear.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -10874,7 +10973,7 @@
         <x:v>Fashion scarcity</x:v>
       </x:c>
       <x:c r="B73" s="4" t="str">
-        <x:v>Fashion items are very rare and expensive because production consumes very large quantities of material and very large amounts of time; hide/fur conversion remains extremely low yield.</x:v>
+        <x:v>Elaborate fashion clothing is very rare and expensive because production consumes very large quantities of material/time. Ordinary simple wraps and metal-based wear with minimal fur are the everyday baseline.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="70" customHeight="1">
@@ -10949,10 +11048,34 @@
         <x:v>Game deposits could be exposed ancient mineral-bearing strata. These concepts add no present-day water cycle, plant gem source, terrain generation or special elemental powers.</x:v>
       </x:c>
     </x:row>
+    <x:row r="83" ht="70" customHeight="1">
+      <x:c r="A83" s="4" t="str">
+        <x:v>Everyday clothing baseline</x:v>
+      </x:c>
+      <x:c r="B83" s="4" t="str">
+        <x:v>Ordinary clothing includes simple wraps, metal chainmail and practical metal-based wear with minimal fur. No ordinary-wear price/rarity numbers or cloth supply are introduced.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="70" customHeight="1">
+      <x:c r="A84" s="4" t="str">
+        <x:v>Fashion distinction</x:v>
+      </x:c>
+      <x:c r="B84" s="4" t="str">
+        <x:v>Elaborate husk-fiber/fur/hide garments retain very rare, expensive fashion status. The same material family can support sparse ordinary use and high-input luxury workmanship.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="70" customHeight="1">
+      <x:c r="A85" s="4" t="str">
+        <x:v>No duplicate chainmail</x:v>
+      </x:c>
+      <x:c r="B85" s="4" t="str">
+        <x:v>The existing chainmail-shirt family now records everyday use; only simple wraps adds a master entry. Equipment patterns, fit, protection and runtime slots remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304b902371224a1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa0b1526190d4383"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11796,7 +11919,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f3c66835ce94565"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84e3a1974c494412"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12039,7 +12162,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cebd52385c84789"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70bb47da346b40b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12443,7 +12566,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R061ce0042b42449e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55908b29a6804d8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13119,7 +13242,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fd53b0ee1664203"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd676b9e52a364515"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add wing shade resources cheap shell and canister economy concepts
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R7d8c70ce9d124981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rf01557ecfe454c92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R48d4ccdb42b845b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rc6c9d63612734444"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R282df88cc1b2428f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R838ab625eee54ebe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R7f9ada08577d4c49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R411f56eeacc84545"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R47b9cf5d70404141"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R319b00919f9547ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R11ebf62b31b44cac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rd97c21860168434a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Re7809c16e9fb492e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R584a453dec2e41da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R69d4cffcbfb84576"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R961cfe3b4f4845df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R8a8713b3bf284b05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R371b5e68f236432b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R103e454549a84d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R82d8682a3185403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="Rbc4adb0d2c654907"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +56,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="28">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -192,6 +193,11 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF423B35"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -205,7 +211,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="52">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -369,6 +375,12 @@
     <x:xf numFmtId="0" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -431,7 +443,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V140" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V157" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -478,6 +490,22 @@
 </x:table>
 </file>
 
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="CanisterConceptsTable" displayName="CanisterConceptsTable" ref="A5:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Concept ID"/>
+    <x:tableColumn id="2" name="Part / item"/>
+    <x:tableColumn id="3" name="Category"/>
+    <x:tableColumn id="4" name="Proposed role"/>
+    <x:tableColumn id="5" name="Source relationship"/>
+    <x:tableColumn id="6" name="Material candidates"/>
+    <x:tableColumn id="7" name="Compatibility / boundary"/>
+    <x:tableColumn id="8" name="Source proposal"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="VariantsTable" displayName="VariantsTable" ref="A5:M25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
@@ -517,7 +545,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -529,7 +557,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B85" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -1659,7 +1687,7 @@
       <x:c r="R17" s="17"/>
       <x:c r="S17" s="17"/>
       <x:c r="T17" s="4" t="str">
-        <x:v>Final camp kit and upgrade design</x:v>
+        <x:v>Final camp kit and upgrade design; author shade-material direction: delicate inner wings. Existing prototype art/recipe unchanged; no duplicate shade item.</x:v>
       </x:c>
       <x:c r="U17" s="11"/>
       <x:c r="V17" s="4" t="str">
@@ -2848,10 +2876,10 @@
         <x:v>Molted exoskeleton</x:v>
       </x:c>
       <x:c r="E40" s="9" t="str">
-        <x:v>New proposal</x:v>
+        <x:v>User direction; not implemented</x:v>
       </x:c>
       <x:c r="F40" s="9" t="str">
-        <x:v>Source of abundant scraped chitin and icore fibers; possible structural plate uses.</x:v>
+        <x:v>Cheap raw shell/husk material; source of scraped fibers and candidate basic casing/guards.</x:v>
       </x:c>
       <x:c r="G40" s="9" t="str">
         <x:v>None</x:v>
@@ -2879,11 +2907,11 @@
       <x:c r="R40" s="22"/>
       <x:c r="S40" s="22"/>
       <x:c r="T40" s="9" t="str">
-        <x:v>Species-specific shell properties and structural uses remain proposals</x:v>
+        <x:v>Ordinary raw shells are cheap bulk material. Processed fibers, exceptional selected material and precision finished parts have separate value; no numeric price set.</x:v>
       </x:c>
       <x:c r="U40" s="23"/>
       <x:c r="V40" s="9" t="str">
-        <x:v>Docs/WORLD_BASIS.md#material-culture; author direction October 14, 2026. Process details and specific product forms remain unimplemented.</x:v>
+        <x:v>Direct author direction October 14, 2026; Docs/WORLD_BASIS.md#material-culture</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="66" customHeight="1">
@@ -8102,6 +8130,890 @@
       <x:c r="U140" s="11"/>
       <x:c r="V140" s="9" t="str">
         <x:v>Direct author clarification, October 14, 2026; Docs/WORLD_BASIS.md#material-culture. Ordinary wear: simple wraps, metal chainmail and practical metal-based pieces with minimal fur. Elaborate fashion remains rare/expensive; no cloth.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="95" customHeight="1">
+      <x:c r="A141" s="9" t="str">
+        <x:v>proposal.bio.inner_wing</x:v>
+      </x:c>
+      <x:c r="B141" s="9" t="str">
+        <x:v>Delicate inner wing</x:v>
+      </x:c>
+      <x:c r="C141" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D141" s="9" t="str">
+        <x:v>Wing material</x:v>
+      </x:c>
+      <x:c r="E141" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F141" s="9" t="str">
+        <x:v>Gathered insectoid megafauna inner-wing membrane for vertical sun shades.</x:v>
+      </x:c>
+      <x:c r="G141" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H141" s="9" t="str">
+        <x:v>Raw resource: Legger / local storage</x:v>
+      </x:c>
+      <x:c r="I141" s="13"/>
+      <x:c r="J141" s="15"/>
+      <x:c r="K141" s="9" t="str">
+        <x:v>Megafauna inner wings; collection details TBD</x:v>
+      </x:c>
+      <x:c r="L141" s="9" t="str">
+        <x:v>Prepare/join into shade panels; method and yield undefined</x:v>
+      </x:c>
+      <x:c r="M141" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N141" s="9" t="str">
+        <x:v>Delicate resource; no automatic opacity, heat resistance, structural strength or cloth properties assigned.</x:v>
+      </x:c>
+      <x:c r="O141" s="17"/>
+      <x:c r="P141" s="17"/>
+      <x:c r="Q141" s="17"/>
+      <x:c r="R141" s="17"/>
+      <x:c r="S141" s="17"/>
+      <x:c r="T141" s="9" t="str">
+        <x:v>Vertical sun-shade material by author direction; value and processing work remain unspecified.</x:v>
+      </x:c>
+      <x:c r="U141" s="11"/>
+      <x:c r="V141" s="9" t="str">
+        <x:v>Direct author direction October 14, 2026; Docs/WORLD_BASIS.md#material-culture</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="95" customHeight="1">
+      <x:c r="A142" s="9" t="str">
+        <x:v>proposal.bio.wing_panel</x:v>
+      </x:c>
+      <x:c r="B142" s="9" t="str">
+        <x:v>Prepared wing shade panel</x:v>
+      </x:c>
+      <x:c r="C142" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D142" s="9" t="str">
+        <x:v>Wing material</x:v>
+      </x:c>
+      <x:c r="E142" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F142" s="9" t="str">
+        <x:v>Prepared inner-wing material for an assembled vertical sun shade.</x:v>
+      </x:c>
+      <x:c r="G142" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H142" s="9" t="str">
+        <x:v>Component carrier eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I142" s="13"/>
+      <x:c r="J142" s="15"/>
+      <x:c r="K142" s="9" t="str">
+        <x:v>Process delicate inner wings; exact method undecided</x:v>
+      </x:c>
+      <x:c r="L142" s="9" t="str">
+        <x:v>Candidate input for existing popup-camp shade; no recipe authored</x:v>
+      </x:c>
+      <x:c r="M142" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N142" s="9" t="str">
+        <x:v>Panel preparation, joining, frame support and actual shade properties need design; no cloth assumed.</x:v>
+      </x:c>
+      <x:c r="O142" s="17"/>
+      <x:c r="P142" s="17"/>
+      <x:c r="Q142" s="17"/>
+      <x:c r="R142" s="17"/>
+      <x:c r="S142" s="17"/>
+      <x:c r="T142" s="9" t="str">
+        <x:v>Proposed intermediate product; reuse existing popup-camp item instead of duplicating the deployed shade.</x:v>
+      </x:c>
+      <x:c r="U142" s="11"/>
+      <x:c r="V142" s="9" t="str">
+        <x:v>New game proposal derived from author wing-resource direction October 14, 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="95" customHeight="1">
+      <x:c r="A143" s="9" t="str">
+        <x:v>proposal.canister.body_blank</x:v>
+      </x:c>
+      <x:c r="B143" s="9" t="str">
+        <x:v>Canister body blank</x:v>
+      </x:c>
+      <x:c r="C143" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D143" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E143" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F143" s="9" t="str">
+        <x:v>Unfinished body for specialist assembly</x:v>
+      </x:c>
+      <x:c r="G143" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H143" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I143" s="13"/>
+      <x:c r="J143" s="15"/>
+      <x:c r="K143" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L143" s="9" t="str">
+        <x:v>Proposed material: Worked metal/alloy choice TBD; shell outer casing possible</x:v>
+      </x:c>
+      <x:c r="M143" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N143" s="9" t="str">
+        <x:v>Personal life-support canister and raw-chemical vessel are distinct service roles</x:v>
+      </x:c>
+      <x:c r="O143" s="17"/>
+      <x:c r="P143" s="17"/>
+      <x:c r="Q143" s="17"/>
+      <x:c r="R143" s="17"/>
+      <x:c r="S143" s="17"/>
+      <x:c r="T143" s="9" t="str">
+        <x:v>Source explicitly distinguishes body fabrication. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U143" s="11"/>
+      <x:c r="V143" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="95" customHeight="1">
+      <x:c r="A144" s="9" t="str">
+        <x:v>proposal.canister.seal_ring</x:v>
+      </x:c>
+      <x:c r="B144" s="9" t="str">
+        <x:v>Replacement seal ring</x:v>
+      </x:c>
+      <x:c r="C144" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D144" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E144" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F144" s="9" t="str">
+        <x:v>Replaceable fitted sealing part</x:v>
+      </x:c>
+      <x:c r="G144" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H144" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I144" s="13"/>
+      <x:c r="J144" s="15"/>
+      <x:c r="K144" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L144" s="9" t="str">
+        <x:v>Proposed material: Biological/mineral elastic material candidate; formulation TBD</x:v>
+      </x:c>
+      <x:c r="M144" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N144" s="9" t="str">
+        <x:v>Seal diameter, compound and service must match; ancient synthetic input not universally required</x:v>
+      </x:c>
+      <x:c r="O144" s="17"/>
+      <x:c r="P144" s="17"/>
+      <x:c r="Q144" s="17"/>
+      <x:c r="R144" s="17"/>
+      <x:c r="S144" s="17"/>
+      <x:c r="T144" s="9" t="str">
+        <x:v>Source explicitly describes replaceable seal systems. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U144" s="11"/>
+      <x:c r="V144" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="95" customHeight="1">
+      <x:c r="A145" s="9" t="str">
+        <x:v>proposal.canister.seal_seat</x:v>
+      </x:c>
+      <x:c r="B145" s="9" t="str">
+        <x:v>Fitted seal seat</x:v>
+      </x:c>
+      <x:c r="C145" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D145" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E145" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F145" s="9" t="str">
+        <x:v>Precision contact surface supporting a seal</x:v>
+      </x:c>
+      <x:c r="G145" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H145" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I145" s="13"/>
+      <x:c r="J145" s="15"/>
+      <x:c r="K145" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L145" s="9" t="str">
+        <x:v>Proposed material: Worked metal or compatible hard insert TBD</x:v>
+      </x:c>
+      <x:c r="M145" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N145" s="9" t="str">
+        <x:v>A seat supports the seal; not a duplicate compression collar or replacement ring</x:v>
+      </x:c>
+      <x:c r="O145" s="17"/>
+      <x:c r="P145" s="17"/>
+      <x:c r="Q145" s="17"/>
+      <x:c r="R145" s="17"/>
+      <x:c r="S145" s="17"/>
+      <x:c r="T145" s="9" t="str">
+        <x:v>New explicit part derived from source seal-system precision. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U145" s="11"/>
+      <x:c r="V145" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="95" customHeight="1">
+      <x:c r="A146" s="9" t="str">
+        <x:v>proposal.canister.sealant</x:v>
+      </x:c>
+      <x:c r="B146" s="9" t="str">
+        <x:v>Canister joint sealant</x:v>
+      </x:c>
+      <x:c r="C146" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D146" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E146" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F146" s="9" t="str">
+        <x:v>Prepared compound for compatible joints</x:v>
+      </x:c>
+      <x:c r="G146" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H146" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I146" s="13"/>
+      <x:c r="J146" s="15"/>
+      <x:c r="K146" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L146" s="9" t="str">
+        <x:v>Proposed material: Compatible biological/mineral binder formulation TBD</x:v>
+      </x:c>
+      <x:c r="M146" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N146" s="9" t="str">
+        <x:v>Not interchangeable with glue, toxic shell binder or a failed pressure seal; exact applications unresolved</x:v>
+      </x:c>
+      <x:c r="O146" s="17"/>
+      <x:c r="P146" s="17"/>
+      <x:c r="Q146" s="17"/>
+      <x:c r="R146" s="17"/>
+      <x:c r="S146" s="17"/>
+      <x:c r="T146" s="9" t="str">
+        <x:v>Author requests sealant; source describes biological seal compounds. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U146" s="11"/>
+      <x:c r="V146" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="95" customHeight="1">
+      <x:c r="A147" s="9" t="str">
+        <x:v>proposal.canister.feed_line</x:v>
+      </x:c>
+      <x:c r="B147" s="9" t="str">
+        <x:v>Feed-line section</x:v>
+      </x:c>
+      <x:c r="C147" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D147" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E147" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F147" s="9" t="str">
+        <x:v>Replacement contained conduit for a personal canister</x:v>
+      </x:c>
+      <x:c r="G147" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H147" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I147" s="13"/>
+      <x:c r="J147" s="15"/>
+      <x:c r="K147" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L147" s="9" t="str">
+        <x:v>Proposed material: Flexible biological/mineral component or recovered part TBD</x:v>
+      </x:c>
+      <x:c r="M147" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N147" s="9" t="str">
+        <x:v>No ordinary rubber/cloth or new respiratory system assumed; service and purity matter</x:v>
+      </x:c>
+      <x:c r="O147" s="17"/>
+      <x:c r="P147" s="17"/>
+      <x:c r="Q147" s="17"/>
+      <x:c r="R147" s="17"/>
+      <x:c r="S147" s="17"/>
+      <x:c r="T147" s="9" t="str">
+        <x:v>Source explicitly describes feed-line routing and material quality. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U147" s="11"/>
+      <x:c r="V147" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="95" customHeight="1">
+      <x:c r="A148" s="9" t="str">
+        <x:v>proposal.canister.coupling</x:v>
+      </x:c>
+      <x:c r="B148" s="9" t="str">
+        <x:v>Feed-line coupling</x:v>
+      </x:c>
+      <x:c r="C148" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D148" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E148" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F148" s="9" t="str">
+        <x:v>Connect a line to a matching canister/interface</x:v>
+      </x:c>
+      <x:c r="G148" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H148" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I148" s="13"/>
+      <x:c r="J148" s="15"/>
+      <x:c r="K148" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L148" s="9" t="str">
+        <x:v>Proposed material: Machined metal with qualified sealing insert TBD</x:v>
+      </x:c>
+      <x:c r="M148" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N148" s="9" t="str">
+        <x:v>Match intended service; not a generic connector for every toxic liquid</x:v>
+      </x:c>
+      <x:c r="O148" s="17"/>
+      <x:c r="P148" s="17"/>
+      <x:c r="Q148" s="17"/>
+      <x:c r="R148" s="17"/>
+      <x:c r="S148" s="17"/>
+      <x:c r="T148" s="9" t="str">
+        <x:v>New explicit fitting from source connection systems. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U148" s="11"/>
+      <x:c r="V148" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="95" customHeight="1">
+      <x:c r="A149" s="9" t="str">
+        <x:v>proposal.canister.mouthpiece</x:v>
+      </x:c>
+      <x:c r="B149" s="9" t="str">
+        <x:v>Canister mouthpiece interface</x:v>
+      </x:c>
+      <x:c r="C149" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D149" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E149" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F149" s="9" t="str">
+        <x:v>Personal delivery interface candidate</x:v>
+      </x:c>
+      <x:c r="G149" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H149" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I149" s="13"/>
+      <x:c r="J149" s="15"/>
+      <x:c r="K149" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L149" s="9" t="str">
+        <x:v>Proposed material: Qualified body-contact material TBD</x:v>
+      </x:c>
+      <x:c r="M149" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N149" s="9" t="str">
+        <x:v>Game algae-use and breathing systems are unchanged; anatomy and hygiene design needed</x:v>
+      </x:c>
+      <x:c r="O149" s="17"/>
+      <x:c r="P149" s="17"/>
+      <x:c r="Q149" s="17"/>
+      <x:c r="R149" s="17"/>
+      <x:c r="S149" s="17"/>
+      <x:c r="T149" s="9" t="str">
+        <x:v>Source describes mouthpiece/collar interfaces. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U149" s="11"/>
+      <x:c r="V149" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="95" customHeight="1">
+      <x:c r="A150" s="9" t="str">
+        <x:v>proposal.canister.window</x:v>
+      </x:c>
+      <x:c r="B150" s="9" t="str">
+        <x:v>Canister viewing-port insert</x:v>
+      </x:c>
+      <x:c r="C150" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D150" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E150" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F150" s="9" t="str">
+        <x:v>Inspect a compatible interior without opening it</x:v>
+      </x:c>
+      <x:c r="G150" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H150" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I150" s="13"/>
+      <x:c r="J150" s="15"/>
+      <x:c r="K150" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L150" s="9" t="str">
+        <x:v>Proposed material: Clear glass and fitted retaining seat</x:v>
+      </x:c>
+      <x:c r="M150" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N150" s="9" t="str">
+        <x:v>Clear glass craft cost; no automatic fill sensor, pressure certification or new HUD</x:v>
+      </x:c>
+      <x:c r="O150" s="17"/>
+      <x:c r="P150" s="17"/>
+      <x:c r="Q150" s="17"/>
+      <x:c r="R150" s="17"/>
+      <x:c r="S150" s="17"/>
+      <x:c r="T150" s="9" t="str">
+        <x:v>Glass source and canister craft describe viewing ports. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U150" s="11"/>
+      <x:c r="V150" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="95" customHeight="1">
+      <x:c r="A151" s="9" t="str">
+        <x:v>proposal.canister.mount</x:v>
+      </x:c>
+      <x:c r="B151" s="9" t="str">
+        <x:v>Canister mounting bracket</x:v>
+      </x:c>
+      <x:c r="C151" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D151" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E151" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F151" s="9" t="str">
+        <x:v>Attach one canister to a fitted carrier</x:v>
+      </x:c>
+      <x:c r="G151" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H151" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I151" s="13"/>
+      <x:c r="J151" s="15"/>
+      <x:c r="K151" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L151" s="9" t="str">
+        <x:v>Proposed material: Metal bracket and retainers</x:v>
+      </x:c>
+      <x:c r="M151" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N151" s="9" t="str">
+        <x:v>Coexist with armor, cloak, backpack, magnets and grounding equipment; no new slot authority</x:v>
+      </x:c>
+      <x:c r="O151" s="17"/>
+      <x:c r="P151" s="17"/>
+      <x:c r="Q151" s="17"/>
+      <x:c r="R151" s="17"/>
+      <x:c r="S151" s="17"/>
+      <x:c r="T151" s="9" t="str">
+        <x:v>Source explicitly separates fitments from body/seal. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U151" s="11"/>
+      <x:c r="V151" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="95" customHeight="1">
+      <x:c r="A152" s="9" t="str">
+        <x:v>proposal.canister.harness</x:v>
+      </x:c>
+      <x:c r="B152" s="9" t="str">
+        <x:v>Fitted canister harness</x:v>
+      </x:c>
+      <x:c r="C152" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D152" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E152" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F152" s="9" t="str">
+        <x:v>Wear a canister in a selected carry arrangement</x:v>
+      </x:c>
+      <x:c r="G152" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H152" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I152" s="13"/>
+      <x:c r="J152" s="15"/>
+      <x:c r="K152" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L152" s="9" t="str">
+        <x:v>Proposed material: Metal/shell carrier; minimal-fur contact material or difficult husk material proposed</x:v>
+      </x:c>
+      <x:c r="M152" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N152" s="9" t="str">
+        <x:v>Exact harness material and capacities unresolved; no cloth straps or changed trial equipment slots</x:v>
+      </x:c>
+      <x:c r="O152" s="17"/>
+      <x:c r="P152" s="17"/>
+      <x:c r="Q152" s="17"/>
+      <x:c r="R152" s="17"/>
+      <x:c r="S152" s="17"/>
+      <x:c r="T152" s="9" t="str">
+        <x:v>Source chest/hip/back/cross-body carry styles. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U152" s="11"/>
+      <x:c r="V152" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="95" customHeight="1">
+      <x:c r="A153" s="9" t="str">
+        <x:v>proposal.canister.inspection_gauge</x:v>
+      </x:c>
+      <x:c r="B153" s="9" t="str">
+        <x:v>Seal inspection gauge</x:v>
+      </x:c>
+      <x:c r="C153" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D153" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E153" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F153" s="9" t="str">
+        <x:v>Specialist workshop inspection aid</x:v>
+      </x:c>
+      <x:c r="G153" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H153" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I153" s="13"/>
+      <x:c r="J153" s="15"/>
+      <x:c r="K153" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L153" s="9" t="str">
+        <x:v>Proposed material: Precision metal/glass tool candidate</x:v>
+      </x:c>
+      <x:c r="M153" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N153" s="9" t="str">
+        <x:v>No numerical pressure behavior or mandatory recurring inspection chore introduced</x:v>
+      </x:c>
+      <x:c r="O153" s="17"/>
+      <x:c r="P153" s="17"/>
+      <x:c r="Q153" s="17"/>
+      <x:c r="R153" s="17"/>
+      <x:c r="S153" s="17"/>
+      <x:c r="T153" s="9" t="str">
+        <x:v>New tool idea inspired by source seal checks/testing. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U153" s="11"/>
+      <x:c r="V153" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/daily-ritual.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="95" customHeight="1">
+      <x:c r="A154" s="9" t="str">
+        <x:v>proposal.canister.service_kit</x:v>
+      </x:c>
+      <x:c r="B154" s="9" t="str">
+        <x:v>Canister service kit</x:v>
+      </x:c>
+      <x:c r="C154" s="9" t="str">
+        <x:v>Field supplies</x:v>
+      </x:c>
+      <x:c r="D154" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E154" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F154" s="9" t="str">
+        <x:v>Carry a selected set of compatible spare seals/fittings</x:v>
+      </x:c>
+      <x:c r="G154" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H154" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I154" s="13"/>
+      <x:c r="J154" s="15"/>
+      <x:c r="K154" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L154" s="9" t="str">
+        <x:v>Proposed material: Existing candidate parts in a fitted case</x:v>
+      </x:c>
+      <x:c r="M154" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N154" s="9" t="str">
+        <x:v>Bundle contents count once and occupy finite capacity; recipe/quantity and repair action unapproved</x:v>
+      </x:c>
+      <x:c r="O154" s="17"/>
+      <x:c r="P154" s="17"/>
+      <x:c r="Q154" s="17"/>
+      <x:c r="R154" s="17"/>
+      <x:c r="S154" s="17"/>
+      <x:c r="T154" s="9" t="str">
+        <x:v>Source caravan carry includes repair kits/spare seals. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U154" s="11"/>
+      <x:c r="V154" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="95" customHeight="1">
+      <x:c r="A155" s="9" t="str">
+        <x:v>proposal.canister.maker_plate</x:v>
+      </x:c>
+      <x:c r="B155" s="9" t="str">
+        <x:v>Canister maker plate</x:v>
+      </x:c>
+      <x:c r="C155" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D155" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E155" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F155" s="9" t="str">
+        <x:v>Visible craft provenance or personal decoration</x:v>
+      </x:c>
+      <x:c r="G155" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H155" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I155" s="13"/>
+      <x:c r="J155" s="15"/>
+      <x:c r="K155" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L155" s="9" t="str">
+        <x:v>Proposed material: Engraved metal; exact format TBD</x:v>
+      </x:c>
+      <x:c r="M155" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N155" s="9" t="str">
+        <x:v>Not functional seal quality, an achievement award or a verified authenticity system by itself</x:v>
+      </x:c>
+      <x:c r="O155" s="17"/>
+      <x:c r="P155" s="17"/>
+      <x:c r="Q155" s="17"/>
+      <x:c r="R155" s="17"/>
+      <x:c r="S155" s="17"/>
+      <x:c r="T155" s="9" t="str">
+        <x:v>Source guild marks and maker reputation. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U155" s="11"/>
+      <x:c r="V155" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister-identity.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="95" customHeight="1">
+      <x:c r="A156" s="9" t="str">
+        <x:v>proposal.canister.trim</x:v>
+      </x:c>
+      <x:c r="B156" s="9" t="str">
+        <x:v>Decorative canister panel</x:v>
+      </x:c>
+      <x:c r="C156" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D156" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E156" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F156" s="9" t="str">
+        <x:v>Nonstructural custom finish candidate</x:v>
+      </x:c>
+      <x:c r="G156" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H156" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I156" s="13"/>
+      <x:c r="J156" s="15"/>
+      <x:c r="K156" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L156" s="9" t="str">
+        <x:v>Proposed material: Worked metal/shell; fashion-grade inlay optional</x:v>
+      </x:c>
+      <x:c r="M156" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N156" s="9" t="str">
+        <x:v>Decoration remains separate from seal/body functionality; material requirements and price TBD</x:v>
+      </x:c>
+      <x:c r="O156" s="17"/>
+      <x:c r="P156" s="17"/>
+      <x:c r="Q156" s="17"/>
+      <x:c r="R156" s="17"/>
+      <x:c r="S156" s="17"/>
+      <x:c r="T156" s="9" t="str">
+        <x:v>Source engravings, surface work and identity. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U156" s="11"/>
+      <x:c r="V156" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister-identity.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="95" customHeight="1">
+      <x:c r="A157" s="9" t="str">
+        <x:v>proposal.canister.endcap</x:v>
+      </x:c>
+      <x:c r="B157" s="9" t="str">
+        <x:v>Canister protective endcap</x:v>
+      </x:c>
+      <x:c r="C157" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D157" s="9" t="str">
+        <x:v>Canister economy concept</x:v>
+      </x:c>
+      <x:c r="E157" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F157" s="9" t="str">
+        <x:v>Outer impact/dust guard candidate</x:v>
+      </x:c>
+      <x:c r="G157" s="9" t="str">
+        <x:v>Unassigned; part/fit ownership TBD</x:v>
+      </x:c>
+      <x:c r="H157" s="9" t="str">
+        <x:v>Resource/component cargo or permitted Booter kit; policy TBD</x:v>
+      </x:c>
+      <x:c r="I157" s="13"/>
+      <x:c r="J157" s="15"/>
+      <x:c r="K157" s="9" t="str">
+        <x:v>Specialist craft/trade/service candidate; no recipe authored</x:v>
+      </x:c>
+      <x:c r="L157" s="9" t="str">
+        <x:v>Proposed material: Cheap shell outer guard or metal form proposed</x:v>
+      </x:c>
+      <x:c r="M157" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N157" s="9" t="str">
+        <x:v>Protective casing is not a pressure seal; no damage/breakage simulation approved</x:v>
+      </x:c>
+      <x:c r="O157" s="17"/>
+      <x:c r="P157" s="17"/>
+      <x:c r="Q157" s="17"/>
+      <x:c r="R157" s="17"/>
+      <x:c r="S157" s="17"/>
+      <x:c r="T157" s="9" t="str">
+        <x:v>New part inspired by source protective deep-operation casing. Source systems are proposals; precision skill and suitable material may affect value, but no prices or lifetime values assigned.</x:v>
+      </x:c>
+      <x:c r="U157" s="11"/>
+      <x:c r="V157" s="9" t="str">
+        <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8127,7 +9039,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7406d226711453b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra96a3825c6364c08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8779,7 +9691,489 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36a2655abdf04317"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R049954675f444f3d"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="35" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="55" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="65" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="82" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="115" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Canister parts, service and craft</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="1" t="str">
+        <x:v>New item proposals from source drafts. Existing algae/dust canisters and gameplay remain unchanged.</x:v>
+      </x:c>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="51" t="str">
+        <x:v>Concept ID</x:v>
+      </x:c>
+      <x:c r="B5" s="51" t="str">
+        <x:v>Part / item</x:v>
+      </x:c>
+      <x:c r="C5" s="51" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="D5" s="51" t="str">
+        <x:v>Proposed role</x:v>
+      </x:c>
+      <x:c r="E5" s="51" t="str">
+        <x:v>Source relationship</x:v>
+      </x:c>
+      <x:c r="F5" s="51" t="str">
+        <x:v>Material candidates</x:v>
+      </x:c>
+      <x:c r="G5" s="51" t="str">
+        <x:v>Compatibility / boundary</x:v>
+      </x:c>
+      <x:c r="H5" s="51" t="str">
+        <x:v>Source proposal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="95" customHeight="1">
+      <x:c r="A6" s="4" t="str">
+        <x:v>proposal.canister.body_blank</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>Canister body blank</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>Unfinished body for specialist assembly</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>Source explicitly distinguishes body fabrication</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>Worked metal/alloy choice TBD; shell outer casing possible</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="str">
+        <x:v>Personal life-support canister and raw-chemical vessel are distinct service roles</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="95" customHeight="1">
+      <x:c r="A7" s="4" t="str">
+        <x:v>proposal.canister.seal_ring</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>Replacement seal ring</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>Replaceable fitted sealing part</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>Source explicitly describes replaceable seal systems</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>Biological/mineral elastic material candidate; formulation TBD</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="str">
+        <x:v>Seal diameter, compound and service must match; ancient synthetic input not universally required</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="95" customHeight="1">
+      <x:c r="A8" s="4" t="str">
+        <x:v>proposal.canister.seal_seat</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>Fitted seal seat</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>Precision contact surface supporting a seal</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>New explicit part derived from source seal-system precision</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>Worked metal or compatible hard insert TBD</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="str">
+        <x:v>A seat supports the seal; not a duplicate compression collar or replacement ring</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="95" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>proposal.canister.sealant</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>Canister joint sealant</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Prepared compound for compatible joints</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Author requests sealant; source describes biological seal compounds</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>Compatible biological/mineral binder formulation TBD</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="str">
+        <x:v>Not interchangeable with glue, toxic shell binder or a failed pressure seal; exact applications unresolved</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="95" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>proposal.canister.feed_line</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>Feed-line section</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Replacement contained conduit for a personal canister</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>Source explicitly describes feed-line routing and material quality</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>Flexible biological/mineral component or recovered part TBD</x:v>
+      </x:c>
+      <x:c r="G10" s="4" t="str">
+        <x:v>No ordinary rubber/cloth or new respiratory system assumed; service and purity matter</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="95" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>proposal.canister.coupling</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>Feed-line coupling</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>Connect a line to a matching canister/interface</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>New explicit fitting from source connection systems</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>Machined metal with qualified sealing insert TBD</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str">
+        <x:v>Match intended service; not a generic connector for every toxic liquid</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="95" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>proposal.canister.mouthpiece</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>Canister mouthpiece interface</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>Personal delivery interface candidate</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>Source describes mouthpiece/collar interfaces</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>Qualified body-contact material TBD</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="str">
+        <x:v>Game algae-use and breathing systems are unchanged; anatomy and hygiene design needed</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="95" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>proposal.canister.window</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>Canister viewing-port insert</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Inspect a compatible interior without opening it</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>Glass source and canister craft describe viewing ports</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>Clear glass and fitted retaining seat</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>Clear glass craft cost; no automatic fill sensor, pressure certification or new HUD</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/glass.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="95" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>proposal.canister.mount</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>Canister mounting bracket</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>Attach one canister to a fitted carrier</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>Source explicitly separates fitments from body/seal</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>Metal bracket and retainers</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="str">
+        <x:v>Coexist with armor, cloak, backpack, magnets and grounding equipment; no new slot authority</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/caster-craft.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="95" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>proposal.canister.harness</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>Fitted canister harness</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Wear a canister in a selected carry arrangement</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>Source chest/hip/back/cross-body carry styles</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>Metal/shell carrier; minimal-fur contact material or difficult husk material proposed</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>Exact harness material and capacities unresolved; no cloth straps or changed trial equipment slots</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="95" customHeight="1">
+      <x:c r="A16" s="4" t="str">
+        <x:v>proposal.canister.inspection_gauge</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>Seal inspection gauge</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Specialist workshop inspection aid</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>New tool idea inspired by source seal checks/testing</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>Precision metal/glass tool candidate</x:v>
+      </x:c>
+      <x:c r="G16" s="4" t="str">
+        <x:v>No numerical pressure behavior or mandatory recurring inspection chore introduced</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/daily-ritual.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="95" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>proposal.canister.service_kit</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>Canister service kit</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>Field supplies</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Carry a selected set of compatible spare seals/fittings</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Source caravan carry includes repair kits/spare seals</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>Existing candidate parts in a fitted case</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>Bundle contents count once and occupy finite capacity; recipe/quantity and repair action unapproved</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="95" customHeight="1">
+      <x:c r="A18" s="4" t="str">
+        <x:v>proposal.canister.maker_plate</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>Canister maker plate</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>Visible craft provenance or personal decoration</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>Source guild marks and maker reputation</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>Engraved metal; exact format TBD</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="str">
+        <x:v>Not functional seal quality, an achievement award or a verified authenticity system by itself</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister-identity.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="95" customHeight="1">
+      <x:c r="A19" s="4" t="str">
+        <x:v>proposal.canister.trim</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>Decorative canister panel</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Nonstructural custom finish candidate</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>Source engravings, surface work and identity</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="str">
+        <x:v>Worked metal/shell; fashion-grade inlay optional</x:v>
+      </x:c>
+      <x:c r="G19" s="4" t="str">
+        <x:v>Decoration remains separate from seal/body functionality; material requirements and price TBD</x:v>
+      </x:c>
+      <x:c r="H19" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister-identity.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="95" customHeight="1">
+      <x:c r="A20" s="4" t="str">
+        <x:v>proposal.canister.endcap</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>Canister protective endcap</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>Outer impact/dust guard candidate</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>New part inspired by source protective deep-operation casing</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="str">
+        <x:v>Cheap shell outer guard or metal form proposed</x:v>
+      </x:c>
+      <x:c r="G20" s="4" t="str">
+        <x:v>Protective casing is not a pressure seal; no damage/breakage simulation approved</x:v>
+      </x:c>
+      <x:c r="H20" s="4" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dcf33107c174b70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9687,7 +11081,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53746a952862460e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba2710e225b34293"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10053,7 +11447,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R568e319411824edf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4ee2e8d828a43ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10114,7 +11508,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>25</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>Existing gear plus armor, carriers, rare eyewear/headwear and very rare fashion families</x:v>
@@ -10129,7 +11523,7 @@
       </x:c>
       <x:c r="B7" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A7)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C7" s="4" t="str">
         <x:v>Pop-up camp and two battery states</x:v>
@@ -10144,7 +11538,7 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>76</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Minerals, biological resources, generic chemistry placeholders and twelve new chemical concepts</x:v>
@@ -10159,7 +11553,7 @@
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A9)</x:f>
-        <x:v>14</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>Existing salvage and proposed materials, including husk-fiber paper and difficult pressed textiles</x:v>
@@ -10387,10 +11781,40 @@
         <x:v>Chainmail already has an item-family entry; no duplicate mail item or cloth input added.</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="85" customHeight="1">
+      <x:c r="A25" s="4" t="str">
+        <x:v>Canister economy</x:v>
+      </x:c>
+      <x:c r="B25" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Canister economy concept")</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C25" s="4" t="str">
+        <x:v>Bodies, seals, seats, sealant, lines, couplings, mouthpieces, viewing inserts, mounts, harnesses, inspection/service and identity pieces</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>15 new proposals from source canister craft/carry/ritual records; no automatic air-reserve or maintenance simulation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="85" customHeight="1">
+      <x:c r="A26" s="4" t="str">
+        <x:v>Megafauna wing materials</x:v>
+      </x:c>
+      <x:c r="B26" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Wing material")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C26" s="4" t="str">
+        <x:v>Delicate inner wings and proposed prepared shade panels</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:v>Vertical shade uses the existing popup-camp family. Ordinary shells separately become cheap bulk resource.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb98a99993c514421"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61e6d6ccb016431b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10453,7 +11877,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>135 design entries: 18 existing item IDs and 117 design concepts. Simple wraps are the new everyday-wear entry; existing chainmail is reused. Three fashion-garment entries explicitly describe elaborate wear.</x:v>
+        <x:v>152 design entries: 18 existing item IDs and 134 design concepts. Added two wing-material concepts and fifteen canister-economy candidates; existing popup camp reused for vertical shades.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -11072,10 +12496,58 @@
         <x:v>The existing chainmail-shirt family now records everyday use; only simple wraps adds a master entry. Equipment patterns, fit, protection and runtime slots remain unimplemented.</x:v>
       </x:c>
     </x:row>
+    <x:row r="86" ht="75" customHeight="1">
+      <x:c r="A86" s="4" t="str">
+        <x:v>Wing sun shades</x:v>
+      </x:c>
+      <x:c r="B86" s="4" t="str">
+        <x:v>Author direction: delicate insectoid megafauna inner wings are resources for vertical sun shades. The prepared panel is a proposed intermediate; existing popup camp owns the shade item concept.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="75" customHeight="1">
+      <x:c r="A87" s="4" t="str">
+        <x:v>Cheap shells</x:v>
+      </x:c>
+      <x:c r="B87" s="4" t="str">
+        <x:v>Ordinary raw shells are cheap bulk material. Processing, selected fiber quality and skilled precision work can still produce valuable outputs. Raw-shell price and fashion-fiber value are separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="75" customHeight="1">
+      <x:c r="A88" s="4" t="str">
+        <x:v>Canister source status</x:v>
+      </x:c>
+      <x:c r="B88" s="4" t="str">
+        <x:v>Read WLD-0037/0038/0039/0044 and WLD-0016 at source revision f6f98515. These are proposals, including Phagia/air-reserve systems and seal materials; no automatic game adoption.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="75" customHeight="1">
+      <x:c r="A89" s="4" t="str">
+        <x:v>Seal distinctions</x:v>
+      </x:c>
+      <x:c r="B89" s="4" t="str">
+        <x:v>Seal rings, hard seats, closure collars, sealant and protective endcaps have different roles. Existing compression seal collar is reused conceptually; it is not duplicated as a new item.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="75" customHeight="1">
+      <x:c r="A90" s="4" t="str">
+        <x:v>Scarcity and service</x:v>
+      </x:c>
+      <x:c r="B90" s="4" t="str">
+        <x:v>Ancient synthetics remain extremely rare. Routine canister seals do not automatically require ancient material. No maintenance frequency, random failure, lifespan, pressure mechanic or recipe approved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="75" customHeight="1">
+      <x:c r="A91" s="4" t="str">
+        <x:v>Body and payload ownership</x:v>
+      </x:c>
+      <x:c r="B91" s="4" t="str">
+        <x:v>Personal survival canister, dust device and toxic-material vessel are distinct roles. Parts do not create extra liquid reserves, shared storage or duplicate owned canisters. All trial systems remain unchanged.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa0b1526190d4383"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34f33dbc0dfd4290"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11919,7 +13391,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84e3a1974c494412"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53bce0257e2043ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12162,7 +13634,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70bb47da346b40b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4616b48d5e0645f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12566,7 +14038,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55908b29a6804d8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fcf34cb044f4fe8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13242,7 +14714,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd676b9e52a364515"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc139173f1f464ff9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add cultural and everyday item proposals
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R11ebf62b31b44cac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rd97c21860168434a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Re7809c16e9fb492e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R584a453dec2e41da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R69d4cffcbfb84576"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R961cfe3b4f4845df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R8a8713b3bf284b05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R371b5e68f236432b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R103e454549a84d62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R82d8682a3185403c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="Rbc4adb0d2c654907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R192f4debe9b9491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R391de0ceb5614c7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R84bed178fb60476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rc122d9cfd57e44c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R0c8868e27bbd403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R4e373c608ef74687"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rb889f8f5ebb244b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R30c1c7f3817842c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Rc13d4d9e6b2c4a88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="Rfd7029adf03e4e00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R1eff6102dc824ebc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -443,7 +443,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V157" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ItemsTable" displayName="ItemsTable" ref="A5:V181" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -545,7 +545,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -557,7 +557,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B96" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -9016,6 +9016,1254 @@
         <x:v>New game item concept October 14, 2026. Source proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/carry-styles.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="158" ht="100" customHeight="1">
+      <x:c r="A158" s="9" t="str">
+        <x:v>proposal.culture.icon</x:v>
+      </x:c>
+      <x:c r="B158" s="9" t="str">
+        <x:v>Preserver icon token</x:v>
+      </x:c>
+      <x:c r="C158" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D158" s="9" t="str">
+        <x:v>Religious</x:v>
+      </x:c>
+      <x:c r="E158" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F158" s="9" t="str">
+        <x:v>Small devotional image carried or displayed</x:v>
+      </x:c>
+      <x:c r="G158" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H158" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I158" s="13"/>
+      <x:c r="J158" s="15"/>
+      <x:c r="K158" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L158" s="9" t="str">
+        <x:v>Material candidate: Stamped metal or carved shell</x:v>
+      </x:c>
+      <x:c r="M158" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N158" s="9" t="str">
+        <x:v>Symbolic object; no protective buff</x:v>
+      </x:c>
+      <x:c r="O158" s="17"/>
+      <x:c r="P158" s="17"/>
+      <x:c r="Q158" s="17"/>
+      <x:c r="R158" s="17"/>
+      <x:c r="S158" s="17"/>
+      <x:c r="T158" s="9" t="str">
+        <x:v>Plain stamped examples could be accessible; fine engraving is prestige work. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U158" s="11"/>
+      <x:c r="V158" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/religious-traditions.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="100" customHeight="1">
+      <x:c r="A159" s="9" t="str">
+        <x:v>proposal.culture.shrine</x:v>
+      </x:c>
+      <x:c r="B159" s="9" t="str">
+        <x:v>Household shrine plaque</x:v>
+      </x:c>
+      <x:c r="C159" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D159" s="9" t="str">
+        <x:v>Religious</x:v>
+      </x:c>
+      <x:c r="E159" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F159" s="9" t="str">
+        <x:v>Small fixed place for household remembrance and devotion</x:v>
+      </x:c>
+      <x:c r="G159" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H159" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I159" s="13"/>
+      <x:c r="J159" s="15"/>
+      <x:c r="K159" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L159" s="9" t="str">
+        <x:v>Material candidate: Shell backing and metal motif</x:v>
+      </x:c>
+      <x:c r="M159" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N159" s="9" t="str">
+        <x:v>Household object; no temple system assumed</x:v>
+      </x:c>
+      <x:c r="O159" s="17"/>
+      <x:c r="P159" s="17"/>
+      <x:c r="Q159" s="17"/>
+      <x:c r="R159" s="17"/>
+      <x:c r="S159" s="17"/>
+      <x:c r="T159" s="9" t="str">
+        <x:v>Simple versions versus elaborate commissioned pieces. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U159" s="11"/>
+      <x:c r="V159" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/religious-traditions.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="100" customHeight="1">
+      <x:c r="A160" s="9" t="str">
+        <x:v>proposal.culture.altar_vial</x:v>
+      </x:c>
+      <x:c r="B160" s="9" t="str">
+        <x:v>Altar display vial</x:v>
+      </x:c>
+      <x:c r="C160" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D160" s="9" t="str">
+        <x:v>Religious</x:v>
+      </x:c>
+      <x:c r="E160" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F160" s="9" t="str">
+        <x:v>Ceremonial display of a deliberately contained sacred sample</x:v>
+      </x:c>
+      <x:c r="G160" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H160" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I160" s="13"/>
+      <x:c r="J160" s="15"/>
+      <x:c r="K160" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L160" s="9" t="str">
+        <x:v>Material candidate: Fine sealed glass vessel and metal cradle</x:v>
+      </x:c>
+      <x:c r="M160" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N160" s="9" t="str">
+        <x:v>Source altar-vial concept; payload identity and viability unresolved; reuse vessel parts</x:v>
+      </x:c>
+      <x:c r="O160" s="17"/>
+      <x:c r="P160" s="17"/>
+      <x:c r="Q160" s="17"/>
+      <x:c r="R160" s="17"/>
+      <x:c r="S160" s="17"/>
+      <x:c r="T160" s="9" t="str">
+        <x:v>Fine glass and precision sealing suggest costly craftsmanship. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U160" s="11"/>
+      <x:c r="V160" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/religious-traditions.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="100" customHeight="1">
+      <x:c r="A161" s="9" t="str">
+        <x:v>proposal.culture.reliquary</x:v>
+      </x:c>
+      <x:c r="B161" s="9" t="str">
+        <x:v>Relic case</x:v>
+      </x:c>
+      <x:c r="C161" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D161" s="9" t="str">
+        <x:v>Religious</x:v>
+      </x:c>
+      <x:c r="E161" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F161" s="9" t="str">
+        <x:v>Protect and display a claimed ancestral relic</x:v>
+      </x:c>
+      <x:c r="G161" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H161" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I161" s="13"/>
+      <x:c r="J161" s="15"/>
+      <x:c r="K161" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L161" s="9" t="str">
+        <x:v>Material candidate: Metal or shell case; rare clear window optional</x:v>
+      </x:c>
+      <x:c r="M161" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N161" s="9" t="str">
+        <x:v>A claim of authenticity is not proof or a magical property</x:v>
+      </x:c>
+      <x:c r="O161" s="17"/>
+      <x:c r="P161" s="17"/>
+      <x:c r="Q161" s="17"/>
+      <x:c r="R161" s="17"/>
+      <x:c r="S161" s="17"/>
+      <x:c r="T161" s="9" t="str">
+        <x:v>Plain keepsake boxes through rare institutional commissions. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U161" s="11"/>
+      <x:c r="V161" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/spiritual-economy.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="100" customHeight="1">
+      <x:c r="A162" s="9" t="str">
+        <x:v>proposal.culture.prayer_leaf</x:v>
+      </x:c>
+      <x:c r="B162" s="9" t="str">
+        <x:v>Husk-paper prayer leaf</x:v>
+      </x:c>
+      <x:c r="C162" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D162" s="9" t="str">
+        <x:v>Religious</x:v>
+      </x:c>
+      <x:c r="E162" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F162" s="9" t="str">
+        <x:v>Portable prayers or devotional images</x:v>
+      </x:c>
+      <x:c r="G162" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H162" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I162" s="13"/>
+      <x:c r="J162" s="15"/>
+      <x:c r="K162" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L162" s="9" t="str">
+        <x:v>Material candidate: Scraped husk-fiber paper and mineral marking medium</x:v>
+      </x:c>
+      <x:c r="M162" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N162" s="9" t="str">
+        <x:v>No ordinary pulp paper or cloth; text and faith acceptance TBD</x:v>
+      </x:c>
+      <x:c r="O162" s="17"/>
+      <x:c r="P162" s="17"/>
+      <x:c r="Q162" s="17"/>
+      <x:c r="R162" s="17"/>
+      <x:c r="S162" s="17"/>
+      <x:c r="T162" s="9" t="str">
+        <x:v>Paper processing and copying consume scarce skilled work. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U162" s="11"/>
+      <x:c r="V162" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/religious-traditions.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="100" customHeight="1">
+      <x:c r="A163" s="9" t="str">
+        <x:v>proposal.culture.offering</x:v>
+      </x:c>
+      <x:c r="B163" s="9" t="str">
+        <x:v>Votive shell token</x:v>
+      </x:c>
+      <x:c r="C163" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D163" s="9" t="str">
+        <x:v>Religious</x:v>
+      </x:c>
+      <x:c r="E163" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F163" s="9" t="str">
+        <x:v>Small dedicated offering left at a shrine</x:v>
+      </x:c>
+      <x:c r="G163" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H163" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I163" s="13"/>
+      <x:c r="J163" s="15"/>
+      <x:c r="K163" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L163" s="9" t="str">
+        <x:v>Material candidate: Worked shed shell; metal inlay optional</x:v>
+      </x:c>
+      <x:c r="M163" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N163" s="9" t="str">
+        <x:v>New game object idea; no mandatory tithe or survival payment</x:v>
+      </x:c>
+      <x:c r="O163" s="17"/>
+      <x:c r="P163" s="17"/>
+      <x:c r="Q163" s="17"/>
+      <x:c r="R163" s="17"/>
+      <x:c r="S163" s="17"/>
+      <x:c r="T163" s="9" t="str">
+        <x:v>Simple shell version can be modest; embellished versions expensive. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U163" s="11"/>
+      <x:c r="V163" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/spiritual-economy.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="100" customHeight="1">
+      <x:c r="A164" s="9" t="str">
+        <x:v>proposal.culture.badge</x:v>
+      </x:c>
+      <x:c r="B164" s="9" t="str">
+        <x:v>Civic office badge</x:v>
+      </x:c>
+      <x:c r="C164" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D164" s="9" t="str">
+        <x:v>Political / civic</x:v>
+      </x:c>
+      <x:c r="E164" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F164" s="9" t="str">
+        <x:v>Visible sign of a delegated public role</x:v>
+      </x:c>
+      <x:c r="G164" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H164" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I164" s="13"/>
+      <x:c r="J164" s="15"/>
+      <x:c r="K164" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L164" s="9" t="str">
+        <x:v>Material candidate: Stamped metal or carved shell</x:v>
+      </x:c>
+      <x:c r="M164" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N164" s="9" t="str">
+        <x:v>Office names and authority unresolved; no automatic access rules</x:v>
+      </x:c>
+      <x:c r="O164" s="17"/>
+      <x:c r="P164" s="17"/>
+      <x:c r="Q164" s="17"/>
+      <x:c r="R164" s="17"/>
+      <x:c r="S164" s="17"/>
+      <x:c r="T164" s="9" t="str">
+        <x:v>Plain office issue or costly ceremonial version. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U164" s="11"/>
+      <x:c r="V164" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/civic-contract.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="100" customHeight="1">
+      <x:c r="A165" s="9" t="str">
+        <x:v>proposal.culture.stamp</x:v>
+      </x:c>
+      <x:c r="B165" s="9" t="str">
+        <x:v>Official seal stamp</x:v>
+      </x:c>
+      <x:c r="C165" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D165" s="9" t="str">
+        <x:v>Political / civic</x:v>
+      </x:c>
+      <x:c r="E165" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F165" s="9" t="str">
+        <x:v>Mark a record or notice with an office symbol</x:v>
+      </x:c>
+      <x:c r="G165" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H165" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I165" s="13"/>
+      <x:c r="J165" s="15"/>
+      <x:c r="K165" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L165" s="9" t="str">
+        <x:v>Material candidate: Engraved metal stamping face</x:v>
+      </x:c>
+      <x:c r="M165" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N165" s="9" t="str">
+        <x:v>Document mark only; distinct from a canister pressure seal</x:v>
+      </x:c>
+      <x:c r="O165" s="17"/>
+      <x:c r="P165" s="17"/>
+      <x:c r="Q165" s="17"/>
+      <x:c r="R165" s="17"/>
+      <x:c r="S165" s="17"/>
+      <x:c r="T165" s="9" t="str">
+        <x:v>Skilled engraving; actual trade restrictions unresolved. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U165" s="11"/>
+      <x:c r="V165" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/civic-contract.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="100" customHeight="1">
+      <x:c r="A166" s="9" t="str">
+        <x:v>proposal.culture.register</x:v>
+      </x:c>
+      <x:c r="B166" s="9" t="str">
+        <x:v>Civic register folio</x:v>
+      </x:c>
+      <x:c r="C166" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D166" s="9" t="str">
+        <x:v>Political / civic</x:v>
+      </x:c>
+      <x:c r="E166" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F166" s="9" t="str">
+        <x:v>Record voluntary contributions, membership and commendations</x:v>
+      </x:c>
+      <x:c r="G166" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H166" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I166" s="13"/>
+      <x:c r="J166" s="15"/>
+      <x:c r="K166" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L166" s="9" t="str">
+        <x:v>Material candidate: Husk-paper leaves between shell covers</x:v>
+      </x:c>
+      <x:c r="M166" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N166" s="9" t="str">
+        <x:v>Source civic register inspiration; no legal survival obligation or permission gate</x:v>
+      </x:c>
+      <x:c r="O166" s="17"/>
+      <x:c r="P166" s="17"/>
+      <x:c r="Q166" s="17"/>
+      <x:c r="R166" s="17"/>
+      <x:c r="S166" s="17"/>
+      <x:c r="T166" s="9" t="str">
+        <x:v>Labor-intensive communal record; not assumed universal personal kit. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U166" s="11"/>
+      <x:c r="V166" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/civic-contract.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="100" customHeight="1">
+      <x:c r="A167" s="9" t="str">
+        <x:v>proposal.culture.notice</x:v>
+      </x:c>
+      <x:c r="B167" s="9" t="str">
+        <x:v>Public notice plate</x:v>
+      </x:c>
+      <x:c r="C167" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D167" s="9" t="str">
+        <x:v>Political / civic</x:v>
+      </x:c>
+      <x:c r="E167" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F167" s="9" t="str">
+        <x:v>Display civic announcements, rules or meeting notices</x:v>
+      </x:c>
+      <x:c r="G167" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H167" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I167" s="13"/>
+      <x:c r="J167" s="15"/>
+      <x:c r="K167" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L167" s="9" t="str">
+        <x:v>Material candidate: Incised shell or thin worked metal</x:v>
+      </x:c>
+      <x:c r="M167" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N167" s="9" t="str">
+        <x:v>Government and literacy practices unresolved</x:v>
+      </x:c>
+      <x:c r="O167" s="17"/>
+      <x:c r="P167" s="17"/>
+      <x:c r="Q167" s="17"/>
+      <x:c r="R167" s="17"/>
+      <x:c r="S167" s="17"/>
+      <x:c r="T167" s="9" t="str">
+        <x:v>Durable reusable public object; exact cost TBD. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U167" s="11"/>
+      <x:c r="V167" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/civic-contract.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="100" customHeight="1">
+      <x:c r="A168" s="9" t="str">
+        <x:v>proposal.culture.petition</x:v>
+      </x:c>
+      <x:c r="B168" s="9" t="str">
+        <x:v>Petition leaf</x:v>
+      </x:c>
+      <x:c r="C168" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D168" s="9" t="str">
+        <x:v>Political / civic</x:v>
+      </x:c>
+      <x:c r="E168" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F168" s="9" t="str">
+        <x:v>Carry a written request or collective statement</x:v>
+      </x:c>
+      <x:c r="G168" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H168" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I168" s="13"/>
+      <x:c r="J168" s="15"/>
+      <x:c r="K168" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L168" s="9" t="str">
+        <x:v>Material candidate: Husk-fiber paper and mineral marks</x:v>
+      </x:c>
+      <x:c r="M168" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N168" s="9" t="str">
+        <x:v>Political disagreement need not imply repression or a named faction</x:v>
+      </x:c>
+      <x:c r="O168" s="17"/>
+      <x:c r="P168" s="17"/>
+      <x:c r="Q168" s="17"/>
+      <x:c r="R168" s="17"/>
+      <x:c r="S168" s="17"/>
+      <x:c r="T168" s="9" t="str">
+        <x:v>Paper cost and copying effort; no numeric price. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U168" s="11"/>
+      <x:c r="V168" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/civic-contract.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="100" customHeight="1">
+      <x:c r="A169" s="9" t="str">
+        <x:v>proposal.culture.commendation</x:v>
+      </x:c>
+      <x:c r="B169" s="9" t="str">
+        <x:v>Community service medallion</x:v>
+      </x:c>
+      <x:c r="C169" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D169" s="9" t="str">
+        <x:v>Political / civic</x:v>
+      </x:c>
+      <x:c r="E169" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F169" s="9" t="str">
+        <x:v>Public recognition of voluntary service</x:v>
+      </x:c>
+      <x:c r="G169" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H169" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I169" s="13"/>
+      <x:c r="J169" s="15"/>
+      <x:c r="K169" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L169" s="9" t="str">
+        <x:v>Material candidate: Stamped metal; optional fine inlay</x:v>
+      </x:c>
+      <x:c r="M169" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N169" s="9" t="str">
+        <x:v>Not a maker plate; award eligibility and issuing body undefined</x:v>
+      </x:c>
+      <x:c r="O169" s="17"/>
+      <x:c r="P169" s="17"/>
+      <x:c r="Q169" s="17"/>
+      <x:c r="R169" s="17"/>
+      <x:c r="S169" s="17"/>
+      <x:c r="T169" s="9" t="str">
+        <x:v>Basic award to elaborate exceptional commission. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U169" s="11"/>
+      <x:c r="V169" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/civic-contract.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="100" customHeight="1">
+      <x:c r="A170" s="9" t="str">
+        <x:v>proposal.culture.pilgrim_die</x:v>
+      </x:c>
+      <x:c r="B170" s="9" t="str">
+        <x:v>Pilgrimage marking die</x:v>
+      </x:c>
+      <x:c r="C170" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D170" s="9" t="str">
+        <x:v>Ritual</x:v>
+      </x:c>
+      <x:c r="E170" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F170" s="9" t="str">
+        <x:v>Apply a sacred-site mark to a suitable record surface</x:v>
+      </x:c>
+      <x:c r="G170" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H170" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I170" s="13"/>
+      <x:c r="J170" s="15"/>
+      <x:c r="K170" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L170" s="9" t="str">
+        <x:v>Material candidate: Engraved metal die</x:v>
+      </x:c>
+      <x:c r="M170" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N170" s="9" t="str">
+        <x:v>No hammering on a live vessel assumed; safe application and faith adoption TBD</x:v>
+      </x:c>
+      <x:c r="O170" s="17"/>
+      <x:c r="P170" s="17"/>
+      <x:c r="Q170" s="17"/>
+      <x:c r="R170" s="17"/>
+      <x:c r="S170" s="17"/>
+      <x:c r="T170" s="9" t="str">
+        <x:v>Specialist institutional tool. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U170" s="11"/>
+      <x:c r="V170" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/religious-traditions.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="100" customHeight="1">
+      <x:c r="A171" s="9" t="str">
+        <x:v>proposal.culture.memorial</x:v>
+      </x:c>
+      <x:c r="B171" s="9" t="str">
+        <x:v>Memorial name plate</x:v>
+      </x:c>
+      <x:c r="C171" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D171" s="9" t="str">
+        <x:v>Ritual</x:v>
+      </x:c>
+      <x:c r="E171" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F171" s="9" t="str">
+        <x:v>Remember a deceased person or missing traveler</x:v>
+      </x:c>
+      <x:c r="G171" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H171" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I171" s="13"/>
+      <x:c r="J171" s="15"/>
+      <x:c r="K171" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L171" s="9" t="str">
+        <x:v>Material candidate: Incised metal or shell</x:v>
+      </x:c>
+      <x:c r="M171" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N171" s="9" t="str">
+        <x:v>Cultural keepsake; no resurrection or supernatural effect</x:v>
+      </x:c>
+      <x:c r="O171" s="17"/>
+      <x:c r="P171" s="17"/>
+      <x:c r="Q171" s="17"/>
+      <x:c r="R171" s="17"/>
+      <x:c r="S171" s="17"/>
+      <x:c r="T171" s="9" t="str">
+        <x:v>Plain family marker to elaborate memorial commission. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U171" s="11"/>
+      <x:c r="V171" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/spiritual-economy.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="100" customHeight="1">
+      <x:c r="A172" s="9" t="str">
+        <x:v>proposal.culture.oath_ring</x:v>
+      </x:c>
+      <x:c r="B172" s="9" t="str">
+        <x:v>Oath exchange ring</x:v>
+      </x:c>
+      <x:c r="C172" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D172" s="9" t="str">
+        <x:v>Ritual</x:v>
+      </x:c>
+      <x:c r="E172" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F172" s="9" t="str">
+        <x:v>Exchange a visible token at a vow or commitment</x:v>
+      </x:c>
+      <x:c r="G172" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H172" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I172" s="13"/>
+      <x:c r="J172" s="15"/>
+      <x:c r="K172" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L172" s="9" t="str">
+        <x:v>Material candidate: Worked metal; shell inset optional</x:v>
+      </x:c>
+      <x:c r="M172" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N172" s="9" t="str">
+        <x:v>New game ritual proposal; exact marriage or guild customs undecided</x:v>
+      </x:c>
+      <x:c r="O172" s="17"/>
+      <x:c r="P172" s="17"/>
+      <x:c r="Q172" s="17"/>
+      <x:c r="R172" s="17"/>
+      <x:c r="S172" s="17"/>
+      <x:c r="T172" s="9" t="str">
+        <x:v>Simple bands through expensive engraved work. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U172" s="11"/>
+      <x:c r="V172" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/spiritual-economy.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="100" customHeight="1">
+      <x:c r="A173" s="9" t="str">
+        <x:v>proposal.culture.milestone</x:v>
+      </x:c>
+      <x:c r="B173" s="9" t="str">
+        <x:v>Life-event charm</x:v>
+      </x:c>
+      <x:c r="C173" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D173" s="9" t="str">
+        <x:v>Ritual</x:v>
+      </x:c>
+      <x:c r="E173" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F173" s="9" t="str">
+        <x:v>Record coming of age, apprenticeship or return</x:v>
+      </x:c>
+      <x:c r="G173" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H173" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I173" s="13"/>
+      <x:c r="J173" s="15"/>
+      <x:c r="K173" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L173" s="9" t="str">
+        <x:v>Material candidate: Stamped metal or carved shell</x:v>
+      </x:c>
+      <x:c r="M173" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N173" s="9" t="str">
+        <x:v>Use existing mounts where appropriate; not a new functional canister</x:v>
+      </x:c>
+      <x:c r="O173" s="17"/>
+      <x:c r="P173" s="17"/>
+      <x:c r="Q173" s="17"/>
+      <x:c r="R173" s="17"/>
+      <x:c r="S173" s="17"/>
+      <x:c r="T173" s="9" t="str">
+        <x:v>Small plain charm to fine engraved keepsake. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U173" s="11"/>
+      <x:c r="V173" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/religious-traditions.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="100" customHeight="1">
+      <x:c r="A174" s="9" t="str">
+        <x:v>proposal.culture.rattle</x:v>
+      </x:c>
+      <x:c r="B174" s="9" t="str">
+        <x:v>Ceremonial shell rattle</x:v>
+      </x:c>
+      <x:c r="C174" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D174" s="9" t="str">
+        <x:v>Ritual</x:v>
+      </x:c>
+      <x:c r="E174" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F174" s="9" t="str">
+        <x:v>Provide a dry percussive sound for gatherings</x:v>
+      </x:c>
+      <x:c r="G174" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H174" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I174" s="13"/>
+      <x:c r="J174" s="15"/>
+      <x:c r="K174" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L174" s="9" t="str">
+        <x:v>Material candidate: Hollow shell with mineral chips and metal fasteners</x:v>
+      </x:c>
+      <x:c r="M174" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N174" s="9" t="str">
+        <x:v>Sound rituals and fauna reactions undecided; no weapon mechanic</x:v>
+      </x:c>
+      <x:c r="O174" s="17"/>
+      <x:c r="P174" s="17"/>
+      <x:c r="Q174" s="17"/>
+      <x:c r="R174" s="17"/>
+      <x:c r="S174" s="17"/>
+      <x:c r="T174" s="9" t="str">
+        <x:v>Plain community instrument; decorated pieces may be costly. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U174" s="11"/>
+      <x:c r="V174" s="9" t="str">
+        <x:v>New game proposal; author request October 14, 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="100" customHeight="1">
+      <x:c r="A175" s="9" t="str">
+        <x:v>proposal.culture.gift_case</x:v>
+      </x:c>
+      <x:c r="B175" s="9" t="str">
+        <x:v>Ceremonial gift case</x:v>
+      </x:c>
+      <x:c r="C175" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D175" s="9" t="str">
+        <x:v>Ritual</x:v>
+      </x:c>
+      <x:c r="E175" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F175" s="9" t="str">
+        <x:v>Present and retain a life-event gift</x:v>
+      </x:c>
+      <x:c r="G175" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H175" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I175" s="13"/>
+      <x:c r="J175" s="15"/>
+      <x:c r="K175" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L175" s="9" t="str">
+        <x:v>Material candidate: Fitted shell or worked metal; minimal lining if needed</x:v>
+      </x:c>
+      <x:c r="M175" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N175" s="9" t="str">
+        <x:v>Reuse existing box/container family as craft basis; contents counted separately</x:v>
+      </x:c>
+      <x:c r="O175" s="17"/>
+      <x:c r="P175" s="17"/>
+      <x:c r="Q175" s="17"/>
+      <x:c r="R175" s="17"/>
+      <x:c r="S175" s="17"/>
+      <x:c r="T175" s="9" t="str">
+        <x:v>Labor-intensive fitted finish differentiates it from basic storage. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U175" s="11"/>
+      <x:c r="V175" s="9" t="str">
+        <x:v>New game proposal inspired by proposal-stage lore: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/canister/religious-traditions.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="100" customHeight="1">
+      <x:c r="A176" s="9" t="str">
+        <x:v>proposal.culture.bowl</x:v>
+      </x:c>
+      <x:c r="B176" s="9" t="str">
+        <x:v>Everyday shell bowl</x:v>
+      </x:c>
+      <x:c r="C176" s="9" t="str">
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D176" s="9" t="str">
+        <x:v>Everyday household</x:v>
+      </x:c>
+      <x:c r="E176" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F176" s="9" t="str">
+        <x:v>Hold an algae meal or sorted small goods</x:v>
+      </x:c>
+      <x:c r="G176" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H176" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I176" s="13"/>
+      <x:c r="J176" s="15"/>
+      <x:c r="K176" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L176" s="9" t="str">
+        <x:v>Material candidate: Prepared shell; safe metal version possible</x:v>
+      </x:c>
+      <x:c r="M176" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N176" s="9" t="str">
+        <x:v>Shell must be assessed for toxic residues; no assumed water supply</x:v>
+      </x:c>
+      <x:c r="O176" s="17"/>
+      <x:c r="P176" s="17"/>
+      <x:c r="Q176" s="17"/>
+      <x:c r="R176" s="17"/>
+      <x:c r="S176" s="17"/>
+      <x:c r="T176" s="9" t="str">
+        <x:v>Cheap raw shell; food-contact preparation has its own cost. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U176" s="11"/>
+      <x:c r="V176" s="9" t="str">
+        <x:v>New game proposal; author request October 14, 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="100" customHeight="1">
+      <x:c r="A177" s="9" t="str">
+        <x:v>proposal.culture.spoon</x:v>
+      </x:c>
+      <x:c r="B177" s="9" t="str">
+        <x:v>Algae spoon / scraper</x:v>
+      </x:c>
+      <x:c r="C177" s="9" t="str">
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D177" s="9" t="str">
+        <x:v>Everyday household</x:v>
+      </x:c>
+      <x:c r="E177" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F177" s="9" t="str">
+        <x:v>Eat or scrape a contained algae portion</x:v>
+      </x:c>
+      <x:c r="G177" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H177" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I177" s="13"/>
+      <x:c r="J177" s="15"/>
+      <x:c r="K177" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L177" s="9" t="str">
+        <x:v>Material candidate: Formed metal or prepared shell</x:v>
+      </x:c>
+      <x:c r="M177" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N177" s="9" t="str">
+        <x:v>Food-safe finish TBD; no duplicate algae supply</x:v>
+      </x:c>
+      <x:c r="O177" s="17"/>
+      <x:c r="P177" s="17"/>
+      <x:c r="Q177" s="17"/>
+      <x:c r="R177" s="17"/>
+      <x:c r="S177" s="17"/>
+      <x:c r="T177" s="9" t="str">
+        <x:v>Practical simple tool; workmanship and material determine value. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U177" s="11"/>
+      <x:c r="V177" s="9" t="str">
+        <x:v>New game proposal; author request October 14, 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="100" customHeight="1">
+      <x:c r="A178" s="9" t="str">
+        <x:v>proposal.culture.brush</x:v>
+      </x:c>
+      <x:c r="B178" s="9" t="str">
+        <x:v>Dust brush</x:v>
+      </x:c>
+      <x:c r="C178" s="9" t="str">
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D178" s="9" t="str">
+        <x:v>Everyday household</x:v>
+      </x:c>
+      <x:c r="E178" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F178" s="9" t="str">
+        <x:v>Sweep dust from possessions and living areas</x:v>
+      </x:c>
+      <x:c r="G178" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H178" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I178" s="13"/>
+      <x:c r="J178" s="15"/>
+      <x:c r="K178" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L178" s="9" t="str">
+        <x:v>Material candidate: Selected fauna bristles in a shell/metal head</x:v>
+      </x:c>
+      <x:c r="M178" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N178" s="9" t="str">
+        <x:v>Bristle safety and assembly unresolved; no cloth required</x:v>
+      </x:c>
+      <x:c r="O178" s="17"/>
+      <x:c r="P178" s="17"/>
+      <x:c r="Q178" s="17"/>
+      <x:c r="R178" s="17"/>
+      <x:c r="S178" s="17"/>
+      <x:c r="T178" s="9" t="str">
+        <x:v>Raw bristles and finished brush have separate value. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U178" s="11"/>
+      <x:c r="V178" s="9" t="str">
+        <x:v>New game proposal; author request October 14, 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="100" customHeight="1">
+      <x:c r="A179" s="9" t="str">
+        <x:v>proposal.culture.comb</x:v>
+      </x:c>
+      <x:c r="B179" s="9" t="str">
+        <x:v>Shell comb</x:v>
+      </x:c>
+      <x:c r="C179" s="9" t="str">
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D179" s="9" t="str">
+        <x:v>Everyday household</x:v>
+      </x:c>
+      <x:c r="E179" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F179" s="9" t="str">
+        <x:v>Personal grooming</x:v>
+      </x:c>
+      <x:c r="G179" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H179" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I179" s="13"/>
+      <x:c r="J179" s="15"/>
+      <x:c r="K179" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L179" s="9" t="str">
+        <x:v>Material candidate: Carved shell or metal</x:v>
+      </x:c>
+      <x:c r="M179" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N179" s="9" t="str">
+        <x:v>No fur textile input or clothing slot implied</x:v>
+      </x:c>
+      <x:c r="O179" s="17"/>
+      <x:c r="P179" s="17"/>
+      <x:c r="Q179" s="17"/>
+      <x:c r="R179" s="17"/>
+      <x:c r="S179" s="17"/>
+      <x:c r="T179" s="9" t="str">
+        <x:v>Simple cheap-material craft; elaborate fine-tooth versions possible. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U179" s="11"/>
+      <x:c r="V179" s="9" t="str">
+        <x:v>New game proposal; author request October 14, 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="100" customHeight="1">
+      <x:c r="A180" s="9" t="str">
+        <x:v>proposal.culture.tablet</x:v>
+      </x:c>
+      <x:c r="B180" s="9" t="str">
+        <x:v>Reusable tally tablet</x:v>
+      </x:c>
+      <x:c r="C180" s="9" t="str">
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D180" s="9" t="str">
+        <x:v>Everyday household</x:v>
+      </x:c>
+      <x:c r="E180" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F180" s="9" t="str">
+        <x:v>Practice marks, keep counts or leave short messages</x:v>
+      </x:c>
+      <x:c r="G180" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H180" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I180" s="13"/>
+      <x:c r="J180" s="15"/>
+      <x:c r="K180" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L180" s="9" t="str">
+        <x:v>Material candidate: Incised shell or soft mineral plate</x:v>
+      </x:c>
+      <x:c r="M180" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N180" s="9" t="str">
+        <x:v>Writing method must match surface; not an electronic tablet</x:v>
+      </x:c>
+      <x:c r="O180" s="17"/>
+      <x:c r="P180" s="17"/>
+      <x:c r="Q180" s="17"/>
+      <x:c r="R180" s="17"/>
+      <x:c r="S180" s="17"/>
+      <x:c r="T180" s="9" t="str">
+        <x:v>Paper-saving reusable surface; exact erasability TBD. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U180" s="11"/>
+      <x:c r="V180" s="9" t="str">
+        <x:v>New game proposal; author request October 14, 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="100" customHeight="1">
+      <x:c r="A181" s="9" t="str">
+        <x:v>proposal.culture.stylus</x:v>
+      </x:c>
+      <x:c r="B181" s="9" t="str">
+        <x:v>Marking stylus</x:v>
+      </x:c>
+      <x:c r="C181" s="9" t="str">
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D181" s="9" t="str">
+        <x:v>Everyday household</x:v>
+      </x:c>
+      <x:c r="E181" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F181" s="9" t="str">
+        <x:v>Incise compatible tablets, labels or simple designs</x:v>
+      </x:c>
+      <x:c r="G181" s="9" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H181" s="9" t="str">
+        <x:v>Personal kit / local storage eligibility TBD</x:v>
+      </x:c>
+      <x:c r="I181" s="13"/>
+      <x:c r="J181" s="15"/>
+      <x:c r="K181" s="9" t="str">
+        <x:v>Craft, trade, gift or institutional custody; exact source TBD</x:v>
+      </x:c>
+      <x:c r="L181" s="9" t="str">
+        <x:v>Material candidate: Worked metal point in a shell/metal grip</x:v>
+      </x:c>
+      <x:c r="M181" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N181" s="9" t="str">
+        <x:v>No ink chemistry or universal writing compatibility assumed</x:v>
+      </x:c>
+      <x:c r="O181" s="17"/>
+      <x:c r="P181" s="17"/>
+      <x:c r="Q181" s="17"/>
+      <x:c r="R181" s="17"/>
+      <x:c r="S181" s="17"/>
+      <x:c r="T181" s="9" t="str">
+        <x:v>Simple durable tool; fine engraving tools are separate specialist grades. Faith, political authority, ritual practice and prices remain proposals.</x:v>
+      </x:c>
+      <x:c r="U181" s="11"/>
+      <x:c r="V181" s="9" t="str">
+        <x:v>New game proposal; author request October 14, 2026</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
@@ -9039,7 +10287,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra96a3825c6364c08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d312667e2254ae4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9691,7 +10939,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R049954675f444f3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f30ee417c894dfa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10173,7 +11421,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dcf33107c174b70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3407710b21c9458b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11081,7 +12329,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba2710e225b34293"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaca4e4c034246dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11447,7 +12695,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4ee2e8d828a43ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3dfa8e5dad04137"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11811,10 +13059,70 @@
         <x:v>Vertical shade uses the existing popup-camp family. Ordinary shells separately become cheap bulk resource.</x:v>
       </x:c>
     </x:row>
+    <x:row r="27" ht="85" customHeight="1">
+      <x:c r="A27" s="4" t="str">
+        <x:v>Religious objects</x:v>
+      </x:c>
+      <x:c r="B27" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Religious")</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C27" s="4" t="str">
+        <x:v>Icons, shrine plaques, altar vials, relic cases, prayer leaves and votive tokens</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="str">
+        <x:v>All six are game proposals; source faith records are proposal-stage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="85" customHeight="1">
+      <x:c r="A28" s="4" t="str">
+        <x:v>Political / civic objects</x:v>
+      </x:c>
+      <x:c r="B28" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Political / civic")</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C28" s="4" t="str">
+        <x:v>Office badges, seal stamps, registers, notices, petitions and service medallions</x:v>
+      </x:c>
+      <x:c r="D28" s="4" t="str">
+        <x:v>Institutions, rights and public roles remain undecided.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="85" customHeight="1">
+      <x:c r="A29" s="4" t="str">
+        <x:v>Ritual objects</x:v>
+      </x:c>
+      <x:c r="B29" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Ritual")</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C29" s="4" t="str">
+        <x:v>Pilgrimage dies, memorial plates, oath rings, milestone charms, rattles and gift cases</x:v>
+      </x:c>
+      <x:c r="D29" s="4" t="str">
+        <x:v>Objects of ceremony and memory; no automatic supernatural effects.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="85" customHeight="1">
+      <x:c r="A30" s="4" t="str">
+        <x:v>Everyday household</x:v>
+      </x:c>
+      <x:c r="B30" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Everyday household")</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C30" s="4" t="str">
+        <x:v>Bowls, algae spoons, dust brushes, combs, tally tablets and marking tools</x:v>
+      </x:c>
+      <x:c r="D30" s="4" t="str">
+        <x:v>Simple shell/metal forms; no wood or ordinary cloth assumed.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61e6d6ccb016431b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40cb6e8346d64b5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11877,7 +13185,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>152 design entries: 18 existing item IDs and 134 design concepts. Added two wing-material concepts and fifteen canister-economy candidates; existing popup camp reused for vertical shades.</x:v>
+        <x:v>176 design entries: 18 existing item IDs and 158 design concepts. Includes 24 religious, civic, ritual and everyday object proposals.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -12544,10 +13852,50 @@
         <x:v>Personal survival canister, dust device and toxic-material vessel are distinct roles. Parts do not create extra liquid reserves, shared storage or duplicate owned canisters. All trial systems remain unchanged.</x:v>
       </x:c>
     </x:row>
+    <x:row r="92" ht="80" customHeight="1">
+      <x:c r="A92" s="4" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="B92" s="4" t="str">
+        <x:v>Religious, political/civic and ritual objects are working game proposals inspired by source drafts WLD-0018, WLD-0036 and WLD-0042. Named faith and institutional details are not silently adopted as game canon.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="80" customHeight="1">
+      <x:c r="A93" s="4" t="str">
+        <x:v>Ordinary and ceremonial grades</x:v>
+      </x:c>
+      <x:c r="B93" s="4" t="str">
+        <x:v>Simple shell and stamped-metal forms may serve everyday use. Fine engraving, clear glass, selected inlay and processed husk paper create potential prestige craft variants; no rarity or value numbers assigned.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="80" customHeight="1">
+      <x:c r="A94" s="4" t="str">
+        <x:v>Symbol and function</x:v>
+      </x:c>
+      <x:c r="B94" s="4" t="str">
+        <x:v>Blessings, relic claims, oath tokens and authority badges do not automatically grant buffs, proof of authenticity or access. Document seal stamps are distinct from liquid-container sealing parts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="80" customHeight="1">
+      <x:c r="A95" s="4" t="str">
+        <x:v>Household materials</x:v>
+      </x:c>
+      <x:c r="B95" s="4" t="str">
+        <x:v>No ordinary cloth, timber, plant paper, free water or automatic food-safe shell is introduced. Household shell needs suitable preparation; paper uses difficult husk-fiber processing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="80" customHeight="1">
+      <x:c r="A96" s="4" t="str">
+        <x:v>Item-family reuse</x:v>
+      </x:c>
+      <x:c r="B96" s="4" t="str">
+        <x:v>Altar vessels and ceremonial gift cases build on existing container families. A blessing or pilgrimage mark is a potential provenance/variant of a canister rather than an extra survival canister or new mechanical reserve.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34f33dbc0dfd4290"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d2e10e8dd704e1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13391,7 +14739,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53bce0257e2043ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7ab387b92dd42bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13634,7 +14982,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4616b48d5e0645f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cd0e37c25024783"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14038,7 +15386,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fcf34cb044f4fe8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R053911fcd78e407c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14714,7 +16062,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc139173f1f464ff9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b050816035a4ce6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: expand ceramic materials and item families
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R88591b5a728e4604"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R2454f2ae713d48b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R4936551bf90b40d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R9b16a1d1ee3040c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R38b3bf21c68440a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R2b3b9880e9d4493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R7f05e57765fb4660"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Ra0f8c55000c34733"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Rae5b6feb8fb548f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R89cb2e4e30ca4bd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R1f0a7bec0d644b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R96c4ebcf05784d3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="Rf0f09ecc79bb4cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R370a4633e2694528"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rd9e12b4fe7a445da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R68d0fe190343488e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rdf171a3efea24e3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R6f131b9db7f04e73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rc18f9de7d0544b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R511b5b6f4d3f4730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R89c95e3337734d0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R4339eb6410e94dea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R2b4f480e1f6448df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R543f669186554f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R77e4abe573524374"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="R8e51d6ef392a460f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,8 +476,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE181" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AE181"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE209" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AE209"/>
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -550,7 +550,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C163" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C166" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Field"/>
     <x:tableColumn id="2" name="Allowed value"/>
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F236" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F236"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F283" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F283"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -614,7 +614,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -626,7 +626,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B108" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -986,7 +986,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>176 items. Filter W:AC for type, stage, origin, use, material, form and status. Search AD; use Item uses for multiple purposes.</x:v>
+        <x:v>204 items. Filter W:AC for type, stage, origin, use, material, form and status. Search AD; use Item uses for multiple purposes.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -3712,7 +3712,7 @@
         <x:v>Electrical insulation</x:v>
       </x:c>
       <x:c r="AA37" s="4" t="str">
-        <x:v>Mineral</x:v>
+        <x:v>Ceramic</x:v>
       </x:c>
       <x:c r="AB37" s="4" t="str">
         <x:v>Solid part</x:v>
@@ -15119,6 +15119,2218 @@
       </x:c>
       <x:c r="AE181" s="4" t="str">
         <x:v>From current item description. Proposed uses retain their existing approval status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="105" customHeight="1">
+      <x:c r="A182" s="9" t="str">
+        <x:v>proposal.ceramic.grog</x:v>
+      </x:c>
+      <x:c r="B182" s="9" t="str">
+        <x:v>Crushed fired ceramic grit</x:v>
+      </x:c>
+      <x:c r="C182" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D182" s="9" t="str">
+        <x:v>Ceramic feedstock</x:v>
+      </x:c>
+      <x:c r="E182" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F182" s="9" t="str">
+        <x:v>Selected broken fired ceramic, sorted and crushed for candidate body mixes.</x:v>
+      </x:c>
+      <x:c r="G182" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H182" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I182" s="13"/>
+      <x:c r="J182" s="15"/>
+      <x:c r="K182" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L182" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M182" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N182" s="9" t="str">
+        <x:v>Composition and contamination must be identified; not every broken vessel is reusable feed.</x:v>
+      </x:c>
+      <x:c r="O182" s="17"/>
+      <x:c r="P182" s="17"/>
+      <x:c r="Q182" s="17"/>
+      <x:c r="R182" s="17"/>
+      <x:c r="S182" s="17"/>
+      <x:c r="T182" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U182" s="11"/>
+      <x:c r="V182" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W182" s="4" t="str">
+        <x:v>Processed material</x:v>
+      </x:c>
+      <x:c r="X182" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y182" s="4" t="str">
+        <x:v>Geological</x:v>
+      </x:c>
+      <x:c r="Z182" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="AA182" s="4" t="str">
+        <x:v>Ceramic feed mixture</x:v>
+      </x:c>
+      <x:c r="AB182" s="4" t="str">
+        <x:v>Particles</x:v>
+      </x:c>
+      <x:c r="AC182" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD182" s="4" t="str">
+        <x:v>crushed fired ceramic grit; fabrication; glass and ceramics; ceramic; pottery; ceramic feedstock; processed material; ceramic feed mixture</x:v>
+      </x:c>
+      <x:c r="AE182" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="105" customHeight="1">
+      <x:c r="A183" s="9" t="str">
+        <x:v>proposal.ceramic.body_feed</x:v>
+      </x:c>
+      <x:c r="B183" s="9" t="str">
+        <x:v>Prepared ceramic body feed</x:v>
+      </x:c>
+      <x:c r="C183" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D183" s="9" t="str">
+        <x:v>Ceramic feedstock</x:v>
+      </x:c>
+      <x:c r="E183" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F183" s="9" t="str">
+        <x:v>Selected mineral feed blended for a chosen ceramic product.</x:v>
+      </x:c>
+      <x:c r="G183" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H183" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I183" s="13"/>
+      <x:c r="J183" s="15"/>
+      <x:c r="K183" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L183" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M183" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N183" s="9" t="str">
+        <x:v>Forming and binder method unresolved under the no-free-water rule; no recipe ratios.</x:v>
+      </x:c>
+      <x:c r="O183" s="17"/>
+      <x:c r="P183" s="17"/>
+      <x:c r="Q183" s="17"/>
+      <x:c r="R183" s="17"/>
+      <x:c r="S183" s="17"/>
+      <x:c r="T183" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U183" s="11"/>
+      <x:c r="V183" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W183" s="4" t="str">
+        <x:v>Processed material</x:v>
+      </x:c>
+      <x:c r="X183" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y183" s="4" t="str">
+        <x:v>Geological</x:v>
+      </x:c>
+      <x:c r="Z183" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="AA183" s="4" t="str">
+        <x:v>Ceramic feed mixture</x:v>
+      </x:c>
+      <x:c r="AB183" s="4" t="str">
+        <x:v>Particles</x:v>
+      </x:c>
+      <x:c r="AC183" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD183" s="4" t="str">
+        <x:v>prepared ceramic body feed; fabrication; glass and ceramics; ceramic; pottery; ceramic feedstock; processed material; ceramic feed mixture</x:v>
+      </x:c>
+      <x:c r="AE183" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="105" customHeight="1">
+      <x:c r="A184" s="9" t="str">
+        <x:v>proposal.ceramic.glaze_feed</x:v>
+      </x:c>
+      <x:c r="B184" s="9" t="str">
+        <x:v>Prepared glaze feed</x:v>
+      </x:c>
+      <x:c r="C184" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D184" s="9" t="str">
+        <x:v>Ceramic feedstock</x:v>
+      </x:c>
+      <x:c r="E184" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F184" s="9" t="str">
+        <x:v>Selected mineral finishing feed for compatible ceramic surfaces.</x:v>
+      </x:c>
+      <x:c r="G184" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H184" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I184" s="13"/>
+      <x:c r="J184" s="15"/>
+      <x:c r="K184" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L184" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M184" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N184" s="9" t="str">
+        <x:v>No universal glaze, toxin barrier or food-safe finish assumed.</x:v>
+      </x:c>
+      <x:c r="O184" s="17"/>
+      <x:c r="P184" s="17"/>
+      <x:c r="Q184" s="17"/>
+      <x:c r="R184" s="17"/>
+      <x:c r="S184" s="17"/>
+      <x:c r="T184" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U184" s="11"/>
+      <x:c r="V184" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W184" s="4" t="str">
+        <x:v>Processed material</x:v>
+      </x:c>
+      <x:c r="X184" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y184" s="4" t="str">
+        <x:v>Geological</x:v>
+      </x:c>
+      <x:c r="Z184" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="AA184" s="4" t="str">
+        <x:v>Ceramic feed mixture</x:v>
+      </x:c>
+      <x:c r="AB184" s="4" t="str">
+        <x:v>Particles</x:v>
+      </x:c>
+      <x:c r="AC184" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD184" s="4" t="str">
+        <x:v>prepared glaze feed; surface finishing; glass and ceramics; ceramic; pottery; ceramic feedstock; processed material; ceramic feed mixture</x:v>
+      </x:c>
+      <x:c r="AE184" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="105" customHeight="1">
+      <x:c r="A185" s="9" t="str">
+        <x:v>proposal.ceramic.unfired_blank</x:v>
+      </x:c>
+      <x:c r="B185" s="9" t="str">
+        <x:v>Unfired shaped ceramic blank</x:v>
+      </x:c>
+      <x:c r="C185" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D185" s="9" t="str">
+        <x:v>Ceramic intermediate</x:v>
+      </x:c>
+      <x:c r="E185" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F185" s="9" t="str">
+        <x:v>A shaped intermediate awaiting its designed firing process.</x:v>
+      </x:c>
+      <x:c r="G185" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H185" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I185" s="13"/>
+      <x:c r="J185" s="15"/>
+      <x:c r="K185" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L185" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M185" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N185" s="9" t="str">
+        <x:v>Forming method and required binders remain proposals; not a usable finished part.</x:v>
+      </x:c>
+      <x:c r="O185" s="17"/>
+      <x:c r="P185" s="17"/>
+      <x:c r="Q185" s="17"/>
+      <x:c r="R185" s="17"/>
+      <x:c r="S185" s="17"/>
+      <x:c r="T185" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U185" s="11"/>
+      <x:c r="V185" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W185" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X185" s="4" t="str">
+        <x:v>Unfired intermediate</x:v>
+      </x:c>
+      <x:c r="Y185" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z185" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="AA185" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB185" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC185" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD185" s="4" t="str">
+        <x:v>unfired shaped ceramic blank; glass and ceramics; ceramic; pottery; ceramic intermediate; crafting component; ceramic</x:v>
+      </x:c>
+      <x:c r="AE185" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="105" customHeight="1">
+      <x:c r="A186" s="9" t="str">
+        <x:v>proposal.ceramic.bowl</x:v>
+      </x:c>
+      <x:c r="B186" s="9" t="str">
+        <x:v>Plain ceramic eating bowl</x:v>
+      </x:c>
+      <x:c r="C186" s="9" t="str">
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D186" s="9" t="str">
+        <x:v>Ceramic household</x:v>
+      </x:c>
+      <x:c r="E186" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F186" s="9" t="str">
+        <x:v>Simple ceramic bowl for contained algae portions.</x:v>
+      </x:c>
+      <x:c r="G186" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H186" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I186" s="13"/>
+      <x:c r="J186" s="15"/>
+      <x:c r="K186" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L186" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M186" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N186" s="9" t="str">
+        <x:v>Food-contact grade and surface finish require design; not a water vessel assumption.</x:v>
+      </x:c>
+      <x:c r="O186" s="17"/>
+      <x:c r="P186" s="17"/>
+      <x:c r="Q186" s="17"/>
+      <x:c r="R186" s="17"/>
+      <x:c r="S186" s="17"/>
+      <x:c r="T186" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U186" s="11"/>
+      <x:c r="V186" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W186" s="4" t="str">
+        <x:v>Household utensil</x:v>
+      </x:c>
+      <x:c r="X186" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y186" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z186" s="4" t="str">
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="AA186" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB186" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC186" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD186" s="4" t="str">
+        <x:v>plain ceramic eating bowl; food service; ceramic; pottery; ceramic household; household utensil; ceramic</x:v>
+      </x:c>
+      <x:c r="AE186" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="105" customHeight="1">
+      <x:c r="A187" s="9" t="str">
+        <x:v>proposal.ceramic.cup</x:v>
+      </x:c>
+      <x:c r="B187" s="9" t="str">
+        <x:v>Small ceramic cup</x:v>
+      </x:c>
+      <x:c r="C187" s="9" t="str">
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D187" s="9" t="str">
+        <x:v>Ceramic household</x:v>
+      </x:c>
+      <x:c r="E187" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F187" s="9" t="str">
+        <x:v>Small cup for a contained food portion or other assigned household use.</x:v>
+      </x:c>
+      <x:c r="G187" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H187" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I187" s="13"/>
+      <x:c r="J187" s="15"/>
+      <x:c r="K187" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L187" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M187" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N187" s="9" t="str">
+        <x:v>Contents and food-contact suitability must be defined; no natural water introduced.</x:v>
+      </x:c>
+      <x:c r="O187" s="17"/>
+      <x:c r="P187" s="17"/>
+      <x:c r="Q187" s="17"/>
+      <x:c r="R187" s="17"/>
+      <x:c r="S187" s="17"/>
+      <x:c r="T187" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U187" s="11"/>
+      <x:c r="V187" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W187" s="4" t="str">
+        <x:v>Household utensil</x:v>
+      </x:c>
+      <x:c r="X187" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y187" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z187" s="4" t="str">
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="AA187" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB187" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC187" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD187" s="4" t="str">
+        <x:v>small ceramic cup; food service; ceramic; pottery; ceramic household; household utensil; ceramic</x:v>
+      </x:c>
+      <x:c r="AE187" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="105" customHeight="1">
+      <x:c r="A188" s="9" t="str">
+        <x:v>proposal.ceramic.plate</x:v>
+      </x:c>
+      <x:c r="B188" s="9" t="str">
+        <x:v>Ceramic serving plate</x:v>
+      </x:c>
+      <x:c r="C188" s="9" t="str">
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D188" s="9" t="str">
+        <x:v>Ceramic household</x:v>
+      </x:c>
+      <x:c r="E188" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F188" s="9" t="str">
+        <x:v>Shallow plate for serving or separating food portions.</x:v>
+      </x:c>
+      <x:c r="G188" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H188" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I188" s="13"/>
+      <x:c r="J188" s="15"/>
+      <x:c r="K188" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L188" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M188" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N188" s="9" t="str">
+        <x:v>No edible-fauna nutritional improvement or cleanliness mechanic granted.</x:v>
+      </x:c>
+      <x:c r="O188" s="17"/>
+      <x:c r="P188" s="17"/>
+      <x:c r="Q188" s="17"/>
+      <x:c r="R188" s="17"/>
+      <x:c r="S188" s="17"/>
+      <x:c r="T188" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U188" s="11"/>
+      <x:c r="V188" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W188" s="4" t="str">
+        <x:v>Household utensil</x:v>
+      </x:c>
+      <x:c r="X188" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y188" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z188" s="4" t="str">
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="AA188" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB188" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC188" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD188" s="4" t="str">
+        <x:v>ceramic serving plate; food service; ceramic; pottery; ceramic household; household utensil; ceramic</x:v>
+      </x:c>
+      <x:c r="AE188" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="105" customHeight="1">
+      <x:c r="A189" s="9" t="str">
+        <x:v>proposal.ceramic.storage_crock</x:v>
+      </x:c>
+      <x:c r="B189" s="9" t="str">
+        <x:v>Ceramic dry-storage crock</x:v>
+      </x:c>
+      <x:c r="C189" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D189" s="9" t="str">
+        <x:v>Ceramic storage</x:v>
+      </x:c>
+      <x:c r="E189" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F189" s="9" t="str">
+        <x:v>Lidded vessel for selected dry household goods.</x:v>
+      </x:c>
+      <x:c r="G189" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H189" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I189" s="13"/>
+      <x:c r="J189" s="15"/>
+      <x:c r="K189" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L189" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M189" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N189" s="9" t="str">
+        <x:v>Not automatically sealed, airtight, pressure-rated or chemically compatible.</x:v>
+      </x:c>
+      <x:c r="O189" s="17"/>
+      <x:c r="P189" s="17"/>
+      <x:c r="Q189" s="17"/>
+      <x:c r="R189" s="17"/>
+      <x:c r="S189" s="17"/>
+      <x:c r="T189" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U189" s="11"/>
+      <x:c r="V189" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W189" s="4" t="str">
+        <x:v>Container</x:v>
+      </x:c>
+      <x:c r="X189" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y189" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z189" s="4" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="AA189" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB189" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC189" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD189" s="4" t="str">
+        <x:v>ceramic dry-storage crock; liquid and bulk containment; cargo organization; ceramic; pottery; ceramic storage; container; ceramic</x:v>
+      </x:c>
+      <x:c r="AE189" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="105" customHeight="1">
+      <x:c r="A190" s="9" t="str">
+        <x:v>proposal.ceramic.crucible</x:v>
+      </x:c>
+      <x:c r="B190" s="9" t="str">
+        <x:v>Ceramic crucible</x:v>
+      </x:c>
+      <x:c r="C190" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D190" s="9" t="str">
+        <x:v>Ceramic workshop</x:v>
+      </x:c>
+      <x:c r="E190" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F190" s="9" t="str">
+        <x:v>Specialist vessel candidate for a selected high-temperature material process.</x:v>
+      </x:c>
+      <x:c r="G190" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H190" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I190" s="13"/>
+      <x:c r="J190" s="15"/>
+      <x:c r="K190" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L190" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M190" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N190" s="9" t="str">
+        <x:v>Composition, supported contents and temperature range unresolved; ordinary pottery is not interchangeable.</x:v>
+      </x:c>
+      <x:c r="O190" s="17"/>
+      <x:c r="P190" s="17"/>
+      <x:c r="Q190" s="17"/>
+      <x:c r="R190" s="17"/>
+      <x:c r="S190" s="17"/>
+      <x:c r="T190" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U190" s="11"/>
+      <x:c r="V190" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W190" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X190" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y190" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z190" s="4" t="str">
+        <x:v>Metal refining</x:v>
+      </x:c>
+      <x:c r="AA190" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB190" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC190" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD190" s="4" t="str">
+        <x:v>ceramic crucible; glass and ceramics; metal refining; ceramic; pottery; ceramic workshop; tool; ceramic</x:v>
+      </x:c>
+      <x:c r="AE190" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="105" customHeight="1">
+      <x:c r="A191" s="9" t="str">
+        <x:v>proposal.ceramic.casting_mold</x:v>
+      </x:c>
+      <x:c r="B191" s="9" t="str">
+        <x:v>Ceramic casting mold</x:v>
+      </x:c>
+      <x:c r="C191" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D191" s="9" t="str">
+        <x:v>Ceramic workshop</x:v>
+      </x:c>
+      <x:c r="E191" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F191" s="9" t="str">
+        <x:v>A shaped mold for a specifically chosen casting process.</x:v>
+      </x:c>
+      <x:c r="G191" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H191" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I191" s="13"/>
+      <x:c r="J191" s="15"/>
+      <x:c r="K191" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L191" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M191" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N191" s="9" t="str">
+        <x:v>Process compatibility, release, lifetime and reusable versus expendable construction TBD.</x:v>
+      </x:c>
+      <x:c r="O191" s="17"/>
+      <x:c r="P191" s="17"/>
+      <x:c r="Q191" s="17"/>
+      <x:c r="R191" s="17"/>
+      <x:c r="S191" s="17"/>
+      <x:c r="T191" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U191" s="11"/>
+      <x:c r="V191" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W191" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X191" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y191" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z191" s="4" t="str">
+        <x:v>Fabrication</x:v>
+      </x:c>
+      <x:c r="AA191" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB191" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC191" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD191" s="4" t="str">
+        <x:v>ceramic casting mold; metal refining; fabrication; ceramic; pottery; ceramic workshop; tool; ceramic</x:v>
+      </x:c>
+      <x:c r="AE191" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="105" customHeight="1">
+      <x:c r="A192" s="9" t="str">
+        <x:v>proposal.ceramic.mortar</x:v>
+      </x:c>
+      <x:c r="B192" s="9" t="str">
+        <x:v>Ceramic grinding mortar</x:v>
+      </x:c>
+      <x:c r="C192" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D192" s="9" t="str">
+        <x:v>Ceramic workshop</x:v>
+      </x:c>
+      <x:c r="E192" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F192" s="9" t="str">
+        <x:v>Bowl-shaped workshop tool for controlled grinding of selected feed.</x:v>
+      </x:c>
+      <x:c r="G192" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H192" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I192" s="13"/>
+      <x:c r="J192" s="15"/>
+      <x:c r="K192" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L192" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M192" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N192" s="9" t="str">
+        <x:v>Grinding suitability and contamination matter; not interchangeable with an eating bowl.</x:v>
+      </x:c>
+      <x:c r="O192" s="17"/>
+      <x:c r="P192" s="17"/>
+      <x:c r="Q192" s="17"/>
+      <x:c r="R192" s="17"/>
+      <x:c r="S192" s="17"/>
+      <x:c r="T192" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U192" s="11"/>
+      <x:c r="V192" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W192" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X192" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y192" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z192" s="4" t="str">
+        <x:v>Chemical processing</x:v>
+      </x:c>
+      <x:c r="AA192" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB192" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC192" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD192" s="4" t="str">
+        <x:v>ceramic grinding mortar; glass and ceramics; chemical processing; ceramic; pottery; ceramic workshop; tool; ceramic</x:v>
+      </x:c>
+      <x:c r="AE192" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="105" customHeight="1">
+      <x:c r="A193" s="9" t="str">
+        <x:v>proposal.ceramic.pestle</x:v>
+      </x:c>
+      <x:c r="B193" s="9" t="str">
+        <x:v>Ceramic pestle</x:v>
+      </x:c>
+      <x:c r="C193" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D193" s="9" t="str">
+        <x:v>Ceramic workshop</x:v>
+      </x:c>
+      <x:c r="E193" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F193" s="9" t="str">
+        <x:v>Grinding tool used with a compatible mortar.</x:v>
+      </x:c>
+      <x:c r="G193" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H193" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I193" s="13"/>
+      <x:c r="J193" s="15"/>
+      <x:c r="K193" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L193" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M193" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N193" s="9" t="str">
+        <x:v>Companion mortar remains separately owned; no automatic processing recipe.</x:v>
+      </x:c>
+      <x:c r="O193" s="17"/>
+      <x:c r="P193" s="17"/>
+      <x:c r="Q193" s="17"/>
+      <x:c r="R193" s="17"/>
+      <x:c r="S193" s="17"/>
+      <x:c r="T193" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U193" s="11"/>
+      <x:c r="V193" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W193" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X193" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y193" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z193" s="4" t="str">
+        <x:v>Chemical processing</x:v>
+      </x:c>
+      <x:c r="AA193" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB193" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC193" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD193" s="4" t="str">
+        <x:v>ceramic pestle; glass and ceramics; chemical processing; ceramic; pottery; ceramic workshop; tool; ceramic</x:v>
+      </x:c>
+      <x:c r="AE193" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="105" customHeight="1">
+      <x:c r="A194" s="9" t="str">
+        <x:v>proposal.ceramic.firing_tray</x:v>
+      </x:c>
+      <x:c r="B194" s="9" t="str">
+        <x:v>Ceramic firing tray</x:v>
+      </x:c>
+      <x:c r="C194" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D194" s="9" t="str">
+        <x:v>Ceramic workshop</x:v>
+      </x:c>
+      <x:c r="E194" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F194" s="9" t="str">
+        <x:v>Support selected small parts in a proposed firing setup.</x:v>
+      </x:c>
+      <x:c r="G194" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H194" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I194" s="13"/>
+      <x:c r="J194" s="15"/>
+      <x:c r="K194" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L194" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M194" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N194" s="9" t="str">
+        <x:v>Suitable ceramic grade, kiln system and firing behavior are undefined.</x:v>
+      </x:c>
+      <x:c r="O194" s="17"/>
+      <x:c r="P194" s="17"/>
+      <x:c r="Q194" s="17"/>
+      <x:c r="R194" s="17"/>
+      <x:c r="S194" s="17"/>
+      <x:c r="T194" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U194" s="11"/>
+      <x:c r="V194" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W194" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X194" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y194" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z194" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="AA194" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB194" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC194" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD194" s="4" t="str">
+        <x:v>ceramic firing tray; glass and ceramics; ceramic; pottery; ceramic workshop; tool; ceramic</x:v>
+      </x:c>
+      <x:c r="AE194" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="105" customHeight="1">
+      <x:c r="A195" s="9" t="str">
+        <x:v>proposal.ceramic.refractory_brick</x:v>
+      </x:c>
+      <x:c r="B195" s="9" t="str">
+        <x:v>Refractory ceramic brick</x:v>
+      </x:c>
+      <x:c r="C195" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D195" s="9" t="str">
+        <x:v>Ceramic thermal component</x:v>
+      </x:c>
+      <x:c r="E195" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F195" s="9" t="str">
+        <x:v>Specialist lining brick for a compatible furnace or kiln.</x:v>
+      </x:c>
+      <x:c r="G195" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H195" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I195" s="13"/>
+      <x:c r="J195" s="15"/>
+      <x:c r="K195" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L195" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M195" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N195" s="9" t="str">
+        <x:v>Heat-service composition and installation unresolved; no universal fire immunity.</x:v>
+      </x:c>
+      <x:c r="O195" s="17"/>
+      <x:c r="P195" s="17"/>
+      <x:c r="Q195" s="17"/>
+      <x:c r="R195" s="17"/>
+      <x:c r="S195" s="17"/>
+      <x:c r="T195" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U195" s="11"/>
+      <x:c r="V195" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W195" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X195" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y195" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z195" s="4" t="str">
+        <x:v>Protective fabrication</x:v>
+      </x:c>
+      <x:c r="AA195" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB195" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC195" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD195" s="4" t="str">
+        <x:v>refractory ceramic brick; glass and ceramics; metal refining; protective fabrication; ceramic; pottery; ceramic thermal component; crafting component; ceramic</x:v>
+      </x:c>
+      <x:c r="AE195" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="105" customHeight="1">
+      <x:c r="A196" s="9" t="str">
+        <x:v>proposal.ceramic.kiln_liner</x:v>
+      </x:c>
+      <x:c r="B196" s="9" t="str">
+        <x:v>Ceramic kiln lining panel</x:v>
+      </x:c>
+      <x:c r="C196" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D196" s="9" t="str">
+        <x:v>Ceramic thermal component</x:v>
+      </x:c>
+      <x:c r="E196" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F196" s="9" t="str">
+        <x:v>Replaceable shaped hot-face panel for a proposed stationary kiln.</x:v>
+      </x:c>
+      <x:c r="G196" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H196" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I196" s="13"/>
+      <x:c r="J196" s="15"/>
+      <x:c r="K196" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L196" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M196" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N196" s="9" t="str">
+        <x:v>Panel differs from brick geometry; kiln implementation and thermal properties TBD.</x:v>
+      </x:c>
+      <x:c r="O196" s="17"/>
+      <x:c r="P196" s="17"/>
+      <x:c r="Q196" s="17"/>
+      <x:c r="R196" s="17"/>
+      <x:c r="S196" s="17"/>
+      <x:c r="T196" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U196" s="11"/>
+      <x:c r="V196" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W196" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X196" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y196" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z196" s="4" t="str">
+        <x:v>Protective fabrication</x:v>
+      </x:c>
+      <x:c r="AA196" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB196" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC196" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD196" s="4" t="str">
+        <x:v>ceramic kiln lining panel; glass and ceramics; protective fabrication; ceramic; pottery; ceramic thermal component; crafting component; ceramic</x:v>
+      </x:c>
+      <x:c r="AE196" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="105" customHeight="1">
+      <x:c r="A197" s="9" t="str">
+        <x:v>proposal.ceramic.bead</x:v>
+      </x:c>
+      <x:c r="B197" s="9" t="str">
+        <x:v>Ceramic insulating bead</x:v>
+      </x:c>
+      <x:c r="C197" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D197" s="9" t="str">
+        <x:v>Ceramic electrical component</x:v>
+      </x:c>
+      <x:c r="E197" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F197" s="9" t="str">
+        <x:v>Small fitted bead candidate for separating selected conductor sections.</x:v>
+      </x:c>
+      <x:c r="G197" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H197" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I197" s="13"/>
+      <x:c r="J197" s="15"/>
+      <x:c r="K197" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L197" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M197" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N197" s="9" t="str">
+        <x:v>Voltage, contamination, geometry and mounting unresolved; no lightning immunity.</x:v>
+      </x:c>
+      <x:c r="O197" s="17"/>
+      <x:c r="P197" s="17"/>
+      <x:c r="Q197" s="17"/>
+      <x:c r="R197" s="17"/>
+      <x:c r="S197" s="17"/>
+      <x:c r="T197" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U197" s="11"/>
+      <x:c r="V197" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W197" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X197" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y197" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z197" s="4" t="str">
+        <x:v>Electrical insulation</x:v>
+      </x:c>
+      <x:c r="AA197" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB197" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC197" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD197" s="4" t="str">
+        <x:v>ceramic insulating bead; electrical work; electrical insulation; ceramic; pottery; ceramic electrical component; crafting component; ceramic</x:v>
+      </x:c>
+      <x:c r="AE197" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="105" customHeight="1">
+      <x:c r="A198" s="9" t="str">
+        <x:v>proposal.ceramic.spacer</x:v>
+      </x:c>
+      <x:c r="B198" s="9" t="str">
+        <x:v>Ceramic insulating spacer</x:v>
+      </x:c>
+      <x:c r="C198" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D198" s="9" t="str">
+        <x:v>Ceramic electrical component</x:v>
+      </x:c>
+      <x:c r="E198" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F198" s="9" t="str">
+        <x:v>Hard standoff separating compatible conductive parts.</x:v>
+      </x:c>
+      <x:c r="G198" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H198" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I198" s="13"/>
+      <x:c r="J198" s="15"/>
+      <x:c r="K198" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L198" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M198" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N198" s="9" t="str">
+        <x:v>Shape-specific part within existing insulating-blank family; no universal substitution.</x:v>
+      </x:c>
+      <x:c r="O198" s="17"/>
+      <x:c r="P198" s="17"/>
+      <x:c r="Q198" s="17"/>
+      <x:c r="R198" s="17"/>
+      <x:c r="S198" s="17"/>
+      <x:c r="T198" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U198" s="11"/>
+      <x:c r="V198" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W198" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X198" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y198" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z198" s="4" t="str">
+        <x:v>Electrical insulation</x:v>
+      </x:c>
+      <x:c r="AA198" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB198" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC198" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD198" s="4" t="str">
+        <x:v>ceramic insulating spacer; electrical work; electrical insulation; ceramic; pottery; ceramic electrical component; crafting component; ceramic</x:v>
+      </x:c>
+      <x:c r="AE198" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="105" customHeight="1">
+      <x:c r="A199" s="9" t="str">
+        <x:v>proposal.ceramic.feedthrough</x:v>
+      </x:c>
+      <x:c r="B199" s="9" t="str">
+        <x:v>Ceramic electrical feedthrough</x:v>
+      </x:c>
+      <x:c r="C199" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D199" s="9" t="str">
+        <x:v>Ceramic electrical component</x:v>
+      </x:c>
+      <x:c r="E199" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F199" s="9" t="str">
+        <x:v>Fitted ceramic/conductor assembly routing an electrical connection through a housing.</x:v>
+      </x:c>
+      <x:c r="G199" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H199" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I199" s="13"/>
+      <x:c r="J199" s="15"/>
+      <x:c r="K199" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L199" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M199" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N199" s="9" t="str">
+        <x:v>Material, seals, voltage and intended service unresolved.</x:v>
+      </x:c>
+      <x:c r="O199" s="17"/>
+      <x:c r="P199" s="17"/>
+      <x:c r="Q199" s="17"/>
+      <x:c r="R199" s="17"/>
+      <x:c r="S199" s="17"/>
+      <x:c r="T199" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U199" s="11"/>
+      <x:c r="V199" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W199" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X199" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y199" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z199" s="4" t="str">
+        <x:v>Electrical insulation</x:v>
+      </x:c>
+      <x:c r="AA199" s="4" t="str">
+        <x:v>Ceramic and metal</x:v>
+      </x:c>
+      <x:c r="AB199" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC199" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD199" s="4" t="str">
+        <x:v>ceramic electrical feedthrough; electrical conduction; electrical insulation; ceramic; pottery; ceramic electrical component; crafting component; ceramic and metal</x:v>
+      </x:c>
+      <x:c r="AE199" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="105" customHeight="1">
+      <x:c r="A200" s="9" t="str">
+        <x:v>proposal.ceramic.stopper</x:v>
+      </x:c>
+      <x:c r="B200" s="9" t="str">
+        <x:v>Fitted ceramic stopper</x:v>
+      </x:c>
+      <x:c r="C200" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D200" s="9" t="str">
+        <x:v>Ceramic vessel fitting</x:v>
+      </x:c>
+      <x:c r="E200" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F200" s="9" t="str">
+        <x:v>Hard closure shaped for its matching vessel.</x:v>
+      </x:c>
+      <x:c r="G200" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H200" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I200" s="13"/>
+      <x:c r="J200" s="15"/>
+      <x:c r="K200" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L200" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M200" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N200" s="9" t="str">
+        <x:v>Not automatically leak-tight; compatible seat and sealing material may be required.</x:v>
+      </x:c>
+      <x:c r="O200" s="17"/>
+      <x:c r="P200" s="17"/>
+      <x:c r="Q200" s="17"/>
+      <x:c r="R200" s="17"/>
+      <x:c r="S200" s="17"/>
+      <x:c r="T200" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U200" s="11"/>
+      <x:c r="V200" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W200" s="4" t="str">
+        <x:v>Container part</x:v>
+      </x:c>
+      <x:c r="X200" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y200" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z200" s="4" t="str">
+        <x:v>Sealing</x:v>
+      </x:c>
+      <x:c r="AA200" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB200" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC200" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD200" s="4" t="str">
+        <x:v>fitted ceramic stopper; sealing; ceramic; pottery; ceramic vessel fitting; container part; ceramic</x:v>
+      </x:c>
+      <x:c r="AE200" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="105" customHeight="1">
+      <x:c r="A201" s="9" t="str">
+        <x:v>proposal.ceramic.lid</x:v>
+      </x:c>
+      <x:c r="B201" s="9" t="str">
+        <x:v>Ceramic vessel lid</x:v>
+      </x:c>
+      <x:c r="C201" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D201" s="9" t="str">
+        <x:v>Ceramic vessel fitting</x:v>
+      </x:c>
+      <x:c r="E201" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F201" s="9" t="str">
+        <x:v>Removable cover matched to an open-topped ceramic vessel.</x:v>
+      </x:c>
+      <x:c r="G201" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H201" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I201" s="13"/>
+      <x:c r="J201" s="15"/>
+      <x:c r="K201" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L201" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M201" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N201" s="9" t="str">
+        <x:v>A cover is distinct from a pressure seal or a matched neck stopper.</x:v>
+      </x:c>
+      <x:c r="O201" s="17"/>
+      <x:c r="P201" s="17"/>
+      <x:c r="Q201" s="17"/>
+      <x:c r="R201" s="17"/>
+      <x:c r="S201" s="17"/>
+      <x:c r="T201" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U201" s="11"/>
+      <x:c r="V201" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W201" s="4" t="str">
+        <x:v>Container part</x:v>
+      </x:c>
+      <x:c r="X201" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y201" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z201" s="4" t="str">
+        <x:v>Liquid and bulk containment</x:v>
+      </x:c>
+      <x:c r="AA201" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB201" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC201" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD201" s="4" t="str">
+        <x:v>ceramic vessel lid; dust exclusion; liquid and bulk containment; ceramic; pottery; ceramic vessel fitting; container part; ceramic</x:v>
+      </x:c>
+      <x:c r="AE201" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="105" customHeight="1">
+      <x:c r="A202" s="9" t="str">
+        <x:v>proposal.ceramic.pour_spout</x:v>
+      </x:c>
+      <x:c r="B202" s="9" t="str">
+        <x:v>Ceramic pouring spout</x:v>
+      </x:c>
+      <x:c r="C202" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D202" s="9" t="str">
+        <x:v>Ceramic vessel fitting</x:v>
+      </x:c>
+      <x:c r="E202" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F202" s="9" t="str">
+        <x:v>Replaceable outlet candidate for compatible contained material.</x:v>
+      </x:c>
+      <x:c r="G202" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H202" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I202" s="13"/>
+      <x:c r="J202" s="15"/>
+      <x:c r="K202" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L202" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M202" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N202" s="9" t="str">
+        <x:v>Viscosity, joints and chemical suitability unresolved; not a universal ichor fitting.</x:v>
+      </x:c>
+      <x:c r="O202" s="17"/>
+      <x:c r="P202" s="17"/>
+      <x:c r="Q202" s="17"/>
+      <x:c r="R202" s="17"/>
+      <x:c r="S202" s="17"/>
+      <x:c r="T202" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U202" s="11"/>
+      <x:c r="V202" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W202" s="4" t="str">
+        <x:v>Container part</x:v>
+      </x:c>
+      <x:c r="X202" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y202" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z202" s="4" t="str">
+        <x:v>Material transfer</x:v>
+      </x:c>
+      <x:c r="AA202" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB202" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC202" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD202" s="4" t="str">
+        <x:v>ceramic pouring spout; material transfer; ceramic; pottery; ceramic vessel fitting; container part; ceramic</x:v>
+      </x:c>
+      <x:c r="AE202" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="105" customHeight="1">
+      <x:c r="A203" s="9" t="str">
+        <x:v>proposal.ceramic.conduit</x:v>
+      </x:c>
+      <x:c r="B203" s="9" t="str">
+        <x:v>Ceramic conduit section</x:v>
+      </x:c>
+      <x:c r="C203" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D203" s="9" t="str">
+        <x:v>Ceramic vessel fitting</x:v>
+      </x:c>
+      <x:c r="E203" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F203" s="9" t="str">
+        <x:v>Rigid channel candidate for an assigned industrial transfer route.</x:v>
+      </x:c>
+      <x:c r="G203" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H203" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I203" s="13"/>
+      <x:c r="J203" s="15"/>
+      <x:c r="K203" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L203" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M203" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N203" s="9" t="str">
+        <x:v>Contents, joints and installation TBD; does not establish outdoor liquid streams.</x:v>
+      </x:c>
+      <x:c r="O203" s="17"/>
+      <x:c r="P203" s="17"/>
+      <x:c r="Q203" s="17"/>
+      <x:c r="R203" s="17"/>
+      <x:c r="S203" s="17"/>
+      <x:c r="T203" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U203" s="11"/>
+      <x:c r="V203" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W203" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X203" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y203" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z203" s="4" t="str">
+        <x:v>Material transfer</x:v>
+      </x:c>
+      <x:c r="AA203" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB203" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC203" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD203" s="4" t="str">
+        <x:v>ceramic conduit section; material transfer; ceramic; pottery; ceramic vessel fitting; crafting component; ceramic</x:v>
+      </x:c>
+      <x:c r="AE203" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="105" customHeight="1">
+      <x:c r="A204" s="9" t="str">
+        <x:v>proposal.ceramic.votive_plaque</x:v>
+      </x:c>
+      <x:c r="B204" s="9" t="str">
+        <x:v>Ceramic votive plaque</x:v>
+      </x:c>
+      <x:c r="C204" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D204" s="9" t="str">
+        <x:v>Ceramic ceremonial</x:v>
+      </x:c>
+      <x:c r="E204" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F204" s="9" t="str">
+        <x:v>Small ceramic offering or devotional image.</x:v>
+      </x:c>
+      <x:c r="G204" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H204" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I204" s="13"/>
+      <x:c r="J204" s="15"/>
+      <x:c r="K204" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L204" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M204" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N204" s="9" t="str">
+        <x:v>New material-specific craft family; iconography and institutional acceptance remain proposals.</x:v>
+      </x:c>
+      <x:c r="O204" s="17"/>
+      <x:c r="P204" s="17"/>
+      <x:c r="Q204" s="17"/>
+      <x:c r="R204" s="17"/>
+      <x:c r="S204" s="17"/>
+      <x:c r="T204" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U204" s="11"/>
+      <x:c r="V204" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W204" s="4" t="str">
+        <x:v>Cultural object</x:v>
+      </x:c>
+      <x:c r="X204" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y204" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z204" s="4" t="str">
+        <x:v>Devotion</x:v>
+      </x:c>
+      <x:c r="AA204" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB204" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC204" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD204" s="4" t="str">
+        <x:v>ceramic votive plaque; decoration; devotion; ceramic; pottery; ceramic ceremonial; cultural object; ceramic</x:v>
+      </x:c>
+      <x:c r="AE204" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="105" customHeight="1">
+      <x:c r="A205" s="9" t="str">
+        <x:v>proposal.ceramic.figurine</x:v>
+      </x:c>
+      <x:c r="B205" s="9" t="str">
+        <x:v>Ceramic commemorative figurine</x:v>
+      </x:c>
+      <x:c r="C205" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D205" s="9" t="str">
+        <x:v>Ceramic ceremonial</x:v>
+      </x:c>
+      <x:c r="E205" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F205" s="9" t="str">
+        <x:v>Sculpted keepsake of a person, creature or significant event.</x:v>
+      </x:c>
+      <x:c r="G205" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H205" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I205" s="13"/>
+      <x:c r="J205" s="15"/>
+      <x:c r="K205" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L205" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M205" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N205" s="9" t="str">
+        <x:v>Subject matter and style TBD; no relic authenticity or supernatural property.</x:v>
+      </x:c>
+      <x:c r="O205" s="17"/>
+      <x:c r="P205" s="17"/>
+      <x:c r="Q205" s="17"/>
+      <x:c r="R205" s="17"/>
+      <x:c r="S205" s="17"/>
+      <x:c r="T205" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U205" s="11"/>
+      <x:c r="V205" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W205" s="4" t="str">
+        <x:v>Cultural object</x:v>
+      </x:c>
+      <x:c r="X205" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y205" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z205" s="4" t="str">
+        <x:v>Remembrance</x:v>
+      </x:c>
+      <x:c r="AA205" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB205" s="4" t="str">
+        <x:v>Solid piece</x:v>
+      </x:c>
+      <x:c r="AC205" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD205" s="4" t="str">
+        <x:v>ceramic commemorative figurine; decoration; remembrance; ceramic; pottery; ceramic ceremonial; cultural object; ceramic</x:v>
+      </x:c>
+      <x:c r="AE205" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="105" customHeight="1">
+      <x:c r="A206" s="9" t="str">
+        <x:v>proposal.ceramic.ceremony_bowl</x:v>
+      </x:c>
+      <x:c r="B206" s="9" t="str">
+        <x:v>Ceremonial ceramic bowl</x:v>
+      </x:c>
+      <x:c r="C206" s="9" t="str">
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D206" s="9" t="str">
+        <x:v>Ceramic ceremonial</x:v>
+      </x:c>
+      <x:c r="E206" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F206" s="9" t="str">
+        <x:v>Dedicated presentation bowl with selected finish or engraving.</x:v>
+      </x:c>
+      <x:c r="G206" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H206" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I206" s="13"/>
+      <x:c r="J206" s="15"/>
+      <x:c r="K206" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L206" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M206" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N206" s="9" t="str">
+        <x:v>Ceremonial workmanship distinguishes this from ordinary tableware; contents unspecified.</x:v>
+      </x:c>
+      <x:c r="O206" s="17"/>
+      <x:c r="P206" s="17"/>
+      <x:c r="Q206" s="17"/>
+      <x:c r="R206" s="17"/>
+      <x:c r="S206" s="17"/>
+      <x:c r="T206" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U206" s="11"/>
+      <x:c r="V206" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W206" s="4" t="str">
+        <x:v>Cultural object</x:v>
+      </x:c>
+      <x:c r="X206" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y206" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z206" s="4" t="str">
+        <x:v>Ceremony</x:v>
+      </x:c>
+      <x:c r="AA206" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB206" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC206" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD206" s="4" t="str">
+        <x:v>ceremonial ceramic bowl; decoration; ceremony; ceramic; pottery; ceramic ceremonial; cultural object; ceramic</x:v>
+      </x:c>
+      <x:c r="AE206" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="105" customHeight="1">
+      <x:c r="A207" s="9" t="str">
+        <x:v>proposal.ceramic.armor_insert</x:v>
+      </x:c>
+      <x:c r="B207" s="9" t="str">
+        <x:v>Specialist ceramic armor insert</x:v>
+      </x:c>
+      <x:c r="C207" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D207" s="9" t="str">
+        <x:v>Ceramic protection</x:v>
+      </x:c>
+      <x:c r="E207" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F207" s="9" t="str">
+        <x:v>Candidate fitted insert in the existing specialized-armor-plate family.</x:v>
+      </x:c>
+      <x:c r="G207" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H207" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I207" s="13"/>
+      <x:c r="J207" s="15"/>
+      <x:c r="K207" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L207" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M207" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N207" s="9" t="str">
+        <x:v>Performance, brittleness, mounting and damage behavior undecided; no protection stats.</x:v>
+      </x:c>
+      <x:c r="O207" s="17"/>
+      <x:c r="P207" s="17"/>
+      <x:c r="Q207" s="17"/>
+      <x:c r="R207" s="17"/>
+      <x:c r="S207" s="17"/>
+      <x:c r="T207" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U207" s="11"/>
+      <x:c r="V207" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W207" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X207" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y207" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z207" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA207" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB207" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC207" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD207" s="4" t="str">
+        <x:v>specialist ceramic armor insert; protection; ceramic; pottery; ceramic protection; armor; ceramic</x:v>
+      </x:c>
+      <x:c r="AE207" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="105" customHeight="1">
+      <x:c r="A208" s="9" t="str">
+        <x:v>proposal.ceramic.fastener</x:v>
+      </x:c>
+      <x:c r="B208" s="9" t="str">
+        <x:v>Ceramic toggle fastener</x:v>
+      </x:c>
+      <x:c r="C208" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D208" s="9" t="str">
+        <x:v>Ceramic household fitting</x:v>
+      </x:c>
+      <x:c r="E208" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F208" s="9" t="str">
+        <x:v>Shaped toggle for a compatible wrap or fitted carrier.</x:v>
+      </x:c>
+      <x:c r="G208" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H208" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I208" s="13"/>
+      <x:c r="J208" s="15"/>
+      <x:c r="K208" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L208" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M208" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N208" s="9" t="str">
+        <x:v>No cloth required; joining method, strength and wear properties unresolved.</x:v>
+      </x:c>
+      <x:c r="O208" s="17"/>
+      <x:c r="P208" s="17"/>
+      <x:c r="Q208" s="17"/>
+      <x:c r="R208" s="17"/>
+      <x:c r="S208" s="17"/>
+      <x:c r="T208" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U208" s="11"/>
+      <x:c r="V208" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W208" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X208" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y208" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z208" s="4" t="str">
+        <x:v>Clothing fabrication</x:v>
+      </x:c>
+      <x:c r="AA208" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB208" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC208" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD208" s="4" t="str">
+        <x:v>ceramic toggle fastener; equipment mounting; clothing fabrication; ceramic; pottery; ceramic household fitting; crafting component; ceramic</x:v>
+      </x:c>
+      <x:c r="AE208" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="105" customHeight="1">
+      <x:c r="A209" s="9" t="str">
+        <x:v>proposal.ceramic.grinding_disc</x:v>
+      </x:c>
+      <x:c r="B209" s="9" t="str">
+        <x:v>Ceramic abrasive disc</x:v>
+      </x:c>
+      <x:c r="C209" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D209" s="9" t="str">
+        <x:v>Ceramic workshop</x:v>
+      </x:c>
+      <x:c r="E209" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F209" s="9" t="str">
+        <x:v>Replaceable shaped abrasive for a chosen workshop tool.</x:v>
+      </x:c>
+      <x:c r="G209" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H209" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I209" s="13"/>
+      <x:c r="J209" s="15"/>
+      <x:c r="K209" s="9" t="str">
+        <x:v>Specialist ceramic craft or trade; exact production route TBD</x:v>
+      </x:c>
+      <x:c r="L209" s="9" t="str">
+        <x:v>Build on existing claystone, alumina, mineral feeds and insulating blanks where appropriate. No recipe authored.</x:v>
+      </x:c>
+      <x:c r="M209" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N209" s="9" t="str">
+        <x:v>Abrasive grade, drive method and safe operating limits unresolved; no powered tool granted.</x:v>
+      </x:c>
+      <x:c r="O209" s="17"/>
+      <x:c r="P209" s="17"/>
+      <x:c r="Q209" s="17"/>
+      <x:c r="R209" s="17"/>
+      <x:c r="S209" s="17"/>
+      <x:c r="T209" s="9" t="str">
+        <x:v>Ceramics requested as a broad item family. Specific objects, grades, sourcing, yield and value remain proposals.</x:v>
+      </x:c>
+      <x:c r="U209" s="11"/>
+      <x:c r="V209" s="9" t="str">
+        <x:v>Author ceramics direction October 14, 2026; local game item proposal. Existing mineral/ceramic entries reused where applicable.</x:v>
+      </x:c>
+      <x:c r="W209" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X209" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y209" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z209" s="4" t="str">
+        <x:v>Surface finishing</x:v>
+      </x:c>
+      <x:c r="AA209" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB209" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC209" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD209" s="4" t="str">
+        <x:v>ceramic abrasive disc; surface finishing; ceramic; pottery; ceramic workshop; tool; ceramic</x:v>
+      </x:c>
+      <x:c r="AE209" s="4" t="str">
+        <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15142,27 +17354,27 @@
       <x:formula1>'Taxonomy'!$B$14:$B$34</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="X6:X1005">
-      <x:formula1>'Taxonomy'!$B$35:$B$42</x:formula1>
+      <x:formula1>'Taxonomy'!$B$35:$B$43</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Y6:Y1005">
-      <x:formula1>'Taxonomy'!$B$43:$B$50</x:formula1>
+      <x:formula1>'Taxonomy'!$B$44:$B$51</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Z6:Z1005">
-      <x:formula1>'Taxonomy'!$B$51:$B$113</x:formula1>
+      <x:formula1>'Taxonomy'!$B$52:$B$114</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AA6:AA1005">
-      <x:formula1>'Taxonomy'!$B$114:$B$140</x:formula1>
+      <x:formula1>'Taxonomy'!$B$115:$B$143</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AB6:AB1005">
-      <x:formula1>'Taxonomy'!$B$141:$B$159</x:formula1>
+      <x:formula1>'Taxonomy'!$B$144:$B$162</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AC6:AC1005">
-      <x:formula1>'Taxonomy'!$B$160:$B$163</x:formula1>
+      <x:formula1>'Taxonomy'!$B$163:$B$166</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc4c813a8d3b4dca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5501e6d9e0d43c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15814,7 +18026,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ea629fbf35241f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46709f5344f24c0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16296,7 +18508,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8309fcd26d924935"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35bcf7942e314fd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16721,7 +18933,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B41" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Unfired intermediate</x:v>
       </x:c>
       <x:c r="C41" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -16732,7 +18944,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B42" s="4" t="str">
-        <x:v>Unworked metal</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C42" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -16740,13 +18952,13 @@
     </x:row>
     <x:row r="43" ht="45" customHeight="1">
       <x:c r="A43" s="4" t="str">
-        <x:v>Origin family</x:v>
+        <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B43" s="4" t="str">
-        <x:v>Ancient technology</x:v>
+        <x:v>Unworked metal</x:v>
       </x:c>
       <x:c r="C43" s="4" t="str">
-        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
+        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="45" customHeight="1">
@@ -16754,7 +18966,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B44" s="4" t="str">
-        <x:v>Atmospheric</x:v>
+        <x:v>Ancient technology</x:v>
       </x:c>
       <x:c r="C44" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -16765,7 +18977,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B45" s="4" t="str">
-        <x:v>Fauna</x:v>
+        <x:v>Atmospheric</x:v>
       </x:c>
       <x:c r="C45" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -16776,7 +18988,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B46" s="4" t="str">
-        <x:v>Geological</x:v>
+        <x:v>Fauna</x:v>
       </x:c>
       <x:c r="C46" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -16787,7 +18999,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B47" s="4" t="str">
-        <x:v>Living culture</x:v>
+        <x:v>Geological</x:v>
       </x:c>
       <x:c r="C47" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -16798,7 +19010,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B48" s="4" t="str">
-        <x:v>Manufactured / unresolved</x:v>
+        <x:v>Living culture</x:v>
       </x:c>
       <x:c r="C48" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -16809,7 +19021,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B49" s="4" t="str">
-        <x:v>Recovered machinery</x:v>
+        <x:v>Manufactured / unresolved</x:v>
       </x:c>
       <x:c r="C49" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -16820,7 +19032,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B50" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Recovered machinery</x:v>
       </x:c>
       <x:c r="C50" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -16828,13 +19040,13 @@
     </x:row>
     <x:row r="51" ht="45" customHeight="1">
       <x:c r="A51" s="4" t="str">
-        <x:v>Primary use</x:v>
+        <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B51" s="4" t="str">
-        <x:v>Area denial</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C51" s="4" t="str">
-        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
+        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="45" customHeight="1">
@@ -16842,7 +19054,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B52" s="4" t="str">
-        <x:v>Binding and construction</x:v>
+        <x:v>Area denial</x:v>
       </x:c>
       <x:c r="C52" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16853,7 +19065,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B53" s="4" t="str">
-        <x:v>Camp rest</x:v>
+        <x:v>Binding and construction</x:v>
       </x:c>
       <x:c r="C53" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16864,7 +19076,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B54" s="4" t="str">
-        <x:v>Cargo organization</x:v>
+        <x:v>Camp rest</x:v>
       </x:c>
       <x:c r="C54" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16875,7 +19087,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B55" s="4" t="str">
-        <x:v>Ceremony</x:v>
+        <x:v>Cargo organization</x:v>
       </x:c>
       <x:c r="C55" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16886,7 +19098,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B56" s="4" t="str">
-        <x:v>Chemical processing</x:v>
+        <x:v>Ceremony</x:v>
       </x:c>
       <x:c r="C56" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16897,7 +19109,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B57" s="4" t="str">
-        <x:v>Civic identification</x:v>
+        <x:v>Chemical processing</x:v>
       </x:c>
       <x:c r="C57" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16908,7 +19120,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B58" s="4" t="str">
-        <x:v>Civic recognition</x:v>
+        <x:v>Civic identification</x:v>
       </x:c>
       <x:c r="C58" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16919,7 +19131,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B59" s="4" t="str">
-        <x:v>Cleaning</x:v>
+        <x:v>Civic recognition</x:v>
       </x:c>
       <x:c r="C59" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16930,7 +19142,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B60" s="4" t="str">
-        <x:v>Clothing</x:v>
+        <x:v>Cleaning</x:v>
       </x:c>
       <x:c r="C60" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16941,7 +19153,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B61" s="4" t="str">
-        <x:v>Clothing fabrication</x:v>
+        <x:v>Clothing</x:v>
       </x:c>
       <x:c r="C61" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16952,7 +19164,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B62" s="4" t="str">
-        <x:v>Culture support</x:v>
+        <x:v>Clothing fabrication</x:v>
       </x:c>
       <x:c r="C62" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16963,7 +19175,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B63" s="4" t="str">
-        <x:v>Decoration</x:v>
+        <x:v>Culture support</x:v>
       </x:c>
       <x:c r="C63" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16974,7 +19186,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B64" s="4" t="str">
-        <x:v>Devotion</x:v>
+        <x:v>Decoration</x:v>
       </x:c>
       <x:c r="C64" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16985,7 +19197,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B65" s="4" t="str">
-        <x:v>Dust exclusion</x:v>
+        <x:v>Devotion</x:v>
       </x:c>
       <x:c r="C65" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -16996,7 +19208,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B66" s="4" t="str">
-        <x:v>Electrical conduction</x:v>
+        <x:v>Dust exclusion</x:v>
       </x:c>
       <x:c r="C66" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17007,7 +19219,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B67" s="4" t="str">
-        <x:v>Electrical insulation</x:v>
+        <x:v>Electrical conduction</x:v>
       </x:c>
       <x:c r="C67" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17018,7 +19230,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B68" s="4" t="str">
-        <x:v>Electrical work</x:v>
+        <x:v>Electrical insulation</x:v>
       </x:c>
       <x:c r="C68" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17029,7 +19241,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B69" s="4" t="str">
-        <x:v>Energy processing</x:v>
+        <x:v>Electrical work</x:v>
       </x:c>
       <x:c r="C69" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17040,7 +19252,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B70" s="4" t="str">
-        <x:v>Energy storage</x:v>
+        <x:v>Energy processing</x:v>
       </x:c>
       <x:c r="C70" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17051,7 +19263,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B71" s="4" t="str">
-        <x:v>Equipment mounting</x:v>
+        <x:v>Energy storage</x:v>
       </x:c>
       <x:c r="C71" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17062,7 +19274,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B72" s="4" t="str">
-        <x:v>Equipment repair</x:v>
+        <x:v>Equipment mounting</x:v>
       </x:c>
       <x:c r="C72" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17073,7 +19285,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B73" s="4" t="str">
-        <x:v>Excavation</x:v>
+        <x:v>Equipment repair</x:v>
       </x:c>
       <x:c r="C73" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17084,7 +19296,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B74" s="4" t="str">
-        <x:v>Fabrication</x:v>
+        <x:v>Excavation</x:v>
       </x:c>
       <x:c r="C74" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17095,7 +19307,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B75" s="4" t="str">
-        <x:v>Fashion</x:v>
+        <x:v>Fabrication</x:v>
       </x:c>
       <x:c r="C75" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17106,7 +19318,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B76" s="4" t="str">
-        <x:v>Fauna interaction</x:v>
+        <x:v>Fashion</x:v>
       </x:c>
       <x:c r="C76" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17117,7 +19329,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B77" s="4" t="str">
-        <x:v>Fiber processing</x:v>
+        <x:v>Fauna interaction</x:v>
       </x:c>
       <x:c r="C77" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17128,7 +19340,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B78" s="4" t="str">
-        <x:v>Food service</x:v>
+        <x:v>Fiber processing</x:v>
       </x:c>
       <x:c r="C78" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17139,7 +19351,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B79" s="4" t="str">
-        <x:v>Fuel</x:v>
+        <x:v>Food service</x:v>
       </x:c>
       <x:c r="C79" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17150,7 +19362,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B80" s="4" t="str">
-        <x:v>Glass and ceramics</x:v>
+        <x:v>Fuel</x:v>
       </x:c>
       <x:c r="C80" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17161,7 +19373,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B81" s="4" t="str">
-        <x:v>Grooming</x:v>
+        <x:v>Glass and ceramics</x:v>
       </x:c>
       <x:c r="C81" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17172,7 +19384,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B82" s="4" t="str">
-        <x:v>Injury treatment</x:v>
+        <x:v>Grooming</x:v>
       </x:c>
       <x:c r="C82" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17183,7 +19395,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B83" s="4" t="str">
-        <x:v>Inspection</x:v>
+        <x:v>Injury treatment</x:v>
       </x:c>
       <x:c r="C83" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17194,7 +19406,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B84" s="4" t="str">
-        <x:v>Keepsake storage</x:v>
+        <x:v>Inspection</x:v>
       </x:c>
       <x:c r="C84" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17205,7 +19417,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B85" s="4" t="str">
-        <x:v>Liquid and bulk containment</x:v>
+        <x:v>Keepsake storage</x:v>
       </x:c>
       <x:c r="C85" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17216,7 +19428,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B86" s="4" t="str">
-        <x:v>Lubrication</x:v>
+        <x:v>Liquid and bulk containment</x:v>
       </x:c>
       <x:c r="C86" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17227,7 +19439,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B87" s="4" t="str">
-        <x:v>Machinery repair</x:v>
+        <x:v>Lubrication</x:v>
       </x:c>
       <x:c r="C87" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17238,7 +19450,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B88" s="4" t="str">
-        <x:v>Magnetic tools</x:v>
+        <x:v>Machinery repair</x:v>
       </x:c>
       <x:c r="C88" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17249,7 +19461,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B89" s="4" t="str">
-        <x:v>Material exclusion</x:v>
+        <x:v>Magnetic tools</x:v>
       </x:c>
       <x:c r="C89" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17260,7 +19472,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B90" s="4" t="str">
-        <x:v>Material transfer</x:v>
+        <x:v>Material exclusion</x:v>
       </x:c>
       <x:c r="C90" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17271,7 +19483,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B91" s="4" t="str">
-        <x:v>Metal refining</x:v>
+        <x:v>Material transfer</x:v>
       </x:c>
       <x:c r="C91" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17282,7 +19494,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B92" s="4" t="str">
-        <x:v>Music</x:v>
+        <x:v>Metal refining</x:v>
       </x:c>
       <x:c r="C92" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17293,7 +19505,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B93" s="4" t="str">
-        <x:v>Nutrition</x:v>
+        <x:v>Music</x:v>
       </x:c>
       <x:c r="C93" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17304,7 +19516,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B94" s="4" t="str">
-        <x:v>Paper making</x:v>
+        <x:v>Nutrition</x:v>
       </x:c>
       <x:c r="C94" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17315,7 +19527,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B95" s="4" t="str">
-        <x:v>Protection</x:v>
+        <x:v>Paper making</x:v>
       </x:c>
       <x:c r="C95" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17326,7 +19538,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B96" s="4" t="str">
-        <x:v>Protective fabrication</x:v>
+        <x:v>Protection</x:v>
       </x:c>
       <x:c r="C96" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17337,7 +19549,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Provenance</x:v>
+        <x:v>Protective fabrication</x:v>
       </x:c>
       <x:c r="C97" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17348,7 +19560,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B98" s="4" t="str">
-        <x:v>Public communication</x:v>
+        <x:v>Provenance</x:v>
       </x:c>
       <x:c r="C98" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17359,7 +19571,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B99" s="4" t="str">
-        <x:v>Remembrance</x:v>
+        <x:v>Public communication</x:v>
       </x:c>
       <x:c r="C99" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17370,7 +19582,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B100" s="4" t="str">
-        <x:v>Resource collection</x:v>
+        <x:v>Remembrance</x:v>
       </x:c>
       <x:c r="C100" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17381,7 +19593,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B101" s="4" t="str">
-        <x:v>Sealing</x:v>
+        <x:v>Resource collection</x:v>
       </x:c>
       <x:c r="C101" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17392,7 +19604,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B102" s="4" t="str">
-        <x:v>Specialist samples</x:v>
+        <x:v>Sealing</x:v>
       </x:c>
       <x:c r="C102" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17403,7 +19615,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B103" s="4" t="str">
-        <x:v>Static management</x:v>
+        <x:v>Specialist samples</x:v>
       </x:c>
       <x:c r="C103" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17414,7 +19626,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B104" s="4" t="str">
-        <x:v>Sun shading</x:v>
+        <x:v>Static management</x:v>
       </x:c>
       <x:c r="C104" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17425,7 +19637,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B105" s="4" t="str">
-        <x:v>Surface finishing</x:v>
+        <x:v>Sun shading</x:v>
       </x:c>
       <x:c r="C105" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17436,7 +19648,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B106" s="4" t="str">
-        <x:v>Survival provision</x:v>
+        <x:v>Surface finishing</x:v>
       </x:c>
       <x:c r="C106" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17447,7 +19659,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B107" s="4" t="str">
-        <x:v>Textile processing</x:v>
+        <x:v>Survival provision</x:v>
       </x:c>
       <x:c r="C107" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17458,7 +19670,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B108" s="4" t="str">
-        <x:v>Tool fabrication</x:v>
+        <x:v>Textile processing</x:v>
       </x:c>
       <x:c r="C108" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17469,7 +19681,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B109" s="4" t="str">
-        <x:v>Traversal</x:v>
+        <x:v>Tool fabrication</x:v>
       </x:c>
       <x:c r="C109" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17480,7 +19692,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B110" s="4" t="str">
-        <x:v>Use unresolved</x:v>
+        <x:v>Traversal</x:v>
       </x:c>
       <x:c r="C110" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17491,7 +19703,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B111" s="4" t="str">
-        <x:v>Vision</x:v>
+        <x:v>Use unresolved</x:v>
       </x:c>
       <x:c r="C111" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17502,7 +19714,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B112" s="4" t="str">
-        <x:v>Work holding</x:v>
+        <x:v>Vision</x:v>
       </x:c>
       <x:c r="C112" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17513,7 +19725,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B113" s="4" t="str">
-        <x:v>Writing and records</x:v>
+        <x:v>Work holding</x:v>
       </x:c>
       <x:c r="C113" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -17521,13 +19733,13 @@
     </x:row>
     <x:row r="114" ht="45" customHeight="1">
       <x:c r="A114" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B114" s="4" t="str">
-        <x:v>Ancient composite</x:v>
+        <x:v>Writing and records</x:v>
       </x:c>
       <x:c r="C114" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="45" customHeight="1">
@@ -17535,7 +19747,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B115" s="4" t="str">
-        <x:v>Biological chemical</x:v>
+        <x:v>Ancient composite</x:v>
       </x:c>
       <x:c r="C115" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17546,7 +19758,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B116" s="4" t="str">
-        <x:v>Carbonaceous material</x:v>
+        <x:v>Biological chemical</x:v>
       </x:c>
       <x:c r="C116" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17557,7 +19769,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B117" s="4" t="str">
-        <x:v>Ceramic</x:v>
+        <x:v>Carbonaceous material</x:v>
       </x:c>
       <x:c r="C117" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17568,7 +19780,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B118" s="4" t="str">
-        <x:v>Faunal fiber</x:v>
+        <x:v>Ceramic</x:v>
       </x:c>
       <x:c r="C118" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17579,7 +19791,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B119" s="4" t="str">
-        <x:v>Faunal fiber and shell</x:v>
+        <x:v>Ceramic and metal</x:v>
       </x:c>
       <x:c r="C119" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17590,7 +19802,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B120" s="4" t="str">
-        <x:v>Faunal membrane</x:v>
+        <x:v>Ceramic feed mixture</x:v>
       </x:c>
       <x:c r="C120" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17601,7 +19813,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B121" s="4" t="str">
-        <x:v>Faunal tissue</x:v>
+        <x:v>Faunal fiber</x:v>
       </x:c>
       <x:c r="C121" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17612,7 +19824,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B122" s="4" t="str">
-        <x:v>Fur</x:v>
+        <x:v>Faunal fiber and shell</x:v>
       </x:c>
       <x:c r="C122" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17623,7 +19835,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B123" s="4" t="str">
-        <x:v>Gemstone</x:v>
+        <x:v>Faunal membrane</x:v>
       </x:c>
       <x:c r="C123" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17634,7 +19846,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B124" s="4" t="str">
-        <x:v>Glass</x:v>
+        <x:v>Faunal tissue</x:v>
       </x:c>
       <x:c r="C124" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17645,7 +19857,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B125" s="4" t="str">
-        <x:v>Glass and metal</x:v>
+        <x:v>Fur</x:v>
       </x:c>
       <x:c r="C125" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17656,7 +19868,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B126" s="4" t="str">
-        <x:v>Glass and shell</x:v>
+        <x:v>Gemstone</x:v>
       </x:c>
       <x:c r="C126" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17667,7 +19879,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B127" s="4" t="str">
-        <x:v>Glass with unresolved casing</x:v>
+        <x:v>Glass</x:v>
       </x:c>
       <x:c r="C127" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17678,7 +19890,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B128" s="4" t="str">
-        <x:v>Hide</x:v>
+        <x:v>Glass and metal</x:v>
       </x:c>
       <x:c r="C128" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17689,7 +19901,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B129" s="4" t="str">
-        <x:v>Husk fiber</x:v>
+        <x:v>Glass and shell</x:v>
       </x:c>
       <x:c r="C129" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17700,7 +19912,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B130" s="4" t="str">
-        <x:v>Husk fiber and shell</x:v>
+        <x:v>Glass with unresolved casing</x:v>
       </x:c>
       <x:c r="C130" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17711,7 +19923,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B131" s="4" t="str">
-        <x:v>Metal</x:v>
+        <x:v>Hide</x:v>
       </x:c>
       <x:c r="C131" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17722,7 +19934,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B132" s="4" t="str">
-        <x:v>Metal and shell</x:v>
+        <x:v>Husk fiber</x:v>
       </x:c>
       <x:c r="C132" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17733,7 +19945,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B133" s="4" t="str">
-        <x:v>Metal or shell</x:v>
+        <x:v>Husk fiber and shell</x:v>
       </x:c>
       <x:c r="C133" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17744,7 +19956,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B134" s="4" t="str">
-        <x:v>Mineral</x:v>
+        <x:v>Metal</x:v>
       </x:c>
       <x:c r="C134" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17755,7 +19967,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B135" s="4" t="str">
-        <x:v>Mineral or shell</x:v>
+        <x:v>Metal and shell</x:v>
       </x:c>
       <x:c r="C135" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17766,7 +19978,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B136" s="4" t="str">
-        <x:v>Mixed / unresolved</x:v>
+        <x:v>Metal or shell</x:v>
       </x:c>
       <x:c r="C136" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17777,7 +19989,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B137" s="4" t="str">
-        <x:v>Shell / chitin</x:v>
+        <x:v>Mineral</x:v>
       </x:c>
       <x:c r="C137" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17788,7 +20000,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B138" s="4" t="str">
-        <x:v>Shell and mineral</x:v>
+        <x:v>Mineral or shell</x:v>
       </x:c>
       <x:c r="C138" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17799,7 +20011,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B139" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Mixed / unresolved</x:v>
       </x:c>
       <x:c r="C139" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17810,7 +20022,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B140" s="4" t="str">
-        <x:v>Wing membrane</x:v>
+        <x:v>Shell / chitin</x:v>
       </x:c>
       <x:c r="C140" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -17818,35 +20030,35 @@
     </x:row>
     <x:row r="141" ht="45" customHeight="1">
       <x:c r="A141" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B141" s="4" t="str">
-        <x:v>Assembly</x:v>
+        <x:v>Shell and mineral</x:v>
       </x:c>
       <x:c r="C141" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="45" customHeight="1">
       <x:c r="A142" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B142" s="4" t="str">
-        <x:v>Bundle</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C142" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="143" ht="45" customHeight="1">
       <x:c r="A143" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B143" s="4" t="str">
-        <x:v>Cord</x:v>
+        <x:v>Wing membrane</x:v>
       </x:c>
       <x:c r="C143" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="45" customHeight="1">
@@ -17854,7 +20066,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B144" s="4" t="str">
-        <x:v>Fiber</x:v>
+        <x:v>Assembly</x:v>
       </x:c>
       <x:c r="C144" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17865,7 +20077,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B145" s="4" t="str">
-        <x:v>Folio</x:v>
+        <x:v>Bundle</x:v>
       </x:c>
       <x:c r="C145" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17876,7 +20088,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B146" s="4" t="str">
-        <x:v>Garment</x:v>
+        <x:v>Cord</x:v>
       </x:c>
       <x:c r="C146" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17887,7 +20099,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B147" s="4" t="str">
-        <x:v>Gel</x:v>
+        <x:v>Fiber</x:v>
       </x:c>
       <x:c r="C147" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17898,7 +20110,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B148" s="4" t="str">
-        <x:v>Liquid</x:v>
+        <x:v>Folio</x:v>
       </x:c>
       <x:c r="C148" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17909,7 +20121,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B149" s="4" t="str">
-        <x:v>Membrane</x:v>
+        <x:v>Garment</x:v>
       </x:c>
       <x:c r="C149" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17920,7 +20132,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B150" s="4" t="str">
-        <x:v>Panel</x:v>
+        <x:v>Gel</x:v>
       </x:c>
       <x:c r="C150" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17931,7 +20143,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B151" s="4" t="str">
-        <x:v>Particles</x:v>
+        <x:v>Liquid</x:v>
       </x:c>
       <x:c r="C151" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17942,7 +20154,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B152" s="4" t="str">
-        <x:v>Patch</x:v>
+        <x:v>Membrane</x:v>
       </x:c>
       <x:c r="C152" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17953,7 +20165,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B153" s="4" t="str">
-        <x:v>Rock</x:v>
+        <x:v>Panel</x:v>
       </x:c>
       <x:c r="C153" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17964,7 +20176,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B154" s="4" t="str">
-        <x:v>Sheet</x:v>
+        <x:v>Particles</x:v>
       </x:c>
       <x:c r="C154" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17975,7 +20187,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B155" s="4" t="str">
-        <x:v>Shell plate</x:v>
+        <x:v>Patch</x:v>
       </x:c>
       <x:c r="C155" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17986,7 +20198,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B156" s="4" t="str">
-        <x:v>Solid part</x:v>
+        <x:v>Rock</x:v>
       </x:c>
       <x:c r="C156" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -17997,7 +20209,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B157" s="4" t="str">
-        <x:v>Solid piece</x:v>
+        <x:v>Sheet</x:v>
       </x:c>
       <x:c r="C157" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -18008,7 +20220,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B158" s="4" t="str">
-        <x:v>Strip</x:v>
+        <x:v>Shell plate</x:v>
       </x:c>
       <x:c r="C158" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -18019,7 +20231,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B159" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Solid part</x:v>
       </x:c>
       <x:c r="C159" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -18027,35 +20239,35 @@
     </x:row>
     <x:row r="160" ht="45" customHeight="1">
       <x:c r="A160" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B160" s="4" t="str">
-        <x:v>Author direction</x:v>
+        <x:v>Solid piece</x:v>
       </x:c>
       <x:c r="C160" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="45" customHeight="1">
       <x:c r="A161" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B161" s="4" t="str">
-        <x:v>Existing definition</x:v>
+        <x:v>Strip</x:v>
       </x:c>
       <x:c r="C161" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="45" customHeight="1">
       <x:c r="A162" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B162" s="4" t="str">
-        <x:v>Proposal</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C162" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="163" ht="45" customHeight="1">
@@ -18063,16 +20275,49 @@
         <x:v>Design status</x:v>
       </x:c>
       <x:c r="B163" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="C163" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="45" customHeight="1">
+      <x:c r="A164" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B164" s="4" t="str">
+        <x:v>Existing definition</x:v>
+      </x:c>
+      <x:c r="C164" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="45" customHeight="1">
+      <x:c r="A165" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B165" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="C165" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="45" customHeight="1">
+      <x:c r="A166" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B166" s="4" t="str">
         <x:v>Withheld assumption</x:v>
       </x:c>
-      <x:c r="C163" s="4" t="str">
+      <x:c r="C166" s="4" t="str">
         <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d78aae0c5b44e0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6cca720bb1c4704"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23377,21 +25622,1083 @@
         <x:v>Current item description. Catalog intent, not implemented actions.</x:v>
       </x:c>
     </x:row>
+    <x:row r="237" ht="50" customHeight="1">
+      <x:c r="A237" s="4" t="str">
+        <x:v>proposal.ceramic.grog</x:v>
+      </x:c>
+      <x:c r="B237" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A237,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crushed fired ceramic grit</x:v>
+      </x:c>
+      <x:c r="C237" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A237,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D237" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E237" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A237,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F237" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="50" customHeight="1">
+      <x:c r="A238" s="4" t="str">
+        <x:v>proposal.ceramic.grog</x:v>
+      </x:c>
+      <x:c r="B238" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A238,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crushed fired ceramic grit</x:v>
+      </x:c>
+      <x:c r="C238" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A238,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D238" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E238" s="4" t="str">
+        <x:v>Fabrication</x:v>
+      </x:c>
+      <x:c r="F238" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="50" customHeight="1">
+      <x:c r="A239" s="4" t="str">
+        <x:v>proposal.ceramic.body_feed</x:v>
+      </x:c>
+      <x:c r="B239" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A239,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared ceramic body feed</x:v>
+      </x:c>
+      <x:c r="C239" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A239,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D239" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E239" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A239,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F239" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="50" customHeight="1">
+      <x:c r="A240" s="4" t="str">
+        <x:v>proposal.ceramic.body_feed</x:v>
+      </x:c>
+      <x:c r="B240" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A240,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared ceramic body feed</x:v>
+      </x:c>
+      <x:c r="C240" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A240,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D240" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E240" s="4" t="str">
+        <x:v>Fabrication</x:v>
+      </x:c>
+      <x:c r="F240" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="50" customHeight="1">
+      <x:c r="A241" s="4" t="str">
+        <x:v>proposal.ceramic.glaze_feed</x:v>
+      </x:c>
+      <x:c r="B241" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A241,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared glaze feed</x:v>
+      </x:c>
+      <x:c r="C241" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A241,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D241" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E241" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A241,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F241" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="50" customHeight="1">
+      <x:c r="A242" s="4" t="str">
+        <x:v>proposal.ceramic.glaze_feed</x:v>
+      </x:c>
+      <x:c r="B242" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A242,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared glaze feed</x:v>
+      </x:c>
+      <x:c r="C242" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A242,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D242" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E242" s="4" t="str">
+        <x:v>Surface finishing</x:v>
+      </x:c>
+      <x:c r="F242" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="50" customHeight="1">
+      <x:c r="A243" s="4" t="str">
+        <x:v>proposal.ceramic.unfired_blank</x:v>
+      </x:c>
+      <x:c r="B243" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A243,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Unfired shaped ceramic blank</x:v>
+      </x:c>
+      <x:c r="C243" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A243,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D243" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E243" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A243,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F243" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="50" customHeight="1">
+      <x:c r="A244" s="4" t="str">
+        <x:v>proposal.ceramic.bowl</x:v>
+      </x:c>
+      <x:c r="B244" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A244,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Plain ceramic eating bowl</x:v>
+      </x:c>
+      <x:c r="C244" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A244,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D244" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E244" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A244,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="F244" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="50" customHeight="1">
+      <x:c r="A245" s="4" t="str">
+        <x:v>proposal.ceramic.cup</x:v>
+      </x:c>
+      <x:c r="B245" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A245,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Small ceramic cup</x:v>
+      </x:c>
+      <x:c r="C245" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A245,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D245" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E245" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A245,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="F245" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="50" customHeight="1">
+      <x:c r="A246" s="4" t="str">
+        <x:v>proposal.ceramic.plate</x:v>
+      </x:c>
+      <x:c r="B246" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A246,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic serving plate</x:v>
+      </x:c>
+      <x:c r="C246" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A246,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Everyday objects</x:v>
+      </x:c>
+      <x:c r="D246" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E246" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A246,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="F246" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="50" customHeight="1">
+      <x:c r="A247" s="4" t="str">
+        <x:v>proposal.ceramic.storage_crock</x:v>
+      </x:c>
+      <x:c r="B247" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A247,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic dry-storage crock</x:v>
+      </x:c>
+      <x:c r="C247" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A247,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D247" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E247" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A247,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F247" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="50" customHeight="1">
+      <x:c r="A248" s="4" t="str">
+        <x:v>proposal.ceramic.storage_crock</x:v>
+      </x:c>
+      <x:c r="B248" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A248,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic dry-storage crock</x:v>
+      </x:c>
+      <x:c r="C248" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A248,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D248" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E248" s="4" t="str">
+        <x:v>Liquid and bulk containment</x:v>
+      </x:c>
+      <x:c r="F248" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="50" customHeight="1">
+      <x:c r="A249" s="4" t="str">
+        <x:v>proposal.ceramic.crucible</x:v>
+      </x:c>
+      <x:c r="B249" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A249,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic crucible</x:v>
+      </x:c>
+      <x:c r="C249" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A249,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D249" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E249" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A249,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Metal refining</x:v>
+      </x:c>
+      <x:c r="F249" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="50" customHeight="1">
+      <x:c r="A250" s="4" t="str">
+        <x:v>proposal.ceramic.crucible</x:v>
+      </x:c>
+      <x:c r="B250" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A250,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic crucible</x:v>
+      </x:c>
+      <x:c r="C250" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A250,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D250" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E250" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F250" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="50" customHeight="1">
+      <x:c r="A251" s="4" t="str">
+        <x:v>proposal.ceramic.casting_mold</x:v>
+      </x:c>
+      <x:c r="B251" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A251,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic casting mold</x:v>
+      </x:c>
+      <x:c r="C251" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A251,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D251" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E251" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A251,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Fabrication</x:v>
+      </x:c>
+      <x:c r="F251" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="50" customHeight="1">
+      <x:c r="A252" s="4" t="str">
+        <x:v>proposal.ceramic.casting_mold</x:v>
+      </x:c>
+      <x:c r="B252" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A252,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic casting mold</x:v>
+      </x:c>
+      <x:c r="C252" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A252,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D252" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E252" s="4" t="str">
+        <x:v>Metal refining</x:v>
+      </x:c>
+      <x:c r="F252" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="50" customHeight="1">
+      <x:c r="A253" s="4" t="str">
+        <x:v>proposal.ceramic.mortar</x:v>
+      </x:c>
+      <x:c r="B253" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A253,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic grinding mortar</x:v>
+      </x:c>
+      <x:c r="C253" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A253,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D253" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E253" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A253,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chemical processing</x:v>
+      </x:c>
+      <x:c r="F253" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="50" customHeight="1">
+      <x:c r="A254" s="4" t="str">
+        <x:v>proposal.ceramic.mortar</x:v>
+      </x:c>
+      <x:c r="B254" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A254,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic grinding mortar</x:v>
+      </x:c>
+      <x:c r="C254" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A254,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D254" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E254" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F254" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255" ht="50" customHeight="1">
+      <x:c r="A255" s="4" t="str">
+        <x:v>proposal.ceramic.pestle</x:v>
+      </x:c>
+      <x:c r="B255" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A255,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic pestle</x:v>
+      </x:c>
+      <x:c r="C255" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A255,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D255" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E255" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A255,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chemical processing</x:v>
+      </x:c>
+      <x:c r="F255" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256" ht="50" customHeight="1">
+      <x:c r="A256" s="4" t="str">
+        <x:v>proposal.ceramic.pestle</x:v>
+      </x:c>
+      <x:c r="B256" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A256,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic pestle</x:v>
+      </x:c>
+      <x:c r="C256" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A256,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D256" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E256" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F256" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257" ht="50" customHeight="1">
+      <x:c r="A257" s="4" t="str">
+        <x:v>proposal.ceramic.firing_tray</x:v>
+      </x:c>
+      <x:c r="B257" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A257,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic firing tray</x:v>
+      </x:c>
+      <x:c r="C257" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A257,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D257" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E257" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A257,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F257" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258" ht="50" customHeight="1">
+      <x:c r="A258" s="4" t="str">
+        <x:v>proposal.ceramic.refractory_brick</x:v>
+      </x:c>
+      <x:c r="B258" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A258,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Refractory ceramic brick</x:v>
+      </x:c>
+      <x:c r="C258" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A258,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D258" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E258" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A258,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protective fabrication</x:v>
+      </x:c>
+      <x:c r="F258" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259" ht="50" customHeight="1">
+      <x:c r="A259" s="4" t="str">
+        <x:v>proposal.ceramic.refractory_brick</x:v>
+      </x:c>
+      <x:c r="B259" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A259,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Refractory ceramic brick</x:v>
+      </x:c>
+      <x:c r="C259" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A259,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D259" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E259" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F259" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260" ht="50" customHeight="1">
+      <x:c r="A260" s="4" t="str">
+        <x:v>proposal.ceramic.refractory_brick</x:v>
+      </x:c>
+      <x:c r="B260" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A260,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Refractory ceramic brick</x:v>
+      </x:c>
+      <x:c r="C260" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A260,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D260" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E260" s="4" t="str">
+        <x:v>Metal refining</x:v>
+      </x:c>
+      <x:c r="F260" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="261" ht="50" customHeight="1">
+      <x:c r="A261" s="4" t="str">
+        <x:v>proposal.ceramic.kiln_liner</x:v>
+      </x:c>
+      <x:c r="B261" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A261,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic kiln lining panel</x:v>
+      </x:c>
+      <x:c r="C261" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A261,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D261" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E261" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A261,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protective fabrication</x:v>
+      </x:c>
+      <x:c r="F261" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262" ht="50" customHeight="1">
+      <x:c r="A262" s="4" t="str">
+        <x:v>proposal.ceramic.kiln_liner</x:v>
+      </x:c>
+      <x:c r="B262" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A262,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic kiln lining panel</x:v>
+      </x:c>
+      <x:c r="C262" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A262,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D262" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E262" s="4" t="str">
+        <x:v>Glass and ceramics</x:v>
+      </x:c>
+      <x:c r="F262" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263" ht="50" customHeight="1">
+      <x:c r="A263" s="4" t="str">
+        <x:v>proposal.ceramic.bead</x:v>
+      </x:c>
+      <x:c r="B263" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A263,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic insulating bead</x:v>
+      </x:c>
+      <x:c r="C263" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A263,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D263" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E263" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A263,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Electrical insulation</x:v>
+      </x:c>
+      <x:c r="F263" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264" ht="50" customHeight="1">
+      <x:c r="A264" s="4" t="str">
+        <x:v>proposal.ceramic.bead</x:v>
+      </x:c>
+      <x:c r="B264" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A264,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic insulating bead</x:v>
+      </x:c>
+      <x:c r="C264" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A264,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D264" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E264" s="4" t="str">
+        <x:v>Electrical work</x:v>
+      </x:c>
+      <x:c r="F264" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265" ht="50" customHeight="1">
+      <x:c r="A265" s="4" t="str">
+        <x:v>proposal.ceramic.spacer</x:v>
+      </x:c>
+      <x:c r="B265" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A265,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic insulating spacer</x:v>
+      </x:c>
+      <x:c r="C265" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A265,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D265" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E265" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A265,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Electrical insulation</x:v>
+      </x:c>
+      <x:c r="F265" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266" ht="50" customHeight="1">
+      <x:c r="A266" s="4" t="str">
+        <x:v>proposal.ceramic.spacer</x:v>
+      </x:c>
+      <x:c r="B266" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A266,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic insulating spacer</x:v>
+      </x:c>
+      <x:c r="C266" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A266,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D266" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E266" s="4" t="str">
+        <x:v>Electrical work</x:v>
+      </x:c>
+      <x:c r="F266" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267" ht="50" customHeight="1">
+      <x:c r="A267" s="4" t="str">
+        <x:v>proposal.ceramic.feedthrough</x:v>
+      </x:c>
+      <x:c r="B267" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A267,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic electrical feedthrough</x:v>
+      </x:c>
+      <x:c r="C267" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A267,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D267" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E267" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A267,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Electrical insulation</x:v>
+      </x:c>
+      <x:c r="F267" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268" ht="50" customHeight="1">
+      <x:c r="A268" s="4" t="str">
+        <x:v>proposal.ceramic.feedthrough</x:v>
+      </x:c>
+      <x:c r="B268" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A268,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic electrical feedthrough</x:v>
+      </x:c>
+      <x:c r="C268" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A268,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D268" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E268" s="4" t="str">
+        <x:v>Electrical conduction</x:v>
+      </x:c>
+      <x:c r="F268" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269" ht="50" customHeight="1">
+      <x:c r="A269" s="4" t="str">
+        <x:v>proposal.ceramic.stopper</x:v>
+      </x:c>
+      <x:c r="B269" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A269,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Fitted ceramic stopper</x:v>
+      </x:c>
+      <x:c r="C269" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A269,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D269" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E269" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A269,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Sealing</x:v>
+      </x:c>
+      <x:c r="F269" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="50" customHeight="1">
+      <x:c r="A270" s="4" t="str">
+        <x:v>proposal.ceramic.lid</x:v>
+      </x:c>
+      <x:c r="B270" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A270,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic vessel lid</x:v>
+      </x:c>
+      <x:c r="C270" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A270,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D270" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E270" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A270,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Liquid and bulk containment</x:v>
+      </x:c>
+      <x:c r="F270" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="271" ht="50" customHeight="1">
+      <x:c r="A271" s="4" t="str">
+        <x:v>proposal.ceramic.lid</x:v>
+      </x:c>
+      <x:c r="B271" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A271,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic vessel lid</x:v>
+      </x:c>
+      <x:c r="C271" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A271,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D271" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E271" s="4" t="str">
+        <x:v>Dust exclusion</x:v>
+      </x:c>
+      <x:c r="F271" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272" ht="50" customHeight="1">
+      <x:c r="A272" s="4" t="str">
+        <x:v>proposal.ceramic.pour_spout</x:v>
+      </x:c>
+      <x:c r="B272" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A272,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic pouring spout</x:v>
+      </x:c>
+      <x:c r="C272" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A272,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D272" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E272" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A272,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Material transfer</x:v>
+      </x:c>
+      <x:c r="F272" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="273" ht="50" customHeight="1">
+      <x:c r="A273" s="4" t="str">
+        <x:v>proposal.ceramic.conduit</x:v>
+      </x:c>
+      <x:c r="B273" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A273,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic conduit section</x:v>
+      </x:c>
+      <x:c r="C273" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A273,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D273" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E273" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A273,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Material transfer</x:v>
+      </x:c>
+      <x:c r="F273" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="274" ht="50" customHeight="1">
+      <x:c r="A274" s="4" t="str">
+        <x:v>proposal.ceramic.votive_plaque</x:v>
+      </x:c>
+      <x:c r="B274" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A274,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic votive plaque</x:v>
+      </x:c>
+      <x:c r="C274" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A274,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D274" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E274" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A274,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Devotion</x:v>
+      </x:c>
+      <x:c r="F274" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="275" ht="50" customHeight="1">
+      <x:c r="A275" s="4" t="str">
+        <x:v>proposal.ceramic.votive_plaque</x:v>
+      </x:c>
+      <x:c r="B275" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A275,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic votive plaque</x:v>
+      </x:c>
+      <x:c r="C275" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A275,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D275" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E275" s="4" t="str">
+        <x:v>Decoration</x:v>
+      </x:c>
+      <x:c r="F275" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="276" ht="50" customHeight="1">
+      <x:c r="A276" s="4" t="str">
+        <x:v>proposal.ceramic.figurine</x:v>
+      </x:c>
+      <x:c r="B276" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A276,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic commemorative figurine</x:v>
+      </x:c>
+      <x:c r="C276" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A276,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D276" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E276" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A276,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Remembrance</x:v>
+      </x:c>
+      <x:c r="F276" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="277" ht="50" customHeight="1">
+      <x:c r="A277" s="4" t="str">
+        <x:v>proposal.ceramic.figurine</x:v>
+      </x:c>
+      <x:c r="B277" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A277,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic commemorative figurine</x:v>
+      </x:c>
+      <x:c r="C277" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A277,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D277" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E277" s="4" t="str">
+        <x:v>Decoration</x:v>
+      </x:c>
+      <x:c r="F277" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="278" ht="50" customHeight="1">
+      <x:c r="A278" s="4" t="str">
+        <x:v>proposal.ceramic.ceremony_bowl</x:v>
+      </x:c>
+      <x:c r="B278" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A278,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceremonial ceramic bowl</x:v>
+      </x:c>
+      <x:c r="C278" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A278,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D278" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E278" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A278,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceremony</x:v>
+      </x:c>
+      <x:c r="F278" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="279" ht="50" customHeight="1">
+      <x:c r="A279" s="4" t="str">
+        <x:v>proposal.ceramic.ceremony_bowl</x:v>
+      </x:c>
+      <x:c r="B279" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A279,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceremonial ceramic bowl</x:v>
+      </x:c>
+      <x:c r="C279" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A279,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cultural objects</x:v>
+      </x:c>
+      <x:c r="D279" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E279" s="4" t="str">
+        <x:v>Decoration</x:v>
+      </x:c>
+      <x:c r="F279" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="280" ht="50" customHeight="1">
+      <x:c r="A280" s="4" t="str">
+        <x:v>proposal.ceramic.armor_insert</x:v>
+      </x:c>
+      <x:c r="B280" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A280,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Specialist ceramic armor insert</x:v>
+      </x:c>
+      <x:c r="C280" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A280,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D280" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E280" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A280,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F280" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="281" ht="50" customHeight="1">
+      <x:c r="A281" s="4" t="str">
+        <x:v>proposal.ceramic.fastener</x:v>
+      </x:c>
+      <x:c r="B281" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A281,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic toggle fastener</x:v>
+      </x:c>
+      <x:c r="C281" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A281,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D281" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E281" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A281,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Clothing fabrication</x:v>
+      </x:c>
+      <x:c r="F281" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282" ht="50" customHeight="1">
+      <x:c r="A282" s="4" t="str">
+        <x:v>proposal.ceramic.fastener</x:v>
+      </x:c>
+      <x:c r="B282" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A282,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic toggle fastener</x:v>
+      </x:c>
+      <x:c r="C282" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A282,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D282" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E282" s="4" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F282" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="283" ht="50" customHeight="1">
+      <x:c r="A283" s="4" t="str">
+        <x:v>proposal.ceramic.grinding_disc</x:v>
+      </x:c>
+      <x:c r="B283" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A283,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic abrasive disc</x:v>
+      </x:c>
+      <x:c r="C283" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A283,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D283" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E283" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A283,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Surface finishing</x:v>
+      </x:c>
+      <x:c r="F283" s="4" t="str">
+        <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A6:A1005">
-      <x:formula1>'Items'!$A$6:$A$181</x:formula1>
+      <x:formula1>'Items'!$A$6:$A$209</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D6:D1005">
       <x:formula1>"Primary,Secondary"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E6:E1005">
-      <x:formula1>'Taxonomy'!$B$51:$B$113</x:formula1>
+      <x:formula1>'Taxonomy'!$B$52:$B$114</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8eee2912255424f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04bde21282a04393"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24299,7 +27606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ffb57d55c5b49f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R347efa8692354fae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24665,7 +27972,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c6c44d5f58a481a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R892de91be3d54486"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24726,7 +28033,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>27</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>Existing gear plus armor, carriers, rare eyewear/headwear and very rare fashion families</x:v>
@@ -24756,7 +28063,7 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>77</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Minerals, biological resources, generic chemistry placeholders and twelve new chemical concepts</x:v>
@@ -24771,7 +28078,7 @@
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A9)</x:f>
-        <x:v>27</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>Existing salvage and proposed materials, including husk-fiber paper and difficult pressed textiles</x:v>
@@ -24870,7 +28177,7 @@
       </x:c>
       <x:c r="B16" s="41" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A16)</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C16" s="41" t="str">
         <x:v>Primary vessels, protective carriers, transfer glassware and closures</x:v>
@@ -25089,10 +28396,25 @@
         <x:v>Simple shell/metal forms; no wood or ordinary cloth assumed.</x:v>
       </x:c>
     </x:row>
+    <x:row r="31" ht="110" customHeight="1">
+      <x:c r="A31" s="3" t="str">
+        <x:v>Ceramics</x:v>
+      </x:c>
+      <x:c r="B31" s="3" t="n">
+        <x:f>COUNTIF(Items!$AA$6:$AA$1005,"Ceramic")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic feed mixture")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic and metal")</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C31" s="3" t="str">
+        <x:v>28 new ceramic-specific feeds, intermediate blanks, tableware, storage, workshop tools, thermal/electrical parts, vessel fittings, ceremonial work and protection candidates</x:v>
+      </x:c>
+      <x:c r="D31" s="3" t="str">
+        <x:v>Existing claystone, alumina, borate, insulating blanks and ceramic reagent jar remain their original entries.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc619958b5f65455d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5644ebef854b44dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25155,7 +28477,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>176 design entries: 18 existing item IDs and 158 design concepts. Includes 24 religious, civic, ritual and everyday object proposals.</x:v>
+        <x:v>204 design entries: 18 existing item IDs and 186 design concepts. Includes 28 ceramic item proposals; classifications and item-use relationships populated.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -25867,7 +29189,7 @@
         <x:v>Filtering the master</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Items is one native filterable table, A5:AE181. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
+        <x:v>Items is one native filterable table, A5:AE209. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="85" customHeight="1">
@@ -25926,10 +29248,42 @@
         <x:v>Sort whole native tables with header arrows so IDs, sources and notes move together. Item uses resolves links by ID after master sorting. Do not sort an isolated column. Classification does not change serialized variants, recipes, carrier policy or Unity gameplay.</x:v>
       </x:c>
     </x:row>
+    <x:row r="105" ht="85" customHeight="1">
+      <x:c r="A105" s="4" t="str">
+        <x:v>Ceramic family</x:v>
+      </x:c>
+      <x:c r="B105" s="4" t="str">
+        <x:v>Author requests many ceramics and ceramic items. Specific feeds, forms, parts, vessels, tools and cultural pieces are new proposals. Reuse existing claystone, alumina, borate, insulating ceramic blanks and glazed reagent-jar entries rather than duplicating them.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="85" customHeight="1">
+      <x:c r="A106" s="4" t="str">
+        <x:v>Ceramic grades</x:v>
+      </x:c>
+      <x:c r="B106" s="4" t="str">
+        <x:v>Ordinary tableware, specialist chemical-service ware, thermal parts, electrical parts and armor candidates have distinct service requirements. The Ceramic material label does not grant universal insulation, heat resistance, food safety, liquid tightness or protection.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="85" customHeight="1">
+      <x:c r="A107" s="4" t="str">
+        <x:v>Ceramic processing</x:v>
+      </x:c>
+      <x:c r="B107" s="4" t="str">
+        <x:v>No free-water pottery/slip/glaze recipe is assumed. Feed selection, forming, binder, finishing and firing remain design work. Chemical compatibility and residue checks remain relevant. Crushed ceramic feed is a proposed recycling product, not a universal salvage yield.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="85" customHeight="1">
+      <x:c r="A108" s="4" t="str">
+        <x:v>Ceramic filters</x:v>
+      </x:c>
+      <x:c r="B108" s="4" t="str">
+        <x:v>Filter Items &gt; Material family for Ceramic, Ceramic feed mixture or Ceramic and metal. Use Subtype for feedstock, household, storage, workshop, thermal, electrical, vessel-fitting, ceremonial, protection and household-fitting branches. Item uses includes primary and secondary ceramic uses.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd392db2f205452d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra233638769404052"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26773,7 +30127,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra99fcbc1ef344f98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32f75a2da65c416b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27016,7 +30370,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e4c29491b2e400b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R393307912f304807"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27420,7 +30774,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R055768a65c56464e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ca8ad4fb9064235"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28096,7 +31450,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b719cebe1f34775"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71110eebd28c4e2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: register lore currency and unresolved denominations
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R370a4633e2694528"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rd9e12b4fe7a445da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R68d0fe190343488e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rdf171a3efea24e3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R6f131b9db7f04e73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rc18f9de7d0544b61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R511b5b6f4d3f4730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R89c95e3337734d0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R4339eb6410e94dea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R2b4f480e1f6448df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R543f669186554f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R77e4abe573524374"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="R8e51d6ef392a460f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R1f3bda4708bb4624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Re123dea67a0d4ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rcf89d166a7244452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rcb5d82861f614ecd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Ra6d192d5b5dd42da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rb8bd761487da4207"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R8d08824eb7da4859"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Ra123ca8fec514178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R022893996caa4fce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="Rc1c776f477604034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R0f47a3a993434baf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="Rfc74994854e3490b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="Rebf0ed6d38354e13"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,8 +476,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE209" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AE209"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE210" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AE210"/>
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -550,7 +550,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C166" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C170" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Field"/>
     <x:tableColumn id="2" name="Allowed value"/>
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F283" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F283"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F284" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F284"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -614,7 +614,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -626,7 +626,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B108" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B111" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -986,7 +986,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>204 items. Filter W:AC for type, stage, origin, use, material, form and status. Search AD; use Item uses for multiple purposes.</x:v>
+        <x:v>205 entries. Filter W:AC for type, stage, origin, use, material, form and status. Currency denominations remain unresolved.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -17333,6 +17333,85 @@
         <x:v>Specific item proposed from author ceramics direction; functional and material limits remain unresolved.</x:v>
       </x:c>
     </x:row>
+    <x:row r="210" ht="115" customHeight="1">
+      <x:c r="A210" s="9" t="str">
+        <x:v>source.currency.imperial_commons</x:v>
+      </x:c>
+      <x:c r="B210" s="9" t="str">
+        <x:v>Imperial Commons</x:v>
+      </x:c>
+      <x:c r="C210" s="9" t="str">
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="D210" s="9" t="str">
+        <x:v>Currency family; denominations unspecified</x:v>
+      </x:c>
+      <x:c r="E210" s="9" t="str">
+        <x:v>Source proposal; not implemented</x:v>
+      </x:c>
+      <x:c r="F210" s="9" t="str">
+        <x:v>Imperial currency for exchange. Source everyday name: Commons; commercial shorthand: marks.</x:v>
+      </x:c>
+      <x:c r="G210" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H210" s="9" t="str">
+        <x:v>Physical form and carrier policy unresolved</x:v>
+      </x:c>
+      <x:c r="I210" s="13"/>
+      <x:c r="J210" s="15"/>
+      <x:c r="K210" s="9" t="str">
+        <x:v>Source issuer: Empire. Issuance and acquisition are not game systems.</x:v>
+      </x:c>
+      <x:c r="L210" s="9" t="str">
+        <x:v>No minting or crafting recipe authored</x:v>
+      </x:c>
+      <x:c r="M210" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N210" s="9" t="str">
+        <x:v>Source WLD-0032 is draft/proposal. No denomination names, face values, ratios, coin/note materials, dimensions or physical form are specified.</x:v>
+      </x:c>
+      <x:c r="O210" s="17"/>
+      <x:c r="P210" s="17"/>
+      <x:c r="Q210" s="17"/>
+      <x:c r="R210" s="17"/>
+      <x:c r="S210" s="17"/>
+      <x:c r="T210" s="9" t="str">
+        <x:v>Currency-family placeholder, not a claimed one-Common coin or note. Commons and marks are aliases, not separate denominations. Leave face values, item prices, stack/mass and wallet behavior undefined.</x:v>
+      </x:c>
+      <x:c r="U210" s="11"/>
+      <x:c r="V210" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/economy/currency.md; WLD-0032 status=draft, canon_status=proposal; remote master revision verified October 14, 2026.</x:v>
+      </x:c>
+      <x:c r="W210" s="4" t="str">
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="X210" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="Y210" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z210" s="4" t="str">
+        <x:v>Trade</x:v>
+      </x:c>
+      <x:c r="AA210" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AB210" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AC210" s="4" t="str">
+        <x:v>Source proposal</x:v>
+      </x:c>
+      <x:c r="AD210" s="4" t="str">
+        <x:v>imperial commons; commons; marks; currency; money; trade; exchange; denomination unspecified</x:v>
+      </x:c>
+      <x:c r="AE210" s="4" t="str">
+        <x:v>Source record explicitly names the currency and aliases; no physical denomination item inferred.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
@@ -17348,33 +17427,33 @@
   </x:conditionalFormatting>
   <x:dataValidations count="8">
     <x:dataValidation type="list" sqref="C6:C1005">
-      <x:formula1>'Taxonomy'!$B$6:$B$13</x:formula1>
+      <x:formula1>'Taxonomy'!$B$6:$B$14</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="W6:W1005">
-      <x:formula1>'Taxonomy'!$B$14:$B$34</x:formula1>
+      <x:formula1>'Taxonomy'!$B$15:$B$36</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="X6:X1005">
-      <x:formula1>'Taxonomy'!$B$35:$B$43</x:formula1>
+      <x:formula1>'Taxonomy'!$B$37:$B$45</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Y6:Y1005">
-      <x:formula1>'Taxonomy'!$B$44:$B$51</x:formula1>
+      <x:formula1>'Taxonomy'!$B$46:$B$53</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Z6:Z1005">
-      <x:formula1>'Taxonomy'!$B$52:$B$114</x:formula1>
+      <x:formula1>'Taxonomy'!$B$54:$B$117</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AA6:AA1005">
-      <x:formula1>'Taxonomy'!$B$115:$B$143</x:formula1>
+      <x:formula1>'Taxonomy'!$B$118:$B$146</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AB6:AB1005">
-      <x:formula1>'Taxonomy'!$B$144:$B$162</x:formula1>
+      <x:formula1>'Taxonomy'!$B$147:$B$165</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AC6:AC1005">
-      <x:formula1>'Taxonomy'!$B$163:$B$166</x:formula1>
+      <x:formula1>'Taxonomy'!$B$166:$B$170</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5501e6d9e0d43c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8e23eba34944339"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18026,7 +18105,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46709f5344f24c0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf81072c62a5e4aeb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18508,7 +18587,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35bcf7942e314fd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f9ad8a0a1a34d3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18581,7 +18660,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B9" s="4" t="str">
-        <x:v>Equipment</x:v>
+        <x:v>Currency</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -18592,7 +18671,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B10" s="4" t="str">
-        <x:v>Everyday objects</x:v>
+        <x:v>Equipment</x:v>
       </x:c>
       <x:c r="C10" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -18603,7 +18682,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B11" s="4" t="str">
-        <x:v>Field supplies</x:v>
+        <x:v>Everyday objects</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -18614,7 +18693,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B12" s="4" t="str">
-        <x:v>Resources</x:v>
+        <x:v>Field supplies</x:v>
       </x:c>
       <x:c r="C12" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -18625,7 +18704,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B13" s="4" t="str">
-        <x:v>Weapons</x:v>
+        <x:v>Resources</x:v>
       </x:c>
       <x:c r="C13" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -18633,13 +18712,13 @@
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
       <x:c r="A14" s="4" t="str">
-        <x:v>Item type</x:v>
+        <x:v>Category</x:v>
       </x:c>
       <x:c r="B14" s="4" t="str">
-        <x:v>Armor</x:v>
+        <x:v>Weapons</x:v>
       </x:c>
       <x:c r="C14" s="4" t="str">
-        <x:v>What the object is, independent of material, culture and use.</x:v>
+        <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="45" customHeight="1">
@@ -18647,7 +18726,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B15" s="4" t="str">
-        <x:v>Carrier</x:v>
+        <x:v>Armor</x:v>
       </x:c>
       <x:c r="C15" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18658,7 +18737,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B16" s="4" t="str">
-        <x:v>Chemical material</x:v>
+        <x:v>Carrier</x:v>
       </x:c>
       <x:c r="C16" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18669,7 +18748,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B17" s="4" t="str">
-        <x:v>Container</x:v>
+        <x:v>Chemical material</x:v>
       </x:c>
       <x:c r="C17" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18680,7 +18759,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B18" s="4" t="str">
-        <x:v>Container part</x:v>
+        <x:v>Container</x:v>
       </x:c>
       <x:c r="C18" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18691,7 +18770,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B19" s="4" t="str">
-        <x:v>Crafting component</x:v>
+        <x:v>Container part</x:v>
       </x:c>
       <x:c r="C19" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18702,7 +18781,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B20" s="4" t="str">
-        <x:v>Cultural object</x:v>
+        <x:v>Crafting component</x:v>
       </x:c>
       <x:c r="C20" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18713,7 +18792,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B21" s="4" t="str">
-        <x:v>Document</x:v>
+        <x:v>Cultural object</x:v>
       </x:c>
       <x:c r="C21" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18724,7 +18803,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B22" s="4" t="str">
-        <x:v>Energy storage</x:v>
+        <x:v>Currency</x:v>
       </x:c>
       <x:c r="C22" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18735,7 +18814,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B23" s="4" t="str">
-        <x:v>Food material</x:v>
+        <x:v>Document</x:v>
       </x:c>
       <x:c r="C23" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18746,7 +18825,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B24" s="4" t="str">
-        <x:v>Gem material</x:v>
+        <x:v>Energy storage</x:v>
       </x:c>
       <x:c r="C24" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18757,7 +18836,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B25" s="4" t="str">
-        <x:v>Household utensil</x:v>
+        <x:v>Food material</x:v>
       </x:c>
       <x:c r="C25" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18768,7 +18847,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B26" s="4" t="str">
-        <x:v>Musical instrument</x:v>
+        <x:v>Gem material</x:v>
       </x:c>
       <x:c r="C26" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18779,7 +18858,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B27" s="4" t="str">
-        <x:v>Processed material</x:v>
+        <x:v>Household utensil</x:v>
       </x:c>
       <x:c r="C27" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18790,7 +18869,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B28" s="4" t="str">
-        <x:v>Raw material</x:v>
+        <x:v>Musical instrument</x:v>
       </x:c>
       <x:c r="C28" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18801,7 +18880,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B29" s="4" t="str">
-        <x:v>Service kit</x:v>
+        <x:v>Processed material</x:v>
       </x:c>
       <x:c r="C29" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18812,7 +18891,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B30" s="4" t="str">
-        <x:v>Shelter kit</x:v>
+        <x:v>Raw material</x:v>
       </x:c>
       <x:c r="C30" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18823,7 +18902,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B31" s="4" t="str">
-        <x:v>Shield</x:v>
+        <x:v>Service kit</x:v>
       </x:c>
       <x:c r="C31" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18834,7 +18913,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B32" s="4" t="str">
-        <x:v>Tool</x:v>
+        <x:v>Shelter kit</x:v>
       </x:c>
       <x:c r="C32" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18845,7 +18924,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B33" s="4" t="str">
-        <x:v>Trip hazard</x:v>
+        <x:v>Shield</x:v>
       </x:c>
       <x:c r="C33" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18856,7 +18935,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B34" s="4" t="str">
-        <x:v>Wearable</x:v>
+        <x:v>Tool</x:v>
       </x:c>
       <x:c r="C34" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -18864,24 +18943,24 @@
     </x:row>
     <x:row r="35" ht="45" customHeight="1">
       <x:c r="A35" s="4" t="str">
-        <x:v>Processing stage</x:v>
+        <x:v>Item type</x:v>
       </x:c>
       <x:c r="B35" s="4" t="str">
-        <x:v>Ancient manufactured</x:v>
+        <x:v>Trip hazard</x:v>
       </x:c>
       <x:c r="C35" s="4" t="str">
-        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
+        <x:v>What the object is, independent of material, culture and use.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="45" customHeight="1">
       <x:c r="A36" s="4" t="str">
-        <x:v>Processing stage</x:v>
+        <x:v>Item type</x:v>
       </x:c>
       <x:c r="B36" s="4" t="str">
-        <x:v>Extracted material</x:v>
+        <x:v>Wearable</x:v>
       </x:c>
       <x:c r="C36" s="4" t="str">
-        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
+        <x:v>What the object is, independent of material, culture and use.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="45" customHeight="1">
@@ -18889,7 +18968,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B37" s="4" t="str">
-        <x:v>Finished item</x:v>
+        <x:v>Ancient manufactured</x:v>
       </x:c>
       <x:c r="C37" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -18900,7 +18979,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B38" s="4" t="str">
-        <x:v>Processed intermediate</x:v>
+        <x:v>Extracted material</x:v>
       </x:c>
       <x:c r="C38" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -18911,7 +18990,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B39" s="4" t="str">
-        <x:v>Raw</x:v>
+        <x:v>Finished item</x:v>
       </x:c>
       <x:c r="C39" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -18922,7 +19001,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B40" s="4" t="str">
-        <x:v>Recovered part</x:v>
+        <x:v>Processed intermediate</x:v>
       </x:c>
       <x:c r="C40" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -18933,7 +19012,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B41" s="4" t="str">
-        <x:v>Unfired intermediate</x:v>
+        <x:v>Raw</x:v>
       </x:c>
       <x:c r="C41" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -18944,7 +19023,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B42" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Recovered part</x:v>
       </x:c>
       <x:c r="C42" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -18955,7 +19034,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B43" s="4" t="str">
-        <x:v>Unworked metal</x:v>
+        <x:v>Unfired intermediate</x:v>
       </x:c>
       <x:c r="C43" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -18963,24 +19042,24 @@
     </x:row>
     <x:row r="44" ht="45" customHeight="1">
       <x:c r="A44" s="4" t="str">
-        <x:v>Origin family</x:v>
+        <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B44" s="4" t="str">
-        <x:v>Ancient technology</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C44" s="4" t="str">
-        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
+        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="45" customHeight="1">
       <x:c r="A45" s="4" t="str">
-        <x:v>Origin family</x:v>
+        <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B45" s="4" t="str">
-        <x:v>Atmospheric</x:v>
+        <x:v>Unworked metal</x:v>
       </x:c>
       <x:c r="C45" s="4" t="str">
-        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
+        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="45" customHeight="1">
@@ -18988,7 +19067,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B46" s="4" t="str">
-        <x:v>Fauna</x:v>
+        <x:v>Ancient technology</x:v>
       </x:c>
       <x:c r="C46" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -18999,7 +19078,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B47" s="4" t="str">
-        <x:v>Geological</x:v>
+        <x:v>Atmospheric</x:v>
       </x:c>
       <x:c r="C47" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -19010,7 +19089,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B48" s="4" t="str">
-        <x:v>Living culture</x:v>
+        <x:v>Fauna</x:v>
       </x:c>
       <x:c r="C48" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -19021,7 +19100,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B49" s="4" t="str">
-        <x:v>Manufactured / unresolved</x:v>
+        <x:v>Geological</x:v>
       </x:c>
       <x:c r="C49" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -19032,7 +19111,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B50" s="4" t="str">
-        <x:v>Recovered machinery</x:v>
+        <x:v>Living culture</x:v>
       </x:c>
       <x:c r="C50" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -19043,7 +19122,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B51" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Manufactured / unresolved</x:v>
       </x:c>
       <x:c r="C51" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -19051,24 +19130,24 @@
     </x:row>
     <x:row r="52" ht="45" customHeight="1">
       <x:c r="A52" s="4" t="str">
-        <x:v>Primary use</x:v>
+        <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B52" s="4" t="str">
-        <x:v>Area denial</x:v>
+        <x:v>Recovered machinery</x:v>
       </x:c>
       <x:c r="C52" s="4" t="str">
-        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
+        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="45" customHeight="1">
       <x:c r="A53" s="4" t="str">
-        <x:v>Primary use</x:v>
+        <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B53" s="4" t="str">
-        <x:v>Binding and construction</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C53" s="4" t="str">
-        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
+        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="45" customHeight="1">
@@ -19076,7 +19155,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B54" s="4" t="str">
-        <x:v>Camp rest</x:v>
+        <x:v>Area denial</x:v>
       </x:c>
       <x:c r="C54" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19087,7 +19166,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B55" s="4" t="str">
-        <x:v>Cargo organization</x:v>
+        <x:v>Binding and construction</x:v>
       </x:c>
       <x:c r="C55" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19098,7 +19177,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B56" s="4" t="str">
-        <x:v>Ceremony</x:v>
+        <x:v>Camp rest</x:v>
       </x:c>
       <x:c r="C56" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19109,7 +19188,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B57" s="4" t="str">
-        <x:v>Chemical processing</x:v>
+        <x:v>Cargo organization</x:v>
       </x:c>
       <x:c r="C57" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19120,7 +19199,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B58" s="4" t="str">
-        <x:v>Civic identification</x:v>
+        <x:v>Ceremony</x:v>
       </x:c>
       <x:c r="C58" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19131,7 +19210,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B59" s="4" t="str">
-        <x:v>Civic recognition</x:v>
+        <x:v>Chemical processing</x:v>
       </x:c>
       <x:c r="C59" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19142,7 +19221,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B60" s="4" t="str">
-        <x:v>Cleaning</x:v>
+        <x:v>Civic identification</x:v>
       </x:c>
       <x:c r="C60" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19153,7 +19232,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B61" s="4" t="str">
-        <x:v>Clothing</x:v>
+        <x:v>Civic recognition</x:v>
       </x:c>
       <x:c r="C61" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19164,7 +19243,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B62" s="4" t="str">
-        <x:v>Clothing fabrication</x:v>
+        <x:v>Cleaning</x:v>
       </x:c>
       <x:c r="C62" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19175,7 +19254,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B63" s="4" t="str">
-        <x:v>Culture support</x:v>
+        <x:v>Clothing</x:v>
       </x:c>
       <x:c r="C63" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19186,7 +19265,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B64" s="4" t="str">
-        <x:v>Decoration</x:v>
+        <x:v>Clothing fabrication</x:v>
       </x:c>
       <x:c r="C64" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19197,7 +19276,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B65" s="4" t="str">
-        <x:v>Devotion</x:v>
+        <x:v>Culture support</x:v>
       </x:c>
       <x:c r="C65" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19208,7 +19287,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B66" s="4" t="str">
-        <x:v>Dust exclusion</x:v>
+        <x:v>Decoration</x:v>
       </x:c>
       <x:c r="C66" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19219,7 +19298,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B67" s="4" t="str">
-        <x:v>Electrical conduction</x:v>
+        <x:v>Devotion</x:v>
       </x:c>
       <x:c r="C67" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19230,7 +19309,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B68" s="4" t="str">
-        <x:v>Electrical insulation</x:v>
+        <x:v>Dust exclusion</x:v>
       </x:c>
       <x:c r="C68" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19241,7 +19320,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B69" s="4" t="str">
-        <x:v>Electrical work</x:v>
+        <x:v>Electrical conduction</x:v>
       </x:c>
       <x:c r="C69" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19252,7 +19331,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B70" s="4" t="str">
-        <x:v>Energy processing</x:v>
+        <x:v>Electrical insulation</x:v>
       </x:c>
       <x:c r="C70" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19263,7 +19342,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B71" s="4" t="str">
-        <x:v>Energy storage</x:v>
+        <x:v>Electrical work</x:v>
       </x:c>
       <x:c r="C71" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19274,7 +19353,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B72" s="4" t="str">
-        <x:v>Equipment mounting</x:v>
+        <x:v>Energy processing</x:v>
       </x:c>
       <x:c r="C72" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19285,7 +19364,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B73" s="4" t="str">
-        <x:v>Equipment repair</x:v>
+        <x:v>Energy storage</x:v>
       </x:c>
       <x:c r="C73" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19296,7 +19375,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B74" s="4" t="str">
-        <x:v>Excavation</x:v>
+        <x:v>Equipment mounting</x:v>
       </x:c>
       <x:c r="C74" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19307,7 +19386,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B75" s="4" t="str">
-        <x:v>Fabrication</x:v>
+        <x:v>Equipment repair</x:v>
       </x:c>
       <x:c r="C75" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19318,7 +19397,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B76" s="4" t="str">
-        <x:v>Fashion</x:v>
+        <x:v>Excavation</x:v>
       </x:c>
       <x:c r="C76" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19329,7 +19408,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B77" s="4" t="str">
-        <x:v>Fauna interaction</x:v>
+        <x:v>Fabrication</x:v>
       </x:c>
       <x:c r="C77" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19340,7 +19419,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B78" s="4" t="str">
-        <x:v>Fiber processing</x:v>
+        <x:v>Fashion</x:v>
       </x:c>
       <x:c r="C78" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19351,7 +19430,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B79" s="4" t="str">
-        <x:v>Food service</x:v>
+        <x:v>Fauna interaction</x:v>
       </x:c>
       <x:c r="C79" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19362,7 +19441,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B80" s="4" t="str">
-        <x:v>Fuel</x:v>
+        <x:v>Fiber processing</x:v>
       </x:c>
       <x:c r="C80" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19373,7 +19452,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B81" s="4" t="str">
-        <x:v>Glass and ceramics</x:v>
+        <x:v>Food service</x:v>
       </x:c>
       <x:c r="C81" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19384,7 +19463,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B82" s="4" t="str">
-        <x:v>Grooming</x:v>
+        <x:v>Fuel</x:v>
       </x:c>
       <x:c r="C82" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19395,7 +19474,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B83" s="4" t="str">
-        <x:v>Injury treatment</x:v>
+        <x:v>Glass and ceramics</x:v>
       </x:c>
       <x:c r="C83" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19406,7 +19485,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B84" s="4" t="str">
-        <x:v>Inspection</x:v>
+        <x:v>Grooming</x:v>
       </x:c>
       <x:c r="C84" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19417,7 +19496,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B85" s="4" t="str">
-        <x:v>Keepsake storage</x:v>
+        <x:v>Injury treatment</x:v>
       </x:c>
       <x:c r="C85" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19428,7 +19507,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B86" s="4" t="str">
-        <x:v>Liquid and bulk containment</x:v>
+        <x:v>Inspection</x:v>
       </x:c>
       <x:c r="C86" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19439,7 +19518,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B87" s="4" t="str">
-        <x:v>Lubrication</x:v>
+        <x:v>Keepsake storage</x:v>
       </x:c>
       <x:c r="C87" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19450,7 +19529,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B88" s="4" t="str">
-        <x:v>Machinery repair</x:v>
+        <x:v>Liquid and bulk containment</x:v>
       </x:c>
       <x:c r="C88" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19461,7 +19540,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B89" s="4" t="str">
-        <x:v>Magnetic tools</x:v>
+        <x:v>Lubrication</x:v>
       </x:c>
       <x:c r="C89" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19472,7 +19551,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B90" s="4" t="str">
-        <x:v>Material exclusion</x:v>
+        <x:v>Machinery repair</x:v>
       </x:c>
       <x:c r="C90" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19483,7 +19562,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B91" s="4" t="str">
-        <x:v>Material transfer</x:v>
+        <x:v>Magnetic tools</x:v>
       </x:c>
       <x:c r="C91" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19494,7 +19573,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B92" s="4" t="str">
-        <x:v>Metal refining</x:v>
+        <x:v>Material exclusion</x:v>
       </x:c>
       <x:c r="C92" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19505,7 +19584,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B93" s="4" t="str">
-        <x:v>Music</x:v>
+        <x:v>Material transfer</x:v>
       </x:c>
       <x:c r="C93" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19516,7 +19595,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B94" s="4" t="str">
-        <x:v>Nutrition</x:v>
+        <x:v>Metal refining</x:v>
       </x:c>
       <x:c r="C94" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19527,7 +19606,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B95" s="4" t="str">
-        <x:v>Paper making</x:v>
+        <x:v>Music</x:v>
       </x:c>
       <x:c r="C95" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19538,7 +19617,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B96" s="4" t="str">
-        <x:v>Protection</x:v>
+        <x:v>Nutrition</x:v>
       </x:c>
       <x:c r="C96" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19549,7 +19628,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Protective fabrication</x:v>
+        <x:v>Paper making</x:v>
       </x:c>
       <x:c r="C97" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19560,7 +19639,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B98" s="4" t="str">
-        <x:v>Provenance</x:v>
+        <x:v>Protection</x:v>
       </x:c>
       <x:c r="C98" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19571,7 +19650,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B99" s="4" t="str">
-        <x:v>Public communication</x:v>
+        <x:v>Protective fabrication</x:v>
       </x:c>
       <x:c r="C99" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19582,7 +19661,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B100" s="4" t="str">
-        <x:v>Remembrance</x:v>
+        <x:v>Provenance</x:v>
       </x:c>
       <x:c r="C100" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19593,7 +19672,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B101" s="4" t="str">
-        <x:v>Resource collection</x:v>
+        <x:v>Public communication</x:v>
       </x:c>
       <x:c r="C101" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19604,7 +19683,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B102" s="4" t="str">
-        <x:v>Sealing</x:v>
+        <x:v>Remembrance</x:v>
       </x:c>
       <x:c r="C102" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19615,7 +19694,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B103" s="4" t="str">
-        <x:v>Specialist samples</x:v>
+        <x:v>Resource collection</x:v>
       </x:c>
       <x:c r="C103" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19626,7 +19705,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B104" s="4" t="str">
-        <x:v>Static management</x:v>
+        <x:v>Sealing</x:v>
       </x:c>
       <x:c r="C104" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19637,7 +19716,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B105" s="4" t="str">
-        <x:v>Sun shading</x:v>
+        <x:v>Specialist samples</x:v>
       </x:c>
       <x:c r="C105" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19648,7 +19727,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B106" s="4" t="str">
-        <x:v>Surface finishing</x:v>
+        <x:v>Static management</x:v>
       </x:c>
       <x:c r="C106" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19659,7 +19738,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B107" s="4" t="str">
-        <x:v>Survival provision</x:v>
+        <x:v>Sun shading</x:v>
       </x:c>
       <x:c r="C107" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19670,7 +19749,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B108" s="4" t="str">
-        <x:v>Textile processing</x:v>
+        <x:v>Surface finishing</x:v>
       </x:c>
       <x:c r="C108" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19681,7 +19760,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B109" s="4" t="str">
-        <x:v>Tool fabrication</x:v>
+        <x:v>Survival provision</x:v>
       </x:c>
       <x:c r="C109" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19692,7 +19771,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B110" s="4" t="str">
-        <x:v>Traversal</x:v>
+        <x:v>Textile processing</x:v>
       </x:c>
       <x:c r="C110" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19703,7 +19782,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B111" s="4" t="str">
-        <x:v>Use unresolved</x:v>
+        <x:v>Tool fabrication</x:v>
       </x:c>
       <x:c r="C111" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19714,7 +19793,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B112" s="4" t="str">
-        <x:v>Vision</x:v>
+        <x:v>Trade</x:v>
       </x:c>
       <x:c r="C112" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19725,7 +19804,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B113" s="4" t="str">
-        <x:v>Work holding</x:v>
+        <x:v>Traversal</x:v>
       </x:c>
       <x:c r="C113" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19736,7 +19815,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B114" s="4" t="str">
-        <x:v>Writing and records</x:v>
+        <x:v>Use unresolved</x:v>
       </x:c>
       <x:c r="C114" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19744,35 +19823,35 @@
     </x:row>
     <x:row r="115" ht="45" customHeight="1">
       <x:c r="A115" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B115" s="4" t="str">
-        <x:v>Ancient composite</x:v>
+        <x:v>Vision</x:v>
       </x:c>
       <x:c r="C115" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="45" customHeight="1">
       <x:c r="A116" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B116" s="4" t="str">
-        <x:v>Biological chemical</x:v>
+        <x:v>Work holding</x:v>
       </x:c>
       <x:c r="C116" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="45" customHeight="1">
       <x:c r="A117" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B117" s="4" t="str">
-        <x:v>Carbonaceous material</x:v>
+        <x:v>Writing and records</x:v>
       </x:c>
       <x:c r="C117" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="45" customHeight="1">
@@ -19780,7 +19859,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B118" s="4" t="str">
-        <x:v>Ceramic</x:v>
+        <x:v>Ancient composite</x:v>
       </x:c>
       <x:c r="C118" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19791,7 +19870,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B119" s="4" t="str">
-        <x:v>Ceramic and metal</x:v>
+        <x:v>Biological chemical</x:v>
       </x:c>
       <x:c r="C119" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19802,7 +19881,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B120" s="4" t="str">
-        <x:v>Ceramic feed mixture</x:v>
+        <x:v>Carbonaceous material</x:v>
       </x:c>
       <x:c r="C120" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19813,7 +19892,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B121" s="4" t="str">
-        <x:v>Faunal fiber</x:v>
+        <x:v>Ceramic</x:v>
       </x:c>
       <x:c r="C121" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19824,7 +19903,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B122" s="4" t="str">
-        <x:v>Faunal fiber and shell</x:v>
+        <x:v>Ceramic and metal</x:v>
       </x:c>
       <x:c r="C122" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19835,7 +19914,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B123" s="4" t="str">
-        <x:v>Faunal membrane</x:v>
+        <x:v>Ceramic feed mixture</x:v>
       </x:c>
       <x:c r="C123" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19846,7 +19925,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B124" s="4" t="str">
-        <x:v>Faunal tissue</x:v>
+        <x:v>Faunal fiber</x:v>
       </x:c>
       <x:c r="C124" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19857,7 +19936,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B125" s="4" t="str">
-        <x:v>Fur</x:v>
+        <x:v>Faunal fiber and shell</x:v>
       </x:c>
       <x:c r="C125" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19868,7 +19947,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B126" s="4" t="str">
-        <x:v>Gemstone</x:v>
+        <x:v>Faunal membrane</x:v>
       </x:c>
       <x:c r="C126" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19879,7 +19958,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B127" s="4" t="str">
-        <x:v>Glass</x:v>
+        <x:v>Faunal tissue</x:v>
       </x:c>
       <x:c r="C127" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19890,7 +19969,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B128" s="4" t="str">
-        <x:v>Glass and metal</x:v>
+        <x:v>Fur</x:v>
       </x:c>
       <x:c r="C128" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19901,7 +19980,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B129" s="4" t="str">
-        <x:v>Glass and shell</x:v>
+        <x:v>Gemstone</x:v>
       </x:c>
       <x:c r="C129" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19912,7 +19991,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B130" s="4" t="str">
-        <x:v>Glass with unresolved casing</x:v>
+        <x:v>Glass</x:v>
       </x:c>
       <x:c r="C130" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19923,7 +20002,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B131" s="4" t="str">
-        <x:v>Hide</x:v>
+        <x:v>Glass and metal</x:v>
       </x:c>
       <x:c r="C131" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19934,7 +20013,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B132" s="4" t="str">
-        <x:v>Husk fiber</x:v>
+        <x:v>Glass and shell</x:v>
       </x:c>
       <x:c r="C132" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19945,7 +20024,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B133" s="4" t="str">
-        <x:v>Husk fiber and shell</x:v>
+        <x:v>Glass with unresolved casing</x:v>
       </x:c>
       <x:c r="C133" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19956,7 +20035,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B134" s="4" t="str">
-        <x:v>Metal</x:v>
+        <x:v>Hide</x:v>
       </x:c>
       <x:c r="C134" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19967,7 +20046,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B135" s="4" t="str">
-        <x:v>Metal and shell</x:v>
+        <x:v>Husk fiber</x:v>
       </x:c>
       <x:c r="C135" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19978,7 +20057,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B136" s="4" t="str">
-        <x:v>Metal or shell</x:v>
+        <x:v>Husk fiber and shell</x:v>
       </x:c>
       <x:c r="C136" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19989,7 +20068,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B137" s="4" t="str">
-        <x:v>Mineral</x:v>
+        <x:v>Metal</x:v>
       </x:c>
       <x:c r="C137" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20000,7 +20079,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B138" s="4" t="str">
-        <x:v>Mineral or shell</x:v>
+        <x:v>Metal and shell</x:v>
       </x:c>
       <x:c r="C138" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20011,7 +20090,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B139" s="4" t="str">
-        <x:v>Mixed / unresolved</x:v>
+        <x:v>Metal or shell</x:v>
       </x:c>
       <x:c r="C139" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20022,7 +20101,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B140" s="4" t="str">
-        <x:v>Shell / chitin</x:v>
+        <x:v>Mineral</x:v>
       </x:c>
       <x:c r="C140" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20033,7 +20112,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B141" s="4" t="str">
-        <x:v>Shell and mineral</x:v>
+        <x:v>Mineral or shell</x:v>
       </x:c>
       <x:c r="C141" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20044,7 +20123,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B142" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Mixed / unresolved</x:v>
       </x:c>
       <x:c r="C142" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20055,7 +20134,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B143" s="4" t="str">
-        <x:v>Wing membrane</x:v>
+        <x:v>Shell / chitin</x:v>
       </x:c>
       <x:c r="C143" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20063,35 +20142,35 @@
     </x:row>
     <x:row r="144" ht="45" customHeight="1">
       <x:c r="A144" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B144" s="4" t="str">
-        <x:v>Assembly</x:v>
+        <x:v>Shell and mineral</x:v>
       </x:c>
       <x:c r="C144" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="45" customHeight="1">
       <x:c r="A145" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B145" s="4" t="str">
-        <x:v>Bundle</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C145" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="146" ht="45" customHeight="1">
       <x:c r="A146" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B146" s="4" t="str">
-        <x:v>Cord</x:v>
+        <x:v>Wing membrane</x:v>
       </x:c>
       <x:c r="C146" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="147" ht="45" customHeight="1">
@@ -20099,7 +20178,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B147" s="4" t="str">
-        <x:v>Fiber</x:v>
+        <x:v>Assembly</x:v>
       </x:c>
       <x:c r="C147" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20110,7 +20189,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B148" s="4" t="str">
-        <x:v>Folio</x:v>
+        <x:v>Bundle</x:v>
       </x:c>
       <x:c r="C148" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20121,7 +20200,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B149" s="4" t="str">
-        <x:v>Garment</x:v>
+        <x:v>Cord</x:v>
       </x:c>
       <x:c r="C149" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20132,7 +20211,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B150" s="4" t="str">
-        <x:v>Gel</x:v>
+        <x:v>Fiber</x:v>
       </x:c>
       <x:c r="C150" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20143,7 +20222,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B151" s="4" t="str">
-        <x:v>Liquid</x:v>
+        <x:v>Folio</x:v>
       </x:c>
       <x:c r="C151" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20154,7 +20233,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B152" s="4" t="str">
-        <x:v>Membrane</x:v>
+        <x:v>Garment</x:v>
       </x:c>
       <x:c r="C152" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20165,7 +20244,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B153" s="4" t="str">
-        <x:v>Panel</x:v>
+        <x:v>Gel</x:v>
       </x:c>
       <x:c r="C153" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20176,7 +20255,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B154" s="4" t="str">
-        <x:v>Particles</x:v>
+        <x:v>Liquid</x:v>
       </x:c>
       <x:c r="C154" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20187,7 +20266,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B155" s="4" t="str">
-        <x:v>Patch</x:v>
+        <x:v>Membrane</x:v>
       </x:c>
       <x:c r="C155" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20198,7 +20277,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B156" s="4" t="str">
-        <x:v>Rock</x:v>
+        <x:v>Panel</x:v>
       </x:c>
       <x:c r="C156" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20209,7 +20288,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B157" s="4" t="str">
-        <x:v>Sheet</x:v>
+        <x:v>Particles</x:v>
       </x:c>
       <x:c r="C157" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20220,7 +20299,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B158" s="4" t="str">
-        <x:v>Shell plate</x:v>
+        <x:v>Patch</x:v>
       </x:c>
       <x:c r="C158" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20231,7 +20310,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B159" s="4" t="str">
-        <x:v>Solid part</x:v>
+        <x:v>Rock</x:v>
       </x:c>
       <x:c r="C159" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20242,7 +20321,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B160" s="4" t="str">
-        <x:v>Solid piece</x:v>
+        <x:v>Sheet</x:v>
       </x:c>
       <x:c r="C160" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20253,7 +20332,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B161" s="4" t="str">
-        <x:v>Strip</x:v>
+        <x:v>Shell plate</x:v>
       </x:c>
       <x:c r="C161" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20264,7 +20343,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B162" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Solid part</x:v>
       </x:c>
       <x:c r="C162" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20272,35 +20351,35 @@
     </x:row>
     <x:row r="163" ht="45" customHeight="1">
       <x:c r="A163" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B163" s="4" t="str">
-        <x:v>Author direction</x:v>
+        <x:v>Solid piece</x:v>
       </x:c>
       <x:c r="C163" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="45" customHeight="1">
       <x:c r="A164" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B164" s="4" t="str">
-        <x:v>Existing definition</x:v>
+        <x:v>Strip</x:v>
       </x:c>
       <x:c r="C164" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="165" ht="45" customHeight="1">
       <x:c r="A165" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B165" s="4" t="str">
-        <x:v>Proposal</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C165" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="166" ht="45" customHeight="1">
@@ -20308,16 +20387,60 @@
         <x:v>Design status</x:v>
       </x:c>
       <x:c r="B166" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="C166" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="45" customHeight="1">
+      <x:c r="A167" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B167" s="4" t="str">
+        <x:v>Existing definition</x:v>
+      </x:c>
+      <x:c r="C167" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="45" customHeight="1">
+      <x:c r="A168" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B168" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="C168" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="45" customHeight="1">
+      <x:c r="A169" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B169" s="4" t="str">
+        <x:v>Source proposal</x:v>
+      </x:c>
+      <x:c r="C169" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="45" customHeight="1">
+      <x:c r="A170" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B170" s="4" t="str">
         <x:v>Withheld assumption</x:v>
       </x:c>
-      <x:c r="C166" s="4" t="str">
+      <x:c r="C170" s="4" t="str">
         <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6cca720bb1c4704"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49d646966f6e4f5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26684,21 +26807,44 @@
         <x:v>Ceramic item proposal. Catalog intent; compatibility and properties unresolved.</x:v>
       </x:c>
     </x:row>
+    <x:row r="284" ht="70" customHeight="1">
+      <x:c r="A284" s="4" t="str">
+        <x:v>source.currency.imperial_commons</x:v>
+      </x:c>
+      <x:c r="B284" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A284,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Imperial Commons</x:v>
+      </x:c>
+      <x:c r="C284" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A284,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="D284" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E284" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A284,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Trade</x:v>
+      </x:c>
+      <x:c r="F284" s="4" t="str">
+        <x:v>WLD-0032 currency proposal. Unit/denomination and physical form unresolved.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A6:A1005">
-      <x:formula1>'Items'!$A$6:$A$209</x:formula1>
+      <x:formula1>'Items'!$A$6:$A$210</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D6:D1005">
       <x:formula1>"Primary,Secondary"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E6:E1005">
-      <x:formula1>'Taxonomy'!$B$52:$B$114</x:formula1>
+      <x:formula1>'Taxonomy'!$B$54:$B$117</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04bde21282a04393"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a17e7aa52c4348"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27606,7 +27752,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R347efa8692354fae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc183ef2e2fa34cd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27972,7 +28118,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R892de91be3d54486"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5211754261c14b1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28411,10 +28557,25 @@
         <x:v>Existing claystone, alumina, borate, insulating blanks and ceramic reagent jar remain their original entries.</x:v>
       </x:c>
     </x:row>
+    <x:row r="32" ht="90" customHeight="1">
+      <x:c r="A32" s="3" t="str">
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="B32" s="3" t="n">
+        <x:f>COUNTIF(Items!$C$6:$C$1005,"Currency")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C32" s="3" t="str">
+        <x:v>Imperial Commons currency family; aliases Commons and marks</x:v>
+      </x:c>
+      <x:c r="D32" s="3" t="str">
+        <x:v>WLD-0032 draft/proposal names the currency but does not define denominations, physical tokens or exchange ratios.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5644ebef854b44dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb57bcde49740455f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28477,7 +28638,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>204 design entries: 18 existing item IDs and 186 design concepts. Includes 28 ceramic item proposals; classifications and item-use relationships populated.</x:v>
+        <x:v>205 design entries: 18 existing item IDs and 187 design/source concepts. Currency-family entry added from WLD-0032; denominations unresolved.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -29189,7 +29350,7 @@
         <x:v>Filtering the master</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Items is one native filterable table, A5:AE209. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
+        <x:v>Items is one native filterable table, A5:AE210. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="85" customHeight="1">
@@ -29280,10 +29441,34 @@
         <x:v>Filter Items &gt; Material family for Ceramic, Ceramic feed mixture or Ceramic and metal. Use Subtype for feedstock, household, storage, workshop, thermal, electrical, vessel-fitting, ceremonial, protection and household-fitting branches. Item uses includes primary and secondary ceramic uses.</x:v>
       </x:c>
     </x:row>
+    <x:row r="109" ht="90" customHeight="1">
+      <x:c r="A109" s="4" t="str">
+        <x:v>Currency source</x:v>
+      </x:c>
+      <x:c r="B109" s="4" t="str">
+        <x:v>WLD-0032 Currency in Arc &amp; Dust, draft/proposal at verified master revision f6f98515c005dc3c73cccd9cbc031691745740c6, names Imperial Commons, everyday Commons and commercial shorthand marks. These are one currency, not three denominations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="90" customHeight="1">
+      <x:c r="A110" s="4" t="str">
+        <x:v>Denominations unresolved</x:v>
+      </x:c>
+      <x:c r="B110" s="4" t="str">
+        <x:v>The inspected currency record and economy index do not specify denominations, face values, exchange ratios, token materials or whether the currency is coins, notes or account balances. One currency-family placeholder is registered. Do not derive copper/silver/gold tiers, assign a one-Common coin or populate trade prices without a source or author decision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="90" customHeight="1">
+      <x:c r="A111" s="4" t="str">
+        <x:v>Source economy boundary</x:v>
+      </x:c>
+      <x:c r="B111" s="4" t="str">
+        <x:v>The source discusses above-baseline craft, expertise and prestige purchases, non-commodity backing, and survival outside monetary exchange. These remain source proposals; the currency entry does not change the game survival economy, wallet, loot or inventory behavior.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra233638769404052"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7a41cf74834ccd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30127,7 +30312,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32f75a2da65c416b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553e1e47f82b4ef1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30370,7 +30555,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R393307912f304807"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5049846909a4947"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30774,7 +30959,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ca8ad4fb9064235"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R251c5f10292541e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31450,7 +31635,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71110eebd28c4e2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R484393edd28440f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add special stones and lore-constrained cooking items
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R1f3bda4708bb4624"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Re123dea67a0d4ddd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rcf89d166a7244452"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rcb5d82861f614ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Ra6d192d5b5dd42da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rb8bd761487da4207"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R8d08824eb7da4859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Ra123ca8fec514178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R022893996caa4fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="Rc1c776f477604034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R0f47a3a993434baf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="Rfc74994854e3490b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="Rebf0ed6d38354e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="Rafec7c372fa94a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Radae3cc1878f4246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R897e4ff09bff433b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rd27023370c4d4730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R5e53ab5e151b404d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rae5b84966dcc4436"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rf51acec02207439d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Re7f89e76855c4244"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Rccae3676c6874cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R347f758c74f0480f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R8d281f37a6874e1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R33b2bde451f4439f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="Rfce68271b1014adc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,8 +476,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE210" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AE210"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE226" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AE226"/>
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -550,7 +550,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C170" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C175" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Field"/>
     <x:tableColumn id="2" name="Allowed value"/>
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F284" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F284"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F305" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F305"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -614,7 +614,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -626,7 +626,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B111" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -986,7 +986,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>205 entries. Filter W:AC for type, stage, origin, use, material, form and status. Currency denominations remain unresolved.</x:v>
+        <x:v>221 entries. Filter W:AC for classifications; search AD. Cooking and fire uses retain source/author distinctions.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -17410,6 +17410,1270 @@
       </x:c>
       <x:c r="AE210" s="4" t="str">
         <x:v>Source record explicitly names the currency and aliases; no physical denomination item inferred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="115" customHeight="1">
+      <x:c r="A211" s="9" t="str">
+        <x:v>proposal.fire.oxygen_stone</x:v>
+      </x:c>
+      <x:c r="B211" s="9" t="str">
+        <x:v>Oxygen-releasing stone</x:v>
+      </x:c>
+      <x:c r="C211" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D211" s="9" t="str">
+        <x:v>Special stone</x:v>
+      </x:c>
+      <x:c r="E211" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F211" s="9" t="str">
+        <x:v>Stone family that releases oxygen, as requested by author.</x:v>
+      </x:c>
+      <x:c r="G211" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H211" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I211" s="13"/>
+      <x:c r="J211" s="15"/>
+      <x:c r="K211" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L211" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M211" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N211" s="9" t="str">
+        <x:v>Source describes active bedrock under geothermal heat/pressure. Continued output after extraction, rate, exhaustion and activation unresolved; no portable infinite air supply.</x:v>
+      </x:c>
+      <x:c r="O211" s="17"/>
+      <x:c r="P211" s="17"/>
+      <x:c r="Q211" s="17"/>
+      <x:c r="R211" s="17"/>
+      <x:c r="S211" s="17"/>
+      <x:c r="T211" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U211" s="11"/>
+      <x:c r="V211" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+      <x:c r="W211" s="4" t="str">
+        <x:v>Raw material</x:v>
+      </x:c>
+      <x:c r="X211" s="4" t="str">
+        <x:v>Raw</x:v>
+      </x:c>
+      <x:c r="Y211" s="4" t="str">
+        <x:v>Geological</x:v>
+      </x:c>
+      <x:c r="Z211" s="4" t="str">
+        <x:v>Atmospheric support</x:v>
+      </x:c>
+      <x:c r="AA211" s="4" t="str">
+        <x:v>Mineral</x:v>
+      </x:c>
+      <x:c r="AB211" s="4" t="str">
+        <x:v>Rock</x:v>
+      </x:c>
+      <x:c r="AC211" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD211" s="4" t="str">
+        <x:v>oxygen-releasing stone; special stone; raw material; mineral; atmospheric support</x:v>
+      </x:c>
+      <x:c r="AE211" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="115" customHeight="1">
+      <x:c r="A212" s="9" t="str">
+        <x:v>proposal.fire.glow_stone</x:v>
+      </x:c>
+      <x:c r="B212" s="9" t="str">
+        <x:v>Glowing stone</x:v>
+      </x:c>
+      <x:c r="C212" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D212" s="9" t="str">
+        <x:v>Special stone</x:v>
+      </x:c>
+      <x:c r="E212" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F212" s="9" t="str">
+        <x:v>Stone family that emits light, as requested by author.</x:v>
+      </x:c>
+      <x:c r="G212" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H212" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I212" s="13"/>
+      <x:c r="J212" s="15"/>
+      <x:c r="K212" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L212" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M212" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N212" s="9" t="str">
+        <x:v>No owning glow-stone record found in inspected material/atmosphere records. Color, brightness, duration, charging, depletion and heat unresolved; glow does not imply combustion.</x:v>
+      </x:c>
+      <x:c r="O212" s="17"/>
+      <x:c r="P212" s="17"/>
+      <x:c r="Q212" s="17"/>
+      <x:c r="R212" s="17"/>
+      <x:c r="S212" s="17"/>
+      <x:c r="T212" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U212" s="11"/>
+      <x:c r="V212" s="9" t="str">
+        <x:v>Direct author direction October 14, 2026</x:v>
+      </x:c>
+      <x:c r="W212" s="4" t="str">
+        <x:v>Raw material</x:v>
+      </x:c>
+      <x:c r="X212" s="4" t="str">
+        <x:v>Raw</x:v>
+      </x:c>
+      <x:c r="Y212" s="4" t="str">
+        <x:v>Geological</x:v>
+      </x:c>
+      <x:c r="Z212" s="4" t="str">
+        <x:v>Illumination</x:v>
+      </x:c>
+      <x:c r="AA212" s="4" t="str">
+        <x:v>Mineral</x:v>
+      </x:c>
+      <x:c r="AB212" s="4" t="str">
+        <x:v>Rock</x:v>
+      </x:c>
+      <x:c r="AC212" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD212" s="4" t="str">
+        <x:v>glowing stone; special stone; raw material; mineral; illumination</x:v>
+      </x:c>
+      <x:c r="AE212" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="115" customHeight="1">
+      <x:c r="A213" s="9" t="str">
+        <x:v>proposal.fire.flint</x:v>
+      </x:c>
+      <x:c r="B213" s="9" t="str">
+        <x:v>Flint stone</x:v>
+      </x:c>
+      <x:c r="C213" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D213" s="9" t="str">
+        <x:v>Special stone</x:v>
+      </x:c>
+      <x:c r="E213" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F213" s="9" t="str">
+        <x:v>Flint resource requested by author; candidate sparking and worked-edge uses.</x:v>
+      </x:c>
+      <x:c r="G213" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H213" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I213" s="13"/>
+      <x:c r="J213" s="15"/>
+      <x:c r="K213" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L213" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M213" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N213" s="9" t="str">
+        <x:v>No matched striker, tinder, guaranteed ignition or crafting recipe assigned. Atmospheric conditions still matter.</x:v>
+      </x:c>
+      <x:c r="O213" s="17"/>
+      <x:c r="P213" s="17"/>
+      <x:c r="Q213" s="17"/>
+      <x:c r="R213" s="17"/>
+      <x:c r="S213" s="17"/>
+      <x:c r="T213" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U213" s="11"/>
+      <x:c r="V213" s="9" t="str">
+        <x:v>Direct author direction October 14, 2026</x:v>
+      </x:c>
+      <x:c r="W213" s="4" t="str">
+        <x:v>Raw material</x:v>
+      </x:c>
+      <x:c r="X213" s="4" t="str">
+        <x:v>Raw</x:v>
+      </x:c>
+      <x:c r="Y213" s="4" t="str">
+        <x:v>Geological</x:v>
+      </x:c>
+      <x:c r="Z213" s="4" t="str">
+        <x:v>Ignition</x:v>
+      </x:c>
+      <x:c r="AA213" s="4" t="str">
+        <x:v>Mineral</x:v>
+      </x:c>
+      <x:c r="AB213" s="4" t="str">
+        <x:v>Rock</x:v>
+      </x:c>
+      <x:c r="AC213" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD213" s="4" t="str">
+        <x:v>flint stone; special stone; raw material; mineral; ignition; tool fabrication</x:v>
+      </x:c>
+      <x:c r="AE213" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="115" customHeight="1">
+      <x:c r="A214" s="9" t="str">
+        <x:v>proposal.fire.striker</x:v>
+      </x:c>
+      <x:c r="B214" s="9" t="str">
+        <x:v>Flint striking tool</x:v>
+      </x:c>
+      <x:c r="C214" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D214" s="9" t="str">
+        <x:v>Ignition tool</x:v>
+      </x:c>
+      <x:c r="E214" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F214" s="9" t="str">
+        <x:v>Worked striking implement candidate used with compatible flint.</x:v>
+      </x:c>
+      <x:c r="G214" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H214" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I214" s="13"/>
+      <x:c r="J214" s="15"/>
+      <x:c r="K214" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L214" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M214" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N214" s="9" t="str">
+        <x:v>Striking-face composition and fuel/tinder pairing TBD; a spark does not guarantee a sustained cooking fire.</x:v>
+      </x:c>
+      <x:c r="O214" s="17"/>
+      <x:c r="P214" s="17"/>
+      <x:c r="Q214" s="17"/>
+      <x:c r="R214" s="17"/>
+      <x:c r="S214" s="17"/>
+      <x:c r="T214" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U214" s="11"/>
+      <x:c r="V214" s="9" t="str">
+        <x:v>New game proposal from author flint direction</x:v>
+      </x:c>
+      <x:c r="W214" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X214" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y214" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z214" s="4" t="str">
+        <x:v>Ignition</x:v>
+      </x:c>
+      <x:c r="AA214" s="4" t="str">
+        <x:v>Metal or shell</x:v>
+      </x:c>
+      <x:c r="AB214" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC214" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD214" s="4" t="str">
+        <x:v>flint striking tool; ignition tool; tool; metal or shell; ignition</x:v>
+      </x:c>
+      <x:c r="AE214" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="115" customHeight="1">
+      <x:c r="A215" s="9" t="str">
+        <x:v>proposal.fire.chitin_char</x:v>
+      </x:c>
+      <x:c r="B215" s="9" t="str">
+        <x:v>Chitin-char</x:v>
+      </x:c>
+      <x:c r="C215" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D215" s="9" t="str">
+        <x:v>Fire fuel</x:v>
+      </x:c>
+      <x:c r="E215" s="9" t="str">
+        <x:v>Source proposal; not implemented</x:v>
+      </x:c>
+      <x:c r="F215" s="9" t="str">
+        <x:v>Carbonized chitin material described in the chitin source record.</x:v>
+      </x:c>
+      <x:c r="G215" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H215" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I215" s="13"/>
+      <x:c r="J215" s="15"/>
+      <x:c r="K215" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L215" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M215" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N215" s="9" t="str">
+        <x:v>Exact preparation and fuel performance unapproved. Existing generic Charcoal is retained; decide whether these become a material variant or separate resources before implementation.</x:v>
+      </x:c>
+      <x:c r="O215" s="17"/>
+      <x:c r="P215" s="17"/>
+      <x:c r="Q215" s="17"/>
+      <x:c r="R215" s="17"/>
+      <x:c r="S215" s="17"/>
+      <x:c r="T215" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U215" s="11"/>
+      <x:c r="V215" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+      <x:c r="W215" s="4" t="str">
+        <x:v>Processed material</x:v>
+      </x:c>
+      <x:c r="X215" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y215" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z215" s="4" t="str">
+        <x:v>Fuel</x:v>
+      </x:c>
+      <x:c r="AA215" s="4" t="str">
+        <x:v>Carbonaceous material</x:v>
+      </x:c>
+      <x:c r="AB215" s="4" t="str">
+        <x:v>Solid piece</x:v>
+      </x:c>
+      <x:c r="AC215" s="4" t="str">
+        <x:v>Source proposal</x:v>
+      </x:c>
+      <x:c r="AD215" s="4" t="str">
+        <x:v>chitin-char; fire fuel; processed material; carbonaceous material; fuel</x:v>
+      </x:c>
+      <x:c r="AE215" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="115" customHeight="1">
+      <x:c r="A216" s="9" t="str">
+        <x:v>proposal.fire.cooking_pot</x:v>
+      </x:c>
+      <x:c r="B216" s="9" t="str">
+        <x:v>Ceramic cooking pot</x:v>
+      </x:c>
+      <x:c r="C216" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D216" s="9" t="str">
+        <x:v>Cooking vessel</x:v>
+      </x:c>
+      <x:c r="E216" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F216" s="9" t="str">
+        <x:v>Purpose-made ceramic vessel candidate for heating a contained food portion.</x:v>
+      </x:c>
+      <x:c r="G216" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H216" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I216" s="13"/>
+      <x:c r="J216" s="15"/>
+      <x:c r="K216" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L216" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M216" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N216" s="9" t="str">
+        <x:v>Food-contact suitability, supported contents, heat grade and process TBD. Distinct from cold serving bowl, storage crock and chemical-service jar.</x:v>
+      </x:c>
+      <x:c r="O216" s="17"/>
+      <x:c r="P216" s="17"/>
+      <x:c r="Q216" s="17"/>
+      <x:c r="R216" s="17"/>
+      <x:c r="S216" s="17"/>
+      <x:c r="T216" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U216" s="11"/>
+      <x:c r="V216" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+      <x:c r="W216" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X216" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y216" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z216" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="AA216" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB216" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC216" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD216" s="4" t="str">
+        <x:v>ceramic cooking pot; cooking vessel; tool; ceramic; cooking</x:v>
+      </x:c>
+      <x:c r="AE216" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="115" customHeight="1">
+      <x:c r="A217" s="9" t="str">
+        <x:v>proposal.fire.cooking_slab</x:v>
+      </x:c>
+      <x:c r="B217" s="9" t="str">
+        <x:v>Cooking stone slab</x:v>
+      </x:c>
+      <x:c r="C217" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D217" s="9" t="str">
+        <x:v>Cooking tool</x:v>
+      </x:c>
+      <x:c r="E217" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F217" s="9" t="str">
+        <x:v>Selected worked stone surface candidate for food heating.</x:v>
+      </x:c>
+      <x:c r="G217" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H217" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I217" s="13"/>
+      <x:c r="J217" s="15"/>
+      <x:c r="K217" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L217" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M217" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N217" s="9" t="str">
+        <x:v>Stone selection and thermal behavior undefined; oxygen/glow stones are not automatically suitable cooking surfaces.</x:v>
+      </x:c>
+      <x:c r="O217" s="17"/>
+      <x:c r="P217" s="17"/>
+      <x:c r="Q217" s="17"/>
+      <x:c r="R217" s="17"/>
+      <x:c r="S217" s="17"/>
+      <x:c r="T217" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U217" s="11"/>
+      <x:c r="V217" s="9" t="str">
+        <x:v>New game proposal from author cooking direction</x:v>
+      </x:c>
+      <x:c r="W217" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X217" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y217" s="4" t="str">
+        <x:v>Geological</x:v>
+      </x:c>
+      <x:c r="Z217" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="AA217" s="4" t="str">
+        <x:v>Mineral</x:v>
+      </x:c>
+      <x:c r="AB217" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC217" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD217" s="4" t="str">
+        <x:v>cooking stone slab; cooking tool; tool; mineral; cooking</x:v>
+      </x:c>
+      <x:c r="AE217" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="115" customHeight="1">
+      <x:c r="A218" s="9" t="str">
+        <x:v>proposal.fire.lidded_pan</x:v>
+      </x:c>
+      <x:c r="B218" s="9" t="str">
+        <x:v>Lidded cooking pan</x:v>
+      </x:c>
+      <x:c r="C218" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D218" s="9" t="str">
+        <x:v>Cooking vessel</x:v>
+      </x:c>
+      <x:c r="E218" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F218" s="9" t="str">
+        <x:v>Metal cooking pan with matched cover for controlled heating.</x:v>
+      </x:c>
+      <x:c r="G218" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H218" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I218" s="13"/>
+      <x:c r="J218" s="15"/>
+      <x:c r="K218" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L218" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M218" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N218" s="9" t="str">
+        <x:v>Lid is part of the item family; heat requirements and food process unresolved. No water-boiling recipe assumed.</x:v>
+      </x:c>
+      <x:c r="O218" s="17"/>
+      <x:c r="P218" s="17"/>
+      <x:c r="Q218" s="17"/>
+      <x:c r="R218" s="17"/>
+      <x:c r="S218" s="17"/>
+      <x:c r="T218" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U218" s="11"/>
+      <x:c r="V218" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+      <x:c r="W218" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X218" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y218" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z218" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="AA218" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB218" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC218" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD218" s="4" t="str">
+        <x:v>lidded cooking pan; cooking vessel; tool; metal; cooking</x:v>
+      </x:c>
+      <x:c r="AE218" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="115" customHeight="1">
+      <x:c r="A219" s="9" t="str">
+        <x:v>proposal.fire.rack</x:v>
+      </x:c>
+      <x:c r="B219" s="9" t="str">
+        <x:v>Cooking rack</x:v>
+      </x:c>
+      <x:c r="C219" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D219" s="9" t="str">
+        <x:v>Cooking tool</x:v>
+      </x:c>
+      <x:c r="E219" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F219" s="9" t="str">
+        <x:v>Open rack for a specifically supported food-heating method.</x:v>
+      </x:c>
+      <x:c r="G219" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H219" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I219" s="13"/>
+      <x:c r="J219" s="15"/>
+      <x:c r="K219" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L219" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M219" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N219" s="9" t="str">
+        <x:v>Compatible food and heat source TBD; cooking does not automatically detoxify fauna.</x:v>
+      </x:c>
+      <x:c r="O219" s="17"/>
+      <x:c r="P219" s="17"/>
+      <x:c r="Q219" s="17"/>
+      <x:c r="R219" s="17"/>
+      <x:c r="S219" s="17"/>
+      <x:c r="T219" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U219" s="11"/>
+      <x:c r="V219" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+      <x:c r="W219" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X219" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y219" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z219" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="AA219" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB219" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC219" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD219" s="4" t="str">
+        <x:v>cooking rack; cooking tool; tool; metal; cooking</x:v>
+      </x:c>
+      <x:c r="AE219" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="115" customHeight="1">
+      <x:c r="A220" s="9" t="str">
+        <x:v>proposal.fire.pot_stand</x:v>
+      </x:c>
+      <x:c r="B220" s="9" t="str">
+        <x:v>Cooking pot stand</x:v>
+      </x:c>
+      <x:c r="C220" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D220" s="9" t="str">
+        <x:v>Cooking tool</x:v>
+      </x:c>
+      <x:c r="E220" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F220" s="9" t="str">
+        <x:v>Support a compatible vessel above a managed heat source.</x:v>
+      </x:c>
+      <x:c r="G220" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H220" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I220" s="13"/>
+      <x:c r="J220" s="15"/>
+      <x:c r="K220" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L220" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M220" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N220" s="9" t="str">
+        <x:v>Footprint, heat clearance and field deployment unresolved; no free-standing workstation service implied.</x:v>
+      </x:c>
+      <x:c r="O220" s="17"/>
+      <x:c r="P220" s="17"/>
+      <x:c r="Q220" s="17"/>
+      <x:c r="R220" s="17"/>
+      <x:c r="S220" s="17"/>
+      <x:c r="T220" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U220" s="11"/>
+      <x:c r="V220" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+      <x:c r="W220" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X220" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y220" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z220" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="AA220" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB220" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC220" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD220" s="4" t="str">
+        <x:v>cooking pot stand; cooking tool; tool; metal; cooking</x:v>
+      </x:c>
+      <x:c r="AE220" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="115" customHeight="1">
+      <x:c r="A221" s="9" t="str">
+        <x:v>proposal.fire.tongs</x:v>
+      </x:c>
+      <x:c r="B221" s="9" t="str">
+        <x:v>Cooking tongs</x:v>
+      </x:c>
+      <x:c r="C221" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D221" s="9" t="str">
+        <x:v>Cooking tool</x:v>
+      </x:c>
+      <x:c r="E221" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F221" s="9" t="str">
+        <x:v>Handle compatible hot cooking items.</x:v>
+      </x:c>
+      <x:c r="G221" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H221" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I221" s="13"/>
+      <x:c r="J221" s="15"/>
+      <x:c r="K221" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L221" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M221" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N221" s="9" t="str">
+        <x:v>Contact surfaces, reach and handling behavior TBD; no automatic immunity to heat.</x:v>
+      </x:c>
+      <x:c r="O221" s="17"/>
+      <x:c r="P221" s="17"/>
+      <x:c r="Q221" s="17"/>
+      <x:c r="R221" s="17"/>
+      <x:c r="S221" s="17"/>
+      <x:c r="T221" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U221" s="11"/>
+      <x:c r="V221" s="9" t="str">
+        <x:v>New game proposal from author cooking direction</x:v>
+      </x:c>
+      <x:c r="W221" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X221" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y221" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z221" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="AA221" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB221" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC221" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD221" s="4" t="str">
+        <x:v>cooking tongs; cooking tool; tool; metal; cooking</x:v>
+      </x:c>
+      <x:c r="AE221" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="115" customHeight="1">
+      <x:c r="A222" s="9" t="str">
+        <x:v>proposal.fire.firebox</x:v>
+      </x:c>
+      <x:c r="B222" s="9" t="str">
+        <x:v>Managed cooking firebox</x:v>
+      </x:c>
+      <x:c r="C222" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D222" s="9" t="str">
+        <x:v>Fire management</x:v>
+      </x:c>
+      <x:c r="E222" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F222" s="9" t="str">
+        <x:v>Contained fire-bed assembly candidate for a chosen low-oxygen cooking setup.</x:v>
+      </x:c>
+      <x:c r="G222" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H222" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I222" s="13"/>
+      <x:c r="J222" s="15"/>
+      <x:c r="K222" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L222" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M222" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N222" s="9" t="str">
+        <x:v>Fuel, intake, exhaust and usable surroundings need design. A box does not create oxygen or make a sealed camp safe.</x:v>
+      </x:c>
+      <x:c r="O222" s="17"/>
+      <x:c r="P222" s="17"/>
+      <x:c r="Q222" s="17"/>
+      <x:c r="R222" s="17"/>
+      <x:c r="S222" s="17"/>
+      <x:c r="T222" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U222" s="11"/>
+      <x:c r="V222" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+      <x:c r="W222" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X222" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y222" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z222" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="AA222" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB222" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC222" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD222" s="4" t="str">
+        <x:v>managed cooking firebox; fire management; tool; mixed / unresolved; cooking; fire management</x:v>
+      </x:c>
+      <x:c r="AE222" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="115" customHeight="1">
+      <x:c r="A223" s="9" t="str">
+        <x:v>proposal.fire.wind_baffle</x:v>
+      </x:c>
+      <x:c r="B223" s="9" t="str">
+        <x:v>Cooking wind baffle</x:v>
+      </x:c>
+      <x:c r="C223" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D223" s="9" t="str">
+        <x:v>Fire management</x:v>
+      </x:c>
+      <x:c r="E223" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F223" s="9" t="str">
+        <x:v>Shaped screen candidate to reduce disruptive crosswind around a cooking setup.</x:v>
+      </x:c>
+      <x:c r="G223" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H223" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I223" s="13"/>
+      <x:c r="J223" s="15"/>
+      <x:c r="K223" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L223" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M223" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N223" s="9" t="str">
+        <x:v>Airflow and exhaust must remain part of design; wind protection must not be treated as airtight enclosure.</x:v>
+      </x:c>
+      <x:c r="O223" s="17"/>
+      <x:c r="P223" s="17"/>
+      <x:c r="Q223" s="17"/>
+      <x:c r="R223" s="17"/>
+      <x:c r="S223" s="17"/>
+      <x:c r="T223" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U223" s="11"/>
+      <x:c r="V223" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+      <x:c r="W223" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X223" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y223" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z223" s="4" t="str">
+        <x:v>Fire management</x:v>
+      </x:c>
+      <x:c r="AA223" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB223" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC223" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD223" s="4" t="str">
+        <x:v>cooking wind baffle; fire management; crafting component; metal; fire management; cooking</x:v>
+      </x:c>
+      <x:c r="AE223" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="115" customHeight="1">
+      <x:c r="A224" s="9" t="str">
+        <x:v>proposal.fire.draft_collar</x:v>
+      </x:c>
+      <x:c r="B224" s="9" t="str">
+        <x:v>Cooking draft collar</x:v>
+      </x:c>
+      <x:c r="C224" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D224" s="9" t="str">
+        <x:v>Fire management</x:v>
+      </x:c>
+      <x:c r="E224" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F224" s="9" t="str">
+        <x:v>Fitted intake/draft part candidate for a compatible cooking firebox.</x:v>
+      </x:c>
+      <x:c r="G224" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H224" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I224" s="13"/>
+      <x:c r="J224" s="15"/>
+      <x:c r="K224" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L224" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M224" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N224" s="9" t="str">
+        <x:v>Proposed small-cooker adaptation of source draft engineering, not a proven design or oxygen-generating device.</x:v>
+      </x:c>
+      <x:c r="O224" s="17"/>
+      <x:c r="P224" s="17"/>
+      <x:c r="Q224" s="17"/>
+      <x:c r="R224" s="17"/>
+      <x:c r="S224" s="17"/>
+      <x:c r="T224" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U224" s="11"/>
+      <x:c r="V224" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+      <x:c r="W224" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X224" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y224" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z224" s="4" t="str">
+        <x:v>Fire management</x:v>
+      </x:c>
+      <x:c r="AA224" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB224" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC224" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD224" s="4" t="str">
+        <x:v>cooking draft collar; fire management; crafting component; ceramic; fire management; cooking</x:v>
+      </x:c>
+      <x:c r="AE224" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="115" customHeight="1">
+      <x:c r="A225" s="9" t="str">
+        <x:v>proposal.fire.heat_shroud</x:v>
+      </x:c>
+      <x:c r="B225" s="9" t="str">
+        <x:v>Cooking heat shroud</x:v>
+      </x:c>
+      <x:c r="C225" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D225" s="9" t="str">
+        <x:v>Fire management</x:v>
+      </x:c>
+      <x:c r="E225" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F225" s="9" t="str">
+        <x:v>Shaped ceramic panel candidate around a selected heat path.</x:v>
+      </x:c>
+      <x:c r="G225" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H225" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I225" s="13"/>
+      <x:c r="J225" s="15"/>
+      <x:c r="K225" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L225" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M225" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N225" s="9" t="str">
+        <x:v>Service grade, mounting and actual heat performance undefined; reuse ceramic lining craft family where possible.</x:v>
+      </x:c>
+      <x:c r="O225" s="17"/>
+      <x:c r="P225" s="17"/>
+      <x:c r="Q225" s="17"/>
+      <x:c r="R225" s="17"/>
+      <x:c r="S225" s="17"/>
+      <x:c r="T225" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U225" s="11"/>
+      <x:c r="V225" s="9" t="str">
+        <x:v>https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+      <x:c r="W225" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X225" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y225" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z225" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="AA225" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB225" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC225" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD225" s="4" t="str">
+        <x:v>cooking heat shroud; fire management; crafting component; ceramic; cooking; protective fabrication</x:v>
+      </x:c>
+      <x:c r="AE225" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="115" customHeight="1">
+      <x:c r="A226" s="9" t="str">
+        <x:v>proposal.fire.glow_holder</x:v>
+      </x:c>
+      <x:c r="B226" s="9" t="str">
+        <x:v>Shuttered glow-stone holder</x:v>
+      </x:c>
+      <x:c r="C226" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D226" s="9" t="str">
+        <x:v>Mineral light</x:v>
+      </x:c>
+      <x:c r="E226" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F226" s="9" t="str">
+        <x:v>Carrier with a movable cover for a selected glowing stone.</x:v>
+      </x:c>
+      <x:c r="G226" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H226" s="9" t="str">
+        <x:v>Carrier / placement policy TBD</x:v>
+      </x:c>
+      <x:c r="I226" s="13"/>
+      <x:c r="J226" s="15"/>
+      <x:c r="K226" s="9" t="str">
+        <x:v>Gathering, specialist craft or trade; exact acquisition TBD</x:v>
+      </x:c>
+      <x:c r="L226" s="9" t="str">
+        <x:v>No cooking, ignition or oxygen-release recipe authored</x:v>
+      </x:c>
+      <x:c r="M226" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N226" s="9" t="str">
+        <x:v>Holder is separate from its stone payload. It may expose or cover light, but does not establish charging, fuel, heat or brightness behavior.</x:v>
+      </x:c>
+      <x:c r="O226" s="17"/>
+      <x:c r="P226" s="17"/>
+      <x:c r="Q226" s="17"/>
+      <x:c r="R226" s="17"/>
+      <x:c r="S226" s="17"/>
+      <x:c r="T226" s="9" t="str">
+        <x:v>Names are descriptive working labels. Fire-dependent uses are constrained by source atmosphere proposals; no oxygen/flame simulation, nutrition bonus or automatic detoxification.</x:v>
+      </x:c>
+      <x:c r="U226" s="11"/>
+      <x:c r="V226" s="9" t="str">
+        <x:v>New game proposal from author glowing-stone direction</x:v>
+      </x:c>
+      <x:c r="W226" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X226" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y226" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z226" s="4" t="str">
+        <x:v>Illumination</x:v>
+      </x:c>
+      <x:c r="AA226" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB226" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC226" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD226" s="4" t="str">
+        <x:v>shuttered glow-stone holder; mineral light; tool; mixed / unresolved; illumination</x:v>
+      </x:c>
+      <x:c r="AE226" s="4" t="str">
+        <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17439,21 +18703,21 @@
       <x:formula1>'Taxonomy'!$B$46:$B$53</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Z6:Z1005">
-      <x:formula1>'Taxonomy'!$B$54:$B$117</x:formula1>
+      <x:formula1>'Taxonomy'!$B$54:$B$122</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AA6:AA1005">
-      <x:formula1>'Taxonomy'!$B$118:$B$146</x:formula1>
+      <x:formula1>'Taxonomy'!$B$123:$B$151</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AB6:AB1005">
-      <x:formula1>'Taxonomy'!$B$147:$B$165</x:formula1>
+      <x:formula1>'Taxonomy'!$B$152:$B$170</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AC6:AC1005">
-      <x:formula1>'Taxonomy'!$B$166:$B$170</x:formula1>
+      <x:formula1>'Taxonomy'!$B$171:$B$175</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8e23eba34944339"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81cdd21ffb674dcf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18105,7 +19369,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf81072c62a5e4aeb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98a7574a27cd45db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18587,7 +19851,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f9ad8a0a1a34d3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b2fdef3127a4026"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19166,7 +20430,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B55" s="4" t="str">
-        <x:v>Binding and construction</x:v>
+        <x:v>Atmospheric support</x:v>
       </x:c>
       <x:c r="C55" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19177,7 +20441,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B56" s="4" t="str">
-        <x:v>Camp rest</x:v>
+        <x:v>Binding and construction</x:v>
       </x:c>
       <x:c r="C56" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19188,7 +20452,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B57" s="4" t="str">
-        <x:v>Cargo organization</x:v>
+        <x:v>Camp rest</x:v>
       </x:c>
       <x:c r="C57" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19199,7 +20463,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B58" s="4" t="str">
-        <x:v>Ceremony</x:v>
+        <x:v>Cargo organization</x:v>
       </x:c>
       <x:c r="C58" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19210,7 +20474,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B59" s="4" t="str">
-        <x:v>Chemical processing</x:v>
+        <x:v>Ceremony</x:v>
       </x:c>
       <x:c r="C59" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19221,7 +20485,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B60" s="4" t="str">
-        <x:v>Civic identification</x:v>
+        <x:v>Chemical processing</x:v>
       </x:c>
       <x:c r="C60" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19232,7 +20496,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B61" s="4" t="str">
-        <x:v>Civic recognition</x:v>
+        <x:v>Civic identification</x:v>
       </x:c>
       <x:c r="C61" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19243,7 +20507,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B62" s="4" t="str">
-        <x:v>Cleaning</x:v>
+        <x:v>Civic recognition</x:v>
       </x:c>
       <x:c r="C62" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19254,7 +20518,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B63" s="4" t="str">
-        <x:v>Clothing</x:v>
+        <x:v>Cleaning</x:v>
       </x:c>
       <x:c r="C63" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19265,7 +20529,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B64" s="4" t="str">
-        <x:v>Clothing fabrication</x:v>
+        <x:v>Clothing</x:v>
       </x:c>
       <x:c r="C64" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19276,7 +20540,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B65" s="4" t="str">
-        <x:v>Culture support</x:v>
+        <x:v>Clothing fabrication</x:v>
       </x:c>
       <x:c r="C65" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19287,7 +20551,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B66" s="4" t="str">
-        <x:v>Decoration</x:v>
+        <x:v>Cooking</x:v>
       </x:c>
       <x:c r="C66" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19298,7 +20562,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B67" s="4" t="str">
-        <x:v>Devotion</x:v>
+        <x:v>Culture support</x:v>
       </x:c>
       <x:c r="C67" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19309,7 +20573,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B68" s="4" t="str">
-        <x:v>Dust exclusion</x:v>
+        <x:v>Decoration</x:v>
       </x:c>
       <x:c r="C68" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19320,7 +20584,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B69" s="4" t="str">
-        <x:v>Electrical conduction</x:v>
+        <x:v>Devotion</x:v>
       </x:c>
       <x:c r="C69" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19331,7 +20595,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B70" s="4" t="str">
-        <x:v>Electrical insulation</x:v>
+        <x:v>Dust exclusion</x:v>
       </x:c>
       <x:c r="C70" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19342,7 +20606,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B71" s="4" t="str">
-        <x:v>Electrical work</x:v>
+        <x:v>Electrical conduction</x:v>
       </x:c>
       <x:c r="C71" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19353,7 +20617,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B72" s="4" t="str">
-        <x:v>Energy processing</x:v>
+        <x:v>Electrical insulation</x:v>
       </x:c>
       <x:c r="C72" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19364,7 +20628,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B73" s="4" t="str">
-        <x:v>Energy storage</x:v>
+        <x:v>Electrical work</x:v>
       </x:c>
       <x:c r="C73" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19375,7 +20639,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B74" s="4" t="str">
-        <x:v>Equipment mounting</x:v>
+        <x:v>Energy processing</x:v>
       </x:c>
       <x:c r="C74" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19386,7 +20650,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B75" s="4" t="str">
-        <x:v>Equipment repair</x:v>
+        <x:v>Energy storage</x:v>
       </x:c>
       <x:c r="C75" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19397,7 +20661,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B76" s="4" t="str">
-        <x:v>Excavation</x:v>
+        <x:v>Equipment mounting</x:v>
       </x:c>
       <x:c r="C76" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19408,7 +20672,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B77" s="4" t="str">
-        <x:v>Fabrication</x:v>
+        <x:v>Equipment repair</x:v>
       </x:c>
       <x:c r="C77" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19419,7 +20683,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B78" s="4" t="str">
-        <x:v>Fashion</x:v>
+        <x:v>Excavation</x:v>
       </x:c>
       <x:c r="C78" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19430,7 +20694,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B79" s="4" t="str">
-        <x:v>Fauna interaction</x:v>
+        <x:v>Fabrication</x:v>
       </x:c>
       <x:c r="C79" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19441,7 +20705,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B80" s="4" t="str">
-        <x:v>Fiber processing</x:v>
+        <x:v>Fashion</x:v>
       </x:c>
       <x:c r="C80" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19452,7 +20716,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B81" s="4" t="str">
-        <x:v>Food service</x:v>
+        <x:v>Fauna interaction</x:v>
       </x:c>
       <x:c r="C81" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19463,7 +20727,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B82" s="4" t="str">
-        <x:v>Fuel</x:v>
+        <x:v>Fiber processing</x:v>
       </x:c>
       <x:c r="C82" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19474,7 +20738,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B83" s="4" t="str">
-        <x:v>Glass and ceramics</x:v>
+        <x:v>Fire management</x:v>
       </x:c>
       <x:c r="C83" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19485,7 +20749,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B84" s="4" t="str">
-        <x:v>Grooming</x:v>
+        <x:v>Food service</x:v>
       </x:c>
       <x:c r="C84" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19496,7 +20760,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B85" s="4" t="str">
-        <x:v>Injury treatment</x:v>
+        <x:v>Fuel</x:v>
       </x:c>
       <x:c r="C85" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19507,7 +20771,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B86" s="4" t="str">
-        <x:v>Inspection</x:v>
+        <x:v>Glass and ceramics</x:v>
       </x:c>
       <x:c r="C86" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19518,7 +20782,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B87" s="4" t="str">
-        <x:v>Keepsake storage</x:v>
+        <x:v>Grooming</x:v>
       </x:c>
       <x:c r="C87" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19529,7 +20793,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B88" s="4" t="str">
-        <x:v>Liquid and bulk containment</x:v>
+        <x:v>Ignition</x:v>
       </x:c>
       <x:c r="C88" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19540,7 +20804,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B89" s="4" t="str">
-        <x:v>Lubrication</x:v>
+        <x:v>Illumination</x:v>
       </x:c>
       <x:c r="C89" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19551,7 +20815,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B90" s="4" t="str">
-        <x:v>Machinery repair</x:v>
+        <x:v>Injury treatment</x:v>
       </x:c>
       <x:c r="C90" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19562,7 +20826,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B91" s="4" t="str">
-        <x:v>Magnetic tools</x:v>
+        <x:v>Inspection</x:v>
       </x:c>
       <x:c r="C91" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19573,7 +20837,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B92" s="4" t="str">
-        <x:v>Material exclusion</x:v>
+        <x:v>Keepsake storage</x:v>
       </x:c>
       <x:c r="C92" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19584,7 +20848,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B93" s="4" t="str">
-        <x:v>Material transfer</x:v>
+        <x:v>Liquid and bulk containment</x:v>
       </x:c>
       <x:c r="C93" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19595,7 +20859,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B94" s="4" t="str">
-        <x:v>Metal refining</x:v>
+        <x:v>Lubrication</x:v>
       </x:c>
       <x:c r="C94" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19606,7 +20870,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B95" s="4" t="str">
-        <x:v>Music</x:v>
+        <x:v>Machinery repair</x:v>
       </x:c>
       <x:c r="C95" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19617,7 +20881,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B96" s="4" t="str">
-        <x:v>Nutrition</x:v>
+        <x:v>Magnetic tools</x:v>
       </x:c>
       <x:c r="C96" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19628,7 +20892,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Paper making</x:v>
+        <x:v>Material exclusion</x:v>
       </x:c>
       <x:c r="C97" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19639,7 +20903,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B98" s="4" t="str">
-        <x:v>Protection</x:v>
+        <x:v>Material transfer</x:v>
       </x:c>
       <x:c r="C98" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19650,7 +20914,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B99" s="4" t="str">
-        <x:v>Protective fabrication</x:v>
+        <x:v>Metal refining</x:v>
       </x:c>
       <x:c r="C99" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19661,7 +20925,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B100" s="4" t="str">
-        <x:v>Provenance</x:v>
+        <x:v>Music</x:v>
       </x:c>
       <x:c r="C100" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19672,7 +20936,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B101" s="4" t="str">
-        <x:v>Public communication</x:v>
+        <x:v>Nutrition</x:v>
       </x:c>
       <x:c r="C101" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19683,7 +20947,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B102" s="4" t="str">
-        <x:v>Remembrance</x:v>
+        <x:v>Paper making</x:v>
       </x:c>
       <x:c r="C102" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19694,7 +20958,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B103" s="4" t="str">
-        <x:v>Resource collection</x:v>
+        <x:v>Protection</x:v>
       </x:c>
       <x:c r="C103" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19705,7 +20969,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B104" s="4" t="str">
-        <x:v>Sealing</x:v>
+        <x:v>Protective fabrication</x:v>
       </x:c>
       <x:c r="C104" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19716,7 +20980,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B105" s="4" t="str">
-        <x:v>Specialist samples</x:v>
+        <x:v>Provenance</x:v>
       </x:c>
       <x:c r="C105" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19727,7 +20991,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B106" s="4" t="str">
-        <x:v>Static management</x:v>
+        <x:v>Public communication</x:v>
       </x:c>
       <x:c r="C106" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19738,7 +21002,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B107" s="4" t="str">
-        <x:v>Sun shading</x:v>
+        <x:v>Remembrance</x:v>
       </x:c>
       <x:c r="C107" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19749,7 +21013,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B108" s="4" t="str">
-        <x:v>Surface finishing</x:v>
+        <x:v>Resource collection</x:v>
       </x:c>
       <x:c r="C108" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19760,7 +21024,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B109" s="4" t="str">
-        <x:v>Survival provision</x:v>
+        <x:v>Sealing</x:v>
       </x:c>
       <x:c r="C109" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19771,7 +21035,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B110" s="4" t="str">
-        <x:v>Textile processing</x:v>
+        <x:v>Specialist samples</x:v>
       </x:c>
       <x:c r="C110" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19782,7 +21046,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B111" s="4" t="str">
-        <x:v>Tool fabrication</x:v>
+        <x:v>Static management</x:v>
       </x:c>
       <x:c r="C111" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19793,7 +21057,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B112" s="4" t="str">
-        <x:v>Trade</x:v>
+        <x:v>Sun shading</x:v>
       </x:c>
       <x:c r="C112" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19804,7 +21068,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B113" s="4" t="str">
-        <x:v>Traversal</x:v>
+        <x:v>Surface finishing</x:v>
       </x:c>
       <x:c r="C113" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19815,7 +21079,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B114" s="4" t="str">
-        <x:v>Use unresolved</x:v>
+        <x:v>Survival provision</x:v>
       </x:c>
       <x:c r="C114" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19826,7 +21090,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B115" s="4" t="str">
-        <x:v>Vision</x:v>
+        <x:v>Textile processing</x:v>
       </x:c>
       <x:c r="C115" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19837,7 +21101,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B116" s="4" t="str">
-        <x:v>Work holding</x:v>
+        <x:v>Tool fabrication</x:v>
       </x:c>
       <x:c r="C116" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19848,7 +21112,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B117" s="4" t="str">
-        <x:v>Writing and records</x:v>
+        <x:v>Trade</x:v>
       </x:c>
       <x:c r="C117" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -19856,57 +21120,57 @@
     </x:row>
     <x:row r="118" ht="45" customHeight="1">
       <x:c r="A118" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B118" s="4" t="str">
-        <x:v>Ancient composite</x:v>
+        <x:v>Traversal</x:v>
       </x:c>
       <x:c r="C118" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="45" customHeight="1">
       <x:c r="A119" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B119" s="4" t="str">
-        <x:v>Biological chemical</x:v>
+        <x:v>Use unresolved</x:v>
       </x:c>
       <x:c r="C119" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="45" customHeight="1">
       <x:c r="A120" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B120" s="4" t="str">
-        <x:v>Carbonaceous material</x:v>
+        <x:v>Vision</x:v>
       </x:c>
       <x:c r="C120" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="45" customHeight="1">
       <x:c r="A121" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B121" s="4" t="str">
-        <x:v>Ceramic</x:v>
+        <x:v>Work holding</x:v>
       </x:c>
       <x:c r="C121" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="45" customHeight="1">
       <x:c r="A122" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B122" s="4" t="str">
-        <x:v>Ceramic and metal</x:v>
+        <x:v>Writing and records</x:v>
       </x:c>
       <x:c r="C122" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="45" customHeight="1">
@@ -19914,7 +21178,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B123" s="4" t="str">
-        <x:v>Ceramic feed mixture</x:v>
+        <x:v>Ancient composite</x:v>
       </x:c>
       <x:c r="C123" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19925,7 +21189,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B124" s="4" t="str">
-        <x:v>Faunal fiber</x:v>
+        <x:v>Biological chemical</x:v>
       </x:c>
       <x:c r="C124" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19936,7 +21200,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B125" s="4" t="str">
-        <x:v>Faunal fiber and shell</x:v>
+        <x:v>Carbonaceous material</x:v>
       </x:c>
       <x:c r="C125" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19947,7 +21211,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B126" s="4" t="str">
-        <x:v>Faunal membrane</x:v>
+        <x:v>Ceramic</x:v>
       </x:c>
       <x:c r="C126" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19958,7 +21222,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B127" s="4" t="str">
-        <x:v>Faunal tissue</x:v>
+        <x:v>Ceramic and metal</x:v>
       </x:c>
       <x:c r="C127" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19969,7 +21233,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B128" s="4" t="str">
-        <x:v>Fur</x:v>
+        <x:v>Ceramic feed mixture</x:v>
       </x:c>
       <x:c r="C128" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19980,7 +21244,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B129" s="4" t="str">
-        <x:v>Gemstone</x:v>
+        <x:v>Faunal fiber</x:v>
       </x:c>
       <x:c r="C129" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -19991,7 +21255,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B130" s="4" t="str">
-        <x:v>Glass</x:v>
+        <x:v>Faunal fiber and shell</x:v>
       </x:c>
       <x:c r="C130" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20002,7 +21266,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B131" s="4" t="str">
-        <x:v>Glass and metal</x:v>
+        <x:v>Faunal membrane</x:v>
       </x:c>
       <x:c r="C131" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20013,7 +21277,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B132" s="4" t="str">
-        <x:v>Glass and shell</x:v>
+        <x:v>Faunal tissue</x:v>
       </x:c>
       <x:c r="C132" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20024,7 +21288,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B133" s="4" t="str">
-        <x:v>Glass with unresolved casing</x:v>
+        <x:v>Fur</x:v>
       </x:c>
       <x:c r="C133" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20035,7 +21299,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B134" s="4" t="str">
-        <x:v>Hide</x:v>
+        <x:v>Gemstone</x:v>
       </x:c>
       <x:c r="C134" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20046,7 +21310,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B135" s="4" t="str">
-        <x:v>Husk fiber</x:v>
+        <x:v>Glass</x:v>
       </x:c>
       <x:c r="C135" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20057,7 +21321,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B136" s="4" t="str">
-        <x:v>Husk fiber and shell</x:v>
+        <x:v>Glass and metal</x:v>
       </x:c>
       <x:c r="C136" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20068,7 +21332,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B137" s="4" t="str">
-        <x:v>Metal</x:v>
+        <x:v>Glass and shell</x:v>
       </x:c>
       <x:c r="C137" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20079,7 +21343,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B138" s="4" t="str">
-        <x:v>Metal and shell</x:v>
+        <x:v>Glass with unresolved casing</x:v>
       </x:c>
       <x:c r="C138" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20090,7 +21354,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B139" s="4" t="str">
-        <x:v>Metal or shell</x:v>
+        <x:v>Hide</x:v>
       </x:c>
       <x:c r="C139" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20101,7 +21365,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B140" s="4" t="str">
-        <x:v>Mineral</x:v>
+        <x:v>Husk fiber</x:v>
       </x:c>
       <x:c r="C140" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20112,7 +21376,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B141" s="4" t="str">
-        <x:v>Mineral or shell</x:v>
+        <x:v>Husk fiber and shell</x:v>
       </x:c>
       <x:c r="C141" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20123,7 +21387,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B142" s="4" t="str">
-        <x:v>Mixed / unresolved</x:v>
+        <x:v>Metal</x:v>
       </x:c>
       <x:c r="C142" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20134,7 +21398,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B143" s="4" t="str">
-        <x:v>Shell / chitin</x:v>
+        <x:v>Metal and shell</x:v>
       </x:c>
       <x:c r="C143" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20145,7 +21409,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B144" s="4" t="str">
-        <x:v>Shell and mineral</x:v>
+        <x:v>Metal or shell</x:v>
       </x:c>
       <x:c r="C144" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20156,7 +21420,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B145" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Mineral</x:v>
       </x:c>
       <x:c r="C145" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20167,7 +21431,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B146" s="4" t="str">
-        <x:v>Wing membrane</x:v>
+        <x:v>Mineral or shell</x:v>
       </x:c>
       <x:c r="C146" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -20175,57 +21439,57 @@
     </x:row>
     <x:row r="147" ht="45" customHeight="1">
       <x:c r="A147" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B147" s="4" t="str">
-        <x:v>Assembly</x:v>
+        <x:v>Mixed / unresolved</x:v>
       </x:c>
       <x:c r="C147" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="148" ht="45" customHeight="1">
       <x:c r="A148" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B148" s="4" t="str">
-        <x:v>Bundle</x:v>
+        <x:v>Shell / chitin</x:v>
       </x:c>
       <x:c r="C148" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="149" ht="45" customHeight="1">
       <x:c r="A149" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B149" s="4" t="str">
-        <x:v>Cord</x:v>
+        <x:v>Shell and mineral</x:v>
       </x:c>
       <x:c r="C149" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="45" customHeight="1">
       <x:c r="A150" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B150" s="4" t="str">
-        <x:v>Fiber</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C150" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="151" ht="45" customHeight="1">
       <x:c r="A151" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B151" s="4" t="str">
-        <x:v>Folio</x:v>
+        <x:v>Wing membrane</x:v>
       </x:c>
       <x:c r="C151" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="152" ht="45" customHeight="1">
@@ -20233,7 +21497,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B152" s="4" t="str">
-        <x:v>Garment</x:v>
+        <x:v>Assembly</x:v>
       </x:c>
       <x:c r="C152" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20244,7 +21508,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B153" s="4" t="str">
-        <x:v>Gel</x:v>
+        <x:v>Bundle</x:v>
       </x:c>
       <x:c r="C153" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20255,7 +21519,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B154" s="4" t="str">
-        <x:v>Liquid</x:v>
+        <x:v>Cord</x:v>
       </x:c>
       <x:c r="C154" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20266,7 +21530,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B155" s="4" t="str">
-        <x:v>Membrane</x:v>
+        <x:v>Fiber</x:v>
       </x:c>
       <x:c r="C155" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20277,7 +21541,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B156" s="4" t="str">
-        <x:v>Panel</x:v>
+        <x:v>Folio</x:v>
       </x:c>
       <x:c r="C156" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20288,7 +21552,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B157" s="4" t="str">
-        <x:v>Particles</x:v>
+        <x:v>Garment</x:v>
       </x:c>
       <x:c r="C157" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20299,7 +21563,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B158" s="4" t="str">
-        <x:v>Patch</x:v>
+        <x:v>Gel</x:v>
       </x:c>
       <x:c r="C158" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20310,7 +21574,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B159" s="4" t="str">
-        <x:v>Rock</x:v>
+        <x:v>Liquid</x:v>
       </x:c>
       <x:c r="C159" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20321,7 +21585,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B160" s="4" t="str">
-        <x:v>Sheet</x:v>
+        <x:v>Membrane</x:v>
       </x:c>
       <x:c r="C160" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20332,7 +21596,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B161" s="4" t="str">
-        <x:v>Shell plate</x:v>
+        <x:v>Panel</x:v>
       </x:c>
       <x:c r="C161" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20343,7 +21607,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B162" s="4" t="str">
-        <x:v>Solid part</x:v>
+        <x:v>Particles</x:v>
       </x:c>
       <x:c r="C162" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20354,7 +21618,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B163" s="4" t="str">
-        <x:v>Solid piece</x:v>
+        <x:v>Patch</x:v>
       </x:c>
       <x:c r="C163" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20365,7 +21629,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B164" s="4" t="str">
-        <x:v>Strip</x:v>
+        <x:v>Rock</x:v>
       </x:c>
       <x:c r="C164" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20376,7 +21640,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B165" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Sheet</x:v>
       </x:c>
       <x:c r="C165" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -20384,63 +21648,118 @@
     </x:row>
     <x:row r="166" ht="45" customHeight="1">
       <x:c r="A166" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B166" s="4" t="str">
-        <x:v>Author direction</x:v>
+        <x:v>Shell plate</x:v>
       </x:c>
       <x:c r="C166" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="167" ht="45" customHeight="1">
       <x:c r="A167" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B167" s="4" t="str">
-        <x:v>Existing definition</x:v>
+        <x:v>Solid part</x:v>
       </x:c>
       <x:c r="C167" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="168" ht="45" customHeight="1">
       <x:c r="A168" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B168" s="4" t="str">
-        <x:v>Proposal</x:v>
+        <x:v>Solid piece</x:v>
       </x:c>
       <x:c r="C168" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="169" ht="45" customHeight="1">
       <x:c r="A169" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B169" s="4" t="str">
-        <x:v>Source proposal</x:v>
+        <x:v>Strip</x:v>
       </x:c>
       <x:c r="C169" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="170" ht="45" customHeight="1">
       <x:c r="A170" s="4" t="str">
+        <x:v>Physical form</x:v>
+      </x:c>
+      <x:c r="B170" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="C170" s="4" t="str">
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="45" customHeight="1">
+      <x:c r="A171" s="4" t="str">
         <x:v>Design status</x:v>
       </x:c>
-      <x:c r="B170" s="4" t="str">
+      <x:c r="B171" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="C171" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="45" customHeight="1">
+      <x:c r="A172" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B172" s="4" t="str">
+        <x:v>Existing definition</x:v>
+      </x:c>
+      <x:c r="C172" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="45" customHeight="1">
+      <x:c r="A173" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B173" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="C173" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="45" customHeight="1">
+      <x:c r="A174" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B174" s="4" t="str">
+        <x:v>Source proposal</x:v>
+      </x:c>
+      <x:c r="C174" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="45" customHeight="1">
+      <x:c r="A175" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B175" s="4" t="str">
         <x:v>Withheld assumption</x:v>
       </x:c>
-      <x:c r="C170" s="4" t="str">
+      <x:c r="C175" s="4" t="str">
         <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49d646966f6e4f5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a7117340824833"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26830,21 +28149,499 @@
         <x:v>WLD-0032 currency proposal. Unit/denomination and physical form unresolved.</x:v>
       </x:c>
     </x:row>
+    <x:row r="285" ht="65" customHeight="1">
+      <x:c r="A285" s="4" t="str">
+        <x:v>proposal.fire.oxygen_stone</x:v>
+      </x:c>
+      <x:c r="B285" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A285,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Oxygen-releasing stone</x:v>
+      </x:c>
+      <x:c r="C285" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A285,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D285" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E285" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A285,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Atmospheric support</x:v>
+      </x:c>
+      <x:c r="F285" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="286" ht="65" customHeight="1">
+      <x:c r="A286" s="4" t="str">
+        <x:v>proposal.fire.glow_stone</x:v>
+      </x:c>
+      <x:c r="B286" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A286,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Glowing stone</x:v>
+      </x:c>
+      <x:c r="C286" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A286,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D286" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E286" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A286,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Illumination</x:v>
+      </x:c>
+      <x:c r="F286" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="287" ht="65" customHeight="1">
+      <x:c r="A287" s="4" t="str">
+        <x:v>proposal.fire.flint</x:v>
+      </x:c>
+      <x:c r="B287" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A287,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Flint stone</x:v>
+      </x:c>
+      <x:c r="C287" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A287,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D287" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E287" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A287,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ignition</x:v>
+      </x:c>
+      <x:c r="F287" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="288" ht="65" customHeight="1">
+      <x:c r="A288" s="4" t="str">
+        <x:v>proposal.fire.flint</x:v>
+      </x:c>
+      <x:c r="B288" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A288,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Flint stone</x:v>
+      </x:c>
+      <x:c r="C288" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A288,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D288" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E288" s="4" t="str">
+        <x:v>Tool fabrication</x:v>
+      </x:c>
+      <x:c r="F288" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="289" ht="65" customHeight="1">
+      <x:c r="A289" s="4" t="str">
+        <x:v>proposal.fire.striker</x:v>
+      </x:c>
+      <x:c r="B289" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A289,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Flint striking tool</x:v>
+      </x:c>
+      <x:c r="C289" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A289,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D289" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E289" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A289,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ignition</x:v>
+      </x:c>
+      <x:c r="F289" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="290" ht="65" customHeight="1">
+      <x:c r="A290" s="4" t="str">
+        <x:v>proposal.fire.chitin_char</x:v>
+      </x:c>
+      <x:c r="B290" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A290,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chitin-char</x:v>
+      </x:c>
+      <x:c r="C290" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A290,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D290" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E290" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A290,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Fuel</x:v>
+      </x:c>
+      <x:c r="F290" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="291" ht="65" customHeight="1">
+      <x:c r="A291" s="4" t="str">
+        <x:v>proposal.fire.cooking_pot</x:v>
+      </x:c>
+      <x:c r="B291" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A291,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic cooking pot</x:v>
+      </x:c>
+      <x:c r="C291" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A291,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D291" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E291" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A291,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F291" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="292" ht="65" customHeight="1">
+      <x:c r="A292" s="4" t="str">
+        <x:v>proposal.fire.cooking_slab</x:v>
+      </x:c>
+      <x:c r="B292" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A292,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking stone slab</x:v>
+      </x:c>
+      <x:c r="C292" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A292,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D292" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E292" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A292,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F292" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="293" ht="65" customHeight="1">
+      <x:c r="A293" s="4" t="str">
+        <x:v>proposal.fire.lidded_pan</x:v>
+      </x:c>
+      <x:c r="B293" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A293,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lidded cooking pan</x:v>
+      </x:c>
+      <x:c r="C293" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A293,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D293" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E293" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A293,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F293" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="294" ht="65" customHeight="1">
+      <x:c r="A294" s="4" t="str">
+        <x:v>proposal.fire.rack</x:v>
+      </x:c>
+      <x:c r="B294" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A294,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking rack</x:v>
+      </x:c>
+      <x:c r="C294" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A294,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D294" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E294" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A294,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F294" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="295" ht="65" customHeight="1">
+      <x:c r="A295" s="4" t="str">
+        <x:v>proposal.fire.pot_stand</x:v>
+      </x:c>
+      <x:c r="B295" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A295,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking pot stand</x:v>
+      </x:c>
+      <x:c r="C295" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A295,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D295" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E295" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A295,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F295" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="296" ht="65" customHeight="1">
+      <x:c r="A296" s="4" t="str">
+        <x:v>proposal.fire.tongs</x:v>
+      </x:c>
+      <x:c r="B296" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A296,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking tongs</x:v>
+      </x:c>
+      <x:c r="C296" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A296,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D296" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E296" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A296,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F296" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="297" ht="65" customHeight="1">
+      <x:c r="A297" s="4" t="str">
+        <x:v>proposal.fire.firebox</x:v>
+      </x:c>
+      <x:c r="B297" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A297,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Managed cooking firebox</x:v>
+      </x:c>
+      <x:c r="C297" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A297,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D297" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E297" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A297,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F297" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="298" ht="65" customHeight="1">
+      <x:c r="A298" s="4" t="str">
+        <x:v>proposal.fire.firebox</x:v>
+      </x:c>
+      <x:c r="B298" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A298,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Managed cooking firebox</x:v>
+      </x:c>
+      <x:c r="C298" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A298,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D298" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E298" s="4" t="str">
+        <x:v>Fire management</x:v>
+      </x:c>
+      <x:c r="F298" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="299" ht="65" customHeight="1">
+      <x:c r="A299" s="4" t="str">
+        <x:v>proposal.fire.wind_baffle</x:v>
+      </x:c>
+      <x:c r="B299" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A299,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking wind baffle</x:v>
+      </x:c>
+      <x:c r="C299" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A299,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D299" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E299" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A299,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Fire management</x:v>
+      </x:c>
+      <x:c r="F299" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="300" ht="65" customHeight="1">
+      <x:c r="A300" s="4" t="str">
+        <x:v>proposal.fire.wind_baffle</x:v>
+      </x:c>
+      <x:c r="B300" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A300,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking wind baffle</x:v>
+      </x:c>
+      <x:c r="C300" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A300,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D300" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E300" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F300" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="301" ht="65" customHeight="1">
+      <x:c r="A301" s="4" t="str">
+        <x:v>proposal.fire.draft_collar</x:v>
+      </x:c>
+      <x:c r="B301" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A301,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking draft collar</x:v>
+      </x:c>
+      <x:c r="C301" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A301,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D301" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E301" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A301,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Fire management</x:v>
+      </x:c>
+      <x:c r="F301" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="302" ht="65" customHeight="1">
+      <x:c r="A302" s="4" t="str">
+        <x:v>proposal.fire.draft_collar</x:v>
+      </x:c>
+      <x:c r="B302" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A302,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking draft collar</x:v>
+      </x:c>
+      <x:c r="C302" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A302,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D302" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E302" s="4" t="str">
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F302" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="303" ht="65" customHeight="1">
+      <x:c r="A303" s="4" t="str">
+        <x:v>proposal.fire.heat_shroud</x:v>
+      </x:c>
+      <x:c r="B303" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A303,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking heat shroud</x:v>
+      </x:c>
+      <x:c r="C303" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A303,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D303" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E303" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A303,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking</x:v>
+      </x:c>
+      <x:c r="F303" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="304" ht="65" customHeight="1">
+      <x:c r="A304" s="4" t="str">
+        <x:v>proposal.fire.heat_shroud</x:v>
+      </x:c>
+      <x:c r="B304" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A304,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cooking heat shroud</x:v>
+      </x:c>
+      <x:c r="C304" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A304,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D304" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E304" s="4" t="str">
+        <x:v>Protective fabrication</x:v>
+      </x:c>
+      <x:c r="F304" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="305" ht="65" customHeight="1">
+      <x:c r="A305" s="4" t="str">
+        <x:v>proposal.fire.glow_holder</x:v>
+      </x:c>
+      <x:c r="B305" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A305,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Shuttered glow-stone holder</x:v>
+      </x:c>
+      <x:c r="C305" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A305,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D305" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E305" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A305,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Illumination</x:v>
+      </x:c>
+      <x:c r="F305" s="4" t="str">
+        <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A6:A1005">
-      <x:formula1>'Items'!$A$6:$A$210</x:formula1>
+      <x:formula1>'Items'!$A$6:$A$226</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D6:D1005">
       <x:formula1>"Primary,Secondary"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E6:E1005">
-      <x:formula1>'Taxonomy'!$B$54:$B$117</x:formula1>
+      <x:formula1>'Taxonomy'!$B$54:$B$122</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a17e7aa52c4348"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4ac972e757149b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27752,7 +29549,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc183ef2e2fa34cd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c693b60662d4bd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28118,7 +29915,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5211754261c14b1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd26ab7ba87ab4d03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28179,7 +29976,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>34</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>Existing gear plus armor, carriers, rare eyewear/headwear and very rare fashion families</x:v>
@@ -28209,7 +30006,7 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>80</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Minerals, biological resources, generic chemistry placeholders and twelve new chemical concepts</x:v>
@@ -28224,7 +30021,7 @@
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A9)</x:f>
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>Existing salvage and proposed materials, including husk-fiber paper and difficult pressed textiles</x:v>
@@ -28548,7 +30345,7 @@
       </x:c>
       <x:c r="B31" s="3" t="n">
         <x:f>COUNTIF(Items!$AA$6:$AA$1005,"Ceramic")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic feed mixture")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic and metal")</x:f>
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
         <x:v>28 new ceramic-specific feeds, intermediate blanks, tableware, storage, workshop tools, thermal/electrical parts, vessel fittings, ceremonial work and protection candidates</x:v>
@@ -28572,10 +30369,25 @@
         <x:v>WLD-0032 draft/proposal names the currency but does not define denominations, physical tokens or exchange ratios.</x:v>
       </x:c>
     </x:row>
+    <x:row r="33" ht="110" customHeight="1">
+      <x:c r="A33" s="3" t="str">
+        <x:v>Special stones, fire and cooking</x:v>
+      </x:c>
+      <x:c r="B33" s="3" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Special stone")+COUNTIF(Items!$D$6:$D$1005,"Ignition tool")+COUNTIF(Items!$D$6:$D$1005,"Fire fuel")+COUNTIF(Items!$D$6:$D$1005,"Cooking vessel")+COUNTIF(Items!$D$6:$D$1005,"Cooking tool")+COUNTIF(Items!$D$6:$D$1005,"Fire management")+COUNTIF(Items!$D$6:$D$1005,"Mineral light")</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C33" s="3" t="str">
+        <x:v>Oxygen-releasing rock, glow stone, flint, ignition, chitin-char, food-heating vessels/tools and managed-fire parts</x:v>
+      </x:c>
+      <x:c r="D33" s="3" t="str">
+        <x:v>Source fire behavior is proposal-stage. Extracted-stone behavior, fuel/air supply, cooking effects and equipment performance unresolved.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb57bcde49740455f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R338f2205ffdf4a9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28638,7 +30450,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>205 design entries: 18 existing item IDs and 187 design/source concepts. Currency-family entry added from WLD-0032; denominations unresolved.</x:v>
+        <x:v>221 design entries: 18 existing item IDs and 203 design/source concepts. Sixteen special-stone, fuel, cooking and fire-management entries added.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -29350,7 +31162,7 @@
         <x:v>Filtering the master</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Items is one native filterable table, A5:AE210. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
+        <x:v>Items is one native filterable table, A5:AE226. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="85" customHeight="1">
@@ -29465,10 +31277,74 @@
         <x:v>The source discusses above-baseline craft, expertise and prestige purchases, non-commodity backing, and survival outside monetary exchange. These remain source proposals; the currency entry does not change the game survival economy, wallet, loot or inventory behavior.</x:v>
       </x:c>
     </x:row>
+    <x:row r="112" ht="105" customHeight="1">
+      <x:c r="A112" s="4" t="str">
+        <x:v>Fire source</x:v>
+      </x:c>
+      <x:c r="B112" s="4" t="str">
+        <x:v>WLD-0083 Atmosphere of the Broken World, draft/proposal at revision f6f98515, describes weaker, slower, dimmer/smokier and more easily extinguished ordinary fires in oxygen-poor air. Cooking and sustained industrial heat need deliberate engineering. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/geography/atmosphere.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="105" customHeight="1">
+      <x:c r="A113" s="4" t="str">
+        <x:v>Fire varies by place</x:v>
+      </x:c>
+      <x:c r="B113" s="4" t="str">
+        <x:v>Source geology describes greater oxygen output deeper in canyons, low oxygen at the open surface, and hydrogen concentration toward upper zones. The record proposes stronger ignition behavior in hydrogen-rich areas. This is source world design, not a quantitative combustion model.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="105" customHeight="1">
+      <x:c r="A114" s="4" t="str">
+        <x:v>Enclosed fire</x:v>
+      </x:c>
+      <x:c r="B114" s="4" t="str">
+        <x:v>The source describes oxygen consumption and dangerous gas accumulation in enclosed spaces. No firebox, wind screen, ordinary canister or oxygen stone automatically makes an enclosed camp safe. Source flame-test folklore is not adopted as a reliable detector or implemented action.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="105" customHeight="1">
+      <x:c r="A115" s="4" t="str">
+        <x:v>Oxygen stone boundary</x:v>
+      </x:c>
+      <x:c r="B115" s="4" t="str">
+        <x:v>Author confirms oxygen-releasing stone families. Source geology relies on sustained geothermal heat/pressure and recharge within formations. Output of detached pieces, activation, rate, depletion, recharge, storage and portable usefulness remain undecided.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="105" customHeight="1">
+      <x:c r="A116" s="4" t="str">
+        <x:v>Glow and flint</x:v>
+      </x:c>
+      <x:c r="B116" s="4" t="str">
+        <x:v>Glowing stone and flint are author-directed resources. No named glow-stone owning record was located in the inspected material/atmosphere neighborhood. Light need not imply flame or heat; charging and lifetime TBD. Flint has candidate sparking/tool uses but no guaranteed ignition.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="105" customHeight="1">
+      <x:c r="A117" s="4" t="str">
+        <x:v>Cooking and survival</x:v>
+      </x:c>
+      <x:c r="B117" s="4" t="str">
+        <x:v>Heating food is a use category, not automatic nutrition improvement or detoxification. Some fauna remains poor food and much internal chemistry is toxic. Reuse eating bowls for serving; cooking pots/pans are heat-service concepts. Recipes and food effects remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="105" customHeight="1">
+      <x:c r="A118" s="4" t="str">
+        <x:v>Fuel and furnace distinction</x:v>
+      </x:c>
+      <x:c r="B118" s="4" t="str">
+        <x:v>Chitin source WLD-0063 describes chitin-char, a plant-free carbonized material. Reconcile with generic Charcoal before runtime implementation. Source furnace craft uses specific fuels, draft and furnace designs; no ordinary campfire grants metallurgy capability. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chitin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="105" customHeight="1">
+      <x:c r="A119" s="4" t="str">
+        <x:v>Source water-vapor conflict</x:v>
+      </x:c>
+      <x:c r="B119" s="4" t="str">
+        <x:v>WLD-0083 proposes trace humidity from hydrogen combustion, alongside other source food/water language. The game no-free-water rule remains controlling. No collectable water, condensation recipe or water supply is added by this task.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7a41cf74834ccd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ccab4361ab44aed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30312,7 +32188,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553e1e47f82b4ef1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcced88e419214fee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30555,7 +32431,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5049846909a4947"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b76f65595004b5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30959,7 +32835,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R251c5f10292541e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba8f04fa49854165"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31635,7 +33511,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R484393edd28440f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a939e103f914243"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: develop faunal lubricant processing and item concepts
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="Rafec7c372fa94a2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Radae3cc1878f4246"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R897e4ff09bff433b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rd27023370c4d4730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R5e53ab5e151b404d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rae5b84966dcc4436"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rf51acec02207439d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Re7f89e76855c4244"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Rccae3676c6874cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R347f758c74f0480f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R8d281f37a6874e1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R33b2bde451f4439f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="Rfce68271b1014adc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R9303566c63ba4a1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rf336aa35dc404d4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rfe9a96ddb92b4918"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rb76f65d1ca5e4a56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rd3ced0d9f93c4fc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rdb7e5429b9324151"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rf1c2911a84884c77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Rf918468f81744fdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R9daaadfb56ee4945"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="Ra64bf09f63984375"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R2a57572d4e3e43ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="Rb4f190fdcd8a459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="R03663e600a6947ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,8 +476,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE226" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AE226"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE234" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AE234"/>
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -550,7 +550,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C175" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C177" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Field"/>
     <x:tableColumn id="2" name="Allowed value"/>
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F305" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F305"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F321" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F321"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -614,7 +614,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -626,7 +626,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B126" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -986,7 +986,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>221 entries. Filter W:AC for classifications; search AD. Cooking and fire uses retain source/author distinctions.</x:v>
+        <x:v>229 entries. Filter W:AC for classifications; search AD. Lubricants include proposed base fractions, grease, oil and film grades.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -18674,6 +18674,638 @@
       </x:c>
       <x:c r="AE226" s="4" t="str">
         <x:v>Author direction establishes stone families. Source mechanisms remain proposal-stage; specific equipment functions are proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="115" customHeight="1">
+      <x:c r="A227" s="9" t="str">
+        <x:v>proposal.lubricant.base</x:v>
+      </x:c>
+      <x:c r="B227" s="9" t="str">
+        <x:v>Clarified faunal lubricant base</x:v>
+      </x:c>
+      <x:c r="C227" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D227" s="9" t="str">
+        <x:v>Lubricant intermediate</x:v>
+      </x:c>
+      <x:c r="E227" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F227" s="9" t="str">
+        <x:v>Select a candidate lubricating liquid fraction from existing joint secretion or a suitable species-specific metabolic fluid.</x:v>
+      </x:c>
+      <x:c r="G227" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H227" s="9" t="str">
+        <x:v>Contained chemical cargo; carrier policy TBD</x:v>
+      </x:c>
+      <x:c r="I227" s="13"/>
+      <x:c r="J227" s="15"/>
+      <x:c r="K227" s="9" t="str">
+        <x:v>Process existing faunal secretions in a specialist workshop; exact species and route TBD</x:v>
+      </x:c>
+      <x:c r="L227" s="9" t="str">
+        <x:v>Proposed stages: segregated collection, separation, selected-fraction preparation, compatible formulation, service-specific testing. No formula or numeric yield.</x:v>
+      </x:c>
+      <x:c r="M227" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N227" s="9" t="str">
+        <x:v>Separate grit, hard-clotting fractions and unwanted chemistry; exact apparatus, stabilization, yield and residual toxicity unresolved.</x:v>
+      </x:c>
+      <x:c r="O227" s="17"/>
+      <x:c r="P227" s="17"/>
+      <x:c r="Q227" s="17"/>
+      <x:c r="R227" s="17"/>
+      <x:c r="S227" s="17"/>
+      <x:c r="T227" s="9" t="str">
+        <x:v>Toxic industrial chemistry remains separate from food. Quality, batch consistency and specialist refinement may drive value; no price, spoilage or maintenance timer assigned.</x:v>
+      </x:c>
+      <x:c r="U227" s="11"/>
+      <x:c r="V227" s="9" t="str">
+        <x:v>New game proposal. Source WLD-0061 processing-agent record describes metabolic oil for machinery; source draft/proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+      <x:c r="W227" s="4" t="str">
+        <x:v>Chemical material</x:v>
+      </x:c>
+      <x:c r="X227" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y227" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z227" s="4" t="str">
+        <x:v>Chemical processing</x:v>
+      </x:c>
+      <x:c r="AA227" s="4" t="str">
+        <x:v>Biological chemical</x:v>
+      </x:c>
+      <x:c r="AB227" s="4" t="str">
+        <x:v>Liquid</x:v>
+      </x:c>
+      <x:c r="AC227" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD227" s="4" t="str">
+        <x:v>clarified faunal lubricant base; grease; lubricant; fauna chemistry; lubrication; chemical processing</x:v>
+      </x:c>
+      <x:c r="AE227" s="4" t="str">
+        <x:v>Specific formulation is proposed; source oils and existing joint secretion are references, not validated recipes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="115" customHeight="1">
+      <x:c r="A228" s="9" t="str">
+        <x:v>proposal.lubricant.thickener</x:v>
+      </x:c>
+      <x:c r="B228" s="9" t="str">
+        <x:v>Prepared secretion thickener</x:v>
+      </x:c>
+      <x:c r="C228" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D228" s="9" t="str">
+        <x:v>Lubricant intermediate</x:v>
+      </x:c>
+      <x:c r="E228" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F228" s="9" t="str">
+        <x:v>Selected biological fraction proposed to give a compatible lubricant body and retention.</x:v>
+      </x:c>
+      <x:c r="G228" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H228" s="9" t="str">
+        <x:v>Contained chemical cargo; carrier policy TBD</x:v>
+      </x:c>
+      <x:c r="I228" s="13"/>
+      <x:c r="J228" s="15"/>
+      <x:c r="K228" s="9" t="str">
+        <x:v>Process existing faunal secretions in a specialist workshop; exact species and route TBD</x:v>
+      </x:c>
+      <x:c r="L228" s="9" t="str">
+        <x:v>Proposed stages: segregated collection, separation, selected-fraction preparation, compatible formulation, service-specific testing. No formula or numeric yield.</x:v>
+      </x:c>
+      <x:c r="M228" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N228" s="9" t="str">
+        <x:v>New research candidate, not automatic use of shell glue, husk enzymes, wax or conventional animal fat. It must remain workable rather than cure hard.</x:v>
+      </x:c>
+      <x:c r="O228" s="17"/>
+      <x:c r="P228" s="17"/>
+      <x:c r="Q228" s="17"/>
+      <x:c r="R228" s="17"/>
+      <x:c r="S228" s="17"/>
+      <x:c r="T228" s="9" t="str">
+        <x:v>Toxic industrial chemistry remains separate from food. Quality, batch consistency and specialist refinement may drive value; no price, spoilage or maintenance timer assigned.</x:v>
+      </x:c>
+      <x:c r="U228" s="11"/>
+      <x:c r="V228" s="9" t="str">
+        <x:v>New game proposal. Source WLD-0061 processing-agent record describes metabolic oil for machinery; source draft/proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+      <x:c r="W228" s="4" t="str">
+        <x:v>Chemical material</x:v>
+      </x:c>
+      <x:c r="X228" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y228" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z228" s="4" t="str">
+        <x:v>Chemical processing</x:v>
+      </x:c>
+      <x:c r="AA228" s="4" t="str">
+        <x:v>Biological chemical</x:v>
+      </x:c>
+      <x:c r="AB228" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AC228" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD228" s="4" t="str">
+        <x:v>prepared secretion thickener; grease; lubricant; fauna chemistry; lubrication; chemical processing</x:v>
+      </x:c>
+      <x:c r="AE228" s="4" t="str">
+        <x:v>Specific formulation is proposed; source oils and existing joint secretion are references, not validated recipes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="115" customHeight="1">
+      <x:c r="A229" s="9" t="str">
+        <x:v>proposal.lubricant.joint_grease</x:v>
+      </x:c>
+      <x:c r="B229" s="9" t="str">
+        <x:v>Faunal joint grease</x:v>
+      </x:c>
+      <x:c r="C229" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D229" s="9" t="str">
+        <x:v>Finished lubricant</x:v>
+      </x:c>
+      <x:c r="E229" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F229" s="9" t="str">
+        <x:v>Lubricant base plus a compatible prepared thickener, proposed for slow mechanical pivots and heavy joints.</x:v>
+      </x:c>
+      <x:c r="G229" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H229" s="9" t="str">
+        <x:v>Contained chemical cargo; carrier policy TBD</x:v>
+      </x:c>
+      <x:c r="I229" s="13"/>
+      <x:c r="J229" s="15"/>
+      <x:c r="K229" s="9" t="str">
+        <x:v>Process existing faunal secretions in a specialist workshop; exact species and route TBD</x:v>
+      </x:c>
+      <x:c r="L229" s="9" t="str">
+        <x:v>Proposed stages: segregated collection, separation, selected-fraction preparation, compatible formulation, service-specific testing. No formula or numeric yield.</x:v>
+      </x:c>
+      <x:c r="M229" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N229" s="9" t="str">
+        <x:v>Application, consistency, seal fit and service interval TBD. Raw secretion is not ready-to-use universal grease.</x:v>
+      </x:c>
+      <x:c r="O229" s="17"/>
+      <x:c r="P229" s="17"/>
+      <x:c r="Q229" s="17"/>
+      <x:c r="R229" s="17"/>
+      <x:c r="S229" s="17"/>
+      <x:c r="T229" s="9" t="str">
+        <x:v>Toxic industrial chemistry remains separate from food. Quality, batch consistency and specialist refinement may drive value; no price, spoilage or maintenance timer assigned.</x:v>
+      </x:c>
+      <x:c r="U229" s="11"/>
+      <x:c r="V229" s="9" t="str">
+        <x:v>New game proposal. Source WLD-0061 processing-agent record describes metabolic oil for machinery; source draft/proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+      <x:c r="W229" s="4" t="str">
+        <x:v>Chemical material</x:v>
+      </x:c>
+      <x:c r="X229" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y229" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z229" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="AA229" s="4" t="str">
+        <x:v>Biological chemical</x:v>
+      </x:c>
+      <x:c r="AB229" s="4" t="str">
+        <x:v>Paste</x:v>
+      </x:c>
+      <x:c r="AC229" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD229" s="4" t="str">
+        <x:v>faunal joint grease; grease; lubricant; fauna chemistry; equipment repair; lubrication</x:v>
+      </x:c>
+      <x:c r="AE229" s="4" t="str">
+        <x:v>Specific formulation is proposed; source oils and existing joint secretion are references, not validated recipes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230" ht="115" customHeight="1">
+      <x:c r="A230" s="9" t="str">
+        <x:v>proposal.lubricant.dust_film</x:v>
+      </x:c>
+      <x:c r="B230" s="9" t="str">
+        <x:v>Dust-shedding lubricant film</x:v>
+      </x:c>
+      <x:c r="C230" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D230" s="9" t="str">
+        <x:v>Finished lubricant</x:v>
+      </x:c>
+      <x:c r="E230" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F230" s="9" t="str">
+        <x:v>Candidate thin-film finish for exposed tool slides and guides in dusty terrain.</x:v>
+      </x:c>
+      <x:c r="G230" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H230" s="9" t="str">
+        <x:v>Contained chemical cargo; carrier policy TBD</x:v>
+      </x:c>
+      <x:c r="I230" s="13"/>
+      <x:c r="J230" s="15"/>
+      <x:c r="K230" s="9" t="str">
+        <x:v>Process existing faunal secretions in a specialist workshop; exact species and route TBD</x:v>
+      </x:c>
+      <x:c r="L230" s="9" t="str">
+        <x:v>Proposed stages: segregated collection, separation, selected-fraction preparation, compatible formulation, service-specific testing. No formula or numeric yield.</x:v>
+      </x:c>
+      <x:c r="M230" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N230" s="9" t="str">
+        <x:v>Design goal: avoid a persistent sticky exposed coating. Film formation, dust behavior and reapplication remain unverified.</x:v>
+      </x:c>
+      <x:c r="O230" s="17"/>
+      <x:c r="P230" s="17"/>
+      <x:c r="Q230" s="17"/>
+      <x:c r="R230" s="17"/>
+      <x:c r="S230" s="17"/>
+      <x:c r="T230" s="9" t="str">
+        <x:v>Toxic industrial chemistry remains separate from food. Quality, batch consistency and specialist refinement may drive value; no price, spoilage or maintenance timer assigned.</x:v>
+      </x:c>
+      <x:c r="U230" s="11"/>
+      <x:c r="V230" s="9" t="str">
+        <x:v>New game proposal. Source WLD-0061 processing-agent record describes metabolic oil for machinery; source draft/proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+      <x:c r="W230" s="4" t="str">
+        <x:v>Chemical material</x:v>
+      </x:c>
+      <x:c r="X230" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y230" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z230" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="AA230" s="4" t="str">
+        <x:v>Biological chemical</x:v>
+      </x:c>
+      <x:c r="AB230" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AC230" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD230" s="4" t="str">
+        <x:v>dust-shedding lubricant film; grease; lubricant; fauna chemistry; dust exclusion; lubrication</x:v>
+      </x:c>
+      <x:c r="AE230" s="4" t="str">
+        <x:v>Specific formulation is proposed; source oils and existing joint secretion are references, not validated recipes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231" ht="115" customHeight="1">
+      <x:c r="A231" s="9" t="str">
+        <x:v>proposal.lubricant.seal_paste</x:v>
+      </x:c>
+      <x:c r="B231" s="9" t="str">
+        <x:v>Seal-conditioning paste</x:v>
+      </x:c>
+      <x:c r="C231" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D231" s="9" t="str">
+        <x:v>Finished lubricant</x:v>
+      </x:c>
+      <x:c r="E231" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F231" s="9" t="str">
+        <x:v>Candidate small-dose conditioner for a specifically compatible canister seal material.</x:v>
+      </x:c>
+      <x:c r="G231" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H231" s="9" t="str">
+        <x:v>Contained chemical cargo; carrier policy TBD</x:v>
+      </x:c>
+      <x:c r="I231" s="13"/>
+      <x:c r="J231" s="15"/>
+      <x:c r="K231" s="9" t="str">
+        <x:v>Process existing faunal secretions in a specialist workshop; exact species and route TBD</x:v>
+      </x:c>
+      <x:c r="L231" s="9" t="str">
+        <x:v>Proposed stages: segregated collection, separation, selected-fraction preparation, compatible formulation, service-specific testing. No formula or numeric yield.</x:v>
+      </x:c>
+      <x:c r="M231" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N231" s="9" t="str">
+        <x:v>Not a sealant, adhesive or repair for a broken seal. Must not contaminate the payload or damage the selected seal.</x:v>
+      </x:c>
+      <x:c r="O231" s="17"/>
+      <x:c r="P231" s="17"/>
+      <x:c r="Q231" s="17"/>
+      <x:c r="R231" s="17"/>
+      <x:c r="S231" s="17"/>
+      <x:c r="T231" s="9" t="str">
+        <x:v>Toxic industrial chemistry remains separate from food. Quality, batch consistency and specialist refinement may drive value; no price, spoilage or maintenance timer assigned.</x:v>
+      </x:c>
+      <x:c r="U231" s="11"/>
+      <x:c r="V231" s="9" t="str">
+        <x:v>New game proposal. Source WLD-0061 processing-agent record describes metabolic oil for machinery; source draft/proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+      <x:c r="W231" s="4" t="str">
+        <x:v>Chemical material</x:v>
+      </x:c>
+      <x:c r="X231" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y231" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z231" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="AA231" s="4" t="str">
+        <x:v>Biological chemical</x:v>
+      </x:c>
+      <x:c r="AB231" s="4" t="str">
+        <x:v>Paste</x:v>
+      </x:c>
+      <x:c r="AC231" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD231" s="4" t="str">
+        <x:v>seal-conditioning paste; grease; lubricant; fauna chemistry; sealing; lubrication</x:v>
+      </x:c>
+      <x:c r="AE231" s="4" t="str">
+        <x:v>Specific formulation is proposed; source oils and existing joint secretion are references, not validated recipes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="115" customHeight="1">
+      <x:c r="A232" s="9" t="str">
+        <x:v>proposal.lubricant.graphite_grease</x:v>
+      </x:c>
+      <x:c r="B232" s="9" t="str">
+        <x:v>Graphite faunal grease</x:v>
+      </x:c>
+      <x:c r="C232" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D232" s="9" t="str">
+        <x:v>Finished lubricant</x:v>
+      </x:c>
+      <x:c r="E232" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F232" s="9" t="str">
+        <x:v>Candidate lubricating blend using existing graded graphite flakes in a compatible faunal carrier.</x:v>
+      </x:c>
+      <x:c r="G232" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H232" s="9" t="str">
+        <x:v>Contained chemical cargo; carrier policy TBD</x:v>
+      </x:c>
+      <x:c r="I232" s="13"/>
+      <x:c r="J232" s="15"/>
+      <x:c r="K232" s="9" t="str">
+        <x:v>Process existing faunal secretions in a specialist workshop; exact species and route TBD</x:v>
+      </x:c>
+      <x:c r="L232" s="9" t="str">
+        <x:v>Proposed stages: segregated collection, separation, selected-fraction preparation, compatible formulation, service-specific testing. No formula or numeric yield.</x:v>
+      </x:c>
+      <x:c r="M232" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N232" s="9" t="str">
+        <x:v>Particle grade and part compatibility TBD. Keep electrical-contact behavior separate; no universal lubricant for every machine.</x:v>
+      </x:c>
+      <x:c r="O232" s="17"/>
+      <x:c r="P232" s="17"/>
+      <x:c r="Q232" s="17"/>
+      <x:c r="R232" s="17"/>
+      <x:c r="S232" s="17"/>
+      <x:c r="T232" s="9" t="str">
+        <x:v>Toxic industrial chemistry remains separate from food. Quality, batch consistency and specialist refinement may drive value; no price, spoilage or maintenance timer assigned.</x:v>
+      </x:c>
+      <x:c r="U232" s="11"/>
+      <x:c r="V232" s="9" t="str">
+        <x:v>New game proposal. Source WLD-0061 processing-agent record describes metabolic oil for machinery; source draft/proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+      <x:c r="W232" s="4" t="str">
+        <x:v>Chemical material</x:v>
+      </x:c>
+      <x:c r="X232" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y232" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z232" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="AA232" s="4" t="str">
+        <x:v>Biological and mineral mixture</x:v>
+      </x:c>
+      <x:c r="AB232" s="4" t="str">
+        <x:v>Paste</x:v>
+      </x:c>
+      <x:c r="AC232" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD232" s="4" t="str">
+        <x:v>graphite faunal grease; grease; lubricant; fauna chemistry; equipment repair; lubrication</x:v>
+      </x:c>
+      <x:c r="AE232" s="4" t="str">
+        <x:v>Specific formulation is proposed; source oils and existing joint secretion are references, not validated recipes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="115" customHeight="1">
+      <x:c r="A233" s="9" t="str">
+        <x:v>proposal.lubricant.insulating_grease</x:v>
+      </x:c>
+      <x:c r="B233" s="9" t="str">
+        <x:v>Electrically insulating grease</x:v>
+      </x:c>
+      <x:c r="C233" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D233" s="9" t="str">
+        <x:v>Finished lubricant</x:v>
+      </x:c>
+      <x:c r="E233" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F233" s="9" t="str">
+        <x:v>Candidate grease formulated for a selected insulating joint or equipment interface.</x:v>
+      </x:c>
+      <x:c r="G233" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H233" s="9" t="str">
+        <x:v>Contained chemical cargo; carrier policy TBD</x:v>
+      </x:c>
+      <x:c r="I233" s="13"/>
+      <x:c r="J233" s="15"/>
+      <x:c r="K233" s="9" t="str">
+        <x:v>Process existing faunal secretions in a specialist workshop; exact species and route TBD</x:v>
+      </x:c>
+      <x:c r="L233" s="9" t="str">
+        <x:v>Proposed stages: segregated collection, separation, selected-fraction preparation, compatible formulation, service-specific testing. No formula or numeric yield.</x:v>
+      </x:c>
+      <x:c r="M233" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N233" s="9" t="str">
+        <x:v>Insulation is a design target needing material selection and testing; not inferred from ordinary ichor or graphite grease.</x:v>
+      </x:c>
+      <x:c r="O233" s="17"/>
+      <x:c r="P233" s="17"/>
+      <x:c r="Q233" s="17"/>
+      <x:c r="R233" s="17"/>
+      <x:c r="S233" s="17"/>
+      <x:c r="T233" s="9" t="str">
+        <x:v>Toxic industrial chemistry remains separate from food. Quality, batch consistency and specialist refinement may drive value; no price, spoilage or maintenance timer assigned.</x:v>
+      </x:c>
+      <x:c r="U233" s="11"/>
+      <x:c r="V233" s="9" t="str">
+        <x:v>New game proposal. Source WLD-0061 processing-agent record describes metabolic oil for machinery; source draft/proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+      <x:c r="W233" s="4" t="str">
+        <x:v>Chemical material</x:v>
+      </x:c>
+      <x:c r="X233" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y233" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z233" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="AA233" s="4" t="str">
+        <x:v>Biological chemical</x:v>
+      </x:c>
+      <x:c r="AB233" s="4" t="str">
+        <x:v>Paste</x:v>
+      </x:c>
+      <x:c r="AC233" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD233" s="4" t="str">
+        <x:v>electrically insulating grease; grease; lubricant; fauna chemistry; electrical insulation; lubrication</x:v>
+      </x:c>
+      <x:c r="AE233" s="4" t="str">
+        <x:v>Specific formulation is proposed; source oils and existing joint secretion are references, not validated recipes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="115" customHeight="1">
+      <x:c r="A234" s="9" t="str">
+        <x:v>proposal.lubricant.precision_oil</x:v>
+      </x:c>
+      <x:c r="B234" s="9" t="str">
+        <x:v>Fine mechanism oil</x:v>
+      </x:c>
+      <x:c r="C234" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D234" s="9" t="str">
+        <x:v>Finished lubricant</x:v>
+      </x:c>
+      <x:c r="E234" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F234" s="9" t="str">
+        <x:v>Highly selected liquid lubricant candidate for small mechanisms and specialist workshop work.</x:v>
+      </x:c>
+      <x:c r="G234" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H234" s="9" t="str">
+        <x:v>Contained chemical cargo; carrier policy TBD</x:v>
+      </x:c>
+      <x:c r="I234" s="13"/>
+      <x:c r="J234" s="15"/>
+      <x:c r="K234" s="9" t="str">
+        <x:v>Process existing faunal secretions in a specialist workshop; exact species and route TBD</x:v>
+      </x:c>
+      <x:c r="L234" s="9" t="str">
+        <x:v>Proposed stages: segregated collection, separation, selected-fraction preparation, compatible formulation, service-specific testing. No formula or numeric yield.</x:v>
+      </x:c>
+      <x:c r="M234" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N234" s="9" t="str">
+        <x:v>Precision and low residue are proposed craft grades. No assumed food safety, optical suitability, shelf life or ancient-tech repair capability.</x:v>
+      </x:c>
+      <x:c r="O234" s="17"/>
+      <x:c r="P234" s="17"/>
+      <x:c r="Q234" s="17"/>
+      <x:c r="R234" s="17"/>
+      <x:c r="S234" s="17"/>
+      <x:c r="T234" s="9" t="str">
+        <x:v>Toxic industrial chemistry remains separate from food. Quality, batch consistency and specialist refinement may drive value; no price, spoilage or maintenance timer assigned.</x:v>
+      </x:c>
+      <x:c r="U234" s="11"/>
+      <x:c r="V234" s="9" t="str">
+        <x:v>New game proposal. Source WLD-0061 processing-agent record describes metabolic oil for machinery; source draft/proposal: https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+      <x:c r="W234" s="4" t="str">
+        <x:v>Chemical material</x:v>
+      </x:c>
+      <x:c r="X234" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y234" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z234" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="AA234" s="4" t="str">
+        <x:v>Biological chemical</x:v>
+      </x:c>
+      <x:c r="AB234" s="4" t="str">
+        <x:v>Liquid</x:v>
+      </x:c>
+      <x:c r="AC234" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD234" s="4" t="str">
+        <x:v>fine mechanism oil; grease; lubricant; fauna chemistry; equipment repair; lubrication</x:v>
+      </x:c>
+      <x:c r="AE234" s="4" t="str">
+        <x:v>Specific formulation is proposed; source oils and existing joint secretion are references, not validated recipes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18706,18 +19338,18 @@
       <x:formula1>'Taxonomy'!$B$54:$B$122</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AA6:AA1005">
-      <x:formula1>'Taxonomy'!$B$123:$B$151</x:formula1>
+      <x:formula1>'Taxonomy'!$B$123:$B$152</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AB6:AB1005">
-      <x:formula1>'Taxonomy'!$B$152:$B$170</x:formula1>
+      <x:formula1>'Taxonomy'!$B$153:$B$172</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AC6:AC1005">
-      <x:formula1>'Taxonomy'!$B$171:$B$175</x:formula1>
+      <x:formula1>'Taxonomy'!$B$173:$B$177</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81cdd21ffb674dcf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc456060523d44fca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19369,7 +20001,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98a7574a27cd45db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf065479cf473434b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19851,7 +20483,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b2fdef3127a4026"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c16fe2a6b8b4f40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21189,7 +21821,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B124" s="4" t="str">
-        <x:v>Biological chemical</x:v>
+        <x:v>Biological and mineral mixture</x:v>
       </x:c>
       <x:c r="C124" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21200,7 +21832,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B125" s="4" t="str">
-        <x:v>Carbonaceous material</x:v>
+        <x:v>Biological chemical</x:v>
       </x:c>
       <x:c r="C125" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21211,7 +21843,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B126" s="4" t="str">
-        <x:v>Ceramic</x:v>
+        <x:v>Carbonaceous material</x:v>
       </x:c>
       <x:c r="C126" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21222,7 +21854,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B127" s="4" t="str">
-        <x:v>Ceramic and metal</x:v>
+        <x:v>Ceramic</x:v>
       </x:c>
       <x:c r="C127" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21233,7 +21865,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B128" s="4" t="str">
-        <x:v>Ceramic feed mixture</x:v>
+        <x:v>Ceramic and metal</x:v>
       </x:c>
       <x:c r="C128" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21244,7 +21876,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B129" s="4" t="str">
-        <x:v>Faunal fiber</x:v>
+        <x:v>Ceramic feed mixture</x:v>
       </x:c>
       <x:c r="C129" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21255,7 +21887,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B130" s="4" t="str">
-        <x:v>Faunal fiber and shell</x:v>
+        <x:v>Faunal fiber</x:v>
       </x:c>
       <x:c r="C130" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21266,7 +21898,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B131" s="4" t="str">
-        <x:v>Faunal membrane</x:v>
+        <x:v>Faunal fiber and shell</x:v>
       </x:c>
       <x:c r="C131" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21277,7 +21909,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B132" s="4" t="str">
-        <x:v>Faunal tissue</x:v>
+        <x:v>Faunal membrane</x:v>
       </x:c>
       <x:c r="C132" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21288,7 +21920,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B133" s="4" t="str">
-        <x:v>Fur</x:v>
+        <x:v>Faunal tissue</x:v>
       </x:c>
       <x:c r="C133" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21299,7 +21931,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B134" s="4" t="str">
-        <x:v>Gemstone</x:v>
+        <x:v>Fur</x:v>
       </x:c>
       <x:c r="C134" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21310,7 +21942,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B135" s="4" t="str">
-        <x:v>Glass</x:v>
+        <x:v>Gemstone</x:v>
       </x:c>
       <x:c r="C135" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21321,7 +21953,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B136" s="4" t="str">
-        <x:v>Glass and metal</x:v>
+        <x:v>Glass</x:v>
       </x:c>
       <x:c r="C136" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21332,7 +21964,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B137" s="4" t="str">
-        <x:v>Glass and shell</x:v>
+        <x:v>Glass and metal</x:v>
       </x:c>
       <x:c r="C137" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21343,7 +21975,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B138" s="4" t="str">
-        <x:v>Glass with unresolved casing</x:v>
+        <x:v>Glass and shell</x:v>
       </x:c>
       <x:c r="C138" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21354,7 +21986,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B139" s="4" t="str">
-        <x:v>Hide</x:v>
+        <x:v>Glass with unresolved casing</x:v>
       </x:c>
       <x:c r="C139" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21365,7 +21997,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B140" s="4" t="str">
-        <x:v>Husk fiber</x:v>
+        <x:v>Hide</x:v>
       </x:c>
       <x:c r="C140" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21376,7 +22008,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B141" s="4" t="str">
-        <x:v>Husk fiber and shell</x:v>
+        <x:v>Husk fiber</x:v>
       </x:c>
       <x:c r="C141" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21387,7 +22019,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B142" s="4" t="str">
-        <x:v>Metal</x:v>
+        <x:v>Husk fiber and shell</x:v>
       </x:c>
       <x:c r="C142" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21398,7 +22030,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B143" s="4" t="str">
-        <x:v>Metal and shell</x:v>
+        <x:v>Metal</x:v>
       </x:c>
       <x:c r="C143" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21409,7 +22041,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B144" s="4" t="str">
-        <x:v>Metal or shell</x:v>
+        <x:v>Metal and shell</x:v>
       </x:c>
       <x:c r="C144" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21420,7 +22052,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B145" s="4" t="str">
-        <x:v>Mineral</x:v>
+        <x:v>Metal or shell</x:v>
       </x:c>
       <x:c r="C145" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21431,7 +22063,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B146" s="4" t="str">
-        <x:v>Mineral or shell</x:v>
+        <x:v>Mineral</x:v>
       </x:c>
       <x:c r="C146" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21442,7 +22074,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B147" s="4" t="str">
-        <x:v>Mixed / unresolved</x:v>
+        <x:v>Mineral or shell</x:v>
       </x:c>
       <x:c r="C147" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21453,7 +22085,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B148" s="4" t="str">
-        <x:v>Shell / chitin</x:v>
+        <x:v>Mixed / unresolved</x:v>
       </x:c>
       <x:c r="C148" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21464,7 +22096,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B149" s="4" t="str">
-        <x:v>Shell and mineral</x:v>
+        <x:v>Shell / chitin</x:v>
       </x:c>
       <x:c r="C149" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21475,7 +22107,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B150" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Shell and mineral</x:v>
       </x:c>
       <x:c r="C150" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21486,7 +22118,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B151" s="4" t="str">
-        <x:v>Wing membrane</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C151" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21494,13 +22126,13 @@
     </x:row>
     <x:row r="152" ht="45" customHeight="1">
       <x:c r="A152" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B152" s="4" t="str">
-        <x:v>Assembly</x:v>
+        <x:v>Wing membrane</x:v>
       </x:c>
       <x:c r="C152" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="153" ht="45" customHeight="1">
@@ -21508,7 +22140,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B153" s="4" t="str">
-        <x:v>Bundle</x:v>
+        <x:v>Assembly</x:v>
       </x:c>
       <x:c r="C153" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21519,7 +22151,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B154" s="4" t="str">
-        <x:v>Cord</x:v>
+        <x:v>Bundle</x:v>
       </x:c>
       <x:c r="C154" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21530,7 +22162,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B155" s="4" t="str">
-        <x:v>Fiber</x:v>
+        <x:v>Cord</x:v>
       </x:c>
       <x:c r="C155" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21541,7 +22173,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B156" s="4" t="str">
-        <x:v>Folio</x:v>
+        <x:v>Fiber</x:v>
       </x:c>
       <x:c r="C156" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21552,7 +22184,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B157" s="4" t="str">
-        <x:v>Garment</x:v>
+        <x:v>Folio</x:v>
       </x:c>
       <x:c r="C157" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21563,7 +22195,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B158" s="4" t="str">
-        <x:v>Gel</x:v>
+        <x:v>Garment</x:v>
       </x:c>
       <x:c r="C158" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21574,7 +22206,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B159" s="4" t="str">
-        <x:v>Liquid</x:v>
+        <x:v>Gel</x:v>
       </x:c>
       <x:c r="C159" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21585,7 +22217,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B160" s="4" t="str">
-        <x:v>Membrane</x:v>
+        <x:v>Liquid</x:v>
       </x:c>
       <x:c r="C160" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21596,7 +22228,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B161" s="4" t="str">
-        <x:v>Panel</x:v>
+        <x:v>Membrane</x:v>
       </x:c>
       <x:c r="C161" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21607,7 +22239,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B162" s="4" t="str">
-        <x:v>Particles</x:v>
+        <x:v>Panel</x:v>
       </x:c>
       <x:c r="C162" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21618,7 +22250,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B163" s="4" t="str">
-        <x:v>Patch</x:v>
+        <x:v>Particles</x:v>
       </x:c>
       <x:c r="C163" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21629,7 +22261,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B164" s="4" t="str">
-        <x:v>Rock</x:v>
+        <x:v>Paste</x:v>
       </x:c>
       <x:c r="C164" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21640,7 +22272,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B165" s="4" t="str">
-        <x:v>Sheet</x:v>
+        <x:v>Patch</x:v>
       </x:c>
       <x:c r="C165" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21651,7 +22283,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B166" s="4" t="str">
-        <x:v>Shell plate</x:v>
+        <x:v>Rock</x:v>
       </x:c>
       <x:c r="C166" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21662,7 +22294,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B167" s="4" t="str">
-        <x:v>Solid part</x:v>
+        <x:v>Sheet</x:v>
       </x:c>
       <x:c r="C167" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21673,7 +22305,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B168" s="4" t="str">
-        <x:v>Solid piece</x:v>
+        <x:v>Shell plate</x:v>
       </x:c>
       <x:c r="C168" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21684,7 +22316,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B169" s="4" t="str">
-        <x:v>Strip</x:v>
+        <x:v>Solid part</x:v>
       </x:c>
       <x:c r="C169" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21695,7 +22327,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B170" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Solid piece</x:v>
       </x:c>
       <x:c r="C170" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -21703,24 +22335,24 @@
     </x:row>
     <x:row r="171" ht="45" customHeight="1">
       <x:c r="A171" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B171" s="4" t="str">
-        <x:v>Author direction</x:v>
+        <x:v>Strip</x:v>
       </x:c>
       <x:c r="C171" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="172" ht="45" customHeight="1">
       <x:c r="A172" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B172" s="4" t="str">
-        <x:v>Existing definition</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C172" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="173" ht="45" customHeight="1">
@@ -21728,7 +22360,7 @@
         <x:v>Design status</x:v>
       </x:c>
       <x:c r="B173" s="4" t="str">
-        <x:v>Proposal</x:v>
+        <x:v>Author direction</x:v>
       </x:c>
       <x:c r="C173" s="4" t="str">
         <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
@@ -21739,7 +22371,7 @@
         <x:v>Design status</x:v>
       </x:c>
       <x:c r="B174" s="4" t="str">
-        <x:v>Source proposal</x:v>
+        <x:v>Existing definition</x:v>
       </x:c>
       <x:c r="C174" s="4" t="str">
         <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
@@ -21750,16 +22382,38 @@
         <x:v>Design status</x:v>
       </x:c>
       <x:c r="B175" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="C175" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="45" customHeight="1">
+      <x:c r="A176" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B176" s="4" t="str">
+        <x:v>Source proposal</x:v>
+      </x:c>
+      <x:c r="C176" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="45" customHeight="1">
+      <x:c r="A177" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B177" s="4" t="str">
         <x:v>Withheld assumption</x:v>
       </x:c>
-      <x:c r="C175" s="4" t="str">
+      <x:c r="C177" s="4" t="str">
         <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a7117340824833"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fb3b42a70bc4a02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28627,10 +29281,370 @@
         <x:v>Catalog intent. Source/author distinction and fire constraints are recorded in Items.</x:v>
       </x:c>
     </x:row>
+    <x:row r="306" ht="65" customHeight="1">
+      <x:c r="A306" s="4" t="str">
+        <x:v>proposal.lubricant.base</x:v>
+      </x:c>
+      <x:c r="B306" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A306,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Clarified faunal lubricant base</x:v>
+      </x:c>
+      <x:c r="C306" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A306,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D306" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E306" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A306,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chemical processing</x:v>
+      </x:c>
+      <x:c r="F306" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="307" ht="65" customHeight="1">
+      <x:c r="A307" s="4" t="str">
+        <x:v>proposal.lubricant.base</x:v>
+      </x:c>
+      <x:c r="B307" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A307,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Clarified faunal lubricant base</x:v>
+      </x:c>
+      <x:c r="C307" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A307,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D307" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E307" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F307" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="308" ht="65" customHeight="1">
+      <x:c r="A308" s="4" t="str">
+        <x:v>proposal.lubricant.thickener</x:v>
+      </x:c>
+      <x:c r="B308" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A308,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared secretion thickener</x:v>
+      </x:c>
+      <x:c r="C308" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A308,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D308" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E308" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A308,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chemical processing</x:v>
+      </x:c>
+      <x:c r="F308" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="309" ht="65" customHeight="1">
+      <x:c r="A309" s="4" t="str">
+        <x:v>proposal.lubricant.thickener</x:v>
+      </x:c>
+      <x:c r="B309" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A309,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared secretion thickener</x:v>
+      </x:c>
+      <x:c r="C309" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A309,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D309" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E309" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F309" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="310" ht="65" customHeight="1">
+      <x:c r="A310" s="4" t="str">
+        <x:v>proposal.lubricant.joint_grease</x:v>
+      </x:c>
+      <x:c r="B310" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A310,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Faunal joint grease</x:v>
+      </x:c>
+      <x:c r="C310" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A310,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D310" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E310" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A310,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F310" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="311" ht="65" customHeight="1">
+      <x:c r="A311" s="4" t="str">
+        <x:v>proposal.lubricant.joint_grease</x:v>
+      </x:c>
+      <x:c r="B311" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A311,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Faunal joint grease</x:v>
+      </x:c>
+      <x:c r="C311" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A311,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D311" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E311" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F311" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="312" ht="65" customHeight="1">
+      <x:c r="A312" s="4" t="str">
+        <x:v>proposal.lubricant.dust_film</x:v>
+      </x:c>
+      <x:c r="B312" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A312,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dust-shedding lubricant film</x:v>
+      </x:c>
+      <x:c r="C312" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A312,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D312" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E312" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A312,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F312" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="313" ht="65" customHeight="1">
+      <x:c r="A313" s="4" t="str">
+        <x:v>proposal.lubricant.dust_film</x:v>
+      </x:c>
+      <x:c r="B313" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A313,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dust-shedding lubricant film</x:v>
+      </x:c>
+      <x:c r="C313" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A313,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D313" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E313" s="4" t="str">
+        <x:v>Dust exclusion</x:v>
+      </x:c>
+      <x:c r="F313" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="314" ht="65" customHeight="1">
+      <x:c r="A314" s="4" t="str">
+        <x:v>proposal.lubricant.seal_paste</x:v>
+      </x:c>
+      <x:c r="B314" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A314,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Seal-conditioning paste</x:v>
+      </x:c>
+      <x:c r="C314" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A314,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D314" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E314" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A314,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F314" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="315" ht="65" customHeight="1">
+      <x:c r="A315" s="4" t="str">
+        <x:v>proposal.lubricant.seal_paste</x:v>
+      </x:c>
+      <x:c r="B315" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A315,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Seal-conditioning paste</x:v>
+      </x:c>
+      <x:c r="C315" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A315,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D315" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E315" s="4" t="str">
+        <x:v>Sealing</x:v>
+      </x:c>
+      <x:c r="F315" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="316" ht="65" customHeight="1">
+      <x:c r="A316" s="4" t="str">
+        <x:v>proposal.lubricant.graphite_grease</x:v>
+      </x:c>
+      <x:c r="B316" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A316,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Graphite faunal grease</x:v>
+      </x:c>
+      <x:c r="C316" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A316,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D316" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E316" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A316,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F316" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="317" ht="65" customHeight="1">
+      <x:c r="A317" s="4" t="str">
+        <x:v>proposal.lubricant.graphite_grease</x:v>
+      </x:c>
+      <x:c r="B317" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A317,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Graphite faunal grease</x:v>
+      </x:c>
+      <x:c r="C317" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A317,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D317" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E317" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F317" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="318" ht="65" customHeight="1">
+      <x:c r="A318" s="4" t="str">
+        <x:v>proposal.lubricant.insulating_grease</x:v>
+      </x:c>
+      <x:c r="B318" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A318,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Electrically insulating grease</x:v>
+      </x:c>
+      <x:c r="C318" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A318,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D318" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E318" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A318,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F318" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="319" ht="65" customHeight="1">
+      <x:c r="A319" s="4" t="str">
+        <x:v>proposal.lubricant.insulating_grease</x:v>
+      </x:c>
+      <x:c r="B319" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A319,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Electrically insulating grease</x:v>
+      </x:c>
+      <x:c r="C319" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A319,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D319" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E319" s="4" t="str">
+        <x:v>Electrical insulation</x:v>
+      </x:c>
+      <x:c r="F319" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="320" ht="65" customHeight="1">
+      <x:c r="A320" s="4" t="str">
+        <x:v>proposal.lubricant.precision_oil</x:v>
+      </x:c>
+      <x:c r="B320" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A320,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Fine mechanism oil</x:v>
+      </x:c>
+      <x:c r="C320" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A320,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D320" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E320" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A320,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F320" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="321" ht="65" customHeight="1">
+      <x:c r="A321" s="4" t="str">
+        <x:v>proposal.lubricant.precision_oil</x:v>
+      </x:c>
+      <x:c r="B321" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A321,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Fine mechanism oil</x:v>
+      </x:c>
+      <x:c r="C321" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A321,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D321" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E321" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F321" s="4" t="str">
+        <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A6:A1005">
-      <x:formula1>'Items'!$A$6:$A$226</x:formula1>
+      <x:formula1>'Items'!$A$6:$A$234</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D6:D1005">
       <x:formula1>"Primary,Secondary"</x:formula1>
@@ -28641,7 +29655,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4ac972e757149b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R870c405a556f47df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29549,7 +30563,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c693b60662d4bd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8d4d0fb74da455a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29915,7 +30929,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd26ab7ba87ab4d03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re22361b4452c457f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30006,7 +31020,7 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>84</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Minerals, biological resources, generic chemistry placeholders and twelve new chemical concepts</x:v>
@@ -30384,10 +31398,25 @@
         <x:v>Source fire behavior is proposal-stage. Extracted-stone behavior, fuel/air supply, cooking effects and equipment performance unresolved.</x:v>
       </x:c>
     </x:row>
+    <x:row r="34" ht="105" customHeight="1">
+      <x:c r="A34" s="3" t="str">
+        <x:v>Faunal lubricants</x:v>
+      </x:c>
+      <x:c r="B34" s="3" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Lubricant intermediate")+COUNTIF(Items!$D$6:$D$1005,"Finished lubricant")</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C34" s="3" t="str">
+        <x:v>Two candidate processing intermediates and six finished oil/grease/film families</x:v>
+      </x:c>
+      <x:c r="D34" s="3" t="str">
+        <x:v>Reuse existing raw joint secretion and graphite flakes. Industrial lubricant is distinct from adhesives, sealant, food and conductive gel.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R338f2205ffdf4a9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf15802da327a4d21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30450,7 +31479,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>221 design entries: 18 existing item IDs and 203 design/source concepts. Sixteen special-stone, fuel, cooking and fire-management entries added.</x:v>
+        <x:v>229 design entries: 18 existing item IDs and 211 design/source concepts. Eight faunal lubricant intermediates and products proposed.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -31162,7 +32191,7 @@
         <x:v>Filtering the master</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Items is one native filterable table, A5:AE226. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
+        <x:v>Items is one native filterable table, A5:AE234. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="85" customHeight="1">
@@ -31341,10 +32370,66 @@
         <x:v>WLD-0083 proposes trace humidity from hydrogen combustion, alongside other source food/water language. The game no-free-water rule remains controlling. No collectable water, condensation recipe or water supply is added by this task.</x:v>
       </x:c>
     </x:row>
+    <x:row r="120" ht="105" customHeight="1">
+      <x:c r="A120" s="4" t="str">
+        <x:v>Lubricant starting material</x:v>
+      </x:c>
+      <x:c r="B120" s="4" t="str">
+        <x:v>Reuse existing Joint-lubricating secretion. Source chemical-processing record proposes a scarce metabolic oil fraction used in industrial machinery. Neither establishes that most fauna contains conventional fat, or reinstates withheld fat/wax concepts. https://github.com/sleepyseamonster/Arc-Dust/blob/f6f98515c005dc3c73cccd9cbc031691745740c6/02-Arc-Dust-Worldbuilding/world/materials/chemical-processing-agents.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="105" customHeight="1">
+      <x:c r="A121" s="4" t="str">
+        <x:v>Proposed harvest and separation</x:v>
+      </x:c>
+      <x:c r="B121" s="4" t="str">
+        <x:v>Collect species/organ-specific fluids into separately marked compatible vessels. Proposed workshop sorting removes grit and hard-clotting fractions, then selects candidate slippery liquid. Vessel/strainer/settling methods, recovery losses and chemistry must be designed; no water wash or guaranteed purification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="105" customHeight="1">
+      <x:c r="A122" s="4" t="str">
+        <x:v>Proposed stabilization</x:v>
+      </x:c>
+      <x:c r="B122" s="4" t="str">
+        <x:v>Selected fractions would need preparation that limits unwanted hard-setting, corrosion, biological change and separation during storage. These are research requirements, not properties already solved by heating. No open-fire boiling, recipe temperatures, doses or proven detoxification are assigned.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="105" customHeight="1">
+      <x:c r="A123" s="4" t="str">
+        <x:v>Oil, grease and film</x:v>
+      </x:c>
+      <x:c r="B123" s="4" t="str">
+        <x:v>Keep selected liquid for fine oil; investigate a compatible non-curing thickener for grease; investigate a less persistent exposed film for dusty slides. Do not assume shell-binding glue makes grease: adhesion, curing and lubricity are different requirements.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="105" customHeight="1">
+      <x:c r="A124" s="4" t="str">
+        <x:v>Specialist formulations</x:v>
+      </x:c>
+      <x:c r="B124" s="4" t="str">
+        <x:v>Use-specific candidates: slow-joint grease, dust-shedding film, seal conditioner, graphite carrier grease, insulating grease and fine mechanism oil. Existing conductive gel remains a separate electrical material. One formulation cannot be assumed to serve all seals, temperatures, mechanisms and electrical roles.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="105" customHeight="1">
+      <x:c r="A125" s="4" t="str">
+        <x:v>Lubricant compatibility and economy</x:v>
+      </x:c>
+      <x:c r="B125" s="4" t="str">
+        <x:v>Candidate batch checks: grit, separation, hard-setting, flow/retention, wear, corrosion and compatibility with the intended seal/part. Exact tests and grades TBD. Consistent specialist batches could be valuable even when raw fluid is cheap; no price or maintenance timer set.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="105" customHeight="1">
+      <x:c r="A126" s="4" t="str">
+        <x:v>Lubricant handling and residue</x:v>
+      </x:c>
+      <x:c r="B126" s="4" t="str">
+        <x:v>Use existing marked bottles/jars and fitted transfer tools. Segregate chemical-processing and food-service vessels. Filter cake, clot residue and rejected fractions are waste streams requiring design, not automatic valuable new items. Lubricants remain potentially toxic and unsuitable as food.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ccab4361ab44aed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93578bfedbca42c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32188,7 +33273,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcced88e419214fee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bfa15faebbd4bfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32431,7 +33516,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b76f65595004b5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87e6615e737d4fd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32835,7 +33920,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba8f04fa49854165"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06b33fdf586647c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33511,7 +34596,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a939e103f914243"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95a52959ce4c4ac6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add wind sails turbines and dirtboard gear
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R9303566c63ba4a1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rf336aa35dc404d4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rfe9a96ddb92b4918"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rb76f65d1ca5e4a56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rd3ced0d9f93c4fc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rdb7e5429b9324151"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Rf1c2911a84884c77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Rf918468f81744fdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R9daaadfb56ee4945"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="Ra64bf09f63984375"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R2a57572d4e3e43ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="Rb4f190fdcd8a459b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="R03663e600a6947ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R3c0a606f599c44b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rdaddc019125b49e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rd4b8460b959f4bf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R73c8d592b5d949e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rd24d60e15d2a4d28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R45b7d35be5924168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R5eab30abb33546e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R082472f04ffd418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Rfffc6a24106d4e17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R2ae2f1f1c86e4c51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R9655a3c9df924ce6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R56bf436b598440cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="R1c7d15b65a1945ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,8 +476,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE234" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AE234"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE244" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AE244"/>
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -550,7 +550,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C177" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C184" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Field"/>
     <x:tableColumn id="2" name="Allowed value"/>
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F321" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F321"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F340" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F340"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -614,7 +614,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -626,7 +626,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B126" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -986,7 +986,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>229 entries. Filter W:AC for classifications; search AD. Lubricants include proposed base fractions, grease, oil and film grades.</x:v>
+        <x:v>239 entries. Wind machines, collapsible wing sails and four-wheel dirtboard gear classified in W:AC; search terms in AD.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -11899,7 +11899,7 @@
         <x:v>User direction; not implemented</x:v>
       </x:c>
       <x:c r="F141" s="9" t="str">
-        <x:v>Gathered insectoid megafauna inner-wing membrane for vertical sun shades.</x:v>
+        <x:v>Gathered insectoid megafauna inner-wing membrane for vertical sun shades. Also author-directed input for wind sails.</x:v>
       </x:c>
       <x:c r="G141" s="9" t="str">
         <x:v>None</x:v>
@@ -11955,7 +11955,7 @@
         <x:v>Author direction</x:v>
       </x:c>
       <x:c r="AD141" s="4" t="str">
-        <x:v>proposal bio inner wing; delicate inner wing; resources; wing material; sun shading; raw material; raw; fauna; sun shading; wing membrane; membrane; author direction</x:v>
+        <x:v>proposal bio inner wing; delicate inner wing; resources; wing material; sun shading; raw material; raw; fauna; sun shading; wing membrane; membrane; author direction; sail membrane; wind propulsion</x:v>
       </x:c>
       <x:c r="AE141" s="4" t="str">
         <x:v>From current item description. Proposed uses retain their existing approval status.</x:v>
@@ -19306,6 +19306,796 @@
       </x:c>
       <x:c r="AE234" s="4" t="str">
         <x:v>Specific formulation is proposed; source oils and existing joint secretion are references, not validated recipes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="115" customHeight="1">
+      <x:c r="A235" s="9" t="str">
+        <x:v>proposal.wind.turbine</x:v>
+      </x:c>
+      <x:c r="B235" s="9" t="str">
+        <x:v>Salvaged wind turbine</x:v>
+      </x:c>
+      <x:c r="C235" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D235" s="9" t="str">
+        <x:v>Wind machine</x:v>
+      </x:c>
+      <x:c r="E235" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F235" s="9" t="str">
+        <x:v>Wind turbine assembled from fallen/salvaged parts, as requested by author.</x:v>
+      </x:c>
+      <x:c r="G235" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H235" s="9" t="str">
+        <x:v>Physical part / installation ownership TBD</x:v>
+      </x:c>
+      <x:c r="I235" s="13"/>
+      <x:c r="J235" s="15"/>
+      <x:c r="K235" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L235" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M235" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N235" s="9" t="str">
+        <x:v>Stationary versus deployable installation, mounting, rotor form, wind response and useful output unresolved. Existing drive salvage is a candidate input, not a mandatory recipe.</x:v>
+      </x:c>
+      <x:c r="O235" s="17"/>
+      <x:c r="P235" s="17"/>
+      <x:c r="Q235" s="17"/>
+      <x:c r="R235" s="17"/>
+      <x:c r="S235" s="17"/>
+      <x:c r="T235" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U235" s="11"/>
+      <x:c r="V235" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W235" s="4" t="str">
+        <x:v>Machine</x:v>
+      </x:c>
+      <x:c r="X235" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y235" s="4" t="str">
+        <x:v>Recovered machinery</x:v>
+      </x:c>
+      <x:c r="Z235" s="4" t="str">
+        <x:v>Wind power</x:v>
+      </x:c>
+      <x:c r="AA235" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB235" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC235" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD235" s="4" t="str">
+        <x:v>salvaged wind turbine; wind machine; wind power; machinery drive; wind; sail; </x:v>
+      </x:c>
+      <x:c r="AE235" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="115" customHeight="1">
+      <x:c r="A236" s="9" t="str">
+        <x:v>proposal.wind.sail_panel</x:v>
+      </x:c>
+      <x:c r="B236" s="9" t="str">
+        <x:v>Prepared insect-wing sail panel</x:v>
+      </x:c>
+      <x:c r="C236" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D236" s="9" t="str">
+        <x:v>Wind sail material</x:v>
+      </x:c>
+      <x:c r="E236" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F236" s="9" t="str">
+        <x:v>Prepared delicate insectoid-wing membrane intended for a sail.</x:v>
+      </x:c>
+      <x:c r="G236" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H236" s="9" t="str">
+        <x:v>Physical part / installation ownership TBD</x:v>
+      </x:c>
+      <x:c r="I236" s="13"/>
+      <x:c r="J236" s="15"/>
+      <x:c r="K236" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L236" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M236" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N236" s="9" t="str">
+        <x:v>Reuse existing inner-wing resource. Sail panel and shade panel are service-specific intermediate concepts; decide later whether their preparation can share a product.</x:v>
+      </x:c>
+      <x:c r="O236" s="17"/>
+      <x:c r="P236" s="17"/>
+      <x:c r="Q236" s="17"/>
+      <x:c r="R236" s="17"/>
+      <x:c r="S236" s="17"/>
+      <x:c r="T236" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U236" s="11"/>
+      <x:c r="V236" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W236" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X236" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y236" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z236" s="4" t="str">
+        <x:v>Wind propulsion</x:v>
+      </x:c>
+      <x:c r="AA236" s="4" t="str">
+        <x:v>Wing membrane</x:v>
+      </x:c>
+      <x:c r="AB236" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC236" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD236" s="4" t="str">
+        <x:v>prepared insect-wing sail panel; wind sail material; wind propulsion; wind; sail; </x:v>
+      </x:c>
+      <x:c r="AE236" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="115" customHeight="1">
+      <x:c r="A237" s="9" t="str">
+        <x:v>proposal.wind.hand_sail</x:v>
+      </x:c>
+      <x:c r="B237" s="9" t="str">
+        <x:v>Collapsible handheld wind sail</x:v>
+      </x:c>
+      <x:c r="C237" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D237" s="9" t="str">
+        <x:v>Wind traversal gear</x:v>
+      </x:c>
+      <x:c r="E237" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F237" s="9" t="str">
+        <x:v>Booter handheld sail that collapses for carrying and opens for wind-driven dirtboard travel.</x:v>
+      </x:c>
+      <x:c r="G237" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H237" s="9" t="str">
+        <x:v>Booter personal gear intended; stowage policy TBD</x:v>
+      </x:c>
+      <x:c r="I237" s="13"/>
+      <x:c r="J237" s="15"/>
+      <x:c r="K237" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L237" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M237" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N237" s="9" t="str">
+        <x:v>One gear item with carried/deployed configurations. Frame geometry, hand use, steering, stowage and carry policy undefined.</x:v>
+      </x:c>
+      <x:c r="O237" s="17"/>
+      <x:c r="P237" s="17"/>
+      <x:c r="Q237" s="17"/>
+      <x:c r="R237" s="17"/>
+      <x:c r="S237" s="17"/>
+      <x:c r="T237" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U237" s="11"/>
+      <x:c r="V237" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W237" s="4" t="str">
+        <x:v>Traversal device</x:v>
+      </x:c>
+      <x:c r="X237" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y237" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z237" s="4" t="str">
+        <x:v>Wind propulsion</x:v>
+      </x:c>
+      <x:c r="AA237" s="4" t="str">
+        <x:v>Wing membrane and frame</x:v>
+      </x:c>
+      <x:c r="AB237" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC237" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD237" s="4" t="str">
+        <x:v>collapsible handheld wind sail; wind traversal gear; wind propulsion; traversal; wind; sail; </x:v>
+      </x:c>
+      <x:c r="AE237" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="115" customHeight="1">
+      <x:c r="A238" s="9" t="str">
+        <x:v>proposal.wind.dirtboard</x:v>
+      </x:c>
+      <x:c r="B238" s="9" t="str">
+        <x:v>Four-wheel all-terrain dirtboard</x:v>
+      </x:c>
+      <x:c r="C238" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D238" s="9" t="str">
+        <x:v>Wind traversal gear</x:v>
+      </x:c>
+      <x:c r="E238" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F238" s="9" t="str">
+        <x:v>Booter all-terrain skateboard with four wheels, used with the handheld sail across large flat areas.</x:v>
+      </x:c>
+      <x:c r="G238" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H238" s="9" t="str">
+        <x:v>Booter personal gear intended; stowage policy TBD</x:v>
+      </x:c>
+      <x:c r="I238" s="13"/>
+      <x:c r="J238" s="15"/>
+      <x:c r="K238" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L238" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M238" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N238" s="9" t="str">
+        <x:v>Wheel material, steering, braking, traction, terrain limits, speed and cargo effects remain open. Sail and board are separately owned companion items.</x:v>
+      </x:c>
+      <x:c r="O238" s="17"/>
+      <x:c r="P238" s="17"/>
+      <x:c r="Q238" s="17"/>
+      <x:c r="R238" s="17"/>
+      <x:c r="S238" s="17"/>
+      <x:c r="T238" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U238" s="11"/>
+      <x:c r="V238" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W238" s="4" t="str">
+        <x:v>Traversal device</x:v>
+      </x:c>
+      <x:c r="X238" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y238" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z238" s="4" t="str">
+        <x:v>Traversal</x:v>
+      </x:c>
+      <x:c r="AA238" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB238" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC238" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD238" s="4" t="str">
+        <x:v>four-wheel all-terrain dirtboard; wind traversal gear; traversal; wind propulsion; wind; sail; skateboard mountainboard four wheel dirt board</x:v>
+      </x:c>
+      <x:c r="AE238" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="115" customHeight="1">
+      <x:c r="A239" s="9" t="str">
+        <x:v>proposal.wind.folding_frame</x:v>
+      </x:c>
+      <x:c r="B239" s="9" t="str">
+        <x:v>Collapsible sail frame</x:v>
+      </x:c>
+      <x:c r="C239" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D239" s="9" t="str">
+        <x:v>Wind sail component</x:v>
+      </x:c>
+      <x:c r="E239" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F239" s="9" t="str">
+        <x:v>Proposed folding spars, joints and retainers supporting a wing sail.</x:v>
+      </x:c>
+      <x:c r="G239" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H239" s="9" t="str">
+        <x:v>Physical part / installation ownership TBD</x:v>
+      </x:c>
+      <x:c r="I239" s="13"/>
+      <x:c r="J239" s="15"/>
+      <x:c r="K239" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L239" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M239" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N239" s="9" t="str">
+        <x:v>Use metal/salvaged parts as candidates; folding geometry, weight and membrane attachment require design.</x:v>
+      </x:c>
+      <x:c r="O239" s="17"/>
+      <x:c r="P239" s="17"/>
+      <x:c r="Q239" s="17"/>
+      <x:c r="R239" s="17"/>
+      <x:c r="S239" s="17"/>
+      <x:c r="T239" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U239" s="11"/>
+      <x:c r="V239" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W239" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X239" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y239" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z239" s="4" t="str">
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="AA239" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB239" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC239" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD239" s="4" t="str">
+        <x:v>collapsible sail frame; wind sail component; equipment fabrication; wind; sail; </x:v>
+      </x:c>
+      <x:c r="AE239" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="115" customHeight="1">
+      <x:c r="A240" s="9" t="str">
+        <x:v>proposal.wind.sail_grip</x:v>
+      </x:c>
+      <x:c r="B240" s="9" t="str">
+        <x:v>Hand-sail grip assembly</x:v>
+      </x:c>
+      <x:c r="C240" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D240" s="9" t="str">
+        <x:v>Wind sail component</x:v>
+      </x:c>
+      <x:c r="E240" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F240" s="9" t="str">
+        <x:v>Proposed hand interface and control attachment for the collapsible sail.</x:v>
+      </x:c>
+      <x:c r="G240" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H240" s="9" t="str">
+        <x:v>Physical part / installation ownership TBD</x:v>
+      </x:c>
+      <x:c r="I240" s="13"/>
+      <x:c r="J240" s="15"/>
+      <x:c r="K240" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L240" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M240" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N240" s="9" t="str">
+        <x:v>Grip arrangement, release behavior and hand occupancy undecided; no body harness or bindings assumed.</x:v>
+      </x:c>
+      <x:c r="O240" s="17"/>
+      <x:c r="P240" s="17"/>
+      <x:c r="Q240" s="17"/>
+      <x:c r="R240" s="17"/>
+      <x:c r="S240" s="17"/>
+      <x:c r="T240" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U240" s="11"/>
+      <x:c r="V240" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W240" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X240" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y240" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z240" s="4" t="str">
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="AA240" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB240" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC240" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD240" s="4" t="str">
+        <x:v>hand-sail grip assembly; wind sail component; equipment fabrication; equipment mounting; wind; sail; </x:v>
+      </x:c>
+      <x:c r="AE240" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="115" customHeight="1">
+      <x:c r="A241" s="9" t="str">
+        <x:v>proposal.wind.wheel</x:v>
+      </x:c>
+      <x:c r="B241" s="9" t="str">
+        <x:v>Dirtboard wheel assembly</x:v>
+      </x:c>
+      <x:c r="C241" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D241" s="9" t="str">
+        <x:v>Dirtboard component</x:v>
+      </x:c>
+      <x:c r="E241" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F241" s="9" t="str">
+        <x:v>Replaceable wheel-and-bearing unit candidate for the four-wheel dirtboard.</x:v>
+      </x:c>
+      <x:c r="G241" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H241" s="9" t="str">
+        <x:v>Physical part / installation ownership TBD</x:v>
+      </x:c>
+      <x:c r="I241" s="13"/>
+      <x:c r="J241" s="15"/>
+      <x:c r="K241" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L241" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M241" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N241" s="9" t="str">
+        <x:v>Exactly four wheels on the assembled board by author direction. Wheel composition unresolved; no ordinary rubber supply assumed.</x:v>
+      </x:c>
+      <x:c r="O241" s="17"/>
+      <x:c r="P241" s="17"/>
+      <x:c r="Q241" s="17"/>
+      <x:c r="R241" s="17"/>
+      <x:c r="S241" s="17"/>
+      <x:c r="T241" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U241" s="11"/>
+      <x:c r="V241" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W241" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X241" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y241" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z241" s="4" t="str">
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="AA241" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB241" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC241" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD241" s="4" t="str">
+        <x:v>dirtboard wheel assembly; dirtboard component; equipment fabrication; equipment repair; wind; sail; </x:v>
+      </x:c>
+      <x:c r="AE241" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="115" customHeight="1">
+      <x:c r="A242" s="9" t="str">
+        <x:v>proposal.wind.truck</x:v>
+      </x:c>
+      <x:c r="B242" s="9" t="str">
+        <x:v>Dirtboard axle / steering assembly</x:v>
+      </x:c>
+      <x:c r="C242" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D242" s="9" t="str">
+        <x:v>Dirtboard component</x:v>
+      </x:c>
+      <x:c r="E242" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F242" s="9" t="str">
+        <x:v>Proposed mount joining wheels to the board and supporting a chosen steering method.</x:v>
+      </x:c>
+      <x:c r="G242" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H242" s="9" t="str">
+        <x:v>Physical part / installation ownership TBD</x:v>
+      </x:c>
+      <x:c r="I242" s="13"/>
+      <x:c r="J242" s="15"/>
+      <x:c r="K242" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L242" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M242" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N242" s="9" t="str">
+        <x:v>Axle/truck geometry, suspension and steering response are design questions; component count unassigned.</x:v>
+      </x:c>
+      <x:c r="O242" s="17"/>
+      <x:c r="P242" s="17"/>
+      <x:c r="Q242" s="17"/>
+      <x:c r="R242" s="17"/>
+      <x:c r="S242" s="17"/>
+      <x:c r="T242" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U242" s="11"/>
+      <x:c r="V242" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W242" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X242" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y242" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z242" s="4" t="str">
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="AA242" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB242" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC242" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD242" s="4" t="str">
+        <x:v>dirtboard axle / steering assembly; dirtboard component; equipment fabrication; equipment repair; wind; sail; </x:v>
+      </x:c>
+      <x:c r="AE242" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="115" customHeight="1">
+      <x:c r="A243" s="9" t="str">
+        <x:v>proposal.wind.rotor</x:v>
+      </x:c>
+      <x:c r="B243" s="9" t="str">
+        <x:v>Salvaged turbine rotor assembly</x:v>
+      </x:c>
+      <x:c r="C243" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D243" s="9" t="str">
+        <x:v>Wind machine component</x:v>
+      </x:c>
+      <x:c r="E243" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F243" s="9" t="str">
+        <x:v>Recovered or reworked rotor components for a compatible wind turbine.</x:v>
+      </x:c>
+      <x:c r="G243" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H243" s="9" t="str">
+        <x:v>Physical part / installation ownership TBD</x:v>
+      </x:c>
+      <x:c r="I243" s="13"/>
+      <x:c r="J243" s="15"/>
+      <x:c r="K243" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L243" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M243" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N243" s="9" t="str">
+        <x:v>Blade versus membrane rotor design undecided; not automatically a complete operating turbine.</x:v>
+      </x:c>
+      <x:c r="O243" s="17"/>
+      <x:c r="P243" s="17"/>
+      <x:c r="Q243" s="17"/>
+      <x:c r="R243" s="17"/>
+      <x:c r="S243" s="17"/>
+      <x:c r="T243" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U243" s="11"/>
+      <x:c r="V243" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W243" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X243" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y243" s="4" t="str">
+        <x:v>Recovered machinery</x:v>
+      </x:c>
+      <x:c r="Z243" s="4" t="str">
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="AA243" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB243" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC243" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD243" s="4" t="str">
+        <x:v>salvaged turbine rotor assembly; wind machine component; equipment fabrication; wind power; wind; sail; </x:v>
+      </x:c>
+      <x:c r="AE243" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="115" customHeight="1">
+      <x:c r="A244" s="9" t="str">
+        <x:v>proposal.wind.generator</x:v>
+      </x:c>
+      <x:c r="B244" s="9" t="str">
+        <x:v>Salvaged generator assembly</x:v>
+      </x:c>
+      <x:c r="C244" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D244" s="9" t="str">
+        <x:v>Wind machine component</x:v>
+      </x:c>
+      <x:c r="E244" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F244" s="9" t="str">
+        <x:v>Optional recovered electromechanical conversion unit for a future electrical-output turbine design.</x:v>
+      </x:c>
+      <x:c r="G244" s="9" t="str">
+        <x:v>Unassigned; no new slot approved</x:v>
+      </x:c>
+      <x:c r="H244" s="9" t="str">
+        <x:v>Physical part / installation ownership TBD</x:v>
+      </x:c>
+      <x:c r="I244" s="13"/>
+      <x:c r="J244" s="15"/>
+      <x:c r="K244" s="9" t="str">
+        <x:v>Salvage, insect-wing processing and specialist assembly; exact routes TBD</x:v>
+      </x:c>
+      <x:c r="L244" s="9" t="str">
+        <x:v>No recipe authored. Existing metal stock, drive salvage, fasteners and compatible lubricant concepts may support later design.</x:v>
+      </x:c>
+      <x:c r="M244" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N244" s="9" t="str">
+        <x:v>Wind output may instead drive machinery directly. Electrical output, connections and Arc Battery compatibility are undefined.</x:v>
+      </x:c>
+      <x:c r="O244" s="17"/>
+      <x:c r="P244" s="17"/>
+      <x:c r="Q244" s="17"/>
+      <x:c r="R244" s="17"/>
+      <x:c r="S244" s="17"/>
+      <x:c r="T244" s="9" t="str">
+        <x:v>Working labels; material quantities, durability and value unspecified. Fallen parts is interpreted as recoverable salvage, not proof of mandatory ancient technology.</x:v>
+      </x:c>
+      <x:c r="U244" s="11"/>
+      <x:c r="V244" s="9" t="str">
+        <x:v>Direct author wind-turbine, insect-wing sail and four-wheel dirtboard direction October 14, 2026; specific component breakdown is proposed.</x:v>
+      </x:c>
+      <x:c r="W244" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X244" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y244" s="4" t="str">
+        <x:v>Recovered machinery</x:v>
+      </x:c>
+      <x:c r="Z244" s="4" t="str">
+        <x:v>Energy processing</x:v>
+      </x:c>
+      <x:c r="AA244" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB244" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC244" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD244" s="4" t="str">
+        <x:v>salvaged generator assembly; wind machine component; energy processing; wind power; wind; sail; </x:v>
+      </x:c>
+      <x:c r="AE244" s="4" t="str">
+        <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19326,30 +20116,30 @@
       <x:formula1>'Taxonomy'!$B$6:$B$14</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="W6:W1005">
-      <x:formula1>'Taxonomy'!$B$15:$B$36</x:formula1>
+      <x:formula1>'Taxonomy'!$B$15:$B$38</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="X6:X1005">
-      <x:formula1>'Taxonomy'!$B$37:$B$45</x:formula1>
+      <x:formula1>'Taxonomy'!$B$39:$B$47</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Y6:Y1005">
-      <x:formula1>'Taxonomy'!$B$46:$B$53</x:formula1>
+      <x:formula1>'Taxonomy'!$B$48:$B$55</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Z6:Z1005">
-      <x:formula1>'Taxonomy'!$B$54:$B$122</x:formula1>
+      <x:formula1>'Taxonomy'!$B$56:$B$128</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AA6:AA1005">
-      <x:formula1>'Taxonomy'!$B$123:$B$152</x:formula1>
+      <x:formula1>'Taxonomy'!$B$129:$B$159</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AB6:AB1005">
-      <x:formula1>'Taxonomy'!$B$153:$B$172</x:formula1>
+      <x:formula1>'Taxonomy'!$B$160:$B$179</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AC6:AC1005">
-      <x:formula1>'Taxonomy'!$B$173:$B$177</x:formula1>
+      <x:formula1>'Taxonomy'!$B$180:$B$184</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc456060523d44fca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R906d8f39e56b4b7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20001,7 +20791,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf065479cf473434b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe7b27f3fe944253"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20483,7 +21273,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c16fe2a6b8b4f40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56216e5a95554486"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20765,7 +21555,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B28" s="4" t="str">
-        <x:v>Musical instrument</x:v>
+        <x:v>Machine</x:v>
       </x:c>
       <x:c r="C28" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -20776,7 +21566,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B29" s="4" t="str">
-        <x:v>Processed material</x:v>
+        <x:v>Musical instrument</x:v>
       </x:c>
       <x:c r="C29" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -20787,7 +21577,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B30" s="4" t="str">
-        <x:v>Raw material</x:v>
+        <x:v>Processed material</x:v>
       </x:c>
       <x:c r="C30" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -20798,7 +21588,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B31" s="4" t="str">
-        <x:v>Service kit</x:v>
+        <x:v>Raw material</x:v>
       </x:c>
       <x:c r="C31" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -20809,7 +21599,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B32" s="4" t="str">
-        <x:v>Shelter kit</x:v>
+        <x:v>Service kit</x:v>
       </x:c>
       <x:c r="C32" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -20820,7 +21610,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B33" s="4" t="str">
-        <x:v>Shield</x:v>
+        <x:v>Shelter kit</x:v>
       </x:c>
       <x:c r="C33" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -20831,7 +21621,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B34" s="4" t="str">
-        <x:v>Tool</x:v>
+        <x:v>Shield</x:v>
       </x:c>
       <x:c r="C34" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -20842,7 +21632,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B35" s="4" t="str">
-        <x:v>Trip hazard</x:v>
+        <x:v>Tool</x:v>
       </x:c>
       <x:c r="C35" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -20853,7 +21643,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B36" s="4" t="str">
-        <x:v>Wearable</x:v>
+        <x:v>Traversal device</x:v>
       </x:c>
       <x:c r="C36" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -20861,24 +21651,24 @@
     </x:row>
     <x:row r="37" ht="45" customHeight="1">
       <x:c r="A37" s="4" t="str">
-        <x:v>Processing stage</x:v>
+        <x:v>Item type</x:v>
       </x:c>
       <x:c r="B37" s="4" t="str">
-        <x:v>Ancient manufactured</x:v>
+        <x:v>Trip hazard</x:v>
       </x:c>
       <x:c r="C37" s="4" t="str">
-        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
+        <x:v>What the object is, independent of material, culture and use.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="45" customHeight="1">
       <x:c r="A38" s="4" t="str">
-        <x:v>Processing stage</x:v>
+        <x:v>Item type</x:v>
       </x:c>
       <x:c r="B38" s="4" t="str">
-        <x:v>Extracted material</x:v>
+        <x:v>Wearable</x:v>
       </x:c>
       <x:c r="C38" s="4" t="str">
-        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
+        <x:v>What the object is, independent of material, culture and use.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="45" customHeight="1">
@@ -20886,7 +21676,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B39" s="4" t="str">
-        <x:v>Finished item</x:v>
+        <x:v>Ancient manufactured</x:v>
       </x:c>
       <x:c r="C39" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -20897,7 +21687,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B40" s="4" t="str">
-        <x:v>Processed intermediate</x:v>
+        <x:v>Extracted material</x:v>
       </x:c>
       <x:c r="C40" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -20908,7 +21698,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B41" s="4" t="str">
-        <x:v>Raw</x:v>
+        <x:v>Finished item</x:v>
       </x:c>
       <x:c r="C41" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -20919,7 +21709,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B42" s="4" t="str">
-        <x:v>Recovered part</x:v>
+        <x:v>Processed intermediate</x:v>
       </x:c>
       <x:c r="C42" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -20930,7 +21720,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B43" s="4" t="str">
-        <x:v>Unfired intermediate</x:v>
+        <x:v>Raw</x:v>
       </x:c>
       <x:c r="C43" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -20941,7 +21731,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B44" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Recovered part</x:v>
       </x:c>
       <x:c r="C44" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -20952,7 +21742,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B45" s="4" t="str">
-        <x:v>Unworked metal</x:v>
+        <x:v>Unfired intermediate</x:v>
       </x:c>
       <x:c r="C45" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -20960,24 +21750,24 @@
     </x:row>
     <x:row r="46" ht="45" customHeight="1">
       <x:c r="A46" s="4" t="str">
-        <x:v>Origin family</x:v>
+        <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B46" s="4" t="str">
-        <x:v>Ancient technology</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C46" s="4" t="str">
-        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
+        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="45" customHeight="1">
       <x:c r="A47" s="4" t="str">
-        <x:v>Origin family</x:v>
+        <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B47" s="4" t="str">
-        <x:v>Atmospheric</x:v>
+        <x:v>Unworked metal</x:v>
       </x:c>
       <x:c r="C47" s="4" t="str">
-        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
+        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="45" customHeight="1">
@@ -20985,7 +21775,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B48" s="4" t="str">
-        <x:v>Fauna</x:v>
+        <x:v>Ancient technology</x:v>
       </x:c>
       <x:c r="C48" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -20996,7 +21786,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B49" s="4" t="str">
-        <x:v>Geological</x:v>
+        <x:v>Atmospheric</x:v>
       </x:c>
       <x:c r="C49" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -21007,7 +21797,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B50" s="4" t="str">
-        <x:v>Living culture</x:v>
+        <x:v>Fauna</x:v>
       </x:c>
       <x:c r="C50" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -21018,7 +21808,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B51" s="4" t="str">
-        <x:v>Manufactured / unresolved</x:v>
+        <x:v>Geological</x:v>
       </x:c>
       <x:c r="C51" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -21029,7 +21819,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B52" s="4" t="str">
-        <x:v>Recovered machinery</x:v>
+        <x:v>Living culture</x:v>
       </x:c>
       <x:c r="C52" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -21040,7 +21830,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B53" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Manufactured / unresolved</x:v>
       </x:c>
       <x:c r="C53" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -21048,24 +21838,24 @@
     </x:row>
     <x:row r="54" ht="45" customHeight="1">
       <x:c r="A54" s="4" t="str">
-        <x:v>Primary use</x:v>
+        <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B54" s="4" t="str">
-        <x:v>Area denial</x:v>
+        <x:v>Recovered machinery</x:v>
       </x:c>
       <x:c r="C54" s="4" t="str">
-        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
+        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="45" customHeight="1">
       <x:c r="A55" s="4" t="str">
-        <x:v>Primary use</x:v>
+        <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B55" s="4" t="str">
-        <x:v>Atmospheric support</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C55" s="4" t="str">
-        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
+        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="45" customHeight="1">
@@ -21073,7 +21863,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B56" s="4" t="str">
-        <x:v>Binding and construction</x:v>
+        <x:v>Area denial</x:v>
       </x:c>
       <x:c r="C56" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21084,7 +21874,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B57" s="4" t="str">
-        <x:v>Camp rest</x:v>
+        <x:v>Atmospheric support</x:v>
       </x:c>
       <x:c r="C57" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21095,7 +21885,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B58" s="4" t="str">
-        <x:v>Cargo organization</x:v>
+        <x:v>Binding and construction</x:v>
       </x:c>
       <x:c r="C58" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21106,7 +21896,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B59" s="4" t="str">
-        <x:v>Ceremony</x:v>
+        <x:v>Camp rest</x:v>
       </x:c>
       <x:c r="C59" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21117,7 +21907,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B60" s="4" t="str">
-        <x:v>Chemical processing</x:v>
+        <x:v>Cargo organization</x:v>
       </x:c>
       <x:c r="C60" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21128,7 +21918,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B61" s="4" t="str">
-        <x:v>Civic identification</x:v>
+        <x:v>Ceremony</x:v>
       </x:c>
       <x:c r="C61" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21139,7 +21929,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B62" s="4" t="str">
-        <x:v>Civic recognition</x:v>
+        <x:v>Chemical processing</x:v>
       </x:c>
       <x:c r="C62" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21150,7 +21940,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B63" s="4" t="str">
-        <x:v>Cleaning</x:v>
+        <x:v>Civic identification</x:v>
       </x:c>
       <x:c r="C63" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21161,7 +21951,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B64" s="4" t="str">
-        <x:v>Clothing</x:v>
+        <x:v>Civic recognition</x:v>
       </x:c>
       <x:c r="C64" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21172,7 +21962,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B65" s="4" t="str">
-        <x:v>Clothing fabrication</x:v>
+        <x:v>Cleaning</x:v>
       </x:c>
       <x:c r="C65" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21183,7 +21973,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B66" s="4" t="str">
-        <x:v>Cooking</x:v>
+        <x:v>Clothing</x:v>
       </x:c>
       <x:c r="C66" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21194,7 +21984,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B67" s="4" t="str">
-        <x:v>Culture support</x:v>
+        <x:v>Clothing fabrication</x:v>
       </x:c>
       <x:c r="C67" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21205,7 +21995,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B68" s="4" t="str">
-        <x:v>Decoration</x:v>
+        <x:v>Cooking</x:v>
       </x:c>
       <x:c r="C68" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21216,7 +22006,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B69" s="4" t="str">
-        <x:v>Devotion</x:v>
+        <x:v>Culture support</x:v>
       </x:c>
       <x:c r="C69" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21227,7 +22017,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B70" s="4" t="str">
-        <x:v>Dust exclusion</x:v>
+        <x:v>Decoration</x:v>
       </x:c>
       <x:c r="C70" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21238,7 +22028,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B71" s="4" t="str">
-        <x:v>Electrical conduction</x:v>
+        <x:v>Devotion</x:v>
       </x:c>
       <x:c r="C71" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21249,7 +22039,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B72" s="4" t="str">
-        <x:v>Electrical insulation</x:v>
+        <x:v>Dust exclusion</x:v>
       </x:c>
       <x:c r="C72" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21260,7 +22050,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B73" s="4" t="str">
-        <x:v>Electrical work</x:v>
+        <x:v>Electrical conduction</x:v>
       </x:c>
       <x:c r="C73" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21271,7 +22061,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B74" s="4" t="str">
-        <x:v>Energy processing</x:v>
+        <x:v>Electrical insulation</x:v>
       </x:c>
       <x:c r="C74" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21282,7 +22072,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B75" s="4" t="str">
-        <x:v>Energy storage</x:v>
+        <x:v>Electrical work</x:v>
       </x:c>
       <x:c r="C75" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21293,7 +22083,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B76" s="4" t="str">
-        <x:v>Equipment mounting</x:v>
+        <x:v>Energy processing</x:v>
       </x:c>
       <x:c r="C76" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21304,7 +22094,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B77" s="4" t="str">
-        <x:v>Equipment repair</x:v>
+        <x:v>Energy storage</x:v>
       </x:c>
       <x:c r="C77" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21315,7 +22105,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B78" s="4" t="str">
-        <x:v>Excavation</x:v>
+        <x:v>Equipment fabrication</x:v>
       </x:c>
       <x:c r="C78" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21326,7 +22116,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B79" s="4" t="str">
-        <x:v>Fabrication</x:v>
+        <x:v>Equipment mounting</x:v>
       </x:c>
       <x:c r="C79" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21337,7 +22127,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B80" s="4" t="str">
-        <x:v>Fashion</x:v>
+        <x:v>Equipment repair</x:v>
       </x:c>
       <x:c r="C80" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21348,7 +22138,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B81" s="4" t="str">
-        <x:v>Fauna interaction</x:v>
+        <x:v>Excavation</x:v>
       </x:c>
       <x:c r="C81" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21359,7 +22149,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B82" s="4" t="str">
-        <x:v>Fiber processing</x:v>
+        <x:v>Fabrication</x:v>
       </x:c>
       <x:c r="C82" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21370,7 +22160,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B83" s="4" t="str">
-        <x:v>Fire management</x:v>
+        <x:v>Fashion</x:v>
       </x:c>
       <x:c r="C83" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21381,7 +22171,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B84" s="4" t="str">
-        <x:v>Food service</x:v>
+        <x:v>Fauna interaction</x:v>
       </x:c>
       <x:c r="C84" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21392,7 +22182,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B85" s="4" t="str">
-        <x:v>Fuel</x:v>
+        <x:v>Fiber processing</x:v>
       </x:c>
       <x:c r="C85" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21403,7 +22193,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B86" s="4" t="str">
-        <x:v>Glass and ceramics</x:v>
+        <x:v>Fire management</x:v>
       </x:c>
       <x:c r="C86" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21414,7 +22204,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B87" s="4" t="str">
-        <x:v>Grooming</x:v>
+        <x:v>Food service</x:v>
       </x:c>
       <x:c r="C87" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21425,7 +22215,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B88" s="4" t="str">
-        <x:v>Ignition</x:v>
+        <x:v>Fuel</x:v>
       </x:c>
       <x:c r="C88" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21436,7 +22226,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B89" s="4" t="str">
-        <x:v>Illumination</x:v>
+        <x:v>Glass and ceramics</x:v>
       </x:c>
       <x:c r="C89" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21447,7 +22237,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B90" s="4" t="str">
-        <x:v>Injury treatment</x:v>
+        <x:v>Grooming</x:v>
       </x:c>
       <x:c r="C90" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21458,7 +22248,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B91" s="4" t="str">
-        <x:v>Inspection</x:v>
+        <x:v>Ignition</x:v>
       </x:c>
       <x:c r="C91" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21469,7 +22259,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B92" s="4" t="str">
-        <x:v>Keepsake storage</x:v>
+        <x:v>Illumination</x:v>
       </x:c>
       <x:c r="C92" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21480,7 +22270,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B93" s="4" t="str">
-        <x:v>Liquid and bulk containment</x:v>
+        <x:v>Injury treatment</x:v>
       </x:c>
       <x:c r="C93" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21491,7 +22281,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B94" s="4" t="str">
-        <x:v>Lubrication</x:v>
+        <x:v>Inspection</x:v>
       </x:c>
       <x:c r="C94" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21502,7 +22292,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B95" s="4" t="str">
-        <x:v>Machinery repair</x:v>
+        <x:v>Keepsake storage</x:v>
       </x:c>
       <x:c r="C95" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21513,7 +22303,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B96" s="4" t="str">
-        <x:v>Magnetic tools</x:v>
+        <x:v>Liquid and bulk containment</x:v>
       </x:c>
       <x:c r="C96" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21524,7 +22314,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Material exclusion</x:v>
+        <x:v>Lubrication</x:v>
       </x:c>
       <x:c r="C97" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21535,7 +22325,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B98" s="4" t="str">
-        <x:v>Material transfer</x:v>
+        <x:v>Machinery drive</x:v>
       </x:c>
       <x:c r="C98" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21546,7 +22336,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B99" s="4" t="str">
-        <x:v>Metal refining</x:v>
+        <x:v>Machinery repair</x:v>
       </x:c>
       <x:c r="C99" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21557,7 +22347,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B100" s="4" t="str">
-        <x:v>Music</x:v>
+        <x:v>Magnetic tools</x:v>
       </x:c>
       <x:c r="C100" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21568,7 +22358,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B101" s="4" t="str">
-        <x:v>Nutrition</x:v>
+        <x:v>Material exclusion</x:v>
       </x:c>
       <x:c r="C101" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21579,7 +22369,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B102" s="4" t="str">
-        <x:v>Paper making</x:v>
+        <x:v>Material transfer</x:v>
       </x:c>
       <x:c r="C102" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21590,7 +22380,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B103" s="4" t="str">
-        <x:v>Protection</x:v>
+        <x:v>Metal refining</x:v>
       </x:c>
       <x:c r="C103" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21601,7 +22391,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B104" s="4" t="str">
-        <x:v>Protective fabrication</x:v>
+        <x:v>Music</x:v>
       </x:c>
       <x:c r="C104" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21612,7 +22402,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B105" s="4" t="str">
-        <x:v>Provenance</x:v>
+        <x:v>Nutrition</x:v>
       </x:c>
       <x:c r="C105" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21623,7 +22413,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B106" s="4" t="str">
-        <x:v>Public communication</x:v>
+        <x:v>Paper making</x:v>
       </x:c>
       <x:c r="C106" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21634,7 +22424,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B107" s="4" t="str">
-        <x:v>Remembrance</x:v>
+        <x:v>Protection</x:v>
       </x:c>
       <x:c r="C107" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21645,7 +22435,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B108" s="4" t="str">
-        <x:v>Resource collection</x:v>
+        <x:v>Protective fabrication</x:v>
       </x:c>
       <x:c r="C108" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21656,7 +22446,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B109" s="4" t="str">
-        <x:v>Sealing</x:v>
+        <x:v>Provenance</x:v>
       </x:c>
       <x:c r="C109" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21667,7 +22457,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B110" s="4" t="str">
-        <x:v>Specialist samples</x:v>
+        <x:v>Public communication</x:v>
       </x:c>
       <x:c r="C110" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21678,7 +22468,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B111" s="4" t="str">
-        <x:v>Static management</x:v>
+        <x:v>Remembrance</x:v>
       </x:c>
       <x:c r="C111" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21689,7 +22479,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B112" s="4" t="str">
-        <x:v>Sun shading</x:v>
+        <x:v>Resource collection</x:v>
       </x:c>
       <x:c r="C112" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21700,7 +22490,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B113" s="4" t="str">
-        <x:v>Surface finishing</x:v>
+        <x:v>Sealing</x:v>
       </x:c>
       <x:c r="C113" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21711,7 +22501,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B114" s="4" t="str">
-        <x:v>Survival provision</x:v>
+        <x:v>Specialist samples</x:v>
       </x:c>
       <x:c r="C114" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21722,7 +22512,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B115" s="4" t="str">
-        <x:v>Textile processing</x:v>
+        <x:v>Static management</x:v>
       </x:c>
       <x:c r="C115" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21733,7 +22523,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B116" s="4" t="str">
-        <x:v>Tool fabrication</x:v>
+        <x:v>Sun shading</x:v>
       </x:c>
       <x:c r="C116" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21744,7 +22534,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B117" s="4" t="str">
-        <x:v>Trade</x:v>
+        <x:v>Surface finishing</x:v>
       </x:c>
       <x:c r="C117" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21755,7 +22545,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B118" s="4" t="str">
-        <x:v>Traversal</x:v>
+        <x:v>Survival provision</x:v>
       </x:c>
       <x:c r="C118" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21766,7 +22556,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B119" s="4" t="str">
-        <x:v>Use unresolved</x:v>
+        <x:v>Textile processing</x:v>
       </x:c>
       <x:c r="C119" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21777,7 +22567,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B120" s="4" t="str">
-        <x:v>Vision</x:v>
+        <x:v>Tool fabrication</x:v>
       </x:c>
       <x:c r="C120" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21788,7 +22578,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B121" s="4" t="str">
-        <x:v>Work holding</x:v>
+        <x:v>Trade</x:v>
       </x:c>
       <x:c r="C121" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21799,7 +22589,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B122" s="4" t="str">
-        <x:v>Writing and records</x:v>
+        <x:v>Traversal</x:v>
       </x:c>
       <x:c r="C122" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -21807,68 +22597,68 @@
     </x:row>
     <x:row r="123" ht="45" customHeight="1">
       <x:c r="A123" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B123" s="4" t="str">
-        <x:v>Ancient composite</x:v>
+        <x:v>Use unresolved</x:v>
       </x:c>
       <x:c r="C123" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="45" customHeight="1">
       <x:c r="A124" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B124" s="4" t="str">
-        <x:v>Biological and mineral mixture</x:v>
+        <x:v>Vision</x:v>
       </x:c>
       <x:c r="C124" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="45" customHeight="1">
       <x:c r="A125" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B125" s="4" t="str">
-        <x:v>Biological chemical</x:v>
+        <x:v>Wind power</x:v>
       </x:c>
       <x:c r="C125" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="45" customHeight="1">
       <x:c r="A126" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B126" s="4" t="str">
-        <x:v>Carbonaceous material</x:v>
+        <x:v>Wind propulsion</x:v>
       </x:c>
       <x:c r="C126" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="45" customHeight="1">
       <x:c r="A127" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B127" s="4" t="str">
-        <x:v>Ceramic</x:v>
+        <x:v>Work holding</x:v>
       </x:c>
       <x:c r="C127" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="45" customHeight="1">
       <x:c r="A128" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B128" s="4" t="str">
-        <x:v>Ceramic and metal</x:v>
+        <x:v>Writing and records</x:v>
       </x:c>
       <x:c r="C128" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="45" customHeight="1">
@@ -21876,7 +22666,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B129" s="4" t="str">
-        <x:v>Ceramic feed mixture</x:v>
+        <x:v>Ancient composite</x:v>
       </x:c>
       <x:c r="C129" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21887,7 +22677,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B130" s="4" t="str">
-        <x:v>Faunal fiber</x:v>
+        <x:v>Biological and mineral mixture</x:v>
       </x:c>
       <x:c r="C130" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21898,7 +22688,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B131" s="4" t="str">
-        <x:v>Faunal fiber and shell</x:v>
+        <x:v>Biological chemical</x:v>
       </x:c>
       <x:c r="C131" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21909,7 +22699,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B132" s="4" t="str">
-        <x:v>Faunal membrane</x:v>
+        <x:v>Carbonaceous material</x:v>
       </x:c>
       <x:c r="C132" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21920,7 +22710,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B133" s="4" t="str">
-        <x:v>Faunal tissue</x:v>
+        <x:v>Ceramic</x:v>
       </x:c>
       <x:c r="C133" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21931,7 +22721,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B134" s="4" t="str">
-        <x:v>Fur</x:v>
+        <x:v>Ceramic and metal</x:v>
       </x:c>
       <x:c r="C134" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21942,7 +22732,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B135" s="4" t="str">
-        <x:v>Gemstone</x:v>
+        <x:v>Ceramic feed mixture</x:v>
       </x:c>
       <x:c r="C135" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21953,7 +22743,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B136" s="4" t="str">
-        <x:v>Glass</x:v>
+        <x:v>Faunal fiber</x:v>
       </x:c>
       <x:c r="C136" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21964,7 +22754,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B137" s="4" t="str">
-        <x:v>Glass and metal</x:v>
+        <x:v>Faunal fiber and shell</x:v>
       </x:c>
       <x:c r="C137" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21975,7 +22765,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B138" s="4" t="str">
-        <x:v>Glass and shell</x:v>
+        <x:v>Faunal membrane</x:v>
       </x:c>
       <x:c r="C138" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21986,7 +22776,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B139" s="4" t="str">
-        <x:v>Glass with unresolved casing</x:v>
+        <x:v>Faunal tissue</x:v>
       </x:c>
       <x:c r="C139" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -21997,7 +22787,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B140" s="4" t="str">
-        <x:v>Hide</x:v>
+        <x:v>Fur</x:v>
       </x:c>
       <x:c r="C140" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22008,7 +22798,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B141" s="4" t="str">
-        <x:v>Husk fiber</x:v>
+        <x:v>Gemstone</x:v>
       </x:c>
       <x:c r="C141" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22019,7 +22809,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B142" s="4" t="str">
-        <x:v>Husk fiber and shell</x:v>
+        <x:v>Glass</x:v>
       </x:c>
       <x:c r="C142" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22030,7 +22820,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B143" s="4" t="str">
-        <x:v>Metal</x:v>
+        <x:v>Glass and metal</x:v>
       </x:c>
       <x:c r="C143" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22041,7 +22831,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B144" s="4" t="str">
-        <x:v>Metal and shell</x:v>
+        <x:v>Glass and shell</x:v>
       </x:c>
       <x:c r="C144" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22052,7 +22842,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B145" s="4" t="str">
-        <x:v>Metal or shell</x:v>
+        <x:v>Glass with unresolved casing</x:v>
       </x:c>
       <x:c r="C145" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22063,7 +22853,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B146" s="4" t="str">
-        <x:v>Mineral</x:v>
+        <x:v>Hide</x:v>
       </x:c>
       <x:c r="C146" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22074,7 +22864,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B147" s="4" t="str">
-        <x:v>Mineral or shell</x:v>
+        <x:v>Husk fiber</x:v>
       </x:c>
       <x:c r="C147" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22085,7 +22875,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B148" s="4" t="str">
-        <x:v>Mixed / unresolved</x:v>
+        <x:v>Husk fiber and shell</x:v>
       </x:c>
       <x:c r="C148" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22096,7 +22886,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B149" s="4" t="str">
-        <x:v>Shell / chitin</x:v>
+        <x:v>Metal</x:v>
       </x:c>
       <x:c r="C149" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22107,7 +22897,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B150" s="4" t="str">
-        <x:v>Shell and mineral</x:v>
+        <x:v>Metal and shell</x:v>
       </x:c>
       <x:c r="C150" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22118,7 +22908,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B151" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Metal or shell</x:v>
       </x:c>
       <x:c r="C151" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22129,7 +22919,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B152" s="4" t="str">
-        <x:v>Wing membrane</x:v>
+        <x:v>Mineral</x:v>
       </x:c>
       <x:c r="C152" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -22137,79 +22927,79 @@
     </x:row>
     <x:row r="153" ht="45" customHeight="1">
       <x:c r="A153" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B153" s="4" t="str">
-        <x:v>Assembly</x:v>
+        <x:v>Mineral or shell</x:v>
       </x:c>
       <x:c r="C153" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="154" ht="45" customHeight="1">
       <x:c r="A154" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B154" s="4" t="str">
-        <x:v>Bundle</x:v>
+        <x:v>Mixed / unresolved</x:v>
       </x:c>
       <x:c r="C154" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="155" ht="45" customHeight="1">
       <x:c r="A155" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B155" s="4" t="str">
-        <x:v>Cord</x:v>
+        <x:v>Shell / chitin</x:v>
       </x:c>
       <x:c r="C155" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="156" ht="45" customHeight="1">
       <x:c r="A156" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B156" s="4" t="str">
-        <x:v>Fiber</x:v>
+        <x:v>Shell and mineral</x:v>
       </x:c>
       <x:c r="C156" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="157" ht="45" customHeight="1">
       <x:c r="A157" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B157" s="4" t="str">
-        <x:v>Folio</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C157" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="158" ht="45" customHeight="1">
       <x:c r="A158" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B158" s="4" t="str">
-        <x:v>Garment</x:v>
+        <x:v>Wing membrane</x:v>
       </x:c>
       <x:c r="C158" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="159" ht="45" customHeight="1">
       <x:c r="A159" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B159" s="4" t="str">
-        <x:v>Gel</x:v>
+        <x:v>Wing membrane and frame</x:v>
       </x:c>
       <x:c r="C159" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="45" customHeight="1">
@@ -22217,7 +23007,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B160" s="4" t="str">
-        <x:v>Liquid</x:v>
+        <x:v>Assembly</x:v>
       </x:c>
       <x:c r="C160" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22228,7 +23018,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B161" s="4" t="str">
-        <x:v>Membrane</x:v>
+        <x:v>Bundle</x:v>
       </x:c>
       <x:c r="C161" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22239,7 +23029,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B162" s="4" t="str">
-        <x:v>Panel</x:v>
+        <x:v>Cord</x:v>
       </x:c>
       <x:c r="C162" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22250,7 +23040,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B163" s="4" t="str">
-        <x:v>Particles</x:v>
+        <x:v>Fiber</x:v>
       </x:c>
       <x:c r="C163" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22261,7 +23051,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B164" s="4" t="str">
-        <x:v>Paste</x:v>
+        <x:v>Folio</x:v>
       </x:c>
       <x:c r="C164" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22272,7 +23062,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B165" s="4" t="str">
-        <x:v>Patch</x:v>
+        <x:v>Garment</x:v>
       </x:c>
       <x:c r="C165" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22283,7 +23073,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B166" s="4" t="str">
-        <x:v>Rock</x:v>
+        <x:v>Gel</x:v>
       </x:c>
       <x:c r="C166" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22294,7 +23084,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B167" s="4" t="str">
-        <x:v>Sheet</x:v>
+        <x:v>Liquid</x:v>
       </x:c>
       <x:c r="C167" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22305,7 +23095,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B168" s="4" t="str">
-        <x:v>Shell plate</x:v>
+        <x:v>Membrane</x:v>
       </x:c>
       <x:c r="C168" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22316,7 +23106,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B169" s="4" t="str">
-        <x:v>Solid part</x:v>
+        <x:v>Panel</x:v>
       </x:c>
       <x:c r="C169" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22327,7 +23117,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B170" s="4" t="str">
-        <x:v>Solid piece</x:v>
+        <x:v>Particles</x:v>
       </x:c>
       <x:c r="C170" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22338,7 +23128,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B171" s="4" t="str">
-        <x:v>Strip</x:v>
+        <x:v>Paste</x:v>
       </x:c>
       <x:c r="C171" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22349,7 +23139,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B172" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Patch</x:v>
       </x:c>
       <x:c r="C172" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -22357,63 +23147,140 @@
     </x:row>
     <x:row r="173" ht="45" customHeight="1">
       <x:c r="A173" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B173" s="4" t="str">
-        <x:v>Author direction</x:v>
+        <x:v>Rock</x:v>
       </x:c>
       <x:c r="C173" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="174" ht="45" customHeight="1">
       <x:c r="A174" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B174" s="4" t="str">
-        <x:v>Existing definition</x:v>
+        <x:v>Sheet</x:v>
       </x:c>
       <x:c r="C174" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="175" ht="45" customHeight="1">
       <x:c r="A175" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B175" s="4" t="str">
-        <x:v>Proposal</x:v>
+        <x:v>Shell plate</x:v>
       </x:c>
       <x:c r="C175" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="176" ht="45" customHeight="1">
       <x:c r="A176" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B176" s="4" t="str">
-        <x:v>Source proposal</x:v>
+        <x:v>Solid part</x:v>
       </x:c>
       <x:c r="C176" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="45" customHeight="1">
       <x:c r="A177" s="4" t="str">
+        <x:v>Physical form</x:v>
+      </x:c>
+      <x:c r="B177" s="4" t="str">
+        <x:v>Solid piece</x:v>
+      </x:c>
+      <x:c r="C177" s="4" t="str">
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="45" customHeight="1">
+      <x:c r="A178" s="4" t="str">
+        <x:v>Physical form</x:v>
+      </x:c>
+      <x:c r="B178" s="4" t="str">
+        <x:v>Strip</x:v>
+      </x:c>
+      <x:c r="C178" s="4" t="str">
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="45" customHeight="1">
+      <x:c r="A179" s="4" t="str">
+        <x:v>Physical form</x:v>
+      </x:c>
+      <x:c r="B179" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="C179" s="4" t="str">
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="45" customHeight="1">
+      <x:c r="A180" s="4" t="str">
         <x:v>Design status</x:v>
       </x:c>
-      <x:c r="B177" s="4" t="str">
+      <x:c r="B180" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="C180" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="45" customHeight="1">
+      <x:c r="A181" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B181" s="4" t="str">
+        <x:v>Existing definition</x:v>
+      </x:c>
+      <x:c r="C181" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="45" customHeight="1">
+      <x:c r="A182" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B182" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="C182" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="45" customHeight="1">
+      <x:c r="A183" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B183" s="4" t="str">
+        <x:v>Source proposal</x:v>
+      </x:c>
+      <x:c r="C183" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="45" customHeight="1">
+      <x:c r="A184" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B184" s="4" t="str">
         <x:v>Withheld assumption</x:v>
       </x:c>
-      <x:c r="C177" s="4" t="str">
+      <x:c r="C184" s="4" t="str">
         <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fb3b42a70bc4a02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd675c714a04c495e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29641,21 +30508,449 @@
         <x:v>Proposed industrial use. Exact compatibility, properties and refinement unresolved.</x:v>
       </x:c>
     </x:row>
+    <x:row r="322" ht="65" customHeight="1">
+      <x:c r="A322" s="4" t="str">
+        <x:v>proposal.wind.turbine</x:v>
+      </x:c>
+      <x:c r="B322" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A322,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Salvaged wind turbine</x:v>
+      </x:c>
+      <x:c r="C322" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A322,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D322" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E322" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A322,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Wind power</x:v>
+      </x:c>
+      <x:c r="F322" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="323" ht="65" customHeight="1">
+      <x:c r="A323" s="4" t="str">
+        <x:v>proposal.wind.turbine</x:v>
+      </x:c>
+      <x:c r="B323" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A323,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Salvaged wind turbine</x:v>
+      </x:c>
+      <x:c r="C323" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A323,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D323" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E323" s="4" t="str">
+        <x:v>Machinery drive</x:v>
+      </x:c>
+      <x:c r="F323" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="324" ht="65" customHeight="1">
+      <x:c r="A324" s="4" t="str">
+        <x:v>proposal.wind.sail_panel</x:v>
+      </x:c>
+      <x:c r="B324" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A324,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared insect-wing sail panel</x:v>
+      </x:c>
+      <x:c r="C324" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A324,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D324" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E324" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A324,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Wind propulsion</x:v>
+      </x:c>
+      <x:c r="F324" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="325" ht="65" customHeight="1">
+      <x:c r="A325" s="4" t="str">
+        <x:v>proposal.wind.hand_sail</x:v>
+      </x:c>
+      <x:c r="B325" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A325,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Collapsible handheld wind sail</x:v>
+      </x:c>
+      <x:c r="C325" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A325,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D325" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E325" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A325,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Wind propulsion</x:v>
+      </x:c>
+      <x:c r="F325" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="326" ht="65" customHeight="1">
+      <x:c r="A326" s="4" t="str">
+        <x:v>proposal.wind.hand_sail</x:v>
+      </x:c>
+      <x:c r="B326" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A326,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Collapsible handheld wind sail</x:v>
+      </x:c>
+      <x:c r="C326" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A326,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D326" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E326" s="4" t="str">
+        <x:v>Traversal</x:v>
+      </x:c>
+      <x:c r="F326" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="327" ht="65" customHeight="1">
+      <x:c r="A327" s="4" t="str">
+        <x:v>proposal.wind.dirtboard</x:v>
+      </x:c>
+      <x:c r="B327" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A327,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Four-wheel all-terrain dirtboard</x:v>
+      </x:c>
+      <x:c r="C327" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A327,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D327" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E327" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A327,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Traversal</x:v>
+      </x:c>
+      <x:c r="F327" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="328" ht="65" customHeight="1">
+      <x:c r="A328" s="4" t="str">
+        <x:v>proposal.wind.dirtboard</x:v>
+      </x:c>
+      <x:c r="B328" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A328,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Four-wheel all-terrain dirtboard</x:v>
+      </x:c>
+      <x:c r="C328" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A328,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D328" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E328" s="4" t="str">
+        <x:v>Wind propulsion</x:v>
+      </x:c>
+      <x:c r="F328" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="329" ht="65" customHeight="1">
+      <x:c r="A329" s="4" t="str">
+        <x:v>proposal.wind.folding_frame</x:v>
+      </x:c>
+      <x:c r="B329" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A329,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Collapsible sail frame</x:v>
+      </x:c>
+      <x:c r="C329" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A329,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D329" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E329" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A329,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="F329" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="330" ht="65" customHeight="1">
+      <x:c r="A330" s="4" t="str">
+        <x:v>proposal.wind.sail_grip</x:v>
+      </x:c>
+      <x:c r="B330" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A330,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Hand-sail grip assembly</x:v>
+      </x:c>
+      <x:c r="C330" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A330,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D330" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E330" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A330,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="F330" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="331" ht="65" customHeight="1">
+      <x:c r="A331" s="4" t="str">
+        <x:v>proposal.wind.sail_grip</x:v>
+      </x:c>
+      <x:c r="B331" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A331,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Hand-sail grip assembly</x:v>
+      </x:c>
+      <x:c r="C331" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A331,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D331" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E331" s="4" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F331" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="332" ht="65" customHeight="1">
+      <x:c r="A332" s="4" t="str">
+        <x:v>proposal.wind.wheel</x:v>
+      </x:c>
+      <x:c r="B332" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A332,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dirtboard wheel assembly</x:v>
+      </x:c>
+      <x:c r="C332" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A332,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D332" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E332" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A332,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="F332" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="333" ht="65" customHeight="1">
+      <x:c r="A333" s="4" t="str">
+        <x:v>proposal.wind.wheel</x:v>
+      </x:c>
+      <x:c r="B333" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A333,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dirtboard wheel assembly</x:v>
+      </x:c>
+      <x:c r="C333" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A333,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D333" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E333" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F333" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="334" ht="65" customHeight="1">
+      <x:c r="A334" s="4" t="str">
+        <x:v>proposal.wind.truck</x:v>
+      </x:c>
+      <x:c r="B334" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A334,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dirtboard axle / steering assembly</x:v>
+      </x:c>
+      <x:c r="C334" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A334,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D334" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E334" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A334,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="F334" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="335" ht="65" customHeight="1">
+      <x:c r="A335" s="4" t="str">
+        <x:v>proposal.wind.truck</x:v>
+      </x:c>
+      <x:c r="B335" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A335,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dirtboard axle / steering assembly</x:v>
+      </x:c>
+      <x:c r="C335" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A335,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D335" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E335" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F335" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="336" ht="65" customHeight="1">
+      <x:c r="A336" s="4" t="str">
+        <x:v>proposal.wind.rotor</x:v>
+      </x:c>
+      <x:c r="B336" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A336,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Salvaged turbine rotor assembly</x:v>
+      </x:c>
+      <x:c r="C336" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A336,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D336" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E336" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A336,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="F336" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="337" ht="65" customHeight="1">
+      <x:c r="A337" s="4" t="str">
+        <x:v>proposal.wind.rotor</x:v>
+      </x:c>
+      <x:c r="B337" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A337,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Salvaged turbine rotor assembly</x:v>
+      </x:c>
+      <x:c r="C337" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A337,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D337" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E337" s="4" t="str">
+        <x:v>Wind power</x:v>
+      </x:c>
+      <x:c r="F337" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="338" ht="65" customHeight="1">
+      <x:c r="A338" s="4" t="str">
+        <x:v>proposal.wind.generator</x:v>
+      </x:c>
+      <x:c r="B338" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A338,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Salvaged generator assembly</x:v>
+      </x:c>
+      <x:c r="C338" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A338,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D338" s="4" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E338" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A338,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Energy processing</x:v>
+      </x:c>
+      <x:c r="F338" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="339" ht="65" customHeight="1">
+      <x:c r="A339" s="4" t="str">
+        <x:v>proposal.wind.generator</x:v>
+      </x:c>
+      <x:c r="B339" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A339,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Salvaged generator assembly</x:v>
+      </x:c>
+      <x:c r="C339" s="4" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A339,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D339" s="4" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E339" s="4" t="str">
+        <x:v>Wind power</x:v>
+      </x:c>
+      <x:c r="F339" s="4" t="str">
+        <x:v>Author-directed family or proposed component. Runtime movement and energy behavior undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="340" ht="65" customHeight="1">
+      <x:c r="A340" s="3" t="str">
+        <x:v>proposal.bio.inner_wing</x:v>
+      </x:c>
+      <x:c r="B340" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A340,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Delicate inner wing</x:v>
+      </x:c>
+      <x:c r="C340" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A340,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D340" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E340" s="3" t="str">
+        <x:v>Wind propulsion</x:v>
+      </x:c>
+      <x:c r="F340" s="3" t="str">
+        <x:v>Author direction: delicate insectoid wings supply sails as well as shade material.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A6:A1005">
-      <x:formula1>'Items'!$A$6:$A$234</x:formula1>
+      <x:formula1>'Items'!$A$6:$A$244</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D6:D1005">
       <x:formula1>"Primary,Secondary"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E6:E1005">
-      <x:formula1>'Taxonomy'!$B$54:$B$122</x:formula1>
+      <x:formula1>'Taxonomy'!$B$56:$B$128</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R870c405a556f47df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd51cfacb15740df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30563,7 +31858,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8d4d0fb74da455a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8b691af0cd34e7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30929,7 +32224,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re22361b4452c457f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31eaca0734394a69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30990,7 +32285,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>43</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>Existing gear plus armor, carriers, rare eyewear/headwear and very rare fashion families</x:v>
@@ -31035,7 +32330,7 @@
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A9)</x:f>
-        <x:v>41</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>Existing salvage and proposed materials, including husk-fiber paper and difficult pressed textiles</x:v>
@@ -31413,10 +32708,25 @@
         <x:v>Reuse existing raw joint secretion and graphite flakes. Industrial lubricant is distinct from adhesives, sealant, food and conductive gel.</x:v>
       </x:c>
     </x:row>
+    <x:row r="35" ht="115" customHeight="1">
+      <x:c r="A35" s="3" t="str">
+        <x:v>Wind gear and machines</x:v>
+      </x:c>
+      <x:c r="B35" s="3" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Wind machine")+COUNTIF(Items!$D$6:$D$1005,"Wind sail material")+COUNTIF(Items!$D$6:$D$1005,"Wind traversal gear")+COUNTIF(Items!$D$6:$D$1005,"Wind sail component")+COUNTIF(Items!$D$6:$D$1005,"Dirtboard component")+COUNTIF(Items!$D$6:$D$1005,"Wind machine component")</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C35" s="3" t="str">
+        <x:v>Salvaged turbine; wing sail panel; collapsible handheld sail; four-wheel dirtboard; proposed frame, grip, wheels, steering, rotor and generator parts</x:v>
+      </x:c>
+      <x:c r="D35" s="3" t="str">
+        <x:v>Existing delicate inner-wing resource gains sail use. Author-directed equipment is catalog design; assembly, movement and energy conversion remain unimplemented.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf15802da327a4d21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ed05bc06191421d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31479,7 +32789,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>229 design entries: 18 existing item IDs and 211 design/source concepts. Eight faunal lubricant intermediates and products proposed.</x:v>
+        <x:v>239 design entries: 18 existing item IDs and 221 design/source concepts. Wind turbine, sail, four-wheel dirtboard and component families added.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -32191,7 +33501,7 @@
         <x:v>Filtering the master</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Items is one native filterable table, A5:AE234. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
+        <x:v>Items is one native filterable table, A5:AE244. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="85" customHeight="1">
@@ -32426,10 +33736,50 @@
         <x:v>Use existing marked bottles/jars and fitted transfer tools. Segregate chemical-processing and food-service vessels. Filter cake, clot residue and rejected fractions are waste streams requiring design, not automatic valuable new items. Lubricants remain potentially toxic and unsuitable as food.</x:v>
       </x:c>
     </x:row>
+    <x:row r="127" ht="105" customHeight="1">
+      <x:c r="A127" s="4" t="str">
+        <x:v>Wing-sail direction</x:v>
+      </x:c>
+      <x:c r="B127" s="4" t="str">
+        <x:v>Author directs sails made from delicate insectoid wings. Reuse existing raw inner-wing item. Prepared sail panel and prepared shade panel distinguish service requirements; shared preparation versus separate products remains open. Metal/salvaged supporting frames avoid assuming ordinary cloth.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="105" customHeight="1">
+      <x:c r="A128" s="4" t="str">
+        <x:v>Booter wind traversal</x:v>
+      </x:c>
+      <x:c r="B128" s="4" t="str">
+        <x:v>Author directs a collapsible handheld sail and four-wheel all-terrain dirtboard for Booter to sail across large flat areas. The sail is one item with carried/deployed configurations; board and sail have separate ownership. Buddha in the spoken brief is interpreted as Booter.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="105" customHeight="1">
+      <x:c r="A129" s="4" t="str">
+        <x:v>Traversal design questions</x:v>
+      </x:c>
+      <x:c r="B129" s="4" t="str">
+        <x:v>Wind direction/strength, sail handling, steering, braking, traction, wheel material, slopes, rough-terrain limits, deployment, hand occupancy, storage, damage and cargo load remain design work. No speed, bindings, brake hardware, equipment slot or runtime vehicle controller is approved by this catalog update.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="105" customHeight="1">
+      <x:c r="A130" s="4" t="str">
+        <x:v>Wind power and salvage</x:v>
+      </x:c>
+      <x:c r="B130" s="4" t="str">
+        <x:v>Author directs turbines made from fallen/salvaged parts. Rotor design, installation and useful output remain open. Optional generator is a proposed component; wind need not produce Arc Energy or charge existing batteries. Existing drive salvage may support later craft design.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="105" customHeight="1">
+      <x:c r="A131" s="4" t="str">
+        <x:v>World and partnership scope</x:v>
+      </x:c>
+      <x:c r="B131" s="4" t="str">
+        <x:v>Catalog/document work only; no generated placement, world identity, unload/reload, persistence or terrain change occurs. Future placed machines and deployable gear will need stable ownership and saved state on the fixed, always-loaded terrain. Booter board travel does not change the Legger into a vehicle or give it remote cargo access.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93578bfedbca42c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1369f2baa07443c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33273,7 +34623,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bfa15faebbd4bfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4c35040b966442f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33516,7 +34866,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87e6615e737d4fd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ad1958bfacc489d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33920,7 +35270,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06b33fdf586647c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04299839df864bdc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34596,7 +35946,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95a52959ce4c4ac6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3262c20f7ba846b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: brainstorm Legger rigging replacements and armor
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R3c0a606f599c44b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rdaddc019125b49e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rd4b8460b959f4bf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R73c8d592b5d949e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rd24d60e15d2a4d28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R45b7d35be5924168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R5eab30abb33546e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R082472f04ffd418f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Rfffc6a24106d4e17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R2ae2f1f1c86e4c51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R9655a3c9df924ce6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R56bf436b598440cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="R1c7d15b65a1945ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R04083613f3454fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R21470474509f4330"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rc596a779cb4e428e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R42d00a8d3f2f4d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R03cc37416e1e46ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Re52eac4c8a4e44b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R70845a9ab0c547e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R266fb9edfc7743da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Rb27f584c645d4eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R5292bf5ede2549a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R5a2307731cdc4f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R343cb6e3bd1d431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="Ra1c232f0a1f741fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,8 +476,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE244" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AE244"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE268" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AE268"/>
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F340" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F340"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F372" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F372"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -614,7 +614,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CategoriesTable" displayName="CategoriesTable" ref="A5:D36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -626,7 +626,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B137" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -986,7 +986,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>239 entries. Wind machines, collapsible wing sails and four-wheel dirtboard gear classified in W:AC; search terms in AD.</x:v>
+        <x:v>263 entries. Legger cargo rigging, chassis, replacements, service parts and armor are classified proposals. Search Legger or filter Subtype.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -20096,6 +20096,1910 @@
       </x:c>
       <x:c r="AE244" s="4" t="str">
         <x:v>Author direction for equipment families; proposed components and unimplemented behavior remain explicitly separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="115" customHeight="1">
+      <x:c r="A245" s="9" t="str">
+        <x:v>proposal.legger.sling</x:v>
+      </x:c>
+      <x:c r="B245" s="9" t="str">
+        <x:v>Legger cargo sling</x:v>
+      </x:c>
+      <x:c r="C245" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D245" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E245" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F245" s="9" t="str">
+        <x:v>Flexible cradle carrying a physically supported load.</x:v>
+      </x:c>
+      <x:c r="G245" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H245" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I245" s="13"/>
+      <x:c r="J245" s="15"/>
+      <x:c r="K245" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L245" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M245" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N245" s="9" t="str">
+        <x:v>Metal links, biological cord or scarce processed hide are candidates; no ordinary cloth. Cargo envelope and fit TBD.</x:v>
+      </x:c>
+      <x:c r="O245" s="17"/>
+      <x:c r="P245" s="17"/>
+      <x:c r="Q245" s="17"/>
+      <x:c r="R245" s="17"/>
+      <x:c r="S245" s="17"/>
+      <x:c r="T245" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U245" s="11"/>
+      <x:c r="V245" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W245" s="4" t="str">
+        <x:v>Carrier</x:v>
+      </x:c>
+      <x:c r="X245" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y245" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z245" s="4" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="AA245" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB245" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC245" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD245" s="4" t="str">
+        <x:v>legger cargo sling; legger cargo rigging; carrier; mixed / unresolved; cargo organization; equipment mounting; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE245" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="115" customHeight="1">
+      <x:c r="A246" s="9" t="str">
+        <x:v>proposal.legger.cradle</x:v>
+      </x:c>
+      <x:c r="B246" s="9" t="str">
+        <x:v>Legger rigid cargo cradle</x:v>
+      </x:c>
+      <x:c r="C246" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D246" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E246" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F246" s="9" t="str">
+        <x:v>Fitted frame for an awkward piece of salvage or a compatible container.</x:v>
+      </x:c>
+      <x:c r="G246" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H246" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I246" s="13"/>
+      <x:c r="J246" s="15"/>
+      <x:c r="K246" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L246" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M246" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N246" s="9" t="str">
+        <x:v>Shape-specific support differs from a flexible sling; dimensions and capacity undecided.</x:v>
+      </x:c>
+      <x:c r="O246" s="17"/>
+      <x:c r="P246" s="17"/>
+      <x:c r="Q246" s="17"/>
+      <x:c r="R246" s="17"/>
+      <x:c r="S246" s="17"/>
+      <x:c r="T246" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U246" s="11"/>
+      <x:c r="V246" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W246" s="4" t="str">
+        <x:v>Carrier</x:v>
+      </x:c>
+      <x:c r="X246" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y246" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z246" s="4" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="AA246" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB246" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC246" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD246" s="4" t="str">
+        <x:v>legger rigid cargo cradle; legger cargo rigging; carrier; metal; cargo organization; equipment mounting; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE246" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="115" customHeight="1">
+      <x:c r="A247" s="9" t="str">
+        <x:v>proposal.legger.anchors</x:v>
+      </x:c>
+      <x:c r="B247" s="9" t="str">
+        <x:v>Legger lashing-anchor set</x:v>
+      </x:c>
+      <x:c r="C247" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D247" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E247" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F247" s="9" t="str">
+        <x:v>Attachment eyes and retainers for a chosen cargo rig.</x:v>
+      </x:c>
+      <x:c r="G247" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H247" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I247" s="13"/>
+      <x:c r="J247" s="15"/>
+      <x:c r="K247" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L247" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M247" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N247" s="9" t="str">
+        <x:v>Anchor geometry, fastening and loads unresolved; item is a set with quantity not yet defined.</x:v>
+      </x:c>
+      <x:c r="O247" s="17"/>
+      <x:c r="P247" s="17"/>
+      <x:c r="Q247" s="17"/>
+      <x:c r="R247" s="17"/>
+      <x:c r="S247" s="17"/>
+      <x:c r="T247" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U247" s="11"/>
+      <x:c r="V247" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W247" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X247" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y247" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z247" s="4" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="AA247" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB247" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC247" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD247" s="4" t="str">
+        <x:v>legger lashing-anchor set; legger cargo rigging; crafting component; metal; equipment mounting; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE247" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="115" customHeight="1">
+      <x:c r="A248" s="9" t="str">
+        <x:v>proposal.legger.balance_link</x:v>
+      </x:c>
+      <x:c r="B248" s="9" t="str">
+        <x:v>Legger load-balance linkage</x:v>
+      </x:c>
+      <x:c r="C248" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D248" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E248" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F248" s="9" t="str">
+        <x:v>Mechanical linkage candidate to distribute a supported cargo load.</x:v>
+      </x:c>
+      <x:c r="G248" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H248" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I248" s="13"/>
+      <x:c r="J248" s="15"/>
+      <x:c r="K248" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L248" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M248" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N248" s="9" t="str">
+        <x:v>A design goal rather than active self-balancing behavior; no increased capacity or stability stat assigned.</x:v>
+      </x:c>
+      <x:c r="O248" s="17"/>
+      <x:c r="P248" s="17"/>
+      <x:c r="Q248" s="17"/>
+      <x:c r="R248" s="17"/>
+      <x:c r="S248" s="17"/>
+      <x:c r="T248" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U248" s="11"/>
+      <x:c r="V248" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W248" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X248" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y248" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z248" s="4" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="AA248" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB248" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC248" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD248" s="4" t="str">
+        <x:v>legger load-balance linkage; legger cargo rigging; crafting component; metal; cargo organization; equipment mounting; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE248" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="115" customHeight="1">
+      <x:c r="A249" s="9" t="str">
+        <x:v>proposal.legger.iron_rib</x:v>
+      </x:c>
+      <x:c r="B249" s="9" t="str">
+        <x:v>Iron chassis replacement rib</x:v>
+      </x:c>
+      <x:c r="C249" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D249" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E249" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F249" s="9" t="str">
+        <x:v>Locally worked iron replacement for a selected damaged chassis member.</x:v>
+      </x:c>
+      <x:c r="G249" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H249" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I249" s="13"/>
+      <x:c r="J249" s="15"/>
+      <x:c r="K249" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L249" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M249" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N249" s="9" t="str">
+        <x:v>Geometry, weight and compatibility must match the selected host; iron is not an automatic drop-in substitute.</x:v>
+      </x:c>
+      <x:c r="O249" s="17"/>
+      <x:c r="P249" s="17"/>
+      <x:c r="Q249" s="17"/>
+      <x:c r="R249" s="17"/>
+      <x:c r="S249" s="17"/>
+      <x:c r="T249" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U249" s="11"/>
+      <x:c r="V249" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W249" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X249" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y249" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z249" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA249" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB249" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC249" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD249" s="4" t="str">
+        <x:v>iron chassis replacement rib; legger chassis; crafting component; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE249" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="115" customHeight="1">
+      <x:c r="A250" s="9" t="str">
+        <x:v>proposal.legger.crossbrace</x:v>
+      </x:c>
+      <x:c r="B250" s="9" t="str">
+        <x:v>Chassis crossbrace</x:v>
+      </x:c>
+      <x:c r="C250" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D250" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E250" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F250" s="9" t="str">
+        <x:v>Brace joining selected chassis members.</x:v>
+      </x:c>
+      <x:c r="G250" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H250" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I250" s="13"/>
+      <x:c r="J250" s="15"/>
+      <x:c r="K250" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L250" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M250" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N250" s="9" t="str">
+        <x:v>Mounting pattern, material grade and repair procedure TBD.</x:v>
+      </x:c>
+      <x:c r="O250" s="17"/>
+      <x:c r="P250" s="17"/>
+      <x:c r="Q250" s="17"/>
+      <x:c r="R250" s="17"/>
+      <x:c r="S250" s="17"/>
+      <x:c r="T250" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U250" s="11"/>
+      <x:c r="V250" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W250" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X250" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y250" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z250" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA250" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB250" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC250" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD250" s="4" t="str">
+        <x:v>chassis crossbrace; legger chassis; crafting component; metal; equipment repair; equipment fabrication; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE250" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="115" customHeight="1">
+      <x:c r="A251" s="9" t="str">
+        <x:v>proposal.legger.belly_pan</x:v>
+      </x:c>
+      <x:c r="B251" s="9" t="str">
+        <x:v>Legger chassis belly pan</x:v>
+      </x:c>
+      <x:c r="C251" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D251" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E251" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F251" s="9" t="str">
+        <x:v>Lower chassis cover candidate for debris and contact exposure.</x:v>
+      </x:c>
+      <x:c r="G251" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H251" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I251" s="13"/>
+      <x:c r="J251" s="15"/>
+      <x:c r="K251" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L251" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M251" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N251" s="9" t="str">
+        <x:v>Clearance, access and actual protection remain undecided.</x:v>
+      </x:c>
+      <x:c r="O251" s="17"/>
+      <x:c r="P251" s="17"/>
+      <x:c r="Q251" s="17"/>
+      <x:c r="R251" s="17"/>
+      <x:c r="S251" s="17"/>
+      <x:c r="T251" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U251" s="11"/>
+      <x:c r="V251" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W251" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X251" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y251" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z251" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA251" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB251" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC251" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD251" s="4" t="str">
+        <x:v>legger chassis belly pan; legger chassis; armor; metal; protection; dust exclusion; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE251" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="115" customHeight="1">
+      <x:c r="A252" s="9" t="str">
+        <x:v>proposal.legger.mount_rail</x:v>
+      </x:c>
+      <x:c r="B252" s="9" t="str">
+        <x:v>Legger attachment rail</x:v>
+      </x:c>
+      <x:c r="C252" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D252" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E252" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F252" s="9" t="str">
+        <x:v>Standardized mounting surface candidate for selected Legger attachments.</x:v>
+      </x:c>
+      <x:c r="G252" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H252" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I252" s="13"/>
+      <x:c r="J252" s="15"/>
+      <x:c r="K252" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L252" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M252" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N252" s="9" t="str">
+        <x:v>Compatibility is a future design choice; does not create universal sockets or unlimited attachments.</x:v>
+      </x:c>
+      <x:c r="O252" s="17"/>
+      <x:c r="P252" s="17"/>
+      <x:c r="Q252" s="17"/>
+      <x:c r="R252" s="17"/>
+      <x:c r="S252" s="17"/>
+      <x:c r="T252" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U252" s="11"/>
+      <x:c r="V252" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W252" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X252" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y252" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z252" s="4" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="AA252" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB252" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC252" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD252" s="4" t="str">
+        <x:v>legger attachment rail; legger chassis; crafting component; metal; equipment mounting; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE252" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="115" customHeight="1">
+      <x:c r="A253" s="9" t="str">
+        <x:v>proposal.legger.joint_bush</x:v>
+      </x:c>
+      <x:c r="B253" s="9" t="str">
+        <x:v>Iron joint bushing</x:v>
+      </x:c>
+      <x:c r="C253" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D253" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E253" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F253" s="9" t="str">
+        <x:v>Replaceable wear sleeve in a specifically matched joint.</x:v>
+      </x:c>
+      <x:c r="G253" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H253" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I253" s="13"/>
+      <x:c r="J253" s="15"/>
+      <x:c r="K253" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L253" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M253" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N253" s="9" t="str">
+        <x:v>Material grade, fit and lubrication are unresolved; separate from a full bearing cassette.</x:v>
+      </x:c>
+      <x:c r="O253" s="17"/>
+      <x:c r="P253" s="17"/>
+      <x:c r="Q253" s="17"/>
+      <x:c r="R253" s="17"/>
+      <x:c r="S253" s="17"/>
+      <x:c r="T253" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U253" s="11"/>
+      <x:c r="V253" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W253" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X253" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y253" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z253" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA253" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB253" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC253" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD253" s="4" t="str">
+        <x:v>iron joint bushing; legger mechanical parts; crafting component; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE253" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="115" customHeight="1">
+      <x:c r="A254" s="9" t="str">
+        <x:v>proposal.legger.bearing</x:v>
+      </x:c>
+      <x:c r="B254" s="9" t="str">
+        <x:v>Replacement bearing assembly</x:v>
+      </x:c>
+      <x:c r="C254" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D254" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E254" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F254" s="9" t="str">
+        <x:v>Locally serviceable bearing assembly for a selected mechanical joint.</x:v>
+      </x:c>
+      <x:c r="G254" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H254" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I254" s="13"/>
+      <x:c r="J254" s="15"/>
+      <x:c r="K254" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L254" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M254" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N254" s="9" t="str">
+        <x:v>Load, geometry, grit exclusion and suitable lubricant TBD; no bearing standard assumed.</x:v>
+      </x:c>
+      <x:c r="O254" s="17"/>
+      <x:c r="P254" s="17"/>
+      <x:c r="Q254" s="17"/>
+      <x:c r="R254" s="17"/>
+      <x:c r="S254" s="17"/>
+      <x:c r="T254" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U254" s="11"/>
+      <x:c r="V254" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W254" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X254" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y254" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z254" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA254" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB254" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC254" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD254" s="4" t="str">
+        <x:v>replacement bearing assembly; legger mechanical parts; crafting component; mixed / unresolved; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE254" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255" ht="115" customHeight="1">
+      <x:c r="A255" s="9" t="str">
+        <x:v>proposal.legger.foot_plate</x:v>
+      </x:c>
+      <x:c r="B255" s="9" t="str">
+        <x:v>Replaceable foot contact plate</x:v>
+      </x:c>
+      <x:c r="C255" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D255" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E255" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F255" s="9" t="str">
+        <x:v>Wear plate at an existing foot-ground contact surface.</x:v>
+      </x:c>
+      <x:c r="G255" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H255" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I255" s="13"/>
+      <x:c r="J255" s="15"/>
+      <x:c r="K255" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L255" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M255" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N255" s="9" t="str">
+        <x:v>Foot anatomy and attachment need inspection before implementation; traction and ground effects unassigned.</x:v>
+      </x:c>
+      <x:c r="O255" s="17"/>
+      <x:c r="P255" s="17"/>
+      <x:c r="Q255" s="17"/>
+      <x:c r="R255" s="17"/>
+      <x:c r="S255" s="17"/>
+      <x:c r="T255" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U255" s="11"/>
+      <x:c r="V255" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W255" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X255" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y255" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z255" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA255" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB255" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC255" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD255" s="4" t="str">
+        <x:v>replaceable foot contact plate; legger mechanical parts; crafting component; metal; equipment repair; traversal; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE255" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256" ht="115" customHeight="1">
+      <x:c r="A256" s="9" t="str">
+        <x:v>proposal.legger.actuator_rod</x:v>
+      </x:c>
+      <x:c r="B256" s="9" t="str">
+        <x:v>Replacement actuator link</x:v>
+      </x:c>
+      <x:c r="C256" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D256" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E256" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F256" s="9" t="str">
+        <x:v>Mechanical link candidate within a compatible existing movement assembly.</x:v>
+      </x:c>
+      <x:c r="G256" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H256" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I256" s="13"/>
+      <x:c r="J256" s="15"/>
+      <x:c r="K256" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L256" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M256" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N256" s="9" t="str">
+        <x:v>Does not establish hydraulic, pneumatic or electric actuation; host mechanism remains TBD.</x:v>
+      </x:c>
+      <x:c r="O256" s="17"/>
+      <x:c r="P256" s="17"/>
+      <x:c r="Q256" s="17"/>
+      <x:c r="R256" s="17"/>
+      <x:c r="S256" s="17"/>
+      <x:c r="T256" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U256" s="11"/>
+      <x:c r="V256" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W256" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X256" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y256" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z256" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA256" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB256" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC256" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD256" s="4" t="str">
+        <x:v>replacement actuator link; legger mechanical parts; crafting component; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE256" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257" ht="115" customHeight="1">
+      <x:c r="A257" s="9" t="str">
+        <x:v>proposal.legger.joint_shroud</x:v>
+      </x:c>
+      <x:c r="B257" s="9" t="str">
+        <x:v>Joint dust shroud</x:v>
+      </x:c>
+      <x:c r="C257" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D257" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E257" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F257" s="9" t="str">
+        <x:v>Protective cover candidate around a moving joint.</x:v>
+      </x:c>
+      <x:c r="G257" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H257" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I257" s="13"/>
+      <x:c r="J257" s="15"/>
+      <x:c r="K257" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L257" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M257" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N257" s="9" t="str">
+        <x:v>Selected membrane or segmented metal geometry; no rubber or cloth supply presumed.</x:v>
+      </x:c>
+      <x:c r="O257" s="17"/>
+      <x:c r="P257" s="17"/>
+      <x:c r="Q257" s="17"/>
+      <x:c r="R257" s="17"/>
+      <x:c r="S257" s="17"/>
+      <x:c r="T257" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U257" s="11"/>
+      <x:c r="V257" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W257" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X257" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y257" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z257" s="4" t="str">
+        <x:v>Dust exclusion</x:v>
+      </x:c>
+      <x:c r="AA257" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB257" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC257" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD257" s="4" t="str">
+        <x:v>joint dust shroud; legger service parts; crafting component; mixed / unresolved; dust exclusion; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE257" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258" ht="115" customHeight="1">
+      <x:c r="A258" s="9" t="str">
+        <x:v>proposal.legger.grease_cup</x:v>
+      </x:c>
+      <x:c r="B258" s="9" t="str">
+        <x:v>Fitted joint lubricant cup</x:v>
+      </x:c>
+      <x:c r="C258" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D258" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E258" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F258" s="9" t="str">
+        <x:v>Small fitted reservoir candidate for a selected joint lubricant.</x:v>
+      </x:c>
+      <x:c r="G258" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H258" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I258" s="13"/>
+      <x:c r="J258" s="15"/>
+      <x:c r="K258" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L258" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M258" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N258" s="9" t="str">
+        <x:v>Supply path, dose and grease compatibility TBD. No automatic replenishment or maintenance timer.</x:v>
+      </x:c>
+      <x:c r="O258" s="17"/>
+      <x:c r="P258" s="17"/>
+      <x:c r="Q258" s="17"/>
+      <x:c r="R258" s="17"/>
+      <x:c r="S258" s="17"/>
+      <x:c r="T258" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U258" s="11"/>
+      <x:c r="V258" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W258" s="4" t="str">
+        <x:v>Container part</x:v>
+      </x:c>
+      <x:c r="X258" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y258" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z258" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="AA258" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB258" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC258" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD258" s="4" t="str">
+        <x:v>fitted joint lubricant cup; legger service parts; container part; metal; lubrication; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE258" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259" ht="115" customHeight="1">
+      <x:c r="A259" s="9" t="str">
+        <x:v>proposal.legger.seal_cartridge</x:v>
+      </x:c>
+      <x:c r="B259" s="9" t="str">
+        <x:v>Replaceable joint-seal cartridge</x:v>
+      </x:c>
+      <x:c r="C259" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D259" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E259" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F259" s="9" t="str">
+        <x:v>Serviceable dust/lubricant retention unit for a specific joint.</x:v>
+      </x:c>
+      <x:c r="G259" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H259" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I259" s="13"/>
+      <x:c r="J259" s="15"/>
+      <x:c r="K259" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L259" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M259" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N259" s="9" t="str">
+        <x:v>Different service from a survival-canister seal; materials and fit unresolved.</x:v>
+      </x:c>
+      <x:c r="O259" s="17"/>
+      <x:c r="P259" s="17"/>
+      <x:c r="Q259" s="17"/>
+      <x:c r="R259" s="17"/>
+      <x:c r="S259" s="17"/>
+      <x:c r="T259" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U259" s="11"/>
+      <x:c r="V259" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W259" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X259" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y259" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z259" s="4" t="str">
+        <x:v>Sealing</x:v>
+      </x:c>
+      <x:c r="AA259" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB259" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC259" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD259" s="4" t="str">
+        <x:v>replaceable joint-seal cartridge; legger service parts; crafting component; mixed / unresolved; sealing; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE259" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260" ht="115" customHeight="1">
+      <x:c r="A260" s="9" t="str">
+        <x:v>proposal.legger.fastener_pack</x:v>
+      </x:c>
+      <x:c r="B260" s="9" t="str">
+        <x:v>Legger service fastener pack</x:v>
+      </x:c>
+      <x:c r="C260" s="9" t="str">
+        <x:v>Field supplies</x:v>
+      </x:c>
+      <x:c r="D260" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E260" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F260" s="9" t="str">
+        <x:v>Selected matching pins, retainers and fasteners for a bounded repair job.</x:v>
+      </x:c>
+      <x:c r="G260" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H260" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I260" s="13"/>
+      <x:c r="J260" s="15"/>
+      <x:c r="K260" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L260" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M260" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N260" s="9" t="str">
+        <x:v>Pack contents and quantity TBD; no generic ability to repair every part or duplicate uncounted contents.</x:v>
+      </x:c>
+      <x:c r="O260" s="17"/>
+      <x:c r="P260" s="17"/>
+      <x:c r="Q260" s="17"/>
+      <x:c r="R260" s="17"/>
+      <x:c r="S260" s="17"/>
+      <x:c r="T260" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U260" s="11"/>
+      <x:c r="V260" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W260" s="4" t="str">
+        <x:v>Service kit</x:v>
+      </x:c>
+      <x:c r="X260" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y260" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z260" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA260" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB260" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC260" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD260" s="4" t="str">
+        <x:v>legger service fastener pack; legger service parts; service kit; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE260" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="261" ht="115" customHeight="1">
+      <x:c r="A261" s="9" t="str">
+        <x:v>proposal.legger.shell_guard</x:v>
+      </x:c>
+      <x:c r="B261" s="9" t="str">
+        <x:v>Chitin chassis guard</x:v>
+      </x:c>
+      <x:c r="C261" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D261" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E261" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F261" s="9" t="str">
+        <x:v>Worked shell panel candidate covering a selected exposed surface.</x:v>
+      </x:c>
+      <x:c r="G261" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H261" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I261" s="13"/>
+      <x:c r="J261" s="15"/>
+      <x:c r="K261" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L261" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M261" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N261" s="9" t="str">
+        <x:v>Cheap raw shell still needs fitting; no numeric protection, durability or ballistic rating.</x:v>
+      </x:c>
+      <x:c r="O261" s="17"/>
+      <x:c r="P261" s="17"/>
+      <x:c r="Q261" s="17"/>
+      <x:c r="R261" s="17"/>
+      <x:c r="S261" s="17"/>
+      <x:c r="T261" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U261" s="11"/>
+      <x:c r="V261" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W261" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X261" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y261" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z261" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA261" s="4" t="str">
+        <x:v>Shell / chitin</x:v>
+      </x:c>
+      <x:c r="AB261" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC261" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD261" s="4" t="str">
+        <x:v>chitin chassis guard; legger armor; armor; shell / chitin; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE261" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262" ht="115" customHeight="1">
+      <x:c r="A262" s="9" t="str">
+        <x:v>proposal.legger.iron_guard</x:v>
+      </x:c>
+      <x:c r="B262" s="9" t="str">
+        <x:v>Iron chassis guard</x:v>
+      </x:c>
+      <x:c r="C262" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D262" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E262" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F262" s="9" t="str">
+        <x:v>Worked iron panel candidate for a selected Legger mount.</x:v>
+      </x:c>
+      <x:c r="G262" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H262" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I262" s="13"/>
+      <x:c r="J262" s="15"/>
+      <x:c r="K262" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L262" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M262" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N262" s="9" t="str">
+        <x:v>Mass, articulation, shielding and replacement tradeoffs require design.</x:v>
+      </x:c>
+      <x:c r="O262" s="17"/>
+      <x:c r="P262" s="17"/>
+      <x:c r="Q262" s="17"/>
+      <x:c r="R262" s="17"/>
+      <x:c r="S262" s="17"/>
+      <x:c r="T262" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U262" s="11"/>
+      <x:c r="V262" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W262" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X262" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y262" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z262" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA262" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB262" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC262" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD262" s="4" t="str">
+        <x:v>iron chassis guard; legger armor; armor; metal; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE262" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263" ht="115" customHeight="1">
+      <x:c r="A263" s="9" t="str">
+        <x:v>proposal.legger.joint_guard</x:v>
+      </x:c>
+      <x:c r="B263" s="9" t="str">
+        <x:v>Articulated joint guard</x:v>
+      </x:c>
+      <x:c r="C263" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D263" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E263" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F263" s="9" t="str">
+        <x:v>Overlapping or articulated cover candidate around a moving joint.</x:v>
+      </x:c>
+      <x:c r="G263" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H263" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I263" s="13"/>
+      <x:c r="J263" s="15"/>
+      <x:c r="K263" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L263" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M263" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N263" s="9" t="str">
+        <x:v>Geometry must preserve movement and maintenance access; no proven protective effect.</x:v>
+      </x:c>
+      <x:c r="O263" s="17"/>
+      <x:c r="P263" s="17"/>
+      <x:c r="Q263" s="17"/>
+      <x:c r="R263" s="17"/>
+      <x:c r="S263" s="17"/>
+      <x:c r="T263" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U263" s="11"/>
+      <x:c r="V263" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W263" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X263" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y263" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z263" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA263" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB263" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC263" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD263" s="4" t="str">
+        <x:v>articulated joint guard; legger armor; armor; mixed / unresolved; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE263" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264" ht="115" customHeight="1">
+      <x:c r="A264" s="9" t="str">
+        <x:v>proposal.legger.ceramic_backing</x:v>
+      </x:c>
+      <x:c r="B264" s="9" t="str">
+        <x:v>Ceramic armor backing insert</x:v>
+      </x:c>
+      <x:c r="C264" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D264" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E264" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F264" s="9" t="str">
+        <x:v>Fitted ceramic backing candidate within a selected composite guard assembly.</x:v>
+      </x:c>
+      <x:c r="G264" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H264" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I264" s="13"/>
+      <x:c r="J264" s="15"/>
+      <x:c r="K264" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L264" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M264" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N264" s="9" t="str">
+        <x:v>An application of the existing ceramic-armor family; layer order, damage and service limits TBD.</x:v>
+      </x:c>
+      <x:c r="O264" s="17"/>
+      <x:c r="P264" s="17"/>
+      <x:c r="Q264" s="17"/>
+      <x:c r="R264" s="17"/>
+      <x:c r="S264" s="17"/>
+      <x:c r="T264" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U264" s="11"/>
+      <x:c r="V264" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W264" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X264" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y264" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z264" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA264" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB264" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC264" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD264" s="4" t="str">
+        <x:v>ceramic armor backing insert; legger armor; armor; ceramic; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE264" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265" ht="115" customHeight="1">
+      <x:c r="A265" s="9" t="str">
+        <x:v>proposal.legger.plasteel_rib</x:v>
+      </x:c>
+      <x:c r="B265" s="9" t="str">
+        <x:v>Ancient plasteel replacement member</x:v>
+      </x:c>
+      <x:c r="C265" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D265" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E265" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F265" s="9" t="str">
+        <x:v>Recovered plasteel structural piece considered for a compatible chassis replacement.</x:v>
+      </x:c>
+      <x:c r="G265" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H265" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I265" s="13"/>
+      <x:c r="J265" s="15"/>
+      <x:c r="K265" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L265" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M265" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N265" s="9" t="str">
+        <x:v>Extremely rare; fit, identification, rework and attachment remain unresolved. Recovery does not grant manufacture.</x:v>
+      </x:c>
+      <x:c r="O265" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P265" s="17"/>
+      <x:c r="Q265" s="17"/>
+      <x:c r="R265" s="17"/>
+      <x:c r="S265" s="17"/>
+      <x:c r="T265" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U265" s="11"/>
+      <x:c r="V265" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W265" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X265" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y265" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z265" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA265" s="4" t="str">
+        <x:v>Ancient composite</x:v>
+      </x:c>
+      <x:c r="AB265" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC265" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD265" s="4" t="str">
+        <x:v>ancient plasteel replacement member; legger ancient replacement; crafting component; ancient composite; equipment repair; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE265" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266" ht="115" customHeight="1">
+      <x:c r="A266" s="9" t="str">
+        <x:v>proposal.legger.nanocarbon_panel</x:v>
+      </x:c>
+      <x:c r="B266" s="9" t="str">
+        <x:v>Ancient nanocarbon armor panel</x:v>
+      </x:c>
+      <x:c r="C266" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D266" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E266" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F266" s="9" t="str">
+        <x:v>Recovered nanotube/nanocarbon composite protective panel candidate.</x:v>
+      </x:c>
+      <x:c r="G266" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H266" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I266" s="13"/>
+      <x:c r="J266" s="15"/>
+      <x:c r="K266" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L266" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M266" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N266" s="9" t="str">
+        <x:v>Extremely rare; ballistic response and degradation must be designed, with no automatic immunity or reproducibility.</x:v>
+      </x:c>
+      <x:c r="O266" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P266" s="17"/>
+      <x:c r="Q266" s="17"/>
+      <x:c r="R266" s="17"/>
+      <x:c r="S266" s="17"/>
+      <x:c r="T266" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U266" s="11"/>
+      <x:c r="V266" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W266" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X266" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y266" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z266" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA266" s="4" t="str">
+        <x:v>Ancient composite</x:v>
+      </x:c>
+      <x:c r="AB266" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC266" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD266" s="4" t="str">
+        <x:v>ancient nanocarbon armor panel; legger ancient replacement; armor; ancient composite; protection; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE266" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267" ht="115" customHeight="1">
+      <x:c r="A267" s="9" t="str">
+        <x:v>proposal.legger.ancient_bearing</x:v>
+      </x:c>
+      <x:c r="B267" s="9" t="str">
+        <x:v>Ancient bearing cassette</x:v>
+      </x:c>
+      <x:c r="C267" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D267" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E267" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F267" s="9" t="str">
+        <x:v>Recovered precision bearing module considered for an appropriate joint.</x:v>
+      </x:c>
+      <x:c r="G267" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H267" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I267" s="13"/>
+      <x:c r="J267" s="15"/>
+      <x:c r="K267" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L267" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M267" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N267" s="9" t="str">
+        <x:v>Extremely rare; compatibility, remaining life and ability to service it are unknown. Material makeup unspecified.</x:v>
+      </x:c>
+      <x:c r="O267" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P267" s="17"/>
+      <x:c r="Q267" s="17"/>
+      <x:c r="R267" s="17"/>
+      <x:c r="S267" s="17"/>
+      <x:c r="T267" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U267" s="11"/>
+      <x:c r="V267" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W267" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X267" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y267" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z267" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA267" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AB267" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC267" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD267" s="4" t="str">
+        <x:v>ancient bearing cassette; legger ancient replacement; crafting component; unresolved; equipment repair; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE267" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268" ht="115" customHeight="1">
+      <x:c r="A268" s="9" t="str">
+        <x:v>proposal.legger.ballistic_guard</x:v>
+      </x:c>
+      <x:c r="B268" s="9" t="str">
+        <x:v>Ancient ballistic-deflecting guard</x:v>
+      </x:c>
+      <x:c r="C268" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D268" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E268" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F268" s="9" t="str">
+        <x:v>Working concept for plasteel/nanocarbon armor intended to resist or deflect projectiles.</x:v>
+      </x:c>
+      <x:c r="G268" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H268" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I268" s="13"/>
+      <x:c r="J268" s="15"/>
+      <x:c r="K268" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L268" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M268" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N268" s="9" t="str">
+        <x:v>Extremely rare. Passive layering, geometry or another mechanism is undecided; no force-field system, guaranteed deflection or armor statistics established.</x:v>
+      </x:c>
+      <x:c r="O268" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P268" s="17"/>
+      <x:c r="Q268" s="17"/>
+      <x:c r="R268" s="17"/>
+      <x:c r="S268" s="17"/>
+      <x:c r="T268" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U268" s="11"/>
+      <x:c r="V268" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W268" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X268" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y268" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z268" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA268" s="4" t="str">
+        <x:v>Ancient composite</x:v>
+      </x:c>
+      <x:c r="AB268" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC268" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD268" s="4" t="str">
+        <x:v>ancient ballistic-deflecting guard; legger ancient replacement; armor; ancient composite; protection; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE268" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20139,7 +22043,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R906d8f39e56b4b7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbfbdf116d8a4d0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20791,7 +22695,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe7b27f3fe944253"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17d3326ef41f42eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21273,7 +23177,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56216e5a95554486"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccb776a39f17488d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23280,7 +25184,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd675c714a04c495e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ec566f944364d48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30936,10 +32840,738 @@
         <x:v>Author direction: delicate insectoid wings supply sails as well as shade material.</x:v>
       </x:c>
     </x:row>
+    <x:row r="341" ht="65" customHeight="1">
+      <x:c r="A341" s="3" t="str">
+        <x:v>proposal.legger.sling</x:v>
+      </x:c>
+      <x:c r="B341" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A341,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger cargo sling</x:v>
+      </x:c>
+      <x:c r="C341" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A341,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D341" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E341" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A341,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F341" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="342" ht="65" customHeight="1">
+      <x:c r="A342" s="3" t="str">
+        <x:v>proposal.legger.sling</x:v>
+      </x:c>
+      <x:c r="B342" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A342,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger cargo sling</x:v>
+      </x:c>
+      <x:c r="C342" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A342,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D342" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E342" s="3" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F342" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="343" ht="65" customHeight="1">
+      <x:c r="A343" s="3" t="str">
+        <x:v>proposal.legger.cradle</x:v>
+      </x:c>
+      <x:c r="B343" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A343,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger rigid cargo cradle</x:v>
+      </x:c>
+      <x:c r="C343" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A343,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D343" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E343" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A343,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F343" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="344" ht="65" customHeight="1">
+      <x:c r="A344" s="3" t="str">
+        <x:v>proposal.legger.cradle</x:v>
+      </x:c>
+      <x:c r="B344" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A344,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger rigid cargo cradle</x:v>
+      </x:c>
+      <x:c r="C344" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A344,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D344" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E344" s="3" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F344" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="345" ht="65" customHeight="1">
+      <x:c r="A345" s="3" t="str">
+        <x:v>proposal.legger.anchors</x:v>
+      </x:c>
+      <x:c r="B345" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A345,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger lashing-anchor set</x:v>
+      </x:c>
+      <x:c r="C345" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A345,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D345" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E345" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A345,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F345" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="346" ht="65" customHeight="1">
+      <x:c r="A346" s="3" t="str">
+        <x:v>proposal.legger.balance_link</x:v>
+      </x:c>
+      <x:c r="B346" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A346,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger load-balance linkage</x:v>
+      </x:c>
+      <x:c r="C346" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A346,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D346" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E346" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A346,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F346" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="347" ht="65" customHeight="1">
+      <x:c r="A347" s="3" t="str">
+        <x:v>proposal.legger.balance_link</x:v>
+      </x:c>
+      <x:c r="B347" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A347,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger load-balance linkage</x:v>
+      </x:c>
+      <x:c r="C347" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A347,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D347" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E347" s="3" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F347" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="348" ht="65" customHeight="1">
+      <x:c r="A348" s="3" t="str">
+        <x:v>proposal.legger.iron_rib</x:v>
+      </x:c>
+      <x:c r="B348" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A348,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Iron chassis replacement rib</x:v>
+      </x:c>
+      <x:c r="C348" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A348,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D348" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E348" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A348,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F348" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="349" ht="65" customHeight="1">
+      <x:c r="A349" s="3" t="str">
+        <x:v>proposal.legger.crossbrace</x:v>
+      </x:c>
+      <x:c r="B349" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A349,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chassis crossbrace</x:v>
+      </x:c>
+      <x:c r="C349" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A349,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D349" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E349" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A349,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F349" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="350" ht="65" customHeight="1">
+      <x:c r="A350" s="3" t="str">
+        <x:v>proposal.legger.crossbrace</x:v>
+      </x:c>
+      <x:c r="B350" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A350,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chassis crossbrace</x:v>
+      </x:c>
+      <x:c r="C350" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A350,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D350" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E350" s="3" t="str">
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="F350" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="351" ht="65" customHeight="1">
+      <x:c r="A351" s="3" t="str">
+        <x:v>proposal.legger.belly_pan</x:v>
+      </x:c>
+      <x:c r="B351" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A351,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger chassis belly pan</x:v>
+      </x:c>
+      <x:c r="C351" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A351,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D351" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E351" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A351,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F351" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="352" ht="65" customHeight="1">
+      <x:c r="A352" s="3" t="str">
+        <x:v>proposal.legger.belly_pan</x:v>
+      </x:c>
+      <x:c r="B352" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A352,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger chassis belly pan</x:v>
+      </x:c>
+      <x:c r="C352" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A352,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D352" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E352" s="3" t="str">
+        <x:v>Dust exclusion</x:v>
+      </x:c>
+      <x:c r="F352" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="353" ht="65" customHeight="1">
+      <x:c r="A353" s="3" t="str">
+        <x:v>proposal.legger.mount_rail</x:v>
+      </x:c>
+      <x:c r="B353" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A353,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger attachment rail</x:v>
+      </x:c>
+      <x:c r="C353" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A353,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D353" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E353" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A353,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F353" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="354" ht="65" customHeight="1">
+      <x:c r="A354" s="3" t="str">
+        <x:v>proposal.legger.joint_bush</x:v>
+      </x:c>
+      <x:c r="B354" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A354,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Iron joint bushing</x:v>
+      </x:c>
+      <x:c r="C354" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A354,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D354" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E354" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A354,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F354" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355" ht="65" customHeight="1">
+      <x:c r="A355" s="3" t="str">
+        <x:v>proposal.legger.bearing</x:v>
+      </x:c>
+      <x:c r="B355" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A355,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replacement bearing assembly</x:v>
+      </x:c>
+      <x:c r="C355" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A355,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D355" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E355" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A355,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F355" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356" ht="65" customHeight="1">
+      <x:c r="A356" s="3" t="str">
+        <x:v>proposal.legger.foot_plate</x:v>
+      </x:c>
+      <x:c r="B356" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A356,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replaceable foot contact plate</x:v>
+      </x:c>
+      <x:c r="C356" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A356,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D356" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E356" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A356,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F356" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="357" ht="65" customHeight="1">
+      <x:c r="A357" s="3" t="str">
+        <x:v>proposal.legger.foot_plate</x:v>
+      </x:c>
+      <x:c r="B357" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A357,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replaceable foot contact plate</x:v>
+      </x:c>
+      <x:c r="C357" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A357,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D357" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E357" s="3" t="str">
+        <x:v>Traversal</x:v>
+      </x:c>
+      <x:c r="F357" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358" ht="65" customHeight="1">
+      <x:c r="A358" s="3" t="str">
+        <x:v>proposal.legger.actuator_rod</x:v>
+      </x:c>
+      <x:c r="B358" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A358,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replacement actuator link</x:v>
+      </x:c>
+      <x:c r="C358" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A358,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D358" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E358" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A358,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F358" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="359" ht="65" customHeight="1">
+      <x:c r="A359" s="3" t="str">
+        <x:v>proposal.legger.joint_shroud</x:v>
+      </x:c>
+      <x:c r="B359" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A359,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Joint dust shroud</x:v>
+      </x:c>
+      <x:c r="C359" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A359,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D359" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E359" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A359,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dust exclusion</x:v>
+      </x:c>
+      <x:c r="F359" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="360" ht="65" customHeight="1">
+      <x:c r="A360" s="3" t="str">
+        <x:v>proposal.legger.joint_shroud</x:v>
+      </x:c>
+      <x:c r="B360" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A360,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Joint dust shroud</x:v>
+      </x:c>
+      <x:c r="C360" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A360,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D360" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E360" s="3" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F360" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="361" ht="65" customHeight="1">
+      <x:c r="A361" s="3" t="str">
+        <x:v>proposal.legger.grease_cup</x:v>
+      </x:c>
+      <x:c r="B361" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A361,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Fitted joint lubricant cup</x:v>
+      </x:c>
+      <x:c r="C361" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A361,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D361" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E361" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A361,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F361" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362" ht="65" customHeight="1">
+      <x:c r="A362" s="3" t="str">
+        <x:v>proposal.legger.seal_cartridge</x:v>
+      </x:c>
+      <x:c r="B362" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A362,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replaceable joint-seal cartridge</x:v>
+      </x:c>
+      <x:c r="C362" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A362,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D362" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E362" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A362,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Sealing</x:v>
+      </x:c>
+      <x:c r="F362" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="363" ht="65" customHeight="1">
+      <x:c r="A363" s="3" t="str">
+        <x:v>proposal.legger.seal_cartridge</x:v>
+      </x:c>
+      <x:c r="B363" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A363,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replaceable joint-seal cartridge</x:v>
+      </x:c>
+      <x:c r="C363" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A363,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D363" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E363" s="3" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F363" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="364" ht="65" customHeight="1">
+      <x:c r="A364" s="3" t="str">
+        <x:v>proposal.legger.fastener_pack</x:v>
+      </x:c>
+      <x:c r="B364" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A364,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger service fastener pack</x:v>
+      </x:c>
+      <x:c r="C364" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A364,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Field supplies</x:v>
+      </x:c>
+      <x:c r="D364" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E364" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A364,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F364" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="365" ht="65" customHeight="1">
+      <x:c r="A365" s="3" t="str">
+        <x:v>proposal.legger.shell_guard</x:v>
+      </x:c>
+      <x:c r="B365" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A365,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chitin chassis guard</x:v>
+      </x:c>
+      <x:c r="C365" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A365,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D365" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E365" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A365,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F365" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="366" ht="65" customHeight="1">
+      <x:c r="A366" s="3" t="str">
+        <x:v>proposal.legger.iron_guard</x:v>
+      </x:c>
+      <x:c r="B366" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A366,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Iron chassis guard</x:v>
+      </x:c>
+      <x:c r="C366" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A366,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D366" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E366" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A366,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F366" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="367" ht="65" customHeight="1">
+      <x:c r="A367" s="3" t="str">
+        <x:v>proposal.legger.joint_guard</x:v>
+      </x:c>
+      <x:c r="B367" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A367,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Articulated joint guard</x:v>
+      </x:c>
+      <x:c r="C367" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A367,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D367" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E367" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A367,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F367" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="368" ht="65" customHeight="1">
+      <x:c r="A368" s="3" t="str">
+        <x:v>proposal.legger.ceramic_backing</x:v>
+      </x:c>
+      <x:c r="B368" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A368,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ceramic armor backing insert</x:v>
+      </x:c>
+      <x:c r="C368" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A368,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D368" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E368" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A368,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F368" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="369" ht="65" customHeight="1">
+      <x:c r="A369" s="3" t="str">
+        <x:v>proposal.legger.plasteel_rib</x:v>
+      </x:c>
+      <x:c r="B369" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A369,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient plasteel replacement member</x:v>
+      </x:c>
+      <x:c r="C369" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A369,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D369" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E369" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A369,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F369" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="370" ht="65" customHeight="1">
+      <x:c r="A370" s="3" t="str">
+        <x:v>proposal.legger.nanocarbon_panel</x:v>
+      </x:c>
+      <x:c r="B370" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A370,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient nanocarbon armor panel</x:v>
+      </x:c>
+      <x:c r="C370" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A370,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D370" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E370" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A370,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F370" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="371" ht="65" customHeight="1">
+      <x:c r="A371" s="3" t="str">
+        <x:v>proposal.legger.ancient_bearing</x:v>
+      </x:c>
+      <x:c r="B371" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A371,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient bearing cassette</x:v>
+      </x:c>
+      <x:c r="C371" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A371,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D371" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E371" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A371,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F371" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="372" ht="65" customHeight="1">
+      <x:c r="A372" s="3" t="str">
+        <x:v>proposal.legger.ballistic_guard</x:v>
+      </x:c>
+      <x:c r="B372" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A372,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient ballistic-deflecting guard</x:v>
+      </x:c>
+      <x:c r="C372" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A372,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D372" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E372" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A372,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F372" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A6:A1005">
-      <x:formula1>'Items'!$A$6:$A$244</x:formula1>
+      <x:formula1>'Items'!$A$6:$A$268</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D6:D1005">
       <x:formula1>"Primary,Secondary"</x:formula1>
@@ -30950,7 +33582,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd51cfacb15740df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb650c84453cf4e32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31858,7 +34490,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8b691af0cd34e7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b1f1157290d4092"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32224,7 +34856,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31eaca0734394a69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36c05c50b9b4462e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32285,7 +34917,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>46</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>Existing gear plus armor, carriers, rare eyewear/headwear and very rare fashion families</x:v>
@@ -32300,7 +34932,7 @@
       </x:c>
       <x:c r="B7" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A7)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C7" s="4" t="str">
         <x:v>Pop-up camp and two battery states</x:v>
@@ -32330,7 +34962,7 @@
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A9)</x:f>
-        <x:v>48</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>Existing salvage and proposed materials, including husk-fiber paper and difficult pressed textiles</x:v>
@@ -32654,7 +35286,7 @@
       </x:c>
       <x:c r="B31" s="3" t="n">
         <x:f>COUNTIF(Items!$AA$6:$AA$1005,"Ceramic")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic feed mixture")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic and metal")</x:f>
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
         <x:v>28 new ceramic-specific feeds, intermediate blanks, tableware, storage, workshop tools, thermal/electrical parts, vessel fittings, ceremonial work and protection candidates</x:v>
@@ -32723,10 +35355,25 @@
         <x:v>Existing delicate inner-wing resource gains sail use. Author-directed equipment is catalog design; assembly, movement and energy conversion remain unimplemented.</x:v>
       </x:c>
     </x:row>
+    <x:row r="36" ht="115" customHeight="1">
+      <x:c r="A36" s="3" t="str">
+        <x:v>Legger parts and fitments</x:v>
+      </x:c>
+      <x:c r="B36" s="3" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Legger cargo rigging")+COUNTIF(Items!$D$6:$D$1005,"Legger chassis")+COUNTIF(Items!$D$6:$D$1005,"Legger mechanical parts")+COUNTIF(Items!$D$6:$D$1005,"Legger service parts")+COUNTIF(Items!$D$6:$D$1005,"Legger armor")+COUNTIF(Items!$D$6:$D$1005,"Legger ancient replacement")</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C36" s="3" t="str">
+        <x:v>24 proposals across cargo rigging, chassis, mechanical parts, service parts, armor and ancient replacements</x:v>
+      </x:c>
+      <x:c r="D36" s="3" t="str">
+        <x:v>Legger-specific fit and physical ownership retained; ordinary iron repairs and extremely rare ancient replacements do not imply a linear upgrade ladder.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ed05bc06191421d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b0576aad39641e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32789,7 +35436,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>239 design entries: 18 existing item IDs and 221 design/source concepts. Wind turbine, sail, four-wheel dirtboard and component families added.</x:v>
+        <x:v>263 design entries: 18 existing item IDs and 245 design/source concepts. Includes 24 Legger fitment and replacement proposals.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -33501,7 +36148,7 @@
         <x:v>Filtering the master</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Items is one native filterable table, A5:AE244. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
+        <x:v>Items is one native filterable table, A5:AE268. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="85" customHeight="1">
@@ -33776,10 +36423,58 @@
         <x:v>Catalog/document work only; no generated placement, world identity, unload/reload, persistence or terrain change occurs. Future placed machines and deployable gear will need stable ownership and saved state on the fixed, always-loaded terrain. Booter board travel does not change the Legger into a vehicle or give it remote cargo access.</x:v>
       </x:c>
     </x:row>
+    <x:row r="132" ht="105" customHeight="1">
+      <x:c r="A132" s="4" t="str">
+        <x:v>Legger concept families</x:v>
+      </x:c>
+      <x:c r="B132" s="4" t="str">
+        <x:v>24 proposals: cargo slings/cradles/anchors/balance linkage; iron ribs/braces/covers/mount rails; bushings/bearings/foot plates/actuator links; dust shrouds/lubricant cups/seal cartridges/service fasteners; shell/iron/articulated/ceramic guards; rare ancient members, panels and bearing modules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="105" customHeight="1">
+      <x:c r="A133" s="4" t="str">
+        <x:v>Legger proposal status</x:v>
+      </x:c>
+      <x:c r="B133" s="4" t="str">
+        <x:v>The author explicitly brainstorms. Specific part list, anatomy, interfaces, geometry, attributes, recipes, quantities, maintenance and installed slots are not accepted runtime designs. Consult the actual Legger model and architecture before implementing fitted replacements.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="105" customHeight="1">
+      <x:c r="A134" s="4" t="str">
+        <x:v>Iron versus ancient</x:v>
+      </x:c>
+      <x:c r="B134" s="4" t="str">
+        <x:v>Iron repairs could be locally serviceable; ancient plasteel/nanocarbon and other recovered high-tech parts remain extremely rare. Weight, fit, availability, repairability and performance are open tradeoffs rather than a guaranteed upgrade ladder. Ancient salvage does not grant manufacturing capability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="105" customHeight="1">
+      <x:c r="A135" s="4" t="str">
+        <x:v>Ballistic armor concept</x:v>
+      </x:c>
+      <x:c r="B135" s="4" t="str">
+        <x:v>Nanotube/plasteel ballistic-repelling or deflecting armor is a working goal. Specific mechanism, layering, projectile interaction and protection remain undefined. Do not infer force fields, invulnerability, a percent deflection chance or that every ancient panel has the same property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="105" customHeight="1">
+      <x:c r="A136" s="4" t="str">
+        <x:v>Fit and reuse</x:v>
+      </x:c>
+      <x:c r="B136" s="4" t="str">
+        <x:v>Use existing raw metal, shell, ceramic and lubricant families. Host-specific finished parts differ from raw stock. Components inside an assembled Legger, spare cargo parts and removed salvage must not be counted as duplicate owned items. Filter Subtype for Legger branches or Search terms for Legger/Leger.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="105" customHeight="1">
+      <x:c r="A137" s="4" t="str">
+        <x:v>Legger world scope</x:v>
+      </x:c>
+      <x:c r="B137" s="4" t="str">
+        <x:v>Catalog work changes no world identity, chunk/terrain loading, persistent state, carrier limit or companion movement. Future installed parts need stable physical ownership, replacement/save behavior and compatibility. The Legger remains the same finite mobile carrier with local access.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1369f2baa07443c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb18fc306c55d4317"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34623,7 +37318,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4c35040b966442f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2064bc84fd74a15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34866,7 +37561,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ad1958bfacc489d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc803812decfa4bf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35270,7 +37965,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04299839df864bdc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R460f93cf9bcd4d86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35946,7 +38641,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3262c20f7ba846b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49061129120245c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: expand all six Legger item families
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R04083613f3454fd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R21470474509f4330"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="Rc596a779cb4e428e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R42d00a8d3f2f4d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R03cc37416e1e46ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Re52eac4c8a4e44b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R70845a9ab0c547e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R266fb9edfc7743da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Rb27f584c645d4eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R5292bf5ede2549a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R5a2307731cdc4f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R343cb6e3bd1d431b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="Ra1c232f0a1f741fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R99e700a71b434630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="R803d3ed2bcee47d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R834a1454682649e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R68d95eb0a9fa4eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rf33880317c06453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="Rca05e0b06c6b4c52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="Re84dba76b8814251"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R5af1967a1649474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="Rcd891f40069c4efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="Rd6a7ecd86d6041d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R4480450986514777"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R1421fd5faa0f45da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="R7f9331eb50e64578"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,8 +476,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE268" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AE268"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ItemsTable" displayName="ItemsTable" ref="A5:AE304" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AE304"/>
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F372" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F372"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F422" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F422"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -626,7 +626,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B137" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B143" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -986,7 +986,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>263 entries. Legger cargo rigging, chassis, replacements, service parts and armor are classified proposals. Search Legger or filter Subtype.</x:v>
+        <x:v>299 entries. Legger cargo rigging, chassis, replacements, service parts and armor are classified proposals. Search Legger or filter Subtype.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -21999,6 +21999,2862 @@
         <x:v>ancient ballistic-deflecting guard; legger ancient replacement; armor; ancient composite; protection; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
       </x:c>
       <x:c r="AE268" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269" ht="115" customHeight="1">
+      <x:c r="A269" s="9" t="str">
+        <x:v>proposal.legger.pannier_frame</x:v>
+      </x:c>
+      <x:c r="B269" s="9" t="str">
+        <x:v>Legger side-pannier frame</x:v>
+      </x:c>
+      <x:c r="C269" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D269" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E269" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F269" s="9" t="str">
+        <x:v>Side-mounted support for a matched bounded cargo container.</x:v>
+      </x:c>
+      <x:c r="G269" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H269" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I269" s="13"/>
+      <x:c r="J269" s="15"/>
+      <x:c r="K269" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L269" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M269" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N269" s="9" t="str">
+        <x:v>Side clearance, load placement and attachment remain open; distinct from a general cargo cradle.</x:v>
+      </x:c>
+      <x:c r="O269" s="17"/>
+      <x:c r="P269" s="17"/>
+      <x:c r="Q269" s="17"/>
+      <x:c r="R269" s="17"/>
+      <x:c r="S269" s="17"/>
+      <x:c r="T269" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U269" s="11"/>
+      <x:c r="V269" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W269" s="4" t="str">
+        <x:v>Carrier</x:v>
+      </x:c>
+      <x:c r="X269" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y269" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z269" s="4" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="AA269" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB269" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC269" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD269" s="4" t="str">
+        <x:v>legger side-pannier frame; legger cargo rigging; carrier; metal; cargo organization; equipment mounting; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE269" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="115" customHeight="1">
+      <x:c r="A270" s="9" t="str">
+        <x:v>proposal.legger.sample_rack</x:v>
+      </x:c>
+      <x:c r="B270" s="9" t="str">
+        <x:v>Legger sample-vial rack</x:v>
+      </x:c>
+      <x:c r="C270" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D270" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E270" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F270" s="9" t="str">
+        <x:v>Fitted rack holding existing separately sealed sample vessels.</x:v>
+      </x:c>
+      <x:c r="G270" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H270" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I270" s="13"/>
+      <x:c r="J270" s="15"/>
+      <x:c r="K270" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L270" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M270" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N270" s="9" t="str">
+        <x:v>Rack geometry, shock isolation and chemistry segregation TBD; vials remain separately counted.</x:v>
+      </x:c>
+      <x:c r="O270" s="17"/>
+      <x:c r="P270" s="17"/>
+      <x:c r="Q270" s="17"/>
+      <x:c r="R270" s="17"/>
+      <x:c r="S270" s="17"/>
+      <x:c r="T270" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U270" s="11"/>
+      <x:c r="V270" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W270" s="4" t="str">
+        <x:v>Carrier</x:v>
+      </x:c>
+      <x:c r="X270" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y270" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z270" s="4" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="AA270" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB270" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC270" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD270" s="4" t="str">
+        <x:v>legger sample-vial rack; legger cargo rigging; carrier; mixed / unresolved; cargo organization; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE270" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="271" ht="115" customHeight="1">
+      <x:c r="A271" s="9" t="str">
+        <x:v>proposal.legger.ore_bin</x:v>
+      </x:c>
+      <x:c r="B271" s="9" t="str">
+        <x:v>Legger removable ore bin</x:v>
+      </x:c>
+      <x:c r="C271" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D271" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E271" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F271" s="9" t="str">
+        <x:v>Removable rigid bin for selected bulk mineral cargo.</x:v>
+      </x:c>
+      <x:c r="G271" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H271" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I271" s="13"/>
+      <x:c r="J271" s="15"/>
+      <x:c r="K271" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L271" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M271" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N271" s="9" t="str">
+        <x:v>Volume and load limit undefined; remains physical Legger cargo, not extra abstract inventory.</x:v>
+      </x:c>
+      <x:c r="O271" s="17"/>
+      <x:c r="P271" s="17"/>
+      <x:c r="Q271" s="17"/>
+      <x:c r="R271" s="17"/>
+      <x:c r="S271" s="17"/>
+      <x:c r="T271" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U271" s="11"/>
+      <x:c r="V271" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W271" s="4" t="str">
+        <x:v>Container</x:v>
+      </x:c>
+      <x:c r="X271" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y271" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z271" s="4" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="AA271" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB271" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC271" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD271" s="4" t="str">
+        <x:v>legger removable ore bin; legger cargo rigging; container; metal; cargo organization; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE271" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272" ht="115" customHeight="1">
+      <x:c r="A272" s="9" t="str">
+        <x:v>proposal.legger.long_load_clamp</x:v>
+      </x:c>
+      <x:c r="B272" s="9" t="str">
+        <x:v>Legger long-load clamp</x:v>
+      </x:c>
+      <x:c r="C272" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D272" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E272" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F272" s="9" t="str">
+        <x:v>A matched clamp for carrying a long salvage member.</x:v>
+      </x:c>
+      <x:c r="G272" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H272" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I272" s="13"/>
+      <x:c r="J272" s="15"/>
+      <x:c r="K272" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L272" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M272" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N272" s="9" t="str">
+        <x:v>Must account for reach, balance and collision envelope; no automatic carrying of arbitrarily large objects.</x:v>
+      </x:c>
+      <x:c r="O272" s="17"/>
+      <x:c r="P272" s="17"/>
+      <x:c r="Q272" s="17"/>
+      <x:c r="R272" s="17"/>
+      <x:c r="S272" s="17"/>
+      <x:c r="T272" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U272" s="11"/>
+      <x:c r="V272" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W272" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X272" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y272" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z272" s="4" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="AA272" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB272" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC272" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD272" s="4" t="str">
+        <x:v>legger long-load clamp; legger cargo rigging; crafting component; metal; equipment mounting; cargo organization; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE272" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="273" ht="115" customHeight="1">
+      <x:c r="A273" s="9" t="str">
+        <x:v>proposal.legger.release_latch</x:v>
+      </x:c>
+      <x:c r="B273" s="9" t="str">
+        <x:v>Cargo quick-release latch</x:v>
+      </x:c>
+      <x:c r="C273" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D273" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E273" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F273" s="9" t="str">
+        <x:v>Serviceable latch securing one compatible cargo carrier.</x:v>
+      </x:c>
+      <x:c r="G273" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H273" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I273" s="13"/>
+      <x:c r="J273" s="15"/>
+      <x:c r="K273" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L273" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M273" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N273" s="9" t="str">
+        <x:v>Release action, retention and failure behavior TBD; distinguish from mounting eyes and lashings.</x:v>
+      </x:c>
+      <x:c r="O273" s="17"/>
+      <x:c r="P273" s="17"/>
+      <x:c r="Q273" s="17"/>
+      <x:c r="R273" s="17"/>
+      <x:c r="S273" s="17"/>
+      <x:c r="T273" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U273" s="11"/>
+      <x:c r="V273" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W273" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X273" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y273" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z273" s="4" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="AA273" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB273" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC273" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD273" s="4" t="str">
+        <x:v>cargo quick-release latch; legger cargo rigging; crafting component; metal; equipment mounting; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE273" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="274" ht="115" customHeight="1">
+      <x:c r="A274" s="9" t="str">
+        <x:v>proposal.legger.board_bracket</x:v>
+      </x:c>
+      <x:c r="B274" s="9" t="str">
+        <x:v>Legger dirtboard carrying bracket</x:v>
+      </x:c>
+      <x:c r="C274" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D274" s="9" t="str">
+        <x:v>Legger cargo rigging</x:v>
+      </x:c>
+      <x:c r="E274" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F274" s="9" t="str">
+        <x:v>Proposed stowage bracket for Booter four-wheel dirtboard.</x:v>
+      </x:c>
+      <x:c r="G274" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H274" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I274" s="13"/>
+      <x:c r="J274" s="15"/>
+      <x:c r="K274" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L274" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M274" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N274" s="9" t="str">
+        <x:v>Fits only after gear/companion carry design; adds no remote board access or capacity.</x:v>
+      </x:c>
+      <x:c r="O274" s="17"/>
+      <x:c r="P274" s="17"/>
+      <x:c r="Q274" s="17"/>
+      <x:c r="R274" s="17"/>
+      <x:c r="S274" s="17"/>
+      <x:c r="T274" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U274" s="11"/>
+      <x:c r="V274" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W274" s="4" t="str">
+        <x:v>Carrier</x:v>
+      </x:c>
+      <x:c r="X274" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y274" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z274" s="4" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="AA274" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB274" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC274" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD274" s="4" t="str">
+        <x:v>legger dirtboard carrying bracket; legger cargo rigging; carrier; metal; cargo organization; equipment mounting; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE274" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="275" ht="115" customHeight="1">
+      <x:c r="A275" s="9" t="str">
+        <x:v>proposal.legger.hinge_plate</x:v>
+      </x:c>
+      <x:c r="B275" s="9" t="str">
+        <x:v>Chassis hinge-mount plate</x:v>
+      </x:c>
+      <x:c r="C275" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D275" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E275" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F275" s="9" t="str">
+        <x:v>Replaceable mounting face for a compatible hinged chassis assembly.</x:v>
+      </x:c>
+      <x:c r="G275" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H275" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I275" s="13"/>
+      <x:c r="J275" s="15"/>
+      <x:c r="K275" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L275" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M275" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N275" s="9" t="str">
+        <x:v>Host joint geometry and fasteners must be established first.</x:v>
+      </x:c>
+      <x:c r="O275" s="17"/>
+      <x:c r="P275" s="17"/>
+      <x:c r="Q275" s="17"/>
+      <x:c r="R275" s="17"/>
+      <x:c r="S275" s="17"/>
+      <x:c r="T275" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U275" s="11"/>
+      <x:c r="V275" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W275" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X275" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y275" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z275" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA275" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB275" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC275" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD275" s="4" t="str">
+        <x:v>chassis hinge-mount plate; legger chassis; crafting component; metal; equipment repair; equipment mounting; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE275" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="276" ht="115" customHeight="1">
+      <x:c r="A276" s="9" t="str">
+        <x:v>proposal.legger.inspection_hatch</x:v>
+      </x:c>
+      <x:c r="B276" s="9" t="str">
+        <x:v>Legger inspection hatch</x:v>
+      </x:c>
+      <x:c r="C276" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D276" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E276" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F276" s="9" t="str">
+        <x:v>Removable chassis access cover for selected service points.</x:v>
+      </x:c>
+      <x:c r="G276" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H276" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I276" s="13"/>
+      <x:c r="J276" s="15"/>
+      <x:c r="K276" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L276" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M276" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N276" s="9" t="str">
+        <x:v>Opening and sealing details remain open; distinct from an armor cover.</x:v>
+      </x:c>
+      <x:c r="O276" s="17"/>
+      <x:c r="P276" s="17"/>
+      <x:c r="Q276" s="17"/>
+      <x:c r="R276" s="17"/>
+      <x:c r="S276" s="17"/>
+      <x:c r="T276" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U276" s="11"/>
+      <x:c r="V276" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W276" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X276" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y276" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z276" s="4" t="str">
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="AA276" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB276" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC276" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD276" s="4" t="str">
+        <x:v>legger inspection hatch; legger chassis; crafting component; metal; inspection; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE276" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="277" ht="115" customHeight="1">
+      <x:c r="A277" s="9" t="str">
+        <x:v>proposal.legger.fracture_patch</x:v>
+      </x:c>
+      <x:c r="B277" s="9" t="str">
+        <x:v>Iron chassis fracture patch</x:v>
+      </x:c>
+      <x:c r="C277" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D277" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E277" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F277" s="9" t="str">
+        <x:v>Shaped bridging piece for a particular damaged frame location.</x:v>
+      </x:c>
+      <x:c r="G277" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H277" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I277" s="13"/>
+      <x:c r="J277" s="15"/>
+      <x:c r="K277" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L277" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M277" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N277" s="9" t="str">
+        <x:v>Temporary versus permanent repair and installation method TBD; not universal structural healing.</x:v>
+      </x:c>
+      <x:c r="O277" s="17"/>
+      <x:c r="P277" s="17"/>
+      <x:c r="Q277" s="17"/>
+      <x:c r="R277" s="17"/>
+      <x:c r="S277" s="17"/>
+      <x:c r="T277" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U277" s="11"/>
+      <x:c r="V277" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W277" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X277" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y277" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z277" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA277" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB277" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC277" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD277" s="4" t="str">
+        <x:v>iron chassis fracture patch; legger chassis; crafting component; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE277" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="278" ht="115" customHeight="1">
+      <x:c r="A278" s="9" t="str">
+        <x:v>proposal.legger.crush_mount</x:v>
+      </x:c>
+      <x:c r="B278" s="9" t="str">
+        <x:v>Sacrificial attachment mount</x:v>
+      </x:c>
+      <x:c r="C278" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D278" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E278" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F278" s="9" t="str">
+        <x:v>Replaceable mount proposed to localize damage at an attachment.</x:v>
+      </x:c>
+      <x:c r="G278" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H278" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I278" s="13"/>
+      <x:c r="J278" s="15"/>
+      <x:c r="K278" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L278" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M278" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N278" s="9" t="str">
+        <x:v>Controlled failure is a design goal; thresholds and damage transfer unresolved.</x:v>
+      </x:c>
+      <x:c r="O278" s="17"/>
+      <x:c r="P278" s="17"/>
+      <x:c r="Q278" s="17"/>
+      <x:c r="R278" s="17"/>
+      <x:c r="S278" s="17"/>
+      <x:c r="T278" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U278" s="11"/>
+      <x:c r="V278" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W278" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X278" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y278" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z278" s="4" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="AA278" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB278" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC278" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD278" s="4" t="str">
+        <x:v>sacrificial attachment mount; legger chassis; crafting component; metal; equipment mounting; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE278" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="279" ht="115" customHeight="1">
+      <x:c r="A279" s="9" t="str">
+        <x:v>proposal.legger.bulkhead_ring</x:v>
+      </x:c>
+      <x:c r="B279" s="9" t="str">
+        <x:v>Chassis reinforcing ring</x:v>
+      </x:c>
+      <x:c r="C279" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D279" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E279" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F279" s="9" t="str">
+        <x:v>Shaped reinforcement around a selected chassis opening.</x:v>
+      </x:c>
+      <x:c r="G279" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H279" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I279" s="13"/>
+      <x:c r="J279" s="15"/>
+      <x:c r="K279" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L279" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M279" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N279" s="9" t="str">
+        <x:v>Requires actual host geometry; reinforcement and mass effects undefined.</x:v>
+      </x:c>
+      <x:c r="O279" s="17"/>
+      <x:c r="P279" s="17"/>
+      <x:c r="Q279" s="17"/>
+      <x:c r="R279" s="17"/>
+      <x:c r="S279" s="17"/>
+      <x:c r="T279" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U279" s="11"/>
+      <x:c r="V279" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W279" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X279" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y279" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z279" s="4" t="str">
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="AA279" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB279" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC279" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD279" s="4" t="str">
+        <x:v>chassis reinforcing ring; legger chassis; crafting component; metal; equipment fabrication; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE279" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="280" ht="115" customHeight="1">
+      <x:c r="A280" s="9" t="str">
+        <x:v>proposal.legger.alignment_shims</x:v>
+      </x:c>
+      <x:c r="B280" s="9" t="str">
+        <x:v>Chassis alignment-shim set</x:v>
+      </x:c>
+      <x:c r="C280" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D280" s="9" t="str">
+        <x:v>Legger chassis</x:v>
+      </x:c>
+      <x:c r="E280" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F280" s="9" t="str">
+        <x:v>Selected thin inserts for matching fitted structural faces.</x:v>
+      </x:c>
+      <x:c r="G280" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H280" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I280" s="13"/>
+      <x:c r="J280" s="15"/>
+      <x:c r="K280" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L280" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M280" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N280" s="9" t="str">
+        <x:v>Set sizes and required tolerances unresolved; no universal-fit interface.</x:v>
+      </x:c>
+      <x:c r="O280" s="17"/>
+      <x:c r="P280" s="17"/>
+      <x:c r="Q280" s="17"/>
+      <x:c r="R280" s="17"/>
+      <x:c r="S280" s="17"/>
+      <x:c r="T280" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U280" s="11"/>
+      <x:c r="V280" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W280" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X280" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y280" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z280" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA280" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB280" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC280" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD280" s="4" t="str">
+        <x:v>chassis alignment-shim set; legger chassis; crafting component; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE280" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="281" ht="115" customHeight="1">
+      <x:c r="A281" s="9" t="str">
+        <x:v>proposal.legger.joint_pin</x:v>
+      </x:c>
+      <x:c r="B281" s="9" t="str">
+        <x:v>Replaceable joint pin</x:v>
+      </x:c>
+      <x:c r="C281" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D281" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E281" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F281" s="9" t="str">
+        <x:v>Matched pivot pin within a selected Legger joint.</x:v>
+      </x:c>
+      <x:c r="G281" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H281" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I281" s="13"/>
+      <x:c r="J281" s="15"/>
+      <x:c r="K281" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L281" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M281" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N281" s="9" t="str">
+        <x:v>Pin, sleeve and bearing are different parts; geometry and material grade unresolved.</x:v>
+      </x:c>
+      <x:c r="O281" s="17"/>
+      <x:c r="P281" s="17"/>
+      <x:c r="Q281" s="17"/>
+      <x:c r="R281" s="17"/>
+      <x:c r="S281" s="17"/>
+      <x:c r="T281" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U281" s="11"/>
+      <x:c r="V281" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W281" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X281" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y281" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z281" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA281" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB281" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC281" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD281" s="4" t="str">
+        <x:v>replaceable joint pin; legger mechanical parts; crafting component; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE281" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282" ht="115" customHeight="1">
+      <x:c r="A282" s="9" t="str">
+        <x:v>proposal.legger.thrust_washer</x:v>
+      </x:c>
+      <x:c r="B282" s="9" t="str">
+        <x:v>Joint thrust washer</x:v>
+      </x:c>
+      <x:c r="C282" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D282" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E282" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F282" s="9" t="str">
+        <x:v>Wear-interface insert proposed for a selected axial contact.</x:v>
+      </x:c>
+      <x:c r="G282" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H282" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I282" s="13"/>
+      <x:c r="J282" s="15"/>
+      <x:c r="K282" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L282" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M282" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N282" s="9" t="str">
+        <x:v>Actual load path, lubrication and service requirements TBD.</x:v>
+      </x:c>
+      <x:c r="O282" s="17"/>
+      <x:c r="P282" s="17"/>
+      <x:c r="Q282" s="17"/>
+      <x:c r="R282" s="17"/>
+      <x:c r="S282" s="17"/>
+      <x:c r="T282" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U282" s="11"/>
+      <x:c r="V282" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W282" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X282" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y282" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z282" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA282" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB282" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC282" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD282" s="4" t="str">
+        <x:v>joint thrust washer; legger mechanical parts; crafting component; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE282" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="283" ht="115" customHeight="1">
+      <x:c r="A283" s="9" t="str">
+        <x:v>proposal.legger.gear_cluster</x:v>
+      </x:c>
+      <x:c r="B283" s="9" t="str">
+        <x:v>Replacement gear cluster</x:v>
+      </x:c>
+      <x:c r="C283" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D283" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E283" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F283" s="9" t="str">
+        <x:v>Matched gears for a compatible drive assembly.</x:v>
+      </x:c>
+      <x:c r="G283" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H283" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I283" s="13"/>
+      <x:c r="J283" s="15"/>
+      <x:c r="K283" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L283" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M283" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N283" s="9" t="str">
+        <x:v>A candidate mechanism rather than proof the current Legger uses this transmission.</x:v>
+      </x:c>
+      <x:c r="O283" s="17"/>
+      <x:c r="P283" s="17"/>
+      <x:c r="Q283" s="17"/>
+      <x:c r="R283" s="17"/>
+      <x:c r="S283" s="17"/>
+      <x:c r="T283" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U283" s="11"/>
+      <x:c r="V283" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W283" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X283" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y283" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z283" s="4" t="str">
+        <x:v>Machinery drive</x:v>
+      </x:c>
+      <x:c r="AA283" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB283" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC283" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD283" s="4" t="str">
+        <x:v>replacement gear cluster; legger mechanical parts; crafting component; metal; machinery drive; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE283" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="284" ht="115" customHeight="1">
+      <x:c r="A284" s="9" t="str">
+        <x:v>proposal.legger.linkage_end</x:v>
+      </x:c>
+      <x:c r="B284" s="9" t="str">
+        <x:v>Replacement linkage-end joint</x:v>
+      </x:c>
+      <x:c r="C284" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D284" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E284" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F284" s="9" t="str">
+        <x:v>End connector joining a selected movement link to its mount.</x:v>
+      </x:c>
+      <x:c r="G284" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H284" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I284" s="13"/>
+      <x:c r="J284" s="15"/>
+      <x:c r="K284" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L284" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M284" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N284" s="9" t="str">
+        <x:v>Degrees of movement, fit and service method unresolved.</x:v>
+      </x:c>
+      <x:c r="O284" s="17"/>
+      <x:c r="P284" s="17"/>
+      <x:c r="Q284" s="17"/>
+      <x:c r="R284" s="17"/>
+      <x:c r="S284" s="17"/>
+      <x:c r="T284" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U284" s="11"/>
+      <x:c r="V284" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W284" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X284" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y284" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z284" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA284" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB284" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC284" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD284" s="4" t="str">
+        <x:v>replacement linkage-end joint; legger mechanical parts; crafting component; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE284" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="285" ht="115" customHeight="1">
+      <x:c r="A285" s="9" t="str">
+        <x:v>proposal.legger.tensioner</x:v>
+      </x:c>
+      <x:c r="B285" s="9" t="str">
+        <x:v>Drive tensioner assembly</x:v>
+      </x:c>
+      <x:c r="C285" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D285" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E285" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F285" s="9" t="str">
+        <x:v>Adjustment assembly candidate for a selected mechanical drive path.</x:v>
+      </x:c>
+      <x:c r="G285" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H285" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I285" s="13"/>
+      <x:c r="J285" s="15"/>
+      <x:c r="K285" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L285" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M285" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N285" s="9" t="str">
+        <x:v>Requires a compatible drive architecture; no belt or chain transmission assumed.</x:v>
+      </x:c>
+      <x:c r="O285" s="17"/>
+      <x:c r="P285" s="17"/>
+      <x:c r="Q285" s="17"/>
+      <x:c r="R285" s="17"/>
+      <x:c r="S285" s="17"/>
+      <x:c r="T285" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U285" s="11"/>
+      <x:c r="V285" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W285" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X285" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y285" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z285" s="4" t="str">
+        <x:v>Machinery drive</x:v>
+      </x:c>
+      <x:c r="AA285" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB285" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC285" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD285" s="4" t="str">
+        <x:v>drive tensioner assembly; legger mechanical parts; crafting component; mixed / unresolved; machinery drive; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE285" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="286" ht="115" customHeight="1">
+      <x:c r="A286" s="9" t="str">
+        <x:v>proposal.legger.scraper_ring</x:v>
+      </x:c>
+      <x:c r="B286" s="9" t="str">
+        <x:v>Joint grit-scraper ring</x:v>
+      </x:c>
+      <x:c r="C286" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D286" s="9" t="str">
+        <x:v>Legger mechanical parts</x:v>
+      </x:c>
+      <x:c r="E286" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F286" s="9" t="str">
+        <x:v>Replaceable contact ring proposed to clear grit from a matched moving surface.</x:v>
+      </x:c>
+      <x:c r="G286" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H286" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I286" s="13"/>
+      <x:c r="J286" s="15"/>
+      <x:c r="K286" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L286" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M286" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N286" s="9" t="str">
+        <x:v>Distinct from a seal cartridge or external shroud; contact and wear properties TBD.</x:v>
+      </x:c>
+      <x:c r="O286" s="17"/>
+      <x:c r="P286" s="17"/>
+      <x:c r="Q286" s="17"/>
+      <x:c r="R286" s="17"/>
+      <x:c r="S286" s="17"/>
+      <x:c r="T286" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U286" s="11"/>
+      <x:c r="V286" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W286" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X286" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y286" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z286" s="4" t="str">
+        <x:v>Dust exclusion</x:v>
+      </x:c>
+      <x:c r="AA286" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB286" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC286" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD286" s="4" t="str">
+        <x:v>joint grit-scraper ring; legger mechanical parts; crafting component; mixed / unresolved; dust exclusion; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE286" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="287" ht="115" customHeight="1">
+      <x:c r="A287" s="9" t="str">
+        <x:v>proposal.legger.grease_applicator</x:v>
+      </x:c>
+      <x:c r="B287" s="9" t="str">
+        <x:v>Joint grease applicator</x:v>
+      </x:c>
+      <x:c r="C287" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D287" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E287" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F287" s="9" t="str">
+        <x:v>Hand-operated tool candidate for placing selected faunal grease at a service point.</x:v>
+      </x:c>
+      <x:c r="G287" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H287" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I287" s="13"/>
+      <x:c r="J287" s="15"/>
+      <x:c r="K287" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L287" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M287" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N287" s="9" t="str">
+        <x:v>Pressure, fitting and dose undefined; does not imply hydraulic actuation.</x:v>
+      </x:c>
+      <x:c r="O287" s="17"/>
+      <x:c r="P287" s="17"/>
+      <x:c r="Q287" s="17"/>
+      <x:c r="R287" s="17"/>
+      <x:c r="S287" s="17"/>
+      <x:c r="T287" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U287" s="11"/>
+      <x:c r="V287" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W287" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X287" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y287" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z287" s="4" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="AA287" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB287" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC287" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD287" s="4" t="str">
+        <x:v>joint grease applicator; legger service parts; tool; metal; lubrication; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE287" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="288" ht="115" customHeight="1">
+      <x:c r="A288" s="9" t="str">
+        <x:v>proposal.legger.service_adapter</x:v>
+      </x:c>
+      <x:c r="B288" s="9" t="str">
+        <x:v>Lubricant service-port adapter</x:v>
+      </x:c>
+      <x:c r="C288" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D288" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E288" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F288" s="9" t="str">
+        <x:v>Matched connection between a lubricant tool and a selected service port.</x:v>
+      </x:c>
+      <x:c r="G288" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H288" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I288" s="13"/>
+      <x:c r="J288" s="15"/>
+      <x:c r="K288" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L288" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M288" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N288" s="9" t="str">
+        <x:v>Compatible fitting standard remains open; not a universal chemical connector.</x:v>
+      </x:c>
+      <x:c r="O288" s="17"/>
+      <x:c r="P288" s="17"/>
+      <x:c r="Q288" s="17"/>
+      <x:c r="R288" s="17"/>
+      <x:c r="S288" s="17"/>
+      <x:c r="T288" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U288" s="11"/>
+      <x:c r="V288" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W288" s="4" t="str">
+        <x:v>Container part</x:v>
+      </x:c>
+      <x:c r="X288" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y288" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z288" s="4" t="str">
+        <x:v>Material transfer</x:v>
+      </x:c>
+      <x:c r="AA288" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB288" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC288" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD288" s="4" t="str">
+        <x:v>lubricant service-port adapter; legger service parts; container part; metal; material transfer; lubrication; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE288" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="289" ht="115" customHeight="1">
+      <x:c r="A289" s="9" t="str">
+        <x:v>proposal.legger.service_pick</x:v>
+      </x:c>
+      <x:c r="B289" s="9" t="str">
+        <x:v>Joint-service cleaning pick</x:v>
+      </x:c>
+      <x:c r="C289" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D289" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E289" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F289" s="9" t="str">
+        <x:v>Shaped tool for removing residue from an accessible service recess.</x:v>
+      </x:c>
+      <x:c r="G289" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H289" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I289" s="13"/>
+      <x:c r="J289" s="15"/>
+      <x:c r="K289" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L289" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M289" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N289" s="9" t="str">
+        <x:v>Tool tip and use must preserve the selected seal/contact surface.</x:v>
+      </x:c>
+      <x:c r="O289" s="17"/>
+      <x:c r="P289" s="17"/>
+      <x:c r="Q289" s="17"/>
+      <x:c r="R289" s="17"/>
+      <x:c r="S289" s="17"/>
+      <x:c r="T289" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U289" s="11"/>
+      <x:c r="V289" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W289" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X289" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y289" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z289" s="4" t="str">
+        <x:v>Cleaning</x:v>
+      </x:c>
+      <x:c r="AA289" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB289" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC289" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD289" s="4" t="str">
+        <x:v>joint-service cleaning pick; legger service parts; tool; metal; cleaning; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE289" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="290" ht="115" customHeight="1">
+      <x:c r="A290" s="9" t="str">
+        <x:v>proposal.legger.bearing_puller</x:v>
+      </x:c>
+      <x:c r="B290" s="9" t="str">
+        <x:v>Matched bearing-removal tool</x:v>
+      </x:c>
+      <x:c r="C290" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D290" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E290" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F290" s="9" t="str">
+        <x:v>Workshop tool candidate for removing a selected bearing assembly.</x:v>
+      </x:c>
+      <x:c r="G290" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H290" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I290" s="13"/>
+      <x:c r="J290" s="15"/>
+      <x:c r="K290" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L290" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M290" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N290" s="9" t="str">
+        <x:v>Requires the actual bearing and host fit; does not grant field disassembly of all joints.</x:v>
+      </x:c>
+      <x:c r="O290" s="17"/>
+      <x:c r="P290" s="17"/>
+      <x:c r="Q290" s="17"/>
+      <x:c r="R290" s="17"/>
+      <x:c r="S290" s="17"/>
+      <x:c r="T290" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U290" s="11"/>
+      <x:c r="V290" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W290" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X290" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y290" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z290" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA290" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB290" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC290" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD290" s="4" t="str">
+        <x:v>matched bearing-removal tool; legger service parts; tool; metal; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE290" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="291" ht="115" customHeight="1">
+      <x:c r="A291" s="9" t="str">
+        <x:v>proposal.legger.alignment_gauge</x:v>
+      </x:c>
+      <x:c r="B291" s="9" t="str">
+        <x:v>Legger alignment gauge</x:v>
+      </x:c>
+      <x:c r="C291" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D291" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E291" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F291" s="9" t="str">
+        <x:v>Template or gauge for checking a defined fitted relationship.</x:v>
+      </x:c>
+      <x:c r="G291" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H291" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I291" s="13"/>
+      <x:c r="J291" s="15"/>
+      <x:c r="K291" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L291" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M291" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N291" s="9" t="str">
+        <x:v>Reference geometry and acceptable tolerances unresolved.</x:v>
+      </x:c>
+      <x:c r="O291" s="17"/>
+      <x:c r="P291" s="17"/>
+      <x:c r="Q291" s="17"/>
+      <x:c r="R291" s="17"/>
+      <x:c r="S291" s="17"/>
+      <x:c r="T291" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U291" s="11"/>
+      <x:c r="V291" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W291" s="4" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="X291" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y291" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z291" s="4" t="str">
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="AA291" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB291" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC291" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD291" s="4" t="str">
+        <x:v>legger alignment gauge; legger service parts; tool; metal; inspection; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE291" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="292" ht="115" customHeight="1">
+      <x:c r="A292" s="9" t="str">
+        <x:v>proposal.legger.spares_case</x:v>
+      </x:c>
+      <x:c r="B292" s="9" t="str">
+        <x:v>Legger fitted spares case</x:v>
+      </x:c>
+      <x:c r="C292" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D292" s="9" t="str">
+        <x:v>Legger service parts</x:v>
+      </x:c>
+      <x:c r="E292" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F292" s="9" t="str">
+        <x:v>Partitioned case for selected small replacement parts and service tools.</x:v>
+      </x:c>
+      <x:c r="G292" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H292" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I292" s="13"/>
+      <x:c r="J292" s="15"/>
+      <x:c r="K292" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L292" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M292" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N292" s="9" t="str">
+        <x:v>Contents remain separate items; no uncounted complete repair kit or capacity increase.</x:v>
+      </x:c>
+      <x:c r="O292" s="17"/>
+      <x:c r="P292" s="17"/>
+      <x:c r="Q292" s="17"/>
+      <x:c r="R292" s="17"/>
+      <x:c r="S292" s="17"/>
+      <x:c r="T292" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U292" s="11"/>
+      <x:c r="V292" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W292" s="4" t="str">
+        <x:v>Container</x:v>
+      </x:c>
+      <x:c r="X292" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y292" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z292" s="4" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="AA292" s="4" t="str">
+        <x:v>Metal or shell</x:v>
+      </x:c>
+      <x:c r="AB292" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC292" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD292" s="4" t="str">
+        <x:v>legger fitted spares case; legger service parts; container; metal or shell; cargo organization; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE292" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="293" ht="115" customHeight="1">
+      <x:c r="A293" s="9" t="str">
+        <x:v>proposal.legger.edge_guard</x:v>
+      </x:c>
+      <x:c r="B293" s="9" t="str">
+        <x:v>Chassis leading-edge guard</x:v>
+      </x:c>
+      <x:c r="C293" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D293" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E293" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F293" s="9" t="str">
+        <x:v>Replaceable narrow guard on a selected exposed frame edge.</x:v>
+      </x:c>
+      <x:c r="G293" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H293" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I293" s="13"/>
+      <x:c r="J293" s="15"/>
+      <x:c r="K293" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L293" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M293" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N293" s="9" t="str">
+        <x:v>Coverage and host geometry distinguish it from full chassis plates; protection TBD.</x:v>
+      </x:c>
+      <x:c r="O293" s="17"/>
+      <x:c r="P293" s="17"/>
+      <x:c r="Q293" s="17"/>
+      <x:c r="R293" s="17"/>
+      <x:c r="S293" s="17"/>
+      <x:c r="T293" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U293" s="11"/>
+      <x:c r="V293" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W293" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X293" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y293" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z293" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA293" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB293" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC293" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD293" s="4" t="str">
+        <x:v>chassis leading-edge guard; legger armor; armor; metal; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE293" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="294" ht="115" customHeight="1">
+      <x:c r="A294" s="9" t="str">
+        <x:v>proposal.legger.instrument_guard</x:v>
+      </x:c>
+      <x:c r="B294" s="9" t="str">
+        <x:v>Instrument-face guard</x:v>
+      </x:c>
+      <x:c r="C294" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D294" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E294" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F294" s="9" t="str">
+        <x:v>Protective cage candidate around a selected exposed instrument face.</x:v>
+      </x:c>
+      <x:c r="G294" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H294" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I294" s="13"/>
+      <x:c r="J294" s="15"/>
+      <x:c r="K294" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L294" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M294" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N294" s="9" t="str">
+        <x:v>Requires a real instrument and sight/clearance review; grants no new sensor capability.</x:v>
+      </x:c>
+      <x:c r="O294" s="17"/>
+      <x:c r="P294" s="17"/>
+      <x:c r="Q294" s="17"/>
+      <x:c r="R294" s="17"/>
+      <x:c r="S294" s="17"/>
+      <x:c r="T294" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U294" s="11"/>
+      <x:c r="V294" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W294" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X294" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y294" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z294" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA294" s="4" t="str">
+        <x:v>Mixed / unresolved</x:v>
+      </x:c>
+      <x:c r="AB294" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC294" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD294" s="4" t="str">
+        <x:v>instrument-face guard; legger armor; armor; mixed / unresolved; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE294" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="295" ht="115" customHeight="1">
+      <x:c r="A295" s="9" t="str">
+        <x:v>proposal.legger.seam_guard</x:v>
+      </x:c>
+      <x:c r="B295" s="9" t="str">
+        <x:v>Armor seam-cover strip</x:v>
+      </x:c>
+      <x:c r="C295" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D295" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E295" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F295" s="9" t="str">
+        <x:v>Overlap piece covering a selected gap between fitted guards.</x:v>
+      </x:c>
+      <x:c r="G295" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H295" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I295" s="13"/>
+      <x:c r="J295" s="15"/>
+      <x:c r="K295" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L295" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M295" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N295" s="9" t="str">
+        <x:v>Must preserve movement and service access; no complete gap-free protection inferred.</x:v>
+      </x:c>
+      <x:c r="O295" s="17"/>
+      <x:c r="P295" s="17"/>
+      <x:c r="Q295" s="17"/>
+      <x:c r="R295" s="17"/>
+      <x:c r="S295" s="17"/>
+      <x:c r="T295" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U295" s="11"/>
+      <x:c r="V295" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W295" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X295" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y295" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z295" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA295" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB295" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC295" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD295" s="4" t="str">
+        <x:v>armor seam-cover strip; legger armor; armor; metal; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE295" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="296" ht="115" customHeight="1">
+      <x:c r="A296" s="9" t="str">
+        <x:v>proposal.legger.impact_cap</x:v>
+      </x:c>
+      <x:c r="B296" s="9" t="str">
+        <x:v>Sacrificial impact cap</x:v>
+      </x:c>
+      <x:c r="C296" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D296" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E296" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F296" s="9" t="str">
+        <x:v>Replaceable cap candidate over a selected protruding part.</x:v>
+      </x:c>
+      <x:c r="G296" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H296" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I296" s="13"/>
+      <x:c r="J296" s="15"/>
+      <x:c r="K296" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L296" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M296" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N296" s="9" t="str">
+        <x:v>Damage localization, shell grade and replacement behavior remain proposed.</x:v>
+      </x:c>
+      <x:c r="O296" s="17"/>
+      <x:c r="P296" s="17"/>
+      <x:c r="Q296" s="17"/>
+      <x:c r="R296" s="17"/>
+      <x:c r="S296" s="17"/>
+      <x:c r="T296" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U296" s="11"/>
+      <x:c r="V296" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W296" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X296" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y296" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z296" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA296" s="4" t="str">
+        <x:v>Shell / chitin</x:v>
+      </x:c>
+      <x:c r="AB296" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC296" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD296" s="4" t="str">
+        <x:v>sacrificial impact cap; legger armor; armor; shell / chitin; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE296" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="297" ht="115" customHeight="1">
+      <x:c r="A297" s="9" t="str">
+        <x:v>proposal.legger.fragment_liner</x:v>
+      </x:c>
+      <x:c r="B297" s="9" t="str">
+        <x:v>Pressed-husk fragment liner</x:v>
+      </x:c>
+      <x:c r="C297" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D297" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E297" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F297" s="9" t="str">
+        <x:v>Scarce pressed-fiber backing proposed inside a selected guard.</x:v>
+      </x:c>
+      <x:c r="G297" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H297" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I297" s="13"/>
+      <x:c r="J297" s="15"/>
+      <x:c r="K297" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L297" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M297" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N297" s="9" t="str">
+        <x:v>Fragment retention is a research goal, not proven ballistic protection; difficult textile processing still applies.</x:v>
+      </x:c>
+      <x:c r="O297" s="17"/>
+      <x:c r="P297" s="17"/>
+      <x:c r="Q297" s="17"/>
+      <x:c r="R297" s="17"/>
+      <x:c r="S297" s="17"/>
+      <x:c r="T297" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U297" s="11"/>
+      <x:c r="V297" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W297" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X297" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y297" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z297" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA297" s="4" t="str">
+        <x:v>Husk fiber</x:v>
+      </x:c>
+      <x:c r="AB297" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC297" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD297" s="4" t="str">
+        <x:v>pressed-husk fragment liner; legger armor; armor; husk fiber; protection; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE297" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="298" ht="115" customHeight="1">
+      <x:c r="A298" s="9" t="str">
+        <x:v>proposal.legger.guard_hinge</x:v>
+      </x:c>
+      <x:c r="B298" s="9" t="str">
+        <x:v>Armor-guard hinge assembly</x:v>
+      </x:c>
+      <x:c r="C298" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D298" s="9" t="str">
+        <x:v>Legger armor</x:v>
+      </x:c>
+      <x:c r="E298" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F298" s="9" t="str">
+        <x:v>Hinge/retainer unit candidate for an articulated protective panel.</x:v>
+      </x:c>
+      <x:c r="G298" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H298" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I298" s="13"/>
+      <x:c r="J298" s="15"/>
+      <x:c r="K298" s="9" t="str">
+        <x:v>Local craft, salvage or specialist trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L298" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M298" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N298" s="9" t="str">
+        <x:v>Different from the joint guard itself; geometry and durability TBD.</x:v>
+      </x:c>
+      <x:c r="O298" s="17"/>
+      <x:c r="P298" s="17"/>
+      <x:c r="Q298" s="17"/>
+      <x:c r="R298" s="17"/>
+      <x:c r="S298" s="17"/>
+      <x:c r="T298" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U298" s="11"/>
+      <x:c r="V298" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W298" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X298" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y298" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z298" s="4" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="AA298" s="4" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="AB298" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC298" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD298" s="4" t="str">
+        <x:v>armor-guard hinge assembly; legger armor; crafting component; metal; equipment mounting; equipment repair; legger; leger; companion replacement part; </x:v>
+      </x:c>
+      <x:c r="AE298" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="299" ht="115" customHeight="1">
+      <x:c r="A299" s="9" t="str">
+        <x:v>proposal.legger.plasteel_collar</x:v>
+      </x:c>
+      <x:c r="B299" s="9" t="str">
+        <x:v>Ancient plasteel joint collar</x:v>
+      </x:c>
+      <x:c r="C299" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D299" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E299" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F299" s="9" t="str">
+        <x:v>Recovered shaped collar considered for an appropriate joint housing.</x:v>
+      </x:c>
+      <x:c r="G299" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H299" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I299" s="13"/>
+      <x:c r="J299" s="15"/>
+      <x:c r="K299" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L299" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M299" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N299" s="9" t="str">
+        <x:v>Extremely rare; interfaces, residual condition and rework capability unknown.</x:v>
+      </x:c>
+      <x:c r="O299" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P299" s="17"/>
+      <x:c r="Q299" s="17"/>
+      <x:c r="R299" s="17"/>
+      <x:c r="S299" s="17"/>
+      <x:c r="T299" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U299" s="11"/>
+      <x:c r="V299" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W299" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X299" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y299" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z299" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA299" s="4" t="str">
+        <x:v>Ancient composite</x:v>
+      </x:c>
+      <x:c r="AB299" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC299" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD299" s="4" t="str">
+        <x:v>ancient plasteel joint collar; legger ancient replacement; crafting component; ancient composite; equipment repair; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE299" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="300" ht="115" customHeight="1">
+      <x:c r="A300" s="9" t="str">
+        <x:v>proposal.legger.tension_member</x:v>
+      </x:c>
+      <x:c r="B300" s="9" t="str">
+        <x:v>Ancient nanocarbon tension member</x:v>
+      </x:c>
+      <x:c r="C300" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D300" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E300" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F300" s="9" t="str">
+        <x:v>Recovered fiber/composite member considered for a selected tensile linkage.</x:v>
+      </x:c>
+      <x:c r="G300" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H300" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I300" s="13"/>
+      <x:c r="J300" s="15"/>
+      <x:c r="K300" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L300" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M300" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N300" s="9" t="str">
+        <x:v>Extremely rare; term describes intended structural role, not confirmed strength or active muscle behavior.</x:v>
+      </x:c>
+      <x:c r="O300" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P300" s="17"/>
+      <x:c r="Q300" s="17"/>
+      <x:c r="R300" s="17"/>
+      <x:c r="S300" s="17"/>
+      <x:c r="T300" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U300" s="11"/>
+      <x:c r="V300" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W300" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X300" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y300" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z300" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA300" s="4" t="str">
+        <x:v>Ancient composite</x:v>
+      </x:c>
+      <x:c r="AB300" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC300" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD300" s="4" t="str">
+        <x:v>ancient nanocarbon tension member; legger ancient replacement; crafting component; ancient composite; equipment repair; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE300" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="301" ht="115" customHeight="1">
+      <x:c r="A301" s="9" t="str">
+        <x:v>proposal.legger.friction_insert</x:v>
+      </x:c>
+      <x:c r="B301" s="9" t="str">
+        <x:v>Ancient friction-interface insert</x:v>
+      </x:c>
+      <x:c r="C301" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D301" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E301" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F301" s="9" t="str">
+        <x:v>Recovered contact insert considered for a matched wear interface.</x:v>
+      </x:c>
+      <x:c r="G301" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H301" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I301" s="13"/>
+      <x:c r="J301" s="15"/>
+      <x:c r="K301" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L301" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M301" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N301" s="9" t="str">
+        <x:v>Extremely rare; composition, remaining life and lubricant requirements unknown.</x:v>
+      </x:c>
+      <x:c r="O301" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P301" s="17"/>
+      <x:c r="Q301" s="17"/>
+      <x:c r="R301" s="17"/>
+      <x:c r="S301" s="17"/>
+      <x:c r="T301" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U301" s="11"/>
+      <x:c r="V301" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W301" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X301" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y301" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z301" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA301" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AB301" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC301" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD301" s="4" t="str">
+        <x:v>ancient friction-interface insert; legger ancient replacement; crafting component; unresolved; equipment repair; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE301" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="302" ht="115" customHeight="1">
+      <x:c r="A302" s="9" t="str">
+        <x:v>proposal.legger.ceramic_race</x:v>
+      </x:c>
+      <x:c r="B302" s="9" t="str">
+        <x:v>Ancient precision ceramic bearing race</x:v>
+      </x:c>
+      <x:c r="C302" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D302" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E302" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F302" s="9" t="str">
+        <x:v>Recovered high-precision ceramic race candidate within a compatible bearing.</x:v>
+      </x:c>
+      <x:c r="G302" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H302" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I302" s="13"/>
+      <x:c r="J302" s="15"/>
+      <x:c r="K302" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L302" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M302" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N302" s="9" t="str">
+        <x:v>Extremely rare because of its ancient fabrication; ordinary modern ceramic parts are a separate family.</x:v>
+      </x:c>
+      <x:c r="O302" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P302" s="17"/>
+      <x:c r="Q302" s="17"/>
+      <x:c r="R302" s="17"/>
+      <x:c r="S302" s="17"/>
+      <x:c r="T302" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U302" s="11"/>
+      <x:c r="V302" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W302" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X302" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y302" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z302" s="4" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="AA302" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB302" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC302" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD302" s="4" t="str">
+        <x:v>ancient precision ceramic bearing race; legger ancient replacement; crafting component; ceramic; equipment repair; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE302" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="303" ht="115" customHeight="1">
+      <x:c r="A303" s="9" t="str">
+        <x:v>proposal.legger.impact_lattice</x:v>
+      </x:c>
+      <x:c r="B303" s="9" t="str">
+        <x:v>Ancient impact-lattice backing</x:v>
+      </x:c>
+      <x:c r="C303" s="9" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D303" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E303" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F303" s="9" t="str">
+        <x:v>Recovered structured backing considered for a composite guard.</x:v>
+      </x:c>
+      <x:c r="G303" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H303" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I303" s="13"/>
+      <x:c r="J303" s="15"/>
+      <x:c r="K303" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L303" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M303" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N303" s="9" t="str">
+        <x:v>Extremely rare; energy response, layer compatibility and protection behavior remain undefined.</x:v>
+      </x:c>
+      <x:c r="O303" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P303" s="17"/>
+      <x:c r="Q303" s="17"/>
+      <x:c r="R303" s="17"/>
+      <x:c r="S303" s="17"/>
+      <x:c r="T303" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U303" s="11"/>
+      <x:c r="V303" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W303" s="4" t="str">
+        <x:v>Armor</x:v>
+      </x:c>
+      <x:c r="X303" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y303" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z303" s="4" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="AA303" s="4" t="str">
+        <x:v>Ancient composite</x:v>
+      </x:c>
+      <x:c r="AB303" s="4" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="AC303" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD303" s="4" t="str">
+        <x:v>ancient impact-lattice backing; legger ancient replacement; armor; ancient composite; protection; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE303" s="4" t="str">
+        <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="304" ht="115" customHeight="1">
+      <x:c r="A304" s="9" t="str">
+        <x:v>proposal.legger.interface_adapter</x:v>
+      </x:c>
+      <x:c r="B304" s="9" t="str">
+        <x:v>Ancient module interface adapter</x:v>
+      </x:c>
+      <x:c r="C304" s="9" t="str">
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D304" s="9" t="str">
+        <x:v>Legger ancient replacement</x:v>
+      </x:c>
+      <x:c r="E304" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F304" s="9" t="str">
+        <x:v>Recovered adapter candidate joining one identified ancient module to a matching host.</x:v>
+      </x:c>
+      <x:c r="G304" s="9" t="str">
+        <x:v>Legger fitment unresolved</x:v>
+      </x:c>
+      <x:c r="H304" s="9" t="str">
+        <x:v>Legger attachment / replacement intended; physical cargo policy unchanged</x:v>
+      </x:c>
+      <x:c r="I304" s="13"/>
+      <x:c r="J304" s="15"/>
+      <x:c r="K304" s="9" t="str">
+        <x:v>Extremely rare recovered technology; fitting and recovery method TBD</x:v>
+      </x:c>
+      <x:c r="L304" s="9" t="str">
+        <x:v>No recipe authored. Reuse existing iron stock, biological materials, ceramic craft, lubricant and ancient-material families where appropriate.</x:v>
+      </x:c>
+      <x:c r="M304" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N304" s="9" t="str">
+        <x:v>Extremely rare and interface-specific; does not unlock universal ancient-module compatibility.</x:v>
+      </x:c>
+      <x:c r="O304" s="17" t="str">
+        <x:v>Extremely rare</x:v>
+      </x:c>
+      <x:c r="P304" s="17"/>
+      <x:c r="Q304" s="17"/>
+      <x:c r="R304" s="17"/>
+      <x:c r="S304" s="17"/>
+      <x:c r="T304" s="9" t="str">
+        <x:v>Brainstorming candidate. Geometry, cost, mass, mounting, carrying and replacement behavior remain open. Part belongs to a finite physical companion.</x:v>
+      </x:c>
+      <x:c r="U304" s="11"/>
+      <x:c r="V304" s="9" t="str">
+        <x:v>Author Legger slings/chassis/replacement/iron/ancient-armor brainstorming October 14, 2026; Docs/WORLD_BASIS.md#the-legger; specific item proposal.</x:v>
+      </x:c>
+      <x:c r="W304" s="4" t="str">
+        <x:v>Crafting component</x:v>
+      </x:c>
+      <x:c r="X304" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y304" s="4" t="str">
+        <x:v>Ancient technology</x:v>
+      </x:c>
+      <x:c r="Z304" s="4" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="AA304" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AB304" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="AC304" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD304" s="4" t="str">
+        <x:v>ancient module interface adapter; legger ancient replacement; crafting component; unresolved; equipment mounting; legger; leger; companion replacement part; ancient salvage plasteel nanotube ballistic</x:v>
+      </x:c>
+      <x:c r="AE304" s="4" t="str">
         <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
       </x:c>
     </x:row>
@@ -22043,7 +24899,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbfbdf116d8a4d0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23296d6faaef4cc3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22695,7 +25551,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17d3326ef41f42eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd39132feb60544f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23177,7 +26033,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccb776a39f17488d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb01e4aa290d6403d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25184,7 +28040,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ec566f944364d48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd013d4714d3440f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33568,10 +36424,1146 @@
         <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
       </x:c>
     </x:row>
+    <x:row r="373" ht="65" customHeight="1">
+      <x:c r="A373" s="3" t="str">
+        <x:v>proposal.legger.pannier_frame</x:v>
+      </x:c>
+      <x:c r="B373" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A373,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger side-pannier frame</x:v>
+      </x:c>
+      <x:c r="C373" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A373,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D373" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E373" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A373,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F373" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="374" ht="65" customHeight="1">
+      <x:c r="A374" s="3" t="str">
+        <x:v>proposal.legger.pannier_frame</x:v>
+      </x:c>
+      <x:c r="B374" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A374,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger side-pannier frame</x:v>
+      </x:c>
+      <x:c r="C374" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A374,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D374" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E374" s="3" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F374" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="375" ht="65" customHeight="1">
+      <x:c r="A375" s="3" t="str">
+        <x:v>proposal.legger.sample_rack</x:v>
+      </x:c>
+      <x:c r="B375" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A375,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger sample-vial rack</x:v>
+      </x:c>
+      <x:c r="C375" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A375,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D375" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E375" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A375,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F375" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="376" ht="65" customHeight="1">
+      <x:c r="A376" s="3" t="str">
+        <x:v>proposal.legger.ore_bin</x:v>
+      </x:c>
+      <x:c r="B376" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A376,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger removable ore bin</x:v>
+      </x:c>
+      <x:c r="C376" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A376,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D376" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E376" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A376,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F376" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="377" ht="65" customHeight="1">
+      <x:c r="A377" s="3" t="str">
+        <x:v>proposal.legger.long_load_clamp</x:v>
+      </x:c>
+      <x:c r="B377" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A377,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger long-load clamp</x:v>
+      </x:c>
+      <x:c r="C377" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A377,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D377" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E377" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A377,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F377" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="378" ht="65" customHeight="1">
+      <x:c r="A378" s="3" t="str">
+        <x:v>proposal.legger.long_load_clamp</x:v>
+      </x:c>
+      <x:c r="B378" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A378,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger long-load clamp</x:v>
+      </x:c>
+      <x:c r="C378" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A378,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D378" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E378" s="3" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F378" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="379" ht="65" customHeight="1">
+      <x:c r="A379" s="3" t="str">
+        <x:v>proposal.legger.release_latch</x:v>
+      </x:c>
+      <x:c r="B379" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A379,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo quick-release latch</x:v>
+      </x:c>
+      <x:c r="C379" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A379,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D379" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E379" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A379,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F379" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="380" ht="65" customHeight="1">
+      <x:c r="A380" s="3" t="str">
+        <x:v>proposal.legger.board_bracket</x:v>
+      </x:c>
+      <x:c r="B380" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A380,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger dirtboard carrying bracket</x:v>
+      </x:c>
+      <x:c r="C380" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A380,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D380" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E380" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A380,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F380" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="381" ht="65" customHeight="1">
+      <x:c r="A381" s="3" t="str">
+        <x:v>proposal.legger.board_bracket</x:v>
+      </x:c>
+      <x:c r="B381" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A381,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger dirtboard carrying bracket</x:v>
+      </x:c>
+      <x:c r="C381" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A381,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D381" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E381" s="3" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F381" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="382" ht="65" customHeight="1">
+      <x:c r="A382" s="3" t="str">
+        <x:v>proposal.legger.hinge_plate</x:v>
+      </x:c>
+      <x:c r="B382" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A382,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chassis hinge-mount plate</x:v>
+      </x:c>
+      <x:c r="C382" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A382,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D382" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E382" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A382,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F382" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="383" ht="65" customHeight="1">
+      <x:c r="A383" s="3" t="str">
+        <x:v>proposal.legger.hinge_plate</x:v>
+      </x:c>
+      <x:c r="B383" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A383,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chassis hinge-mount plate</x:v>
+      </x:c>
+      <x:c r="C383" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A383,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D383" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E383" s="3" t="str">
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F383" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="384" ht="65" customHeight="1">
+      <x:c r="A384" s="3" t="str">
+        <x:v>proposal.legger.inspection_hatch</x:v>
+      </x:c>
+      <x:c r="B384" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A384,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger inspection hatch</x:v>
+      </x:c>
+      <x:c r="C384" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A384,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D384" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E384" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A384,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="F384" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="385" ht="65" customHeight="1">
+      <x:c r="A385" s="3" t="str">
+        <x:v>proposal.legger.inspection_hatch</x:v>
+      </x:c>
+      <x:c r="B385" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A385,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger inspection hatch</x:v>
+      </x:c>
+      <x:c r="C385" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A385,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D385" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E385" s="3" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F385" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="386" ht="65" customHeight="1">
+      <x:c r="A386" s="3" t="str">
+        <x:v>proposal.legger.fracture_patch</x:v>
+      </x:c>
+      <x:c r="B386" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A386,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Iron chassis fracture patch</x:v>
+      </x:c>
+      <x:c r="C386" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A386,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D386" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E386" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A386,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F386" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="387" ht="65" customHeight="1">
+      <x:c r="A387" s="3" t="str">
+        <x:v>proposal.legger.crush_mount</x:v>
+      </x:c>
+      <x:c r="B387" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A387,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Sacrificial attachment mount</x:v>
+      </x:c>
+      <x:c r="C387" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A387,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D387" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E387" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A387,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F387" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="388" ht="65" customHeight="1">
+      <x:c r="A388" s="3" t="str">
+        <x:v>proposal.legger.crush_mount</x:v>
+      </x:c>
+      <x:c r="B388" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A388,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Sacrificial attachment mount</x:v>
+      </x:c>
+      <x:c r="C388" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A388,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D388" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E388" s="3" t="str">
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F388" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="389" ht="65" customHeight="1">
+      <x:c r="A389" s="3" t="str">
+        <x:v>proposal.legger.bulkhead_ring</x:v>
+      </x:c>
+      <x:c r="B389" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A389,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chassis reinforcing ring</x:v>
+      </x:c>
+      <x:c r="C389" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A389,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D389" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E389" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A389,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment fabrication</x:v>
+      </x:c>
+      <x:c r="F389" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="390" ht="65" customHeight="1">
+      <x:c r="A390" s="3" t="str">
+        <x:v>proposal.legger.alignment_shims</x:v>
+      </x:c>
+      <x:c r="B390" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A390,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chassis alignment-shim set</x:v>
+      </x:c>
+      <x:c r="C390" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A390,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D390" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E390" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A390,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F390" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="391" ht="65" customHeight="1">
+      <x:c r="A391" s="3" t="str">
+        <x:v>proposal.legger.joint_pin</x:v>
+      </x:c>
+      <x:c r="B391" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A391,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replaceable joint pin</x:v>
+      </x:c>
+      <x:c r="C391" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A391,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D391" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E391" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A391,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F391" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="392" ht="65" customHeight="1">
+      <x:c r="A392" s="3" t="str">
+        <x:v>proposal.legger.thrust_washer</x:v>
+      </x:c>
+      <x:c r="B392" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A392,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Joint thrust washer</x:v>
+      </x:c>
+      <x:c r="C392" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A392,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D392" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E392" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A392,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F392" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="393" ht="65" customHeight="1">
+      <x:c r="A393" s="3" t="str">
+        <x:v>proposal.legger.gear_cluster</x:v>
+      </x:c>
+      <x:c r="B393" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A393,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replacement gear cluster</x:v>
+      </x:c>
+      <x:c r="C393" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A393,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D393" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E393" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A393,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Machinery drive</x:v>
+      </x:c>
+      <x:c r="F393" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="394" ht="65" customHeight="1">
+      <x:c r="A394" s="3" t="str">
+        <x:v>proposal.legger.gear_cluster</x:v>
+      </x:c>
+      <x:c r="B394" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A394,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replacement gear cluster</x:v>
+      </x:c>
+      <x:c r="C394" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A394,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D394" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E394" s="3" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F394" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="395" ht="65" customHeight="1">
+      <x:c r="A395" s="3" t="str">
+        <x:v>proposal.legger.linkage_end</x:v>
+      </x:c>
+      <x:c r="B395" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A395,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Replacement linkage-end joint</x:v>
+      </x:c>
+      <x:c r="C395" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A395,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D395" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E395" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A395,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F395" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="396" ht="65" customHeight="1">
+      <x:c r="A396" s="3" t="str">
+        <x:v>proposal.legger.tensioner</x:v>
+      </x:c>
+      <x:c r="B396" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A396,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Drive tensioner assembly</x:v>
+      </x:c>
+      <x:c r="C396" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A396,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D396" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E396" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A396,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Machinery drive</x:v>
+      </x:c>
+      <x:c r="F396" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="397" ht="65" customHeight="1">
+      <x:c r="A397" s="3" t="str">
+        <x:v>proposal.legger.tensioner</x:v>
+      </x:c>
+      <x:c r="B397" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A397,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Drive tensioner assembly</x:v>
+      </x:c>
+      <x:c r="C397" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A397,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D397" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E397" s="3" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F397" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="398" ht="65" customHeight="1">
+      <x:c r="A398" s="3" t="str">
+        <x:v>proposal.legger.scraper_ring</x:v>
+      </x:c>
+      <x:c r="B398" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A398,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Joint grit-scraper ring</x:v>
+      </x:c>
+      <x:c r="C398" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A398,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D398" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E398" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A398,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dust exclusion</x:v>
+      </x:c>
+      <x:c r="F398" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="399" ht="65" customHeight="1">
+      <x:c r="A399" s="3" t="str">
+        <x:v>proposal.legger.scraper_ring</x:v>
+      </x:c>
+      <x:c r="B399" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A399,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Joint grit-scraper ring</x:v>
+      </x:c>
+      <x:c r="C399" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A399,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D399" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E399" s="3" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F399" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="400" ht="65" customHeight="1">
+      <x:c r="A400" s="3" t="str">
+        <x:v>proposal.legger.grease_applicator</x:v>
+      </x:c>
+      <x:c r="B400" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A400,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Joint grease applicator</x:v>
+      </x:c>
+      <x:c r="C400" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A400,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D400" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E400" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A400,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F400" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="401" ht="65" customHeight="1">
+      <x:c r="A401" s="3" t="str">
+        <x:v>proposal.legger.grease_applicator</x:v>
+      </x:c>
+      <x:c r="B401" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A401,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Joint grease applicator</x:v>
+      </x:c>
+      <x:c r="C401" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A401,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D401" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E401" s="3" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F401" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="402" ht="65" customHeight="1">
+      <x:c r="A402" s="3" t="str">
+        <x:v>proposal.legger.service_adapter</x:v>
+      </x:c>
+      <x:c r="B402" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A402,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubricant service-port adapter</x:v>
+      </x:c>
+      <x:c r="C402" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A402,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D402" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E402" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A402,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Material transfer</x:v>
+      </x:c>
+      <x:c r="F402" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="403" ht="65" customHeight="1">
+      <x:c r="A403" s="3" t="str">
+        <x:v>proposal.legger.service_adapter</x:v>
+      </x:c>
+      <x:c r="B403" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A403,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Lubricant service-port adapter</x:v>
+      </x:c>
+      <x:c r="C403" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A403,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D403" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E403" s="3" t="str">
+        <x:v>Lubrication</x:v>
+      </x:c>
+      <x:c r="F403" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="404" ht="65" customHeight="1">
+      <x:c r="A404" s="3" t="str">
+        <x:v>proposal.legger.service_pick</x:v>
+      </x:c>
+      <x:c r="B404" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A404,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Joint-service cleaning pick</x:v>
+      </x:c>
+      <x:c r="C404" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A404,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D404" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E404" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A404,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cleaning</x:v>
+      </x:c>
+      <x:c r="F404" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="405" ht="65" customHeight="1">
+      <x:c r="A405" s="3" t="str">
+        <x:v>proposal.legger.service_pick</x:v>
+      </x:c>
+      <x:c r="B405" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A405,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Joint-service cleaning pick</x:v>
+      </x:c>
+      <x:c r="C405" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A405,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D405" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E405" s="3" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F405" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="406" ht="65" customHeight="1">
+      <x:c r="A406" s="3" t="str">
+        <x:v>proposal.legger.bearing_puller</x:v>
+      </x:c>
+      <x:c r="B406" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A406,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Matched bearing-removal tool</x:v>
+      </x:c>
+      <x:c r="C406" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A406,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D406" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E406" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A406,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F406" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="407" ht="65" customHeight="1">
+      <x:c r="A407" s="3" t="str">
+        <x:v>proposal.legger.alignment_gauge</x:v>
+      </x:c>
+      <x:c r="B407" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A407,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger alignment gauge</x:v>
+      </x:c>
+      <x:c r="C407" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A407,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D407" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E407" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A407,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="F407" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="408" ht="65" customHeight="1">
+      <x:c r="A408" s="3" t="str">
+        <x:v>proposal.legger.alignment_gauge</x:v>
+      </x:c>
+      <x:c r="B408" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A408,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger alignment gauge</x:v>
+      </x:c>
+      <x:c r="C408" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A408,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D408" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E408" s="3" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F408" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="409" ht="65" customHeight="1">
+      <x:c r="A409" s="3" t="str">
+        <x:v>proposal.legger.spares_case</x:v>
+      </x:c>
+      <x:c r="B409" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A409,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Legger fitted spares case</x:v>
+      </x:c>
+      <x:c r="C409" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A409,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D409" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E409" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A409,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F409" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="410" ht="65" customHeight="1">
+      <x:c r="A410" s="3" t="str">
+        <x:v>proposal.legger.edge_guard</x:v>
+      </x:c>
+      <x:c r="B410" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A410,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Chassis leading-edge guard</x:v>
+      </x:c>
+      <x:c r="C410" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A410,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D410" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E410" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A410,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F410" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="411" ht="65" customHeight="1">
+      <x:c r="A411" s="3" t="str">
+        <x:v>proposal.legger.instrument_guard</x:v>
+      </x:c>
+      <x:c r="B411" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A411,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Instrument-face guard</x:v>
+      </x:c>
+      <x:c r="C411" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A411,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D411" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E411" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A411,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F411" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="412" ht="65" customHeight="1">
+      <x:c r="A412" s="3" t="str">
+        <x:v>proposal.legger.seam_guard</x:v>
+      </x:c>
+      <x:c r="B412" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A412,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Armor seam-cover strip</x:v>
+      </x:c>
+      <x:c r="C412" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A412,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D412" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E412" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A412,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F412" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="413" ht="65" customHeight="1">
+      <x:c r="A413" s="3" t="str">
+        <x:v>proposal.legger.impact_cap</x:v>
+      </x:c>
+      <x:c r="B413" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A413,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Sacrificial impact cap</x:v>
+      </x:c>
+      <x:c r="C413" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A413,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D413" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E413" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A413,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F413" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="414" ht="65" customHeight="1">
+      <x:c r="A414" s="3" t="str">
+        <x:v>proposal.legger.fragment_liner</x:v>
+      </x:c>
+      <x:c r="B414" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A414,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Pressed-husk fragment liner</x:v>
+      </x:c>
+      <x:c r="C414" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A414,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D414" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E414" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A414,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F414" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="415" ht="65" customHeight="1">
+      <x:c r="A415" s="3" t="str">
+        <x:v>proposal.legger.guard_hinge</x:v>
+      </x:c>
+      <x:c r="B415" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A415,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Armor-guard hinge assembly</x:v>
+      </x:c>
+      <x:c r="C415" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A415,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D415" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E415" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A415,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F415" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="416" ht="65" customHeight="1">
+      <x:c r="A416" s="3" t="str">
+        <x:v>proposal.legger.guard_hinge</x:v>
+      </x:c>
+      <x:c r="B416" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A416,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Armor-guard hinge assembly</x:v>
+      </x:c>
+      <x:c r="C416" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A416,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D416" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E416" s="3" t="str">
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F416" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="417" ht="65" customHeight="1">
+      <x:c r="A417" s="3" t="str">
+        <x:v>proposal.legger.plasteel_collar</x:v>
+      </x:c>
+      <x:c r="B417" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A417,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient plasteel joint collar</x:v>
+      </x:c>
+      <x:c r="C417" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A417,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D417" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E417" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A417,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F417" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="418" ht="65" customHeight="1">
+      <x:c r="A418" s="3" t="str">
+        <x:v>proposal.legger.tension_member</x:v>
+      </x:c>
+      <x:c r="B418" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A418,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient nanocarbon tension member</x:v>
+      </x:c>
+      <x:c r="C418" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A418,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D418" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E418" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A418,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F418" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="419" ht="65" customHeight="1">
+      <x:c r="A419" s="3" t="str">
+        <x:v>proposal.legger.friction_insert</x:v>
+      </x:c>
+      <x:c r="B419" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A419,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient friction-interface insert</x:v>
+      </x:c>
+      <x:c r="C419" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A419,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D419" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E419" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A419,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F419" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="420" ht="65" customHeight="1">
+      <x:c r="A420" s="3" t="str">
+        <x:v>proposal.legger.ceramic_race</x:v>
+      </x:c>
+      <x:c r="B420" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A420,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient precision ceramic bearing race</x:v>
+      </x:c>
+      <x:c r="C420" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A420,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D420" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E420" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A420,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment repair</x:v>
+      </x:c>
+      <x:c r="F420" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="421" ht="65" customHeight="1">
+      <x:c r="A421" s="3" t="str">
+        <x:v>proposal.legger.impact_lattice</x:v>
+      </x:c>
+      <x:c r="B421" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A421,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient impact-lattice backing</x:v>
+      </x:c>
+      <x:c r="C421" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A421,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="D421" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E421" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A421,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Protection</x:v>
+      </x:c>
+      <x:c r="F421" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="422" ht="65" customHeight="1">
+      <x:c r="A422" s="3" t="str">
+        <x:v>proposal.legger.interface_adapter</x:v>
+      </x:c>
+      <x:c r="B422" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A422,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Ancient module interface adapter</x:v>
+      </x:c>
+      <x:c r="C422" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A422,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crafting components</x:v>
+      </x:c>
+      <x:c r="D422" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E422" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A422,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Equipment mounting</x:v>
+      </x:c>
+      <x:c r="F422" s="3" t="str">
+        <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A6:A1005">
-      <x:formula1>'Items'!$A$6:$A$268</x:formula1>
+      <x:formula1>'Items'!$A$6:$A$304</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D6:D1005">
       <x:formula1>"Primary,Secondary"</x:formula1>
@@ -33582,7 +37574,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb650c84453cf4e32"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8408375463a45e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34490,7 +38482,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b1f1157290d4092"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a46a4d87fe344df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34856,7 +38848,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36c05c50b9b4462e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10c4e4500c9f4365"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34917,7 +38909,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A6)</x:f>
-        <x:v>55</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>Existing gear plus armor, carriers, rare eyewear/headwear and very rare fashion families</x:v>
@@ -34962,7 +38954,7 @@
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A9)</x:f>
-        <x:v>62</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>Existing salvage and proposed materials, including husk-fiber paper and difficult pressed textiles</x:v>
@@ -35286,7 +39278,7 @@
       </x:c>
       <x:c r="B31" s="3" t="n">
         <x:f>COUNTIF(Items!$AA$6:$AA$1005,"Ceramic")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic feed mixture")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic and metal")</x:f>
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
         <x:v>28 new ceramic-specific feeds, intermediate blanks, tableware, storage, workshop tools, thermal/electrical parts, vessel fittings, ceremonial work and protection candidates</x:v>
@@ -35361,19 +39353,19 @@
       </x:c>
       <x:c r="B36" s="3" t="n">
         <x:f>COUNTIF(Items!$D$6:$D$1005,"Legger cargo rigging")+COUNTIF(Items!$D$6:$D$1005,"Legger chassis")+COUNTIF(Items!$D$6:$D$1005,"Legger mechanical parts")+COUNTIF(Items!$D$6:$D$1005,"Legger service parts")+COUNTIF(Items!$D$6:$D$1005,"Legger armor")+COUNTIF(Items!$D$6:$D$1005,"Legger ancient replacement")</x:f>
-        <x:v>24</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C36" s="3" t="str">
-        <x:v>24 proposals across cargo rigging, chassis, mechanical parts, service parts, armor and ancient replacements</x:v>
+        <x:v>60 proposals across cargo rigging, chassis, mechanical parts, service equipment, armor and ancient replacements</x:v>
       </x:c>
       <x:c r="D36" s="3" t="str">
-        <x:v>Legger-specific fit and physical ownership retained; ordinary iron repairs and extremely rare ancient replacements do not imply a linear upgrade ladder.</x:v>
+        <x:v>Includes 36 additional specific parts. Fit, function, serviceability and protective properties remain proposals.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b0576aad39641e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabefef62f3fd4078"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35436,7 +39428,7 @@
         <x:v>Items</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>263 design entries: 18 existing item IDs and 245 design/source concepts. Includes 24 Legger fitment and replacement proposals.</x:v>
+        <x:v>299 design entries: 18 existing item IDs and 281 design/source concepts. Includes 60 Legger parts and fitment proposals.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -36148,7 +40140,7 @@
         <x:v>Filtering the master</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Items is one native filterable table, A5:AE268. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
+        <x:v>Items is one native filterable table, A5:AE304. Category and Subtype retain earlier detail. New fields W:AC separate item type, processing stage, origin, primary use, material, form and status. Search terms are in AD. Freeze panes keep IDs/names visible while scrolling.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="85" customHeight="1">
@@ -36471,10 +40463,58 @@
         <x:v>Catalog work changes no world identity, chunk/terrain loading, persistent state, carrier limit or companion movement. Future installed parts need stable physical ownership, replacement/save behavior and compatibility. The Legger remains the same finite mobile carrier with local access.</x:v>
       </x:c>
     </x:row>
+    <x:row r="138" ht="105" customHeight="1">
+      <x:c r="A138" s="4" t="str">
+        <x:v>Expanded cargo rigging</x:v>
+      </x:c>
+      <x:c r="B138" s="4" t="str">
+        <x:v>Side pannier frames, sample-vial racks, removable ore bins, long-load clamps, release latches and a proposed dirtboard bracket add cargo-shape-specific ideas. Containers, stored gear and their contents retain separate ownership and finite physical limits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="105" customHeight="1">
+      <x:c r="A139" s="4" t="str">
+        <x:v>Expanded chassis and movement</x:v>
+      </x:c>
+      <x:c r="B139" s="4" t="str">
+        <x:v>Chassis hinge plates, access hatches, fracture patches, sacrificial mounts, reinforcement rings and shim sets address fitting and repair. Joint pins, thrust washers, gear clusters, linkage ends, tensioners and grit scrapers are host-specific mechanical proposals; inspect actual Legger anatomy before implementation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="105" customHeight="1">
+      <x:c r="A140" s="4" t="str">
+        <x:v>Expanded service equipment</x:v>
+      </x:c>
+      <x:c r="B140" s="4" t="str">
+        <x:v>Grease applicator, service-port adapter, cleaning pick, matched bearing-removal tool, alignment gauge and fitted spares case extend the lubricant/repair craft chain. These are tools and containers, distinct from installed service parts or magically complete repair kits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="105" customHeight="1">
+      <x:c r="A141" s="4" t="str">
+        <x:v>Expanded armor</x:v>
+      </x:c>
+      <x:c r="B141" s="4" t="str">
+        <x:v>Edge guards, instrument cages, seam strips, sacrificial caps, pressed-husk fragment liners and guard hinges address coverage and access. Specific wear, fragment retention and impact performance remain unverified; rare processed fiber inputs remain difficult to produce.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="105" customHeight="1">
+      <x:c r="A142" s="4" t="str">
+        <x:v>Expanded ancient replacements</x:v>
+      </x:c>
+      <x:c r="B142" s="4" t="str">
+        <x:v>Plasteel collars, nanocarbon tension members, unknown friction inserts, precision ceramic races, impact-lattice backing and module-specific adapters remain extremely rare recovered candidates. No universal interface, active muscle, self-repair or guaranteed ballistic effect is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="105" customHeight="1">
+      <x:c r="A143" s="4" t="str">
+        <x:v>Filter the expanded Legger set</x:v>
+      </x:c>
+      <x:c r="B143" s="4" t="str">
+        <x:v>60 Legger concepts now share six exact Subtype values: Legger cargo rigging, Legger chassis, Legger mechanical parts, Legger service parts, Legger armor and Legger ancient replacement. Use Item type to separate tools, containers, carriers, installed components and armor, and Item uses for repair, inspection, lubrication, mounting and protection.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb18fc306c55d4317"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec1e03cb1d56472e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37318,7 +41358,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2064bc84fd74a15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9fd875330ef4193"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37561,7 +41601,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc803812decfa4bf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c29314c6b274dfd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37965,7 +42005,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R460f93cf9bcd4d86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2a2bf301f4648e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38641,7 +42681,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49061129120245c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70c274d25e194ec3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add processed Phagia consumables and fauna delicacies
</commit_message>
<xml_diff>
--- a/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
+++ b/Docs/Design/Items/MASTER_ITEM_DATABASE.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R8acb532612b64c20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rf6c4040355514a37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R9b8fb9efc23647c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="R13d537377c714421"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Raa997f589ed242fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R5e0034a23d584f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R35ba0122792d4be6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="Ra1d142274d4d4994"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R988f37e70ff045aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="Rff7df799f7dc4fb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R884abbd129384bb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="R6f97e756b92e40ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="R644af9c6cc4542d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" r:id="R5a4c1fdf0de44bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="2" r:id="Rfcaba7b5b3c9403b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipes" sheetId="3" r:id="R249c3dac5a2841c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="4" r:id="Rc25002a91e2b448e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R7b20586181774de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource chains" sheetId="6" r:id="R8a954f63b63a4250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creature concepts" sheetId="7" r:id="R2a4b152fec79494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemical concepts" sheetId="8" r:id="R1284de7dca04461a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container concepts" sheetId="9" r:id="R5954b3aed9354757"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment concepts" sheetId="10" r:id="R322eb6b9a35b4ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canister concepts" sheetId="11" r:id="R9fd859b39215405a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="12" r:id="Rb1b07698f3534730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item uses" sheetId="13" r:id="R3610a3ba452f4148"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -493,8 +493,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="ItemsTable" displayName="ItemsTable" ref="A5:AE304" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AE304"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="ItemsTable" displayName="ItemsTable" ref="A5:AE318" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AE318"/>
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -569,8 +569,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C184" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:C184"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="ItemTaxonomy" displayName="ItemTaxonomy" ref="A5:C193" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:C193"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Field"/>
     <x:tableColumn id="2" name="Allowed value"/>
@@ -581,8 +581,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F422" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F422"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ItemUseRelationships" displayName="ItemUseRelationships" ref="A5:F441" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F441"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Item name"/>
@@ -636,8 +636,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="CategoriesTable" displayName="CategoriesTable" ref="A5:E40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:E40"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="CategoriesTable" displayName="CategoriesTable" ref="A5:E42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:E42"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Current coverage"/>
@@ -650,8 +650,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B147" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:B147"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GuideTable" displayName="GuideTable" ref="A5:B153" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:B153"/>
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Guidance"/>
@@ -1015,7 +1015,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>299 entries. Legger cargo rigging, chassis, replacements, service parts and armor are classified proposals. Search Legger or filter Subtype.</x:v>
+        <x:v>Prepared Phagia foods, drinks and delicacies extend the catalog. Filter Category/Type/Use; Search terms update from current labels and aliases.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -25524,6 +25524,1154 @@
         <x:v>Specific parts and protective properties remain proposals; ancient-material scarcity is established author direction.</x:v>
       </x:c>
     </x:row>
+    <x:row r="305" ht="115" customHeight="1">
+      <x:c r="A305" s="9" t="str">
+        <x:v>proposal.food.drink_portion</x:v>
+      </x:c>
+      <x:c r="B305" s="9" t="str">
+        <x:v>Prepared Phagia drink portion</x:v>
+      </x:c>
+      <x:c r="C305" s="9" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D305" s="9" t="str">
+        <x:v>Phagia drink</x:v>
+      </x:c>
+      <x:c r="E305" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F305" s="9" t="str">
+        <x:v>Prepared algae drink in a food-service vessel, intended to improve on an unprocessed baseline portion.</x:v>
+      </x:c>
+      <x:c r="G305" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H305" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I305" s="13"/>
+      <x:c r="J305" s="15"/>
+      <x:c r="K305" s="9" t="str">
+        <x:v>Specialist Phagia processing, provisioning or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L305" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M305" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N305" s="9" t="str">
+        <x:v>Serving size, preparation, performance and live-culture requirements TBD. Drinkable biological preparation is not a free-water resource.</x:v>
+      </x:c>
+      <x:c r="O305" s="17"/>
+      <x:c r="P305" s="17"/>
+      <x:c r="Q305" s="17"/>
+      <x:c r="R305" s="17"/>
+      <x:c r="S305" s="17"/>
+      <x:c r="T305" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U305" s="11" t="str">
+        <x:v>nutrition; phagea; algae</x:v>
+      </x:c>
+      <x:c r="V305" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W305" s="4" t="str">
+        <x:v>Drink consumable</x:v>
+      </x:c>
+      <x:c r="X305" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y305" s="4" t="str">
+        <x:v>Living culture</x:v>
+      </x:c>
+      <x:c r="Z305" s="4" t="str">
+        <x:v>Hydration</x:v>
+      </x:c>
+      <x:c r="AA305" s="4" t="str">
+        <x:v>Phagia preparation</x:v>
+      </x:c>
+      <x:c r="AB305" s="4" t="str">
+        <x:v>Liquid</x:v>
+      </x:c>
+      <x:c r="AC305" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD305" s="4" t="str">
+        <x:f>LOWER(A305&amp;"; "&amp;B305&amp;"; "&amp;C305&amp;"; "&amp;D305&amp;"; "&amp;W305&amp;"; "&amp;X305&amp;"; "&amp;Y305&amp;"; "&amp;Z305&amp;"; "&amp;AA305&amp;"; "&amp;AB305&amp;"; "&amp;AC305&amp;"; "&amp;U305)</x:f>
+        <x:v>proposal.food.drink_portion; prepared phagia drink portion; consumables; phagia drink; drink consumable; finished item; living culture; hydration; phagia preparation; liquid; author direction; nutrition; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE305" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="306" ht="115" customHeight="1">
+      <x:c r="A306" s="9" t="str">
+        <x:v>proposal.food.dense_drink</x:v>
+      </x:c>
+      <x:c r="B306" s="9" t="str">
+        <x:v>Dense Phagia nutrient drink</x:v>
+      </x:c>
+      <x:c r="C306" s="9" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D306" s="9" t="str">
+        <x:v>Phagia drink</x:v>
+      </x:c>
+      <x:c r="E306" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F306" s="9" t="str">
+        <x:v>Candidate concentrated drink preparation for a compact food-and-drink serving.</x:v>
+      </x:c>
+      <x:c r="G306" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H306" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I306" s="13"/>
+      <x:c r="J306" s="15"/>
+      <x:c r="K306" s="9" t="str">
+        <x:v>Specialist Phagia processing, provisioning or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L306" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M306" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N306" s="9" t="str">
+        <x:v>Drinkability, concentration process, nutritional benefit and hydration tradeoffs remain proposed; no dilution water or numeric effects assigned.</x:v>
+      </x:c>
+      <x:c r="O306" s="17"/>
+      <x:c r="P306" s="17"/>
+      <x:c r="Q306" s="17"/>
+      <x:c r="R306" s="17"/>
+      <x:c r="S306" s="17"/>
+      <x:c r="T306" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U306" s="11" t="str">
+        <x:v>hydration; phagea; algae</x:v>
+      </x:c>
+      <x:c r="V306" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W306" s="4" t="str">
+        <x:v>Drink consumable</x:v>
+      </x:c>
+      <x:c r="X306" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y306" s="4" t="str">
+        <x:v>Living culture</x:v>
+      </x:c>
+      <x:c r="Z306" s="4" t="str">
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="AA306" s="4" t="str">
+        <x:v>Phagia preparation</x:v>
+      </x:c>
+      <x:c r="AB306" s="4" t="str">
+        <x:v>Liquid</x:v>
+      </x:c>
+      <x:c r="AC306" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD306" s="4" t="str">
+        <x:f>LOWER(A306&amp;"; "&amp;B306&amp;"; "&amp;C306&amp;"; "&amp;D306&amp;"; "&amp;W306&amp;"; "&amp;X306&amp;"; "&amp;Y306&amp;"; "&amp;Z306&amp;"; "&amp;AA306&amp;"; "&amp;AB306&amp;"; "&amp;AC306&amp;"; "&amp;U306)</x:f>
+        <x:v>proposal.food.dense_drink; dense phagia nutrient drink; consumables; phagia drink; drink consumable; finished item; living culture; nutrition; phagia preparation; liquid; proposal; hydration; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE306" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="307" ht="115" customHeight="1">
+      <x:c r="A307" s="9" t="str">
+        <x:v>proposal.food.ration_bar</x:v>
+      </x:c>
+      <x:c r="B307" s="9" t="str">
+        <x:v>Phagia ration bar</x:v>
+      </x:c>
+      <x:c r="C307" s="9" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D307" s="9" t="str">
+        <x:v>Phagia bar</x:v>
+      </x:c>
+      <x:c r="E307" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F307" s="9" t="str">
+        <x:v>Prepared algae bar comparable in use to a protein/meal bar.</x:v>
+      </x:c>
+      <x:c r="G307" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H307" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I307" s="13"/>
+      <x:c r="J307" s="15"/>
+      <x:c r="K307" s="9" t="str">
+        <x:v>Specialist Phagia processing, provisioning or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L307" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M307" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N307" s="9" t="str">
+        <x:v>Comparison describes portable food format; exact protein composition, binding, serving size and benefits unresolved.</x:v>
+      </x:c>
+      <x:c r="O307" s="17"/>
+      <x:c r="P307" s="17"/>
+      <x:c r="Q307" s="17"/>
+      <x:c r="R307" s="17"/>
+      <x:c r="S307" s="17"/>
+      <x:c r="T307" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U307" s="11" t="str">
+        <x:v>phagea; algae</x:v>
+      </x:c>
+      <x:c r="V307" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W307" s="4" t="str">
+        <x:v>Food consumable</x:v>
+      </x:c>
+      <x:c r="X307" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y307" s="4" t="str">
+        <x:v>Living culture</x:v>
+      </x:c>
+      <x:c r="Z307" s="4" t="str">
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="AA307" s="4" t="str">
+        <x:v>Phagia preparation</x:v>
+      </x:c>
+      <x:c r="AB307" s="4" t="str">
+        <x:v>Solid piece</x:v>
+      </x:c>
+      <x:c r="AC307" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD307" s="4" t="str">
+        <x:f>LOWER(A307&amp;"; "&amp;B307&amp;"; "&amp;C307&amp;"; "&amp;D307&amp;"; "&amp;W307&amp;"; "&amp;X307&amp;"; "&amp;Y307&amp;"; "&amp;Z307&amp;"; "&amp;AA307&amp;"; "&amp;AB307&amp;"; "&amp;AC307&amp;"; "&amp;U307)</x:f>
+        <x:v>proposal.food.ration_bar; phagia ration bar; consumables; phagia bar; food consumable; finished item; living culture; nutrition; phagia preparation; solid piece; author direction; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE307" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="308" ht="115" customHeight="1">
+      <x:c r="A308" s="9" t="str">
+        <x:v>proposal.food.dried_bar</x:v>
+      </x:c>
+      <x:c r="B308" s="9" t="str">
+        <x:v>Dried Phagia travel bar</x:v>
+      </x:c>
+      <x:c r="C308" s="9" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D308" s="9" t="str">
+        <x:v>Phagia bar</x:v>
+      </x:c>
+      <x:c r="E308" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F308" s="9" t="str">
+        <x:v>Dried algae bar proposed as a processed travel consumable.</x:v>
+      </x:c>
+      <x:c r="G308" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H308" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I308" s="13"/>
+      <x:c r="J308" s="15"/>
+      <x:c r="K308" s="9" t="str">
+        <x:v>Specialist Phagia processing, provisioning or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L308" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M308" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N308" s="9" t="str">
+        <x:v>Drying method, retained compounds, texture and storage life require design. No hydration restoration inferred from a dry format.</x:v>
+      </x:c>
+      <x:c r="O308" s="17"/>
+      <x:c r="P308" s="17"/>
+      <x:c r="Q308" s="17"/>
+      <x:c r="R308" s="17"/>
+      <x:c r="S308" s="17"/>
+      <x:c r="T308" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U308" s="11" t="str">
+        <x:v>phagea; algae</x:v>
+      </x:c>
+      <x:c r="V308" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W308" s="4" t="str">
+        <x:v>Food consumable</x:v>
+      </x:c>
+      <x:c r="X308" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y308" s="4" t="str">
+        <x:v>Living culture</x:v>
+      </x:c>
+      <x:c r="Z308" s="4" t="str">
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="AA308" s="4" t="str">
+        <x:v>Phagia preparation</x:v>
+      </x:c>
+      <x:c r="AB308" s="4" t="str">
+        <x:v>Solid piece</x:v>
+      </x:c>
+      <x:c r="AC308" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD308" s="4" t="str">
+        <x:f>LOWER(A308&amp;"; "&amp;B308&amp;"; "&amp;C308&amp;"; "&amp;D308&amp;"; "&amp;W308&amp;"; "&amp;X308&amp;"; "&amp;Y308&amp;"; "&amp;Z308&amp;"; "&amp;AA308&amp;"; "&amp;AB308&amp;"; "&amp;AC308&amp;"; "&amp;U308)</x:f>
+        <x:v>proposal.food.dried_bar; dried phagia travel bar; consumables; phagia bar; food consumable; finished item; living culture; nutrition; phagia preparation; solid piece; author direction; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE308" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="309" ht="115" customHeight="1">
+      <x:c r="A309" s="9" t="str">
+        <x:v>proposal.food.meal_paste</x:v>
+      </x:c>
+      <x:c r="B309" s="9" t="str">
+        <x:v>Prepared Phagia meal paste</x:v>
+      </x:c>
+      <x:c r="C309" s="9" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D309" s="9" t="str">
+        <x:v>Phagia prepared meal</x:v>
+      </x:c>
+      <x:c r="E309" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F309" s="9" t="str">
+        <x:v>Smooth prepared algae meal candidate portioned for consumption.</x:v>
+      </x:c>
+      <x:c r="G309" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H309" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I309" s="13"/>
+      <x:c r="J309" s="15"/>
+      <x:c r="K309" s="9" t="str">
+        <x:v>Specialist Phagia processing, provisioning or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L309" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M309" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N309" s="9" t="str">
+        <x:v>Formulation, preparation, containment, food value and serving size remain open.</x:v>
+      </x:c>
+      <x:c r="O309" s="17"/>
+      <x:c r="P309" s="17"/>
+      <x:c r="Q309" s="17"/>
+      <x:c r="R309" s="17"/>
+      <x:c r="S309" s="17"/>
+      <x:c r="T309" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U309" s="11" t="str">
+        <x:v>phagea; algae</x:v>
+      </x:c>
+      <x:c r="V309" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W309" s="4" t="str">
+        <x:v>Food consumable</x:v>
+      </x:c>
+      <x:c r="X309" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y309" s="4" t="str">
+        <x:v>Living culture</x:v>
+      </x:c>
+      <x:c r="Z309" s="4" t="str">
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="AA309" s="4" t="str">
+        <x:v>Phagia preparation</x:v>
+      </x:c>
+      <x:c r="AB309" s="4" t="str">
+        <x:v>Paste</x:v>
+      </x:c>
+      <x:c r="AC309" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD309" s="4" t="str">
+        <x:f>LOWER(A309&amp;"; "&amp;B309&amp;"; "&amp;C309&amp;"; "&amp;D309&amp;"; "&amp;W309&amp;"; "&amp;X309&amp;"; "&amp;Y309&amp;"; "&amp;Z309&amp;"; "&amp;AA309&amp;"; "&amp;AB309&amp;"; "&amp;AC309&amp;"; "&amp;U309)</x:f>
+        <x:v>proposal.food.meal_paste; prepared phagia meal paste; consumables; phagia prepared meal; food consumable; finished item; living culture; nutrition; phagia preparation; paste; proposal; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE309" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="310" ht="115" customHeight="1">
+      <x:c r="A310" s="9" t="str">
+        <x:v>proposal.food.meal_portion</x:v>
+      </x:c>
+      <x:c r="B310" s="9" t="str">
+        <x:v>Prepared Phagia meal portion</x:v>
+      </x:c>
+      <x:c r="C310" s="9" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D310" s="9" t="str">
+        <x:v>Phagia prepared meal</x:v>
+      </x:c>
+      <x:c r="E310" s="9" t="str">
+        <x:v>User direction; not implemented</x:v>
+      </x:c>
+      <x:c r="F310" s="9" t="str">
+        <x:v>Prepared consumable meal based on the survival algae.</x:v>
+      </x:c>
+      <x:c r="G310" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H310" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I310" s="13"/>
+      <x:c r="J310" s="15"/>
+      <x:c r="K310" s="9" t="str">
+        <x:v>Specialist Phagia processing, provisioning or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L310" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M310" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N310" s="9" t="str">
+        <x:v>Warmed, cold-set or other preparation routes remain open; cooking follows the world fire rules. No universal healing or stamina effect.</x:v>
+      </x:c>
+      <x:c r="O310" s="17"/>
+      <x:c r="P310" s="17"/>
+      <x:c r="Q310" s="17"/>
+      <x:c r="R310" s="17"/>
+      <x:c r="S310" s="17"/>
+      <x:c r="T310" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U310" s="11" t="str">
+        <x:v>phagea; algae</x:v>
+      </x:c>
+      <x:c r="V310" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W310" s="4" t="str">
+        <x:v>Food consumable</x:v>
+      </x:c>
+      <x:c r="X310" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y310" s="4" t="str">
+        <x:v>Living culture</x:v>
+      </x:c>
+      <x:c r="Z310" s="4" t="str">
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="AA310" s="4" t="str">
+        <x:v>Phagia preparation</x:v>
+      </x:c>
+      <x:c r="AB310" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AC310" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="AD310" s="4" t="str">
+        <x:f>LOWER(A310&amp;"; "&amp;B310&amp;"; "&amp;C310&amp;"; "&amp;D310&amp;"; "&amp;W310&amp;"; "&amp;X310&amp;"; "&amp;Y310&amp;"; "&amp;Z310&amp;"; "&amp;AA310&amp;"; "&amp;AB310&amp;"; "&amp;AC310&amp;"; "&amp;U310)</x:f>
+        <x:v>proposal.food.meal_portion; prepared phagia meal portion; consumables; phagia prepared meal; food consumable; finished item; living culture; nutrition; phagia preparation; unresolved; author direction; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE310" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="311" ht="115" customHeight="1">
+      <x:c r="A311" s="9" t="str">
+        <x:v>proposal.food.fauna_flake_dish</x:v>
+      </x:c>
+      <x:c r="B311" s="9" t="str">
+        <x:v>Phagia and edible-fauna flake delicacy</x:v>
+      </x:c>
+      <x:c r="C311" s="9" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D311" s="9" t="str">
+        <x:v>Phagia delicacy</x:v>
+      </x:c>
+      <x:c r="E311" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F311" s="9" t="str">
+        <x:v>Candidate fine meal combining algae with selected prepared edible fauna flakes.</x:v>
+      </x:c>
+      <x:c r="G311" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H311" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I311" s="13"/>
+      <x:c r="J311" s="15"/>
+      <x:c r="K311" s="9" t="str">
+        <x:v>Specialist Phagia processing, provisioning or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L311" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M311" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N311" s="9" t="str">
+        <x:v>Species and exact edible fraction unresolved. Fauna contributes culinary character; improved nutritional performance is not assumed to come from fauna.</x:v>
+      </x:c>
+      <x:c r="O311" s="17"/>
+      <x:c r="P311" s="17"/>
+      <x:c r="Q311" s="17"/>
+      <x:c r="R311" s="17"/>
+      <x:c r="S311" s="17"/>
+      <x:c r="T311" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U311" s="11" t="str">
+        <x:v>phagea; algae</x:v>
+      </x:c>
+      <x:c r="V311" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W311" s="4" t="str">
+        <x:v>Food consumable</x:v>
+      </x:c>
+      <x:c r="X311" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y311" s="4" t="str">
+        <x:v>Biological mixture</x:v>
+      </x:c>
+      <x:c r="Z311" s="4" t="str">
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="AA311" s="4" t="str">
+        <x:v>Phagia and edible fauna</x:v>
+      </x:c>
+      <x:c r="AB311" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AC311" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD311" s="4" t="str">
+        <x:f>LOWER(A311&amp;"; "&amp;B311&amp;"; "&amp;C311&amp;"; "&amp;D311&amp;"; "&amp;W311&amp;"; "&amp;X311&amp;"; "&amp;Y311&amp;"; "&amp;Z311&amp;"; "&amp;AA311&amp;"; "&amp;AB311&amp;"; "&amp;AC311&amp;"; "&amp;U311)</x:f>
+        <x:v>proposal.food.fauna_flake_dish; phagia and edible-fauna flake delicacy; consumables; phagia delicacy; food consumable; finished item; biological mixture; nutrition; phagia and edible fauna; unresolved; proposal; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE311" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="312" ht="115" customHeight="1">
+      <x:c r="A312" s="9" t="str">
+        <x:v>proposal.food.layered_delicacy</x:v>
+      </x:c>
+      <x:c r="B312" s="9" t="str">
+        <x:v>Layered Phagia-fauna delicacy</x:v>
+      </x:c>
+      <x:c r="C312" s="9" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D312" s="9" t="str">
+        <x:v>Phagia delicacy</x:v>
+      </x:c>
+      <x:c r="E312" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F312" s="9" t="str">
+        <x:v>Candidate composed meal using distinct prepared algae and edible-fauna layers.</x:v>
+      </x:c>
+      <x:c r="G312" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H312" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I312" s="13"/>
+      <x:c r="J312" s="15"/>
+      <x:c r="K312" s="9" t="str">
+        <x:v>Specialist Phagia processing, provisioning or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L312" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M312" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N312" s="9" t="str">
+        <x:v>Layering, texture, service method and skilled preparation differentiate this culinary concept; no accepted recipe or rarity.</x:v>
+      </x:c>
+      <x:c r="O312" s="17"/>
+      <x:c r="P312" s="17"/>
+      <x:c r="Q312" s="17"/>
+      <x:c r="R312" s="17"/>
+      <x:c r="S312" s="17"/>
+      <x:c r="T312" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U312" s="11" t="str">
+        <x:v>phagea; algae</x:v>
+      </x:c>
+      <x:c r="V312" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W312" s="4" t="str">
+        <x:v>Food consumable</x:v>
+      </x:c>
+      <x:c r="X312" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y312" s="4" t="str">
+        <x:v>Biological mixture</x:v>
+      </x:c>
+      <x:c r="Z312" s="4" t="str">
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="AA312" s="4" t="str">
+        <x:v>Phagia and edible fauna</x:v>
+      </x:c>
+      <x:c r="AB312" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="AC312" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD312" s="4" t="str">
+        <x:f>LOWER(A312&amp;"; "&amp;B312&amp;"; "&amp;C312&amp;"; "&amp;D312&amp;"; "&amp;W312&amp;"; "&amp;X312&amp;"; "&amp;Y312&amp;"; "&amp;Z312&amp;"; "&amp;AA312&amp;"; "&amp;AB312&amp;"; "&amp;AC312&amp;"; "&amp;U312)</x:f>
+        <x:v>proposal.food.layered_delicacy; layered phagia-fauna delicacy; consumables; phagia delicacy; food consumable; finished item; biological mixture; nutrition; phagia and edible fauna; unresolved; proposal; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE312" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="313" ht="115" customHeight="1">
+      <x:c r="A313" s="9" t="str">
+        <x:v>proposal.food.crisp_delicacy</x:v>
+      </x:c>
+      <x:c r="B313" s="9" t="str">
+        <x:v>Crisp Phagia-fauna wafer</x:v>
+      </x:c>
+      <x:c r="C313" s="9" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D313" s="9" t="str">
+        <x:v>Phagia delicacy</x:v>
+      </x:c>
+      <x:c r="E313" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F313" s="9" t="str">
+        <x:v>Candidate delicate crisp combining processed algae and a selected edible fauna ingredient.</x:v>
+      </x:c>
+      <x:c r="G313" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H313" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I313" s="13"/>
+      <x:c r="J313" s="15"/>
+      <x:c r="K313" s="9" t="str">
+        <x:v>Specialist Phagia processing, provisioning or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L313" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M313" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N313" s="9" t="str">
+        <x:v>Edible binders, crisping method and food safety remain open. It is a proposed delicacy, not an automatic dried-bar ingredient substitution.</x:v>
+      </x:c>
+      <x:c r="O313" s="17"/>
+      <x:c r="P313" s="17"/>
+      <x:c r="Q313" s="17"/>
+      <x:c r="R313" s="17"/>
+      <x:c r="S313" s="17"/>
+      <x:c r="T313" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U313" s="11" t="str">
+        <x:v>phagea; algae</x:v>
+      </x:c>
+      <x:c r="V313" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W313" s="4" t="str">
+        <x:v>Food consumable</x:v>
+      </x:c>
+      <x:c r="X313" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y313" s="4" t="str">
+        <x:v>Biological mixture</x:v>
+      </x:c>
+      <x:c r="Z313" s="4" t="str">
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="AA313" s="4" t="str">
+        <x:v>Phagia and edible fauna</x:v>
+      </x:c>
+      <x:c r="AB313" s="4" t="str">
+        <x:v>Solid piece</x:v>
+      </x:c>
+      <x:c r="AC313" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD313" s="4" t="str">
+        <x:f>LOWER(A313&amp;"; "&amp;B313&amp;"; "&amp;C313&amp;"; "&amp;D313&amp;"; "&amp;W313&amp;"; "&amp;X313&amp;"; "&amp;Y313&amp;"; "&amp;Z313&amp;"; "&amp;AA313&amp;"; "&amp;AB313&amp;"; "&amp;AC313&amp;"; "&amp;U313)</x:f>
+        <x:v>proposal.food.crisp_delicacy; crisp phagia-fauna wafer; consumables; phagia delicacy; food consumable; finished item; biological mixture; nutrition; phagia and edible fauna; solid piece; proposal; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE313" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="314" ht="115" customHeight="1">
+      <x:c r="A314" s="9" t="str">
+        <x:v>proposal.food.edible_flakes</x:v>
+      </x:c>
+      <x:c r="B314" s="9" t="str">
+        <x:v>Prepared edible-fauna flakes</x:v>
+      </x:c>
+      <x:c r="C314" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D314" s="9" t="str">
+        <x:v>Prepared fauna food ingredient</x:v>
+      </x:c>
+      <x:c r="E314" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F314" s="9" t="str">
+        <x:v>Selected known-edible fauna fraction prepared as a possible Phagia meal ingredient.</x:v>
+      </x:c>
+      <x:c r="G314" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H314" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I314" s="13"/>
+      <x:c r="J314" s="15"/>
+      <x:c r="K314" s="9" t="str">
+        <x:v>Prepare selected edible-fauna fraction; method TBD</x:v>
+      </x:c>
+      <x:c r="L314" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M314" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N314" s="9" t="str">
+        <x:v>Reuses existing generic edible fauna fraction. Selection, preparation and retained toxicity require species-specific design; conventional meat is not assumed.</x:v>
+      </x:c>
+      <x:c r="O314" s="17"/>
+      <x:c r="P314" s="17"/>
+      <x:c r="Q314" s="17"/>
+      <x:c r="R314" s="17"/>
+      <x:c r="S314" s="17"/>
+      <x:c r="T314" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U314" s="11" t="str">
+        <x:v>phagea; algae</x:v>
+      </x:c>
+      <x:c r="V314" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W314" s="4" t="str">
+        <x:v>Food material</x:v>
+      </x:c>
+      <x:c r="X314" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y314" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z314" s="4" t="str">
+        <x:v>Food preparation</x:v>
+      </x:c>
+      <x:c r="AA314" s="4" t="str">
+        <x:v>Faunal tissue</x:v>
+      </x:c>
+      <x:c r="AB314" s="4" t="str">
+        <x:v>Particles</x:v>
+      </x:c>
+      <x:c r="AC314" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD314" s="4" t="str">
+        <x:f>LOWER(A314&amp;"; "&amp;B314&amp;"; "&amp;C314&amp;"; "&amp;D314&amp;"; "&amp;W314&amp;"; "&amp;X314&amp;"; "&amp;Y314&amp;"; "&amp;Z314&amp;"; "&amp;AA314&amp;"; "&amp;AB314&amp;"; "&amp;AC314&amp;"; "&amp;U314)</x:f>
+        <x:v>proposal.food.edible_flakes; prepared edible-fauna flakes; resources; prepared fauna food ingredient; food material; processed intermediate; fauna; food preparation; faunal tissue; particles; proposal; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE314" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="315" ht="115" customHeight="1">
+      <x:c r="A315" s="9" t="str">
+        <x:v>proposal.food.edible_paste</x:v>
+      </x:c>
+      <x:c r="B315" s="9" t="str">
+        <x:v>Prepared edible-fauna paste</x:v>
+      </x:c>
+      <x:c r="C315" s="9" t="str">
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D315" s="9" t="str">
+        <x:v>Prepared fauna food ingredient</x:v>
+      </x:c>
+      <x:c r="E315" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F315" s="9" t="str">
+        <x:v>Selected edible fauna fraction prepared for mixing or layering with algae.</x:v>
+      </x:c>
+      <x:c r="G315" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H315" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I315" s="13"/>
+      <x:c r="J315" s="15"/>
+      <x:c r="K315" s="9" t="str">
+        <x:v>Prepare selected edible-fauna fraction; method TBD</x:v>
+      </x:c>
+      <x:c r="L315" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M315" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N315" s="9" t="str">
+        <x:v>Preparation is not automatic detoxification. Nutritional contribution remains low; chemistry used for machinery is not a food substitute.</x:v>
+      </x:c>
+      <x:c r="O315" s="17"/>
+      <x:c r="P315" s="17"/>
+      <x:c r="Q315" s="17"/>
+      <x:c r="R315" s="17"/>
+      <x:c r="S315" s="17"/>
+      <x:c r="T315" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U315" s="11" t="str">
+        <x:v>phagea; algae</x:v>
+      </x:c>
+      <x:c r="V315" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W315" s="4" t="str">
+        <x:v>Food material</x:v>
+      </x:c>
+      <x:c r="X315" s="4" t="str">
+        <x:v>Processed intermediate</x:v>
+      </x:c>
+      <x:c r="Y315" s="4" t="str">
+        <x:v>Fauna</x:v>
+      </x:c>
+      <x:c r="Z315" s="4" t="str">
+        <x:v>Food preparation</x:v>
+      </x:c>
+      <x:c r="AA315" s="4" t="str">
+        <x:v>Faunal tissue</x:v>
+      </x:c>
+      <x:c r="AB315" s="4" t="str">
+        <x:v>Paste</x:v>
+      </x:c>
+      <x:c r="AC315" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD315" s="4" t="str">
+        <x:f>LOWER(A315&amp;"; "&amp;B315&amp;"; "&amp;C315&amp;"; "&amp;D315&amp;"; "&amp;W315&amp;"; "&amp;X315&amp;"; "&amp;Y315&amp;"; "&amp;Z315&amp;"; "&amp;AA315&amp;"; "&amp;AB315&amp;"; "&amp;AC315&amp;"; "&amp;U315)</x:f>
+        <x:v>proposal.food.edible_paste; prepared edible-fauna paste; resources; prepared fauna food ingredient; food material; processed intermediate; fauna; food preparation; faunal tissue; paste; proposal; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE315" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="316" ht="115" customHeight="1">
+      <x:c r="A316" s="9" t="str">
+        <x:v>proposal.food.drink_flask</x:v>
+      </x:c>
+      <x:c r="B316" s="9" t="str">
+        <x:v>Reusable Phagia drinking flask</x:v>
+      </x:c>
+      <x:c r="C316" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D316" s="9" t="str">
+        <x:v>Food packaging</x:v>
+      </x:c>
+      <x:c r="E316" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F316" s="9" t="str">
+        <x:v>Dedicated food-contact vessel for a prepared Phagia drink portion.</x:v>
+      </x:c>
+      <x:c r="G316" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H316" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I316" s="13"/>
+      <x:c r="J316" s="15"/>
+      <x:c r="K316" s="9" t="str">
+        <x:v>Food-service craft or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L316" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M316" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N316" s="9" t="str">
+        <x:v>Vessel and edible payload are distinct. Refill, cleaning, seal compatibility and material qualification TBD; do not repurpose a contaminated reagent vessel.</x:v>
+      </x:c>
+      <x:c r="O316" s="17"/>
+      <x:c r="P316" s="17"/>
+      <x:c r="Q316" s="17"/>
+      <x:c r="R316" s="17"/>
+      <x:c r="S316" s="17"/>
+      <x:c r="T316" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U316" s="11" t="str">
+        <x:v>cargo organization; phagea; algae</x:v>
+      </x:c>
+      <x:c r="V316" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W316" s="4" t="str">
+        <x:v>Container</x:v>
+      </x:c>
+      <x:c r="X316" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y316" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z316" s="4" t="str">
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="AA316" s="4" t="str">
+        <x:v>Glass or ceramic</x:v>
+      </x:c>
+      <x:c r="AB316" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC316" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD316" s="4" t="str">
+        <x:f>LOWER(A316&amp;"; "&amp;B316&amp;"; "&amp;C316&amp;"; "&amp;D316&amp;"; "&amp;W316&amp;"; "&amp;X316&amp;"; "&amp;Y316&amp;"; "&amp;Z316&amp;"; "&amp;AA316&amp;"; "&amp;AB316&amp;"; "&amp;AC316&amp;"; "&amp;U316)</x:f>
+        <x:v>proposal.food.drink_flask; reusable phagia drinking flask; containers; food packaging; container; finished item; manufactured / unresolved; food service; glass or ceramic; assembly; proposal; cargo organization; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE316" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="317" ht="115" customHeight="1">
+      <x:c r="A317" s="9" t="str">
+        <x:v>proposal.food.bar_case</x:v>
+      </x:c>
+      <x:c r="B317" s="9" t="str">
+        <x:v>Phagia ration-bar case</x:v>
+      </x:c>
+      <x:c r="C317" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D317" s="9" t="str">
+        <x:v>Food packaging</x:v>
+      </x:c>
+      <x:c r="E317" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F317" s="9" t="str">
+        <x:v>Reusable fitted carrier protecting selected prepared bars from dust and damage.</x:v>
+      </x:c>
+      <x:c r="G317" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H317" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I317" s="13"/>
+      <x:c r="J317" s="15"/>
+      <x:c r="K317" s="9" t="str">
+        <x:v>Food-service craft or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L317" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M317" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N317" s="9" t="str">
+        <x:v>Bars count separately from their case. Food contact and closure remain design work; no cloth wrapper or invisible storage capacity.</x:v>
+      </x:c>
+      <x:c r="O317" s="17"/>
+      <x:c r="P317" s="17"/>
+      <x:c r="Q317" s="17"/>
+      <x:c r="R317" s="17"/>
+      <x:c r="S317" s="17"/>
+      <x:c r="T317" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U317" s="11" t="str">
+        <x:v>cargo organization; phagea; algae</x:v>
+      </x:c>
+      <x:c r="V317" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W317" s="4" t="str">
+        <x:v>Carrier</x:v>
+      </x:c>
+      <x:c r="X317" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y317" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z317" s="4" t="str">
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="AA317" s="4" t="str">
+        <x:v>Metal or shell</x:v>
+      </x:c>
+      <x:c r="AB317" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC317" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD317" s="4" t="str">
+        <x:f>LOWER(A317&amp;"; "&amp;B317&amp;"; "&amp;C317&amp;"; "&amp;D317&amp;"; "&amp;W317&amp;"; "&amp;X317&amp;"; "&amp;Y317&amp;"; "&amp;Z317&amp;"; "&amp;AA317&amp;"; "&amp;AB317&amp;"; "&amp;AC317&amp;"; "&amp;U317)</x:f>
+        <x:v>proposal.food.bar_case; phagia ration-bar case; containers; food packaging; carrier; finished item; manufactured / unresolved; food service; metal or shell; assembly; proposal; cargo organization; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE317" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="318" ht="115" customHeight="1">
+      <x:c r="A318" s="9" t="str">
+        <x:v>proposal.food.meal_carrier</x:v>
+      </x:c>
+      <x:c r="B318" s="9" t="str">
+        <x:v>Prepared-meal carrier</x:v>
+      </x:c>
+      <x:c r="C318" s="9" t="str">
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D318" s="9" t="str">
+        <x:v>Food packaging</x:v>
+      </x:c>
+      <x:c r="E318" s="9" t="str">
+        <x:v>New proposal</x:v>
+      </x:c>
+      <x:c r="F318" s="9" t="str">
+        <x:v>Lidded food-service carrier for a prepared algae meal portion.</x:v>
+      </x:c>
+      <x:c r="G318" s="9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H318" s="9" t="str">
+        <x:v>Prepared portions / vessels; Booter eligibility and capacity TBD</x:v>
+      </x:c>
+      <x:c r="I318" s="13"/>
+      <x:c r="J318" s="15"/>
+      <x:c r="K318" s="9" t="str">
+        <x:v>Food-service craft or trade; exact route TBD</x:v>
+      </x:c>
+      <x:c r="L318" s="9" t="str">
+        <x:v>No recipe, ratio or serving quantity authored. Food processing and any heating need setting-compatible design.</x:v>
+      </x:c>
+      <x:c r="M318" s="9" t="str">
+        <x:v>Not implemented</x:v>
+      </x:c>
+      <x:c r="N318" s="9" t="str">
+        <x:v>Build on existing ceramic lid/vessel craft. It is distinct from meal contents, a cooking pot and an industrial chemical jar.</x:v>
+      </x:c>
+      <x:c r="O318" s="17"/>
+      <x:c r="P318" s="17"/>
+      <x:c r="Q318" s="17"/>
+      <x:c r="R318" s="17"/>
+      <x:c r="S318" s="17"/>
+      <x:c r="T318" s="9" t="str">
+        <x:v>Higher-performing processed Phagia consumables and high-quality fauna-mixed delicacies are author direction. Specific performance, supply costs, value, shelf life and consumption behavior remain unresolved.</x:v>
+      </x:c>
+      <x:c r="U318" s="11" t="str">
+        <x:v>cargo organization; phagea; algae</x:v>
+      </x:c>
+      <x:c r="V318" s="9" t="str">
+        <x:v>Direct author Phagia food/drink processing and fauna-delicacy direction October 14, 2026; Docs/WORLD_BASIS.md#survival-rules. Specific named dishes and packaging are proposals.</x:v>
+      </x:c>
+      <x:c r="W318" s="4" t="str">
+        <x:v>Container</x:v>
+      </x:c>
+      <x:c r="X318" s="4" t="str">
+        <x:v>Finished item</x:v>
+      </x:c>
+      <x:c r="Y318" s="4" t="str">
+        <x:v>Manufactured / unresolved</x:v>
+      </x:c>
+      <x:c r="Z318" s="4" t="str">
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="AA318" s="4" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="AB318" s="4" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="AC318" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="AD318" s="4" t="str">
+        <x:f>LOWER(A318&amp;"; "&amp;B318&amp;"; "&amp;C318&amp;"; "&amp;D318&amp;"; "&amp;W318&amp;"; "&amp;X318&amp;"; "&amp;Y318&amp;"; "&amp;Z318&amp;"; "&amp;AA318&amp;"; "&amp;AB318&amp;"; "&amp;AC318&amp;"; "&amp;U318)</x:f>
+        <x:v>proposal.food.meal_carrier; prepared-meal carrier; containers; food packaging; container; finished item; manufactured / unresolved; food service; ceramic; assembly; proposal; cargo organization; phagea; algae</x:v>
+      </x:c>
+      <x:c r="AE318" s="4" t="str">
+        <x:v>Accepted direction for processed-food families; individual recipes, ingredient qualification and effects remain design proposals.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E6:E23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="trial"/>
@@ -25539,33 +26687,33 @@
   </x:conditionalFormatting>
   <x:dataValidations count="8">
     <x:dataValidation type="list" sqref="C6:C1005">
-      <x:formula1>'Taxonomy'!$B$6:$B$14</x:formula1>
+      <x:formula1>'Taxonomy'!$B$6:$B$15</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="W6:W1005">
-      <x:formula1>'Taxonomy'!$B$15:$B$38</x:formula1>
+      <x:formula1>'Taxonomy'!$B$16:$B$41</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="X6:X1005">
-      <x:formula1>'Taxonomy'!$B$39:$B$47</x:formula1>
+      <x:formula1>'Taxonomy'!$B$42:$B$50</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Y6:Y1005">
-      <x:formula1>'Taxonomy'!$B$48:$B$55</x:formula1>
+      <x:formula1>'Taxonomy'!$B$51:$B$59</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Z6:Z1005">
-      <x:formula1>'Taxonomy'!$B$56:$B$128</x:formula1>
+      <x:formula1>'Taxonomy'!$B$60:$B$134</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AA6:AA1005">
-      <x:formula1>'Taxonomy'!$B$129:$B$159</x:formula1>
+      <x:formula1>'Taxonomy'!$B$135:$B$168</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AB6:AB1005">
-      <x:formula1>'Taxonomy'!$B$160:$B$179</x:formula1>
+      <x:formula1>'Taxonomy'!$B$169:$B$188</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AC6:AC1005">
-      <x:formula1>'Taxonomy'!$B$180:$B$184</x:formula1>
+      <x:formula1>'Taxonomy'!$B$189:$B$193</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910c896bf9f54894"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R649a7e81d6374dea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26217,7 +27365,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R196eed82406e430e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9756e60a11b42f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26699,7 +27847,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3b06221ca0d4d23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb60a25e31f9b44f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26739,7 +27887,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B6" s="4" t="str">
-        <x:v>Containers</x:v>
+        <x:v>Consumables</x:v>
       </x:c>
       <x:c r="C6" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -26750,7 +27898,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B7" s="4" t="str">
-        <x:v>Crafting components</x:v>
+        <x:v>Containers</x:v>
       </x:c>
       <x:c r="C7" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -26761,7 +27909,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B8" s="4" t="str">
-        <x:v>Cultural objects</x:v>
+        <x:v>Crafting components</x:v>
       </x:c>
       <x:c r="C8" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -26772,7 +27920,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B9" s="4" t="str">
-        <x:v>Currency</x:v>
+        <x:v>Cultural objects</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -26783,7 +27931,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B10" s="4" t="str">
-        <x:v>Equipment</x:v>
+        <x:v>Currency</x:v>
       </x:c>
       <x:c r="C10" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -26794,7 +27942,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B11" s="4" t="str">
-        <x:v>Everyday objects</x:v>
+        <x:v>Equipment</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -26805,7 +27953,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B12" s="4" t="str">
-        <x:v>Field supplies</x:v>
+        <x:v>Everyday objects</x:v>
       </x:c>
       <x:c r="C12" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -26816,7 +27964,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B13" s="4" t="str">
-        <x:v>Resources</x:v>
+        <x:v>Field supplies</x:v>
       </x:c>
       <x:c r="C13" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -26827,7 +27975,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B14" s="4" t="str">
-        <x:v>Weapons</x:v>
+        <x:v>Resources</x:v>
       </x:c>
       <x:c r="C14" s="4" t="str">
         <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
@@ -26835,13 +27983,13 @@
     </x:row>
     <x:row r="15" ht="45" customHeight="1">
       <x:c r="A15" s="4" t="str">
-        <x:v>Item type</x:v>
+        <x:v>Category</x:v>
       </x:c>
       <x:c r="B15" s="4" t="str">
-        <x:v>Armor</x:v>
+        <x:v>Weapons</x:v>
       </x:c>
       <x:c r="C15" s="4" t="str">
-        <x:v>What the object is, independent of material, culture and use.</x:v>
+        <x:v>Broad existing inventory/design grouping. One per master item.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="45" customHeight="1">
@@ -26849,7 +27997,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B16" s="4" t="str">
-        <x:v>Carrier</x:v>
+        <x:v>Armor</x:v>
       </x:c>
       <x:c r="C16" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26860,7 +28008,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B17" s="4" t="str">
-        <x:v>Chemical material</x:v>
+        <x:v>Carrier</x:v>
       </x:c>
       <x:c r="C17" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26871,7 +28019,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B18" s="4" t="str">
-        <x:v>Container</x:v>
+        <x:v>Chemical material</x:v>
       </x:c>
       <x:c r="C18" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26882,7 +28030,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B19" s="4" t="str">
-        <x:v>Container part</x:v>
+        <x:v>Container</x:v>
       </x:c>
       <x:c r="C19" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26893,7 +28041,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B20" s="4" t="str">
-        <x:v>Crafting component</x:v>
+        <x:v>Container part</x:v>
       </x:c>
       <x:c r="C20" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26904,7 +28052,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B21" s="4" t="str">
-        <x:v>Cultural object</x:v>
+        <x:v>Crafting component</x:v>
       </x:c>
       <x:c r="C21" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26915,7 +28063,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B22" s="4" t="str">
-        <x:v>Currency</x:v>
+        <x:v>Cultural object</x:v>
       </x:c>
       <x:c r="C22" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26926,7 +28074,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B23" s="4" t="str">
-        <x:v>Document</x:v>
+        <x:v>Currency</x:v>
       </x:c>
       <x:c r="C23" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26937,7 +28085,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B24" s="4" t="str">
-        <x:v>Energy storage</x:v>
+        <x:v>Document</x:v>
       </x:c>
       <x:c r="C24" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26948,7 +28096,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B25" s="4" t="str">
-        <x:v>Food material</x:v>
+        <x:v>Drink consumable</x:v>
       </x:c>
       <x:c r="C25" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26959,7 +28107,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B26" s="4" t="str">
-        <x:v>Gem material</x:v>
+        <x:v>Energy storage</x:v>
       </x:c>
       <x:c r="C26" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26970,7 +28118,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B27" s="4" t="str">
-        <x:v>Household utensil</x:v>
+        <x:v>Food consumable</x:v>
       </x:c>
       <x:c r="C27" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26981,7 +28129,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B28" s="4" t="str">
-        <x:v>Machine</x:v>
+        <x:v>Food material</x:v>
       </x:c>
       <x:c r="C28" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -26992,7 +28140,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B29" s="4" t="str">
-        <x:v>Musical instrument</x:v>
+        <x:v>Gem material</x:v>
       </x:c>
       <x:c r="C29" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27003,7 +28151,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B30" s="4" t="str">
-        <x:v>Processed material</x:v>
+        <x:v>Household utensil</x:v>
       </x:c>
       <x:c r="C30" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27014,7 +28162,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B31" s="4" t="str">
-        <x:v>Raw material</x:v>
+        <x:v>Machine</x:v>
       </x:c>
       <x:c r="C31" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27025,7 +28173,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B32" s="4" t="str">
-        <x:v>Service kit</x:v>
+        <x:v>Musical instrument</x:v>
       </x:c>
       <x:c r="C32" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27036,7 +28184,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B33" s="4" t="str">
-        <x:v>Shelter kit</x:v>
+        <x:v>Processed material</x:v>
       </x:c>
       <x:c r="C33" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27047,7 +28195,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B34" s="4" t="str">
-        <x:v>Shield</x:v>
+        <x:v>Raw material</x:v>
       </x:c>
       <x:c r="C34" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27058,7 +28206,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B35" s="4" t="str">
-        <x:v>Tool</x:v>
+        <x:v>Service kit</x:v>
       </x:c>
       <x:c r="C35" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27069,7 +28217,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B36" s="4" t="str">
-        <x:v>Traversal device</x:v>
+        <x:v>Shelter kit</x:v>
       </x:c>
       <x:c r="C36" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27080,7 +28228,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B37" s="4" t="str">
-        <x:v>Trip hazard</x:v>
+        <x:v>Shield</x:v>
       </x:c>
       <x:c r="C37" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27091,7 +28239,7 @@
         <x:v>Item type</x:v>
       </x:c>
       <x:c r="B38" s="4" t="str">
-        <x:v>Wearable</x:v>
+        <x:v>Tool</x:v>
       </x:c>
       <x:c r="C38" s="4" t="str">
         <x:v>What the object is, independent of material, culture and use.</x:v>
@@ -27099,35 +28247,35 @@
     </x:row>
     <x:row r="39" ht="45" customHeight="1">
       <x:c r="A39" s="4" t="str">
-        <x:v>Processing stage</x:v>
+        <x:v>Item type</x:v>
       </x:c>
       <x:c r="B39" s="4" t="str">
-        <x:v>Ancient manufactured</x:v>
+        <x:v>Traversal device</x:v>
       </x:c>
       <x:c r="C39" s="4" t="str">
-        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
+        <x:v>What the object is, independent of material, culture and use.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="45" customHeight="1">
       <x:c r="A40" s="4" t="str">
-        <x:v>Processing stage</x:v>
+        <x:v>Item type</x:v>
       </x:c>
       <x:c r="B40" s="4" t="str">
-        <x:v>Extracted material</x:v>
+        <x:v>Trip hazard</x:v>
       </x:c>
       <x:c r="C40" s="4" t="str">
-        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
+        <x:v>What the object is, independent of material, culture and use.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="45" customHeight="1">
       <x:c r="A41" s="4" t="str">
-        <x:v>Processing stage</x:v>
+        <x:v>Item type</x:v>
       </x:c>
       <x:c r="B41" s="4" t="str">
-        <x:v>Finished item</x:v>
+        <x:v>Wearable</x:v>
       </x:c>
       <x:c r="C41" s="4" t="str">
-        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
+        <x:v>What the object is, independent of material, culture and use.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="45" customHeight="1">
@@ -27135,7 +28283,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B42" s="4" t="str">
-        <x:v>Processed intermediate</x:v>
+        <x:v>Ancient manufactured</x:v>
       </x:c>
       <x:c r="C42" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -27146,7 +28294,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B43" s="4" t="str">
-        <x:v>Raw</x:v>
+        <x:v>Extracted material</x:v>
       </x:c>
       <x:c r="C43" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -27157,7 +28305,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B44" s="4" t="str">
-        <x:v>Recovered part</x:v>
+        <x:v>Finished item</x:v>
       </x:c>
       <x:c r="C44" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -27168,7 +28316,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B45" s="4" t="str">
-        <x:v>Unfired intermediate</x:v>
+        <x:v>Processed intermediate</x:v>
       </x:c>
       <x:c r="C45" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -27179,7 +28327,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B46" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Raw</x:v>
       </x:c>
       <x:c r="C46" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -27190,7 +28338,7 @@
         <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B47" s="4" t="str">
-        <x:v>Unworked metal</x:v>
+        <x:v>Recovered part</x:v>
       </x:c>
       <x:c r="C47" s="4" t="str">
         <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
@@ -27198,35 +28346,35 @@
     </x:row>
     <x:row r="48" ht="45" customHeight="1">
       <x:c r="A48" s="4" t="str">
-        <x:v>Origin family</x:v>
+        <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B48" s="4" t="str">
-        <x:v>Ancient technology</x:v>
+        <x:v>Unfired intermediate</x:v>
       </x:c>
       <x:c r="C48" s="4" t="str">
-        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
+        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="45" customHeight="1">
       <x:c r="A49" s="4" t="str">
-        <x:v>Origin family</x:v>
+        <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B49" s="4" t="str">
-        <x:v>Atmospheric</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C49" s="4" t="str">
-        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
+        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="45" customHeight="1">
       <x:c r="A50" s="4" t="str">
-        <x:v>Origin family</x:v>
+        <x:v>Processing stage</x:v>
       </x:c>
       <x:c r="B50" s="4" t="str">
-        <x:v>Fauna</x:v>
+        <x:v>Unworked metal</x:v>
       </x:c>
       <x:c r="C50" s="4" t="str">
-        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
+        <x:v>State of the listed item, not its next recipe. Stage unresolved means raw-versus-processed is undecided.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="45" customHeight="1">
@@ -27234,7 +28382,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B51" s="4" t="str">
-        <x:v>Geological</x:v>
+        <x:v>Ancient technology</x:v>
       </x:c>
       <x:c r="C51" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -27245,7 +28393,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B52" s="4" t="str">
-        <x:v>Living culture</x:v>
+        <x:v>Atmospheric</x:v>
       </x:c>
       <x:c r="C52" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -27256,7 +28404,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B53" s="4" t="str">
-        <x:v>Manufactured / unresolved</x:v>
+        <x:v>Biological mixture</x:v>
       </x:c>
       <x:c r="C53" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -27267,7 +28415,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B54" s="4" t="str">
-        <x:v>Recovered machinery</x:v>
+        <x:v>Fauna</x:v>
       </x:c>
       <x:c r="C54" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -27278,7 +28426,7 @@
         <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B55" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Geological</x:v>
       </x:c>
       <x:c r="C55" s="4" t="str">
         <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
@@ -27286,46 +28434,46 @@
     </x:row>
     <x:row r="56" ht="45" customHeight="1">
       <x:c r="A56" s="4" t="str">
-        <x:v>Primary use</x:v>
+        <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B56" s="4" t="str">
-        <x:v>Area denial</x:v>
+        <x:v>Living culture</x:v>
       </x:c>
       <x:c r="C56" s="4" t="str">
-        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
+        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="45" customHeight="1">
       <x:c r="A57" s="4" t="str">
-        <x:v>Primary use</x:v>
+        <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B57" s="4" t="str">
-        <x:v>Atmospheric support</x:v>
+        <x:v>Manufactured / unresolved</x:v>
       </x:c>
       <x:c r="C57" s="4" t="str">
-        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
+        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="45" customHeight="1">
       <x:c r="A58" s="4" t="str">
-        <x:v>Primary use</x:v>
+        <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B58" s="4" t="str">
-        <x:v>Binding and construction</x:v>
+        <x:v>Recovered machinery</x:v>
       </x:c>
       <x:c r="C58" s="4" t="str">
-        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
+        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="45" customHeight="1">
       <x:c r="A59" s="4" t="str">
-        <x:v>Primary use</x:v>
+        <x:v>Origin family</x:v>
       </x:c>
       <x:c r="B59" s="4" t="str">
-        <x:v>Camp rest</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C59" s="4" t="str">
-        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
+        <x:v>Broad provenance. Manufactured / unresolved does not identify raw ingredients.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="45" customHeight="1">
@@ -27333,7 +28481,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B60" s="4" t="str">
-        <x:v>Cargo organization</x:v>
+        <x:v>Area denial</x:v>
       </x:c>
       <x:c r="C60" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27344,7 +28492,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B61" s="4" t="str">
-        <x:v>Ceremony</x:v>
+        <x:v>Atmospheric support</x:v>
       </x:c>
       <x:c r="C61" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27355,7 +28503,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B62" s="4" t="str">
-        <x:v>Chemical processing</x:v>
+        <x:v>Binding and construction</x:v>
       </x:c>
       <x:c r="C62" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27366,7 +28514,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B63" s="4" t="str">
-        <x:v>Civic identification</x:v>
+        <x:v>Camp rest</x:v>
       </x:c>
       <x:c r="C63" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27377,7 +28525,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B64" s="4" t="str">
-        <x:v>Civic recognition</x:v>
+        <x:v>Cargo organization</x:v>
       </x:c>
       <x:c r="C64" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27388,7 +28536,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B65" s="4" t="str">
-        <x:v>Cleaning</x:v>
+        <x:v>Ceremony</x:v>
       </x:c>
       <x:c r="C65" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27399,7 +28547,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B66" s="4" t="str">
-        <x:v>Clothing</x:v>
+        <x:v>Chemical processing</x:v>
       </x:c>
       <x:c r="C66" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27410,7 +28558,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B67" s="4" t="str">
-        <x:v>Clothing fabrication</x:v>
+        <x:v>Civic identification</x:v>
       </x:c>
       <x:c r="C67" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27421,7 +28569,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B68" s="4" t="str">
-        <x:v>Cooking</x:v>
+        <x:v>Civic recognition</x:v>
       </x:c>
       <x:c r="C68" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27432,7 +28580,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B69" s="4" t="str">
-        <x:v>Culture support</x:v>
+        <x:v>Cleaning</x:v>
       </x:c>
       <x:c r="C69" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27443,7 +28591,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B70" s="4" t="str">
-        <x:v>Decoration</x:v>
+        <x:v>Clothing</x:v>
       </x:c>
       <x:c r="C70" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27454,7 +28602,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B71" s="4" t="str">
-        <x:v>Devotion</x:v>
+        <x:v>Clothing fabrication</x:v>
       </x:c>
       <x:c r="C71" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27465,7 +28613,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B72" s="4" t="str">
-        <x:v>Dust exclusion</x:v>
+        <x:v>Cooking</x:v>
       </x:c>
       <x:c r="C72" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27476,7 +28624,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B73" s="4" t="str">
-        <x:v>Electrical conduction</x:v>
+        <x:v>Culture support</x:v>
       </x:c>
       <x:c r="C73" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27487,7 +28635,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B74" s="4" t="str">
-        <x:v>Electrical insulation</x:v>
+        <x:v>Decoration</x:v>
       </x:c>
       <x:c r="C74" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27498,7 +28646,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B75" s="4" t="str">
-        <x:v>Electrical work</x:v>
+        <x:v>Devotion</x:v>
       </x:c>
       <x:c r="C75" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27509,7 +28657,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B76" s="4" t="str">
-        <x:v>Energy processing</x:v>
+        <x:v>Dust exclusion</x:v>
       </x:c>
       <x:c r="C76" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27520,7 +28668,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B77" s="4" t="str">
-        <x:v>Energy storage</x:v>
+        <x:v>Electrical conduction</x:v>
       </x:c>
       <x:c r="C77" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27531,7 +28679,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B78" s="4" t="str">
-        <x:v>Equipment fabrication</x:v>
+        <x:v>Electrical insulation</x:v>
       </x:c>
       <x:c r="C78" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27542,7 +28690,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B79" s="4" t="str">
-        <x:v>Equipment mounting</x:v>
+        <x:v>Electrical work</x:v>
       </x:c>
       <x:c r="C79" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27553,7 +28701,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B80" s="4" t="str">
-        <x:v>Equipment repair</x:v>
+        <x:v>Energy processing</x:v>
       </x:c>
       <x:c r="C80" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27564,7 +28712,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B81" s="4" t="str">
-        <x:v>Excavation</x:v>
+        <x:v>Energy storage</x:v>
       </x:c>
       <x:c r="C81" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27575,7 +28723,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B82" s="4" t="str">
-        <x:v>Fabrication</x:v>
+        <x:v>Equipment fabrication</x:v>
       </x:c>
       <x:c r="C82" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27586,7 +28734,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B83" s="4" t="str">
-        <x:v>Fashion</x:v>
+        <x:v>Equipment mounting</x:v>
       </x:c>
       <x:c r="C83" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27597,7 +28745,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B84" s="4" t="str">
-        <x:v>Fauna interaction</x:v>
+        <x:v>Equipment repair</x:v>
       </x:c>
       <x:c r="C84" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27608,7 +28756,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B85" s="4" t="str">
-        <x:v>Fiber processing</x:v>
+        <x:v>Excavation</x:v>
       </x:c>
       <x:c r="C85" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27619,7 +28767,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B86" s="4" t="str">
-        <x:v>Fire management</x:v>
+        <x:v>Fabrication</x:v>
       </x:c>
       <x:c r="C86" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27630,7 +28778,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B87" s="4" t="str">
-        <x:v>Food service</x:v>
+        <x:v>Fashion</x:v>
       </x:c>
       <x:c r="C87" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27641,7 +28789,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B88" s="4" t="str">
-        <x:v>Fuel</x:v>
+        <x:v>Fauna interaction</x:v>
       </x:c>
       <x:c r="C88" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27652,7 +28800,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B89" s="4" t="str">
-        <x:v>Glass and ceramics</x:v>
+        <x:v>Fiber processing</x:v>
       </x:c>
       <x:c r="C89" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27663,7 +28811,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B90" s="4" t="str">
-        <x:v>Grooming</x:v>
+        <x:v>Fire management</x:v>
       </x:c>
       <x:c r="C90" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27674,7 +28822,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B91" s="4" t="str">
-        <x:v>Ignition</x:v>
+        <x:v>Food preparation</x:v>
       </x:c>
       <x:c r="C91" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27685,7 +28833,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B92" s="4" t="str">
-        <x:v>Illumination</x:v>
+        <x:v>Food service</x:v>
       </x:c>
       <x:c r="C92" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27696,7 +28844,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B93" s="4" t="str">
-        <x:v>Injury treatment</x:v>
+        <x:v>Fuel</x:v>
       </x:c>
       <x:c r="C93" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27707,7 +28855,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B94" s="4" t="str">
-        <x:v>Inspection</x:v>
+        <x:v>Glass and ceramics</x:v>
       </x:c>
       <x:c r="C94" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27718,7 +28866,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B95" s="4" t="str">
-        <x:v>Keepsake storage</x:v>
+        <x:v>Grooming</x:v>
       </x:c>
       <x:c r="C95" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27729,7 +28877,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B96" s="4" t="str">
-        <x:v>Liquid and bulk containment</x:v>
+        <x:v>Hydration</x:v>
       </x:c>
       <x:c r="C96" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27740,7 +28888,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>Lubrication</x:v>
+        <x:v>Ignition</x:v>
       </x:c>
       <x:c r="C97" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27751,7 +28899,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B98" s="4" t="str">
-        <x:v>Machinery drive</x:v>
+        <x:v>Illumination</x:v>
       </x:c>
       <x:c r="C98" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27762,7 +28910,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B99" s="4" t="str">
-        <x:v>Machinery repair</x:v>
+        <x:v>Injury treatment</x:v>
       </x:c>
       <x:c r="C99" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27773,7 +28921,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B100" s="4" t="str">
-        <x:v>Magnetic tools</x:v>
+        <x:v>Inspection</x:v>
       </x:c>
       <x:c r="C100" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27784,7 +28932,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B101" s="4" t="str">
-        <x:v>Material exclusion</x:v>
+        <x:v>Keepsake storage</x:v>
       </x:c>
       <x:c r="C101" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27795,7 +28943,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B102" s="4" t="str">
-        <x:v>Material transfer</x:v>
+        <x:v>Liquid and bulk containment</x:v>
       </x:c>
       <x:c r="C102" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27806,7 +28954,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B103" s="4" t="str">
-        <x:v>Metal refining</x:v>
+        <x:v>Lubrication</x:v>
       </x:c>
       <x:c r="C103" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27817,7 +28965,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B104" s="4" t="str">
-        <x:v>Music</x:v>
+        <x:v>Machinery drive</x:v>
       </x:c>
       <x:c r="C104" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27828,7 +28976,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B105" s="4" t="str">
-        <x:v>Nutrition</x:v>
+        <x:v>Machinery repair</x:v>
       </x:c>
       <x:c r="C105" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27839,7 +28987,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B106" s="4" t="str">
-        <x:v>Paper making</x:v>
+        <x:v>Magnetic tools</x:v>
       </x:c>
       <x:c r="C106" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27850,7 +28998,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B107" s="4" t="str">
-        <x:v>Protection</x:v>
+        <x:v>Material exclusion</x:v>
       </x:c>
       <x:c r="C107" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27861,7 +29009,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B108" s="4" t="str">
-        <x:v>Protective fabrication</x:v>
+        <x:v>Material transfer</x:v>
       </x:c>
       <x:c r="C108" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27872,7 +29020,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B109" s="4" t="str">
-        <x:v>Provenance</x:v>
+        <x:v>Metal refining</x:v>
       </x:c>
       <x:c r="C109" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27883,7 +29031,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B110" s="4" t="str">
-        <x:v>Public communication</x:v>
+        <x:v>Music</x:v>
       </x:c>
       <x:c r="C110" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27894,7 +29042,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B111" s="4" t="str">
-        <x:v>Remembrance</x:v>
+        <x:v>Nutrition</x:v>
       </x:c>
       <x:c r="C111" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27905,7 +29053,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B112" s="4" t="str">
-        <x:v>Resource collection</x:v>
+        <x:v>Paper making</x:v>
       </x:c>
       <x:c r="C112" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27916,7 +29064,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B113" s="4" t="str">
-        <x:v>Sealing</x:v>
+        <x:v>Protection</x:v>
       </x:c>
       <x:c r="C113" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27927,7 +29075,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B114" s="4" t="str">
-        <x:v>Specialist samples</x:v>
+        <x:v>Protective fabrication</x:v>
       </x:c>
       <x:c r="C114" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27938,7 +29086,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B115" s="4" t="str">
-        <x:v>Static management</x:v>
+        <x:v>Provenance</x:v>
       </x:c>
       <x:c r="C115" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27949,7 +29097,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B116" s="4" t="str">
-        <x:v>Sun shading</x:v>
+        <x:v>Public communication</x:v>
       </x:c>
       <x:c r="C116" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27960,7 +29108,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B117" s="4" t="str">
-        <x:v>Surface finishing</x:v>
+        <x:v>Remembrance</x:v>
       </x:c>
       <x:c r="C117" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27971,7 +29119,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B118" s="4" t="str">
-        <x:v>Survival provision</x:v>
+        <x:v>Resource collection</x:v>
       </x:c>
       <x:c r="C118" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27982,7 +29130,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B119" s="4" t="str">
-        <x:v>Textile processing</x:v>
+        <x:v>Sealing</x:v>
       </x:c>
       <x:c r="C119" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -27993,7 +29141,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B120" s="4" t="str">
-        <x:v>Tool fabrication</x:v>
+        <x:v>Specialist samples</x:v>
       </x:c>
       <x:c r="C120" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -28004,7 +29152,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B121" s="4" t="str">
-        <x:v>Trade</x:v>
+        <x:v>Static management</x:v>
       </x:c>
       <x:c r="C121" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -28015,7 +29163,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B122" s="4" t="str">
-        <x:v>Traversal</x:v>
+        <x:v>Sun shading</x:v>
       </x:c>
       <x:c r="C122" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -28026,7 +29174,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B123" s="4" t="str">
-        <x:v>Use unresolved</x:v>
+        <x:v>Surface finishing</x:v>
       </x:c>
       <x:c r="C123" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -28037,7 +29185,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B124" s="4" t="str">
-        <x:v>Vision</x:v>
+        <x:v>Survival provision</x:v>
       </x:c>
       <x:c r="C124" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -28048,7 +29196,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B125" s="4" t="str">
-        <x:v>Wind power</x:v>
+        <x:v>Textile processing</x:v>
       </x:c>
       <x:c r="C125" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -28059,7 +29207,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B126" s="4" t="str">
-        <x:v>Wind propulsion</x:v>
+        <x:v>Tool fabrication</x:v>
       </x:c>
       <x:c r="C126" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -28070,7 +29218,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B127" s="4" t="str">
-        <x:v>Work holding</x:v>
+        <x:v>Trade</x:v>
       </x:c>
       <x:c r="C127" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -28081,7 +29229,7 @@
         <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B128" s="4" t="str">
-        <x:v>Writing and records</x:v>
+        <x:v>Traversal</x:v>
       </x:c>
       <x:c r="C128" s="4" t="str">
         <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
@@ -28089,68 +29237,68 @@
     </x:row>
     <x:row r="129" ht="45" customHeight="1">
       <x:c r="A129" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B129" s="4" t="str">
-        <x:v>Ancient composite</x:v>
+        <x:v>Use unresolved</x:v>
       </x:c>
       <x:c r="C129" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="45" customHeight="1">
       <x:c r="A130" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B130" s="4" t="str">
-        <x:v>Biological and mineral mixture</x:v>
+        <x:v>Vision</x:v>
       </x:c>
       <x:c r="C130" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="45" customHeight="1">
       <x:c r="A131" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B131" s="4" t="str">
-        <x:v>Biological chemical</x:v>
+        <x:v>Wind power</x:v>
       </x:c>
       <x:c r="C131" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="45" customHeight="1">
       <x:c r="A132" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B132" s="4" t="str">
-        <x:v>Carbonaceous material</x:v>
+        <x:v>Wind propulsion</x:v>
       </x:c>
       <x:c r="C132" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="45" customHeight="1">
       <x:c r="A133" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B133" s="4" t="str">
-        <x:v>Ceramic</x:v>
+        <x:v>Work holding</x:v>
       </x:c>
       <x:c r="C133" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="45" customHeight="1">
       <x:c r="A134" s="4" t="str">
-        <x:v>Material family</x:v>
+        <x:v>Primary use</x:v>
       </x:c>
       <x:c r="B134" s="4" t="str">
-        <x:v>Ceramic and metal</x:v>
+        <x:v>Writing and records</x:v>
       </x:c>
       <x:c r="C134" s="4" t="str">
-        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
+        <x:v>Main catalog purpose. Item uses lists additional purposes as separate filterable rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="45" customHeight="1">
@@ -28158,7 +29306,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B135" s="4" t="str">
-        <x:v>Ceramic feed mixture</x:v>
+        <x:v>Ancient composite</x:v>
       </x:c>
       <x:c r="C135" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28169,7 +29317,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B136" s="4" t="str">
-        <x:v>Faunal fiber</x:v>
+        <x:v>Biological and mineral mixture</x:v>
       </x:c>
       <x:c r="C136" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28180,7 +29328,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B137" s="4" t="str">
-        <x:v>Faunal fiber and shell</x:v>
+        <x:v>Biological chemical</x:v>
       </x:c>
       <x:c r="C137" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28191,7 +29339,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B138" s="4" t="str">
-        <x:v>Faunal membrane</x:v>
+        <x:v>Carbonaceous material</x:v>
       </x:c>
       <x:c r="C138" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28202,7 +29350,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B139" s="4" t="str">
-        <x:v>Faunal tissue</x:v>
+        <x:v>Ceramic</x:v>
       </x:c>
       <x:c r="C139" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28213,7 +29361,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B140" s="4" t="str">
-        <x:v>Fur</x:v>
+        <x:v>Ceramic and metal</x:v>
       </x:c>
       <x:c r="C140" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28224,7 +29372,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B141" s="4" t="str">
-        <x:v>Gemstone</x:v>
+        <x:v>Ceramic feed mixture</x:v>
       </x:c>
       <x:c r="C141" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28235,7 +29383,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B142" s="4" t="str">
-        <x:v>Glass</x:v>
+        <x:v>Faunal fiber</x:v>
       </x:c>
       <x:c r="C142" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28246,7 +29394,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B143" s="4" t="str">
-        <x:v>Glass and metal</x:v>
+        <x:v>Faunal fiber and shell</x:v>
       </x:c>
       <x:c r="C143" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28257,7 +29405,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B144" s="4" t="str">
-        <x:v>Glass and shell</x:v>
+        <x:v>Faunal membrane</x:v>
       </x:c>
       <x:c r="C144" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28268,7 +29416,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B145" s="4" t="str">
-        <x:v>Glass with unresolved casing</x:v>
+        <x:v>Faunal tissue</x:v>
       </x:c>
       <x:c r="C145" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28279,7 +29427,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B146" s="4" t="str">
-        <x:v>Hide</x:v>
+        <x:v>Fur</x:v>
       </x:c>
       <x:c r="C146" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28290,7 +29438,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B147" s="4" t="str">
-        <x:v>Husk fiber</x:v>
+        <x:v>Gemstone</x:v>
       </x:c>
       <x:c r="C147" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28301,7 +29449,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B148" s="4" t="str">
-        <x:v>Husk fiber and shell</x:v>
+        <x:v>Glass</x:v>
       </x:c>
       <x:c r="C148" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28312,7 +29460,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B149" s="4" t="str">
-        <x:v>Metal</x:v>
+        <x:v>Glass and metal</x:v>
       </x:c>
       <x:c r="C149" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28323,7 +29471,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B150" s="4" t="str">
-        <x:v>Metal and shell</x:v>
+        <x:v>Glass and shell</x:v>
       </x:c>
       <x:c r="C150" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28334,7 +29482,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B151" s="4" t="str">
-        <x:v>Metal or shell</x:v>
+        <x:v>Glass or ceramic</x:v>
       </x:c>
       <x:c r="C151" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28345,7 +29493,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B152" s="4" t="str">
-        <x:v>Mineral</x:v>
+        <x:v>Glass with unresolved casing</x:v>
       </x:c>
       <x:c r="C152" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28356,7 +29504,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B153" s="4" t="str">
-        <x:v>Mineral or shell</x:v>
+        <x:v>Hide</x:v>
       </x:c>
       <x:c r="C153" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28367,7 +29515,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B154" s="4" t="str">
-        <x:v>Mixed / unresolved</x:v>
+        <x:v>Husk fiber</x:v>
       </x:c>
       <x:c r="C154" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28378,7 +29526,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B155" s="4" t="str">
-        <x:v>Shell / chitin</x:v>
+        <x:v>Husk fiber and shell</x:v>
       </x:c>
       <x:c r="C155" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28389,7 +29537,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B156" s="4" t="str">
-        <x:v>Shell and mineral</x:v>
+        <x:v>Metal</x:v>
       </x:c>
       <x:c r="C156" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28400,7 +29548,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B157" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Metal and shell</x:v>
       </x:c>
       <x:c r="C157" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28411,7 +29559,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B158" s="4" t="str">
-        <x:v>Wing membrane</x:v>
+        <x:v>Metal or shell</x:v>
       </x:c>
       <x:c r="C158" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28422,7 +29570,7 @@
         <x:v>Material family</x:v>
       </x:c>
       <x:c r="B159" s="4" t="str">
-        <x:v>Wing membrane and frame</x:v>
+        <x:v>Mineral</x:v>
       </x:c>
       <x:c r="C159" s="4" t="str">
         <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
@@ -28430,101 +29578,101 @@
     </x:row>
     <x:row r="160" ht="45" customHeight="1">
       <x:c r="A160" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B160" s="4" t="str">
-        <x:v>Assembly</x:v>
+        <x:v>Mineral or shell</x:v>
       </x:c>
       <x:c r="C160" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="45" customHeight="1">
       <x:c r="A161" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B161" s="4" t="str">
-        <x:v>Bundle</x:v>
+        <x:v>Mixed / unresolved</x:v>
       </x:c>
       <x:c r="C161" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="45" customHeight="1">
       <x:c r="A162" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B162" s="4" t="str">
-        <x:v>Cord</x:v>
+        <x:v>Phagia and edible fauna</x:v>
       </x:c>
       <x:c r="C162" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="163" ht="45" customHeight="1">
       <x:c r="A163" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B163" s="4" t="str">
-        <x:v>Fiber</x:v>
+        <x:v>Phagia preparation</x:v>
       </x:c>
       <x:c r="C163" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="45" customHeight="1">
       <x:c r="A164" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B164" s="4" t="str">
-        <x:v>Folio</x:v>
+        <x:v>Shell / chitin</x:v>
       </x:c>
       <x:c r="C164" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="165" ht="45" customHeight="1">
       <x:c r="A165" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B165" s="4" t="str">
-        <x:v>Garment</x:v>
+        <x:v>Shell and mineral</x:v>
       </x:c>
       <x:c r="C165" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="166" ht="45" customHeight="1">
       <x:c r="A166" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B166" s="4" t="str">
-        <x:v>Gel</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="C166" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="167" ht="45" customHeight="1">
       <x:c r="A167" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B167" s="4" t="str">
-        <x:v>Liquid</x:v>
+        <x:v>Wing membrane</x:v>
       </x:c>
       <x:c r="C167" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="168" ht="45" customHeight="1">
       <x:c r="A168" s="4" t="str">
-        <x:v>Physical form</x:v>
+        <x:v>Material family</x:v>
       </x:c>
       <x:c r="B168" s="4" t="str">
-        <x:v>Membrane</x:v>
+        <x:v>Wing membrane and frame</x:v>
       </x:c>
       <x:c r="C168" s="4" t="str">
-        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+        <x:v>Broad descriptive candidate. Mixed, alternative and unresolved values preserve uncertainty.</x:v>
       </x:c>
     </x:row>
     <x:row r="169" ht="45" customHeight="1">
@@ -28532,7 +29680,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B169" s="4" t="str">
-        <x:v>Panel</x:v>
+        <x:v>Assembly</x:v>
       </x:c>
       <x:c r="C169" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28543,7 +29691,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B170" s="4" t="str">
-        <x:v>Particles</x:v>
+        <x:v>Bundle</x:v>
       </x:c>
       <x:c r="C170" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28554,7 +29702,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B171" s="4" t="str">
-        <x:v>Paste</x:v>
+        <x:v>Cord</x:v>
       </x:c>
       <x:c r="C171" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28565,7 +29713,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B172" s="4" t="str">
-        <x:v>Patch</x:v>
+        <x:v>Fiber</x:v>
       </x:c>
       <x:c r="C172" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28576,7 +29724,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B173" s="4" t="str">
-        <x:v>Rock</x:v>
+        <x:v>Folio</x:v>
       </x:c>
       <x:c r="C173" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28587,7 +29735,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B174" s="4" t="str">
-        <x:v>Sheet</x:v>
+        <x:v>Garment</x:v>
       </x:c>
       <x:c r="C174" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28598,7 +29746,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B175" s="4" t="str">
-        <x:v>Shell plate</x:v>
+        <x:v>Gel</x:v>
       </x:c>
       <x:c r="C175" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28609,7 +29757,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B176" s="4" t="str">
-        <x:v>Solid part</x:v>
+        <x:v>Liquid</x:v>
       </x:c>
       <x:c r="C176" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28620,7 +29768,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B177" s="4" t="str">
-        <x:v>Solid piece</x:v>
+        <x:v>Membrane</x:v>
       </x:c>
       <x:c r="C177" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28631,7 +29779,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B178" s="4" t="str">
-        <x:v>Strip</x:v>
+        <x:v>Panel</x:v>
       </x:c>
       <x:c r="C178" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28642,7 +29790,7 @@
         <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B179" s="4" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Particles</x:v>
       </x:c>
       <x:c r="C179" s="4" t="str">
         <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
@@ -28650,63 +29798,162 @@
     </x:row>
     <x:row r="180" ht="45" customHeight="1">
       <x:c r="A180" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B180" s="4" t="str">
-        <x:v>Author direction</x:v>
+        <x:v>Paste</x:v>
       </x:c>
       <x:c r="C180" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="181" ht="45" customHeight="1">
       <x:c r="A181" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B181" s="4" t="str">
-        <x:v>Existing definition</x:v>
+        <x:v>Patch</x:v>
       </x:c>
       <x:c r="C181" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="182" ht="45" customHeight="1">
       <x:c r="A182" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B182" s="4" t="str">
-        <x:v>Proposal</x:v>
+        <x:v>Rock</x:v>
       </x:c>
       <x:c r="C182" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="183" ht="45" customHeight="1">
       <x:c r="A183" s="4" t="str">
-        <x:v>Design status</x:v>
+        <x:v>Physical form</x:v>
       </x:c>
       <x:c r="B183" s="4" t="str">
-        <x:v>Source proposal</x:v>
+        <x:v>Sheet</x:v>
       </x:c>
       <x:c r="C183" s="4" t="str">
-        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="45" customHeight="1">
       <x:c r="A184" s="4" t="str">
+        <x:v>Physical form</x:v>
+      </x:c>
+      <x:c r="B184" s="4" t="str">
+        <x:v>Shell plate</x:v>
+      </x:c>
+      <x:c r="C184" s="4" t="str">
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="45" customHeight="1">
+      <x:c r="A185" s="4" t="str">
+        <x:v>Physical form</x:v>
+      </x:c>
+      <x:c r="B185" s="4" t="str">
+        <x:v>Solid part</x:v>
+      </x:c>
+      <x:c r="C185" s="4" t="str">
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="45" customHeight="1">
+      <x:c r="A186" s="4" t="str">
+        <x:v>Physical form</x:v>
+      </x:c>
+      <x:c r="B186" s="4" t="str">
+        <x:v>Solid piece</x:v>
+      </x:c>
+      <x:c r="C186" s="4" t="str">
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="45" customHeight="1">
+      <x:c r="A187" s="4" t="str">
+        <x:v>Physical form</x:v>
+      </x:c>
+      <x:c r="B187" s="4" t="str">
+        <x:v>Strip</x:v>
+      </x:c>
+      <x:c r="C187" s="4" t="str">
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="45" customHeight="1">
+      <x:c r="A188" s="4" t="str">
+        <x:v>Physical form</x:v>
+      </x:c>
+      <x:c r="B188" s="4" t="str">
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="C188" s="4" t="str">
+        <x:v>Catalog shape/state only; Unresolved avoids inventing a physical or chemical property.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="45" customHeight="1">
+      <x:c r="A189" s="4" t="str">
         <x:v>Design status</x:v>
       </x:c>
-      <x:c r="B184" s="4" t="str">
+      <x:c r="B189" s="4" t="str">
+        <x:v>Author direction</x:v>
+      </x:c>
+      <x:c r="C189" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="45" customHeight="1">
+      <x:c r="A190" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B190" s="4" t="str">
+        <x:v>Existing definition</x:v>
+      </x:c>
+      <x:c r="C190" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="45" customHeight="1">
+      <x:c r="A191" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B191" s="4" t="str">
+        <x:v>Proposal</x:v>
+      </x:c>
+      <x:c r="C191" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="45" customHeight="1">
+      <x:c r="A192" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B192" s="4" t="str">
+        <x:v>Source proposal</x:v>
+      </x:c>
+      <x:c r="C192" s="4" t="str">
+        <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="45" customHeight="1">
+      <x:c r="A193" s="4" t="str">
+        <x:v>Design status</x:v>
+      </x:c>
+      <x:c r="B193" s="4" t="str">
         <x:v>Withheld assumption</x:v>
       </x:c>
-      <x:c r="C184" s="4" t="str">
+      <x:c r="C193" s="4" t="str">
         <x:v>Existing definition means serialized data, not proof all intended uses work. Author direction, Proposal and Withheld assumption remain distinct.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c83a9a2e5ac4c69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76f4ec2d1fd54ea9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38226,21 +39473,453 @@
         <x:v>Legger-specific proposal; intended use is not an implemented companion ability.</x:v>
       </x:c>
     </x:row>
+    <x:row r="423" ht="65" customHeight="1">
+      <x:c r="A423" s="3" t="str">
+        <x:v>proposal.food.drink_portion</x:v>
+      </x:c>
+      <x:c r="B423" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A423,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared Phagia drink portion</x:v>
+      </x:c>
+      <x:c r="C423" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A423,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D423" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E423" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A423,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Hydration</x:v>
+      </x:c>
+      <x:c r="F423" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="424" ht="65" customHeight="1">
+      <x:c r="A424" s="3" t="str">
+        <x:v>proposal.food.drink_portion</x:v>
+      </x:c>
+      <x:c r="B424" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A424,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared Phagia drink portion</x:v>
+      </x:c>
+      <x:c r="C424" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A424,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D424" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E424" s="3" t="str">
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="F424" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="425" ht="65" customHeight="1">
+      <x:c r="A425" s="3" t="str">
+        <x:v>proposal.food.dense_drink</x:v>
+      </x:c>
+      <x:c r="B425" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A425,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dense Phagia nutrient drink</x:v>
+      </x:c>
+      <x:c r="C425" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A425,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D425" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E425" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A425,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="F425" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="426" ht="65" customHeight="1">
+      <x:c r="A426" s="3" t="str">
+        <x:v>proposal.food.dense_drink</x:v>
+      </x:c>
+      <x:c r="B426" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A426,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dense Phagia nutrient drink</x:v>
+      </x:c>
+      <x:c r="C426" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A426,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D426" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E426" s="3" t="str">
+        <x:v>Hydration</x:v>
+      </x:c>
+      <x:c r="F426" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="427" ht="65" customHeight="1">
+      <x:c r="A427" s="3" t="str">
+        <x:v>proposal.food.ration_bar</x:v>
+      </x:c>
+      <x:c r="B427" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A427,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Phagia ration bar</x:v>
+      </x:c>
+      <x:c r="C427" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A427,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D427" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E427" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A427,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="F427" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="428" ht="65" customHeight="1">
+      <x:c r="A428" s="3" t="str">
+        <x:v>proposal.food.dried_bar</x:v>
+      </x:c>
+      <x:c r="B428" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A428,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Dried Phagia travel bar</x:v>
+      </x:c>
+      <x:c r="C428" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A428,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D428" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E428" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A428,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="F428" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="429" ht="65" customHeight="1">
+      <x:c r="A429" s="3" t="str">
+        <x:v>proposal.food.meal_paste</x:v>
+      </x:c>
+      <x:c r="B429" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A429,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared Phagia meal paste</x:v>
+      </x:c>
+      <x:c r="C429" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A429,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D429" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E429" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A429,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="F429" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="430" ht="65" customHeight="1">
+      <x:c r="A430" s="3" t="str">
+        <x:v>proposal.food.meal_portion</x:v>
+      </x:c>
+      <x:c r="B430" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A430,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared Phagia meal portion</x:v>
+      </x:c>
+      <x:c r="C430" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A430,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D430" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E430" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A430,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="F430" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="431" ht="65" customHeight="1">
+      <x:c r="A431" s="3" t="str">
+        <x:v>proposal.food.fauna_flake_dish</x:v>
+      </x:c>
+      <x:c r="B431" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A431,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Phagia and edible-fauna flake delicacy</x:v>
+      </x:c>
+      <x:c r="C431" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A431,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D431" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E431" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A431,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="F431" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="432" ht="65" customHeight="1">
+      <x:c r="A432" s="3" t="str">
+        <x:v>proposal.food.layered_delicacy</x:v>
+      </x:c>
+      <x:c r="B432" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A432,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Layered Phagia-fauna delicacy</x:v>
+      </x:c>
+      <x:c r="C432" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A432,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D432" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E432" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A432,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="F432" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="433" ht="65" customHeight="1">
+      <x:c r="A433" s="3" t="str">
+        <x:v>proposal.food.crisp_delicacy</x:v>
+      </x:c>
+      <x:c r="B433" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A433,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Crisp Phagia-fauna wafer</x:v>
+      </x:c>
+      <x:c r="C433" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A433,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="D433" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E433" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A433,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Nutrition</x:v>
+      </x:c>
+      <x:c r="F433" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="434" ht="65" customHeight="1">
+      <x:c r="A434" s="3" t="str">
+        <x:v>proposal.food.edible_flakes</x:v>
+      </x:c>
+      <x:c r="B434" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A434,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared edible-fauna flakes</x:v>
+      </x:c>
+      <x:c r="C434" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A434,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D434" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E434" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A434,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Food preparation</x:v>
+      </x:c>
+      <x:c r="F434" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="435" ht="65" customHeight="1">
+      <x:c r="A435" s="3" t="str">
+        <x:v>proposal.food.edible_paste</x:v>
+      </x:c>
+      <x:c r="B435" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A435,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared edible-fauna paste</x:v>
+      </x:c>
+      <x:c r="C435" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A435,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Resources</x:v>
+      </x:c>
+      <x:c r="D435" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E435" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A435,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Food preparation</x:v>
+      </x:c>
+      <x:c r="F435" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="436" ht="65" customHeight="1">
+      <x:c r="A436" s="3" t="str">
+        <x:v>proposal.food.drink_flask</x:v>
+      </x:c>
+      <x:c r="B436" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A436,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Reusable Phagia drinking flask</x:v>
+      </x:c>
+      <x:c r="C436" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A436,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D436" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E436" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A436,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="F436" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="437" ht="65" customHeight="1">
+      <x:c r="A437" s="3" t="str">
+        <x:v>proposal.food.drink_flask</x:v>
+      </x:c>
+      <x:c r="B437" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A437,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Reusable Phagia drinking flask</x:v>
+      </x:c>
+      <x:c r="C437" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A437,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D437" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E437" s="3" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F437" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="438" ht="65" customHeight="1">
+      <x:c r="A438" s="3" t="str">
+        <x:v>proposal.food.bar_case</x:v>
+      </x:c>
+      <x:c r="B438" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A438,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Phagia ration-bar case</x:v>
+      </x:c>
+      <x:c r="C438" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A438,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D438" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E438" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A438,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="F438" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="439" ht="65" customHeight="1">
+      <x:c r="A439" s="3" t="str">
+        <x:v>proposal.food.bar_case</x:v>
+      </x:c>
+      <x:c r="B439" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A439,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Phagia ration-bar case</x:v>
+      </x:c>
+      <x:c r="C439" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A439,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D439" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E439" s="3" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F439" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="440" ht="65" customHeight="1">
+      <x:c r="A440" s="3" t="str">
+        <x:v>proposal.food.meal_carrier</x:v>
+      </x:c>
+      <x:c r="B440" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A440,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared-meal carrier</x:v>
+      </x:c>
+      <x:c r="C440" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A440,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D440" s="3" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="E440" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$Z$6:$Z$1005,MATCH(A440,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Food service</x:v>
+      </x:c>
+      <x:c r="F440" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="441" ht="65" customHeight="1">
+      <x:c r="A441" s="3" t="str">
+        <x:v>proposal.food.meal_carrier</x:v>
+      </x:c>
+      <x:c r="B441" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$B$6:$B$1005,MATCH(A441,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Prepared-meal carrier</x:v>
+      </x:c>
+      <x:c r="C441" s="3" t="str">
+        <x:f>IFERROR(INDEX(Items!$C$6:$C$1005,MATCH(A441,Items!$A$6:$A$1005,0)),"MISSING ITEM ID")</x:f>
+        <x:v>Containers</x:v>
+      </x:c>
+      <x:c r="D441" s="3" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="E441" s="3" t="str">
+        <x:v>Cargo organization</x:v>
+      </x:c>
+      <x:c r="F441" s="3" t="str">
+        <x:v>Food direction / item proposal. Consumption values, ingredient compatibility and packaging behavior unresolved.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A6:A1005">
-      <x:formula1>'Items'!$A$6:$A$304</x:formula1>
+      <x:formula1>'Items'!$A$6:$A$318</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D6:D1005">
       <x:formula1>"Primary,Secondary"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E6:E1005">
-      <x:formula1>'Taxonomy'!$B$56:$B$128</x:formula1>
+      <x:formula1>'Taxonomy'!$B$60:$B$134</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b4b2846244f42bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25201691a7ee45b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39148,7 +40827,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6121a759c0274a56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d943dd22670479d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39514,7 +41193,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcd5659b5a9e4e66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb1bd0be42834fe9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39617,7 +41296,7 @@
       </x:c>
       <x:c r="B8" s="9" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A8)</x:f>
-        <x:v>92</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Raw and processed minerals, fauna materials, fuels, gems and industrial chemistry</x:v>
@@ -39652,13 +41331,13 @@
         <x:v>Survival contents</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>Not discrete items</x:v>
+        <x:v>Baseline reserve remains canister-owned</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>Living algae in its attached personal canister</x:v>
+        <x:v>Existing attached algae reserve is distinct from newly prepared drink/bar/meal servings</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Do not create a duplicate algae stack</x:v>
+        <x:v>Processing quantities and consumption transfers must account for source algae and prepared servings once.</x:v>
       </x:c>
       <x:c r="E10" s="4" t="str">
         <x:v>Planning scope</x:v>
@@ -39756,7 +41435,7 @@
       </x:c>
       <x:c r="B16" s="41" t="n">
         <x:f>COUNTIF(Items!$C$6:$C$1005,A16)</x:f>
-        <x:v>17</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C16" s="41" t="str">
         <x:v>Items assigned to the broad Containers category, including tools/closures in the original vessel family</x:v>
@@ -40026,7 +41705,7 @@
       </x:c>
       <x:c r="B31" s="4" t="n">
         <x:f>COUNTIF(Items!$AA$6:$AA$1005,"Ceramic")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic feed mixture")+COUNTIF(Items!$AA$6:$AA$1005,"Ceramic and metal")</x:f>
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C31" s="4" t="str">
         <x:v>Items classified as Ceramic, Ceramic feed mixture or Ceramic and metal</x:v>
@@ -40200,10 +41879,46 @@
         <x:v>Item family</x:v>
       </x:c>
     </x:row>
+    <x:row r="41" ht="115" customHeight="1">
+      <x:c r="A41" s="4" t="str">
+        <x:v>Consumables</x:v>
+      </x:c>
+      <x:c r="B41" s="4" t="n">
+        <x:f>COUNTIF(Items!$C$6:$C$1005,A41)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C41" s="4" t="str">
+        <x:v>Prepared Phagia drinks, ration/dried bars, meals and fauna-mixed delicacies</x:v>
+      </x:c>
+      <x:c r="D41" s="4" t="str">
+        <x:v>Prepared servings differ from the existing attached baseline algae reserve. Exact consumption effects and serving amounts remain open.</x:v>
+      </x:c>
+      <x:c r="E41" s="4" t="str">
+        <x:v>Primary category</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="115" customHeight="1">
+      <x:c r="A42" s="4" t="str">
+        <x:v>Phagia food and packaging</x:v>
+      </x:c>
+      <x:c r="B42" s="4" t="n">
+        <x:f>COUNTIF(Items!$D$6:$D$1005,"Phagia drink")+COUNTIF(Items!$D$6:$D$1005,"Phagia bar")+COUNTIF(Items!$D$6:$D$1005,"Phagia prepared meal")+COUNTIF(Items!$D$6:$D$1005,"Phagia delicacy")+COUNTIF(Items!$D$6:$D$1005,"Prepared fauna food ingredient")+COUNTIF(Items!$D$6:$D$1005,"Food packaging")</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C42" s="4" t="str">
+        <x:v>Nine prepared consumables, two edible-fauna intermediates and three food-service carriers</x:v>
+      </x:c>
+      <x:c r="D42" s="4" t="str">
+        <x:v>Food/industrial chemistry and payload/container ownership remain distinct.</x:v>
+      </x:c>
+      <x:c r="E42" s="4" t="str">
+        <x:v>Item family</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ca94f1076a441e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R315b061ba3744af3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40267,7 +41982,7 @@
       </x:c>
       <x:c r="B8" s="9" t="str">
         <x:f>COUNTA(Items!$A$6:$A$1005)&amp;" catalog entries: "&amp;COUNTIF(Items!$AC$6:$AC$1005,"Existing definition")&amp;" existing definition IDs and "&amp;(COUNTA(Items!$A$6:$A$1005)-COUNTIF(Items!$AC$6:$AC$1005,"Existing definition"))&amp;" design/source concepts."</x:f>
-        <x:v>299 catalog entries: 18 existing definition IDs and 281 design/source concepts.</x:v>
+        <x:v>313 catalog entries: 18 existing definition IDs and 295 design/source concepts.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -41012,7 +42727,7 @@
         <x:v>Adding a new item</x:v>
       </x:c>
       <x:c r="B101" s="4" t="str">
-        <x:v>Add one row inside ItemsTable with a unique Item ID. Fill category/subtype, source/status, W:AC and optional search aliases U; copy the AD search formula. Add exactly one Primary relationship in Item uses plus any Secondary rows, copying linked formulas. Extend validation sources and bounded references beyond row 1005 when needed. Current dropdown item-ID source ends at row 304.</x:v>
+        <x:v>Add one row inside ItemsTable with a unique Item ID. Fill category/subtype, source/status, W:AC and optional search aliases U; copy the AD search formula. Add exactly one Primary relationship in Item uses plus any Secondary rows, copying linked formulas. Extend validation sources and bounded references beyond row 1005 when needed. Current dropdown item-ID source ends at row 318.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="85" customHeight="1">
@@ -41356,7 +43071,7 @@
         <x:v>Main categories and families</x:v>
       </x:c>
       <x:c r="B144" s="4" t="str">
-        <x:v>Categories &gt; Grouping = Primary category gives nine mutually exclusive groups covering every master entry once. Item family and Planning scope rows may overlap; their counts must not be added to primary category totals.</x:v>
+        <x:v>Categories &gt; Grouping = Primary category gives ten mutually exclusive groups covering every master entry once. Item family and Planning scope rows may overlap; their counts must not be added to primary category totals.</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="90" customHeight="1">
@@ -41383,10 +43098,58 @@
         <x:v>One Primary relationship per item must link back to its master Primary use. Each additional purpose gets one Secondary row; avoid duplicate Item ID + Use pairs. Names/categories are linked by ID. Use native header filters and whole-table sorts to keep rows and source context together.</x:v>
       </x:c>
     </x:row>
+    <x:row r="148" ht="105" customHeight="1">
+      <x:c r="A148" s="4" t="str">
+        <x:v>Processed Phagia direction</x:v>
+      </x:c>
+      <x:c r="B148" s="4" t="str">
+        <x:v>Author confirms that eating/drinking Phagia can be processed into higher-performing consumables, including drinkable portions, algae bars, dried bars and prepared meals. Phagia follows the lore spelling; phagea/algae aliases support search. Intended performance is qualitative, with no assigned nutrition, hydration, healing or stamina numbers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="105" customHeight="1">
+      <x:c r="A149" s="4" t="str">
+        <x:v>Delicacy direction</x:v>
+      </x:c>
+      <x:c r="B149" s="4" t="str">
+        <x:v>Selected edible fauna resources may combine with Phagia to make high-quality delicacies. Fauna remains generally poor nutrition; the algae retains its nutritional foundation. Specific flakes, paste and composed dishes are proposals, not a conventional meat or fat supply.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="105" customHeight="1">
+      <x:c r="A150" s="4" t="str">
+        <x:v>Food qualification</x:v>
+      </x:c>
+      <x:c r="B150" s="4" t="str">
+        <x:v>Only selected species-specific edible fractions are food candidates. Lubricants, venom, etchants, binders and general ichor are not meal ingredients by default. Heating, drying or refining does not automatically establish edibility or remove toxicity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="105" customHeight="1">
+      <x:c r="A151" s="4" t="str">
+        <x:v>Food and vessel ownership</x:v>
+      </x:c>
+      <x:c r="B151" s="4" t="str">
+        <x:v>Prepared servings are new food products rather than a duplicate baseline algae stack. A reusable flask/case/meal carrier and its food payload are separate conceptual records. Future recipes must account for algae inputs, prepared portions, containers and reuse without duplicating material.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="105" customHeight="1">
+      <x:c r="A152" s="4" t="str">
+        <x:v>Preparation and preservation</x:v>
+      </x:c>
+      <x:c r="B152" s="4" t="str">
+        <x:v>Pressing, drying, concentrating, cooking and portioning are candidate processing lanes; no temperatures, ratios, yields, expiry timers or preservation guarantees are approved. Source live-culture/respiratory properties are not automatically retained by prepared meals. Cooking follows the setting fire/air rules; no natural-water or cloth recipe assumed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="105" customHeight="1">
+      <x:c r="A153" s="4" t="str">
+        <x:v>Food filters</x:v>
+      </x:c>
+      <x:c r="B153" s="4" t="str">
+        <x:v>Category = Consumables selects ready food/drink portions. Item type distinguishes Food consumable, Drink consumable, Food material and packaging carriers. Subtype separates Phagia drink/bar/prepared meal/delicacy, prepared edible-fauna ingredients and food packaging. Item uses adds Nutrition, Hydration and Food preparation relationships.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a4510f234c24b6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R247d3d2908ee4ef9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42230,7 +43993,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2165680f86d64d4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40ddb677b8e44e96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42473,7 +44236,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff43dbe606a14e00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29e635a661ad4c43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42877,7 +44640,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd09061fea11472f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63d3cc5b243f4bb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43553,7 +45316,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reea443f4cd564451"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f326e39ae6e4142"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>